<commit_message>
udated with scenario 1004
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="7545"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="145">
   <si>
     <t>1</t>
   </si>
@@ -441,7 +441,16 @@
     <t>Scenario4</t>
   </si>
   <si>
-    <t>4|5</t>
+    <t>ST-G0-01-1-R</t>
+  </si>
+  <si>
+    <t>MoveLPNQty</t>
+  </si>
+  <si>
+    <t>RecQty2</t>
+  </si>
+  <si>
+    <t>Scenario2</t>
   </si>
 </sst>
 </file>
@@ -554,12 +563,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -887,7 +894,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -901,9 +908,10 @@
     <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.5703125" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -937,175 +945,226 @@
       <c r="K1" s="1" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="L1" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="15" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="L2" s="15"/>
+    </row>
+    <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="L3" s="15"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C4" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D4" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E4" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G4" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H4" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I4" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J4" s="15" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C5" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D5" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E5" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F5" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G5" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H5" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I5" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J5" s="15" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C6" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D6" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E6" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G6" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H6" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I6" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J6" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K6" s="15" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="L6" s="15"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C7" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D7" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E7" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F7" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G7" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H7" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="J7" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="K7" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="I6" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>135</v>
-      </c>
+      <c r="L7" s="13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L8" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1115,147 +1174,134 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="2"/>
+    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="3" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="13"/>
+      <c r="G2" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="H2" s="15" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="F3" s="13"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="13"/>
+      <c r="G4" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="H4" s="15" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="E5" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="F5" s="15" t="s">
+      <c r="E5" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G5" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="G5" s="17" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>131</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="G6" s="17" t="s">
+      <c r="H5" s="15" t="s">
         <v>135</v>
       </c>
     </row>
@@ -1270,552 +1316,552 @@
   <dimension ref="A1:B68"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="14"/>
-    <col min="2" max="2" width="39.5703125" style="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="14"/>
+    <col min="1" max="1" width="9.140625" style="12"/>
+    <col min="2" max="2" width="39.5703125" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="7" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="7" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="7" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="7" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="7" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="7" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="7" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="7" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="7" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="7" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="7" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="7" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="7" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="7" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="7" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="7" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="7" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="7" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="7" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="7" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="7" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="8" t="s">
+      <c r="A29" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="7" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="8" t="s">
+      <c r="A30" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="7" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="9" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="8" t="s">
+      <c r="A33" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="9" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B34" s="12" t="s">
+      <c r="B34" s="10" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B35" s="12" t="s">
+      <c r="B35" s="10" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="8" t="s">
+      <c r="A36" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B36" s="12" t="s">
+      <c r="B36" s="10" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="8" t="s">
+      <c r="A37" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B37" s="12" t="s">
+      <c r="B37" s="10" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="10" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="8" t="s">
+      <c r="A39" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B39" s="12" t="s">
+      <c r="B39" s="10" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="8" t="s">
+      <c r="A40" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="B40" s="10" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="8" t="s">
+      <c r="A41" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B41" s="12" t="s">
+      <c r="B41" s="10" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="8" t="s">
+      <c r="A42" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B42" s="12" t="s">
+      <c r="B42" s="10" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="8" t="s">
+      <c r="A43" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B43" s="12" t="s">
+      <c r="B43" s="10" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="8" t="s">
+      <c r="A44" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B44" s="12" t="s">
+      <c r="B44" s="10" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="8" t="s">
+      <c r="A45" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B45" s="12" t="s">
+      <c r="B45" s="10" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="8" t="s">
+      <c r="A46" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B46" s="12" t="s">
+      <c r="B46" s="10" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="8" t="s">
+      <c r="A47" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="B47" s="12" t="s">
+      <c r="B47" s="10" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="8" t="s">
+      <c r="A48" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="B48" s="12" t="s">
+      <c r="B48" s="10" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="8" t="s">
+      <c r="A49" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B49" s="12" t="s">
+      <c r="B49" s="10" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="8" t="s">
+      <c r="A50" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B50" s="12" t="s">
+      <c r="B50" s="10" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" s="8" t="s">
+      <c r="A51" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B51" s="12" t="s">
+      <c r="B51" s="10" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" s="8" t="s">
+      <c r="A52" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B52" s="12" t="s">
+      <c r="B52" s="10" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" s="8" t="s">
+      <c r="A53" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B53" s="12" t="s">
+      <c r="B53" s="10" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" s="8" t="s">
+      <c r="A54" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="B54" s="12" t="s">
+      <c r="B54" s="10" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" s="8" t="s">
+      <c r="A55" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B55" s="12" t="s">
+      <c r="B55" s="10" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" s="8" t="s">
+      <c r="A56" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="B56" s="12" t="s">
+      <c r="B56" s="10" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="8" t="s">
+      <c r="A57" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="B57" s="12" t="s">
+      <c r="B57" s="10" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" s="8" t="s">
+      <c r="A58" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B58" s="12" t="s">
+      <c r="B58" s="10" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" s="8" t="s">
+      <c r="A59" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B59" s="12" t="s">
+      <c r="B59" s="10" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" s="8" t="s">
+      <c r="A60" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B60" s="12" t="s">
+      <c r="B60" s="10" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" s="8" t="s">
+      <c r="A61" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="B61" s="12" t="s">
+      <c r="B61" s="10" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" s="8" t="s">
+      <c r="A62" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B62" s="12" t="s">
+      <c r="B62" s="10" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" s="8" t="s">
+      <c r="A63" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="B63" s="12" t="s">
+      <c r="B63" s="10" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="8" t="s">
+      <c r="A64" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="B64" s="12" t="s">
+      <c r="B64" s="10" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" s="8" t="s">
+      <c r="A65" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B65" s="12" t="s">
+      <c r="B65" s="10" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" s="8" t="s">
+      <c r="A66" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B66" s="13" t="s">
+      <c r="B66" s="11" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="8" t="s">
+      <c r="A67" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B67" s="13" t="s">
+      <c r="B67" s="11" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="8" t="s">
+      <c r="A68" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B68" s="10" t="s">
+      <c r="B68" s="8" t="s">
         <v>55</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated scripts with new scenarios
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="148">
   <si>
     <t>1</t>
   </si>
@@ -39,42 +39,9 @@
     <t>Account</t>
   </si>
   <si>
-    <t>EmployeeID</t>
-  </si>
-  <si>
-    <t>ZipCode</t>
-  </si>
-  <si>
-    <t>FirstName</t>
-  </si>
-  <si>
-    <t>Phone1</t>
-  </si>
-  <si>
-    <t>Address1</t>
-  </si>
-  <si>
-    <t>CustomerPO#</t>
-  </si>
-  <si>
-    <t>ABT</t>
-  </si>
-  <si>
-    <t>123456</t>
-  </si>
-  <si>
-    <t>48755</t>
-  </si>
-  <si>
-    <t>1234567890</t>
-  </si>
-  <si>
     <t>7181E-01</t>
   </si>
   <si>
-    <t>ABT-</t>
-  </si>
-  <si>
     <t>Item_Ref</t>
   </si>
   <si>
@@ -375,18 +342,6 @@
     <t>67</t>
   </si>
   <si>
-    <t>JACK</t>
-  </si>
-  <si>
-    <t>JILL</t>
-  </si>
-  <si>
-    <t>ABC</t>
-  </si>
-  <si>
-    <t>XYZ</t>
-  </si>
-  <si>
     <t>Scenario8</t>
   </si>
   <si>
@@ -414,9 +369,6 @@
     <t>EA</t>
   </si>
   <si>
-    <t>07-12-2022</t>
-  </si>
-  <si>
     <t>Scenario1</t>
   </si>
   <si>
@@ -451,6 +403,63 @@
   </si>
   <si>
     <t>Scenario2</t>
+  </si>
+  <si>
+    <t>Scenario5</t>
+  </si>
+  <si>
+    <t>5|6</t>
+  </si>
+  <si>
+    <t>FG-000246-01</t>
+  </si>
+  <si>
+    <t>ReturnCode</t>
+  </si>
+  <si>
+    <t>FinalDispCode</t>
+  </si>
+  <si>
+    <t>UD</t>
+  </si>
+  <si>
+    <t>ASNId</t>
+  </si>
+  <si>
+    <t>Scenario6</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>Scenario9</t>
+  </si>
+  <si>
+    <t>12-31-2022</t>
+  </si>
+  <si>
+    <t>Scenario7</t>
+  </si>
+  <si>
+    <t>Scenario10</t>
+  </si>
+  <si>
+    <t>DM</t>
+  </si>
+  <si>
+    <t>Scenario11</t>
+  </si>
+  <si>
+    <t>LockCode</t>
+  </si>
+  <si>
+    <t>UD-Undeliverable</t>
+  </si>
+  <si>
+    <t>DT - Damaged in Transit from Supplier</t>
+  </si>
+  <si>
+    <t>DM-Damaged Return</t>
   </si>
 </sst>
 </file>
@@ -510,7 +519,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -557,13 +566,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -588,6 +621,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -894,24 +929,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -919,252 +949,267 @@
         <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>10</v>
+        <v>118</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>126</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>11</v>
+        <v>135</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>14</v>
+        <v>111</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>0</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E2" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="F2" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="H2" s="14" t="s">
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+    </row>
+    <row r="3" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="D3" s="13" t="s">
         <v>2</v>
-      </c>
-      <c r="J2" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="L2" s="15"/>
-    </row>
-    <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>15</v>
       </c>
       <c r="E3" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="F3" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="H3" s="14" t="s">
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="D4" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="L3" s="15"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="I4" s="13" t="s">
+      <c r="B6" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="13" t="s">
         <v>2</v>
-      </c>
-      <c r="J4" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="I5" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>15</v>
       </c>
       <c r="E6" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="F6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="I6" s="13" t="s">
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="J6" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="K6" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="L6" s="15"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="E7" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F8" s="13"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F9" s="13"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="15" t="s">
+      <c r="B10" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E10" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="F7" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="I7" s="13" t="s">
+      <c r="F10" s="13"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="J7" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" s="13" t="s">
+      <c r="E11" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="L7" s="13" t="s">
+      <c r="B12" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C12" s="14" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="L8" s="2"/>
+      <c r="D12" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15" t="s">
+        <v>147</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1174,7 +1219,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
@@ -1183,126 +1228,340 @@
     <col min="6" max="6" width="9.140625" style="2"/>
     <col min="7" max="7" width="13.5703125" customWidth="1"/>
     <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>143</v>
-      </c>
       <c r="G1" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+      <c r="H1" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="F2" s="13"/>
       <c r="G2" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="H2" s="15" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+      <c r="H2" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C3" s="13" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="F3" s="13"/>
       <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H3" s="17"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="F4" s="13"/>
       <c r="G4" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="H4" s="15" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="D5" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="E5" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="H5" s="15" t="s">
-        <v>135</v>
+      <c r="C7" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I8" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="J8" s="15" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="J9" s="15" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I10" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="J10" s="15" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I12" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="J12" s="15" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1323,7 +1582,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>5</v>
@@ -1334,7 +1593,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1342,63 +1601,63 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -1406,463 +1665,463 @@
         <v>3</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="B68" s="8" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added new senarios and updated scripts
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="7545"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="7545" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="165">
   <si>
     <t>1</t>
   </si>
@@ -411,9 +411,6 @@
     <t>5|6</t>
   </si>
   <si>
-    <t>FG-000246-01</t>
-  </si>
-  <si>
     <t>ReturnCode</t>
   </si>
   <si>
@@ -463,6 +460,57 @@
   </si>
   <si>
     <t>Scenario12</t>
+  </si>
+  <si>
+    <t>Scenario13</t>
+  </si>
+  <si>
+    <t>No data found</t>
+  </si>
+  <si>
+    <t>Scenario14</t>
+  </si>
+  <si>
+    <t>ChangeQty</t>
+  </si>
+  <si>
+    <t>ReasonCode</t>
+  </si>
+  <si>
+    <t>CC</t>
+  </si>
+  <si>
+    <t>Scenario15</t>
+  </si>
+  <si>
+    <t>SH</t>
+  </si>
+  <si>
+    <t>MC</t>
+  </si>
+  <si>
+    <t>Scenario16</t>
+  </si>
+  <si>
+    <t>Scenario17</t>
+  </si>
+  <si>
+    <t>Scenario18</t>
+  </si>
+  <si>
+    <t>Scenario19</t>
+  </si>
+  <si>
+    <t>Scenario20</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <t>Scrap Item</t>
+  </si>
+  <si>
+    <t>Scenario21</t>
   </si>
 </sst>
 </file>
@@ -599,7 +647,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -626,6 +674,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -932,7 +985,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -964,10 +1017,10 @@
         <v>126</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1096,7 +1149,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>111</v>
@@ -1111,12 +1164,12 @@
       <c r="F9" s="13"/>
       <c r="G9" s="15"/>
       <c r="H9" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>111</v>
@@ -1134,7 +1187,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>111</v>
@@ -1152,7 +1205,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>111</v>
@@ -1167,12 +1220,12 @@
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
       <c r="H12" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>111</v>
@@ -1187,12 +1240,12 @@
       <c r="F13" s="15"/>
       <c r="G13" s="15"/>
       <c r="H13" s="15" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>111</v>
@@ -1205,7 +1258,181 @@
       <c r="F14" s="15"/>
       <c r="G14" s="15"/>
       <c r="H14" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15" s="13"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" s="13"/>
+      <c r="E16" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="13"/>
+      <c r="E17" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" s="13"/>
+      <c r="E18" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="13"/>
+      <c r="E19" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D22" s="2"/>
+      <c r="E22" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="E23" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="H23" s="15" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -1216,20 +1443,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" customWidth="1"/>
     <col min="6" max="6" width="9.140625" style="2"/>
     <col min="7" max="7" width="13.5703125" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" customWidth="1"/>
     <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>8</v>
       </c>
@@ -1255,13 +1485,22 @@
         <v>118</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="L1" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="M1" s="19" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
@@ -1279,15 +1518,17 @@
       </c>
       <c r="F2" s="13"/>
       <c r="G2" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H2" s="17" t="s">
         <v>119</v>
       </c>
       <c r="I2" s="15"/>
       <c r="J2" s="15"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>2</v>
       </c>
@@ -1308,8 +1549,10 @@
       <c r="H3" s="17"/>
       <c r="I3" s="15"/>
       <c r="J3" s="15"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>45</v>
       </c>
@@ -1327,15 +1570,17 @@
       </c>
       <c r="F4" s="13"/>
       <c r="G4" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H4" s="17" t="s">
         <v>119</v>
       </c>
       <c r="I4" s="15"/>
       <c r="J4" s="15"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>46</v>
       </c>
@@ -1355,15 +1600,17 @@
         <v>62</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H5" s="17" t="s">
         <v>119</v>
       </c>
       <c r="I5" s="15"/>
       <c r="J5" s="15"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>47</v>
       </c>
@@ -1381,20 +1628,22 @@
       </c>
       <c r="F6" s="13"/>
       <c r="G6" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>119</v>
       </c>
       <c r="I6" s="15"/>
       <c r="J6" s="15"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>48</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>61</v>
@@ -1403,19 +1652,21 @@
         <v>116</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="F7" s="13"/>
       <c r="G7" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H7" s="17" t="s">
         <v>119</v>
       </c>
       <c r="I7" s="15"/>
       <c r="J7" s="15"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K7" s="15"/>
+      <c r="L7" s="15"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>49</v>
       </c>
@@ -1433,19 +1684,23 @@
       </c>
       <c r="F8" s="13"/>
       <c r="G8" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H8" s="17" t="s">
         <v>119</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+      <c r="K8" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="L8" s="15"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>50</v>
       </c>
@@ -1459,23 +1714,27 @@
         <v>116</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F9" s="13"/>
       <c r="G9" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H9" s="17" t="s">
         <v>119</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+      <c r="K9" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="L9" s="15"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>51</v>
       </c>
@@ -1493,19 +1752,23 @@
       </c>
       <c r="F10" s="13"/>
       <c r="G10" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H10" s="17" t="s">
         <v>119</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J10" s="15" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+      <c r="K10" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="L10" s="15"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>3</v>
       </c>
@@ -1523,15 +1786,17 @@
       </c>
       <c r="F11" s="13"/>
       <c r="G11" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H11" s="17" t="s">
         <v>119</v>
       </c>
       <c r="I11" s="15"/>
       <c r="J11" s="15"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K11" s="15"/>
+      <c r="L11" s="15"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>52</v>
       </c>
@@ -1549,19 +1814,23 @@
       </c>
       <c r="F12" s="13"/>
       <c r="G12" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H12" s="17" t="s">
         <v>119</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J12" s="15" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+      <c r="K12" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L12" s="15"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>53</v>
       </c>
@@ -1575,11 +1844,285 @@
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H13" s="17"/>
       <c r="I13" s="15"/>
       <c r="J13" s="15"/>
+      <c r="K13" s="15"/>
+      <c r="L13" s="15"/>
+    </row>
+    <row r="14" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="I14" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="J14" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="K14" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="L14" s="15"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" s="15"/>
+      <c r="G15" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="L15" s="15" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F16" s="15"/>
+      <c r="G16" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="L16" s="15" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F17" s="15"/>
+      <c r="G17" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="I17" s="15"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="L17" s="15" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F18" s="15"/>
+      <c r="G18" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="L18" s="15" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F19" s="15"/>
+      <c r="G19" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H19" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="15" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F20" s="15"/>
+      <c r="G20" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H21" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="M21" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C22" s="13"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H22" s="17"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="15"/>
+      <c r="L22" s="15"/>
+      <c r="M22" s="2" t="s">
+        <v>163</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added one more user story scenrio
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="168">
   <si>
     <t>1</t>
   </si>
@@ -511,6 +511,15 @@
   </si>
   <si>
     <t>Scenario21</t>
+  </si>
+  <si>
+    <t>Scenario22</t>
+  </si>
+  <si>
+    <t>Scenario23</t>
+  </si>
+  <si>
+    <t>Scenario24</t>
   </si>
 </sst>
 </file>
@@ -570,7 +579,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -641,13 +650,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -679,6 +697,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -985,7 +1004,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -1435,6 +1454,57 @@
         <v>145</v>
       </c>
     </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="H24" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="H26" s="15" t="s">
+        <v>146</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1443,7 +1513,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
@@ -1457,6 +1527,7 @@
     <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1695,9 +1766,7 @@
       <c r="J8" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="K8" s="15" t="s">
-        <v>133</v>
-      </c>
+      <c r="K8" s="15"/>
       <c r="L8" s="15"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -1729,9 +1798,7 @@
       <c r="J9" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="K9" s="15" t="s">
-        <v>133</v>
-      </c>
+      <c r="K9" s="15"/>
       <c r="L9" s="15"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -1763,9 +1830,7 @@
       <c r="J10" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="K10" s="15" t="s">
-        <v>133</v>
-      </c>
+      <c r="K10" s="15"/>
       <c r="L10" s="15"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -1825,9 +1890,7 @@
       <c r="J12" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="K12" s="15" t="s">
-        <v>141</v>
-      </c>
+      <c r="K12" s="15"/>
       <c r="L12" s="15"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -1881,9 +1944,7 @@
       <c r="J14" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="K14" s="21" t="s">
-        <v>133</v>
-      </c>
+      <c r="K14" s="21"/>
       <c r="L14" s="15"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -2064,7 +2125,9 @@
       <c r="G20" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="H20" s="15"/>
+      <c r="H20" s="15" t="s">
+        <v>119</v>
+      </c>
       <c r="I20" s="15"/>
       <c r="J20" s="15"/>
       <c r="K20" s="15"/>
@@ -2100,7 +2163,7 @@
       </c>
     </row>
     <row r="22" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="18" t="s">
         <v>62</v>
       </c>
       <c r="B22" s="14" t="s">
@@ -2122,6 +2185,90 @@
       <c r="L22" s="15"/>
       <c r="M22" s="2" t="s">
         <v>163</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H23" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I23" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="J23" s="23" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H24" s="17" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H25" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="I25" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="J25" s="23" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated step def rf menu ith product class
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="170">
   <si>
     <t>1</t>
   </si>
@@ -520,6 +520,12 @@
   </si>
   <si>
     <t>Scenario24</t>
+  </si>
+  <si>
+    <t>ProductStatus</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
 </sst>
 </file>
@@ -1513,7 +1519,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
@@ -1524,13 +1530,14 @@
     <col min="7" max="7" width="13.5703125" customWidth="1"/>
     <col min="8" max="8" width="11.7109375" customWidth="1"/>
     <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>8</v>
       </c>
@@ -1559,19 +1566,22 @@
         <v>131</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="L1" s="19" t="s">
+      <c r="M1" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="M1" s="19" t="s">
+      <c r="N1" s="19" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
@@ -1598,8 +1608,9 @@
       <c r="J2" s="15"/>
       <c r="K2" s="15"/>
       <c r="L2" s="15"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M2" s="15"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>2</v>
       </c>
@@ -1622,8 +1633,9 @@
       <c r="J3" s="15"/>
       <c r="K3" s="15"/>
       <c r="L3" s="15"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M3" s="15"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>45</v>
       </c>
@@ -1650,8 +1662,9 @@
       <c r="J4" s="15"/>
       <c r="K4" s="15"/>
       <c r="L4" s="15"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M4" s="15"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>46</v>
       </c>
@@ -1680,8 +1693,9 @@
       <c r="J5" s="15"/>
       <c r="K5" s="15"/>
       <c r="L5" s="15"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M5" s="15"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>47</v>
       </c>
@@ -1708,8 +1722,9 @@
       <c r="J6" s="15"/>
       <c r="K6" s="15"/>
       <c r="L6" s="15"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M6" s="15"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>48</v>
       </c>
@@ -1736,8 +1751,9 @@
       <c r="J7" s="15"/>
       <c r="K7" s="15"/>
       <c r="L7" s="15"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M7" s="15"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>49</v>
       </c>
@@ -1763,13 +1779,14 @@
       <c r="I8" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="J8" s="15" t="s">
+      <c r="J8" s="15"/>
+      <c r="K8" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="K8" s="15"/>
       <c r="L8" s="15"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M8" s="15"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>50</v>
       </c>
@@ -1795,13 +1812,14 @@
       <c r="I9" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="J9" s="15" t="s">
+      <c r="J9" s="15"/>
+      <c r="K9" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="K9" s="15"/>
       <c r="L9" s="15"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M9" s="15"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>51</v>
       </c>
@@ -1827,13 +1845,14 @@
       <c r="I10" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="J10" s="15" t="s">
+      <c r="J10" s="15"/>
+      <c r="K10" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="K10" s="15"/>
       <c r="L10" s="15"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M10" s="15"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>3</v>
       </c>
@@ -1860,8 +1879,9 @@
       <c r="J11" s="15"/>
       <c r="K11" s="15"/>
       <c r="L11" s="15"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M11" s="15"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>52</v>
       </c>
@@ -1887,13 +1907,14 @@
       <c r="I12" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="J12" s="15" t="s">
+      <c r="J12" s="15"/>
+      <c r="K12" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="K12" s="15"/>
       <c r="L12" s="15"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M12" s="15"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>53</v>
       </c>
@@ -1911,11 +1932,14 @@
       </c>
       <c r="H13" s="17"/>
       <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
+      <c r="J13" s="15" t="s">
+        <v>169</v>
+      </c>
       <c r="K13" s="15"/>
       <c r="L13" s="15"/>
-    </row>
-    <row r="14" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="M13" s="15"/>
+    </row>
+    <row r="14" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>54</v>
       </c>
@@ -1941,13 +1965,14 @@
       <c r="I14" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="J14" s="21" t="s">
+      <c r="J14" s="21"/>
+      <c r="K14" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="K14" s="21"/>
-      <c r="L14" s="15"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="L14" s="21"/>
+      <c r="M14" s="15"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>55</v>
       </c>
@@ -1972,14 +1997,15 @@
       </c>
       <c r="I15" s="15"/>
       <c r="J15" s="15"/>
-      <c r="K15" s="13" t="s">
+      <c r="K15" s="15"/>
+      <c r="L15" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="L15" s="15" t="s">
+      <c r="M15" s="15" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
         <v>56</v>
       </c>
@@ -2004,14 +2030,15 @@
       </c>
       <c r="I16" s="15"/>
       <c r="J16" s="15"/>
-      <c r="K16" s="13" t="s">
+      <c r="K16" s="15"/>
+      <c r="L16" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="L16" s="15" t="s">
+      <c r="M16" s="15" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
         <v>57</v>
       </c>
@@ -2036,14 +2063,15 @@
       </c>
       <c r="I17" s="15"/>
       <c r="J17" s="15"/>
-      <c r="K17" s="13" t="s">
+      <c r="K17" s="15"/>
+      <c r="L17" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="L17" s="15" t="s">
+      <c r="M17" s="15" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
         <v>58</v>
       </c>
@@ -2068,14 +2096,15 @@
       </c>
       <c r="I18" s="15"/>
       <c r="J18" s="15"/>
-      <c r="K18" s="13" t="s">
+      <c r="K18" s="15"/>
+      <c r="L18" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="L18" s="15" t="s">
+      <c r="M18" s="15" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>59</v>
       </c>
@@ -2101,11 +2130,12 @@
       <c r="I19" s="15"/>
       <c r="J19" s="15"/>
       <c r="K19" s="15"/>
-      <c r="L19" s="15" t="s">
+      <c r="L19" s="15"/>
+      <c r="M19" s="15" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
         <v>60</v>
       </c>
@@ -2131,11 +2161,12 @@
       <c r="I20" s="15"/>
       <c r="J20" s="15"/>
       <c r="K20" s="15"/>
-      <c r="L20" s="15" t="s">
+      <c r="L20" s="15"/>
+      <c r="M20" s="15" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
         <v>61</v>
       </c>
@@ -2158,11 +2189,11 @@
       <c r="H21" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="M21" t="s">
+      <c r="N21" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="22" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
         <v>62</v>
       </c>
@@ -2180,14 +2211,17 @@
       </c>
       <c r="H22" s="17"/>
       <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
+      <c r="J22" s="15" t="s">
+        <v>169</v>
+      </c>
       <c r="K22" s="15"/>
       <c r="L22" s="15"/>
-      <c r="M22" s="2" t="s">
+      <c r="M22" s="15"/>
+      <c r="N22" s="2" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
         <v>63</v>
       </c>
@@ -2213,11 +2247,12 @@
       <c r="I23" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="J23" s="23" t="s">
+      <c r="J23" s="23"/>
+      <c r="K23" s="23" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
         <v>64</v>
       </c>
@@ -2241,7 +2276,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
         <v>65</v>
       </c>
@@ -2267,7 +2302,8 @@
       <c r="I25" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="J25" s="23" t="s">
+      <c r="J25" s="23"/>
+      <c r="K25" s="23" t="s">
         <v>141</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated with NVI scenarios
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="7545" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="7545"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="171">
   <si>
     <t>1</t>
   </si>
@@ -369,9 +369,6 @@
     <t>EA</t>
   </si>
   <si>
-    <t>Scenario1</t>
-  </si>
-  <si>
     <t>RecLocation</t>
   </si>
   <si>
@@ -387,12 +384,6 @@
     <t>76</t>
   </si>
   <si>
-    <t>Scenario3</t>
-  </si>
-  <si>
-    <t>Scenario4</t>
-  </si>
-  <si>
     <t>ST-G0-01-1-R</t>
   </si>
   <si>
@@ -402,12 +393,6 @@
     <t>RecQty2</t>
   </si>
   <si>
-    <t>Scenario2</t>
-  </si>
-  <si>
-    <t>Scenario5</t>
-  </si>
-  <si>
     <t>5|6</t>
   </si>
   <si>
@@ -423,9 +408,6 @@
     <t>ASNId</t>
   </si>
   <si>
-    <t>Scenario6</t>
-  </si>
-  <si>
     <t>80</t>
   </si>
   <si>
@@ -435,18 +417,9 @@
     <t>12-31-2022</t>
   </si>
   <si>
-    <t>Scenario7</t>
-  </si>
-  <si>
-    <t>Scenario10</t>
-  </si>
-  <si>
     <t>DM</t>
   </si>
   <si>
-    <t>Scenario11</t>
-  </si>
-  <si>
     <t>LockCode</t>
   </si>
   <si>
@@ -459,18 +432,9 @@
     <t>DM-Damaged Return</t>
   </si>
   <si>
-    <t>Scenario12</t>
-  </si>
-  <si>
-    <t>Scenario13</t>
-  </si>
-  <si>
     <t>No data found</t>
   </si>
   <si>
-    <t>Scenario14</t>
-  </si>
-  <si>
     <t>ChangeQty</t>
   </si>
   <si>
@@ -480,52 +444,91 @@
     <t>CC</t>
   </si>
   <si>
-    <t>Scenario15</t>
-  </si>
-  <si>
     <t>SH</t>
   </si>
   <si>
     <t>MC</t>
   </si>
   <si>
-    <t>Scenario16</t>
-  </si>
-  <si>
-    <t>Scenario17</t>
-  </si>
-  <si>
-    <t>Scenario18</t>
-  </si>
-  <si>
-    <t>Scenario19</t>
-  </si>
-  <si>
-    <t>Scenario20</t>
-  </si>
-  <si>
     <t>Reference</t>
   </si>
   <si>
     <t>Scrap Item</t>
   </si>
   <si>
-    <t>Scenario21</t>
-  </si>
-  <si>
-    <t>Scenario22</t>
-  </si>
-  <si>
-    <t>Scenario23</t>
-  </si>
-  <si>
-    <t>Scenario24</t>
-  </si>
-  <si>
     <t>ProductStatus</t>
   </si>
   <si>
     <t>NA</t>
+  </si>
+  <si>
+    <t>QSC_Scenario001</t>
+  </si>
+  <si>
+    <t>QSC_Scenario002</t>
+  </si>
+  <si>
+    <t>QSC_Scenario003</t>
+  </si>
+  <si>
+    <t>QSC_Scenario004</t>
+  </si>
+  <si>
+    <t>QSC_Scenario005</t>
+  </si>
+  <si>
+    <t>QSC_Scenario006</t>
+  </si>
+  <si>
+    <t>QSC_Scenario007</t>
+  </si>
+  <si>
+    <t>QSC_Scenario008</t>
+  </si>
+  <si>
+    <t>QSC_Scenario009</t>
+  </si>
+  <si>
+    <t>QSC_Scenario010</t>
+  </si>
+  <si>
+    <t>QSC_Scenario011</t>
+  </si>
+  <si>
+    <t>QSC_Scenario012</t>
+  </si>
+  <si>
+    <t>QSC_Scenario013</t>
+  </si>
+  <si>
+    <t>QSC_Scenario014</t>
+  </si>
+  <si>
+    <t>QSC_Scenario015</t>
+  </si>
+  <si>
+    <t>QSC_Scenario016</t>
+  </si>
+  <si>
+    <t>QSC_Scenario017</t>
+  </si>
+  <si>
+    <t>QSC_Scenario018</t>
+  </si>
+  <si>
+    <t>QSC_Scenario019</t>
+  </si>
+  <si>
+    <t>QSC_Scenario020</t>
+  </si>
+  <si>
+    <t>QSC_Scenario021</t>
+  </si>
+  <si>
+    <t>QSC_Scenario022</t>
+  </si>
+  <si>
+    <t>QSC_Scenario023</t>
   </si>
 </sst>
 </file>
@@ -1010,10 +1013,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" customWidth="1"/>
     <col min="2" max="2" width="10.85546875" customWidth="1"/>
     <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -1030,27 +1033,27 @@
         <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>134</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>117</v>
+        <v>148</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>111</v>
@@ -1060,7 +1063,7 @@
       </c>
       <c r="D2" s="13"/>
       <c r="E2" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
@@ -1068,7 +1071,7 @@
     </row>
     <row r="3" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>111</v>
@@ -1078,15 +1081,15 @@
       </c>
       <c r="D3" s="13"/>
       <c r="E3" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F3" s="15"/>
       <c r="G3" s="15"/>
       <c r="H3" s="15"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>108</v>
+        <v>150</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>111</v>
@@ -1095,14 +1098,16 @@
         <v>0</v>
       </c>
       <c r="D4" s="13"/>
-      <c r="E4" s="15"/>
+      <c r="E4" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="F4" s="15"/>
       <c r="G4" s="15"/>
       <c r="H4" s="15"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>110</v>
+        <v>151</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>111</v>
@@ -1111,405 +1116,421 @@
         <v>45</v>
       </c>
       <c r="D5" s="13"/>
-      <c r="E5" s="15"/>
+      <c r="E5" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="F5" s="15"/>
       <c r="G5" s="15"/>
       <c r="H5" s="15"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>123</v>
+        <v>152</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D6" s="13"/>
-      <c r="E6" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="F6" s="15"/>
+      <c r="E6" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>3</v>
+      </c>
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>124</v>
+        <v>153</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>46</v>
+        <v>125</v>
       </c>
       <c r="D7" s="13"/>
-      <c r="E7" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>3</v>
-      </c>
+      <c r="E7" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F7" s="13"/>
       <c r="G7" s="15"/>
       <c r="H7" s="15"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>130</v>
+        <v>49</v>
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F8" s="13"/>
       <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H8" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D9" s="13"/>
       <c r="E9" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F9" s="13"/>
       <c r="G9" s="15"/>
-      <c r="H9" s="15" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H9" s="15"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="F10" s="13"/>
+        <v>118</v>
+      </c>
+      <c r="F10" s="15"/>
       <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
+      <c r="H10" s="15" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F11" s="15"/>
       <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
+      <c r="H11" s="15" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>3</v>
+        <v>53</v>
       </c>
       <c r="D12" s="13"/>
-      <c r="E12" s="15" t="s">
-        <v>119</v>
-      </c>
+      <c r="E12" s="15"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
       <c r="H12" s="15" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D13" s="13"/>
-      <c r="E13" s="15" t="s">
-        <v>119</v>
-      </c>
+      <c r="E13" s="15"/>
       <c r="F13" s="15"/>
       <c r="G13" s="15"/>
       <c r="H13" s="15" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D14" s="13"/>
-      <c r="E14" s="15"/>
+      <c r="E14" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="F14" s="15"/>
       <c r="G14" s="15"/>
       <c r="H14" s="15" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D15" s="13"/>
-      <c r="E15" s="15"/>
+      <c r="E15" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="F15" s="15"/>
       <c r="G15" s="15"/>
       <c r="H15" s="15" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D16" s="13"/>
       <c r="E16" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F16" s="15"/>
       <c r="G16" s="15"/>
       <c r="H16" s="15" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D17" s="13"/>
       <c r="E17" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F17" s="15"/>
       <c r="G17" s="15"/>
       <c r="H17" s="15" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="D18" s="13"/>
+        <v>59</v>
+      </c>
       <c r="E18" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="15"/>
       <c r="H18" s="15" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="13"/>
+        <v>60</v>
+      </c>
       <c r="E19" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F19" s="15"/>
       <c r="G19" s="15"/>
       <c r="H19" s="15" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>59</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="D20" s="2"/>
       <c r="E20" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F20" s="15"/>
       <c r="G20" s="15"/>
       <c r="H20" s="15" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>60</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="D21" s="2"/>
       <c r="E21" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
+        <v>118</v>
+      </c>
       <c r="H21" s="15" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="D22" s="2"/>
+        <v>63</v>
+      </c>
       <c r="E22" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
+        <v>118</v>
+      </c>
       <c r="H22" s="15" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="D23" s="2"/>
+        <v>64</v>
+      </c>
       <c r="E23" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H23" s="15" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>111</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="B25" s="15" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B28" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C25" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="H25" s="15" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="B26" s="15" t="s">
+      <c r="C28" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="D28" s="13"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B29" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C26" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="H26" s="15" t="s">
-        <v>146</v>
-      </c>
+      <c r="C29" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" s="13"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="D30" s="13"/>
+      <c r="E30" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1542,7 +1563,7 @@
         <v>8</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>112</v>
@@ -1554,31 +1575,31 @@
         <v>114</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>115</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>168</v>
+        <v>146</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="M1" s="19" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="N1" s="19" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -1599,10 +1620,10 @@
       </c>
       <c r="F2" s="13"/>
       <c r="G2" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I2" s="15"/>
       <c r="J2" s="15"/>
@@ -1649,14 +1670,14 @@
         <v>116</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F4" s="13"/>
       <c r="G4" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I4" s="15"/>
       <c r="J4" s="15"/>
@@ -1684,10 +1705,10 @@
         <v>62</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I5" s="15"/>
       <c r="J5" s="15"/>
@@ -1713,10 +1734,10 @@
       </c>
       <c r="F6" s="13"/>
       <c r="G6" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I6" s="15"/>
       <c r="J6" s="15"/>
@@ -1742,10 +1763,10 @@
       </c>
       <c r="F7" s="13"/>
       <c r="G7" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I7" s="15"/>
       <c r="J7" s="15"/>
@@ -1771,17 +1792,17 @@
       </c>
       <c r="F8" s="13"/>
       <c r="G8" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="J8" s="15"/>
       <c r="K8" s="15" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="L8" s="15"/>
       <c r="M8" s="15"/>
@@ -1800,21 +1821,21 @@
         <v>116</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="F9" s="13"/>
       <c r="G9" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="J9" s="15"/>
       <c r="K9" s="15" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="L9" s="15"/>
       <c r="M9" s="15"/>
@@ -1837,17 +1858,17 @@
       </c>
       <c r="F10" s="13"/>
       <c r="G10" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="J10" s="15"/>
       <c r="K10" s="15" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
@@ -1870,10 +1891,10 @@
       </c>
       <c r="F11" s="13"/>
       <c r="G11" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I11" s="15"/>
       <c r="J11" s="15"/>
@@ -1899,17 +1920,17 @@
       </c>
       <c r="F12" s="13"/>
       <c r="G12" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="J12" s="15"/>
       <c r="K12" s="15" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
@@ -1928,12 +1949,12 @@
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H13" s="17"/>
       <c r="I13" s="15"/>
       <c r="J13" s="15" t="s">
-        <v>169</v>
+        <v>147</v>
       </c>
       <c r="K13" s="15"/>
       <c r="L13" s="15"/>
@@ -1957,17 +1978,17 @@
       </c>
       <c r="F14" s="13"/>
       <c r="G14" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H14" s="20" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I14" s="21" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="J14" s="21"/>
       <c r="K14" s="21" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="L14" s="21"/>
       <c r="M14" s="15"/>
@@ -1990,10 +2011,10 @@
       </c>
       <c r="F15" s="15"/>
       <c r="G15" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I15" s="15"/>
       <c r="J15" s="15"/>
@@ -2002,7 +2023,7 @@
         <v>100</v>
       </c>
       <c r="M15" s="15" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -2023,10 +2044,10 @@
       </c>
       <c r="F16" s="15"/>
       <c r="G16" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I16" s="15"/>
       <c r="J16" s="15"/>
@@ -2035,7 +2056,7 @@
         <v>80</v>
       </c>
       <c r="M16" s="15" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
@@ -2056,10 +2077,10 @@
       </c>
       <c r="F17" s="15"/>
       <c r="G17" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I17" s="15"/>
       <c r="J17" s="15"/>
@@ -2068,7 +2089,7 @@
         <v>100</v>
       </c>
       <c r="M17" s="15" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
@@ -2089,10 +2110,10 @@
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I18" s="15"/>
       <c r="J18" s="15"/>
@@ -2101,7 +2122,7 @@
         <v>80</v>
       </c>
       <c r="M18" s="15" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
@@ -2122,17 +2143,17 @@
       </c>
       <c r="F19" s="15"/>
       <c r="G19" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I19" s="15"/>
       <c r="J19" s="15"/>
       <c r="K19" s="15"/>
       <c r="L19" s="15"/>
       <c r="M19" s="15" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
@@ -2153,17 +2174,17 @@
       </c>
       <c r="F20" s="15"/>
       <c r="G20" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I20" s="15"/>
       <c r="J20" s="15"/>
       <c r="K20" s="15"/>
       <c r="L20" s="15"/>
       <c r="M20" s="15" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
@@ -2184,13 +2205,13 @@
       </c>
       <c r="F21" s="13"/>
       <c r="G21" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H21" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N21" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
     </row>
     <row r="22" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2207,18 +2228,18 @@
       </c>
       <c r="F22" s="13"/>
       <c r="G22" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H22" s="17"/>
       <c r="I22" s="15"/>
       <c r="J22" s="15" t="s">
-        <v>169</v>
+        <v>147</v>
       </c>
       <c r="K22" s="15"/>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
       <c r="N22" s="2" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
@@ -2239,17 +2260,17 @@
       </c>
       <c r="F23" s="13"/>
       <c r="G23" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H23" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I23" s="23" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="J23" s="23"/>
       <c r="K23" s="23" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
@@ -2270,10 +2291,10 @@
       </c>
       <c r="F24" s="13"/>
       <c r="G24" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H24" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
@@ -2294,17 +2315,17 @@
       </c>
       <c r="F25" s="13"/>
       <c r="G25" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H25" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I25" s="23" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="J25" s="23"/>
       <c r="K25" s="23" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated screenshot error and changed env from test to dev
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="174">
   <si>
     <t>1</t>
   </si>
@@ -529,6 +529,15 @@
   </si>
   <si>
     <t>QSC_Scenario023</t>
+  </si>
+  <si>
+    <t>MM3</t>
+  </si>
+  <si>
+    <t>Facility</t>
+  </si>
+  <si>
+    <t>QSC_Scenario000</t>
   </si>
 </sst>
 </file>
@@ -1013,19 +1022,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" customWidth="1"/>
     <col min="2" max="2" width="10.85546875" customWidth="1"/>
-    <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1033,504 +1043,606 @@
         <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>148</v>
+        <v>173</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="13"/>
-      <c r="E2" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F2" s="15"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G2" s="15"/>
       <c r="H2" s="15"/>
-    </row>
-    <row r="3" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I2" s="15"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="13"/>
-      <c r="E3" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F3" s="15"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G3" s="15"/>
       <c r="H3" s="15"/>
-    </row>
-    <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I3" s="15"/>
+    </row>
+    <row r="4" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D4" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F4" s="15"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G4" s="15"/>
       <c r="H4" s="15"/>
-    </row>
-    <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I4" s="15"/>
+    </row>
+    <row r="5" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C5" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F5" s="15"/>
+      <c r="C5" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G5" s="15"/>
       <c r="H5" s="15"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I5" s="15"/>
+    </row>
+    <row r="6" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>3</v>
+      <c r="C6" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="13"/>
+      <c r="F6" s="15" t="s">
+        <v>118</v>
       </c>
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I6" s="15"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C7" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F7" s="13"/>
-      <c r="G7" s="15"/>
+      <c r="C7" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>3</v>
+      </c>
       <c r="H7" s="15"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I7" s="15"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C8" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="13"/>
-      <c r="E8" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F8" s="13"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" s="13"/>
+      <c r="F8" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="G8" s="13"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C9" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="13"/>
-      <c r="E9" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F9" s="13"/>
-      <c r="G9" s="15"/>
+      <c r="C9" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="13"/>
+      <c r="F9" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="G9" s="13"/>
       <c r="H9" s="15"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I9" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C10" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="D10" s="13"/>
-      <c r="E10" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C10" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="13"/>
+      <c r="F10" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="G10" s="13"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="D11" s="13"/>
-      <c r="E11" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F11" s="15"/>
+      <c r="C11" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E11" s="13"/>
+      <c r="F11" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G11" s="15"/>
-      <c r="H11" s="15" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H11" s="15"/>
+      <c r="I11" s="15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C12" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
+      <c r="C12" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="13"/>
+      <c r="F12" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G12" s="15"/>
-      <c r="H12" s="15" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H12" s="15"/>
+      <c r="I12" s="15" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C13" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="D13" s="13"/>
-      <c r="E13" s="15"/>
+      <c r="C13" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="13"/>
       <c r="F13" s="15"/>
       <c r="G13" s="15"/>
-      <c r="H13" s="15" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H13" s="15"/>
+      <c r="I13" s="15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="D14" s="13"/>
-      <c r="E14" s="15" t="s">
-        <v>118</v>
-      </c>
+      <c r="C14" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="13"/>
       <c r="F14" s="15"/>
       <c r="G14" s="15"/>
-      <c r="H14" s="15" t="s">
+      <c r="H14" s="15"/>
+      <c r="I14" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C15" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F15" s="15"/>
+      <c r="C15" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="E15" s="13"/>
+      <c r="F15" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G15" s="15"/>
-      <c r="H15" s="15" t="s">
+      <c r="H15" s="15"/>
+      <c r="I15" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" s="13"/>
-      <c r="E16" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F16" s="15"/>
+      <c r="C16" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="13"/>
+      <c r="F16" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G16" s="15"/>
-      <c r="H16" s="15" t="s">
+      <c r="H16" s="15"/>
+      <c r="I16" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F17" s="15"/>
+      <c r="C17" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E17" s="13"/>
+      <c r="F17" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G17" s="15"/>
-      <c r="H17" s="15" t="s">
+      <c r="H17" s="15"/>
+      <c r="I17" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C18" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F18" s="15"/>
+      <c r="C18" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" s="13"/>
+      <c r="F18" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G18" s="15"/>
-      <c r="H18" s="15" t="s">
+      <c r="H18" s="15"/>
+      <c r="I18" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C19" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F19" s="15"/>
+      <c r="C19" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G19" s="15"/>
-      <c r="H19" s="15" t="s">
+      <c r="H19" s="15"/>
+      <c r="I19" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C20" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F20" s="15"/>
+      <c r="C20" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" s="15" t="s">
+        <v>118</v>
+      </c>
       <c r="G20" s="15"/>
-      <c r="H20" s="15" t="s">
+      <c r="H20" s="15"/>
+      <c r="I20" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C21" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" s="2"/>
-      <c r="E21" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="H21" s="15" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C21" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E21" s="2"/>
+      <c r="F21" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C22" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="E22" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="H22" s="15" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C22" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" s="2"/>
+      <c r="F22" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="I22" s="15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C23" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="H23" s="15" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C23" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="F23" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="I23" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="F24" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="I24" s="15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D25" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="E24" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="H24" s="15" t="s">
+      <c r="F25" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="I25" s="15" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
         <v>108</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="C28" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
-        <v>110</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C29" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="15"/>
+      <c r="C29" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="E29" s="13"/>
       <c r="F29" s="15"/>
       <c r="G29" s="15"/>
       <c r="H29" s="15"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I29" s="15"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C30" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="D30" s="13"/>
-      <c r="E30" s="15" t="s">
-        <v>118</v>
-      </c>
+      <c r="C30" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="E30" s="13"/>
       <c r="F30" s="15"/>
       <c r="G30" s="15"/>
       <c r="H30" s="15"/>
+      <c r="I30" s="15"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E31" s="13"/>
+      <c r="F31" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+      <c r="I31" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated with Kelli upload & Outbound flow scripts
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23530"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA123CFC-811A-429F-9A78-6D8DE7D896FC}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="7545"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -16,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="183">
   <si>
     <t>1</t>
   </si>
@@ -538,12 +539,39 @@
   </si>
   <si>
     <t>QSC_Scenario000</t>
+  </si>
+  <si>
+    <t>QSC_OBScenario001</t>
+  </si>
+  <si>
+    <t>FG-000100-02</t>
+  </si>
+  <si>
+    <t>FAK</t>
+  </si>
+  <si>
+    <t>NMFCFreightClass</t>
+  </si>
+  <si>
+    <t>WaveAllocationType</t>
+  </si>
+  <si>
+    <t>QSC ALLOCATION TYPE</t>
+  </si>
+  <si>
+    <t>InventoryType</t>
+  </si>
+  <si>
+    <t>Normal(N)</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -597,7 +625,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -668,22 +696,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -709,18 +728,19 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
-    <cellStyle name="Normal 3" xfId="2"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -811,6 +831,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -846,6 +883,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1021,8 +1075,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I31"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" customWidth="1"/>
@@ -1460,24 +1514,24 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="22" t="s">
         <v>171</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="F20" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15" t="s">
+      <c r="F20" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22" t="s">
         <v>138</v>
       </c>
     </row>
@@ -1494,7 +1548,7 @@
       <c r="D21" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="E21" s="2"/>
+      <c r="E21" s="15"/>
       <c r="F21" s="15" t="s">
         <v>118</v>
       </c>
@@ -1517,10 +1571,12 @@
       <c r="D22" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="E22" s="2"/>
+      <c r="E22" s="15"/>
       <c r="F22" s="15" t="s">
         <v>118</v>
       </c>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
       <c r="I22" s="15" t="s">
         <v>136</v>
       </c>
@@ -1538,9 +1594,12 @@
       <c r="D23" s="14" t="s">
         <v>63</v>
       </c>
+      <c r="E23" s="15"/>
       <c r="F23" s="15" t="s">
         <v>118</v>
       </c>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
       <c r="I23" s="15" t="s">
         <v>135</v>
       </c>
@@ -1558,9 +1617,12 @@
       <c r="D24" s="14" t="s">
         <v>64</v>
       </c>
+      <c r="E24" s="15"/>
       <c r="F24" s="15" t="s">
         <v>118</v>
       </c>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
       <c r="I24" s="15" t="s">
         <v>136</v>
       </c>
@@ -1578,71 +1640,203 @@
       <c r="D25" s="14" t="s">
         <v>65</v>
       </c>
+      <c r="E25" s="15"/>
       <c r="F25" s="15" t="s">
         <v>118</v>
       </c>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
       <c r="I25" s="15" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="B29" s="15" t="s">
+    <row r="26" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="B26" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C26" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="D29" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="E29" s="13"/>
+      <c r="D26" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15"/>
+    </row>
+    <row r="27" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="15"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+      <c r="I27" s="15"/>
+    </row>
+    <row r="28" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="I28" s="15"/>
+    </row>
+    <row r="29" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="15"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
       <c r="F29" s="15"/>
       <c r="G29" s="15"/>
       <c r="H29" s="15"/>
       <c r="I29" s="15"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="B30" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="E30" s="13"/>
+    <row r="30" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="15"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
       <c r="F30" s="15"/>
       <c r="G30" s="15"/>
       <c r="H30" s="15"/>
       <c r="I30" s="15"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="B31" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="E31" s="13"/>
-      <c r="F31" s="15" t="s">
-        <v>118</v>
-      </c>
+    <row r="31" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="15"/>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
       <c r="G31" s="15"/>
       <c r="H31" s="15"/>
       <c r="I31" s="15"/>
+    </row>
+    <row r="32" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="15"/>
+      <c r="B32" s="15"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="15"/>
+    </row>
+    <row r="33" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="15"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="15"/>
+    </row>
+    <row r="34" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="15"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+      <c r="I34" s="15"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="15"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="15"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+      <c r="I36" s="15"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="E37" s="13"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="15"/>
+      <c r="I37" s="15"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="E38" s="13"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="15"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E39" s="13"/>
+      <c r="F39" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="G39" s="15"/>
+      <c r="H39" s="15"/>
+      <c r="I39" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1651,8 +1845,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
@@ -1668,31 +1862,34 @@
     <col min="12" max="12" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" s="1" t="s">
         <v>117</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -1707,15 +1904,24 @@
       <c r="L1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="M1" s="19" t="s">
+      <c r="M1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="N1" s="19" t="s">
+      <c r="N1" s="1" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="O1" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="14" t="s">
@@ -1730,11 +1936,13 @@
       <c r="E2" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="F2" s="13"/>
+      <c r="F2" s="13" t="s">
+        <v>182</v>
+      </c>
       <c r="G2" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="15" t="s">
         <v>118</v>
       </c>
       <c r="I2" s="15"/>
@@ -1742,9 +1950,13 @@
       <c r="K2" s="15"/>
       <c r="L2" s="15"/>
       <c r="M2" s="15"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="N2" s="15"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="14" t="s">
@@ -1761,15 +1973,19 @@
       </c>
       <c r="F3" s="13"/>
       <c r="G3" s="15"/>
-      <c r="H3" s="17"/>
+      <c r="H3" s="15"/>
       <c r="I3" s="15"/>
       <c r="J3" s="15"/>
       <c r="K3" s="15"/>
       <c r="L3" s="15"/>
       <c r="M3" s="15"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="15"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
         <v>45</v>
       </c>
       <c r="B4" s="14" t="s">
@@ -1788,7 +2004,7 @@
       <c r="G4" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="H4" s="15" t="s">
         <v>118</v>
       </c>
       <c r="I4" s="15"/>
@@ -1796,9 +2012,13 @@
       <c r="K4" s="15"/>
       <c r="L4" s="15"/>
       <c r="M4" s="15"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
         <v>46</v>
       </c>
       <c r="B5" s="14" t="s">
@@ -1819,7 +2039,7 @@
       <c r="G5" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H5" s="17" t="s">
+      <c r="H5" s="15" t="s">
         <v>118</v>
       </c>
       <c r="I5" s="15"/>
@@ -1827,9 +2047,13 @@
       <c r="K5" s="15"/>
       <c r="L5" s="15"/>
       <c r="M5" s="15"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
         <v>47</v>
       </c>
       <c r="B6" s="14" t="s">
@@ -1848,7 +2072,7 @@
       <c r="G6" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" s="15" t="s">
         <v>118</v>
       </c>
       <c r="I6" s="15"/>
@@ -1856,9 +2080,13 @@
       <c r="K6" s="15"/>
       <c r="L6" s="15"/>
       <c r="M6" s="15"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="18" t="s">
         <v>48</v>
       </c>
       <c r="B7" s="14" t="s">
@@ -1877,7 +2105,7 @@
       <c r="G7" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H7" s="17" t="s">
+      <c r="H7" s="15" t="s">
         <v>118</v>
       </c>
       <c r="I7" s="15"/>
@@ -1885,9 +2113,13 @@
       <c r="K7" s="15"/>
       <c r="L7" s="15"/>
       <c r="M7" s="15"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+      <c r="N7" s="15"/>
+      <c r="O7" s="15"/>
+      <c r="P7" s="15"/>
+      <c r="Q7" s="15"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="18" t="s">
         <v>49</v>
       </c>
       <c r="B8" s="14" t="s">
@@ -1906,7 +2138,7 @@
       <c r="G8" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H8" s="17" t="s">
+      <c r="H8" s="15" t="s">
         <v>118</v>
       </c>
       <c r="I8" s="15" t="s">
@@ -1918,9 +2150,13 @@
       </c>
       <c r="L8" s="15"/>
       <c r="M8" s="15"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+      <c r="N8" s="15"/>
+      <c r="O8" s="15"/>
+      <c r="P8" s="15"/>
+      <c r="Q8" s="15"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
         <v>50</v>
       </c>
       <c r="B9" s="14" t="s">
@@ -1939,7 +2175,7 @@
       <c r="G9" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H9" s="17" t="s">
+      <c r="H9" s="15" t="s">
         <v>118</v>
       </c>
       <c r="I9" s="15" t="s">
@@ -1951,9 +2187,13 @@
       </c>
       <c r="L9" s="15"/>
       <c r="M9" s="15"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+      <c r="N9" s="15"/>
+      <c r="O9" s="15"/>
+      <c r="P9" s="15"/>
+      <c r="Q9" s="15"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
         <v>51</v>
       </c>
       <c r="B10" s="14" t="s">
@@ -1972,7 +2212,7 @@
       <c r="G10" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H10" s="17" t="s">
+      <c r="H10" s="15" t="s">
         <v>118</v>
       </c>
       <c r="I10" s="15" t="s">
@@ -1984,9 +2224,13 @@
       </c>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
+      <c r="N10" s="15"/>
+      <c r="O10" s="15"/>
+      <c r="P10" s="15"/>
+      <c r="Q10" s="15"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
         <v>3</v>
       </c>
       <c r="B11" s="14" t="s">
@@ -2005,7 +2249,7 @@
       <c r="G11" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H11" s="17" t="s">
+      <c r="H11" s="15" t="s">
         <v>118</v>
       </c>
       <c r="I11" s="15"/>
@@ -2013,9 +2257,13 @@
       <c r="K11" s="15"/>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="N11" s="15"/>
+      <c r="O11" s="15"/>
+      <c r="P11" s="15"/>
+      <c r="Q11" s="15"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" s="18" t="s">
         <v>52</v>
       </c>
       <c r="B12" s="14" t="s">
@@ -2034,7 +2282,7 @@
       <c r="G12" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H12" s="17" t="s">
+      <c r="H12" s="15" t="s">
         <v>118</v>
       </c>
       <c r="I12" s="15" t="s">
@@ -2046,9 +2294,13 @@
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
+      <c r="N12" s="15"/>
+      <c r="O12" s="15"/>
+      <c r="P12" s="15"/>
+      <c r="Q12" s="15"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" s="18" t="s">
         <v>53</v>
       </c>
       <c r="B13" s="14" t="s">
@@ -2063,7 +2315,7 @@
       <c r="G13" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H13" s="17"/>
+      <c r="H13" s="15"/>
       <c r="I13" s="15"/>
       <c r="J13" s="15" t="s">
         <v>147</v>
@@ -2071,8 +2323,12 @@
       <c r="K13" s="15"/>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
-    </row>
-    <row r="14" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="N13" s="15"/>
+      <c r="O13" s="15"/>
+      <c r="P13" s="15"/>
+      <c r="Q13" s="15"/>
+    </row>
+    <row r="14" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>54</v>
       </c>
@@ -2092,33 +2348,37 @@
       <c r="G14" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H14" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="I14" s="21" t="s">
+      <c r="H14" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="I14" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="J14" s="21"/>
-      <c r="K14" s="21" t="s">
+      <c r="J14" s="15"/>
+      <c r="K14" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="L14" s="21"/>
+      <c r="L14" s="15"/>
       <c r="M14" s="15"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="18" t="s">
+      <c r="N14" s="15"/>
+      <c r="O14" s="15"/>
+      <c r="P14" s="15"/>
+      <c r="Q14" s="15"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" s="17" t="s">
         <v>55</v>
       </c>
       <c r="B15" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="C15" s="17" t="s">
         <v>90</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="E15" s="22" t="s">
+      <c r="E15" s="17" t="s">
         <v>90</v>
       </c>
       <c r="F15" s="15"/>
@@ -2137,21 +2397,25 @@
       <c r="M15" s="15" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="18" t="s">
+      <c r="N15" s="15"/>
+      <c r="O15" s="15"/>
+      <c r="P15" s="15"/>
+      <c r="Q15" s="15"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" s="17" t="s">
         <v>56</v>
       </c>
       <c r="B16" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="17" t="s">
         <v>90</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="E16" s="22" t="s">
+      <c r="E16" s="17" t="s">
         <v>90</v>
       </c>
       <c r="F16" s="15"/>
@@ -2170,21 +2434,25 @@
       <c r="M16" s="15" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
+      <c r="N16" s="15"/>
+      <c r="O16" s="15"/>
+      <c r="P16" s="15"/>
+      <c r="Q16" s="15"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A17" s="17" t="s">
         <v>57</v>
       </c>
       <c r="B17" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="17" t="s">
         <v>90</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="E17" s="22" t="s">
+      <c r="E17" s="17" t="s">
         <v>90</v>
       </c>
       <c r="F17" s="15"/>
@@ -2203,21 +2471,25 @@
       <c r="M17" s="15" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="18" t="s">
+      <c r="N17" s="15"/>
+      <c r="O17" s="15"/>
+      <c r="P17" s="15"/>
+      <c r="Q17" s="15"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A18" s="17" t="s">
         <v>58</v>
       </c>
       <c r="B18" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="17" t="s">
         <v>90</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="17" t="s">
         <v>90</v>
       </c>
       <c r="F18" s="15"/>
@@ -2236,21 +2508,25 @@
       <c r="M18" s="15" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="18" t="s">
+      <c r="N18" s="15"/>
+      <c r="O18" s="15"/>
+      <c r="P18" s="15"/>
+      <c r="Q18" s="15"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A19" s="17" t="s">
         <v>59</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="17" t="s">
         <v>90</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="E19" s="22" t="s">
+      <c r="E19" s="17" t="s">
         <v>90</v>
       </c>
       <c r="F19" s="15"/>
@@ -2267,21 +2543,25 @@
       <c r="M19" s="15" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="18" t="s">
+      <c r="N19" s="15"/>
+      <c r="O19" s="15"/>
+      <c r="P19" s="15"/>
+      <c r="Q19" s="15"/>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A20" s="17" t="s">
         <v>60</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="17" t="s">
         <v>90</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="E20" s="22" t="s">
+      <c r="E20" s="17" t="s">
         <v>90</v>
       </c>
       <c r="F20" s="15"/>
@@ -2298,9 +2578,13 @@
       <c r="M20" s="15" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="18" t="s">
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
+      <c r="P20" s="15"/>
+      <c r="Q20" s="15"/>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A21" s="17" t="s">
         <v>61</v>
       </c>
       <c r="B21" s="14" t="s">
@@ -2319,15 +2603,23 @@
       <c r="G21" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H21" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="N21" t="s">
+      <c r="H21" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="15"/>
+      <c r="L21" s="15"/>
+      <c r="M21" s="15"/>
+      <c r="N21" s="15" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="18" t="s">
+      <c r="O21" s="15"/>
+      <c r="P21" s="15"/>
+      <c r="Q21" s="15"/>
+    </row>
+    <row r="22" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="17" t="s">
         <v>62</v>
       </c>
       <c r="B22" s="14" t="s">
@@ -2342,7 +2634,7 @@
       <c r="G22" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H22" s="17"/>
+      <c r="H22" s="15"/>
       <c r="I22" s="15"/>
       <c r="J22" s="15" t="s">
         <v>147</v>
@@ -2350,12 +2642,15 @@
       <c r="K22" s="15"/>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
-      <c r="N22" s="2" t="s">
+      <c r="N22" s="15" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="18" t="s">
+      <c r="O22" s="15"/>
+      <c r="P22" s="15"/>
+      <c r="Q22" s="15"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A23" s="17" t="s">
         <v>63</v>
       </c>
       <c r="B23" s="14" t="s">
@@ -2374,19 +2669,25 @@
       <c r="G23" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H23" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="I23" s="23" t="s">
+      <c r="H23" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="I23" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23" t="s">
+      <c r="J23" s="19"/>
+      <c r="K23" s="19" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="18" t="s">
+      <c r="L23" s="15"/>
+      <c r="M23" s="15"/>
+      <c r="N23" s="15"/>
+      <c r="O23" s="15"/>
+      <c r="P23" s="15"/>
+      <c r="Q23" s="15"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A24" s="17" t="s">
         <v>64</v>
       </c>
       <c r="B24" s="14" t="s">
@@ -2405,12 +2706,21 @@
       <c r="G24" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H24" s="17" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="18" t="s">
+      <c r="H24" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="15"/>
+      <c r="M24" s="15"/>
+      <c r="N24" s="15"/>
+      <c r="O24" s="15"/>
+      <c r="P24" s="15"/>
+      <c r="Q24" s="15"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A25" s="17" t="s">
         <v>65</v>
       </c>
       <c r="B25" s="14" t="s">
@@ -2429,16 +2739,150 @@
       <c r="G25" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H25" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="I25" s="23" t="s">
+      <c r="H25" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="I25" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="J25" s="23"/>
-      <c r="K25" s="23" t="s">
+      <c r="J25" s="19"/>
+      <c r="K25" s="19" t="s">
         <v>133</v>
       </c>
+      <c r="L25" s="15"/>
+      <c r="M25" s="15"/>
+      <c r="N25" s="15"/>
+      <c r="O25" s="15"/>
+      <c r="P25" s="15"/>
+      <c r="Q25" s="15"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A26" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="15"/>
+      <c r="L26" s="15"/>
+      <c r="M26" s="15"/>
+      <c r="N26" s="15"/>
+      <c r="O26" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="P26" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q26" s="15" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A27" s="15"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+      <c r="I27" s="15"/>
+      <c r="J27" s="15"/>
+      <c r="K27" s="15"/>
+      <c r="L27" s="15"/>
+      <c r="M27" s="15"/>
+      <c r="N27" s="15"/>
+      <c r="O27" s="15"/>
+      <c r="P27" s="15"/>
+      <c r="Q27" s="15"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="I28" s="15"/>
+      <c r="J28" s="15"/>
+      <c r="K28" s="15"/>
+      <c r="L28" s="15"/>
+      <c r="M28" s="15"/>
+      <c r="N28" s="15"/>
+      <c r="O28" s="15"/>
+      <c r="P28" s="15"/>
+      <c r="Q28" s="15"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A29" s="15"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="15"/>
+      <c r="K29" s="15"/>
+      <c r="L29" s="15"/>
+      <c r="M29" s="15"/>
+      <c r="N29" s="15"/>
+      <c r="O29" s="15"/>
+      <c r="P29" s="15"/>
+      <c r="Q29" s="15"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A30" s="15"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
+      <c r="I30" s="15"/>
+      <c r="J30" s="15"/>
+      <c r="K30" s="15"/>
+      <c r="L30" s="15"/>
+      <c r="M30" s="15"/>
+      <c r="N30" s="15"/>
+      <c r="O30" s="15"/>
+      <c r="P30" s="15"/>
+      <c r="Q30" s="15"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A31" s="15"/>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+      <c r="I31" s="15"/>
+      <c r="J31" s="15"/>
+      <c r="K31" s="15"/>
+      <c r="L31" s="15"/>
+      <c r="M31" s="15"/>
+      <c r="N31" s="15"/>
+      <c r="O31" s="15"/>
+      <c r="P31" s="15"/>
+      <c r="Q31" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2447,7 +2891,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B68"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
Chnaged with copying Reports and screenshots to local drive folder
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23628"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA123CFC-811A-429F-9A78-6D8DE7D896FC}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BDB0D68-C7BC-428D-8826-634CBBA4F752}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="186">
   <si>
     <t>1</t>
   </si>
@@ -566,6 +566,15 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>QSC_OBScenario002</t>
+  </si>
+  <si>
+    <t>FG-000412-00</t>
+  </si>
+  <si>
+    <t>26|27</t>
   </si>
 </sst>
 </file>
@@ -1670,10 +1679,18 @@
       <c r="I26" s="15"/>
     </row>
     <row r="27" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
+      <c r="A27" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D27" s="24" t="s">
+        <v>185</v>
+      </c>
       <c r="E27" s="15"/>
       <c r="F27" s="15"/>
       <c r="G27" s="15"/>
@@ -2789,11 +2806,19 @@
         <v>181</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
+    <row r="27" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>116</v>
+      </c>
       <c r="E27" s="15"/>
       <c r="F27" s="15"/>
       <c r="G27" s="15"/>
@@ -2804,15 +2829,29 @@
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
       <c r="N27" s="15"/>
-      <c r="O27" s="15"/>
-      <c r="P27" s="15"/>
-      <c r="Q27" s="15"/>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
+      <c r="O27" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="P27" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q27" s="15" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" s="20" t="s">
+        <v>184</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>116</v>
+      </c>
       <c r="E28" s="15"/>
       <c r="F28" s="15"/>
       <c r="G28" s="15"/>
@@ -2823,9 +2862,15 @@
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
       <c r="N28" s="15"/>
-      <c r="O28" s="15"/>
-      <c r="P28" s="15"/>
-      <c r="Q28" s="15"/>
+      <c r="O28" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="P28" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q28" s="15" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="15"/>

</xml_diff>

<commit_message>
Added few shipping scenarios for QSC
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23628"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BDB0D68-C7BC-428D-8826-634CBBA4F752}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686F5CBE-1D31-4984-9A23-FA076DF2886D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="189">
   <si>
     <t>1</t>
   </si>
@@ -575,6 +575,15 @@
   </si>
   <si>
     <t>26|27</t>
+  </si>
+  <si>
+    <t>FG-000413-01</t>
+  </si>
+  <si>
+    <t>QSC_OBScenario003</t>
+  </si>
+  <si>
+    <t>100</t>
   </si>
 </sst>
 </file>
@@ -1698,10 +1707,18 @@
       <c r="I27" s="15"/>
     </row>
     <row r="28" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
+      <c r="A28" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D28" s="24" t="s">
+        <v>69</v>
+      </c>
       <c r="E28" s="15"/>
       <c r="F28" s="15"/>
       <c r="G28" s="15"/>
@@ -2781,7 +2798,7 @@
         <v>175</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D26" s="17" t="s">
         <v>116</v>
@@ -2872,11 +2889,19 @@
         <v>181</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A29" s="15"/>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
+    <row r="29" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>116</v>
+      </c>
       <c r="E29" s="15"/>
       <c r="F29" s="15"/>
       <c r="G29" s="15"/>
@@ -2887,9 +2912,15 @@
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
       <c r="N29" s="15"/>
-      <c r="O29" s="15"/>
-      <c r="P29" s="15"/>
-      <c r="Q29" s="15"/>
+      <c r="O29" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="P29" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q29" s="15" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" s="15"/>

</xml_diff>

<commit_message>
udated with cancel olpn
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23901"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0841039C-3E3F-4F82-ADBE-ABBB049E283D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48914D2D-02D9-430C-95E5-407A7FE8787E}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="280">
   <si>
     <t>1</t>
   </si>
@@ -379,9 +379,6 @@
     <t>ItemReference</t>
   </si>
   <si>
-    <t>76</t>
-  </si>
-  <si>
     <t>ST-G0-01-1-R</t>
   </si>
   <si>
@@ -406,9 +403,6 @@
     <t>ASNId</t>
   </si>
   <si>
-    <t>80</t>
-  </si>
-  <si>
     <t>Scenario9</t>
   </si>
   <si>
@@ -610,30 +604,9 @@
     <t>QSC_OBScenario007</t>
   </si>
   <si>
-    <t>NVI_Scenario001</t>
-  </si>
-  <si>
     <t>NVI</t>
   </si>
   <si>
-    <t>NVI_Scenario002</t>
-  </si>
-  <si>
-    <t>NVI_Scenario003</t>
-  </si>
-  <si>
-    <t>NVI_Scenario004</t>
-  </si>
-  <si>
-    <t>NVI_Scenario005</t>
-  </si>
-  <si>
-    <t>NVI_Scenario006</t>
-  </si>
-  <si>
-    <t>NVI_Scenario007</t>
-  </si>
-  <si>
     <t>PltQty</t>
   </si>
   <si>
@@ -823,21 +796,6 @@
     <t>808</t>
   </si>
   <si>
-    <t>NVI_Scenario008</t>
-  </si>
-  <si>
-    <t>NVI_Scenario009</t>
-  </si>
-  <si>
-    <t>NVI_Scenario010</t>
-  </si>
-  <si>
-    <t>NVI_Scenario011</t>
-  </si>
-  <si>
-    <t>NVI_Scenario012</t>
-  </si>
-  <si>
     <t>809</t>
   </si>
   <si>
@@ -854,6 +812,51 @@
   </si>
   <si>
     <t>813</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario001</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario002</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario003</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario004</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario005</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario006</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario007</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario008</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario009</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario010</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario011</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario012</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario013</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario014</t>
+  </si>
+  <si>
+    <t>814</t>
   </si>
 </sst>
 </file>
@@ -996,7 +999,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1031,6 +1034,8 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1371,7 +1376,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P72"/>
+  <dimension ref="A1:P74"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.88671875" customWidth="1"/>
@@ -1396,7 +1401,7 @@
         <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>119</v>
@@ -1408,45 +1413,45 @@
         <v>116</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J1" s="24" t="s">
+        <v>164</v>
+      </c>
+      <c r="K1" s="24" t="s">
+        <v>165</v>
+      </c>
+      <c r="L1" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="K1" s="24" t="s">
+      <c r="M1" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="L1" s="24" t="s">
+      <c r="N1" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="M1" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="N1" s="24" t="s">
-        <v>170</v>
-      </c>
       <c r="O1" s="24" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="P1" s="24" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>0</v>
@@ -1468,13 +1473,13 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>0</v>
@@ -1496,13 +1501,13 @@
     </row>
     <row r="4" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>0</v>
@@ -1514,7 +1519,7 @@
       <c r="G4" s="15"/>
       <c r="H4" s="15"/>
       <c r="I4" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J4" s="15"/>
       <c r="K4" s="15"/>
@@ -1526,13 +1531,13 @@
     </row>
     <row r="5" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>0</v>
@@ -1554,13 +1559,13 @@
     </row>
     <row r="6" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>45</v>
@@ -1582,20 +1587,20 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>46</v>
       </c>
       <c r="E7" s="13"/>
       <c r="F7" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G7" s="13" t="s">
         <v>3</v>
@@ -1612,16 +1617,16 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E8" s="13"/>
       <c r="F8" s="15" t="s">
@@ -1630,7 +1635,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="15"/>
       <c r="I8" s="15" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="J8" s="15"/>
       <c r="K8" s="15"/>
@@ -1642,13 +1647,13 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>49</v>
@@ -1660,7 +1665,7 @@
       <c r="G9" s="13"/>
       <c r="H9" s="15"/>
       <c r="I9" s="15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="J9" s="15"/>
       <c r="K9" s="15"/>
@@ -1672,13 +1677,13 @@
     </row>
     <row r="10" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>51</v>
@@ -1700,13 +1705,13 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>3</v>
@@ -1718,7 +1723,7 @@
       <c r="G11" s="15"/>
       <c r="H11" s="15"/>
       <c r="I11" s="15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J11" s="15"/>
       <c r="K11" s="15"/>
@@ -1730,13 +1735,13 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>52</v>
@@ -1748,7 +1753,7 @@
       <c r="G12" s="15"/>
       <c r="H12" s="15"/>
       <c r="I12" s="15" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J12" s="15"/>
       <c r="K12" s="15"/>
@@ -1760,13 +1765,13 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D13" s="14" t="s">
         <v>53</v>
@@ -1776,7 +1781,7 @@
       <c r="G13" s="15"/>
       <c r="H13" s="15"/>
       <c r="I13" s="15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J13" s="15"/>
       <c r="K13" s="15"/>
@@ -1788,13 +1793,13 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>54</v>
@@ -1804,7 +1809,7 @@
       <c r="G14" s="15"/>
       <c r="H14" s="15"/>
       <c r="I14" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J14" s="15"/>
       <c r="K14" s="15"/>
@@ -1816,13 +1821,13 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>55</v>
@@ -1834,7 +1839,7 @@
       <c r="G15" s="15"/>
       <c r="H15" s="15"/>
       <c r="I15" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J15" s="15"/>
       <c r="K15" s="15"/>
@@ -1846,13 +1851,13 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D16" s="14" t="s">
         <v>56</v>
@@ -1864,7 +1869,7 @@
       <c r="G16" s="15"/>
       <c r="H16" s="15"/>
       <c r="I16" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J16" s="15"/>
       <c r="K16" s="15"/>
@@ -1876,13 +1881,13 @@
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="13" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D17" s="14" t="s">
         <v>57</v>
@@ -1894,7 +1899,7 @@
       <c r="G17" s="15"/>
       <c r="H17" s="15"/>
       <c r="I17" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J17" s="15"/>
       <c r="K17" s="15"/>
@@ -1906,13 +1911,13 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D18" s="14" t="s">
         <v>58</v>
@@ -1924,7 +1929,7 @@
       <c r="G18" s="15"/>
       <c r="H18" s="15"/>
       <c r="I18" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J18" s="15"/>
       <c r="K18" s="15"/>
@@ -1936,13 +1941,13 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="13" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>59</v>
@@ -1953,7 +1958,7 @@
       <c r="G19" s="15"/>
       <c r="H19" s="15"/>
       <c r="I19" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J19" s="15"/>
       <c r="K19" s="15"/>
@@ -1965,13 +1970,13 @@
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="13" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="B20" s="21" t="s">
         <v>110</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D20" s="22" t="s">
         <v>60</v>
@@ -1982,7 +1987,7 @@
       <c r="G20" s="21"/>
       <c r="H20" s="21"/>
       <c r="I20" s="21" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J20" s="15"/>
       <c r="K20" s="15"/>
@@ -1994,13 +1999,13 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="13" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>61</v>
@@ -2012,7 +2017,7 @@
       <c r="G21" s="15"/>
       <c r="H21" s="15"/>
       <c r="I21" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J21" s="15"/>
       <c r="K21" s="15"/>
@@ -2024,13 +2029,13 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="13" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D22" s="14" t="s">
         <v>62</v>
@@ -2042,7 +2047,7 @@
       <c r="G22" s="15"/>
       <c r="H22" s="15"/>
       <c r="I22" s="15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J22" s="15"/>
       <c r="K22" s="15"/>
@@ -2054,13 +2059,13 @@
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="13" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>63</v>
@@ -2072,7 +2077,7 @@
       <c r="G23" s="15"/>
       <c r="H23" s="15"/>
       <c r="I23" s="15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="J23" s="15"/>
       <c r="K23" s="15"/>
@@ -2084,13 +2089,13 @@
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="13" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D24" s="14" t="s">
         <v>64</v>
@@ -2102,7 +2107,7 @@
       <c r="G24" s="15"/>
       <c r="H24" s="15"/>
       <c r="I24" s="15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J24" s="15"/>
       <c r="K24" s="15"/>
@@ -2114,13 +2119,13 @@
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" s="13" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D25" s="14" t="s">
         <v>65</v>
@@ -2132,7 +2137,7 @@
       <c r="G25" s="15"/>
       <c r="H25" s="15"/>
       <c r="I25" s="15" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J25" s="15"/>
       <c r="K25" s="15"/>
@@ -2144,13 +2149,13 @@
     </row>
     <row r="26" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="13" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>66</v>
@@ -2172,16 +2177,16 @@
     </row>
     <row r="27" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E27" s="15"/>
       <c r="F27" s="15" t="s">
@@ -2200,16 +2205,16 @@
     </row>
     <row r="28" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="13" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E28" s="15"/>
       <c r="F28" s="15" t="s">
@@ -2228,13 +2233,13 @@
     </row>
     <row r="29" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="13" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>70</v>
@@ -2256,13 +2261,13 @@
     </row>
     <row r="30" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="13" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D30" s="14" t="s">
         <v>71</v>
@@ -2284,13 +2289,13 @@
     </row>
     <row r="31" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="13" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>72</v>
@@ -2312,16 +2317,16 @@
     </row>
     <row r="32" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="13" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E32" s="15"/>
       <c r="F32" s="15" t="s">
@@ -2340,16 +2345,16 @@
     </row>
     <row r="33" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="13" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="B33" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E33" s="15"/>
       <c r="F33" s="15" t="s">
@@ -2368,16 +2373,16 @@
     </row>
     <row r="34" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="15" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="E34" s="15"/>
       <c r="F34" s="15"/>
@@ -2412,16 +2417,16 @@
     </row>
     <row r="36" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="15" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E36" s="15"/>
       <c r="F36" s="15"/>
@@ -2438,16 +2443,16 @@
     </row>
     <row r="37" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="15" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B37" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E37" s="15"/>
       <c r="F37" s="15"/>
@@ -2464,16 +2469,16 @@
     </row>
     <row r="38" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="15" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E38" s="15"/>
       <c r="F38" s="15"/>
@@ -2490,16 +2495,16 @@
     </row>
     <row r="39" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="15" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B39" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E39" s="15"/>
       <c r="F39" s="15"/>
@@ -2512,22 +2517,22 @@
       <c r="M39" s="15"/>
       <c r="N39" s="15"/>
       <c r="O39" s="15" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="P39" s="15"/>
     </row>
     <row r="40" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="15" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E40" s="15"/>
       <c r="F40" s="15"/>
@@ -2540,22 +2545,22 @@
       <c r="M40" s="15"/>
       <c r="N40" s="15"/>
       <c r="O40" s="15" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="P40" s="15"/>
     </row>
     <row r="41" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="15" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B41" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E41" s="15"/>
       <c r="F41" s="15"/>
@@ -2568,22 +2573,22 @@
       <c r="M41" s="15"/>
       <c r="N41" s="15"/>
       <c r="O41" s="15" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="P41" s="15"/>
     </row>
     <row r="42" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="15" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E42" s="15"/>
       <c r="F42" s="15"/>
@@ -2596,22 +2601,22 @@
       <c r="M42" s="15"/>
       <c r="N42" s="15"/>
       <c r="O42" s="15" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="P42" s="15"/>
     </row>
     <row r="43" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="15" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="B43" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C43" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E43" s="15"/>
       <c r="F43" s="15"/>
@@ -2624,22 +2629,22 @@
       <c r="M43" s="15"/>
       <c r="N43" s="15"/>
       <c r="O43" s="15" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="P43" s="15"/>
     </row>
     <row r="44" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="15" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="B44" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="E44" s="15"/>
       <c r="F44" s="15"/>
@@ -2656,16 +2661,16 @@
     </row>
     <row r="45" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="15" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="B45" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C45" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="E45" s="15"/>
       <c r="F45" s="15"/>
@@ -2682,16 +2687,16 @@
     </row>
     <row r="46" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="15" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="B46" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C46" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="E46" s="15"/>
       <c r="F46" s="15"/>
@@ -2708,16 +2713,16 @@
     </row>
     <row r="47" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="15" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="B47" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="E47" s="15"/>
       <c r="F47" s="15"/>
@@ -2770,13 +2775,13 @@
     </row>
     <row r="50" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="15" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B50" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D50" s="15"/>
       <c r="E50" s="15"/>
@@ -2785,7 +2790,7 @@
       <c r="H50" s="15"/>
       <c r="I50" s="15"/>
       <c r="J50" s="13" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="K50" s="15"/>
       <c r="L50" s="15"/>
@@ -2796,13 +2801,13 @@
     </row>
     <row r="51" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="15" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B51" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D51" s="15"/>
       <c r="E51" s="15"/>
@@ -2812,7 +2817,7 @@
       <c r="I51" s="15"/>
       <c r="J51" s="15"/>
       <c r="K51" s="15" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="L51" s="15"/>
       <c r="M51" s="15"/>
@@ -2822,13 +2827,13 @@
     </row>
     <row r="52" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="15" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B52" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D52" s="15"/>
       <c r="E52" s="15"/>
@@ -2839,7 +2844,7 @@
       <c r="J52" s="15"/>
       <c r="K52" s="15"/>
       <c r="L52" s="15" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="M52" s="15"/>
       <c r="N52" s="15"/>
@@ -2848,13 +2853,13 @@
     </row>
     <row r="53" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A53" s="15" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B53" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C53" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D53" s="15"/>
       <c r="E53" s="15"/>
@@ -2866,7 +2871,7 @@
       <c r="K53" s="15"/>
       <c r="L53" s="15"/>
       <c r="M53" s="15" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="N53" s="15"/>
       <c r="O53" s="15"/>
@@ -2874,13 +2879,13 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" s="15" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B54" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C54" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D54" s="15"/>
       <c r="E54" s="15"/>
@@ -2893,7 +2898,7 @@
       <c r="L54" s="15"/>
       <c r="M54" s="15"/>
       <c r="N54" s="13" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="O54" s="15"/>
       <c r="P54" s="15"/>
@@ -2942,7 +2947,7 @@
         <v>110</v>
       </c>
       <c r="C57" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D57" s="14" t="s">
         <v>0</v>
@@ -2968,7 +2973,7 @@
         <v>110</v>
       </c>
       <c r="C58" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D58" s="14" t="s">
         <v>45</v>
@@ -2988,13 +2993,13 @@
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" s="13" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B59" s="15" t="s">
         <v>110</v>
       </c>
       <c r="C59" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D59" s="14" t="s">
         <v>50</v>
@@ -3034,16 +3039,16 @@
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A61" s="15" t="s">
-        <v>197</v>
+        <v>265</v>
       </c>
       <c r="B61" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C61" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D61" s="13" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="E61" s="15"/>
       <c r="F61" s="15" t="s">
@@ -3064,16 +3069,16 @@
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A62" s="15" t="s">
-        <v>199</v>
+        <v>266</v>
       </c>
       <c r="B62" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D62" s="13" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="E62" s="15"/>
       <c r="F62" s="15" t="s">
@@ -3094,16 +3099,16 @@
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A63" s="15" t="s">
-        <v>200</v>
+        <v>267</v>
       </c>
       <c r="B63" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C63" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D63" s="13" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="E63" s="15"/>
       <c r="F63" s="15" t="s">
@@ -3124,16 +3129,16 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A64" s="15" t="s">
-        <v>201</v>
+        <v>268</v>
       </c>
       <c r="B64" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C64" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D64" s="13" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="E64" s="15"/>
       <c r="F64" s="15" t="s">
@@ -3154,16 +3159,16 @@
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A65" s="15" t="s">
-        <v>202</v>
+        <v>269</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C65" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D65" s="13" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="E65" s="15"/>
       <c r="F65" s="15" t="s">
@@ -3184,16 +3189,16 @@
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A66" s="15" t="s">
-        <v>203</v>
+        <v>270</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C66" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D66" s="13" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="E66" s="15"/>
       <c r="F66" s="15" t="s">
@@ -3214,16 +3219,16 @@
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A67" s="15" t="s">
-        <v>204</v>
+        <v>271</v>
       </c>
       <c r="B67" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C67" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D67" s="13" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="E67" s="15"/>
       <c r="F67" s="15" t="s">
@@ -3244,16 +3249,16 @@
     </row>
     <row r="68" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="15" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B68" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C68" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D68" s="13" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="E68" s="15"/>
       <c r="F68" s="15" t="s">
@@ -3272,16 +3277,16 @@
     </row>
     <row r="69" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A69" s="15" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B69" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C69" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D69" s="13" t="s">
-        <v>273</v>
+        <v>259</v>
       </c>
       <c r="E69" s="15"/>
       <c r="F69" s="15" t="s">
@@ -3300,16 +3305,16 @@
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A70" s="15" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C70" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>274</v>
+        <v>260</v>
       </c>
       <c r="E70" s="15"/>
       <c r="F70" s="15" t="s">
@@ -3328,16 +3333,16 @@
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A71" s="15" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B71" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C71" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D71" s="13" t="s">
-        <v>275</v>
+        <v>261</v>
       </c>
       <c r="E71" s="15"/>
       <c r="F71" s="15" t="s">
@@ -3356,16 +3361,16 @@
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A72" s="15" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B72" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C72" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>276</v>
+        <v>262</v>
       </c>
       <c r="E72" s="15"/>
       <c r="F72" s="15" t="s">
@@ -3381,6 +3386,31 @@
       <c r="N72" s="15"/>
       <c r="O72" s="15"/>
       <c r="P72" s="13"/>
+    </row>
+    <row r="73" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A73" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="B73" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="C73" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="D73" s="27" t="s">
+        <v>279</v>
+      </c>
+      <c r="F73" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="P73" s="26" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A74" s="15" t="s">
+        <v>278</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -3431,7 +3461,7 @@
         <v>113</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>114</v>
@@ -3440,37 +3470,37 @@
         <v>116</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>126</v>
-      </c>
       <c r="L1" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="O1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="P1" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="R1" s="1" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
@@ -3478,7 +3508,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C2" s="13" t="s">
         <v>61</v>
@@ -3491,7 +3521,7 @@
       </c>
       <c r="F2" s="13"/>
       <c r="G2" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H2" s="15" t="s">
         <v>117</v>
@@ -3544,20 +3574,20 @@
         <v>45</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>90</v>
+        <v>3</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>120</v>
+        <v>57</v>
       </c>
       <c r="F4" s="13"/>
       <c r="G4" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H4" s="15" t="s">
         <v>117</v>
@@ -3579,7 +3609,7 @@
         <v>46</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>80</v>
@@ -3594,7 +3624,7 @@
         <v>62</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>117</v>
@@ -3616,20 +3646,20 @@
         <v>47</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>80</v>
+        <v>3</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>80</v>
+        <v>3</v>
       </c>
       <c r="F6" s="13"/>
       <c r="G6" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H6" s="15" t="s">
         <v>117</v>
@@ -3651,7 +3681,7 @@
         <v>48</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>61</v>
@@ -3664,7 +3694,7 @@
       </c>
       <c r="F7" s="13"/>
       <c r="G7" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H7" s="15" t="s">
         <v>117</v>
@@ -3686,7 +3716,7 @@
         <v>49</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>3</v>
@@ -3699,17 +3729,17 @@
       </c>
       <c r="F8" s="13"/>
       <c r="G8" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H8" s="15" t="s">
         <v>117</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J8" s="15"/>
       <c r="K8" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="L8" s="15"/>
       <c r="M8" s="15"/>
@@ -3725,30 +3755,30 @@
         <v>50</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>90</v>
+        <v>3</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>129</v>
+        <v>57</v>
       </c>
       <c r="F9" s="13"/>
       <c r="G9" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H9" s="15" t="s">
         <v>117</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J9" s="15"/>
       <c r="K9" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="L9" s="15"/>
       <c r="M9" s="15"/>
@@ -3764,7 +3794,7 @@
         <v>51</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>3</v>
@@ -3777,17 +3807,17 @@
       </c>
       <c r="F10" s="13"/>
       <c r="G10" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H10" s="15" t="s">
         <v>117</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J10" s="15"/>
       <c r="K10" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
@@ -3803,7 +3833,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>3</v>
@@ -3816,7 +3846,7 @@
       </c>
       <c r="F11" s="13"/>
       <c r="G11" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H11" s="15" t="s">
         <v>117</v>
@@ -3838,7 +3868,7 @@
         <v>52</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>3</v>
@@ -3851,17 +3881,17 @@
       </c>
       <c r="F12" s="13"/>
       <c r="G12" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H12" s="15" t="s">
         <v>117</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J12" s="15"/>
       <c r="K12" s="15" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
@@ -3877,7 +3907,7 @@
         <v>53</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="15"/>
@@ -3886,12 +3916,12 @@
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H13" s="15"/>
       <c r="I13" s="15"/>
       <c r="J13" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K13" s="15"/>
       <c r="L13" s="15"/>
@@ -3908,7 +3938,7 @@
         <v>54</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C14" s="13" t="s">
         <v>3</v>
@@ -3921,17 +3951,17 @@
       </c>
       <c r="F14" s="13"/>
       <c r="G14" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>117</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J14" s="15"/>
       <c r="K14" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
@@ -3947,20 +3977,20 @@
         <v>55</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F15" s="15"/>
       <c r="G15" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H15" s="15" t="s">
         <v>117</v>
@@ -3969,10 +3999,10 @@
       <c r="J15" s="15"/>
       <c r="K15" s="15"/>
       <c r="L15" s="13" t="s">
-        <v>100</v>
+        <v>66</v>
       </c>
       <c r="M15" s="15" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="N15" s="15"/>
       <c r="O15" s="15"/>
@@ -3986,20 +4016,20 @@
         <v>56</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F16" s="15"/>
       <c r="G16" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>117</v>
@@ -4008,10 +4038,10 @@
       <c r="J16" s="15"/>
       <c r="K16" s="15"/>
       <c r="L16" s="13" t="s">
-        <v>80</v>
+        <v>56</v>
       </c>
       <c r="M16" s="15" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="N16" s="15"/>
       <c r="O16" s="15"/>
@@ -4025,20 +4055,20 @@
         <v>57</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="F17" s="15"/>
       <c r="G17" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>117</v>
@@ -4047,10 +4077,10 @@
       <c r="J17" s="15"/>
       <c r="K17" s="15"/>
       <c r="L17" s="13" t="s">
-        <v>100</v>
+        <v>66</v>
       </c>
       <c r="M17" s="15" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="N17" s="15"/>
       <c r="O17" s="15"/>
@@ -4064,20 +4094,20 @@
         <v>58</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>117</v>
@@ -4086,10 +4116,10 @@
       <c r="J18" s="15"/>
       <c r="K18" s="15"/>
       <c r="L18" s="13" t="s">
-        <v>80</v>
+        <v>56</v>
       </c>
       <c r="M18" s="15" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="N18" s="15"/>
       <c r="O18" s="15"/>
@@ -4103,20 +4133,20 @@
         <v>59</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F19" s="15"/>
       <c r="G19" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>117</v>
@@ -4126,7 +4156,7 @@
       <c r="K19" s="15"/>
       <c r="L19" s="15"/>
       <c r="M19" s="15" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="N19" s="15"/>
       <c r="O19" s="15"/>
@@ -4140,20 +4170,20 @@
         <v>60</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="F20" s="15"/>
       <c r="G20" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>117</v>
@@ -4163,7 +4193,7 @@
       <c r="K20" s="15"/>
       <c r="L20" s="15"/>
       <c r="M20" s="15" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="N20" s="15"/>
       <c r="O20" s="15"/>
@@ -4177,7 +4207,7 @@
         <v>61</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C21" s="13" t="s">
         <v>61</v>
@@ -4190,7 +4220,7 @@
       </c>
       <c r="F21" s="13"/>
       <c r="G21" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>117</v>
@@ -4201,7 +4231,7 @@
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
       <c r="N21" s="15" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O21" s="15"/>
       <c r="P21" s="15"/>
@@ -4214,7 +4244,7 @@
         <v>62</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="15"/>
@@ -4226,13 +4256,13 @@
       <c r="H22" s="15"/>
       <c r="I22" s="15"/>
       <c r="J22" s="13" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K22" s="15"/>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
       <c r="N22" s="15" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="O22" s="15"/>
       <c r="P22" s="15"/>
@@ -4245,7 +4275,7 @@
         <v>63</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>3</v>
@@ -4258,17 +4288,17 @@
       </c>
       <c r="F23" s="13"/>
       <c r="G23" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H23" s="15" t="s">
         <v>117</v>
       </c>
       <c r="I23" s="19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J23" s="19"/>
       <c r="K23" s="19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
@@ -4284,7 +4314,7 @@
         <v>64</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>3</v>
@@ -4297,7 +4327,7 @@
       </c>
       <c r="F24" s="13"/>
       <c r="G24" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H24" s="15" t="s">
         <v>117</v>
@@ -4319,7 +4349,7 @@
         <v>65</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>3</v>
@@ -4332,17 +4362,17 @@
       </c>
       <c r="F25" s="13"/>
       <c r="G25" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H25" s="15" t="s">
         <v>117</v>
       </c>
       <c r="I25" s="19" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J25" s="19"/>
       <c r="K25" s="19" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
@@ -4358,7 +4388,7 @@
         <v>66</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C26" s="13" t="s">
         <v>3</v>
@@ -4391,7 +4421,7 @@
         <v>67</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>3</v>
@@ -4424,7 +4454,7 @@
         <v>68</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>3</v>
@@ -4457,7 +4487,7 @@
         <v>69</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>3</v>
@@ -4490,7 +4520,7 @@
         <v>36</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>47</v>
@@ -4523,7 +4553,7 @@
         <v>70</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C31" s="13" t="s">
         <v>3</v>
@@ -4556,7 +4586,7 @@
         <v>71</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>3</v>
@@ -4589,7 +4619,7 @@
         <v>72</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C33" s="13" t="s">
         <v>3</v>
@@ -4622,7 +4652,7 @@
         <v>73</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>3</v>
@@ -4655,7 +4685,7 @@
         <v>74</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C35" s="13" t="s">
         <v>3</v>
@@ -4688,7 +4718,7 @@
         <v>75</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C36" s="13" t="s">
         <v>3</v>
@@ -4721,7 +4751,7 @@
         <v>76</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C37" s="13" t="s">
         <v>3</v>
@@ -4751,10 +4781,10 @@
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A38" s="17" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C38" s="17" t="s">
         <v>2</v>
@@ -4768,30 +4798,30 @@
       <c r="H38" s="15"/>
       <c r="I38" s="15"/>
       <c r="J38" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K38" s="15"/>
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
       <c r="N38" s="15"/>
       <c r="O38" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P38" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q38" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R38" s="15"/>
       <c r="S38" s="15"/>
     </row>
     <row r="39" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="17" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C39" s="17" t="s">
         <v>0</v>
@@ -4805,30 +4835,30 @@
       <c r="H39" s="15"/>
       <c r="I39" s="15"/>
       <c r="J39" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K39" s="15"/>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
       <c r="N39" s="15"/>
       <c r="O39" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P39" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q39" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R39" s="15"/>
       <c r="S39" s="15"/>
     </row>
     <row r="40" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="17" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C40" s="17" t="s">
         <v>0</v>
@@ -4842,33 +4872,33 @@
       <c r="H40" s="15"/>
       <c r="I40" s="15"/>
       <c r="J40" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K40" s="15"/>
       <c r="L40" s="15"/>
       <c r="M40" s="15"/>
       <c r="N40" s="15"/>
       <c r="O40" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P40" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q40" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R40" s="15"/>
       <c r="S40" s="15"/>
     </row>
     <row r="41" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B41" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="C41" s="17" t="s">
         <v>158</v>
-      </c>
-      <c r="C41" s="17" t="s">
-        <v>160</v>
       </c>
       <c r="D41" s="17" t="s">
         <v>115</v>
@@ -4879,30 +4909,30 @@
       <c r="H41" s="15"/>
       <c r="I41" s="15"/>
       <c r="J41" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K41" s="15"/>
       <c r="L41" s="15"/>
       <c r="M41" s="15"/>
       <c r="N41" s="15"/>
       <c r="O41" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P41" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q41" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R41" s="15"/>
       <c r="S41" s="15"/>
     </row>
     <row r="42" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="17" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C42" s="17" t="s">
         <v>2</v>
@@ -4916,30 +4946,30 @@
       <c r="H42" s="15"/>
       <c r="I42" s="15"/>
       <c r="J42" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K42" s="15"/>
       <c r="L42" s="15"/>
       <c r="M42" s="15"/>
       <c r="N42" s="15"/>
       <c r="O42" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P42" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q42" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R42" s="15"/>
       <c r="S42" s="15"/>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A43" s="17" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C43" s="17" t="s">
         <v>2</v>
@@ -4953,30 +4983,30 @@
       <c r="H43" s="15"/>
       <c r="I43" s="15"/>
       <c r="J43" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K43" s="15"/>
       <c r="L43" s="15"/>
       <c r="M43" s="15"/>
       <c r="N43" s="15"/>
       <c r="O43" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P43" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q43" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R43" s="15"/>
       <c r="S43" s="15"/>
     </row>
     <row r="44" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="17" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C44" s="17" t="s">
         <v>2</v>
@@ -4990,30 +5020,30 @@
       <c r="H44" s="15"/>
       <c r="I44" s="15"/>
       <c r="J44" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K44" s="15"/>
       <c r="L44" s="15"/>
       <c r="M44" s="15"/>
       <c r="N44" s="15"/>
       <c r="O44" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P44" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q44" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R44" s="15"/>
       <c r="S44" s="15"/>
     </row>
     <row r="45" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="17" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C45" s="17" t="s">
         <v>2</v>
@@ -5027,30 +5057,30 @@
       <c r="H45" s="15"/>
       <c r="I45" s="15"/>
       <c r="J45" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K45" s="15"/>
       <c r="L45" s="15"/>
       <c r="M45" s="15"/>
       <c r="N45" s="15"/>
       <c r="O45" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P45" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q45" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R45" s="15"/>
       <c r="S45" s="15"/>
     </row>
     <row r="46" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="17" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C46" s="17" t="s">
         <v>3</v>
@@ -5064,20 +5094,20 @@
       <c r="H46" s="15"/>
       <c r="I46" s="15"/>
       <c r="J46" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K46" s="15"/>
       <c r="L46" s="15"/>
       <c r="M46" s="15"/>
       <c r="N46" s="15"/>
       <c r="O46" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P46" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q46" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R46" s="13" t="s">
         <v>47</v>
@@ -5086,10 +5116,10 @@
     </row>
     <row r="47" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="17" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C47" s="17" t="s">
         <v>3</v>
@@ -5103,20 +5133,20 @@
       <c r="H47" s="15"/>
       <c r="I47" s="15"/>
       <c r="J47" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K47" s="15"/>
       <c r="L47" s="15"/>
       <c r="M47" s="15"/>
       <c r="N47" s="15"/>
       <c r="O47" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P47" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q47" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R47" s="13" t="s">
         <v>47</v>
@@ -5125,10 +5155,10 @@
     </row>
     <row r="48" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="17" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C48" s="17" t="s">
         <v>3</v>
@@ -5142,20 +5172,20 @@
       <c r="H48" s="15"/>
       <c r="I48" s="15"/>
       <c r="J48" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K48" s="15"/>
       <c r="L48" s="15"/>
       <c r="M48" s="15"/>
       <c r="N48" s="15"/>
       <c r="O48" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P48" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q48" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R48" s="15"/>
       <c r="S48" s="13" t="s">
@@ -5164,10 +5194,10 @@
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A49" s="17" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C49" s="13" t="s">
         <v>47</v>
@@ -5181,30 +5211,30 @@
       <c r="H49" s="15"/>
       <c r="I49" s="15"/>
       <c r="J49" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K49" s="15"/>
       <c r="L49" s="15"/>
       <c r="M49" s="15"/>
       <c r="N49" s="15"/>
       <c r="O49" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P49" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q49" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R49" s="15"/>
       <c r="S49" s="15"/>
     </row>
     <row r="50" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="17" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C50" s="13" t="s">
         <v>47</v>
@@ -5218,20 +5248,20 @@
       <c r="H50" s="15"/>
       <c r="I50" s="15"/>
       <c r="J50" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K50" s="15"/>
       <c r="L50" s="15"/>
       <c r="M50" s="15"/>
       <c r="N50" s="15"/>
       <c r="O50" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P50" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q50" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R50" s="15"/>
       <c r="S50" s="13" t="s">
@@ -5240,10 +5270,10 @@
     </row>
     <row r="51" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="17" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C51" s="13" t="s">
         <v>3</v>
@@ -5257,30 +5287,30 @@
       <c r="H51" s="15"/>
       <c r="I51" s="15"/>
       <c r="J51" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K51" s="15"/>
       <c r="L51" s="15"/>
       <c r="M51" s="15"/>
       <c r="N51" s="15"/>
       <c r="O51" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P51" s="15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="Q51" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R51" s="15"/>
       <c r="S51" s="15"/>
     </row>
     <row r="52" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="17" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C52" s="13" t="s">
         <v>0</v>
@@ -5327,10 +5357,10 @@
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A54" s="13" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C54" s="13" t="s">
         <v>61</v>
@@ -5360,10 +5390,10 @@
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A55" s="13" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C55" s="13" t="s">
         <v>61</v>
@@ -5393,10 +5423,10 @@
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A56" s="13" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C56" s="13" t="s">
         <v>61</v>
@@ -5428,10 +5458,10 @@
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A57" s="13" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="B57" s="13" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C57" s="13" t="s">
         <v>61</v>
@@ -5461,10 +5491,10 @@
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A58" s="13" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C58" s="13" t="s">
         <v>61</v>
@@ -5494,10 +5524,10 @@
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A59" s="13" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="B59" s="13" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C59" s="13" t="s">
         <v>3</v>
@@ -5527,10 +5557,10 @@
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A60" s="13" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="B60" s="13" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="C60" s="13" t="s">
         <v>61</v>
@@ -5560,10 +5590,10 @@
     </row>
     <row r="61" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="13" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="C61" s="13" t="s">
         <v>61</v>
@@ -5593,10 +5623,10 @@
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A62" s="13" t="s">
-        <v>273</v>
+        <v>259</v>
       </c>
       <c r="B62" s="13" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="C62" s="13" t="s">
         <v>61</v>
@@ -5628,10 +5658,10 @@
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A63" s="13" t="s">
-        <v>274</v>
+        <v>260</v>
       </c>
       <c r="B63" s="13" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="C63" s="13" t="s">
         <v>61</v>
@@ -5661,19 +5691,19 @@
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A64" s="13" t="s">
-        <v>275</v>
+        <v>261</v>
       </c>
       <c r="B64" s="13" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="D64" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E64" s="13" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="F64" s="15"/>
       <c r="G64" s="25"/>
@@ -5694,10 +5724,10 @@
     </row>
     <row r="65" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A65" s="13" t="s">
-        <v>277</v>
+        <v>263</v>
       </c>
       <c r="B65" s="13" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C65" s="13" t="s">
         <v>61</v>
@@ -5708,7 +5738,7 @@
       <c r="E65" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="F65" s="15"/>
+      <c r="F65" s="13"/>
       <c r="G65" s="25"/>
       <c r="H65" s="15" t="s">
         <v>117</v>
@@ -5727,10 +5757,10 @@
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A66" s="13" t="s">
-        <v>278</v>
+        <v>264</v>
       </c>
       <c r="B66" s="13" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="C66" s="13" t="s">
         <v>61</v>
@@ -5741,7 +5771,7 @@
       <c r="E66" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="F66" s="15"/>
+      <c r="F66" s="13"/>
       <c r="G66" s="25"/>
       <c r="H66" s="15" t="s">
         <v>117</v>
@@ -5758,15 +5788,27 @@
       <c r="R66" s="15"/>
       <c r="S66" s="15"/>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A67" s="13"/>
-      <c r="B67" s="13"/>
-      <c r="C67" s="13"/>
-      <c r="D67" s="15"/>
-      <c r="E67" s="13"/>
-      <c r="F67" s="15"/>
+    <row r="67" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="B67" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="C67" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D67" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="E67" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="F67" s="13"/>
       <c r="G67" s="25"/>
-      <c r="H67" s="15"/>
+      <c r="H67" s="15" t="s">
+        <v>117</v>
+      </c>
       <c r="I67" s="15"/>
       <c r="J67" s="15"/>
       <c r="K67" s="15"/>

</xml_diff>

<commit_message>
updated script with kelly scenarios
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23901"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93400CF6-73AD-4EA8-8F31-2BF8383C8AED}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E140022D-EEBE-41D0-A2A8-964995F875F2}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1149" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1161" uniqueCount="324">
   <si>
     <t>1</t>
   </si>
@@ -983,6 +983,12 @@
   </si>
   <si>
     <t>825</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario021</t>
+  </si>
+  <si>
+    <t>826</t>
   </si>
 </sst>
 </file>
@@ -1502,7 +1508,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S222"/>
+  <dimension ref="A1:S223"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" customWidth="1"/>
@@ -4276,16 +4282,28 @@
       </c>
       <c r="S90" s="15"/>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A91" s="15"/>
-      <c r="B91" s="15"/>
-      <c r="C91" s="15"/>
-      <c r="D91" s="15"/>
+    <row r="91" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="15" t="s">
+        <v>322</v>
+      </c>
+      <c r="B91" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="C91" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="D91" s="13" t="s">
+        <v>323</v>
+      </c>
       <c r="E91" s="15"/>
-      <c r="F91" s="15"/>
+      <c r="F91" s="15" t="s">
+        <v>117</v>
+      </c>
       <c r="G91" s="15"/>
       <c r="H91" s="15"/>
-      <c r="I91" s="15"/>
+      <c r="I91" s="15" t="s">
+        <v>133</v>
+      </c>
       <c r="J91" s="15"/>
       <c r="K91" s="15"/>
       <c r="L91" s="15"/>
@@ -4294,34 +4312,22 @@
       <c r="O91" s="15"/>
       <c r="P91" s="15"/>
       <c r="Q91" s="15"/>
-      <c r="R91" s="15"/>
+      <c r="R91" s="13"/>
       <c r="S91" s="15"/>
     </row>
-    <row r="92" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="15" t="s">
-        <v>290</v>
-      </c>
-      <c r="B92" s="15" t="s">
-        <v>195</v>
-      </c>
-      <c r="C92" s="15" t="s">
-        <v>145</v>
-      </c>
+    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A92" s="15"/>
+      <c r="B92" s="15"/>
+      <c r="C92" s="15"/>
       <c r="D92" s="15"/>
       <c r="E92" s="15"/>
       <c r="F92" s="15"/>
       <c r="G92" s="15"/>
       <c r="H92" s="15"/>
       <c r="I92" s="15"/>
-      <c r="J92" s="13" t="s">
-        <v>297</v>
-      </c>
-      <c r="K92" s="13" t="s">
-        <v>298</v>
-      </c>
-      <c r="L92" s="13" t="s">
-        <v>299</v>
-      </c>
+      <c r="J92" s="15"/>
+      <c r="K92" s="15"/>
+      <c r="L92" s="15"/>
       <c r="M92" s="15"/>
       <c r="N92" s="15"/>
       <c r="O92" s="15"/>
@@ -4332,7 +4338,7 @@
     </row>
     <row r="93" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="15" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B93" s="15" t="s">
         <v>195</v>
@@ -4347,13 +4353,13 @@
       <c r="H93" s="15"/>
       <c r="I93" s="15"/>
       <c r="J93" s="13" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K93" s="13" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="L93" s="13" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="M93" s="15"/>
       <c r="N93" s="15"/>
@@ -4363,19 +4369,31 @@
       <c r="R93" s="15"/>
       <c r="S93" s="15"/>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A94" s="15"/>
-      <c r="B94" s="15"/>
-      <c r="C94" s="15"/>
+    <row r="94" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="15" t="s">
+        <v>291</v>
+      </c>
+      <c r="B94" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="C94" s="15" t="s">
+        <v>145</v>
+      </c>
       <c r="D94" s="15"/>
       <c r="E94" s="15"/>
       <c r="F94" s="15"/>
       <c r="G94" s="15"/>
       <c r="H94" s="15"/>
       <c r="I94" s="15"/>
-      <c r="J94" s="15"/>
-      <c r="K94" s="15"/>
-      <c r="L94" s="15"/>
+      <c r="J94" s="13" t="s">
+        <v>296</v>
+      </c>
+      <c r="K94" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="L94" s="13" t="s">
+        <v>300</v>
+      </c>
       <c r="M94" s="15"/>
       <c r="N94" s="15"/>
       <c r="O94" s="15"/>
@@ -7071,6 +7089,27 @@
       <c r="Q222" s="15"/>
       <c r="R222" s="15"/>
       <c r="S222" s="15"/>
+    </row>
+    <row r="223" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A223" s="15"/>
+      <c r="B223" s="15"/>
+      <c r="C223" s="15"/>
+      <c r="D223" s="15"/>
+      <c r="E223" s="15"/>
+      <c r="F223" s="15"/>
+      <c r="G223" s="15"/>
+      <c r="H223" s="15"/>
+      <c r="I223" s="15"/>
+      <c r="J223" s="15"/>
+      <c r="K223" s="15"/>
+      <c r="L223" s="15"/>
+      <c r="M223" s="15"/>
+      <c r="N223" s="15"/>
+      <c r="O223" s="15"/>
+      <c r="P223" s="15"/>
+      <c r="Q223" s="15"/>
+      <c r="R223" s="15"/>
+      <c r="S223" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -9001,8 +9040,8 @@
       <c r="B53" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="C53" s="17" t="s">
-        <v>2</v>
+      <c r="C53" s="13" t="s">
+        <v>0</v>
       </c>
       <c r="D53" s="17" t="s">
         <v>115</v>
@@ -9038,8 +9077,8 @@
       <c r="B54" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="C54" s="17" t="s">
-        <v>2</v>
+      <c r="C54" s="13" t="s">
+        <v>0</v>
       </c>
       <c r="D54" s="17" t="s">
         <v>115</v>
@@ -9891,7 +9930,24 @@
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A84" s="13"/>
+      <c r="A84" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="B84" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="C84" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D84" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="E84" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="H84" s="15" t="s">
+        <v>117</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
Added with Fedexnet scenarios
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E140022D-EEBE-41D0-A2A8-964995F875F2}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{322CEA26-22B7-423D-8235-D4C93F18DB60}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1161" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1170" uniqueCount="328">
   <si>
     <t>1</t>
   </si>
@@ -989,13 +989,25 @@
   </si>
   <si>
     <t>826</t>
+  </si>
+  <si>
+    <t>OlpnStatus</t>
+  </si>
+  <si>
+    <t>10 - Printed</t>
+  </si>
+  <si>
+    <t>30 - Weighed</t>
+  </si>
+  <si>
+    <t>90 - Shipped</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1032,6 +1044,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Source Sans Pro"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1131,7 +1149,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1168,6 +1186,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1508,7 +1527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S223"/>
+  <dimension ref="A1:T223"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" customWidth="1"/>
@@ -1525,10 +1544,11 @@
     <col min="13" max="13" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="19.42578125" customWidth="1"/>
-    <col min="19" max="19" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1586,8 +1606,11 @@
       <c r="S1" s="24" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T1" s="24" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>225</v>
       </c>
@@ -1617,8 +1640,9 @@
       <c r="Q2" s="15"/>
       <c r="R2" s="15"/>
       <c r="S2" s="15"/>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T2" s="15"/>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>226</v>
       </c>
@@ -1648,8 +1672,9 @@
       <c r="Q3" s="15"/>
       <c r="R3" s="15"/>
       <c r="S3" s="15"/>
-    </row>
-    <row r="4" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T3" s="15"/>
+    </row>
+    <row r="4" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>227</v>
       </c>
@@ -1681,8 +1706,9 @@
       <c r="Q4" s="15"/>
       <c r="R4" s="15"/>
       <c r="S4" s="15"/>
-    </row>
-    <row r="5" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T4" s="15"/>
+    </row>
+    <row r="5" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>228</v>
       </c>
@@ -1712,8 +1738,9 @@
       <c r="Q5" s="15"/>
       <c r="R5" s="15"/>
       <c r="S5" s="15"/>
-    </row>
-    <row r="6" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T5" s="15"/>
+    </row>
+    <row r="6" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>229</v>
       </c>
@@ -1743,8 +1770,9 @@
       <c r="Q6" s="15"/>
       <c r="R6" s="15"/>
       <c r="S6" s="15"/>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T6" s="15"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>230</v>
       </c>
@@ -1776,8 +1804,9 @@
       <c r="Q7" s="15"/>
       <c r="R7" s="15"/>
       <c r="S7" s="15"/>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T7" s="15"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>231</v>
       </c>
@@ -1809,8 +1838,9 @@
       <c r="Q8" s="15"/>
       <c r="R8" s="15"/>
       <c r="S8" s="15"/>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T8" s="15"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>232</v>
       </c>
@@ -1842,8 +1872,9 @@
       <c r="Q9" s="15"/>
       <c r="R9" s="15"/>
       <c r="S9" s="15"/>
-    </row>
-    <row r="10" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T9" s="15"/>
+    </row>
+    <row r="10" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>233</v>
       </c>
@@ -1873,8 +1904,9 @@
       <c r="Q10" s="15"/>
       <c r="R10" s="15"/>
       <c r="S10" s="15"/>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T10" s="15"/>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>234</v>
       </c>
@@ -1906,8 +1938,9 @@
       <c r="Q11" s="15"/>
       <c r="R11" s="15"/>
       <c r="S11" s="15"/>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T11" s="15"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>235</v>
       </c>
@@ -1939,8 +1972,9 @@
       <c r="Q12" s="15"/>
       <c r="R12" s="15"/>
       <c r="S12" s="15"/>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T12" s="15"/>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>236</v>
       </c>
@@ -1970,8 +2004,9 @@
       <c r="Q13" s="15"/>
       <c r="R13" s="15"/>
       <c r="S13" s="15"/>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T13" s="15"/>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>237</v>
       </c>
@@ -2001,8 +2036,9 @@
       <c r="Q14" s="15"/>
       <c r="R14" s="15"/>
       <c r="S14" s="15"/>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T14" s="15"/>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>238</v>
       </c>
@@ -2034,8 +2070,9 @@
       <c r="Q15" s="15"/>
       <c r="R15" s="15"/>
       <c r="S15" s="15"/>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T15" s="15"/>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>239</v>
       </c>
@@ -2067,8 +2104,9 @@
       <c r="Q16" s="15"/>
       <c r="R16" s="15"/>
       <c r="S16" s="15"/>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T16" s="15"/>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>240</v>
       </c>
@@ -2100,8 +2138,9 @@
       <c r="Q17" s="15"/>
       <c r="R17" s="15"/>
       <c r="S17" s="15"/>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T17" s="15"/>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
         <v>241</v>
       </c>
@@ -2133,8 +2172,9 @@
       <c r="Q18" s="15"/>
       <c r="R18" s="15"/>
       <c r="S18" s="15"/>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T18" s="15"/>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>242</v>
       </c>
@@ -2165,8 +2205,9 @@
       <c r="Q19" s="15"/>
       <c r="R19" s="15"/>
       <c r="S19" s="15"/>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T19" s="15"/>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>243</v>
       </c>
@@ -2197,8 +2238,9 @@
       <c r="Q20" s="15"/>
       <c r="R20" s="15"/>
       <c r="S20" s="15"/>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T20" s="15"/>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
         <v>244</v>
       </c>
@@ -2230,8 +2272,9 @@
       <c r="Q21" s="15"/>
       <c r="R21" s="15"/>
       <c r="S21" s="15"/>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T21" s="15"/>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
         <v>245</v>
       </c>
@@ -2263,8 +2306,9 @@
       <c r="Q22" s="15"/>
       <c r="R22" s="15"/>
       <c r="S22" s="15"/>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T22" s="15"/>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
         <v>246</v>
       </c>
@@ -2296,8 +2340,9 @@
       <c r="Q23" s="15"/>
       <c r="R23" s="15"/>
       <c r="S23" s="15"/>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T23" s="15"/>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
         <v>247</v>
       </c>
@@ -2329,8 +2374,9 @@
       <c r="Q24" s="15"/>
       <c r="R24" s="15"/>
       <c r="S24" s="15"/>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T24" s="15"/>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
         <v>248</v>
       </c>
@@ -2362,8 +2408,9 @@
       <c r="Q25" s="15"/>
       <c r="R25" s="15"/>
       <c r="S25" s="15"/>
-    </row>
-    <row r="26" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T25" s="15"/>
+    </row>
+    <row r="26" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
         <v>249</v>
       </c>
@@ -2393,8 +2440,9 @@
       <c r="Q26" s="15"/>
       <c r="R26" s="15"/>
       <c r="S26" s="15"/>
-    </row>
-    <row r="27" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T26" s="15"/>
+    </row>
+    <row r="27" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
         <v>250</v>
       </c>
@@ -2424,8 +2472,9 @@
       <c r="Q27" s="15"/>
       <c r="R27" s="15"/>
       <c r="S27" s="15"/>
-    </row>
-    <row r="28" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T27" s="15"/>
+    </row>
+    <row r="28" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>251</v>
       </c>
@@ -2455,8 +2504,9 @@
       <c r="Q28" s="15"/>
       <c r="R28" s="15"/>
       <c r="S28" s="15"/>
-    </row>
-    <row r="29" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T28" s="15"/>
+    </row>
+    <row r="29" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
         <v>252</v>
       </c>
@@ -2486,8 +2536,9 @@
       <c r="Q29" s="15"/>
       <c r="R29" s="15"/>
       <c r="S29" s="15"/>
-    </row>
-    <row r="30" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T29" s="15"/>
+    </row>
+    <row r="30" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
         <v>253</v>
       </c>
@@ -2517,8 +2568,9 @@
       <c r="Q30" s="15"/>
       <c r="R30" s="15"/>
       <c r="S30" s="15"/>
-    </row>
-    <row r="31" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T30" s="15"/>
+    </row>
+    <row r="31" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
         <v>254</v>
       </c>
@@ -2548,8 +2600,9 @@
       <c r="Q31" s="15"/>
       <c r="R31" s="15"/>
       <c r="S31" s="15"/>
-    </row>
-    <row r="32" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T31" s="15"/>
+    </row>
+    <row r="32" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
         <v>255</v>
       </c>
@@ -2579,8 +2632,9 @@
       <c r="Q32" s="15"/>
       <c r="R32" s="15"/>
       <c r="S32" s="15"/>
-    </row>
-    <row r="33" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T32" s="15"/>
+    </row>
+    <row r="33" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
         <v>256</v>
       </c>
@@ -2610,8 +2664,9 @@
       <c r="Q33" s="15"/>
       <c r="R33" s="15"/>
       <c r="S33" s="15"/>
-    </row>
-    <row r="34" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T33" s="15"/>
+    </row>
+    <row r="34" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
         <v>257</v>
       </c>
@@ -2639,8 +2694,9 @@
       <c r="Q34" s="15"/>
       <c r="R34" s="15"/>
       <c r="S34" s="15"/>
-    </row>
-    <row r="35" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T34" s="15"/>
+    </row>
+    <row r="35" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="13"/>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
@@ -2660,8 +2716,9 @@
       <c r="Q35" s="15"/>
       <c r="R35" s="15"/>
       <c r="S35" s="15"/>
-    </row>
-    <row r="36" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T35" s="15"/>
+    </row>
+    <row r="36" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
         <v>147</v>
       </c>
@@ -2689,8 +2746,9 @@
       <c r="Q36" s="15"/>
       <c r="R36" s="15"/>
       <c r="S36" s="15"/>
-    </row>
-    <row r="37" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T36" s="15"/>
+    </row>
+    <row r="37" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
         <v>154</v>
       </c>
@@ -2718,8 +2776,9 @@
       <c r="Q37" s="15"/>
       <c r="R37" s="15"/>
       <c r="S37" s="15"/>
-    </row>
-    <row r="38" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T37" s="15"/>
+    </row>
+    <row r="38" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
         <v>157</v>
       </c>
@@ -2747,8 +2806,9 @@
       <c r="Q38" s="15"/>
       <c r="R38" s="15"/>
       <c r="S38" s="15"/>
-    </row>
-    <row r="39" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T38" s="15"/>
+    </row>
+    <row r="39" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
         <v>173</v>
       </c>
@@ -2778,8 +2838,9 @@
       </c>
       <c r="R39" s="15"/>
       <c r="S39" s="15"/>
-    </row>
-    <row r="40" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T39" s="15"/>
+    </row>
+    <row r="40" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
         <v>178</v>
       </c>
@@ -2809,8 +2870,9 @@
       </c>
       <c r="R40" s="15"/>
       <c r="S40" s="15"/>
-    </row>
-    <row r="41" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T40" s="15"/>
+    </row>
+    <row r="41" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="15" t="s">
         <v>190</v>
       </c>
@@ -2840,8 +2902,9 @@
       </c>
       <c r="R41" s="26"/>
       <c r="S41" s="15"/>
-    </row>
-    <row r="42" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T41" s="15"/>
+    </row>
+    <row r="42" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
         <v>194</v>
       </c>
@@ -2871,8 +2934,9 @@
       </c>
       <c r="R42" s="26"/>
       <c r="S42" s="15"/>
-    </row>
-    <row r="43" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T42" s="15"/>
+    </row>
+    <row r="43" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="15" t="s">
         <v>207</v>
       </c>
@@ -2902,8 +2966,9 @@
       </c>
       <c r="R43" s="26"/>
       <c r="S43" s="15"/>
-    </row>
-    <row r="44" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T43" s="15"/>
+    </row>
+    <row r="44" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="15" t="s">
         <v>208</v>
       </c>
@@ -2931,8 +2996,9 @@
       <c r="Q44" s="15"/>
       <c r="R44" s="26"/>
       <c r="S44" s="15"/>
-    </row>
-    <row r="45" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T44" s="15"/>
+    </row>
+    <row r="45" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="15" t="s">
         <v>209</v>
       </c>
@@ -2960,8 +3026,9 @@
       <c r="Q45" s="15"/>
       <c r="R45" s="26"/>
       <c r="S45" s="15"/>
-    </row>
-    <row r="46" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T45" s="15"/>
+    </row>
+    <row r="46" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="15" t="s">
         <v>210</v>
       </c>
@@ -2989,8 +3056,9 @@
       <c r="Q46" s="15"/>
       <c r="R46" s="26"/>
       <c r="S46" s="15"/>
-    </row>
-    <row r="47" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T46" s="15"/>
+    </row>
+    <row r="47" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="15" t="s">
         <v>221</v>
       </c>
@@ -3018,8 +3086,9 @@
       <c r="Q47" s="15"/>
       <c r="R47" s="26"/>
       <c r="S47" s="15"/>
-    </row>
-    <row r="48" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T47" s="15"/>
+    </row>
+    <row r="48" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
         <v>280</v>
       </c>
@@ -3046,9 +3115,14 @@
       <c r="P48" s="15"/>
       <c r="Q48" s="15"/>
       <c r="R48" s="26"/>
-      <c r="S48" s="15"/>
-    </row>
-    <row r="49" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S48" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="T48" s="15" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="49" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="15" t="s">
         <v>281</v>
       </c>
@@ -3075,9 +3149,14 @@
       <c r="P49" s="15"/>
       <c r="Q49" s="15"/>
       <c r="R49" s="26"/>
-      <c r="S49" s="15"/>
-    </row>
-    <row r="50" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S49" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="T49" s="13" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="50" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="15" t="s">
         <v>282</v>
       </c>
@@ -3104,9 +3183,14 @@
       <c r="P50" s="15"/>
       <c r="Q50" s="15"/>
       <c r="R50" s="26"/>
-      <c r="S50" s="15"/>
-    </row>
-    <row r="51" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S50" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="T50" s="28" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
         <v>283</v>
       </c>
@@ -3138,8 +3222,11 @@
       <c r="S51" s="13" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T51" s="15" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="52" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="15" t="s">
         <v>284</v>
       </c>
@@ -3171,8 +3258,11 @@
       <c r="S52" s="13" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T52" s="15" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="15" t="s">
         <v>285</v>
       </c>
@@ -3204,8 +3294,9 @@
       <c r="S53" s="13" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T53" s="15"/>
+    </row>
+    <row r="54" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="15"/>
       <c r="B54" s="15"/>
       <c r="C54" s="15"/>
@@ -3225,8 +3316,9 @@
       <c r="Q54" s="15"/>
       <c r="R54" s="26"/>
       <c r="S54" s="15"/>
-    </row>
-    <row r="55" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T54" s="15"/>
+    </row>
+    <row r="55" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="15"/>
       <c r="B55" s="15"/>
       <c r="C55" s="15"/>
@@ -3246,8 +3338,9 @@
       <c r="Q55" s="15"/>
       <c r="R55" s="26"/>
       <c r="S55" s="15"/>
-    </row>
-    <row r="56" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T55" s="15"/>
+    </row>
+    <row r="56" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="15"/>
       <c r="B56" s="15"/>
       <c r="C56" s="15"/>
@@ -3267,8 +3360,9 @@
       <c r="Q56" s="15"/>
       <c r="R56" s="26"/>
       <c r="S56" s="15"/>
-    </row>
-    <row r="57" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T56" s="15"/>
+    </row>
+    <row r="57" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="15"/>
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
@@ -3288,8 +3382,9 @@
       <c r="Q57" s="15"/>
       <c r="R57" s="26"/>
       <c r="S57" s="15"/>
-    </row>
-    <row r="58" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T57" s="15"/>
+    </row>
+    <row r="58" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="15"/>
       <c r="B58" s="15"/>
       <c r="C58" s="15"/>
@@ -3309,8 +3404,9 @@
       <c r="Q58" s="15"/>
       <c r="R58" s="26"/>
       <c r="S58" s="15"/>
-    </row>
-    <row r="59" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T58" s="15"/>
+    </row>
+    <row r="59" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="15"/>
       <c r="B59" s="15"/>
       <c r="C59" s="15"/>
@@ -3330,8 +3426,9 @@
       <c r="Q59" s="15"/>
       <c r="R59" s="26"/>
       <c r="S59" s="15"/>
-    </row>
-    <row r="60" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T59" s="15"/>
+    </row>
+    <row r="60" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="15" t="s">
         <v>159</v>
       </c>
@@ -3363,8 +3460,9 @@
       <c r="Q60" s="15"/>
       <c r="R60" s="26"/>
       <c r="S60" s="15"/>
-    </row>
-    <row r="61" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T60" s="15"/>
+    </row>
+    <row r="61" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="15" t="s">
         <v>160</v>
       </c>
@@ -3392,8 +3490,9 @@
       <c r="Q61" s="15"/>
       <c r="R61" s="26"/>
       <c r="S61" s="15"/>
-    </row>
-    <row r="62" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T61" s="15"/>
+    </row>
+    <row r="62" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="15" t="s">
         <v>161</v>
       </c>
@@ -3421,8 +3520,9 @@
       <c r="Q62" s="15"/>
       <c r="R62" s="26"/>
       <c r="S62" s="15"/>
-    </row>
-    <row r="63" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T62" s="15"/>
+    </row>
+    <row r="63" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="15" t="s">
         <v>162</v>
       </c>
@@ -3450,8 +3550,9 @@
       <c r="Q63" s="15"/>
       <c r="R63" s="26"/>
       <c r="S63" s="15"/>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T63" s="15"/>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A64" s="15" t="s">
         <v>163</v>
       </c>
@@ -3479,8 +3580,9 @@
       <c r="Q64" s="15"/>
       <c r="R64" s="26"/>
       <c r="S64" s="15"/>
-    </row>
-    <row r="65" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T64" s="15"/>
+    </row>
+    <row r="65" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="15"/>
       <c r="B65" s="15"/>
       <c r="C65" s="15"/>
@@ -3500,8 +3602,9 @@
       <c r="Q65" s="15"/>
       <c r="R65" s="26"/>
       <c r="S65" s="15"/>
-    </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T65" s="15"/>
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A66" s="15"/>
       <c r="B66" s="15"/>
       <c r="C66" s="15"/>
@@ -3521,8 +3624,9 @@
       <c r="Q66" s="15"/>
       <c r="R66" s="26"/>
       <c r="S66" s="15"/>
-    </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T66" s="15"/>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A67" s="13" t="s">
         <v>108</v>
       </c>
@@ -3550,8 +3654,9 @@
       <c r="Q67" s="15"/>
       <c r="R67" s="26"/>
       <c r="S67" s="15"/>
-    </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T67" s="15"/>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A68" s="13" t="s">
         <v>109</v>
       </c>
@@ -3579,8 +3684,9 @@
       <c r="Q68" s="15"/>
       <c r="R68" s="26"/>
       <c r="S68" s="15"/>
-    </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T68" s="15"/>
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A69" s="13" t="s">
         <v>128</v>
       </c>
@@ -3610,8 +3716,9 @@
       <c r="Q69" s="15"/>
       <c r="R69" s="26"/>
       <c r="S69" s="15"/>
-    </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T69" s="15"/>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A70" s="15"/>
       <c r="B70" s="15"/>
       <c r="C70" s="15"/>
@@ -3631,8 +3738,9 @@
       <c r="Q70" s="15"/>
       <c r="R70" s="26"/>
       <c r="S70" s="15"/>
-    </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T70" s="15"/>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A71" s="15" t="s">
         <v>265</v>
       </c>
@@ -3664,8 +3772,9 @@
         <v>0</v>
       </c>
       <c r="S71" s="15"/>
-    </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T71" s="15"/>
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A72" s="15" t="s">
         <v>266</v>
       </c>
@@ -3697,8 +3806,9 @@
         <v>0</v>
       </c>
       <c r="S72" s="15"/>
-    </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T72" s="15"/>
+    </row>
+    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A73" s="15" t="s">
         <v>267</v>
       </c>
@@ -3730,8 +3840,9 @@
         <v>0</v>
       </c>
       <c r="S73" s="15"/>
-    </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T73" s="15"/>
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A74" s="15" t="s">
         <v>268</v>
       </c>
@@ -3763,8 +3874,9 @@
         <v>0</v>
       </c>
       <c r="S74" s="15"/>
-    </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T74" s="15"/>
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A75" s="15" t="s">
         <v>269</v>
       </c>
@@ -3796,8 +3908,9 @@
         <v>0</v>
       </c>
       <c r="S75" s="15"/>
-    </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T75" s="15"/>
+    </row>
+    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A76" s="15" t="s">
         <v>270</v>
       </c>
@@ -3829,8 +3942,9 @@
         <v>0</v>
       </c>
       <c r="S76" s="15"/>
-    </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T76" s="15"/>
+    </row>
+    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A77" s="15" t="s">
         <v>271</v>
       </c>
@@ -3862,8 +3976,9 @@
         <v>2</v>
       </c>
       <c r="S77" s="15"/>
-    </row>
-    <row r="78" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T77" s="15"/>
+    </row>
+    <row r="78" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="15" t="s">
         <v>272</v>
       </c>
@@ -3893,8 +4008,9 @@
       <c r="Q78" s="15"/>
       <c r="R78" s="18"/>
       <c r="S78" s="15"/>
-    </row>
-    <row r="79" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T78" s="15"/>
+    </row>
+    <row r="79" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="15" t="s">
         <v>273</v>
       </c>
@@ -3924,8 +4040,9 @@
       <c r="Q79" s="15"/>
       <c r="R79" s="13"/>
       <c r="S79" s="15"/>
-    </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T79" s="15"/>
+    </row>
+    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A80" s="15" t="s">
         <v>274</v>
       </c>
@@ -3955,8 +4072,9 @@
       <c r="Q80" s="15"/>
       <c r="R80" s="13"/>
       <c r="S80" s="15"/>
-    </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T80" s="15"/>
+    </row>
+    <row r="81" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A81" s="15" t="s">
         <v>275</v>
       </c>
@@ -3986,8 +4104,9 @@
       <c r="Q81" s="15"/>
       <c r="R81" s="13"/>
       <c r="S81" s="15"/>
-    </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T81" s="15"/>
+    </row>
+    <row r="82" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A82" s="15" t="s">
         <v>276</v>
       </c>
@@ -4017,8 +4136,9 @@
       <c r="Q82" s="15"/>
       <c r="R82" s="13"/>
       <c r="S82" s="15"/>
-    </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T82" s="15"/>
+    </row>
+    <row r="83" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="s">
         <v>277</v>
       </c>
@@ -4050,8 +4170,9 @@
         <v>0</v>
       </c>
       <c r="S83" s="15"/>
-    </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T83" s="15"/>
+    </row>
+    <row r="84" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A84" s="15" t="s">
         <v>278</v>
       </c>
@@ -4083,8 +4204,9 @@
         <v>0</v>
       </c>
       <c r="S84" s="15"/>
-    </row>
-    <row r="85" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T84" s="15"/>
+    </row>
+    <row r="85" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="15" t="s">
         <v>302</v>
       </c>
@@ -4116,8 +4238,9 @@
         <v>0</v>
       </c>
       <c r="S85" s="15"/>
-    </row>
-    <row r="86" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T85" s="15"/>
+    </row>
+    <row r="86" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="15" t="s">
         <v>309</v>
       </c>
@@ -4149,8 +4272,9 @@
         <v>2</v>
       </c>
       <c r="S86" s="15"/>
-    </row>
-    <row r="87" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T86" s="15"/>
+    </row>
+    <row r="87" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="15" t="s">
         <v>311</v>
       </c>
@@ -4182,8 +4306,9 @@
         <v>0</v>
       </c>
       <c r="S87" s="15"/>
-    </row>
-    <row r="88" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T87" s="15"/>
+    </row>
+    <row r="88" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="15" t="s">
         <v>312</v>
       </c>
@@ -4215,8 +4340,9 @@
         <v>0</v>
       </c>
       <c r="S88" s="15"/>
-    </row>
-    <row r="89" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T88" s="15"/>
+    </row>
+    <row r="89" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="15" t="s">
         <v>316</v>
       </c>
@@ -4248,8 +4374,9 @@
         <v>2</v>
       </c>
       <c r="S89" s="15"/>
-    </row>
-    <row r="90" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T89" s="15"/>
+    </row>
+    <row r="90" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="15" t="s">
         <v>318</v>
       </c>
@@ -4281,8 +4408,9 @@
         <v>0</v>
       </c>
       <c r="S90" s="15"/>
-    </row>
-    <row r="91" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T90" s="15"/>
+    </row>
+    <row r="91" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="15" t="s">
         <v>322</v>
       </c>
@@ -4314,8 +4442,9 @@
       <c r="Q91" s="15"/>
       <c r="R91" s="13"/>
       <c r="S91" s="15"/>
-    </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T91" s="15"/>
+    </row>
+    <row r="92" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A92" s="15"/>
       <c r="B92" s="15"/>
       <c r="C92" s="15"/>
@@ -4335,8 +4464,9 @@
       <c r="Q92" s="15"/>
       <c r="R92" s="15"/>
       <c r="S92" s="15"/>
-    </row>
-    <row r="93" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T92" s="15"/>
+    </row>
+    <row r="93" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="15" t="s">
         <v>290</v>
       </c>
@@ -4368,8 +4498,9 @@
       <c r="Q93" s="15"/>
       <c r="R93" s="15"/>
       <c r="S93" s="15"/>
-    </row>
-    <row r="94" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="T93" s="15"/>
+    </row>
+    <row r="94" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="15" t="s">
         <v>291</v>
       </c>
@@ -4401,8 +4532,9 @@
       <c r="Q94" s="15"/>
       <c r="R94" s="15"/>
       <c r="S94" s="15"/>
-    </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T94" s="15"/>
+    </row>
+    <row r="95" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A95" s="15"/>
       <c r="B95" s="15"/>
       <c r="C95" s="15"/>
@@ -4422,8 +4554,9 @@
       <c r="Q95" s="15"/>
       <c r="R95" s="15"/>
       <c r="S95" s="15"/>
-    </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T95" s="15"/>
+    </row>
+    <row r="96" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A96" s="15"/>
       <c r="B96" s="15"/>
       <c r="C96" s="15"/>
@@ -4443,8 +4576,9 @@
       <c r="Q96" s="15"/>
       <c r="R96" s="15"/>
       <c r="S96" s="15"/>
-    </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T96" s="15"/>
+    </row>
+    <row r="97" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A97" s="15"/>
       <c r="B97" s="15"/>
       <c r="C97" s="15"/>
@@ -4464,8 +4598,9 @@
       <c r="Q97" s="15"/>
       <c r="R97" s="15"/>
       <c r="S97" s="15"/>
-    </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T97" s="15"/>
+    </row>
+    <row r="98" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A98" s="15"/>
       <c r="B98" s="15"/>
       <c r="C98" s="15"/>
@@ -4485,8 +4620,9 @@
       <c r="Q98" s="15"/>
       <c r="R98" s="15"/>
       <c r="S98" s="15"/>
-    </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T98" s="15"/>
+    </row>
+    <row r="99" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A99" s="15"/>
       <c r="B99" s="15"/>
       <c r="C99" s="15"/>
@@ -4506,8 +4642,9 @@
       <c r="Q99" s="15"/>
       <c r="R99" s="15"/>
       <c r="S99" s="15"/>
-    </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T99" s="15"/>
+    </row>
+    <row r="100" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A100" s="15"/>
       <c r="B100" s="15"/>
       <c r="C100" s="15"/>
@@ -4527,8 +4664,9 @@
       <c r="Q100" s="15"/>
       <c r="R100" s="15"/>
       <c r="S100" s="15"/>
-    </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T100" s="15"/>
+    </row>
+    <row r="101" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A101" s="15"/>
       <c r="B101" s="15"/>
       <c r="C101" s="15"/>
@@ -4548,8 +4686,9 @@
       <c r="Q101" s="15"/>
       <c r="R101" s="15"/>
       <c r="S101" s="15"/>
-    </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T101" s="15"/>
+    </row>
+    <row r="102" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A102" s="15"/>
       <c r="B102" s="15"/>
       <c r="C102" s="15"/>
@@ -4569,8 +4708,9 @@
       <c r="Q102" s="15"/>
       <c r="R102" s="15"/>
       <c r="S102" s="15"/>
-    </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T102" s="15"/>
+    </row>
+    <row r="103" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A103" s="15"/>
       <c r="B103" s="15"/>
       <c r="C103" s="15"/>
@@ -4590,8 +4730,9 @@
       <c r="Q103" s="15"/>
       <c r="R103" s="15"/>
       <c r="S103" s="15"/>
-    </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T103" s="15"/>
+    </row>
+    <row r="104" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A104" s="15"/>
       <c r="B104" s="15"/>
       <c r="C104" s="15"/>
@@ -4611,8 +4752,9 @@
       <c r="Q104" s="15"/>
       <c r="R104" s="15"/>
       <c r="S104" s="15"/>
-    </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T104" s="15"/>
+    </row>
+    <row r="105" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A105" s="15"/>
       <c r="B105" s="15"/>
       <c r="C105" s="15"/>
@@ -4632,8 +4774,9 @@
       <c r="Q105" s="15"/>
       <c r="R105" s="15"/>
       <c r="S105" s="15"/>
-    </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T105" s="15"/>
+    </row>
+    <row r="106" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A106" s="15"/>
       <c r="B106" s="15"/>
       <c r="C106" s="15"/>
@@ -4653,8 +4796,9 @@
       <c r="Q106" s="15"/>
       <c r="R106" s="15"/>
       <c r="S106" s="15"/>
-    </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T106" s="15"/>
+    </row>
+    <row r="107" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A107" s="15"/>
       <c r="B107" s="15"/>
       <c r="C107" s="15"/>
@@ -4674,8 +4818,9 @@
       <c r="Q107" s="15"/>
       <c r="R107" s="15"/>
       <c r="S107" s="15"/>
-    </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T107" s="15"/>
+    </row>
+    <row r="108" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A108" s="15"/>
       <c r="B108" s="15"/>
       <c r="C108" s="15"/>
@@ -4695,8 +4840,9 @@
       <c r="Q108" s="15"/>
       <c r="R108" s="15"/>
       <c r="S108" s="15"/>
-    </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T108" s="15"/>
+    </row>
+    <row r="109" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A109" s="15"/>
       <c r="B109" s="15"/>
       <c r="C109" s="15"/>
@@ -4716,8 +4862,9 @@
       <c r="Q109" s="15"/>
       <c r="R109" s="15"/>
       <c r="S109" s="15"/>
-    </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T109" s="15"/>
+    </row>
+    <row r="110" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A110" s="15"/>
       <c r="B110" s="15"/>
       <c r="C110" s="15"/>
@@ -4737,8 +4884,9 @@
       <c r="Q110" s="15"/>
       <c r="R110" s="15"/>
       <c r="S110" s="15"/>
-    </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T110" s="15"/>
+    </row>
+    <row r="111" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A111" s="15"/>
       <c r="B111" s="15"/>
       <c r="C111" s="15"/>
@@ -4758,8 +4906,9 @@
       <c r="Q111" s="15"/>
       <c r="R111" s="15"/>
       <c r="S111" s="15"/>
-    </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T111" s="15"/>
+    </row>
+    <row r="112" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A112" s="15"/>
       <c r="B112" s="15"/>
       <c r="C112" s="15"/>
@@ -4779,8 +4928,9 @@
       <c r="Q112" s="15"/>
       <c r="R112" s="15"/>
       <c r="S112" s="15"/>
-    </row>
-    <row r="113" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T112" s="15"/>
+    </row>
+    <row r="113" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A113" s="15"/>
       <c r="B113" s="15"/>
       <c r="C113" s="15"/>
@@ -4800,8 +4950,9 @@
       <c r="Q113" s="15"/>
       <c r="R113" s="15"/>
       <c r="S113" s="15"/>
-    </row>
-    <row r="114" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T113" s="15"/>
+    </row>
+    <row r="114" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A114" s="15"/>
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
@@ -4821,8 +4972,9 @@
       <c r="Q114" s="15"/>
       <c r="R114" s="15"/>
       <c r="S114" s="15"/>
-    </row>
-    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T114" s="15"/>
+    </row>
+    <row r="115" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A115" s="15"/>
       <c r="B115" s="15"/>
       <c r="C115" s="15"/>
@@ -4842,8 +4994,9 @@
       <c r="Q115" s="15"/>
       <c r="R115" s="15"/>
       <c r="S115" s="15"/>
-    </row>
-    <row r="116" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T115" s="15"/>
+    </row>
+    <row r="116" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A116" s="15"/>
       <c r="B116" s="15"/>
       <c r="C116" s="15"/>
@@ -4863,8 +5016,9 @@
       <c r="Q116" s="15"/>
       <c r="R116" s="15"/>
       <c r="S116" s="15"/>
-    </row>
-    <row r="117" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T116" s="15"/>
+    </row>
+    <row r="117" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A117" s="15"/>
       <c r="B117" s="15"/>
       <c r="C117" s="15"/>
@@ -4884,8 +5038,9 @@
       <c r="Q117" s="15"/>
       <c r="R117" s="15"/>
       <c r="S117" s="15"/>
-    </row>
-    <row r="118" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T117" s="15"/>
+    </row>
+    <row r="118" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A118" s="15"/>
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
@@ -4905,8 +5060,9 @@
       <c r="Q118" s="15"/>
       <c r="R118" s="15"/>
       <c r="S118" s="15"/>
-    </row>
-    <row r="119" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T118" s="15"/>
+    </row>
+    <row r="119" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A119" s="15"/>
       <c r="B119" s="15"/>
       <c r="C119" s="15"/>
@@ -4926,8 +5082,9 @@
       <c r="Q119" s="15"/>
       <c r="R119" s="15"/>
       <c r="S119" s="15"/>
-    </row>
-    <row r="120" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T119" s="15"/>
+    </row>
+    <row r="120" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A120" s="15"/>
       <c r="B120" s="15"/>
       <c r="C120" s="15"/>
@@ -4947,8 +5104,9 @@
       <c r="Q120" s="15"/>
       <c r="R120" s="15"/>
       <c r="S120" s="15"/>
-    </row>
-    <row r="121" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T120" s="15"/>
+    </row>
+    <row r="121" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A121" s="15"/>
       <c r="B121" s="15"/>
       <c r="C121" s="15"/>
@@ -4968,8 +5126,9 @@
       <c r="Q121" s="15"/>
       <c r="R121" s="15"/>
       <c r="S121" s="15"/>
-    </row>
-    <row r="122" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T121" s="15"/>
+    </row>
+    <row r="122" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A122" s="15"/>
       <c r="B122" s="15"/>
       <c r="C122" s="15"/>
@@ -4989,8 +5148,9 @@
       <c r="Q122" s="15"/>
       <c r="R122" s="15"/>
       <c r="S122" s="15"/>
-    </row>
-    <row r="123" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T122" s="15"/>
+    </row>
+    <row r="123" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A123" s="15"/>
       <c r="B123" s="15"/>
       <c r="C123" s="15"/>
@@ -5010,8 +5170,9 @@
       <c r="Q123" s="15"/>
       <c r="R123" s="15"/>
       <c r="S123" s="15"/>
-    </row>
-    <row r="124" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T123" s="15"/>
+    </row>
+    <row r="124" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A124" s="15"/>
       <c r="B124" s="15"/>
       <c r="C124" s="15"/>
@@ -5031,8 +5192,9 @@
       <c r="Q124" s="15"/>
       <c r="R124" s="15"/>
       <c r="S124" s="15"/>
-    </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T124" s="15"/>
+    </row>
+    <row r="125" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A125" s="15"/>
       <c r="B125" s="15"/>
       <c r="C125" s="15"/>
@@ -5052,8 +5214,9 @@
       <c r="Q125" s="15"/>
       <c r="R125" s="15"/>
       <c r="S125" s="15"/>
-    </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T125" s="15"/>
+    </row>
+    <row r="126" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A126" s="15"/>
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
@@ -5073,8 +5236,9 @@
       <c r="Q126" s="15"/>
       <c r="R126" s="15"/>
       <c r="S126" s="15"/>
-    </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T126" s="15"/>
+    </row>
+    <row r="127" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A127" s="15"/>
       <c r="B127" s="15"/>
       <c r="C127" s="15"/>
@@ -5094,8 +5258,9 @@
       <c r="Q127" s="15"/>
       <c r="R127" s="15"/>
       <c r="S127" s="15"/>
-    </row>
-    <row r="128" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T127" s="15"/>
+    </row>
+    <row r="128" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A128" s="15"/>
       <c r="B128" s="15"/>
       <c r="C128" s="15"/>
@@ -5115,8 +5280,9 @@
       <c r="Q128" s="15"/>
       <c r="R128" s="15"/>
       <c r="S128" s="15"/>
-    </row>
-    <row r="129" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T128" s="15"/>
+    </row>
+    <row r="129" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A129" s="15"/>
       <c r="B129" s="15"/>
       <c r="C129" s="15"/>
@@ -5136,8 +5302,9 @@
       <c r="Q129" s="15"/>
       <c r="R129" s="15"/>
       <c r="S129" s="15"/>
-    </row>
-    <row r="130" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T129" s="15"/>
+    </row>
+    <row r="130" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A130" s="15"/>
       <c r="B130" s="15"/>
       <c r="C130" s="15"/>
@@ -5157,8 +5324,9 @@
       <c r="Q130" s="15"/>
       <c r="R130" s="15"/>
       <c r="S130" s="15"/>
-    </row>
-    <row r="131" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T130" s="15"/>
+    </row>
+    <row r="131" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A131" s="15"/>
       <c r="B131" s="15"/>
       <c r="C131" s="15"/>
@@ -5178,8 +5346,9 @@
       <c r="Q131" s="15"/>
       <c r="R131" s="15"/>
       <c r="S131" s="15"/>
-    </row>
-    <row r="132" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T131" s="15"/>
+    </row>
+    <row r="132" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A132" s="15"/>
       <c r="B132" s="15"/>
       <c r="C132" s="15"/>
@@ -5199,8 +5368,9 @@
       <c r="Q132" s="15"/>
       <c r="R132" s="15"/>
       <c r="S132" s="15"/>
-    </row>
-    <row r="133" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T132" s="15"/>
+    </row>
+    <row r="133" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A133" s="15"/>
       <c r="B133" s="15"/>
       <c r="C133" s="15"/>
@@ -5220,8 +5390,9 @@
       <c r="Q133" s="15"/>
       <c r="R133" s="15"/>
       <c r="S133" s="15"/>
-    </row>
-    <row r="134" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T133" s="15"/>
+    </row>
+    <row r="134" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A134" s="15"/>
       <c r="B134" s="15"/>
       <c r="C134" s="15"/>
@@ -5241,8 +5412,9 @@
       <c r="Q134" s="15"/>
       <c r="R134" s="15"/>
       <c r="S134" s="15"/>
-    </row>
-    <row r="135" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T134" s="15"/>
+    </row>
+    <row r="135" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A135" s="15"/>
       <c r="B135" s="15"/>
       <c r="C135" s="15"/>
@@ -5262,8 +5434,9 @@
       <c r="Q135" s="15"/>
       <c r="R135" s="15"/>
       <c r="S135" s="15"/>
-    </row>
-    <row r="136" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T135" s="15"/>
+    </row>
+    <row r="136" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A136" s="15"/>
       <c r="B136" s="15"/>
       <c r="C136" s="15"/>
@@ -5283,8 +5456,9 @@
       <c r="Q136" s="15"/>
       <c r="R136" s="15"/>
       <c r="S136" s="15"/>
-    </row>
-    <row r="137" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T136" s="15"/>
+    </row>
+    <row r="137" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A137" s="15"/>
       <c r="B137" s="15"/>
       <c r="C137" s="15"/>
@@ -5304,8 +5478,9 @@
       <c r="Q137" s="15"/>
       <c r="R137" s="15"/>
       <c r="S137" s="15"/>
-    </row>
-    <row r="138" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T137" s="15"/>
+    </row>
+    <row r="138" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A138" s="15"/>
       <c r="B138" s="15"/>
       <c r="C138" s="15"/>
@@ -5325,8 +5500,9 @@
       <c r="Q138" s="15"/>
       <c r="R138" s="15"/>
       <c r="S138" s="15"/>
-    </row>
-    <row r="139" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T138" s="15"/>
+    </row>
+    <row r="139" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A139" s="15"/>
       <c r="B139" s="15"/>
       <c r="C139" s="15"/>
@@ -5346,8 +5522,9 @@
       <c r="Q139" s="15"/>
       <c r="R139" s="15"/>
       <c r="S139" s="15"/>
-    </row>
-    <row r="140" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T139" s="15"/>
+    </row>
+    <row r="140" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A140" s="15"/>
       <c r="B140" s="15"/>
       <c r="C140" s="15"/>
@@ -5367,8 +5544,9 @@
       <c r="Q140" s="15"/>
       <c r="R140" s="15"/>
       <c r="S140" s="15"/>
-    </row>
-    <row r="141" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T140" s="15"/>
+    </row>
+    <row r="141" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A141" s="15"/>
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
@@ -5388,8 +5566,9 @@
       <c r="Q141" s="15"/>
       <c r="R141" s="15"/>
       <c r="S141" s="15"/>
-    </row>
-    <row r="142" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T141" s="15"/>
+    </row>
+    <row r="142" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A142" s="15"/>
       <c r="B142" s="15"/>
       <c r="C142" s="15"/>
@@ -5409,8 +5588,9 @@
       <c r="Q142" s="15"/>
       <c r="R142" s="15"/>
       <c r="S142" s="15"/>
-    </row>
-    <row r="143" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T142" s="15"/>
+    </row>
+    <row r="143" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A143" s="15"/>
       <c r="B143" s="15"/>
       <c r="C143" s="15"/>
@@ -5430,8 +5610,9 @@
       <c r="Q143" s="15"/>
       <c r="R143" s="15"/>
       <c r="S143" s="15"/>
-    </row>
-    <row r="144" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T143" s="15"/>
+    </row>
+    <row r="144" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A144" s="15"/>
       <c r="B144" s="15"/>
       <c r="C144" s="15"/>
@@ -5451,8 +5632,9 @@
       <c r="Q144" s="15"/>
       <c r="R144" s="15"/>
       <c r="S144" s="15"/>
-    </row>
-    <row r="145" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T144" s="15"/>
+    </row>
+    <row r="145" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A145" s="15"/>
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
@@ -5472,8 +5654,9 @@
       <c r="Q145" s="15"/>
       <c r="R145" s="15"/>
       <c r="S145" s="15"/>
-    </row>
-    <row r="146" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T145" s="15"/>
+    </row>
+    <row r="146" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A146" s="15"/>
       <c r="B146" s="15"/>
       <c r="C146" s="15"/>
@@ -5493,8 +5676,9 @@
       <c r="Q146" s="15"/>
       <c r="R146" s="15"/>
       <c r="S146" s="15"/>
-    </row>
-    <row r="147" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T146" s="15"/>
+    </row>
+    <row r="147" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A147" s="15"/>
       <c r="B147" s="15"/>
       <c r="C147" s="15"/>
@@ -5514,8 +5698,9 @@
       <c r="Q147" s="15"/>
       <c r="R147" s="15"/>
       <c r="S147" s="15"/>
-    </row>
-    <row r="148" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T147" s="15"/>
+    </row>
+    <row r="148" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A148" s="15"/>
       <c r="B148" s="15"/>
       <c r="C148" s="15"/>
@@ -5535,8 +5720,9 @@
       <c r="Q148" s="15"/>
       <c r="R148" s="15"/>
       <c r="S148" s="15"/>
-    </row>
-    <row r="149" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T148" s="15"/>
+    </row>
+    <row r="149" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A149" s="15"/>
       <c r="B149" s="15"/>
       <c r="C149" s="15"/>
@@ -5556,8 +5742,9 @@
       <c r="Q149" s="15"/>
       <c r="R149" s="15"/>
       <c r="S149" s="15"/>
-    </row>
-    <row r="150" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T149" s="15"/>
+    </row>
+    <row r="150" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A150" s="15"/>
       <c r="B150" s="15"/>
       <c r="C150" s="15"/>
@@ -5577,8 +5764,9 @@
       <c r="Q150" s="15"/>
       <c r="R150" s="15"/>
       <c r="S150" s="15"/>
-    </row>
-    <row r="151" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T150" s="15"/>
+    </row>
+    <row r="151" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A151" s="15"/>
       <c r="B151" s="15"/>
       <c r="C151" s="15"/>
@@ -5598,8 +5786,9 @@
       <c r="Q151" s="15"/>
       <c r="R151" s="15"/>
       <c r="S151" s="15"/>
-    </row>
-    <row r="152" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T151" s="15"/>
+    </row>
+    <row r="152" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A152" s="15"/>
       <c r="B152" s="15"/>
       <c r="C152" s="15"/>
@@ -5619,8 +5808,9 @@
       <c r="Q152" s="15"/>
       <c r="R152" s="15"/>
       <c r="S152" s="15"/>
-    </row>
-    <row r="153" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T152" s="15"/>
+    </row>
+    <row r="153" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A153" s="15"/>
       <c r="B153" s="15"/>
       <c r="C153" s="15"/>
@@ -5640,8 +5830,9 @@
       <c r="Q153" s="15"/>
       <c r="R153" s="15"/>
       <c r="S153" s="15"/>
-    </row>
-    <row r="154" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T153" s="15"/>
+    </row>
+    <row r="154" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A154" s="15"/>
       <c r="B154" s="15"/>
       <c r="C154" s="15"/>
@@ -5661,8 +5852,9 @@
       <c r="Q154" s="15"/>
       <c r="R154" s="15"/>
       <c r="S154" s="15"/>
-    </row>
-    <row r="155" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T154" s="15"/>
+    </row>
+    <row r="155" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A155" s="15"/>
       <c r="B155" s="15"/>
       <c r="C155" s="15"/>
@@ -5682,8 +5874,9 @@
       <c r="Q155" s="15"/>
       <c r="R155" s="15"/>
       <c r="S155" s="15"/>
-    </row>
-    <row r="156" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T155" s="15"/>
+    </row>
+    <row r="156" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A156" s="15"/>
       <c r="B156" s="15"/>
       <c r="C156" s="15"/>
@@ -5703,8 +5896,9 @@
       <c r="Q156" s="15"/>
       <c r="R156" s="15"/>
       <c r="S156" s="15"/>
-    </row>
-    <row r="157" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T156" s="15"/>
+    </row>
+    <row r="157" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A157" s="15"/>
       <c r="B157" s="15"/>
       <c r="C157" s="15"/>
@@ -5724,8 +5918,9 @@
       <c r="Q157" s="15"/>
       <c r="R157" s="15"/>
       <c r="S157" s="15"/>
-    </row>
-    <row r="158" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T157" s="15"/>
+    </row>
+    <row r="158" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A158" s="15"/>
       <c r="B158" s="15"/>
       <c r="C158" s="15"/>
@@ -5745,8 +5940,9 @@
       <c r="Q158" s="15"/>
       <c r="R158" s="15"/>
       <c r="S158" s="15"/>
-    </row>
-    <row r="159" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T158" s="15"/>
+    </row>
+    <row r="159" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A159" s="15"/>
       <c r="B159" s="15"/>
       <c r="C159" s="15"/>
@@ -5766,8 +5962,9 @@
       <c r="Q159" s="15"/>
       <c r="R159" s="15"/>
       <c r="S159" s="15"/>
-    </row>
-    <row r="160" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T159" s="15"/>
+    </row>
+    <row r="160" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A160" s="15"/>
       <c r="B160" s="15"/>
       <c r="C160" s="15"/>
@@ -5787,8 +5984,9 @@
       <c r="Q160" s="15"/>
       <c r="R160" s="15"/>
       <c r="S160" s="15"/>
-    </row>
-    <row r="161" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T160" s="15"/>
+    </row>
+    <row r="161" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A161" s="15"/>
       <c r="B161" s="15"/>
       <c r="C161" s="15"/>
@@ -5808,8 +6006,9 @@
       <c r="Q161" s="15"/>
       <c r="R161" s="15"/>
       <c r="S161" s="15"/>
-    </row>
-    <row r="162" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T161" s="15"/>
+    </row>
+    <row r="162" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A162" s="15"/>
       <c r="B162" s="15"/>
       <c r="C162" s="15"/>
@@ -5829,8 +6028,9 @@
       <c r="Q162" s="15"/>
       <c r="R162" s="15"/>
       <c r="S162" s="15"/>
-    </row>
-    <row r="163" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T162" s="15"/>
+    </row>
+    <row r="163" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A163" s="15"/>
       <c r="B163" s="15"/>
       <c r="C163" s="15"/>
@@ -5850,8 +6050,9 @@
       <c r="Q163" s="15"/>
       <c r="R163" s="15"/>
       <c r="S163" s="15"/>
-    </row>
-    <row r="164" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T163" s="15"/>
+    </row>
+    <row r="164" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A164" s="15"/>
       <c r="B164" s="15"/>
       <c r="C164" s="15"/>
@@ -5871,8 +6072,9 @@
       <c r="Q164" s="15"/>
       <c r="R164" s="15"/>
       <c r="S164" s="15"/>
-    </row>
-    <row r="165" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T164" s="15"/>
+    </row>
+    <row r="165" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A165" s="15"/>
       <c r="B165" s="15"/>
       <c r="C165" s="15"/>
@@ -5892,8 +6094,9 @@
       <c r="Q165" s="15"/>
       <c r="R165" s="15"/>
       <c r="S165" s="15"/>
-    </row>
-    <row r="166" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T165" s="15"/>
+    </row>
+    <row r="166" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A166" s="15"/>
       <c r="B166" s="15"/>
       <c r="C166" s="15"/>
@@ -5913,8 +6116,9 @@
       <c r="Q166" s="15"/>
       <c r="R166" s="15"/>
       <c r="S166" s="15"/>
-    </row>
-    <row r="167" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T166" s="15"/>
+    </row>
+    <row r="167" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A167" s="15"/>
       <c r="B167" s="15"/>
       <c r="C167" s="15"/>
@@ -5934,8 +6138,9 @@
       <c r="Q167" s="15"/>
       <c r="R167" s="15"/>
       <c r="S167" s="15"/>
-    </row>
-    <row r="168" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T167" s="15"/>
+    </row>
+    <row r="168" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A168" s="15"/>
       <c r="B168" s="15"/>
       <c r="C168" s="15"/>
@@ -5955,8 +6160,9 @@
       <c r="Q168" s="15"/>
       <c r="R168" s="15"/>
       <c r="S168" s="15"/>
-    </row>
-    <row r="169" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T168" s="15"/>
+    </row>
+    <row r="169" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A169" s="15"/>
       <c r="B169" s="15"/>
       <c r="C169" s="15"/>
@@ -5976,8 +6182,9 @@
       <c r="Q169" s="15"/>
       <c r="R169" s="15"/>
       <c r="S169" s="15"/>
-    </row>
-    <row r="170" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T169" s="15"/>
+    </row>
+    <row r="170" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A170" s="15"/>
       <c r="B170" s="15"/>
       <c r="C170" s="15"/>
@@ -5997,8 +6204,9 @@
       <c r="Q170" s="15"/>
       <c r="R170" s="15"/>
       <c r="S170" s="15"/>
-    </row>
-    <row r="171" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T170" s="15"/>
+    </row>
+    <row r="171" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A171" s="15"/>
       <c r="B171" s="15"/>
       <c r="C171" s="15"/>
@@ -6018,8 +6226,9 @@
       <c r="Q171" s="15"/>
       <c r="R171" s="15"/>
       <c r="S171" s="15"/>
-    </row>
-    <row r="172" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T171" s="15"/>
+    </row>
+    <row r="172" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A172" s="15"/>
       <c r="B172" s="15"/>
       <c r="C172" s="15"/>
@@ -6039,8 +6248,9 @@
       <c r="Q172" s="15"/>
       <c r="R172" s="15"/>
       <c r="S172" s="15"/>
-    </row>
-    <row r="173" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T172" s="15"/>
+    </row>
+    <row r="173" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A173" s="15"/>
       <c r="B173" s="15"/>
       <c r="C173" s="15"/>
@@ -6060,8 +6270,9 @@
       <c r="Q173" s="15"/>
       <c r="R173" s="15"/>
       <c r="S173" s="15"/>
-    </row>
-    <row r="174" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T173" s="15"/>
+    </row>
+    <row r="174" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A174" s="15"/>
       <c r="B174" s="15"/>
       <c r="C174" s="15"/>
@@ -6081,8 +6292,9 @@
       <c r="Q174" s="15"/>
       <c r="R174" s="15"/>
       <c r="S174" s="15"/>
-    </row>
-    <row r="175" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T174" s="15"/>
+    </row>
+    <row r="175" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A175" s="15"/>
       <c r="B175" s="15"/>
       <c r="C175" s="15"/>
@@ -6102,8 +6314,9 @@
       <c r="Q175" s="15"/>
       <c r="R175" s="15"/>
       <c r="S175" s="15"/>
-    </row>
-    <row r="176" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T175" s="15"/>
+    </row>
+    <row r="176" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A176" s="15"/>
       <c r="B176" s="15"/>
       <c r="C176" s="15"/>
@@ -6123,8 +6336,9 @@
       <c r="Q176" s="15"/>
       <c r="R176" s="15"/>
       <c r="S176" s="15"/>
-    </row>
-    <row r="177" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T176" s="15"/>
+    </row>
+    <row r="177" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A177" s="15"/>
       <c r="B177" s="15"/>
       <c r="C177" s="15"/>
@@ -6144,8 +6358,9 @@
       <c r="Q177" s="15"/>
       <c r="R177" s="15"/>
       <c r="S177" s="15"/>
-    </row>
-    <row r="178" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T177" s="15"/>
+    </row>
+    <row r="178" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A178" s="15"/>
       <c r="B178" s="15"/>
       <c r="C178" s="15"/>
@@ -6165,8 +6380,9 @@
       <c r="Q178" s="15"/>
       <c r="R178" s="15"/>
       <c r="S178" s="15"/>
-    </row>
-    <row r="179" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T178" s="15"/>
+    </row>
+    <row r="179" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A179" s="15"/>
       <c r="B179" s="15"/>
       <c r="C179" s="15"/>
@@ -6186,8 +6402,9 @@
       <c r="Q179" s="15"/>
       <c r="R179" s="15"/>
       <c r="S179" s="15"/>
-    </row>
-    <row r="180" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T179" s="15"/>
+    </row>
+    <row r="180" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A180" s="15"/>
       <c r="B180" s="15"/>
       <c r="C180" s="15"/>
@@ -6207,8 +6424,9 @@
       <c r="Q180" s="15"/>
       <c r="R180" s="15"/>
       <c r="S180" s="15"/>
-    </row>
-    <row r="181" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T180" s="15"/>
+    </row>
+    <row r="181" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A181" s="15"/>
       <c r="B181" s="15"/>
       <c r="C181" s="15"/>
@@ -6228,8 +6446,9 @@
       <c r="Q181" s="15"/>
       <c r="R181" s="15"/>
       <c r="S181" s="15"/>
-    </row>
-    <row r="182" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T181" s="15"/>
+    </row>
+    <row r="182" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A182" s="15"/>
       <c r="B182" s="15"/>
       <c r="C182" s="15"/>
@@ -6249,8 +6468,9 @@
       <c r="Q182" s="15"/>
       <c r="R182" s="15"/>
       <c r="S182" s="15"/>
-    </row>
-    <row r="183" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T182" s="15"/>
+    </row>
+    <row r="183" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A183" s="15"/>
       <c r="B183" s="15"/>
       <c r="C183" s="15"/>
@@ -6270,8 +6490,9 @@
       <c r="Q183" s="15"/>
       <c r="R183" s="15"/>
       <c r="S183" s="15"/>
-    </row>
-    <row r="184" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T183" s="15"/>
+    </row>
+    <row r="184" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A184" s="15"/>
       <c r="B184" s="15"/>
       <c r="C184" s="15"/>
@@ -6291,8 +6512,9 @@
       <c r="Q184" s="15"/>
       <c r="R184" s="15"/>
       <c r="S184" s="15"/>
-    </row>
-    <row r="185" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T184" s="15"/>
+    </row>
+    <row r="185" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A185" s="15"/>
       <c r="B185" s="15"/>
       <c r="C185" s="15"/>
@@ -6312,8 +6534,9 @@
       <c r="Q185" s="15"/>
       <c r="R185" s="15"/>
       <c r="S185" s="15"/>
-    </row>
-    <row r="186" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T185" s="15"/>
+    </row>
+    <row r="186" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A186" s="15"/>
       <c r="B186" s="15"/>
       <c r="C186" s="15"/>
@@ -6333,8 +6556,9 @@
       <c r="Q186" s="15"/>
       <c r="R186" s="15"/>
       <c r="S186" s="15"/>
-    </row>
-    <row r="187" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T186" s="15"/>
+    </row>
+    <row r="187" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A187" s="15"/>
       <c r="B187" s="15"/>
       <c r="C187" s="15"/>
@@ -6354,8 +6578,9 @@
       <c r="Q187" s="15"/>
       <c r="R187" s="15"/>
       <c r="S187" s="15"/>
-    </row>
-    <row r="188" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T187" s="15"/>
+    </row>
+    <row r="188" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A188" s="15"/>
       <c r="B188" s="15"/>
       <c r="C188" s="15"/>
@@ -6375,8 +6600,9 @@
       <c r="Q188" s="15"/>
       <c r="R188" s="15"/>
       <c r="S188" s="15"/>
-    </row>
-    <row r="189" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T188" s="15"/>
+    </row>
+    <row r="189" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A189" s="15"/>
       <c r="B189" s="15"/>
       <c r="C189" s="15"/>
@@ -6396,8 +6622,9 @@
       <c r="Q189" s="15"/>
       <c r="R189" s="15"/>
       <c r="S189" s="15"/>
-    </row>
-    <row r="190" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T189" s="15"/>
+    </row>
+    <row r="190" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A190" s="15"/>
       <c r="B190" s="15"/>
       <c r="C190" s="15"/>
@@ -6417,8 +6644,9 @@
       <c r="Q190" s="15"/>
       <c r="R190" s="15"/>
       <c r="S190" s="15"/>
-    </row>
-    <row r="191" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T190" s="15"/>
+    </row>
+    <row r="191" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A191" s="15"/>
       <c r="B191" s="15"/>
       <c r="C191" s="15"/>
@@ -6438,8 +6666,9 @@
       <c r="Q191" s="15"/>
       <c r="R191" s="15"/>
       <c r="S191" s="15"/>
-    </row>
-    <row r="192" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T191" s="15"/>
+    </row>
+    <row r="192" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A192" s="15"/>
       <c r="B192" s="15"/>
       <c r="C192" s="15"/>
@@ -6459,8 +6688,9 @@
       <c r="Q192" s="15"/>
       <c r="R192" s="15"/>
       <c r="S192" s="15"/>
-    </row>
-    <row r="193" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T192" s="15"/>
+    </row>
+    <row r="193" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A193" s="15"/>
       <c r="B193" s="15"/>
       <c r="C193" s="15"/>
@@ -6480,8 +6710,9 @@
       <c r="Q193" s="15"/>
       <c r="R193" s="15"/>
       <c r="S193" s="15"/>
-    </row>
-    <row r="194" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T193" s="15"/>
+    </row>
+    <row r="194" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A194" s="15"/>
       <c r="B194" s="15"/>
       <c r="C194" s="15"/>
@@ -6501,8 +6732,9 @@
       <c r="Q194" s="15"/>
       <c r="R194" s="15"/>
       <c r="S194" s="15"/>
-    </row>
-    <row r="195" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T194" s="15"/>
+    </row>
+    <row r="195" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A195" s="15"/>
       <c r="B195" s="15"/>
       <c r="C195" s="15"/>
@@ -6522,8 +6754,9 @@
       <c r="Q195" s="15"/>
       <c r="R195" s="15"/>
       <c r="S195" s="15"/>
-    </row>
-    <row r="196" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T195" s="15"/>
+    </row>
+    <row r="196" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A196" s="15"/>
       <c r="B196" s="15"/>
       <c r="C196" s="15"/>
@@ -6543,8 +6776,9 @@
       <c r="Q196" s="15"/>
       <c r="R196" s="15"/>
       <c r="S196" s="15"/>
-    </row>
-    <row r="197" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T196" s="15"/>
+    </row>
+    <row r="197" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A197" s="15"/>
       <c r="B197" s="15"/>
       <c r="C197" s="15"/>
@@ -6564,8 +6798,9 @@
       <c r="Q197" s="15"/>
       <c r="R197" s="15"/>
       <c r="S197" s="15"/>
-    </row>
-    <row r="198" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T197" s="15"/>
+    </row>
+    <row r="198" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A198" s="15"/>
       <c r="B198" s="15"/>
       <c r="C198" s="15"/>
@@ -6585,8 +6820,9 @@
       <c r="Q198" s="15"/>
       <c r="R198" s="15"/>
       <c r="S198" s="15"/>
-    </row>
-    <row r="199" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T198" s="15"/>
+    </row>
+    <row r="199" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A199" s="15"/>
       <c r="B199" s="15"/>
       <c r="C199" s="15"/>
@@ -6606,8 +6842,9 @@
       <c r="Q199" s="15"/>
       <c r="R199" s="15"/>
       <c r="S199" s="15"/>
-    </row>
-    <row r="200" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T199" s="15"/>
+    </row>
+    <row r="200" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A200" s="15"/>
       <c r="B200" s="15"/>
       <c r="C200" s="15"/>
@@ -6627,8 +6864,9 @@
       <c r="Q200" s="15"/>
       <c r="R200" s="15"/>
       <c r="S200" s="15"/>
-    </row>
-    <row r="201" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T200" s="15"/>
+    </row>
+    <row r="201" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A201" s="15"/>
       <c r="B201" s="15"/>
       <c r="C201" s="15"/>
@@ -6648,8 +6886,9 @@
       <c r="Q201" s="15"/>
       <c r="R201" s="15"/>
       <c r="S201" s="15"/>
-    </row>
-    <row r="202" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T201" s="15"/>
+    </row>
+    <row r="202" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A202" s="15"/>
       <c r="B202" s="15"/>
       <c r="C202" s="15"/>
@@ -6669,8 +6908,9 @@
       <c r="Q202" s="15"/>
       <c r="R202" s="15"/>
       <c r="S202" s="15"/>
-    </row>
-    <row r="203" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T202" s="15"/>
+    </row>
+    <row r="203" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A203" s="15"/>
       <c r="B203" s="15"/>
       <c r="C203" s="15"/>
@@ -6690,8 +6930,9 @@
       <c r="Q203" s="15"/>
       <c r="R203" s="15"/>
       <c r="S203" s="15"/>
-    </row>
-    <row r="204" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T203" s="15"/>
+    </row>
+    <row r="204" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A204" s="15"/>
       <c r="B204" s="15"/>
       <c r="C204" s="15"/>
@@ -6711,8 +6952,9 @@
       <c r="Q204" s="15"/>
       <c r="R204" s="15"/>
       <c r="S204" s="15"/>
-    </row>
-    <row r="205" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T204" s="15"/>
+    </row>
+    <row r="205" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A205" s="15"/>
       <c r="B205" s="15"/>
       <c r="C205" s="15"/>
@@ -6732,8 +6974,9 @@
       <c r="Q205" s="15"/>
       <c r="R205" s="15"/>
       <c r="S205" s="15"/>
-    </row>
-    <row r="206" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T205" s="15"/>
+    </row>
+    <row r="206" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A206" s="15"/>
       <c r="B206" s="15"/>
       <c r="C206" s="15"/>
@@ -6753,8 +6996,9 @@
       <c r="Q206" s="15"/>
       <c r="R206" s="15"/>
       <c r="S206" s="15"/>
-    </row>
-    <row r="207" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T206" s="15"/>
+    </row>
+    <row r="207" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A207" s="15"/>
       <c r="B207" s="15"/>
       <c r="C207" s="15"/>
@@ -6774,8 +7018,9 @@
       <c r="Q207" s="15"/>
       <c r="R207" s="15"/>
       <c r="S207" s="15"/>
-    </row>
-    <row r="208" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T207" s="15"/>
+    </row>
+    <row r="208" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A208" s="15"/>
       <c r="B208" s="15"/>
       <c r="C208" s="15"/>
@@ -6795,8 +7040,9 @@
       <c r="Q208" s="15"/>
       <c r="R208" s="15"/>
       <c r="S208" s="15"/>
-    </row>
-    <row r="209" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T208" s="15"/>
+    </row>
+    <row r="209" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A209" s="15"/>
       <c r="B209" s="15"/>
       <c r="C209" s="15"/>
@@ -6816,8 +7062,9 @@
       <c r="Q209" s="15"/>
       <c r="R209" s="15"/>
       <c r="S209" s="15"/>
-    </row>
-    <row r="210" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T209" s="15"/>
+    </row>
+    <row r="210" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A210" s="15"/>
       <c r="B210" s="15"/>
       <c r="C210" s="15"/>
@@ -6837,8 +7084,9 @@
       <c r="Q210" s="15"/>
       <c r="R210" s="15"/>
       <c r="S210" s="15"/>
-    </row>
-    <row r="211" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T210" s="15"/>
+    </row>
+    <row r="211" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A211" s="15"/>
       <c r="B211" s="15"/>
       <c r="C211" s="15"/>
@@ -6858,8 +7106,9 @@
       <c r="Q211" s="15"/>
       <c r="R211" s="15"/>
       <c r="S211" s="15"/>
-    </row>
-    <row r="212" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T211" s="15"/>
+    </row>
+    <row r="212" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A212" s="15"/>
       <c r="B212" s="15"/>
       <c r="C212" s="15"/>
@@ -6879,8 +7128,9 @@
       <c r="Q212" s="15"/>
       <c r="R212" s="15"/>
       <c r="S212" s="15"/>
-    </row>
-    <row r="213" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T212" s="15"/>
+    </row>
+    <row r="213" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A213" s="15"/>
       <c r="B213" s="15"/>
       <c r="C213" s="15"/>
@@ -6900,8 +7150,9 @@
       <c r="Q213" s="15"/>
       <c r="R213" s="15"/>
       <c r="S213" s="15"/>
-    </row>
-    <row r="214" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T213" s="15"/>
+    </row>
+    <row r="214" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A214" s="15"/>
       <c r="B214" s="15"/>
       <c r="C214" s="15"/>
@@ -6921,8 +7172,9 @@
       <c r="Q214" s="15"/>
       <c r="R214" s="15"/>
       <c r="S214" s="15"/>
-    </row>
-    <row r="215" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T214" s="15"/>
+    </row>
+    <row r="215" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A215" s="15"/>
       <c r="B215" s="15"/>
       <c r="C215" s="15"/>
@@ -6942,8 +7194,9 @@
       <c r="Q215" s="15"/>
       <c r="R215" s="15"/>
       <c r="S215" s="15"/>
-    </row>
-    <row r="216" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T215" s="15"/>
+    </row>
+    <row r="216" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A216" s="15"/>
       <c r="B216" s="15"/>
       <c r="C216" s="15"/>
@@ -6963,8 +7216,9 @@
       <c r="Q216" s="15"/>
       <c r="R216" s="15"/>
       <c r="S216" s="15"/>
-    </row>
-    <row r="217" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T216" s="15"/>
+    </row>
+    <row r="217" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A217" s="15"/>
       <c r="B217" s="15"/>
       <c r="C217" s="15"/>
@@ -6984,8 +7238,9 @@
       <c r="Q217" s="15"/>
       <c r="R217" s="15"/>
       <c r="S217" s="15"/>
-    </row>
-    <row r="218" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T217" s="15"/>
+    </row>
+    <row r="218" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A218" s="15"/>
       <c r="B218" s="15"/>
       <c r="C218" s="15"/>
@@ -7005,8 +7260,9 @@
       <c r="Q218" s="15"/>
       <c r="R218" s="15"/>
       <c r="S218" s="15"/>
-    </row>
-    <row r="219" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T218" s="15"/>
+    </row>
+    <row r="219" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A219" s="15"/>
       <c r="B219" s="15"/>
       <c r="C219" s="15"/>
@@ -7026,8 +7282,9 @@
       <c r="Q219" s="15"/>
       <c r="R219" s="15"/>
       <c r="S219" s="15"/>
-    </row>
-    <row r="220" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T219" s="15"/>
+    </row>
+    <row r="220" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A220" s="15"/>
       <c r="B220" s="15"/>
       <c r="C220" s="15"/>
@@ -7047,8 +7304,9 @@
       <c r="Q220" s="15"/>
       <c r="R220" s="15"/>
       <c r="S220" s="15"/>
-    </row>
-    <row r="221" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T220" s="15"/>
+    </row>
+    <row r="221" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A221" s="15"/>
       <c r="B221" s="15"/>
       <c r="C221" s="15"/>
@@ -7068,8 +7326,9 @@
       <c r="Q221" s="15"/>
       <c r="R221" s="15"/>
       <c r="S221" s="15"/>
-    </row>
-    <row r="222" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T221" s="15"/>
+    </row>
+    <row r="222" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A222" s="15"/>
       <c r="B222" s="15"/>
       <c r="C222" s="15"/>
@@ -7089,8 +7348,9 @@
       <c r="Q222" s="15"/>
       <c r="R222" s="15"/>
       <c r="S222" s="15"/>
-    </row>
-    <row r="223" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T222" s="15"/>
+    </row>
+    <row r="223" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A223" s="15"/>
       <c r="B223" s="15"/>
       <c r="C223" s="15"/>
@@ -7110,6 +7370,7 @@
       <c r="Q223" s="15"/>
       <c r="R223" s="15"/>
       <c r="S223" s="15"/>
+      <c r="T223" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -8779,10 +9040,10 @@
         <v>211</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C46" s="17" t="s">
-        <v>3</v>
+        <v>46</v>
       </c>
       <c r="D46" s="17" t="s">
         <v>115</v>
@@ -8809,7 +9070,7 @@
         <v>153</v>
       </c>
       <c r="R46" s="13" t="s">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="S46" s="15"/>
     </row>
@@ -8818,10 +9079,10 @@
         <v>212</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C47" s="17" t="s">
-        <v>3</v>
+        <v>46</v>
       </c>
       <c r="D47" s="17" t="s">
         <v>115</v>
@@ -8848,7 +9109,7 @@
         <v>153</v>
       </c>
       <c r="R47" s="13" t="s">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="S47" s="15"/>
     </row>
@@ -8857,10 +9118,10 @@
         <v>215</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C48" s="17" t="s">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="D48" s="17" t="s">
         <v>115</v>
@@ -8888,7 +9149,7 @@
       </c>
       <c r="R48" s="15"/>
       <c r="S48" s="13" t="s">
-        <v>47</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
@@ -8896,7 +9157,7 @@
         <v>216</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C49" s="13" t="s">
         <v>47</v>
@@ -8933,7 +9194,7 @@
         <v>217</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C50" s="13" t="s">
         <v>47</v>
@@ -8964,7 +9225,7 @@
       </c>
       <c r="R50" s="15"/>
       <c r="S50" s="13" t="s">
-        <v>47</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8972,10 +9233,10 @@
         <v>218</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="D51" s="15" t="s">
         <v>115</v>

</xml_diff>

<commit_message>
Added with iLPN format generate
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC7E3730-72B0-4155-9B8E-9019BB6143D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0D56BDB-C335-4F99-85EC-1AD9764E544B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -373,9 +373,6 @@
     <t>ItemReference</t>
   </si>
   <si>
-    <t>ST-G0-01-1-R</t>
-  </si>
-  <si>
     <t>MoveLPNQty</t>
   </si>
   <si>
@@ -1223,6 +1220,9 @@
   </si>
   <si>
     <t>831</t>
+  </si>
+  <si>
+    <t>ST-G0-0-1-R</t>
   </si>
 </sst>
 </file>
@@ -1770,7 +1770,7 @@
         <v>6</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D1" s="17" t="s">
         <v>117</v>
@@ -1782,78 +1782,78 @@
         <v>114</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J1" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="K1" s="17" t="s">
+        <v>277</v>
+      </c>
+      <c r="L1" s="17" t="s">
+        <v>279</v>
+      </c>
+      <c r="M1" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="K1" s="17" t="s">
-        <v>278</v>
-      </c>
-      <c r="L1" s="17" t="s">
-        <v>280</v>
-      </c>
-      <c r="M1" s="17" t="s">
+      <c r="N1" s="17" t="s">
         <v>156</v>
       </c>
-      <c r="N1" s="17" t="s">
+      <c r="O1" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="O1" s="17" t="s">
+      <c r="P1" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="P1" s="17" t="s">
-        <v>159</v>
-      </c>
       <c r="Q1" s="17" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="R1" s="17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="S1" s="17" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="T1" s="17" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="U1" s="22" t="s">
+        <v>343</v>
+      </c>
+      <c r="V1" s="22" t="s">
         <v>344</v>
       </c>
-      <c r="V1" s="22" t="s">
+      <c r="W1" s="22" t="s">
         <v>345</v>
       </c>
-      <c r="W1" s="22" t="s">
+      <c r="X1" s="22" t="s">
         <v>346</v>
       </c>
-      <c r="X1" s="22" t="s">
+      <c r="Y1" s="22" t="s">
         <v>347</v>
       </c>
-      <c r="Y1" s="22" t="s">
+      <c r="Z1" s="22" t="s">
         <v>348</v>
       </c>
-      <c r="Z1" s="22" t="s">
+      <c r="AA1" s="22" t="s">
         <v>349</v>
-      </c>
-      <c r="AA1" s="22" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="2" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D2" s="18" t="s">
         <v>0</v>
@@ -1886,13 +1886,13 @@
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B3" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D3" s="18" t="s">
         <v>0</v>
@@ -1904,13 +1904,13 @@
     </row>
     <row r="4" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>0</v>
@@ -1922,7 +1922,7 @@
       <c r="G4" s="14"/>
       <c r="H4" s="14"/>
       <c r="I4" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J4" s="14"/>
       <c r="K4" s="14"/>
@@ -1945,13 +1945,13 @@
     </row>
     <row r="5" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B5" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>85</v>
@@ -1963,7 +1963,7 @@
       <c r="G5" s="14"/>
       <c r="H5" s="14"/>
       <c r="I5" s="14" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="J5" s="14"/>
       <c r="K5" s="14"/>
@@ -1986,13 +1986,13 @@
     </row>
     <row r="6" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B6" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D6" s="18" t="s">
         <v>0</v>
@@ -2025,13 +2025,13 @@
     </row>
     <row r="7" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B7" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D7" s="18" t="s">
         <v>45</v>
@@ -2064,20 +2064,20 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D8" s="18" t="s">
         <v>46</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="15" t="s">
-        <v>118</v>
+        <v>401</v>
       </c>
       <c r="G8" s="15" t="s">
         <v>3</v>
@@ -2085,16 +2085,16 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B9" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E9" s="15"/>
       <c r="F9" s="14" t="s">
@@ -2102,18 +2102,18 @@
       </c>
       <c r="G9" s="15"/>
       <c r="I9" s="14" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B10" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D10" s="18" t="s">
         <v>49</v>
@@ -2124,18 +2124,18 @@
       </c>
       <c r="G10" s="15"/>
       <c r="I10" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B11" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D11" s="18" t="s">
         <v>51</v>
@@ -2147,7 +2147,7 @@
       <c r="G11" s="15"/>
       <c r="H11" s="14"/>
       <c r="I11" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J11" s="14"/>
       <c r="K11" s="14"/>
@@ -2170,13 +2170,13 @@
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B12" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D12" s="18" t="s">
         <v>3</v>
@@ -2186,18 +2186,18 @@
         <v>115</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B13" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D13" s="18" t="s">
         <v>52</v>
@@ -2207,54 +2207,54 @@
         <v>115</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B14" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D14" s="18" t="s">
         <v>53</v>
       </c>
       <c r="E14" s="15"/>
       <c r="I14" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B15" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D15" s="18" t="s">
         <v>54</v>
       </c>
       <c r="E15" s="15"/>
       <c r="I15" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B16" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D16" s="18" t="s">
         <v>55</v>
@@ -2264,18 +2264,18 @@
         <v>115</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B17" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D17" s="18" t="s">
         <v>56</v>
@@ -2285,18 +2285,18 @@
         <v>115</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B18" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D18" s="18" t="s">
         <v>57</v>
@@ -2306,18 +2306,18 @@
         <v>115</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D19" s="18" t="s">
         <v>58</v>
@@ -2327,18 +2327,18 @@
         <v>115</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D20" s="18" t="s">
         <v>59</v>
@@ -2347,18 +2347,18 @@
         <v>115</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D21" s="18" t="s">
         <v>60</v>
@@ -2367,18 +2367,18 @@
         <v>115</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D22" s="18" t="s">
         <v>61</v>
@@ -2387,18 +2387,18 @@
         <v>115</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D23" s="18" t="s">
         <v>62</v>
@@ -2407,18 +2407,18 @@
         <v>115</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B24" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D24" s="18" t="s">
         <v>63</v>
@@ -2427,18 +2427,18 @@
         <v>115</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B25" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D25" s="18" t="s">
         <v>64</v>
@@ -2447,18 +2447,18 @@
         <v>115</v>
       </c>
       <c r="I25" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D26" s="18" t="s">
         <v>65</v>
@@ -2467,18 +2467,18 @@
         <v>115</v>
       </c>
       <c r="I26" s="14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="27" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B27" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D27" s="18" t="s">
         <v>66</v>
@@ -2511,16 +2511,16 @@
     </row>
     <row r="28" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B28" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E28" s="14"/>
       <c r="F28" s="14" t="s">
@@ -2550,16 +2550,16 @@
     </row>
     <row r="29" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B29" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E29" s="14"/>
       <c r="F29" s="14" t="s">
@@ -2589,13 +2589,13 @@
     </row>
     <row r="30" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B30" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D30" s="18" t="s">
         <v>70</v>
@@ -2628,13 +2628,13 @@
     </row>
     <row r="31" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B31" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D31" s="18" t="s">
         <v>71</v>
@@ -2667,13 +2667,13 @@
     </row>
     <row r="32" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D32" s="18" t="s">
         <v>72</v>
@@ -2706,16 +2706,16 @@
     </row>
     <row r="33" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E33" s="14"/>
       <c r="F33" s="14" t="s">
@@ -2745,16 +2745,16 @@
     </row>
     <row r="34" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D34" s="18" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E34" s="14"/>
       <c r="F34" s="14" t="s">
@@ -2784,16 +2784,16 @@
     </row>
     <row r="35" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E35" s="14"/>
       <c r="F35" s="14" t="s">
@@ -2823,16 +2823,16 @@
     </row>
     <row r="36" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E36" s="14"/>
       <c r="F36" s="14" t="s">
@@ -2862,16 +2862,16 @@
     </row>
     <row r="37" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D37" s="18" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E37" s="14"/>
       <c r="F37" s="14" t="s">
@@ -2901,16 +2901,16 @@
     </row>
     <row r="38" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B38" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D38" s="18" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E38" s="14"/>
       <c r="F38" s="14" t="s">
@@ -2969,13 +2969,13 @@
     </row>
     <row r="40" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B40" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D40" s="23" t="s">
         <v>0</v>
@@ -3035,16 +3035,16 @@
     </row>
     <row r="42" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E42" s="14"/>
       <c r="F42" s="14"/>
@@ -3072,16 +3072,16 @@
     </row>
     <row r="43" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E43" s="14"/>
       <c r="F43" s="14"/>
@@ -3109,16 +3109,16 @@
     </row>
     <row r="44" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E44" s="14"/>
       <c r="F44" s="14"/>
@@ -3146,16 +3146,16 @@
     </row>
     <row r="45" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E45" s="14"/>
       <c r="F45" s="14"/>
@@ -3170,7 +3170,7 @@
       <c r="O45" s="14"/>
       <c r="P45" s="14"/>
       <c r="Q45" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="R45" s="14"/>
       <c r="S45" s="14"/>
@@ -3185,16 +3185,16 @@
     </row>
     <row r="46" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B46" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E46" s="14"/>
       <c r="F46" s="14"/>
@@ -3209,7 +3209,7 @@
       <c r="O46" s="14"/>
       <c r="P46" s="14"/>
       <c r="Q46" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="R46" s="14"/>
       <c r="S46" s="14"/>
@@ -3224,16 +3224,16 @@
     </row>
     <row r="47" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B47" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E47" s="14"/>
       <c r="F47" s="14"/>
@@ -3248,7 +3248,7 @@
       <c r="O47" s="14"/>
       <c r="P47" s="14"/>
       <c r="Q47" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R47" s="14"/>
       <c r="S47" s="14"/>
@@ -3263,16 +3263,16 @@
     </row>
     <row r="48" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B48" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E48" s="14"/>
       <c r="F48" s="14"/>
@@ -3287,7 +3287,7 @@
       <c r="O48" s="14"/>
       <c r="P48" s="14"/>
       <c r="Q48" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R48" s="14"/>
       <c r="S48" s="14"/>
@@ -3302,16 +3302,16 @@
     </row>
     <row r="49" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B49" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E49" s="14"/>
       <c r="F49" s="14"/>
@@ -3326,7 +3326,7 @@
       <c r="O49" s="14"/>
       <c r="P49" s="14"/>
       <c r="Q49" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="R49" s="14"/>
       <c r="S49" s="14"/>
@@ -3341,16 +3341,16 @@
     </row>
     <row r="50" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B50" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E50" s="14"/>
       <c r="F50" s="14"/>
@@ -3378,16 +3378,16 @@
     </row>
     <row r="51" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B51" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E51" s="14"/>
       <c r="F51" s="14"/>
@@ -3415,16 +3415,16 @@
     </row>
     <row r="52" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B52" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E52" s="14"/>
       <c r="F52" s="14"/>
@@ -3452,16 +3452,16 @@
     </row>
     <row r="53" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B53" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E53" s="14"/>
       <c r="F53" s="14"/>
@@ -3489,16 +3489,16 @@
     </row>
     <row r="54" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B54" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E54" s="14"/>
       <c r="F54" s="14"/>
@@ -3518,7 +3518,7 @@
         <v>0</v>
       </c>
       <c r="T54" s="14" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="U54" s="14"/>
       <c r="V54" s="14"/>
@@ -3530,16 +3530,16 @@
     </row>
     <row r="55" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B55" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D55" s="23" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E55" s="14"/>
       <c r="F55" s="14"/>
@@ -3559,7 +3559,7 @@
         <v>0</v>
       </c>
       <c r="T55" s="15" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="U55" s="14"/>
       <c r="V55" s="14"/>
@@ -3571,16 +3571,16 @@
     </row>
     <row r="56" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B56" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E56" s="14"/>
       <c r="F56" s="14"/>
@@ -3600,7 +3600,7 @@
         <v>0</v>
       </c>
       <c r="T56" s="24" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="U56" s="14"/>
       <c r="V56" s="14"/>
@@ -3612,16 +3612,16 @@
     </row>
     <row r="57" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B57" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D57" s="23" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E57" s="14"/>
       <c r="F57" s="14"/>
@@ -3636,14 +3636,14 @@
       <c r="O57" s="14"/>
       <c r="P57" s="14"/>
       <c r="Q57" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R57" s="14"/>
       <c r="S57" s="15" t="s">
         <v>0</v>
       </c>
       <c r="T57" s="14" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="U57" s="14"/>
       <c r="V57" s="14"/>
@@ -3655,16 +3655,16 @@
     </row>
     <row r="58" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B58" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D58" s="23" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E58" s="14"/>
       <c r="F58" s="14"/>
@@ -3679,14 +3679,14 @@
       <c r="O58" s="14"/>
       <c r="P58" s="14"/>
       <c r="Q58" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R58" s="14"/>
       <c r="S58" s="15" t="s">
         <v>0</v>
       </c>
       <c r="T58" s="14" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="U58" s="14"/>
       <c r="V58" s="14"/>
@@ -3698,16 +3698,16 @@
     </row>
     <row r="59" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B59" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D59" s="23" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E59" s="14"/>
       <c r="F59" s="14"/>
@@ -3722,7 +3722,7 @@
       <c r="O59" s="14"/>
       <c r="P59" s="14"/>
       <c r="Q59" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R59" s="14"/>
       <c r="S59" s="15" t="s">
@@ -3768,13 +3768,13 @@
     </row>
     <row r="61" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B61" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D61" s="18" t="s">
         <v>0</v>
@@ -3805,16 +3805,16 @@
     </row>
     <row r="62" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B62" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D62" s="18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E62" s="14"/>
       <c r="F62" s="14"/>
@@ -3842,13 +3842,13 @@
     </row>
     <row r="63" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B63" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D63" s="18" t="s">
         <v>0</v>
@@ -3860,7 +3860,7 @@
       <c r="G63" s="14"/>
       <c r="H63" s="14"/>
       <c r="I63" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J63" s="14"/>
       <c r="K63" s="14"/>
@@ -3883,16 +3883,16 @@
     </row>
     <row r="64" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B64" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D64" s="18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E64" s="14"/>
       <c r="F64" s="14" t="s">
@@ -3901,7 +3901,7 @@
       <c r="G64" s="14"/>
       <c r="H64" s="14"/>
       <c r="I64" s="14" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="J64" s="14"/>
       <c r="K64" s="14"/>
@@ -3924,16 +3924,16 @@
     </row>
     <row r="65" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B65" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D65" s="25" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E65" s="14"/>
       <c r="F65" s="14"/>
@@ -3961,16 +3961,16 @@
     </row>
     <row r="66" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B66" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D66" s="18" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E66" s="14"/>
       <c r="F66" s="14"/>
@@ -3998,16 +3998,16 @@
     </row>
     <row r="67" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B67" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D67" s="25" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E67" s="14"/>
       <c r="F67" s="14"/>
@@ -4035,16 +4035,16 @@
     </row>
     <row r="68" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B68" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D68" s="18" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E68" s="14"/>
       <c r="F68" s="14"/>
@@ -4072,13 +4072,13 @@
     </row>
     <row r="69" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="14" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B69" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D69" s="18"/>
       <c r="E69" s="14"/>
@@ -4136,13 +4136,13 @@
     </row>
     <row r="71" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="12" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B71" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D71" s="18"/>
       <c r="E71" s="14"/>
@@ -4151,13 +4151,13 @@
       <c r="H71" s="14"/>
       <c r="I71" s="14"/>
       <c r="J71" s="13" t="s">
+        <v>381</v>
+      </c>
+      <c r="K71" s="15" t="s">
+        <v>278</v>
+      </c>
+      <c r="L71" s="14" t="s">
         <v>382</v>
-      </c>
-      <c r="K71" s="15" t="s">
-        <v>279</v>
-      </c>
-      <c r="L71" s="14" t="s">
-        <v>383</v>
       </c>
       <c r="M71" s="14"/>
       <c r="N71" s="14"/>
@@ -4177,13 +4177,13 @@
     </row>
     <row r="72" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="12" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B72" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D72" s="18"/>
       <c r="E72" s="14"/>
@@ -4195,7 +4195,7 @@
       <c r="K72" s="14"/>
       <c r="L72" s="12"/>
       <c r="M72" s="12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="N72" s="12"/>
       <c r="O72" s="12"/>
@@ -4214,13 +4214,13 @@
     </row>
     <row r="73" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="12" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B73" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D73" s="18"/>
       <c r="E73" s="14"/>
@@ -4233,7 +4233,7 @@
       <c r="L73" s="12"/>
       <c r="M73" s="12"/>
       <c r="N73" s="12" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O73" s="12"/>
       <c r="P73" s="12"/>
@@ -4251,13 +4251,13 @@
     </row>
     <row r="74" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="12" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B74" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C74" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D74" s="18"/>
       <c r="E74" s="14"/>
@@ -4271,7 +4271,7 @@
       <c r="M74" s="12"/>
       <c r="N74" s="12"/>
       <c r="O74" s="12" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="P74" s="12"/>
       <c r="Q74" s="14"/>
@@ -4288,13 +4288,13 @@
     </row>
     <row r="75" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="12" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B75" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C75" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D75" s="18"/>
       <c r="E75" s="14"/>
@@ -4309,7 +4309,7 @@
       <c r="N75" s="12"/>
       <c r="O75" s="12"/>
       <c r="P75" s="13" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="Q75" s="14"/>
       <c r="R75" s="14"/>
@@ -4354,13 +4354,13 @@
     </row>
     <row r="77" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="12" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B77" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D77" s="12"/>
       <c r="E77" s="12"/>
@@ -4380,36 +4380,36 @@
       <c r="S77" s="12"/>
       <c r="T77" s="12"/>
       <c r="U77" s="13" t="s">
+        <v>315</v>
+      </c>
+      <c r="V77" s="13" t="s">
         <v>316</v>
       </c>
-      <c r="V77" s="13" t="s">
+      <c r="W77" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="W77" s="12" t="s">
+      <c r="X77" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="X77" s="12" t="s">
+      <c r="Y77" s="12" t="s">
         <v>319</v>
-      </c>
-      <c r="Y77" s="12" t="s">
-        <v>320</v>
       </c>
       <c r="Z77" s="12" t="s">
         <v>108</v>
       </c>
       <c r="AA77" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="78" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="12" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B78" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C78" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D78" s="12"/>
       <c r="E78" s="12"/>
@@ -4429,36 +4429,36 @@
       <c r="S78" s="12"/>
       <c r="T78" s="12"/>
       <c r="U78" s="13" t="s">
+        <v>315</v>
+      </c>
+      <c r="V78" s="13" t="s">
         <v>316</v>
       </c>
-      <c r="V78" s="13" t="s">
+      <c r="W78" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="W78" s="12" t="s">
+      <c r="X78" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="X78" s="12" t="s">
+      <c r="Y78" s="12" t="s">
         <v>319</v>
-      </c>
-      <c r="Y78" s="12" t="s">
-        <v>320</v>
       </c>
       <c r="Z78" s="12" t="s">
         <v>108</v>
       </c>
       <c r="AA78" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="79" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="12" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B79" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D79" s="12"/>
       <c r="E79" s="12"/>
@@ -4478,34 +4478,34 @@
       <c r="S79" s="12"/>
       <c r="T79" s="12"/>
       <c r="U79" s="12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="V79" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="W79" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="X79" s="12" t="s">
         <v>323</v>
       </c>
-      <c r="W79" s="12" t="s">
-        <v>318</v>
-      </c>
-      <c r="X79" s="12" t="s">
-        <v>324</v>
-      </c>
       <c r="Y79" s="12" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="Z79" s="12"/>
       <c r="AA79" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="80" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="12" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B80" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C80" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D80" s="12"/>
       <c r="E80" s="12"/>
@@ -4525,19 +4525,19 @@
       <c r="S80" s="12"/>
       <c r="T80" s="12"/>
       <c r="U80" s="13" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="V80" s="13" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="W80" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="X80" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="X80" s="12" t="s">
+      <c r="Y80" s="12" t="s">
         <v>319</v>
-      </c>
-      <c r="Y80" s="12" t="s">
-        <v>320</v>
       </c>
       <c r="Z80" s="12" t="s">
         <v>108</v>
@@ -4546,13 +4546,13 @@
     </row>
     <row r="81" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="12" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B81" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D81" s="12"/>
       <c r="E81" s="12"/>
@@ -4572,34 +4572,34 @@
       <c r="S81" s="12"/>
       <c r="T81" s="12"/>
       <c r="U81" s="12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="V81" s="12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="W81" s="12" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="X81" s="12"/>
       <c r="Y81" s="12" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="Z81" s="12" t="s">
         <v>108</v>
       </c>
       <c r="AA81" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="82" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="12" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B82" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C82" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D82" s="12"/>
       <c r="E82" s="12"/>
@@ -4620,33 +4620,33 @@
       <c r="T82" s="12"/>
       <c r="U82" s="12"/>
       <c r="V82" s="12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="W82" s="12" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="X82" s="12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="Y82" s="12" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="Z82" s="12" t="s">
         <v>108</v>
       </c>
       <c r="AA82" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="83" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B83" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C83" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D83" s="12"/>
       <c r="E83" s="12"/>
@@ -4666,36 +4666,36 @@
       <c r="S83" s="12"/>
       <c r="T83" s="12"/>
       <c r="U83" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="V83" s="13" t="s">
         <v>331</v>
       </c>
-      <c r="V83" s="13" t="s">
-        <v>332</v>
-      </c>
       <c r="W83" s="13" t="s">
+        <v>317</v>
+      </c>
+      <c r="X83" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="X83" s="12" t="s">
+      <c r="Y83" s="12" t="s">
         <v>319</v>
-      </c>
-      <c r="Y83" s="12" t="s">
-        <v>320</v>
       </c>
       <c r="Z83" s="12" t="s">
         <v>108</v>
       </c>
       <c r="AA83" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="84" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="12" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B84" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C84" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D84" s="12"/>
       <c r="E84" s="12"/>
@@ -4715,36 +4715,36 @@
       <c r="S84" s="12"/>
       <c r="T84" s="12"/>
       <c r="U84" s="13" t="s">
+        <v>315</v>
+      </c>
+      <c r="V84" s="13" t="s">
         <v>316</v>
       </c>
-      <c r="V84" s="13" t="s">
-        <v>317</v>
-      </c>
       <c r="W84" s="13" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="X84" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="Y84" s="12" t="s">
         <v>319</v>
-      </c>
-      <c r="Y84" s="12" t="s">
-        <v>320</v>
       </c>
       <c r="Z84" s="12" t="s">
         <v>108</v>
       </c>
       <c r="AA84" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="85" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="12" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B85" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C85" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D85" s="12"/>
       <c r="E85" s="12"/>
@@ -4764,36 +4764,36 @@
       <c r="S85" s="12"/>
       <c r="T85" s="12"/>
       <c r="U85" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="V85" s="12" t="s">
         <v>316</v>
       </c>
-      <c r="V85" s="12" t="s">
+      <c r="W85" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="W85" s="12" t="s">
-        <v>318</v>
-      </c>
       <c r="X85" s="12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="Y85" s="12" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="Z85" s="12" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AA85" s="12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="86" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="12" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B86" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C86" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D86" s="12"/>
       <c r="E86" s="12"/>
@@ -4813,36 +4813,36 @@
       <c r="S86" s="12"/>
       <c r="T86" s="12"/>
       <c r="U86" s="12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="V86" s="13" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="W86" s="12" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="X86" s="12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="Y86" s="12" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="Z86" s="12" t="s">
         <v>108</v>
       </c>
       <c r="AA86" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="87" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="12" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B87" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C87" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D87" s="12"/>
       <c r="E87" s="12"/>
@@ -4862,36 +4862,36 @@
       <c r="S87" s="12"/>
       <c r="T87" s="12"/>
       <c r="U87" s="12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="V87" s="12" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="W87" s="12" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="X87" s="12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="Y87" s="12" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="Z87" s="12" t="s">
         <v>108</v>
       </c>
       <c r="AA87" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="88" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="12" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B88" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C88" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D88" s="12"/>
       <c r="E88" s="12"/>
@@ -4911,36 +4911,36 @@
       <c r="S88" s="12"/>
       <c r="T88" s="12"/>
       <c r="U88" s="12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="V88" s="12" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="W88" s="12" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="X88" s="12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="Y88" s="12" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="Z88" s="12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="AA88" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="89" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="12" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B89" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D89" s="12"/>
       <c r="E89" s="12"/>
@@ -4960,25 +4960,25 @@
       <c r="S89" s="12"/>
       <c r="T89" s="12"/>
       <c r="U89" s="12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="V89" s="12" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="W89" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="X89" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="X89" s="12" t="s">
+      <c r="Y89" s="12" t="s">
         <v>319</v>
-      </c>
-      <c r="Y89" s="12" t="s">
-        <v>320</v>
       </c>
       <c r="Z89" s="12" t="s">
         <v>108</v>
       </c>
       <c r="AA89" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="90" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -5041,16 +5041,16 @@
     </row>
     <row r="92" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A92" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B92" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C92" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D92" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F92" s="14" t="s">
         <v>115</v>
@@ -5061,16 +5061,16 @@
     </row>
     <row r="93" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A93" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B93" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C93" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D93" s="15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F93" s="14" t="s">
         <v>115</v>
@@ -5081,16 +5081,16 @@
     </row>
     <row r="94" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A94" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B94" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C94" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D94" s="15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F94" s="14" t="s">
         <v>115</v>
@@ -5101,16 +5101,16 @@
     </row>
     <row r="95" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A95" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B95" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C95" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D95" s="15" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F95" s="14" t="s">
         <v>115</v>
@@ -5121,16 +5121,16 @@
     </row>
     <row r="96" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A96" s="14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B96" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C96" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D96" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F96" s="14" t="s">
         <v>115</v>
@@ -5141,16 +5141,16 @@
     </row>
     <row r="97" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A97" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B97" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C97" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D97" s="15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F97" s="14" t="s">
         <v>115</v>
@@ -5161,16 +5161,16 @@
     </row>
     <row r="98" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A98" s="14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B98" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C98" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D98" s="15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F98" s="14" t="s">
         <v>115</v>
@@ -5181,16 +5181,16 @@
     </row>
     <row r="99" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B99" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C99" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D99" s="15" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E99" s="14"/>
       <c r="F99" s="14" t="s">
@@ -5220,16 +5220,16 @@
     </row>
     <row r="100" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B100" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C100" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D100" s="15" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E100" s="14"/>
       <c r="F100" s="14" t="s">
@@ -5259,16 +5259,16 @@
     </row>
     <row r="101" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A101" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B101" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C101" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D101" s="15" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F101" s="14" t="s">
         <v>115</v>
@@ -5277,16 +5277,16 @@
     </row>
     <row r="102" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A102" s="14" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B102" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C102" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D102" s="15" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F102" s="14" t="s">
         <v>115</v>
@@ -5295,16 +5295,16 @@
     </row>
     <row r="103" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A103" s="14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B103" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C103" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D103" s="15" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F103" s="14" t="s">
         <v>115</v>
@@ -5313,16 +5313,16 @@
     </row>
     <row r="104" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A104" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B104" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C104" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D104" s="16" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F104" s="14" t="s">
         <v>115</v>
@@ -5333,16 +5333,16 @@
     </row>
     <row r="105" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A105" s="14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B105" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C105" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D105" s="15" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F105" s="14" t="s">
         <v>115</v>
@@ -5353,16 +5353,16 @@
     </row>
     <row r="106" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="B106" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="C106" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D106" s="15" t="s">
         <v>287</v>
-      </c>
-      <c r="B106" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="C106" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="D106" s="15" t="s">
-        <v>288</v>
       </c>
       <c r="E106" s="14"/>
       <c r="F106" s="14" t="s">
@@ -5394,16 +5394,16 @@
     </row>
     <row r="107" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="14" t="s">
+        <v>293</v>
+      </c>
+      <c r="B107" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="C107" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D107" s="15" t="s">
         <v>294</v>
-      </c>
-      <c r="B107" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="C107" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="D107" s="15" t="s">
-        <v>295</v>
       </c>
       <c r="E107" s="14"/>
       <c r="F107" s="14" t="s">
@@ -5435,16 +5435,16 @@
     </row>
     <row r="108" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="14" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B108" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C108" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D108" s="15" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E108" s="14"/>
       <c r="F108" s="14" t="s">
@@ -5476,16 +5476,16 @@
     </row>
     <row r="109" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="B109" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="C109" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D109" s="15" t="s">
         <v>297</v>
-      </c>
-      <c r="B109" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="C109" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="D109" s="15" t="s">
-        <v>298</v>
       </c>
       <c r="E109" s="14"/>
       <c r="F109" s="14" t="s">
@@ -5517,16 +5517,16 @@
     </row>
     <row r="110" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="14" t="s">
+        <v>300</v>
+      </c>
+      <c r="B110" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="C110" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D110" s="15" t="s">
         <v>301</v>
-      </c>
-      <c r="B110" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="C110" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="D110" s="15" t="s">
-        <v>302</v>
       </c>
       <c r="E110" s="14"/>
       <c r="F110" s="14" t="s">
@@ -5558,16 +5558,16 @@
     </row>
     <row r="111" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="B111" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="C111" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D111" s="15" t="s">
         <v>303</v>
-      </c>
-      <c r="B111" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="C111" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="D111" s="15" t="s">
-        <v>304</v>
       </c>
       <c r="E111" s="14"/>
       <c r="F111" s="14" t="s">
@@ -5599,16 +5599,16 @@
     </row>
     <row r="112" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="14" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B112" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C112" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D112" s="15" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E112" s="14"/>
       <c r="F112" s="14" t="s">
@@ -5617,7 +5617,7 @@
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
       <c r="I112" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J112" s="14"/>
       <c r="K112" s="14"/>
@@ -5640,16 +5640,16 @@
     </row>
     <row r="113" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="14" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B113" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C113" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D113" s="15" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E113" s="14"/>
       <c r="F113" s="14" t="s">
@@ -5658,7 +5658,7 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="14" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="J113" s="14"/>
       <c r="K113" s="14"/>
@@ -5681,16 +5681,16 @@
     </row>
     <row r="114" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="14" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B114" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C114" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D114" s="15" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="E114" s="14"/>
       <c r="F114" s="14" t="s">
@@ -5699,7 +5699,7 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J114" s="14"/>
       <c r="K114" s="14"/>
@@ -5722,16 +5722,16 @@
     </row>
     <row r="115" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="14" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B115" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C115" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D115" s="15" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="E115" s="14"/>
       <c r="F115" s="14" t="s">
@@ -5740,7 +5740,7 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="14" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="J115" s="14"/>
       <c r="K115" s="14"/>
@@ -5879,13 +5879,13 @@
     </row>
     <row r="121" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="14" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B121" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C121" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D121" s="14"/>
       <c r="E121" s="14"/>
@@ -5894,13 +5894,13 @@
       <c r="H121" s="14"/>
       <c r="I121" s="14"/>
       <c r="J121" s="15" t="s">
+        <v>281</v>
+      </c>
+      <c r="K121" s="15" t="s">
         <v>282</v>
       </c>
-      <c r="K121" s="15" t="s">
+      <c r="L121" s="15" t="s">
         <v>283</v>
-      </c>
-      <c r="L121" s="15" t="s">
-        <v>284</v>
       </c>
       <c r="M121" s="14"/>
       <c r="N121" s="14"/>
@@ -5920,13 +5920,13 @@
     </row>
     <row r="122" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="14" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B122" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C122" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D122" s="14"/>
       <c r="E122" s="14"/>
@@ -5935,13 +5935,13 @@
       <c r="H122" s="14"/>
       <c r="I122" s="14"/>
       <c r="J122" s="15" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K122" s="15" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="L122" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="M122" s="14"/>
       <c r="N122" s="14"/>
@@ -5961,58 +5961,58 @@
     </row>
     <row r="123" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A123" s="14" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B123" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C123" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O123" s="15" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="124" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A124" s="14" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B124" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C124" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O124" s="15" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="125" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A125" s="14" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B125" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C125" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O125" s="15" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="126" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A126" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="B126" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="C126" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="M126" s="14" t="s">
         <v>384</v>
-      </c>
-      <c r="B126" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="C126" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="M126" s="14" t="s">
-        <v>385</v>
       </c>
     </row>
   </sheetData>
@@ -6064,7 +6064,7 @@
         <v>111</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G1" s="17" t="s">
         <v>112</v>
@@ -6073,37 +6073,37 @@
         <v>114</v>
       </c>
       <c r="I1" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="J1" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="K1" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="J1" s="17" t="s">
-        <v>139</v>
-      </c>
-      <c r="K1" s="17" t="s">
-        <v>123</v>
-      </c>
       <c r="L1" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="M1" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="M1" s="17" t="s">
-        <v>133</v>
-      </c>
       <c r="N1" s="17" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="O1" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="P1" s="17" t="s">
         <v>146</v>
       </c>
-      <c r="P1" s="17" t="s">
+      <c r="Q1" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="Q1" s="17" t="s">
-        <v>148</v>
-      </c>
       <c r="R1" s="17" t="s">
+        <v>205</v>
+      </c>
+      <c r="S1" s="17" t="s">
         <v>206</v>
-      </c>
-      <c r="S1" s="17" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
@@ -6111,7 +6111,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C2" s="15" t="s">
         <v>61</v>
@@ -6151,7 +6151,7 @@
         <v>45</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>3</v>
@@ -6173,7 +6173,7 @@
         <v>46</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C5" s="15" t="s">
         <v>80</v>
@@ -6197,7 +6197,7 @@
         <v>47</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C6" s="15" t="s">
         <v>3</v>
@@ -6219,7 +6219,7 @@
         <v>48</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>61</v>
@@ -6241,7 +6241,7 @@
         <v>49</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C8" s="15"/>
       <c r="E8" s="15" t="s">
@@ -6253,10 +6253,10 @@
         <v>115</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K8" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
@@ -6264,7 +6264,7 @@
         <v>50</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>3</v>
@@ -6281,10 +6281,10 @@
         <v>115</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -6292,10 +6292,10 @@
         <v>51</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>113</v>
@@ -6309,10 +6309,10 @@
         <v>115</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K10" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
@@ -6320,7 +6320,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C11" s="15" t="s">
         <v>3</v>
@@ -6342,7 +6342,7 @@
         <v>52</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C12" s="15" t="s">
         <v>3</v>
@@ -6359,10 +6359,10 @@
         <v>115</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K12" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
@@ -6370,7 +6370,7 @@
         <v>53</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C13" s="15"/>
       <c r="E13" s="15" t="s">
@@ -6379,7 +6379,7 @@
       <c r="F13" s="15"/>
       <c r="G13" s="15"/>
       <c r="J13" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -6387,7 +6387,7 @@
         <v>54</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C14" s="15" t="s">
         <v>3</v>
@@ -6404,11 +6404,11 @@
         <v>115</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J14" s="14"/>
       <c r="K14" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L14" s="14"/>
       <c r="M14" s="14"/>
@@ -6424,7 +6424,7 @@
         <v>55</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>61</v>
@@ -6443,7 +6443,7 @@
         <v>66</v>
       </c>
       <c r="M15" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
@@ -6451,7 +6451,7 @@
         <v>56</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>61</v>
@@ -6470,7 +6470,7 @@
         <v>56</v>
       </c>
       <c r="M16" s="14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
@@ -6478,7 +6478,7 @@
         <v>57</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>61</v>
@@ -6497,7 +6497,7 @@
         <v>66</v>
       </c>
       <c r="M17" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
@@ -6505,7 +6505,7 @@
         <v>58</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>61</v>
@@ -6524,7 +6524,7 @@
         <v>56</v>
       </c>
       <c r="M18" s="14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
@@ -6532,7 +6532,7 @@
         <v>59</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>61</v>
@@ -6548,7 +6548,7 @@
         <v>115</v>
       </c>
       <c r="M19" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>60</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>61</v>
@@ -6572,7 +6572,7 @@
         <v>115</v>
       </c>
       <c r="M20" s="14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
@@ -6580,7 +6580,7 @@
         <v>61</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C21" s="15" t="s">
         <v>61</v>
@@ -6597,7 +6597,7 @@
         <v>115</v>
       </c>
       <c r="N21" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="22" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -6605,7 +6605,7 @@
         <v>62</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C22" s="15"/>
       <c r="D22" s="14"/>
@@ -6617,13 +6617,13 @@
       <c r="H22" s="14"/>
       <c r="I22" s="14"/>
       <c r="J22" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K22" s="14"/>
       <c r="L22" s="14"/>
       <c r="M22" s="14"/>
       <c r="N22" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="O22" s="14"/>
       <c r="P22" s="14"/>
@@ -6636,10 +6636,10 @@
         <v>63</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>113</v>
@@ -6653,11 +6653,11 @@
         <v>115</v>
       </c>
       <c r="I23" s="19" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J23" s="19"/>
       <c r="K23" s="19" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
@@ -6665,7 +6665,7 @@
         <v>64</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>3</v>
@@ -6687,7 +6687,7 @@
         <v>65</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C25" s="15" t="s">
         <v>3</v>
@@ -6704,11 +6704,11 @@
         <v>115</v>
       </c>
       <c r="I25" s="19" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J25" s="19"/>
       <c r="K25" s="19" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -6716,7 +6716,7 @@
         <v>66</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>3</v>
@@ -6749,7 +6749,7 @@
         <v>67</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>3</v>
@@ -6782,7 +6782,7 @@
         <v>68</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>3</v>
@@ -6815,7 +6815,7 @@
         <v>69</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>3</v>
@@ -6848,7 +6848,7 @@
         <v>36</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C30" s="15" t="s">
         <v>47</v>
@@ -6881,7 +6881,7 @@
         <v>70</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C31" s="15" t="s">
         <v>3</v>
@@ -6914,7 +6914,7 @@
         <v>71</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C32" s="15" t="s">
         <v>3</v>
@@ -6947,7 +6947,7 @@
         <v>72</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C33" s="15" t="s">
         <v>3</v>
@@ -6980,7 +6980,7 @@
         <v>73</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C34" s="15" t="s">
         <v>3</v>
@@ -7013,7 +7013,7 @@
         <v>74</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C35" s="15" t="s">
         <v>3</v>
@@ -7046,7 +7046,7 @@
         <v>75</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C36" s="15" t="s">
         <v>3</v>
@@ -7079,7 +7079,7 @@
         <v>76</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>3</v>
@@ -7112,7 +7112,7 @@
         <v>77</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C38" s="15" t="s">
         <v>3</v>
@@ -7145,7 +7145,7 @@
         <v>78</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C39" s="15" t="s">
         <v>3</v>
@@ -7178,7 +7178,7 @@
         <v>79</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C40" s="15" t="s">
         <v>3</v>
@@ -7211,7 +7211,7 @@
         <v>80</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C41" s="15" t="s">
         <v>47</v>
@@ -7244,7 +7244,7 @@
         <v>81</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C42" s="15" t="s">
         <v>3</v>
@@ -7277,7 +7277,7 @@
         <v>82</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C43" s="15" t="s">
         <v>3</v>
@@ -7310,7 +7310,7 @@
         <v>83</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C44" s="15" t="s">
         <v>3</v>
@@ -7319,7 +7319,7 @@
         <v>113</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F44" s="15"/>
       <c r="G44" s="15"/>
@@ -7343,7 +7343,7 @@
         <v>84</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C45" s="15" t="s">
         <v>47</v>
@@ -7376,7 +7376,7 @@
         <v>85</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C46" s="15" t="s">
         <v>47</v>
@@ -7408,10 +7408,10 @@
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A47" s="16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C47" s="16" t="s">
         <v>0</v>
@@ -7420,24 +7420,24 @@
         <v>113</v>
       </c>
       <c r="J47" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O47" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P47" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q47" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="48" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C48" s="16" t="s">
         <v>0</v>
@@ -7451,30 +7451,30 @@
       <c r="H48" s="14"/>
       <c r="I48" s="14"/>
       <c r="J48" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K48" s="14"/>
       <c r="L48" s="14"/>
       <c r="M48" s="14"/>
       <c r="N48" s="14"/>
       <c r="O48" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P48" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q48" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R48" s="14"/>
       <c r="S48" s="14"/>
     </row>
     <row r="49" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>0</v>
@@ -7488,33 +7488,33 @@
       <c r="H49" s="14"/>
       <c r="I49" s="14"/>
       <c r="J49" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K49" s="14"/>
       <c r="L49" s="14"/>
       <c r="M49" s="14"/>
       <c r="N49" s="14"/>
       <c r="O49" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P49" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q49" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R49" s="14"/>
       <c r="S49" s="14"/>
     </row>
     <row r="50" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D50" s="16" t="s">
         <v>113</v>
@@ -7525,30 +7525,30 @@
       <c r="H50" s="14"/>
       <c r="I50" s="14"/>
       <c r="J50" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K50" s="14"/>
       <c r="L50" s="14"/>
       <c r="M50" s="14"/>
       <c r="N50" s="14"/>
       <c r="O50" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P50" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q50" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R50" s="14"/>
       <c r="S50" s="14"/>
     </row>
     <row r="51" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C51" s="16" t="s">
         <v>2</v>
@@ -7562,30 +7562,30 @@
       <c r="H51" s="14"/>
       <c r="I51" s="14"/>
       <c r="J51" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K51" s="14"/>
       <c r="L51" s="14"/>
       <c r="M51" s="14"/>
       <c r="N51" s="14"/>
       <c r="O51" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P51" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q51" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R51" s="14"/>
       <c r="S51" s="14"/>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="16" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C52" s="16" t="s">
         <v>2</v>
@@ -7594,24 +7594,24 @@
         <v>113</v>
       </c>
       <c r="J52" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O52" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P52" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q52" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="53" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C53" s="16" t="s">
         <v>2</v>
@@ -7625,30 +7625,30 @@
       <c r="H53" s="14"/>
       <c r="I53" s="14"/>
       <c r="J53" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K53" s="14"/>
       <c r="L53" s="14"/>
       <c r="M53" s="14"/>
       <c r="N53" s="14"/>
       <c r="O53" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P53" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q53" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R53" s="14"/>
       <c r="S53" s="14"/>
     </row>
     <row r="54" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="16" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C54" s="16" t="s">
         <v>2</v>
@@ -7662,30 +7662,30 @@
       <c r="H54" s="14"/>
       <c r="I54" s="14"/>
       <c r="J54" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K54" s="14"/>
       <c r="L54" s="14"/>
       <c r="M54" s="14"/>
       <c r="N54" s="14"/>
       <c r="O54" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P54" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q54" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R54" s="14"/>
       <c r="S54" s="14"/>
     </row>
     <row r="55" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C55" s="16" t="s">
         <v>46</v>
@@ -7699,20 +7699,20 @@
       <c r="H55" s="14"/>
       <c r="I55" s="14"/>
       <c r="J55" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K55" s="14"/>
       <c r="L55" s="14"/>
       <c r="M55" s="14"/>
       <c r="N55" s="14"/>
       <c r="O55" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P55" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q55" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R55" s="15" t="s">
         <v>2</v>
@@ -7721,10 +7721,10 @@
     </row>
     <row r="56" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="16" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C56" s="16" t="s">
         <v>46</v>
@@ -7738,20 +7738,20 @@
       <c r="H56" s="14"/>
       <c r="I56" s="14"/>
       <c r="J56" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K56" s="14"/>
       <c r="L56" s="14"/>
       <c r="M56" s="14"/>
       <c r="N56" s="14"/>
       <c r="O56" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P56" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q56" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R56" s="15" t="s">
         <v>2</v>
@@ -7760,10 +7760,10 @@
     </row>
     <row r="57" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B57" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C57" s="16" t="s">
         <v>47</v>
@@ -7777,20 +7777,20 @@
       <c r="H57" s="14"/>
       <c r="I57" s="14"/>
       <c r="J57" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K57" s="14"/>
       <c r="L57" s="14"/>
       <c r="M57" s="14"/>
       <c r="N57" s="14"/>
       <c r="O57" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P57" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q57" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R57" s="14"/>
       <c r="S57" s="15" t="s">
@@ -7799,10 +7799,10 @@
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58" s="16" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B58" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C58" s="15" t="s">
         <v>47</v>
@@ -7811,24 +7811,24 @@
         <v>113</v>
       </c>
       <c r="J58" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O58" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P58" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q58" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="59" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B59" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C59" s="15" t="s">
         <v>47</v>
@@ -7842,20 +7842,20 @@
       <c r="H59" s="14"/>
       <c r="I59" s="14"/>
       <c r="J59" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K59" s="14"/>
       <c r="L59" s="14"/>
       <c r="M59" s="14"/>
       <c r="N59" s="14"/>
       <c r="O59" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P59" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q59" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R59" s="14"/>
       <c r="S59" s="15" t="s">
@@ -7864,10 +7864,10 @@
     </row>
     <row r="60" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C60" s="15" t="s">
         <v>47</v>
@@ -7881,30 +7881,30 @@
       <c r="H60" s="14"/>
       <c r="I60" s="14"/>
       <c r="J60" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K60" s="14"/>
       <c r="L60" s="14"/>
       <c r="M60" s="14"/>
       <c r="N60" s="14"/>
       <c r="O60" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P60" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q60" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R60" s="14"/>
       <c r="S60" s="14"/>
     </row>
     <row r="61" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="16" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C61" s="15" t="s">
         <v>0</v>
@@ -7930,10 +7930,10 @@
     </row>
     <row r="62" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="16" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B62" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C62" s="15" t="s">
         <v>0</v>
@@ -7947,30 +7947,30 @@
       <c r="H62" s="14"/>
       <c r="I62" s="14"/>
       <c r="J62" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K62" s="14"/>
       <c r="L62" s="14"/>
       <c r="M62" s="14"/>
       <c r="N62" s="14"/>
       <c r="O62" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P62" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q62" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R62" s="14"/>
       <c r="S62" s="14"/>
     </row>
     <row r="63" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="16" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B63" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C63" s="15" t="s">
         <v>0</v>
@@ -7984,30 +7984,30 @@
       <c r="H63" s="14"/>
       <c r="I63" s="14"/>
       <c r="J63" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K63" s="14"/>
       <c r="L63" s="14"/>
       <c r="M63" s="14"/>
       <c r="N63" s="14"/>
       <c r="O63" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P63" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q63" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R63" s="14"/>
       <c r="S63" s="14"/>
     </row>
     <row r="64" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="16" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B64" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C64" s="16" t="s">
         <v>0</v>
@@ -8021,30 +8021,30 @@
       <c r="H64" s="14"/>
       <c r="I64" s="14"/>
       <c r="J64" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K64" s="14"/>
       <c r="L64" s="14"/>
       <c r="M64" s="14"/>
       <c r="N64" s="14"/>
       <c r="O64" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P64" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q64" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R64" s="14"/>
       <c r="S64" s="14"/>
     </row>
     <row r="65" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="16" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B65" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C65" s="16" t="s">
         <v>0</v>
@@ -8058,30 +8058,30 @@
       <c r="H65" s="14"/>
       <c r="I65" s="14"/>
       <c r="J65" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K65" s="14"/>
       <c r="L65" s="14"/>
       <c r="M65" s="14"/>
       <c r="N65" s="14"/>
       <c r="O65" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P65" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q65" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R65" s="14"/>
       <c r="S65" s="14"/>
     </row>
     <row r="66" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="16" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C66" s="16" t="s">
         <v>0</v>
@@ -8095,20 +8095,20 @@
       <c r="H66" s="14"/>
       <c r="I66" s="14"/>
       <c r="J66" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K66" s="14"/>
       <c r="L66" s="14"/>
       <c r="M66" s="14"/>
       <c r="N66" s="14"/>
       <c r="O66" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P66" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q66" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="R66" s="14"/>
       <c r="S66" s="14"/>
@@ -8136,10 +8136,10 @@
     </row>
     <row r="69" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A69" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B69" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C69" s="15" t="s">
         <v>61</v>
@@ -8157,10 +8157,10 @@
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C70" s="15" t="s">
         <v>61</v>
@@ -8178,10 +8178,10 @@
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A71" s="15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B71" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C71" s="15" t="s">
         <v>61</v>
@@ -8202,10 +8202,10 @@
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A72" s="15" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B72" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C72" s="15" t="s">
         <v>61</v>
@@ -8223,10 +8223,10 @@
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A73" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B73" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C73" s="15" t="s">
         <v>61</v>
@@ -8244,10 +8244,10 @@
     </row>
     <row r="74" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A74" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B74" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C74" s="15" t="s">
         <v>3</v>
@@ -8265,10 +8265,10 @@
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A75" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B75" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C75" s="15" t="s">
         <v>61</v>
@@ -8286,10 +8286,10 @@
     </row>
     <row r="76" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="15" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C76" s="15" t="s">
         <v>61</v>
@@ -8319,10 +8319,10 @@
     </row>
     <row r="77" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A77" s="15" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B77" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C77" s="15" t="s">
         <v>61</v>
@@ -8343,10 +8343,10 @@
     </row>
     <row r="78" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A78" s="15" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B78" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C78" s="15" t="s">
         <v>61</v>
@@ -8364,10 +8364,10 @@
     </row>
     <row r="79" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A79" s="15" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B79" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C79" s="15" t="s">
         <v>3</v>
@@ -8385,10 +8385,10 @@
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A80" s="15" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B80" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C80" s="15" t="s">
         <v>61</v>
@@ -8407,10 +8407,10 @@
     </row>
     <row r="81" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A81" s="15" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B81" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C81" s="15" t="s">
         <v>61</v>
@@ -8429,10 +8429,10 @@
     </row>
     <row r="82" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="15" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B82" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C82" s="15" t="s">
         <v>61</v>
@@ -8462,10 +8462,10 @@
     </row>
     <row r="83" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B83" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C83" s="15" t="s">
         <v>61</v>
@@ -8486,10 +8486,10 @@
     </row>
     <row r="84" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A84" s="15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B84" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C84" s="15" t="s">
         <v>3</v>
@@ -8507,10 +8507,10 @@
     </row>
     <row r="85" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A85" s="15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B85" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C85" s="15" t="s">
         <v>3</v>
@@ -8528,10 +8528,10 @@
     </row>
     <row r="86" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A86" s="15" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B86" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C86" s="15" t="s">
         <v>3</v>
@@ -8549,10 +8549,10 @@
     </row>
     <row r="87" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A87" s="15" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B87" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C87" s="15" t="s">
         <v>3</v>
@@ -8570,10 +8570,10 @@
     </row>
     <row r="88" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A88" s="15" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B88" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C88" s="15" t="s">
         <v>3</v>
@@ -8591,10 +8591,10 @@
     </row>
     <row r="89" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A89" s="15" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B89" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C89" s="15" t="s">
         <v>3</v>
@@ -8612,10 +8612,10 @@
     </row>
     <row r="90" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A90" s="15" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B90" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C90" s="15" t="s">
         <v>3</v>
@@ -8632,10 +8632,10 @@
     </row>
     <row r="91" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A91" s="15" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B91" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C91" s="15" t="s">
         <v>3</v>
@@ -8652,10 +8652,10 @@
     </row>
     <row r="92" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A92" s="15" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B92" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C92" s="15" t="s">
         <v>3</v>
@@ -8672,10 +8672,10 @@
     </row>
     <row r="93" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A93" s="15" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B93" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C93" s="15" t="s">
         <v>3</v>
@@ -8692,10 +8692,10 @@
     </row>
     <row r="94" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A94" s="15" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B94" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C94" s="15" t="s">
         <v>46</v>
@@ -8712,10 +8712,10 @@
     </row>
     <row r="95" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="15" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B95" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C95" s="15" t="s">
         <v>46</v>
@@ -8745,10 +8745,10 @@
     </row>
     <row r="96" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="15" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B96" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C96" s="15" t="s">
         <v>46</v>
@@ -8778,10 +8778,10 @@
     </row>
     <row r="97" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="15" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B97" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C97" s="15" t="s">
         <v>2</v>
@@ -8798,11 +8798,11 @@
         <v>115</v>
       </c>
       <c r="I97" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J97" s="14"/>
       <c r="K97" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L97" s="14"/>
       <c r="M97" s="14"/>
@@ -8815,10 +8815,10 @@
     </row>
     <row r="98" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="15" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B98" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C98" s="14"/>
       <c r="D98" s="14"/>
@@ -8831,11 +8831,11 @@
         <v>115</v>
       </c>
       <c r="I98" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J98" s="14"/>
       <c r="K98" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L98" s="14"/>
       <c r="M98" s="14"/>
@@ -8848,10 +8848,10 @@
     </row>
     <row r="99" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="15" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B99" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D99" s="14"/>
       <c r="E99" s="15" t="s">
@@ -8863,11 +8863,11 @@
         <v>115</v>
       </c>
       <c r="I99" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J99" s="14"/>
       <c r="K99" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L99" s="14"/>
       <c r="M99" s="14"/>

</xml_diff>

<commit_message>
added script for bulk putaway
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0D56BDB-C335-4F99-85EC-1AD9764E544B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3763EC-ED4E-4685-9D30-2DE9BC63FBA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1477" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="403">
   <si>
     <t>1</t>
   </si>
@@ -469,9 +469,6 @@
     <t>QSC_OBScenario002</t>
   </si>
   <si>
-    <t>FG-000412-00</t>
-  </si>
-  <si>
     <t>FG-000413-01</t>
   </si>
   <si>
@@ -1223,6 +1220,12 @@
   </si>
   <si>
     <t>ST-G0-0-1-R</t>
+  </si>
+  <si>
+    <t>QSC_IBScenario036</t>
+  </si>
+  <si>
+    <t>FG-000003-AC</t>
   </si>
 </sst>
 </file>
@@ -1737,7 +1740,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA126"/>
+  <dimension ref="A1:AA127"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="14" customWidth="1"/>
@@ -1791,63 +1794,63 @@
         <v>126</v>
       </c>
       <c r="J1" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="K1" s="17" t="s">
+        <v>276</v>
+      </c>
+      <c r="L1" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="M1" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="K1" s="17" t="s">
-        <v>277</v>
-      </c>
-      <c r="L1" s="17" t="s">
-        <v>279</v>
-      </c>
-      <c r="M1" s="17" t="s">
+      <c r="N1" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="N1" s="17" t="s">
+      <c r="O1" s="17" t="s">
         <v>156</v>
       </c>
-      <c r="O1" s="17" t="s">
+      <c r="P1" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="P1" s="17" t="s">
-        <v>158</v>
-      </c>
       <c r="Q1" s="17" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R1" s="17" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="S1" s="17" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="T1" s="17" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="U1" s="22" t="s">
+        <v>342</v>
+      </c>
+      <c r="V1" s="22" t="s">
         <v>343</v>
       </c>
-      <c r="V1" s="22" t="s">
+      <c r="W1" s="22" t="s">
         <v>344</v>
       </c>
-      <c r="W1" s="22" t="s">
+      <c r="X1" s="22" t="s">
         <v>345</v>
       </c>
-      <c r="X1" s="22" t="s">
+      <c r="Y1" s="22" t="s">
         <v>346</v>
       </c>
-      <c r="Y1" s="22" t="s">
+      <c r="Z1" s="22" t="s">
         <v>347</v>
       </c>
-      <c r="Z1" s="22" t="s">
+      <c r="AA1" s="22" t="s">
         <v>348</v>
-      </c>
-      <c r="AA1" s="22" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="2" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>108</v>
@@ -1886,7 +1889,7 @@
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B3" s="14" t="s">
         <v>108</v>
@@ -1904,7 +1907,7 @@
     </row>
     <row r="4" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>108</v>
@@ -1945,7 +1948,7 @@
     </row>
     <row r="5" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B5" s="14" t="s">
         <v>108</v>
@@ -1963,7 +1966,7 @@
       <c r="G5" s="14"/>
       <c r="H5" s="14"/>
       <c r="I5" s="14" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="J5" s="14"/>
       <c r="K5" s="14"/>
@@ -1986,7 +1989,7 @@
     </row>
     <row r="6" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B6" s="14" t="s">
         <v>108</v>
@@ -2025,7 +2028,7 @@
     </row>
     <row r="7" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B7" s="14" t="s">
         <v>108</v>
@@ -2064,7 +2067,7 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>108</v>
@@ -2077,7 +2080,7 @@
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="15" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G8" s="15" t="s">
         <v>3</v>
@@ -2085,7 +2088,7 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B9" s="14" t="s">
         <v>108</v>
@@ -2102,12 +2105,12 @@
       </c>
       <c r="G9" s="15"/>
       <c r="I9" s="14" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B10" s="14" t="s">
         <v>108</v>
@@ -2129,7 +2132,7 @@
     </row>
     <row r="11" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B11" s="14" t="s">
         <v>108</v>
@@ -2170,7 +2173,7 @@
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B12" s="14" t="s">
         <v>108</v>
@@ -2191,7 +2194,7 @@
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B13" s="14" t="s">
         <v>108</v>
@@ -2212,7 +2215,7 @@
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B14" s="14" t="s">
         <v>108</v>
@@ -2230,7 +2233,7 @@
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B15" s="14" t="s">
         <v>108</v>
@@ -2248,7 +2251,7 @@
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B16" s="14" t="s">
         <v>108</v>
@@ -2269,7 +2272,7 @@
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B17" s="14" t="s">
         <v>108</v>
@@ -2290,7 +2293,7 @@
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B18" s="14" t="s">
         <v>108</v>
@@ -2311,7 +2314,7 @@
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>108</v>
@@ -2332,7 +2335,7 @@
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>108</v>
@@ -2352,7 +2355,7 @@
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>108</v>
@@ -2372,7 +2375,7 @@
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>108</v>
@@ -2392,7 +2395,7 @@
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>108</v>
@@ -2412,7 +2415,7 @@
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B24" s="14" t="s">
         <v>108</v>
@@ -2432,7 +2435,7 @@
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B25" s="14" t="s">
         <v>108</v>
@@ -2452,7 +2455,7 @@
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>108</v>
@@ -2472,7 +2475,7 @@
     </row>
     <row r="27" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B27" s="14" t="s">
         <v>108</v>
@@ -2511,7 +2514,7 @@
     </row>
     <row r="28" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B28" s="14" t="s">
         <v>108</v>
@@ -2520,7 +2523,7 @@
         <v>140</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E28" s="14"/>
       <c r="F28" s="14" t="s">
@@ -2550,7 +2553,7 @@
     </row>
     <row r="29" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B29" s="14" t="s">
         <v>108</v>
@@ -2559,7 +2562,7 @@
         <v>140</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E29" s="14"/>
       <c r="F29" s="14" t="s">
@@ -2589,7 +2592,7 @@
     </row>
     <row r="30" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B30" s="14" t="s">
         <v>108</v>
@@ -2628,7 +2631,7 @@
     </row>
     <row r="31" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B31" s="14" t="s">
         <v>108</v>
@@ -2667,7 +2670,7 @@
     </row>
     <row r="32" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>108</v>
@@ -2706,7 +2709,7 @@
     </row>
     <row r="33" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>108</v>
@@ -2715,7 +2718,7 @@
         <v>140</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E33" s="14"/>
       <c r="F33" s="14" t="s">
@@ -2745,7 +2748,7 @@
     </row>
     <row r="34" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>108</v>
@@ -2754,7 +2757,7 @@
         <v>140</v>
       </c>
       <c r="D34" s="18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E34" s="14"/>
       <c r="F34" s="14" t="s">
@@ -2784,7 +2787,7 @@
     </row>
     <row r="35" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>108</v>
@@ -2793,7 +2796,7 @@
         <v>140</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E35" s="14"/>
       <c r="F35" s="14" t="s">
@@ -2823,7 +2826,7 @@
     </row>
     <row r="36" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>108</v>
@@ -2832,7 +2835,7 @@
         <v>140</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E36" s="14"/>
       <c r="F36" s="14" t="s">
@@ -2862,7 +2865,7 @@
     </row>
     <row r="37" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>108</v>
@@ -2871,7 +2874,7 @@
         <v>140</v>
       </c>
       <c r="D37" s="18" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E37" s="14"/>
       <c r="F37" s="14" t="s">
@@ -2901,7 +2904,7 @@
     </row>
     <row r="38" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B38" s="14" t="s">
         <v>108</v>
@@ -2910,7 +2913,7 @@
         <v>140</v>
       </c>
       <c r="D38" s="18" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E38" s="14"/>
       <c r="F38" s="14" t="s">
@@ -2939,12 +2942,22 @@
       <c r="AA38" s="14"/>
     </row>
     <row r="39" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="15"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="18"/>
+      <c r="A39" s="15" t="s">
+        <v>401</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D39" s="23" t="s">
+        <v>0</v>
+      </c>
       <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
+      <c r="F39" s="14" t="s">
+        <v>115</v>
+      </c>
       <c r="G39" s="14"/>
       <c r="H39" s="14"/>
       <c r="I39" s="14"/>
@@ -2968,18 +2981,10 @@
       <c r="AA39" s="14"/>
     </row>
     <row r="40" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="14" t="s">
-        <v>359</v>
-      </c>
-      <c r="B40" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="D40" s="23" t="s">
-        <v>0</v>
-      </c>
+      <c r="A40" s="15"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="18"/>
       <c r="E40" s="14"/>
       <c r="F40" s="14"/>
       <c r="G40" s="14"/>
@@ -3005,10 +3010,18 @@
       <c r="AA40" s="14"/>
     </row>
     <row r="41" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="15"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="18"/>
+      <c r="A41" s="14" t="s">
+        <v>358</v>
+      </c>
+      <c r="B41" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C41" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D41" s="23" t="s">
+        <v>0</v>
+      </c>
       <c r="E41" s="14"/>
       <c r="F41" s="14"/>
       <c r="G41" s="14"/>
@@ -3034,18 +3047,10 @@
       <c r="AA41" s="14"/>
     </row>
     <row r="42" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="B42" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="C42" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="D42" s="23" t="s">
-        <v>165</v>
-      </c>
+      <c r="A42" s="15"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="18"/>
       <c r="E42" s="14"/>
       <c r="F42" s="14"/>
       <c r="G42" s="14"/>
@@ -3072,7 +3077,7 @@
     </row>
     <row r="43" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>108</v>
@@ -3081,7 +3086,7 @@
         <v>140</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="E43" s="14"/>
       <c r="F43" s="14"/>
@@ -3109,7 +3114,7 @@
     </row>
     <row r="44" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>108</v>
@@ -3118,7 +3123,7 @@
         <v>140</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E44" s="14"/>
       <c r="F44" s="14"/>
@@ -3146,7 +3151,7 @@
     </row>
     <row r="45" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>108</v>
@@ -3155,7 +3160,7 @@
         <v>140</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E45" s="14"/>
       <c r="F45" s="14"/>
@@ -3169,9 +3174,7 @@
       <c r="N45" s="14"/>
       <c r="O45" s="14"/>
       <c r="P45" s="14"/>
-      <c r="Q45" s="14" t="s">
-        <v>162</v>
-      </c>
+      <c r="Q45" s="14"/>
       <c r="R45" s="14"/>
       <c r="S45" s="14"/>
       <c r="T45" s="14"/>
@@ -3185,7 +3188,7 @@
     </row>
     <row r="46" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B46" s="14" t="s">
         <v>108</v>
@@ -3194,7 +3197,7 @@
         <v>140</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E46" s="14"/>
       <c r="F46" s="14"/>
@@ -3209,7 +3212,7 @@
       <c r="O46" s="14"/>
       <c r="P46" s="14"/>
       <c r="Q46" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="R46" s="14"/>
       <c r="S46" s="14"/>
@@ -3224,7 +3227,7 @@
     </row>
     <row r="47" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="B47" s="14" t="s">
         <v>108</v>
@@ -3233,7 +3236,7 @@
         <v>140</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E47" s="14"/>
       <c r="F47" s="14"/>
@@ -3248,7 +3251,7 @@
       <c r="O47" s="14"/>
       <c r="P47" s="14"/>
       <c r="Q47" s="14" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="R47" s="14"/>
       <c r="S47" s="14"/>
@@ -3263,7 +3266,7 @@
     </row>
     <row r="48" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B48" s="14" t="s">
         <v>108</v>
@@ -3272,7 +3275,7 @@
         <v>140</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="E48" s="14"/>
       <c r="F48" s="14"/>
@@ -3287,7 +3290,7 @@
       <c r="O48" s="14"/>
       <c r="P48" s="14"/>
       <c r="Q48" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="R48" s="14"/>
       <c r="S48" s="14"/>
@@ -3302,7 +3305,7 @@
     </row>
     <row r="49" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="B49" s="14" t="s">
         <v>108</v>
@@ -3311,7 +3314,7 @@
         <v>140</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E49" s="14"/>
       <c r="F49" s="14"/>
@@ -3341,7 +3344,7 @@
     </row>
     <row r="50" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B50" s="14" t="s">
         <v>108</v>
@@ -3350,7 +3353,7 @@
         <v>140</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>197</v>
+        <v>178</v>
       </c>
       <c r="E50" s="14"/>
       <c r="F50" s="14"/>
@@ -3364,7 +3367,9 @@
       <c r="N50" s="14"/>
       <c r="O50" s="14"/>
       <c r="P50" s="14"/>
-      <c r="Q50" s="14"/>
+      <c r="Q50" s="14" t="s">
+        <v>161</v>
+      </c>
       <c r="R50" s="14"/>
       <c r="S50" s="14"/>
       <c r="T50" s="14"/>
@@ -3378,7 +3383,7 @@
     </row>
     <row r="51" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B51" s="14" t="s">
         <v>108</v>
@@ -3387,7 +3392,7 @@
         <v>140</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E51" s="14"/>
       <c r="F51" s="14"/>
@@ -3415,7 +3420,7 @@
     </row>
     <row r="52" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B52" s="14" t="s">
         <v>108</v>
@@ -3424,7 +3429,7 @@
         <v>140</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E52" s="14"/>
       <c r="F52" s="14"/>
@@ -3452,7 +3457,7 @@
     </row>
     <row r="53" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="B53" s="14" t="s">
         <v>108</v>
@@ -3461,7 +3466,7 @@
         <v>140</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="E53" s="14"/>
       <c r="F53" s="14"/>
@@ -3489,7 +3494,7 @@
     </row>
     <row r="54" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>265</v>
+        <v>206</v>
       </c>
       <c r="B54" s="14" t="s">
         <v>108</v>
@@ -3498,7 +3503,7 @@
         <v>140</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="E54" s="14"/>
       <c r="F54" s="14"/>
@@ -3514,12 +3519,8 @@
       <c r="P54" s="14"/>
       <c r="Q54" s="14"/>
       <c r="R54" s="14"/>
-      <c r="S54" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T54" s="14" t="s">
-        <v>307</v>
-      </c>
+      <c r="S54" s="14"/>
+      <c r="T54" s="14"/>
       <c r="U54" s="14"/>
       <c r="V54" s="14"/>
       <c r="W54" s="14"/>
@@ -3530,7 +3531,7 @@
     </row>
     <row r="55" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B55" s="14" t="s">
         <v>108</v>
@@ -3539,7 +3540,7 @@
         <v>140</v>
       </c>
       <c r="D55" s="23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E55" s="14"/>
       <c r="F55" s="14"/>
@@ -3558,8 +3559,8 @@
       <c r="S55" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="T55" s="15" t="s">
-        <v>308</v>
+      <c r="T55" s="14" t="s">
+        <v>306</v>
       </c>
       <c r="U55" s="14"/>
       <c r="V55" s="14"/>
@@ -3571,7 +3572,7 @@
     </row>
     <row r="56" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B56" s="14" t="s">
         <v>108</v>
@@ -3580,7 +3581,7 @@
         <v>140</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E56" s="14"/>
       <c r="F56" s="14"/>
@@ -3599,8 +3600,8 @@
       <c r="S56" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="T56" s="24" t="s">
-        <v>309</v>
+      <c r="T56" s="15" t="s">
+        <v>307</v>
       </c>
       <c r="U56" s="14"/>
       <c r="V56" s="14"/>
@@ -3612,7 +3613,7 @@
     </row>
     <row r="57" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B57" s="14" t="s">
         <v>108</v>
@@ -3621,7 +3622,7 @@
         <v>140</v>
       </c>
       <c r="D57" s="23" t="s">
-        <v>273</v>
+        <v>169</v>
       </c>
       <c r="E57" s="14"/>
       <c r="F57" s="14"/>
@@ -3635,15 +3636,13 @@
       <c r="N57" s="14"/>
       <c r="O57" s="14"/>
       <c r="P57" s="14"/>
-      <c r="Q57" s="14" t="s">
-        <v>163</v>
-      </c>
+      <c r="Q57" s="14"/>
       <c r="R57" s="14"/>
       <c r="S57" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="T57" s="14" t="s">
-        <v>307</v>
+      <c r="T57" s="24" t="s">
+        <v>308</v>
       </c>
       <c r="U57" s="14"/>
       <c r="V57" s="14"/>
@@ -3655,7 +3654,7 @@
     </row>
     <row r="58" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B58" s="14" t="s">
         <v>108</v>
@@ -3664,7 +3663,7 @@
         <v>140</v>
       </c>
       <c r="D58" s="23" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E58" s="14"/>
       <c r="F58" s="14"/>
@@ -3679,14 +3678,14 @@
       <c r="O58" s="14"/>
       <c r="P58" s="14"/>
       <c r="Q58" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="R58" s="14"/>
       <c r="S58" s="15" t="s">
         <v>0</v>
       </c>
       <c r="T58" s="14" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="U58" s="14"/>
       <c r="V58" s="14"/>
@@ -3698,7 +3697,7 @@
     </row>
     <row r="59" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B59" s="14" t="s">
         <v>108</v>
@@ -3707,7 +3706,7 @@
         <v>140</v>
       </c>
       <c r="D59" s="23" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E59" s="14"/>
       <c r="F59" s="14"/>
@@ -3722,13 +3721,15 @@
       <c r="O59" s="14"/>
       <c r="P59" s="14"/>
       <c r="Q59" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="R59" s="14"/>
       <c r="S59" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="T59" s="14"/>
+      <c r="T59" s="14" t="s">
+        <v>307</v>
+      </c>
       <c r="U59" s="14"/>
       <c r="V59" s="14"/>
       <c r="W59" s="14"/>
@@ -3738,10 +3739,18 @@
       <c r="AA59" s="14"/>
     </row>
     <row r="60" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="14"/>
-      <c r="B60" s="14"/>
-      <c r="C60" s="14"/>
-      <c r="D60" s="23"/>
+      <c r="A60" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="B60" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C60" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D60" s="23" t="s">
+        <v>272</v>
+      </c>
       <c r="E60" s="14"/>
       <c r="F60" s="14"/>
       <c r="G60" s="14"/>
@@ -3754,9 +3763,13 @@
       <c r="N60" s="14"/>
       <c r="O60" s="14"/>
       <c r="P60" s="14"/>
-      <c r="Q60" s="14"/>
+      <c r="Q60" s="14" t="s">
+        <v>162</v>
+      </c>
       <c r="R60" s="14"/>
-      <c r="S60" s="14"/>
+      <c r="S60" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="T60" s="14"/>
       <c r="U60" s="14"/>
       <c r="V60" s="14"/>
@@ -3767,19 +3780,11 @@
       <c r="AA60" s="14"/>
     </row>
     <row r="61" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="14" t="s">
-        <v>310</v>
-      </c>
-      <c r="B61" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="C61" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="D61" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="E61" s="15"/>
+      <c r="A61" s="14"/>
+      <c r="B61" s="14"/>
+      <c r="C61" s="14"/>
+      <c r="D61" s="23"/>
+      <c r="E61" s="14"/>
       <c r="F61" s="14"/>
       <c r="G61" s="14"/>
       <c r="H61" s="14"/>
@@ -3805,7 +3810,7 @@
     </row>
     <row r="62" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B62" s="14" t="s">
         <v>108</v>
@@ -3814,9 +3819,9 @@
         <v>140</v>
       </c>
       <c r="D62" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="E62" s="14"/>
+        <v>0</v>
+      </c>
+      <c r="E62" s="15"/>
       <c r="F62" s="14"/>
       <c r="G62" s="14"/>
       <c r="H62" s="14"/>
@@ -3842,7 +3847,7 @@
     </row>
     <row r="63" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B63" s="14" t="s">
         <v>108</v>
@@ -3851,17 +3856,13 @@
         <v>140</v>
       </c>
       <c r="D63" s="18" t="s">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="E63" s="14"/>
-      <c r="F63" s="14" t="s">
-        <v>115</v>
-      </c>
+      <c r="F63" s="14"/>
       <c r="G63" s="14"/>
       <c r="H63" s="14"/>
-      <c r="I63" s="14" t="s">
-        <v>130</v>
-      </c>
+      <c r="I63" s="14"/>
       <c r="J63" s="14"/>
       <c r="K63" s="14"/>
       <c r="L63" s="14"/>
@@ -3883,7 +3884,7 @@
     </row>
     <row r="64" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B64" s="14" t="s">
         <v>108</v>
@@ -3892,7 +3893,7 @@
         <v>140</v>
       </c>
       <c r="D64" s="18" t="s">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="E64" s="14"/>
       <c r="F64" s="14" t="s">
@@ -3901,7 +3902,7 @@
       <c r="G64" s="14"/>
       <c r="H64" s="14"/>
       <c r="I64" s="14" t="s">
-        <v>391</v>
+        <v>130</v>
       </c>
       <c r="J64" s="14"/>
       <c r="K64" s="14"/>
@@ -3924,7 +3925,7 @@
     </row>
     <row r="65" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
-        <v>350</v>
+        <v>312</v>
       </c>
       <c r="B65" s="14" t="s">
         <v>108</v>
@@ -3932,14 +3933,18 @@
       <c r="C65" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="D65" s="25" t="s">
-        <v>354</v>
+      <c r="D65" s="18" t="s">
+        <v>120</v>
       </c>
       <c r="E65" s="14"/>
-      <c r="F65" s="14"/>
+      <c r="F65" s="14" t="s">
+        <v>115</v>
+      </c>
       <c r="G65" s="14"/>
       <c r="H65" s="14"/>
-      <c r="I65" s="14"/>
+      <c r="I65" s="14" t="s">
+        <v>390</v>
+      </c>
       <c r="J65" s="14"/>
       <c r="K65" s="14"/>
       <c r="L65" s="14"/>
@@ -3961,7 +3966,7 @@
     </row>
     <row r="66" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B66" s="14" t="s">
         <v>108</v>
@@ -3969,8 +3974,8 @@
       <c r="C66" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="D66" s="18" t="s">
-        <v>357</v>
+      <c r="D66" s="25" t="s">
+        <v>353</v>
       </c>
       <c r="E66" s="14"/>
       <c r="F66" s="14"/>
@@ -3998,7 +4003,7 @@
     </row>
     <row r="67" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B67" s="14" t="s">
         <v>108</v>
@@ -4006,8 +4011,8 @@
       <c r="C67" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="D67" s="25" t="s">
-        <v>354</v>
+      <c r="D67" s="18" t="s">
+        <v>356</v>
       </c>
       <c r="E67" s="14"/>
       <c r="F67" s="14"/>
@@ -4035,7 +4040,7 @@
     </row>
     <row r="68" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B68" s="14" t="s">
         <v>108</v>
@@ -4043,8 +4048,8 @@
       <c r="C68" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="D68" s="18" t="s">
-        <v>357</v>
+      <c r="D68" s="25" t="s">
+        <v>353</v>
       </c>
       <c r="E68" s="14"/>
       <c r="F68" s="14"/>
@@ -4072,7 +4077,7 @@
     </row>
     <row r="69" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="14" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="B69" s="14" t="s">
         <v>108</v>
@@ -4080,7 +4085,9 @@
       <c r="C69" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="D69" s="18"/>
+      <c r="D69" s="18" t="s">
+        <v>356</v>
+      </c>
       <c r="E69" s="14"/>
       <c r="F69" s="14"/>
       <c r="G69" s="14"/>
@@ -4106,9 +4113,15 @@
       <c r="AA69" s="14"/>
     </row>
     <row r="70" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="14"/>
-      <c r="B70" s="14"/>
-      <c r="C70" s="14"/>
+      <c r="A70" s="14" t="s">
+        <v>357</v>
+      </c>
+      <c r="B70" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C70" s="14" t="s">
+        <v>140</v>
+      </c>
       <c r="D70" s="18"/>
       <c r="E70" s="14"/>
       <c r="F70" s="14"/>
@@ -4135,30 +4148,18 @@
       <c r="AA70" s="14"/>
     </row>
     <row r="71" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="12" t="s">
-        <v>373</v>
-      </c>
-      <c r="B71" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="C71" s="12" t="s">
-        <v>140</v>
-      </c>
+      <c r="A71" s="14"/>
+      <c r="B71" s="14"/>
+      <c r="C71" s="14"/>
       <c r="D71" s="18"/>
       <c r="E71" s="14"/>
       <c r="F71" s="14"/>
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="14"/>
-      <c r="J71" s="13" t="s">
-        <v>381</v>
-      </c>
-      <c r="K71" s="15" t="s">
-        <v>278</v>
-      </c>
-      <c r="L71" s="14" t="s">
-        <v>382</v>
-      </c>
+      <c r="J71" s="14"/>
+      <c r="K71" s="14"/>
+      <c r="L71" s="14"/>
       <c r="M71" s="14"/>
       <c r="N71" s="14"/>
       <c r="O71" s="14"/>
@@ -4177,7 +4178,7 @@
     </row>
     <row r="72" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="12" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B72" s="12" t="s">
         <v>108</v>
@@ -4191,15 +4192,19 @@
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="14"/>
-      <c r="J72" s="14"/>
-      <c r="K72" s="14"/>
-      <c r="L72" s="12"/>
-      <c r="M72" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="N72" s="12"/>
-      <c r="O72" s="12"/>
-      <c r="P72" s="12"/>
+      <c r="J72" s="13" t="s">
+        <v>380</v>
+      </c>
+      <c r="K72" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="L72" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="M72" s="14"/>
+      <c r="N72" s="14"/>
+      <c r="O72" s="14"/>
+      <c r="P72" s="14"/>
       <c r="Q72" s="14"/>
       <c r="R72" s="14"/>
       <c r="S72" s="14"/>
@@ -4214,7 +4219,7 @@
     </row>
     <row r="73" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="12" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B73" s="12" t="s">
         <v>108</v>
@@ -4231,10 +4236,10 @@
       <c r="J73" s="14"/>
       <c r="K73" s="14"/>
       <c r="L73" s="12"/>
-      <c r="M73" s="12"/>
-      <c r="N73" s="12" t="s">
-        <v>378</v>
-      </c>
+      <c r="M73" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="N73" s="12"/>
       <c r="O73" s="12"/>
       <c r="P73" s="12"/>
       <c r="Q73" s="14"/>
@@ -4251,7 +4256,7 @@
     </row>
     <row r="74" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="12" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B74" s="12" t="s">
         <v>108</v>
@@ -4269,10 +4274,10 @@
       <c r="K74" s="14"/>
       <c r="L74" s="12"/>
       <c r="M74" s="12"/>
-      <c r="N74" s="12"/>
-      <c r="O74" s="12" t="s">
-        <v>379</v>
-      </c>
+      <c r="N74" s="12" t="s">
+        <v>377</v>
+      </c>
+      <c r="O74" s="12"/>
       <c r="P74" s="12"/>
       <c r="Q74" s="14"/>
       <c r="R74" s="14"/>
@@ -4288,7 +4293,7 @@
     </row>
     <row r="75" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="12" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B75" s="12" t="s">
         <v>108</v>
@@ -4307,10 +4312,10 @@
       <c r="L75" s="12"/>
       <c r="M75" s="12"/>
       <c r="N75" s="12"/>
-      <c r="O75" s="12"/>
-      <c r="P75" s="13" t="s">
-        <v>380</v>
-      </c>
+      <c r="O75" s="12" t="s">
+        <v>378</v>
+      </c>
+      <c r="P75" s="12"/>
       <c r="Q75" s="14"/>
       <c r="R75" s="14"/>
       <c r="S75" s="14"/>
@@ -4324,10 +4329,16 @@
       <c r="AA75" s="14"/>
     </row>
     <row r="76" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="14"/>
-      <c r="B76" s="14"/>
-      <c r="C76" s="14"/>
-      <c r="D76" s="23"/>
+      <c r="A76" s="12" t="s">
+        <v>376</v>
+      </c>
+      <c r="B76" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C76" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="D76" s="18"/>
       <c r="E76" s="14"/>
       <c r="F76" s="14"/>
       <c r="G76" s="14"/>
@@ -4335,11 +4346,13 @@
       <c r="I76" s="14"/>
       <c r="J76" s="14"/>
       <c r="K76" s="14"/>
-      <c r="L76" s="14"/>
-      <c r="M76" s="14"/>
-      <c r="N76" s="14"/>
-      <c r="O76" s="14"/>
-      <c r="P76" s="14"/>
+      <c r="L76" s="12"/>
+      <c r="M76" s="12"/>
+      <c r="N76" s="12"/>
+      <c r="O76" s="12"/>
+      <c r="P76" s="13" t="s">
+        <v>379</v>
+      </c>
       <c r="Q76" s="14"/>
       <c r="R76" s="14"/>
       <c r="S76" s="14"/>
@@ -4352,58 +4365,38 @@
       <c r="Z76" s="14"/>
       <c r="AA76" s="14"/>
     </row>
-    <row r="77" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="12" t="s">
-        <v>314</v>
-      </c>
-      <c r="B77" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="C77" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="D77" s="12"/>
-      <c r="E77" s="12"/>
-      <c r="F77" s="12"/>
-      <c r="G77" s="12"/>
-      <c r="H77" s="12"/>
-      <c r="I77" s="12"/>
-      <c r="J77" s="12"/>
-      <c r="K77" s="12"/>
-      <c r="L77" s="12"/>
-      <c r="M77" s="12"/>
-      <c r="N77" s="12"/>
-      <c r="O77" s="12"/>
-      <c r="P77" s="12"/>
-      <c r="Q77" s="12"/>
-      <c r="R77" s="12"/>
-      <c r="S77" s="12"/>
-      <c r="T77" s="12"/>
-      <c r="U77" s="13" t="s">
-        <v>315</v>
-      </c>
-      <c r="V77" s="13" t="s">
-        <v>316</v>
-      </c>
-      <c r="W77" s="12" t="s">
-        <v>317</v>
-      </c>
-      <c r="X77" s="12" t="s">
-        <v>318</v>
-      </c>
-      <c r="Y77" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="Z77" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="AA77" s="12" t="s">
-        <v>140</v>
-      </c>
+    <row r="77" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="14"/>
+      <c r="B77" s="14"/>
+      <c r="C77" s="14"/>
+      <c r="D77" s="23"/>
+      <c r="E77" s="14"/>
+      <c r="F77" s="14"/>
+      <c r="G77" s="14"/>
+      <c r="H77" s="14"/>
+      <c r="I77" s="14"/>
+      <c r="J77" s="14"/>
+      <c r="K77" s="14"/>
+      <c r="L77" s="14"/>
+      <c r="M77" s="14"/>
+      <c r="N77" s="14"/>
+      <c r="O77" s="14"/>
+      <c r="P77" s="14"/>
+      <c r="Q77" s="14"/>
+      <c r="R77" s="14"/>
+      <c r="S77" s="14"/>
+      <c r="T77" s="14"/>
+      <c r="U77" s="14"/>
+      <c r="V77" s="14"/>
+      <c r="W77" s="14"/>
+      <c r="X77" s="14"/>
+      <c r="Y77" s="14"/>
+      <c r="Z77" s="14"/>
+      <c r="AA77" s="14"/>
     </row>
     <row r="78" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="12" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="B78" s="12" t="s">
         <v>108</v>
@@ -4429,19 +4422,19 @@
       <c r="S78" s="12"/>
       <c r="T78" s="12"/>
       <c r="U78" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="V78" s="13" t="s">
         <v>315</v>
       </c>
-      <c r="V78" s="13" t="s">
+      <c r="W78" s="12" t="s">
         <v>316</v>
       </c>
-      <c r="W78" s="12" t="s">
+      <c r="X78" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="X78" s="12" t="s">
+      <c r="Y78" s="12" t="s">
         <v>318</v>
-      </c>
-      <c r="Y78" s="12" t="s">
-        <v>319</v>
       </c>
       <c r="Z78" s="12" t="s">
         <v>108</v>
@@ -4452,7 +4445,7 @@
     </row>
     <row r="79" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="12" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B79" s="12" t="s">
         <v>108</v>
@@ -4477,29 +4470,31 @@
       <c r="R79" s="12"/>
       <c r="S79" s="12"/>
       <c r="T79" s="12"/>
-      <c r="U79" s="12" t="s">
+      <c r="U79" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="V79" s="13" t="s">
         <v>315</v>
       </c>
-      <c r="V79" s="12" t="s">
-        <v>322</v>
-      </c>
       <c r="W79" s="12" t="s">
+        <v>316</v>
+      </c>
+      <c r="X79" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="X79" s="12" t="s">
-        <v>323</v>
-      </c>
       <c r="Y79" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="Z79" s="12"/>
+        <v>318</v>
+      </c>
+      <c r="Z79" s="12" t="s">
+        <v>108</v>
+      </c>
       <c r="AA79" s="12" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="80" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="12" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B80" s="12" t="s">
         <v>108</v>
@@ -4524,29 +4519,29 @@
       <c r="R80" s="12"/>
       <c r="S80" s="12"/>
       <c r="T80" s="12"/>
-      <c r="U80" s="13" t="s">
-        <v>315</v>
-      </c>
-      <c r="V80" s="13" t="s">
-        <v>325</v>
+      <c r="U80" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="V80" s="12" t="s">
+        <v>321</v>
       </c>
       <c r="W80" s="12" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="X80" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="Y80" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="Y80" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="Z80" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="AA80" s="12"/>
+      <c r="Z80" s="12"/>
+      <c r="AA80" s="12" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="81" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="12" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="B81" s="12" t="s">
         <v>108</v>
@@ -4571,29 +4566,29 @@
       <c r="R81" s="12"/>
       <c r="S81" s="12"/>
       <c r="T81" s="12"/>
-      <c r="U81" s="12" t="s">
-        <v>315</v>
-      </c>
-      <c r="V81" s="12" t="s">
-        <v>327</v>
+      <c r="U81" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="V81" s="13" t="s">
+        <v>324</v>
       </c>
       <c r="W81" s="12" t="s">
+        <v>316</v>
+      </c>
+      <c r="X81" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="X81" s="12"/>
       <c r="Y81" s="12" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="Z81" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="AA81" s="12" t="s">
-        <v>140</v>
-      </c>
+      <c r="AA81" s="12"/>
     </row>
     <row r="82" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="12" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="B82" s="12" t="s">
         <v>108</v>
@@ -4618,18 +4613,18 @@
       <c r="R82" s="12"/>
       <c r="S82" s="12"/>
       <c r="T82" s="12"/>
-      <c r="U82" s="12"/>
+      <c r="U82" s="12" t="s">
+        <v>314</v>
+      </c>
       <c r="V82" s="12" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="W82" s="12" t="s">
-        <v>317</v>
-      </c>
-      <c r="X82" s="12" t="s">
-        <v>323</v>
-      </c>
+        <v>316</v>
+      </c>
+      <c r="X82" s="12"/>
       <c r="Y82" s="12" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="Z82" s="12" t="s">
         <v>108</v>
@@ -4640,7 +4635,7 @@
     </row>
     <row r="83" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="12" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B83" s="12" t="s">
         <v>108</v>
@@ -4665,20 +4660,18 @@
       <c r="R83" s="12"/>
       <c r="S83" s="12"/>
       <c r="T83" s="12"/>
-      <c r="U83" s="13" t="s">
-        <v>330</v>
-      </c>
-      <c r="V83" s="13" t="s">
-        <v>331</v>
-      </c>
-      <c r="W83" s="13" t="s">
-        <v>317</v>
+      <c r="U83" s="12"/>
+      <c r="V83" s="12" t="s">
+        <v>326</v>
+      </c>
+      <c r="W83" s="12" t="s">
+        <v>316</v>
       </c>
       <c r="X83" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="Y83" s="12" t="s">
         <v>318</v>
-      </c>
-      <c r="Y83" s="12" t="s">
-        <v>319</v>
       </c>
       <c r="Z83" s="12" t="s">
         <v>108</v>
@@ -4689,7 +4682,7 @@
     </row>
     <row r="84" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="12" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B84" s="12" t="s">
         <v>108</v>
@@ -4715,19 +4708,19 @@
       <c r="S84" s="12"/>
       <c r="T84" s="12"/>
       <c r="U84" s="13" t="s">
-        <v>315</v>
+        <v>329</v>
       </c>
       <c r="V84" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="W84" s="13" t="s">
         <v>316</v>
       </c>
-      <c r="W84" s="13" t="s">
-        <v>333</v>
-      </c>
       <c r="X84" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="Y84" s="12" t="s">
         <v>318</v>
-      </c>
-      <c r="Y84" s="12" t="s">
-        <v>319</v>
       </c>
       <c r="Z84" s="12" t="s">
         <v>108</v>
@@ -4738,7 +4731,7 @@
     </row>
     <row r="85" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="12" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="B85" s="12" t="s">
         <v>108</v>
@@ -4763,31 +4756,31 @@
       <c r="R85" s="12"/>
       <c r="S85" s="12"/>
       <c r="T85" s="12"/>
-      <c r="U85" s="12" t="s">
+      <c r="U85" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="V85" s="13" t="s">
         <v>315</v>
       </c>
-      <c r="V85" s="12" t="s">
-        <v>316</v>
-      </c>
-      <c r="W85" s="12" t="s">
+      <c r="W85" s="13" t="s">
+        <v>332</v>
+      </c>
+      <c r="X85" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="X85" s="12" t="s">
-        <v>323</v>
-      </c>
       <c r="Y85" s="12" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="Z85" s="12" t="s">
-        <v>181</v>
+        <v>108</v>
       </c>
       <c r="AA85" s="12" t="s">
-        <v>335</v>
+        <v>140</v>
       </c>
     </row>
     <row r="86" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="12" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="B86" s="12" t="s">
         <v>108</v>
@@ -4813,30 +4806,30 @@
       <c r="S86" s="12"/>
       <c r="T86" s="12"/>
       <c r="U86" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="V86" s="12" t="s">
         <v>315</v>
       </c>
-      <c r="V86" s="13" t="s">
-        <v>337</v>
-      </c>
       <c r="W86" s="12" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="X86" s="12" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="Y86" s="12" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="Z86" s="12" t="s">
-        <v>108</v>
+        <v>180</v>
       </c>
       <c r="AA86" s="12" t="s">
-        <v>140</v>
+        <v>334</v>
       </c>
     </row>
     <row r="87" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="12" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B87" s="12" t="s">
         <v>108</v>
@@ -4862,19 +4855,19 @@
       <c r="S87" s="12"/>
       <c r="T87" s="12"/>
       <c r="U87" s="12" t="s">
-        <v>315</v>
-      </c>
-      <c r="V87" s="12" t="s">
-        <v>339</v>
+        <v>314</v>
+      </c>
+      <c r="V87" s="13" t="s">
+        <v>336</v>
       </c>
       <c r="W87" s="12" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="X87" s="12" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="Y87" s="12" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="Z87" s="12" t="s">
         <v>108</v>
@@ -4885,7 +4878,7 @@
     </row>
     <row r="88" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="12" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="B88" s="12" t="s">
         <v>108</v>
@@ -4911,22 +4904,22 @@
       <c r="S88" s="12"/>
       <c r="T88" s="12"/>
       <c r="U88" s="12" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="V88" s="12" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="W88" s="12" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="X88" s="12" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="Y88" s="12" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="Z88" s="12" t="s">
-        <v>335</v>
+        <v>108</v>
       </c>
       <c r="AA88" s="12" t="s">
         <v>140</v>
@@ -4934,7 +4927,7 @@
     </row>
     <row r="89" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="12" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="B89" s="12" t="s">
         <v>108</v>
@@ -4960,31 +4953,37 @@
       <c r="S89" s="12"/>
       <c r="T89" s="12"/>
       <c r="U89" s="12" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="V89" s="12" t="s">
+        <v>340</v>
+      </c>
+      <c r="W89" s="12" t="s">
+        <v>316</v>
+      </c>
+      <c r="X89" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="Y89" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="Z89" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="AA89" s="12" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="90" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="12" t="s">
         <v>341</v>
       </c>
-      <c r="W89" s="12" t="s">
-        <v>317</v>
-      </c>
-      <c r="X89" s="12" t="s">
-        <v>318</v>
-      </c>
-      <c r="Y89" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="Z89" s="12" t="s">
+      <c r="B90" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="AA89" s="12" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="90" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="12"/>
-      <c r="B90" s="12"/>
-      <c r="C90" s="12"/>
+      <c r="C90" s="12" t="s">
+        <v>140</v>
+      </c>
       <c r="D90" s="12"/>
       <c r="E90" s="12"/>
       <c r="F90" s="12"/>
@@ -5002,13 +5001,27 @@
       <c r="R90" s="12"/>
       <c r="S90" s="12"/>
       <c r="T90" s="12"/>
-      <c r="U90" s="12"/>
-      <c r="V90" s="12"/>
-      <c r="W90" s="12"/>
-      <c r="X90" s="12"/>
-      <c r="Y90" s="12"/>
-      <c r="Z90" s="12"/>
-      <c r="AA90" s="12"/>
+      <c r="U90" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="V90" s="12" t="s">
+        <v>340</v>
+      </c>
+      <c r="W90" s="12" t="s">
+        <v>316</v>
+      </c>
+      <c r="X90" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="Y90" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="Z90" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="AA90" s="12" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="91" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="12"/>
@@ -5039,38 +5052,47 @@
       <c r="Z91" s="12"/>
       <c r="AA91" s="12"/>
     </row>
-    <row r="92" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A92" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="B92" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="C92" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="D92" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="F92" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="R92" s="15" t="s">
-        <v>0</v>
-      </c>
+    <row r="92" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="12"/>
+      <c r="B92" s="12"/>
+      <c r="C92" s="12"/>
+      <c r="D92" s="12"/>
+      <c r="E92" s="12"/>
+      <c r="F92" s="12"/>
+      <c r="G92" s="12"/>
+      <c r="H92" s="12"/>
+      <c r="I92" s="12"/>
+      <c r="J92" s="12"/>
+      <c r="K92" s="12"/>
+      <c r="L92" s="12"/>
+      <c r="M92" s="12"/>
+      <c r="N92" s="12"/>
+      <c r="O92" s="12"/>
+      <c r="P92" s="12"/>
+      <c r="Q92" s="12"/>
+      <c r="R92" s="12"/>
+      <c r="S92" s="12"/>
+      <c r="T92" s="12"/>
+      <c r="U92" s="12"/>
+      <c r="V92" s="12"/>
+      <c r="W92" s="12"/>
+      <c r="X92" s="12"/>
+      <c r="Y92" s="12"/>
+      <c r="Z92" s="12"/>
+      <c r="AA92" s="12"/>
     </row>
     <row r="93" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A93" s="14" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B93" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C93" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D93" s="15" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F93" s="14" t="s">
         <v>115</v>
@@ -5081,16 +5103,16 @@
     </row>
     <row r="94" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A94" s="14" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B94" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C94" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D94" s="15" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F94" s="14" t="s">
         <v>115</v>
@@ -5101,16 +5123,16 @@
     </row>
     <row r="95" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A95" s="14" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B95" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C95" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D95" s="15" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F95" s="14" t="s">
         <v>115</v>
@@ -5121,16 +5143,16 @@
     </row>
     <row r="96" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A96" s="14" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B96" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C96" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D96" s="15" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F96" s="14" t="s">
         <v>115</v>
@@ -5141,16 +5163,16 @@
     </row>
     <row r="97" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A97" s="14" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B97" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C97" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D97" s="15" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="F97" s="14" t="s">
         <v>115</v>
@@ -5161,75 +5183,56 @@
     </row>
     <row r="98" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A98" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B98" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C98" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D98" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F98" s="14" t="s">
         <v>115</v>
       </c>
       <c r="R98" s="15" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A99" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="B99" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="C99" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D99" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="F99" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="R99" s="15" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="99" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="14" t="s">
-        <v>257</v>
-      </c>
-      <c r="B99" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="C99" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="D99" s="15" t="s">
-        <v>243</v>
-      </c>
-      <c r="E99" s="14"/>
-      <c r="F99" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="G99" s="14"/>
-      <c r="H99" s="14"/>
-      <c r="I99" s="14"/>
-      <c r="J99" s="14"/>
-      <c r="K99" s="14"/>
-      <c r="L99" s="14"/>
-      <c r="M99" s="14"/>
-      <c r="N99" s="14"/>
-      <c r="O99" s="14"/>
-      <c r="P99" s="14"/>
-      <c r="Q99" s="14"/>
-      <c r="R99" s="15"/>
-      <c r="S99" s="14"/>
-      <c r="T99" s="14"/>
-      <c r="U99" s="14"/>
-      <c r="V99" s="14"/>
-      <c r="W99" s="14"/>
-      <c r="X99" s="14"/>
-      <c r="Y99" s="14"/>
-      <c r="Z99" s="14"/>
-      <c r="AA99" s="14"/>
     </row>
     <row r="100" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="14" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B100" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C100" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D100" s="15" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E100" s="14"/>
       <c r="F100" s="14" t="s">
@@ -5257,36 +5260,57 @@
       <c r="Z100" s="14"/>
       <c r="AA100" s="14"/>
     </row>
-    <row r="101" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="14" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B101" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C101" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D101" s="15" t="s">
-        <v>245</v>
-      </c>
+        <v>243</v>
+      </c>
+      <c r="E101" s="14"/>
       <c r="F101" s="14" t="s">
         <v>115</v>
       </c>
+      <c r="G101" s="14"/>
+      <c r="H101" s="14"/>
+      <c r="I101" s="14"/>
+      <c r="J101" s="14"/>
+      <c r="K101" s="14"/>
+      <c r="L101" s="14"/>
+      <c r="M101" s="14"/>
+      <c r="N101" s="14"/>
+      <c r="O101" s="14"/>
+      <c r="P101" s="14"/>
+      <c r="Q101" s="14"/>
       <c r="R101" s="15"/>
+      <c r="S101" s="14"/>
+      <c r="T101" s="14"/>
+      <c r="U101" s="14"/>
+      <c r="V101" s="14"/>
+      <c r="W101" s="14"/>
+      <c r="X101" s="14"/>
+      <c r="Y101" s="14"/>
+      <c r="Z101" s="14"/>
+      <c r="AA101" s="14"/>
     </row>
     <row r="102" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A102" s="14" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B102" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C102" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D102" s="15" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="F102" s="14" t="s">
         <v>115</v>
@@ -5295,16 +5319,16 @@
     </row>
     <row r="103" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A103" s="14" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B103" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C103" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D103" s="15" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F103" s="14" t="s">
         <v>115</v>
@@ -5313,36 +5337,34 @@
     </row>
     <row r="104" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A104" s="14" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B104" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C104" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="D104" s="16" t="s">
-        <v>264</v>
+      <c r="D104" s="15" t="s">
+        <v>246</v>
       </c>
       <c r="F104" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="R104" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R104" s="15"/>
     </row>
     <row r="105" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A105" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="B105" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="C105" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D105" s="16" t="s">
         <v>263</v>
-      </c>
-      <c r="B105" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="C105" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="D105" s="15" t="s">
-        <v>285</v>
       </c>
       <c r="F105" s="14" t="s">
         <v>115</v>
@@ -5351,59 +5373,38 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A106" s="14" t="s">
-        <v>286</v>
+        <v>262</v>
       </c>
       <c r="B106" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C106" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D106" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="E106" s="14"/>
+        <v>284</v>
+      </c>
       <c r="F106" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="G106" s="14"/>
-      <c r="H106" s="14"/>
-      <c r="I106" s="14"/>
-      <c r="J106" s="14"/>
-      <c r="K106" s="14"/>
-      <c r="L106" s="14"/>
-      <c r="M106" s="14"/>
-      <c r="N106" s="14"/>
-      <c r="O106" s="14"/>
-      <c r="P106" s="14"/>
-      <c r="Q106" s="14"/>
       <c r="R106" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="S106" s="14"/>
-      <c r="T106" s="14"/>
-      <c r="U106" s="14"/>
-      <c r="V106" s="14"/>
-      <c r="W106" s="14"/>
-      <c r="X106" s="14"/>
-      <c r="Y106" s="14"/>
-      <c r="Z106" s="14"/>
-      <c r="AA106" s="14"/>
     </row>
     <row r="107" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="14" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="B107" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C107" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D107" s="15" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="E107" s="14"/>
       <c r="F107" s="14" t="s">
@@ -5421,7 +5422,7 @@
       <c r="P107" s="14"/>
       <c r="Q107" s="14"/>
       <c r="R107" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S107" s="14"/>
       <c r="T107" s="14"/>
@@ -5435,16 +5436,16 @@
     </row>
     <row r="108" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="14" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B108" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C108" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D108" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E108" s="14"/>
       <c r="F108" s="14" t="s">
@@ -5462,7 +5463,7 @@
       <c r="P108" s="14"/>
       <c r="Q108" s="14"/>
       <c r="R108" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S108" s="14"/>
       <c r="T108" s="14"/>
@@ -5476,16 +5477,16 @@
     </row>
     <row r="109" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B109" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C109" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D109" s="15" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="E109" s="14"/>
       <c r="F109" s="14" t="s">
@@ -5517,16 +5518,16 @@
     </row>
     <row r="110" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="14" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="B110" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C110" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D110" s="15" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="E110" s="14"/>
       <c r="F110" s="14" t="s">
@@ -5544,7 +5545,7 @@
       <c r="P110" s="14"/>
       <c r="Q110" s="14"/>
       <c r="R110" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S110" s="14"/>
       <c r="T110" s="14"/>
@@ -5558,16 +5559,16 @@
     </row>
     <row r="111" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="14" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B111" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C111" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D111" s="15" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="E111" s="14"/>
       <c r="F111" s="14" t="s">
@@ -5585,7 +5586,7 @@
       <c r="P111" s="14"/>
       <c r="Q111" s="14"/>
       <c r="R111" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S111" s="14"/>
       <c r="T111" s="14"/>
@@ -5599,16 +5600,16 @@
     </row>
     <row r="112" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="14" t="s">
-        <v>386</v>
+        <v>301</v>
       </c>
       <c r="B112" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C112" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D112" s="15" t="s">
-        <v>385</v>
+        <v>302</v>
       </c>
       <c r="E112" s="14"/>
       <c r="F112" s="14" t="s">
@@ -5616,9 +5617,7 @@
       </c>
       <c r="G112" s="14"/>
       <c r="H112" s="14"/>
-      <c r="I112" s="14" t="s">
-        <v>128</v>
-      </c>
+      <c r="I112" s="14"/>
       <c r="J112" s="14"/>
       <c r="K112" s="14"/>
       <c r="L112" s="14"/>
@@ -5627,7 +5626,9 @@
       <c r="O112" s="14"/>
       <c r="P112" s="14"/>
       <c r="Q112" s="14"/>
-      <c r="R112" s="15"/>
+      <c r="R112" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S112" s="14"/>
       <c r="T112" s="14"/>
       <c r="U112" s="14"/>
@@ -5640,16 +5641,16 @@
     </row>
     <row r="113" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="14" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="B113" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C113" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D113" s="15" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="E113" s="14"/>
       <c r="F113" s="14" t="s">
@@ -5658,7 +5659,7 @@
       <c r="G113" s="14"/>
       <c r="H113" s="14"/>
       <c r="I113" s="14" t="s">
-        <v>392</v>
+        <v>128</v>
       </c>
       <c r="J113" s="14"/>
       <c r="K113" s="14"/>
@@ -5681,16 +5682,16 @@
     </row>
     <row r="114" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="14" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="B114" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C114" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D114" s="15" t="s">
-        <v>397</v>
+        <v>386</v>
       </c>
       <c r="E114" s="14"/>
       <c r="F114" s="14" t="s">
@@ -5699,7 +5700,7 @@
       <c r="G114" s="14"/>
       <c r="H114" s="14"/>
       <c r="I114" s="14" t="s">
-        <v>127</v>
+        <v>391</v>
       </c>
       <c r="J114" s="14"/>
       <c r="K114" s="14"/>
@@ -5722,16 +5723,16 @@
     </row>
     <row r="115" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="14" t="s">
+        <v>394</v>
+      </c>
+      <c r="B115" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="C115" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D115" s="15" t="s">
         <v>396</v>
-      </c>
-      <c r="B115" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="C115" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="D115" s="15" t="s">
-        <v>398</v>
       </c>
       <c r="E115" s="14"/>
       <c r="F115" s="14" t="s">
@@ -5740,7 +5741,7 @@
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
       <c r="I115" s="14" t="s">
-        <v>394</v>
+        <v>127</v>
       </c>
       <c r="J115" s="14"/>
       <c r="K115" s="14"/>
@@ -5762,15 +5763,27 @@
       <c r="AA115" s="14"/>
     </row>
     <row r="116" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="14"/>
-      <c r="B116" s="14"/>
-      <c r="C116" s="14"/>
-      <c r="D116" s="15"/>
+      <c r="A116" s="14" t="s">
+        <v>395</v>
+      </c>
+      <c r="B116" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="C116" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D116" s="15" t="s">
+        <v>397</v>
+      </c>
       <c r="E116" s="14"/>
-      <c r="F116" s="14"/>
+      <c r="F116" s="14" t="s">
+        <v>115</v>
+      </c>
       <c r="G116" s="14"/>
       <c r="H116" s="14"/>
-      <c r="I116" s="14"/>
+      <c r="I116" s="14" t="s">
+        <v>393</v>
+      </c>
       <c r="J116" s="14"/>
       <c r="K116" s="14"/>
       <c r="L116" s="14"/>
@@ -5877,53 +5890,41 @@
       <c r="Z119" s="14"/>
       <c r="AA119" s="14"/>
     </row>
-    <row r="121" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="14" t="s">
-        <v>275</v>
-      </c>
-      <c r="B121" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="C121" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="D121" s="14"/>
-      <c r="E121" s="14"/>
-      <c r="F121" s="14"/>
-      <c r="G121" s="14"/>
-      <c r="H121" s="14"/>
-      <c r="I121" s="14"/>
-      <c r="J121" s="15" t="s">
-        <v>281</v>
-      </c>
-      <c r="K121" s="15" t="s">
-        <v>282</v>
-      </c>
-      <c r="L121" s="15" t="s">
-        <v>283</v>
-      </c>
-      <c r="M121" s="14"/>
-      <c r="N121" s="14"/>
-      <c r="O121" s="14"/>
-      <c r="P121" s="14"/>
-      <c r="Q121" s="14"/>
-      <c r="R121" s="14"/>
-      <c r="S121" s="14"/>
-      <c r="T121" s="14"/>
-      <c r="U121" s="14"/>
-      <c r="V121" s="14"/>
-      <c r="W121" s="14"/>
-      <c r="X121" s="14"/>
-      <c r="Y121" s="14"/>
-      <c r="Z121" s="14"/>
-      <c r="AA121" s="14"/>
+    <row r="120" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="14"/>
+      <c r="B120" s="14"/>
+      <c r="C120" s="14"/>
+      <c r="D120" s="15"/>
+      <c r="E120" s="14"/>
+      <c r="F120" s="14"/>
+      <c r="G120" s="14"/>
+      <c r="H120" s="14"/>
+      <c r="I120" s="14"/>
+      <c r="J120" s="14"/>
+      <c r="K120" s="14"/>
+      <c r="L120" s="14"/>
+      <c r="M120" s="14"/>
+      <c r="N120" s="14"/>
+      <c r="O120" s="14"/>
+      <c r="P120" s="14"/>
+      <c r="Q120" s="14"/>
+      <c r="R120" s="15"/>
+      <c r="S120" s="14"/>
+      <c r="T120" s="14"/>
+      <c r="U120" s="14"/>
+      <c r="V120" s="14"/>
+      <c r="W120" s="14"/>
+      <c r="X120" s="14"/>
+      <c r="Y120" s="14"/>
+      <c r="Z120" s="14"/>
+      <c r="AA120" s="14"/>
     </row>
     <row r="122" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="14" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B122" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C122" s="14" t="s">
         <v>140</v>
@@ -5938,10 +5939,10 @@
         <v>280</v>
       </c>
       <c r="K122" s="15" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="L122" s="15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="M122" s="14"/>
       <c r="N122" s="14"/>
@@ -5959,60 +5960,101 @@
       <c r="Z122" s="14"/>
       <c r="AA122" s="14"/>
     </row>
-    <row r="123" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="14" t="s">
-        <v>367</v>
+        <v>275</v>
       </c>
       <c r="B123" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C123" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="O123" s="15" t="s">
-        <v>370</v>
-      </c>
+      <c r="D123" s="14"/>
+      <c r="E123" s="14"/>
+      <c r="F123" s="14"/>
+      <c r="G123" s="14"/>
+      <c r="H123" s="14"/>
+      <c r="I123" s="14"/>
+      <c r="J123" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="K123" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="L123" s="15" t="s">
+        <v>283</v>
+      </c>
+      <c r="M123" s="14"/>
+      <c r="N123" s="14"/>
+      <c r="O123" s="14"/>
+      <c r="P123" s="14"/>
+      <c r="Q123" s="14"/>
+      <c r="R123" s="14"/>
+      <c r="S123" s="14"/>
+      <c r="T123" s="14"/>
+      <c r="U123" s="14"/>
+      <c r="V123" s="14"/>
+      <c r="W123" s="14"/>
+      <c r="X123" s="14"/>
+      <c r="Y123" s="14"/>
+      <c r="Z123" s="14"/>
+      <c r="AA123" s="14"/>
     </row>
     <row r="124" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A124" s="14" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B124" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C124" s="14" t="s">
         <v>140</v>
       </c>
       <c r="O124" s="15" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="125" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A125" s="14" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B125" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C125" s="14" t="s">
         <v>140</v>
       </c>
       <c r="O125" s="15" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="126" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A126" s="14" t="s">
+        <v>368</v>
+      </c>
+      <c r="B126" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="C126" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="O126" s="15" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="127" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A127" s="14" t="s">
+        <v>382</v>
+      </c>
+      <c r="B127" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="C127" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="M127" s="14" t="s">
         <v>383</v>
-      </c>
-      <c r="B126" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="C126" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="M126" s="14" t="s">
-        <v>384</v>
       </c>
     </row>
   </sheetData>
@@ -6100,10 +6142,10 @@
         <v>147</v>
       </c>
       <c r="R1" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="S1" s="17" t="s">
         <v>205</v>
-      </c>
-      <c r="S1" s="17" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
@@ -6219,7 +6261,7 @@
         <v>48</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>61</v>
@@ -6264,7 +6306,7 @@
         <v>50</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>3</v>
@@ -6370,7 +6412,7 @@
         <v>53</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C13" s="15"/>
       <c r="E13" s="15" t="s">
@@ -6605,7 +6647,7 @@
         <v>62</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C22" s="15"/>
       <c r="D22" s="14"/>
@@ -6623,7 +6665,7 @@
       <c r="L22" s="14"/>
       <c r="M22" s="14"/>
       <c r="N22" s="14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="O22" s="14"/>
       <c r="P22" s="14"/>
@@ -6782,7 +6824,7 @@
         <v>68</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>3</v>
@@ -6848,7 +6890,7 @@
         <v>36</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C30" s="15" t="s">
         <v>47</v>
@@ -7013,7 +7055,7 @@
         <v>74</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C35" s="15" t="s">
         <v>3</v>
@@ -7079,7 +7121,7 @@
         <v>76</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>3</v>
@@ -7112,7 +7154,7 @@
         <v>77</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C38" s="15" t="s">
         <v>3</v>
@@ -7145,7 +7187,7 @@
         <v>78</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C39" s="15" t="s">
         <v>3</v>
@@ -7211,7 +7253,7 @@
         <v>80</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C41" s="15" t="s">
         <v>47</v>
@@ -7244,7 +7286,7 @@
         <v>81</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C42" s="15" t="s">
         <v>3</v>
@@ -7277,7 +7319,7 @@
         <v>82</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C43" s="15" t="s">
         <v>3</v>
@@ -7310,7 +7352,7 @@
         <v>83</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C44" s="15" t="s">
         <v>3</v>
@@ -7343,7 +7385,7 @@
         <v>84</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C45" s="15" t="s">
         <v>47</v>
@@ -7376,7 +7418,7 @@
         <v>85</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C46" s="15" t="s">
         <v>47</v>
@@ -7408,7 +7450,7 @@
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A47" s="16" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B47" s="20" t="s">
         <v>143</v>
@@ -7426,7 +7468,7 @@
         <v>144</v>
       </c>
       <c r="P47" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q47" s="14" t="s">
         <v>148</v>
@@ -7434,7 +7476,7 @@
     </row>
     <row r="48" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B48" s="20" t="s">
         <v>143</v>
@@ -7461,7 +7503,7 @@
         <v>144</v>
       </c>
       <c r="P48" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q48" s="14" t="s">
         <v>148</v>
@@ -7471,10 +7513,10 @@
     </row>
     <row r="49" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>0</v>
@@ -7498,7 +7540,7 @@
         <v>144</v>
       </c>
       <c r="P49" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q49" s="14" t="s">
         <v>148</v>
@@ -7508,13 +7550,13 @@
     </row>
     <row r="50" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D50" s="16" t="s">
         <v>113</v>
@@ -7535,7 +7577,7 @@
         <v>144</v>
       </c>
       <c r="P50" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q50" s="14" t="s">
         <v>148</v>
@@ -7545,7 +7587,7 @@
     </row>
     <row r="51" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B51" s="20" t="s">
         <v>143</v>
@@ -7572,7 +7614,7 @@
         <v>144</v>
       </c>
       <c r="P51" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q51" s="14" t="s">
         <v>148</v>
@@ -7582,7 +7624,7 @@
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B52" s="20" t="s">
         <v>143</v>
@@ -7600,7 +7642,7 @@
         <v>144</v>
       </c>
       <c r="P52" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q52" s="14" t="s">
         <v>148</v>
@@ -7608,7 +7650,7 @@
     </row>
     <row r="53" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B53" s="20" t="s">
         <v>143</v>
@@ -7635,7 +7677,7 @@
         <v>144</v>
       </c>
       <c r="P53" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q53" s="14" t="s">
         <v>148</v>
@@ -7645,10 +7687,10 @@
     </row>
     <row r="54" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="16" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C54" s="16" t="s">
         <v>2</v>
@@ -7672,7 +7714,7 @@
         <v>144</v>
       </c>
       <c r="P54" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q54" s="14" t="s">
         <v>148</v>
@@ -7682,10 +7724,10 @@
     </row>
     <row r="55" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="16" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C55" s="16" t="s">
         <v>46</v>
@@ -7709,7 +7751,7 @@
         <v>144</v>
       </c>
       <c r="P55" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q55" s="14" t="s">
         <v>148</v>
@@ -7721,10 +7763,10 @@
     </row>
     <row r="56" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C56" s="16" t="s">
         <v>46</v>
@@ -7748,7 +7790,7 @@
         <v>144</v>
       </c>
       <c r="P56" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q56" s="14" t="s">
         <v>148</v>
@@ -7760,10 +7802,10 @@
     </row>
     <row r="57" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B57" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C57" s="16" t="s">
         <v>47</v>
@@ -7787,7 +7829,7 @@
         <v>144</v>
       </c>
       <c r="P57" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q57" s="14" t="s">
         <v>148</v>
@@ -7799,10 +7841,10 @@
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58" s="16" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B58" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C58" s="15" t="s">
         <v>47</v>
@@ -7817,7 +7859,7 @@
         <v>144</v>
       </c>
       <c r="P58" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q58" s="14" t="s">
         <v>148</v>
@@ -7825,10 +7867,10 @@
     </row>
     <row r="59" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B59" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C59" s="15" t="s">
         <v>47</v>
@@ -7852,7 +7894,7 @@
         <v>144</v>
       </c>
       <c r="P59" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q59" s="14" t="s">
         <v>148</v>
@@ -7864,10 +7906,10 @@
     </row>
     <row r="60" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C60" s="15" t="s">
         <v>47</v>
@@ -7891,7 +7933,7 @@
         <v>144</v>
       </c>
       <c r="P60" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q60" s="14" t="s">
         <v>148</v>
@@ -7901,7 +7943,7 @@
     </row>
     <row r="61" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="16" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B61" s="20" t="s">
         <v>143</v>
@@ -7930,7 +7972,7 @@
     </row>
     <row r="62" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="16" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B62" s="20" t="s">
         <v>143</v>
@@ -7957,7 +7999,7 @@
         <v>144</v>
       </c>
       <c r="P62" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q62" s="14" t="s">
         <v>148</v>
@@ -7967,10 +8009,10 @@
     </row>
     <row r="63" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="16" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B63" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C63" s="15" t="s">
         <v>0</v>
@@ -7994,7 +8036,7 @@
         <v>144</v>
       </c>
       <c r="P63" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q63" s="14" t="s">
         <v>148</v>
@@ -8004,7 +8046,7 @@
     </row>
     <row r="64" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="16" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B64" s="20" t="s">
         <v>143</v>
@@ -8031,7 +8073,7 @@
         <v>144</v>
       </c>
       <c r="P64" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q64" s="14" t="s">
         <v>148</v>
@@ -8041,7 +8083,7 @@
     </row>
     <row r="65" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="16" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B65" s="20" t="s">
         <v>143</v>
@@ -8068,7 +8110,7 @@
         <v>144</v>
       </c>
       <c r="P65" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q65" s="14" t="s">
         <v>148</v>
@@ -8078,10 +8120,10 @@
     </row>
     <row r="66" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="16" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>150</v>
+        <v>402</v>
       </c>
       <c r="C66" s="16" t="s">
         <v>0</v>
@@ -8105,7 +8147,7 @@
         <v>144</v>
       </c>
       <c r="P66" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q66" s="14" t="s">
         <v>148</v>
@@ -8136,10 +8178,10 @@
     </row>
     <row r="69" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A69" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B69" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C69" s="15" t="s">
         <v>61</v>
@@ -8157,10 +8199,10 @@
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C70" s="15" t="s">
         <v>61</v>
@@ -8178,10 +8220,10 @@
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A71" s="15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B71" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C71" s="15" t="s">
         <v>61</v>
@@ -8202,10 +8244,10 @@
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A72" s="15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B72" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C72" s="15" t="s">
         <v>61</v>
@@ -8223,10 +8265,10 @@
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A73" s="15" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B73" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C73" s="15" t="s">
         <v>61</v>
@@ -8244,10 +8286,10 @@
     </row>
     <row r="74" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A74" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B74" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C74" s="15" t="s">
         <v>3</v>
@@ -8265,10 +8307,10 @@
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A75" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B75" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C75" s="15" t="s">
         <v>61</v>
@@ -8286,10 +8328,10 @@
     </row>
     <row r="76" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C76" s="15" t="s">
         <v>61</v>
@@ -8319,10 +8361,10 @@
     </row>
     <row r="77" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A77" s="15" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B77" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C77" s="15" t="s">
         <v>61</v>
@@ -8343,10 +8385,10 @@
     </row>
     <row r="78" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A78" s="15" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B78" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C78" s="15" t="s">
         <v>61</v>
@@ -8364,10 +8406,10 @@
     </row>
     <row r="79" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A79" s="15" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B79" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C79" s="15" t="s">
         <v>3</v>
@@ -8385,10 +8427,10 @@
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A80" s="15" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B80" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C80" s="15" t="s">
         <v>61</v>
@@ -8407,10 +8449,10 @@
     </row>
     <row r="81" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A81" s="15" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B81" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C81" s="15" t="s">
         <v>61</v>
@@ -8429,10 +8471,10 @@
     </row>
     <row r="82" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="15" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B82" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C82" s="15" t="s">
         <v>61</v>
@@ -8462,10 +8504,10 @@
     </row>
     <row r="83" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B83" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C83" s="15" t="s">
         <v>61</v>
@@ -8486,10 +8528,10 @@
     </row>
     <row r="84" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A84" s="15" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B84" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C84" s="15" t="s">
         <v>3</v>
@@ -8507,10 +8549,10 @@
     </row>
     <row r="85" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A85" s="15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B85" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C85" s="15" t="s">
         <v>3</v>
@@ -8528,10 +8570,10 @@
     </row>
     <row r="86" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A86" s="15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B86" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C86" s="15" t="s">
         <v>3</v>
@@ -8549,10 +8591,10 @@
     </row>
     <row r="87" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A87" s="15" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B87" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C87" s="15" t="s">
         <v>3</v>
@@ -8570,10 +8612,10 @@
     </row>
     <row r="88" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A88" s="15" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B88" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C88" s="15" t="s">
         <v>3</v>
@@ -8591,10 +8633,10 @@
     </row>
     <row r="89" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A89" s="15" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B89" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C89" s="15" t="s">
         <v>3</v>
@@ -8612,10 +8654,10 @@
     </row>
     <row r="90" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A90" s="15" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B90" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C90" s="15" t="s">
         <v>3</v>
@@ -8632,10 +8674,10 @@
     </row>
     <row r="91" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A91" s="15" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B91" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C91" s="15" t="s">
         <v>3</v>
@@ -8652,10 +8694,10 @@
     </row>
     <row r="92" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A92" s="15" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B92" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C92" s="15" t="s">
         <v>3</v>
@@ -8672,10 +8714,10 @@
     </row>
     <row r="93" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A93" s="15" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B93" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C93" s="15" t="s">
         <v>3</v>
@@ -8692,10 +8734,10 @@
     </row>
     <row r="94" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A94" s="15" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B94" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C94" s="15" t="s">
         <v>46</v>
@@ -8712,10 +8754,10 @@
     </row>
     <row r="95" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="15" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B95" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C95" s="15" t="s">
         <v>46</v>
@@ -8745,10 +8787,10 @@
     </row>
     <row r="96" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="15" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B96" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C96" s="15" t="s">
         <v>46</v>
@@ -8778,10 +8820,10 @@
     </row>
     <row r="97" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="15" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B97" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C97" s="15" t="s">
         <v>2</v>
@@ -8815,10 +8857,10 @@
     </row>
     <row r="98" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="15" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B98" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C98" s="14"/>
       <c r="D98" s="14"/>
@@ -8848,10 +8890,10 @@
     </row>
     <row r="99" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="15" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B99" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D99" s="14"/>
       <c r="E99" s="15" t="s">

</xml_diff>

<commit_message>
updated the scripts for normal item putaway
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24131"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB0F1E7A-9A62-4929-B892-214EC26867CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B57F611B-1B3F-432F-AF90-90D8392A017A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1672" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1684" uniqueCount="440">
   <si>
     <t>1</t>
   </si>
@@ -1328,6 +1328,15 @@
   </si>
   <si>
     <t>Normal</t>
+  </si>
+  <si>
+    <t>FG-200000-00</t>
+  </si>
+  <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>QSC_IBScenario038</t>
   </si>
 </sst>
 </file>
@@ -1843,7 +1852,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE339"/>
+  <dimension ref="A1:AE340"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="14" customWidth="1"/>
@@ -3360,8 +3369,8 @@
       </c>
     </row>
     <row r="42" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
-        <v>354</v>
+      <c r="A42" s="15" t="s">
+        <v>439</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>108</v>
@@ -3370,7 +3379,7 @@
         <v>136</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E42" s="14"/>
       <c r="F42" s="14" t="s">
@@ -3400,15 +3409,27 @@
       <c r="AB42" s="14"/>
       <c r="AC42" s="14"/>
       <c r="AD42" s="14"/>
-      <c r="AE42" s="14"/>
+      <c r="AE42" s="14" t="s">
+        <v>436</v>
+      </c>
     </row>
     <row r="43" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="15"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="18"/>
+      <c r="A43" s="14" t="s">
+        <v>354</v>
+      </c>
+      <c r="B43" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="D43" s="23" t="s">
+        <v>86</v>
+      </c>
       <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
+      <c r="F43" s="14" t="s">
+        <v>424</v>
+      </c>
       <c r="G43" s="14"/>
       <c r="H43" s="14"/>
       <c r="I43" s="14"/>
@@ -3436,18 +3457,10 @@
       <c r="AE43" s="14"/>
     </row>
     <row r="44" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="B44" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="C44" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="D44" s="23" t="s">
-        <v>160</v>
-      </c>
+      <c r="A44" s="15"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="18"/>
       <c r="E44" s="14"/>
       <c r="F44" s="14"/>
       <c r="G44" s="14"/>
@@ -3471,20 +3484,14 @@
       <c r="Y44" s="14"/>
       <c r="Z44" s="14"/>
       <c r="AA44" s="14"/>
-      <c r="AB44" s="14" t="s">
-        <v>399</v>
-      </c>
-      <c r="AC44" s="14" t="s">
-        <v>397</v>
-      </c>
-      <c r="AD44" s="14" t="s">
-        <v>398</v>
-      </c>
+      <c r="AB44" s="14"/>
+      <c r="AC44" s="14"/>
+      <c r="AD44" s="14"/>
       <c r="AE44" s="14"/>
     </row>
     <row r="45" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>108</v>
@@ -3493,7 +3500,7 @@
         <v>136</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="E45" s="14"/>
       <c r="F45" s="14"/>
@@ -3522,16 +3529,16 @@
         <v>399</v>
       </c>
       <c r="AC45" s="14" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="AD45" s="14" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="AE45" s="14"/>
     </row>
     <row r="46" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B46" s="14" t="s">
         <v>108</v>
@@ -3540,7 +3547,7 @@
         <v>136</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E46" s="14"/>
       <c r="F46" s="14"/>
@@ -3578,7 +3585,7 @@
     </row>
     <row r="47" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B47" s="14" t="s">
         <v>108</v>
@@ -3587,7 +3594,7 @@
         <v>136</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E47" s="14"/>
       <c r="F47" s="14"/>
@@ -3601,9 +3608,7 @@
       <c r="N47" s="14"/>
       <c r="O47" s="14"/>
       <c r="P47" s="14"/>
-      <c r="Q47" s="14" t="s">
-        <v>157</v>
-      </c>
+      <c r="Q47" s="14"/>
       <c r="R47" s="14"/>
       <c r="S47" s="14"/>
       <c r="T47" s="14"/>
@@ -3627,7 +3632,7 @@
     </row>
     <row r="48" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="B48" s="14" t="s">
         <v>108</v>
@@ -3676,7 +3681,7 @@
     </row>
     <row r="49" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="B49" s="14" t="s">
         <v>108</v>
@@ -3685,7 +3690,7 @@
         <v>136</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E49" s="14"/>
       <c r="F49" s="14"/>
@@ -3700,7 +3705,7 @@
       <c r="O49" s="14"/>
       <c r="P49" s="14"/>
       <c r="Q49" s="14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="R49" s="14"/>
       <c r="S49" s="14"/>
@@ -3725,7 +3730,7 @@
     </row>
     <row r="50" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B50" s="14" t="s">
         <v>108</v>
@@ -3734,7 +3739,7 @@
         <v>136</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="E50" s="14"/>
       <c r="F50" s="14"/>
@@ -3774,7 +3779,7 @@
     </row>
     <row r="51" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>188</v>
+        <v>175</v>
       </c>
       <c r="B51" s="14" t="s">
         <v>108</v>
@@ -3798,7 +3803,7 @@
       <c r="O51" s="14"/>
       <c r="P51" s="14"/>
       <c r="Q51" s="14" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="R51" s="14"/>
       <c r="S51" s="14"/>
@@ -3823,7 +3828,7 @@
     </row>
     <row r="52" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B52" s="14" t="s">
         <v>108</v>
@@ -3832,7 +3837,7 @@
         <v>136</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>192</v>
+        <v>174</v>
       </c>
       <c r="E52" s="14"/>
       <c r="F52" s="14"/>
@@ -3846,7 +3851,9 @@
       <c r="N52" s="14"/>
       <c r="O52" s="14"/>
       <c r="P52" s="14"/>
-      <c r="Q52" s="14"/>
+      <c r="Q52" s="14" t="s">
+        <v>157</v>
+      </c>
       <c r="R52" s="14"/>
       <c r="S52" s="14"/>
       <c r="T52" s="14"/>
@@ -3870,7 +3877,7 @@
     </row>
     <row r="53" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B53" s="14" t="s">
         <v>108</v>
@@ -3879,7 +3886,7 @@
         <v>136</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E53" s="14"/>
       <c r="F53" s="14"/>
@@ -3917,7 +3924,7 @@
     </row>
     <row r="54" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B54" s="14" t="s">
         <v>108</v>
@@ -3926,7 +3933,7 @@
         <v>136</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E54" s="14"/>
       <c r="F54" s="14"/>
@@ -3964,7 +3971,7 @@
     </row>
     <row r="55" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="B55" s="14" t="s">
         <v>108</v>
@@ -3973,7 +3980,7 @@
         <v>136</v>
       </c>
       <c r="D55" s="23" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E55" s="14"/>
       <c r="F55" s="14"/>
@@ -4011,7 +4018,7 @@
     </row>
     <row r="56" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>260</v>
+        <v>202</v>
       </c>
       <c r="B56" s="14" t="s">
         <v>108</v>
@@ -4020,7 +4027,7 @@
         <v>136</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="E56" s="14"/>
       <c r="F56" s="14"/>
@@ -4036,12 +4043,8 @@
       <c r="P56" s="14"/>
       <c r="Q56" s="14"/>
       <c r="R56" s="14"/>
-      <c r="S56" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T56" s="14" t="s">
-        <v>302</v>
-      </c>
+      <c r="S56" s="14"/>
+      <c r="T56" s="14"/>
       <c r="U56" s="14"/>
       <c r="V56" s="14"/>
       <c r="W56" s="14"/>
@@ -4062,7 +4065,7 @@
     </row>
     <row r="57" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B57" s="14" t="s">
         <v>108</v>
@@ -4090,8 +4093,8 @@
       <c r="S57" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="T57" s="15" t="s">
-        <v>303</v>
+      <c r="T57" s="14" t="s">
+        <v>302</v>
       </c>
       <c r="U57" s="14"/>
       <c r="V57" s="14"/>
@@ -4113,7 +4116,7 @@
     </row>
     <row r="58" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B58" s="14" t="s">
         <v>108</v>
@@ -4141,8 +4144,8 @@
       <c r="S58" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="T58" s="24" t="s">
-        <v>304</v>
+      <c r="T58" s="15" t="s">
+        <v>303</v>
       </c>
       <c r="U58" s="14"/>
       <c r="V58" s="14"/>
@@ -4164,7 +4167,7 @@
     </row>
     <row r="59" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B59" s="14" t="s">
         <v>108</v>
@@ -4173,7 +4176,7 @@
         <v>136</v>
       </c>
       <c r="D59" s="23" t="s">
-        <v>268</v>
+        <v>165</v>
       </c>
       <c r="E59" s="14"/>
       <c r="F59" s="14"/>
@@ -4187,15 +4190,13 @@
       <c r="N59" s="14"/>
       <c r="O59" s="14"/>
       <c r="P59" s="14"/>
-      <c r="Q59" s="14" t="s">
-        <v>158</v>
-      </c>
+      <c r="Q59" s="14"/>
       <c r="R59" s="14"/>
       <c r="S59" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="T59" s="14" t="s">
-        <v>302</v>
+      <c r="T59" s="24" t="s">
+        <v>304</v>
       </c>
       <c r="U59" s="14"/>
       <c r="V59" s="14"/>
@@ -4217,7 +4218,7 @@
     </row>
     <row r="60" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B60" s="14" t="s">
         <v>108</v>
@@ -4248,7 +4249,7 @@
         <v>0</v>
       </c>
       <c r="T60" s="14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="U60" s="14"/>
       <c r="V60" s="14"/>
@@ -4270,7 +4271,7 @@
     </row>
     <row r="61" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B61" s="14" t="s">
         <v>108</v>
@@ -4300,7 +4301,9 @@
       <c r="S61" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="T61" s="14"/>
+      <c r="T61" s="14" t="s">
+        <v>303</v>
+      </c>
       <c r="U61" s="14"/>
       <c r="V61" s="14"/>
       <c r="W61" s="14"/>
@@ -4321,7 +4324,7 @@
     </row>
     <row r="62" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>396</v>
+        <v>265</v>
       </c>
       <c r="B62" s="14" t="s">
         <v>108</v>
@@ -4330,7 +4333,7 @@
         <v>136</v>
       </c>
       <c r="D62" s="23" t="s">
-        <v>160</v>
+        <v>268</v>
       </c>
       <c r="E62" s="14"/>
       <c r="F62" s="14"/>
@@ -4363,16 +4366,16 @@
         <v>399</v>
       </c>
       <c r="AC62" s="14" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="AD62" s="14" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="AE62" s="14"/>
     </row>
     <row r="63" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="B63" s="14" t="s">
         <v>108</v>
@@ -4395,9 +4398,13 @@
       <c r="N63" s="14"/>
       <c r="O63" s="14"/>
       <c r="P63" s="14"/>
-      <c r="Q63" s="14"/>
+      <c r="Q63" s="14" t="s">
+        <v>158</v>
+      </c>
       <c r="R63" s="14"/>
-      <c r="S63" s="14"/>
+      <c r="S63" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="T63" s="14"/>
       <c r="U63" s="14"/>
       <c r="V63" s="14"/>
@@ -4419,7 +4426,7 @@
     </row>
     <row r="64" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B64" s="14" t="s">
         <v>108</v>
@@ -4428,7 +4435,7 @@
         <v>136</v>
       </c>
       <c r="D64" s="23" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="E64" s="14"/>
       <c r="F64" s="14"/>
@@ -4457,16 +4464,16 @@
         <v>399</v>
       </c>
       <c r="AC64" s="14" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="AD64" s="14" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="AE64" s="14"/>
     </row>
     <row r="65" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B65" s="14" t="s">
         <v>108</v>
@@ -4475,7 +4482,7 @@
         <v>136</v>
       </c>
       <c r="D65" s="23" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="E65" s="14"/>
       <c r="F65" s="14"/>
@@ -4501,19 +4508,19 @@
       <c r="Z65" s="14"/>
       <c r="AA65" s="14"/>
       <c r="AB65" s="14" t="s">
-        <v>412</v>
+        <v>399</v>
       </c>
       <c r="AC65" s="14" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="AD65" s="14" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="AE65" s="14"/>
     </row>
     <row r="66" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B66" s="14" t="s">
         <v>108</v>
@@ -4522,7 +4529,7 @@
         <v>136</v>
       </c>
       <c r="D66" s="23" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="E66" s="14"/>
       <c r="F66" s="14"/>
@@ -4551,16 +4558,16 @@
         <v>412</v>
       </c>
       <c r="AC66" s="14" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="AD66" s="14" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="AE66" s="14"/>
     </row>
     <row r="67" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B67" s="14" t="s">
         <v>108</v>
@@ -4569,7 +4576,7 @@
         <v>136</v>
       </c>
       <c r="D67" s="23" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="E67" s="14"/>
       <c r="F67" s="14"/>
@@ -4598,16 +4605,16 @@
         <v>412</v>
       </c>
       <c r="AC67" s="14" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="AD67" s="14" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="AE67" s="14"/>
     </row>
     <row r="68" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B68" s="14" t="s">
         <v>108</v>
@@ -4616,7 +4623,7 @@
         <v>136</v>
       </c>
       <c r="D68" s="23" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="E68" s="14"/>
       <c r="F68" s="14"/>
@@ -4642,19 +4649,19 @@
       <c r="Z68" s="14"/>
       <c r="AA68" s="14"/>
       <c r="AB68" s="14" t="s">
-        <v>399</v>
+        <v>412</v>
       </c>
       <c r="AC68" s="14" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="AD68" s="14" t="s">
-        <v>399</v>
+        <v>410</v>
       </c>
       <c r="AE68" s="14"/>
     </row>
     <row r="69" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="14" t="s">
-        <v>413</v>
+        <v>405</v>
       </c>
       <c r="B69" s="14" t="s">
         <v>108</v>
@@ -4663,7 +4670,7 @@
         <v>136</v>
       </c>
       <c r="D69" s="23" t="s">
-        <v>416</v>
+        <v>166</v>
       </c>
       <c r="E69" s="14"/>
       <c r="F69" s="14"/>
@@ -4700,10 +4707,18 @@
       <c r="AE69" s="14"/>
     </row>
     <row r="70" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="14"/>
-      <c r="B70" s="14"/>
-      <c r="C70" s="14"/>
-      <c r="D70" s="23"/>
+      <c r="A70" s="14" t="s">
+        <v>413</v>
+      </c>
+      <c r="B70" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C70" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="D70" s="23" t="s">
+        <v>416</v>
+      </c>
       <c r="E70" s="14"/>
       <c r="F70" s="14"/>
       <c r="G70" s="14"/>
@@ -4727,25 +4742,23 @@
       <c r="Y70" s="14"/>
       <c r="Z70" s="14"/>
       <c r="AA70" s="14"/>
-      <c r="AB70" s="14"/>
-      <c r="AC70" s="14"/>
-      <c r="AD70" s="14"/>
+      <c r="AB70" s="14" t="s">
+        <v>399</v>
+      </c>
+      <c r="AC70" s="14" t="s">
+        <v>399</v>
+      </c>
+      <c r="AD70" s="14" t="s">
+        <v>399</v>
+      </c>
       <c r="AE70" s="14"/>
     </row>
     <row r="71" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="14" t="s">
-        <v>305</v>
-      </c>
-      <c r="B71" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="C71" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="D71" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="E71" s="15"/>
+      <c r="A71" s="14"/>
+      <c r="B71" s="14"/>
+      <c r="C71" s="14"/>
+      <c r="D71" s="23"/>
+      <c r="E71" s="14"/>
       <c r="F71" s="14"/>
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
@@ -4775,7 +4788,7 @@
     </row>
     <row r="72" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="14" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B72" s="14" t="s">
         <v>108</v>
@@ -4784,9 +4797,9 @@
         <v>136</v>
       </c>
       <c r="D72" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="E72" s="14"/>
+        <v>0</v>
+      </c>
+      <c r="E72" s="15"/>
       <c r="F72" s="14"/>
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
@@ -4816,7 +4829,7 @@
     </row>
     <row r="73" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="14" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B73" s="14" t="s">
         <v>108</v>
@@ -4825,17 +4838,13 @@
         <v>136</v>
       </c>
       <c r="D73" s="18" t="s">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="E73" s="14"/>
-      <c r="F73" s="14" t="s">
-        <v>424</v>
-      </c>
+      <c r="F73" s="14"/>
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
-      <c r="I73" s="14" t="s">
-        <v>129</v>
-      </c>
+      <c r="I73" s="14"/>
       <c r="J73" s="14"/>
       <c r="K73" s="14"/>
       <c r="L73" s="14"/>
@@ -4861,7 +4870,7 @@
     </row>
     <row r="74" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="14" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B74" s="14" t="s">
         <v>108</v>
@@ -4870,7 +4879,7 @@
         <v>136</v>
       </c>
       <c r="D74" s="18" t="s">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="E74" s="14"/>
       <c r="F74" s="14" t="s">
@@ -4879,7 +4888,7 @@
       <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="14" t="s">
-        <v>381</v>
+        <v>129</v>
       </c>
       <c r="J74" s="14"/>
       <c r="K74" s="14"/>
@@ -4906,7 +4915,7 @@
     </row>
     <row r="75" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
-        <v>345</v>
+        <v>308</v>
       </c>
       <c r="B75" s="14" t="s">
         <v>108</v>
@@ -4914,14 +4923,18 @@
       <c r="C75" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="D75" s="25" t="s">
-        <v>349</v>
+      <c r="D75" s="18" t="s">
+        <v>119</v>
       </c>
       <c r="E75" s="14"/>
-      <c r="F75" s="14"/>
+      <c r="F75" s="14" t="s">
+        <v>424</v>
+      </c>
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
-      <c r="I75" s="14"/>
+      <c r="I75" s="14" t="s">
+        <v>381</v>
+      </c>
       <c r="J75" s="14"/>
       <c r="K75" s="14"/>
       <c r="L75" s="14"/>
@@ -4947,7 +4960,7 @@
     </row>
     <row r="76" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="14" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B76" s="14" t="s">
         <v>108</v>
@@ -4955,8 +4968,8 @@
       <c r="C76" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="D76" s="18" t="s">
-        <v>352</v>
+      <c r="D76" s="25" t="s">
+        <v>349</v>
       </c>
       <c r="E76" s="14"/>
       <c r="F76" s="14"/>
@@ -4988,7 +5001,7 @@
     </row>
     <row r="77" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B77" s="14" t="s">
         <v>108</v>
@@ -4996,8 +5009,8 @@
       <c r="C77" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="D77" s="25" t="s">
-        <v>349</v>
+      <c r="D77" s="18" t="s">
+        <v>352</v>
       </c>
       <c r="E77" s="14"/>
       <c r="F77" s="14"/>
@@ -5029,7 +5042,7 @@
     </row>
     <row r="78" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="14" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B78" s="14" t="s">
         <v>108</v>
@@ -5037,8 +5050,8 @@
       <c r="C78" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="D78" s="18" t="s">
-        <v>352</v>
+      <c r="D78" s="25" t="s">
+        <v>349</v>
       </c>
       <c r="E78" s="14"/>
       <c r="F78" s="14"/>
@@ -5070,7 +5083,7 @@
     </row>
     <row r="79" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="14" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B79" s="14" t="s">
         <v>108</v>
@@ -5078,7 +5091,9 @@
       <c r="C79" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="D79" s="18"/>
+      <c r="D79" s="18" t="s">
+        <v>352</v>
+      </c>
       <c r="E79" s="14"/>
       <c r="F79" s="14"/>
       <c r="G79" s="14"/>
@@ -5108,9 +5123,15 @@
       <c r="AE79" s="14"/>
     </row>
     <row r="80" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="14"/>
-      <c r="B80" s="14"/>
-      <c r="C80" s="14"/>
+      <c r="A80" s="14" t="s">
+        <v>353</v>
+      </c>
+      <c r="B80" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C80" s="14" t="s">
+        <v>136</v>
+      </c>
       <c r="D80" s="18"/>
       <c r="E80" s="14"/>
       <c r="F80" s="14"/>
@@ -5141,30 +5162,18 @@
       <c r="AE80" s="14"/>
     </row>
     <row r="81" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="12" t="s">
-        <v>368</v>
-      </c>
-      <c r="B81" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="C81" s="12" t="s">
-        <v>136</v>
-      </c>
+      <c r="A81" s="14"/>
+      <c r="B81" s="14"/>
+      <c r="C81" s="14"/>
       <c r="D81" s="18"/>
       <c r="E81" s="14"/>
       <c r="F81" s="14"/>
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
       <c r="I81" s="14"/>
-      <c r="J81" s="13" t="s">
-        <v>426</v>
-      </c>
-      <c r="K81" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="L81" s="14" t="s">
-        <v>427</v>
-      </c>
+      <c r="J81" s="14"/>
+      <c r="K81" s="14"/>
+      <c r="L81" s="14"/>
       <c r="M81" s="14"/>
       <c r="N81" s="14"/>
       <c r="O81" s="14"/>
@@ -5187,7 +5196,7 @@
     </row>
     <row r="82" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="12" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B82" s="12" t="s">
         <v>108</v>
@@ -5201,15 +5210,19 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="14"/>
-      <c r="J82" s="14"/>
-      <c r="K82" s="14"/>
-      <c r="L82" s="12"/>
-      <c r="M82" s="12" t="s">
-        <v>418</v>
-      </c>
-      <c r="N82" s="12"/>
-      <c r="O82" s="12"/>
-      <c r="P82" s="12"/>
+      <c r="J82" s="13" t="s">
+        <v>426</v>
+      </c>
+      <c r="K82" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="L82" s="14" t="s">
+        <v>427</v>
+      </c>
+      <c r="M82" s="14"/>
+      <c r="N82" s="14"/>
+      <c r="O82" s="14"/>
+      <c r="P82" s="14"/>
       <c r="Q82" s="14"/>
       <c r="R82" s="14"/>
       <c r="S82" s="14"/>
@@ -5228,7 +5241,7 @@
     </row>
     <row r="83" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="12" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B83" s="12" t="s">
         <v>108</v>
@@ -5245,10 +5258,10 @@
       <c r="J83" s="14"/>
       <c r="K83" s="14"/>
       <c r="L83" s="12"/>
-      <c r="M83" s="12"/>
-      <c r="N83" s="12" t="s">
-        <v>431</v>
-      </c>
+      <c r="M83" s="12" t="s">
+        <v>418</v>
+      </c>
+      <c r="N83" s="12"/>
       <c r="O83" s="12"/>
       <c r="P83" s="12"/>
       <c r="Q83" s="14"/>
@@ -5269,7 +5282,7 @@
     </row>
     <row r="84" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="12" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B84" s="12" t="s">
         <v>108</v>
@@ -5287,10 +5300,10 @@
       <c r="K84" s="14"/>
       <c r="L84" s="12"/>
       <c r="M84" s="12"/>
-      <c r="N84" s="12"/>
-      <c r="O84" s="12" t="s">
-        <v>428</v>
-      </c>
+      <c r="N84" s="12" t="s">
+        <v>431</v>
+      </c>
+      <c r="O84" s="12"/>
       <c r="P84" s="12"/>
       <c r="Q84" s="14"/>
       <c r="R84" s="14"/>
@@ -5310,7 +5323,7 @@
     </row>
     <row r="85" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="12" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B85" s="12" t="s">
         <v>108</v>
@@ -5329,10 +5342,10 @@
       <c r="L85" s="12"/>
       <c r="M85" s="12"/>
       <c r="N85" s="12"/>
-      <c r="O85" s="12"/>
-      <c r="P85" s="13" t="s">
-        <v>429</v>
-      </c>
+      <c r="O85" s="12" t="s">
+        <v>428</v>
+      </c>
+      <c r="P85" s="12"/>
       <c r="Q85" s="14"/>
       <c r="R85" s="14"/>
       <c r="S85" s="14"/>
@@ -5350,10 +5363,16 @@
       <c r="AE85" s="14"/>
     </row>
     <row r="86" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="14"/>
-      <c r="B86" s="14"/>
-      <c r="C86" s="14"/>
-      <c r="D86" s="23"/>
+      <c r="A86" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="B86" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C86" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D86" s="18"/>
       <c r="E86" s="14"/>
       <c r="F86" s="14"/>
       <c r="G86" s="14"/>
@@ -5361,11 +5380,13 @@
       <c r="I86" s="14"/>
       <c r="J86" s="14"/>
       <c r="K86" s="14"/>
-      <c r="L86" s="14"/>
-      <c r="M86" s="14"/>
-      <c r="N86" s="14"/>
-      <c r="O86" s="14"/>
-      <c r="P86" s="14"/>
+      <c r="L86" s="12"/>
+      <c r="M86" s="12"/>
+      <c r="N86" s="12"/>
+      <c r="O86" s="12"/>
+      <c r="P86" s="13" t="s">
+        <v>429</v>
+      </c>
       <c r="Q86" s="14"/>
       <c r="R86" s="14"/>
       <c r="S86" s="14"/>
@@ -5382,62 +5403,42 @@
       <c r="AD86" s="14"/>
       <c r="AE86" s="14"/>
     </row>
-    <row r="87" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="12" t="s">
-        <v>309</v>
-      </c>
-      <c r="B87" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="C87" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="D87" s="12"/>
-      <c r="E87" s="12"/>
-      <c r="F87" s="12"/>
-      <c r="G87" s="12"/>
-      <c r="H87" s="12"/>
-      <c r="I87" s="12"/>
-      <c r="J87" s="12"/>
-      <c r="K87" s="12"/>
-      <c r="L87" s="12"/>
-      <c r="M87" s="12"/>
-      <c r="N87" s="12"/>
-      <c r="O87" s="12"/>
-      <c r="P87" s="12"/>
-      <c r="Q87" s="12"/>
-      <c r="R87" s="12"/>
-      <c r="S87" s="12"/>
-      <c r="T87" s="12"/>
-      <c r="U87" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="V87" s="13" t="s">
-        <v>311</v>
-      </c>
-      <c r="W87" s="12" t="s">
-        <v>312</v>
-      </c>
-      <c r="X87" s="12" t="s">
-        <v>313</v>
-      </c>
-      <c r="Y87" s="12" t="s">
-        <v>314</v>
-      </c>
-      <c r="Z87" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="AA87" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="AB87" s="12"/>
-      <c r="AC87" s="12"/>
-      <c r="AD87" s="12"/>
-      <c r="AE87" s="12"/>
+    <row r="87" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="14"/>
+      <c r="B87" s="14"/>
+      <c r="C87" s="14"/>
+      <c r="D87" s="23"/>
+      <c r="E87" s="14"/>
+      <c r="F87" s="14"/>
+      <c r="G87" s="14"/>
+      <c r="H87" s="14"/>
+      <c r="I87" s="14"/>
+      <c r="J87" s="14"/>
+      <c r="K87" s="14"/>
+      <c r="L87" s="14"/>
+      <c r="M87" s="14"/>
+      <c r="N87" s="14"/>
+      <c r="O87" s="14"/>
+      <c r="P87" s="14"/>
+      <c r="Q87" s="14"/>
+      <c r="R87" s="14"/>
+      <c r="S87" s="14"/>
+      <c r="T87" s="14"/>
+      <c r="U87" s="14"/>
+      <c r="V87" s="14"/>
+      <c r="W87" s="14"/>
+      <c r="X87" s="14"/>
+      <c r="Y87" s="14"/>
+      <c r="Z87" s="14"/>
+      <c r="AA87" s="14"/>
+      <c r="AB87" s="14"/>
+      <c r="AC87" s="14"/>
+      <c r="AD87" s="14"/>
+      <c r="AE87" s="14"/>
     </row>
     <row r="88" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="12" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="B88" s="12" t="s">
         <v>108</v>
@@ -5490,7 +5491,7 @@
     </row>
     <row r="89" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B89" s="12" t="s">
         <v>108</v>
@@ -5515,22 +5516,24 @@
       <c r="R89" s="12"/>
       <c r="S89" s="12"/>
       <c r="T89" s="12"/>
-      <c r="U89" s="12" t="s">
+      <c r="U89" s="13" t="s">
         <v>310</v>
       </c>
-      <c r="V89" s="12" t="s">
-        <v>317</v>
+      <c r="V89" s="13" t="s">
+        <v>311</v>
       </c>
       <c r="W89" s="12" t="s">
         <v>312</v>
       </c>
       <c r="X89" s="12" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="Y89" s="12" t="s">
         <v>314</v>
       </c>
-      <c r="Z89" s="12"/>
+      <c r="Z89" s="12" t="s">
+        <v>108</v>
+      </c>
       <c r="AA89" s="12" t="s">
         <v>136</v>
       </c>
@@ -5541,7 +5544,7 @@
     </row>
     <row r="90" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="12" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B90" s="12" t="s">
         <v>108</v>
@@ -5566,25 +5569,25 @@
       <c r="R90" s="12"/>
       <c r="S90" s="12"/>
       <c r="T90" s="12"/>
-      <c r="U90" s="13" t="s">
+      <c r="U90" s="12" t="s">
         <v>310</v>
       </c>
-      <c r="V90" s="13" t="s">
-        <v>320</v>
+      <c r="V90" s="12" t="s">
+        <v>317</v>
       </c>
       <c r="W90" s="12" t="s">
         <v>312</v>
       </c>
       <c r="X90" s="12" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="Y90" s="12" t="s">
         <v>314</v>
       </c>
-      <c r="Z90" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="AA90" s="12"/>
+      <c r="Z90" s="12"/>
+      <c r="AA90" s="12" t="s">
+        <v>136</v>
+      </c>
       <c r="AB90" s="12"/>
       <c r="AC90" s="12"/>
       <c r="AD90" s="12"/>
@@ -5592,7 +5595,7 @@
     </row>
     <row r="91" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="12" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B91" s="12" t="s">
         <v>108</v>
@@ -5617,25 +5620,25 @@
       <c r="R91" s="12"/>
       <c r="S91" s="12"/>
       <c r="T91" s="12"/>
-      <c r="U91" s="12" t="s">
+      <c r="U91" s="13" t="s">
         <v>310</v>
       </c>
-      <c r="V91" s="12" t="s">
-        <v>322</v>
+      <c r="V91" s="13" t="s">
+        <v>320</v>
       </c>
       <c r="W91" s="12" t="s">
         <v>312</v>
       </c>
-      <c r="X91" s="12"/>
+      <c r="X91" s="12" t="s">
+        <v>313</v>
+      </c>
       <c r="Y91" s="12" t="s">
         <v>314</v>
       </c>
       <c r="Z91" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="AA91" s="12" t="s">
-        <v>136</v>
-      </c>
+      <c r="AA91" s="12"/>
       <c r="AB91" s="12"/>
       <c r="AC91" s="12"/>
       <c r="AD91" s="12"/>
@@ -5643,7 +5646,7 @@
     </row>
     <row r="92" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="12" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B92" s="12" t="s">
         <v>108</v>
@@ -5668,16 +5671,16 @@
       <c r="R92" s="12"/>
       <c r="S92" s="12"/>
       <c r="T92" s="12"/>
-      <c r="U92" s="12"/>
+      <c r="U92" s="12" t="s">
+        <v>310</v>
+      </c>
       <c r="V92" s="12" t="s">
         <v>322</v>
       </c>
       <c r="W92" s="12" t="s">
         <v>312</v>
       </c>
-      <c r="X92" s="12" t="s">
-        <v>318</v>
-      </c>
+      <c r="X92" s="12"/>
       <c r="Y92" s="12" t="s">
         <v>314</v>
       </c>
@@ -5694,7 +5697,7 @@
     </row>
     <row r="93" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B93" s="12" t="s">
         <v>108</v>
@@ -5719,17 +5722,15 @@
       <c r="R93" s="12"/>
       <c r="S93" s="12"/>
       <c r="T93" s="12"/>
-      <c r="U93" s="13" t="s">
-        <v>325</v>
-      </c>
-      <c r="V93" s="13" t="s">
-        <v>326</v>
-      </c>
-      <c r="W93" s="13" t="s">
+      <c r="U93" s="12"/>
+      <c r="V93" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="W93" s="12" t="s">
         <v>312</v>
       </c>
       <c r="X93" s="12" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="Y93" s="12" t="s">
         <v>314</v>
@@ -5747,7 +5748,7 @@
     </row>
     <row r="94" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="12" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B94" s="12" t="s">
         <v>108</v>
@@ -5773,13 +5774,13 @@
       <c r="S94" s="12"/>
       <c r="T94" s="12"/>
       <c r="U94" s="13" t="s">
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="V94" s="13" t="s">
-        <v>311</v>
+        <v>326</v>
       </c>
       <c r="W94" s="13" t="s">
-        <v>328</v>
+        <v>312</v>
       </c>
       <c r="X94" s="12" t="s">
         <v>313</v>
@@ -5800,7 +5801,7 @@
     </row>
     <row r="95" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B95" s="12" t="s">
         <v>108</v>
@@ -5825,26 +5826,26 @@
       <c r="R95" s="12"/>
       <c r="S95" s="12"/>
       <c r="T95" s="12"/>
-      <c r="U95" s="12" t="s">
+      <c r="U95" s="13" t="s">
         <v>310</v>
       </c>
-      <c r="V95" s="12" t="s">
+      <c r="V95" s="13" t="s">
         <v>311</v>
       </c>
-      <c r="W95" s="12" t="s">
-        <v>312</v>
+      <c r="W95" s="13" t="s">
+        <v>328</v>
       </c>
       <c r="X95" s="12" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="Y95" s="12" t="s">
         <v>314</v>
       </c>
       <c r="Z95" s="12" t="s">
-        <v>176</v>
+        <v>108</v>
       </c>
       <c r="AA95" s="12" t="s">
-        <v>330</v>
+        <v>136</v>
       </c>
       <c r="AB95" s="12"/>
       <c r="AC95" s="12"/>
@@ -5853,7 +5854,7 @@
     </row>
     <row r="96" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="12" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B96" s="12" t="s">
         <v>108</v>
@@ -5881,8 +5882,8 @@
       <c r="U96" s="12" t="s">
         <v>310</v>
       </c>
-      <c r="V96" s="13" t="s">
-        <v>332</v>
+      <c r="V96" s="12" t="s">
+        <v>311</v>
       </c>
       <c r="W96" s="12" t="s">
         <v>312</v>
@@ -5894,10 +5895,10 @@
         <v>314</v>
       </c>
       <c r="Z96" s="12" t="s">
-        <v>108</v>
+        <v>176</v>
       </c>
       <c r="AA96" s="12" t="s">
-        <v>136</v>
+        <v>330</v>
       </c>
       <c r="AB96" s="12"/>
       <c r="AC96" s="12"/>
@@ -5906,7 +5907,7 @@
     </row>
     <row r="97" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B97" s="12" t="s">
         <v>108</v>
@@ -5934,8 +5935,8 @@
       <c r="U97" s="12" t="s">
         <v>310</v>
       </c>
-      <c r="V97" s="12" t="s">
-        <v>334</v>
+      <c r="V97" s="13" t="s">
+        <v>332</v>
       </c>
       <c r="W97" s="12" t="s">
         <v>312</v>
@@ -5959,7 +5960,7 @@
     </row>
     <row r="98" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="12" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B98" s="12" t="s">
         <v>108</v>
@@ -5988,7 +5989,7 @@
         <v>310</v>
       </c>
       <c r="V98" s="12" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="W98" s="12" t="s">
         <v>312</v>
@@ -6000,7 +6001,7 @@
         <v>314</v>
       </c>
       <c r="Z98" s="12" t="s">
-        <v>330</v>
+        <v>108</v>
       </c>
       <c r="AA98" s="12" t="s">
         <v>136</v>
@@ -6012,7 +6013,7 @@
     </row>
     <row r="99" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="12" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B99" s="12" t="s">
         <v>108</v>
@@ -6047,13 +6048,13 @@
         <v>312</v>
       </c>
       <c r="X99" s="12" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="Y99" s="12" t="s">
         <v>314</v>
       </c>
       <c r="Z99" s="12" t="s">
-        <v>108</v>
+        <v>330</v>
       </c>
       <c r="AA99" s="12" t="s">
         <v>136</v>
@@ -6064,9 +6065,15 @@
       <c r="AE99" s="12"/>
     </row>
     <row r="100" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="12"/>
-      <c r="B100" s="12"/>
-      <c r="C100" s="12"/>
+      <c r="A100" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="B100" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C100" s="12" t="s">
+        <v>136</v>
+      </c>
       <c r="D100" s="12"/>
       <c r="E100" s="12"/>
       <c r="F100" s="12"/>
@@ -6084,13 +6091,27 @@
       <c r="R100" s="12"/>
       <c r="S100" s="12"/>
       <c r="T100" s="12"/>
-      <c r="U100" s="12"/>
-      <c r="V100" s="12"/>
-      <c r="W100" s="12"/>
-      <c r="X100" s="12"/>
-      <c r="Y100" s="12"/>
-      <c r="Z100" s="12"/>
-      <c r="AA100" s="12"/>
+      <c r="U100" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="V100" s="12" t="s">
+        <v>336</v>
+      </c>
+      <c r="W100" s="12" t="s">
+        <v>312</v>
+      </c>
+      <c r="X100" s="12" t="s">
+        <v>313</v>
+      </c>
+      <c r="Y100" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="Z100" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="AA100" s="12" t="s">
+        <v>136</v>
+      </c>
       <c r="AB100" s="12"/>
       <c r="AC100" s="12"/>
       <c r="AD100" s="12"/>
@@ -6129,33 +6150,42 @@
       <c r="AD101" s="12"/>
       <c r="AE101" s="12"/>
     </row>
-    <row r="102" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A102" s="14" t="s">
-        <v>245</v>
-      </c>
-      <c r="B102" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="C102" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="D102" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="F102" s="14" t="s">
-        <v>424</v>
-      </c>
-      <c r="R102" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB102" s="14"/>
-      <c r="AC102" s="14"/>
-      <c r="AD102" s="14"/>
-      <c r="AE102" s="14"/>
+    <row r="102" spans="1:31" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="12"/>
+      <c r="B102" s="12"/>
+      <c r="C102" s="12"/>
+      <c r="D102" s="12"/>
+      <c r="E102" s="12"/>
+      <c r="F102" s="12"/>
+      <c r="G102" s="12"/>
+      <c r="H102" s="12"/>
+      <c r="I102" s="12"/>
+      <c r="J102" s="12"/>
+      <c r="K102" s="12"/>
+      <c r="L102" s="12"/>
+      <c r="M102" s="12"/>
+      <c r="N102" s="12"/>
+      <c r="O102" s="12"/>
+      <c r="P102" s="12"/>
+      <c r="Q102" s="12"/>
+      <c r="R102" s="12"/>
+      <c r="S102" s="12"/>
+      <c r="T102" s="12"/>
+      <c r="U102" s="12"/>
+      <c r="V102" s="12"/>
+      <c r="W102" s="12"/>
+      <c r="X102" s="12"/>
+      <c r="Y102" s="12"/>
+      <c r="Z102" s="12"/>
+      <c r="AA102" s="12"/>
+      <c r="AB102" s="12"/>
+      <c r="AC102" s="12"/>
+      <c r="AD102" s="12"/>
+      <c r="AE102" s="12"/>
     </row>
     <row r="103" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A103" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B103" s="14" t="s">
         <v>176</v>
@@ -6164,7 +6194,7 @@
         <v>136</v>
       </c>
       <c r="D103" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F103" s="14" t="s">
         <v>424</v>
@@ -6179,7 +6209,7 @@
     </row>
     <row r="104" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A104" s="14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B104" s="14" t="s">
         <v>176</v>
@@ -6188,7 +6218,7 @@
         <v>136</v>
       </c>
       <c r="D104" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F104" s="14" t="s">
         <v>424</v>
@@ -6203,7 +6233,7 @@
     </row>
     <row r="105" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A105" s="14" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B105" s="14" t="s">
         <v>176</v>
@@ -6212,7 +6242,7 @@
         <v>136</v>
       </c>
       <c r="D105" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F105" s="14" t="s">
         <v>424</v>
@@ -6227,7 +6257,7 @@
     </row>
     <row r="106" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A106" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B106" s="14" t="s">
         <v>176</v>
@@ -6236,7 +6266,7 @@
         <v>136</v>
       </c>
       <c r="D106" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F106" s="14" t="s">
         <v>424</v>
@@ -6251,7 +6281,7 @@
     </row>
     <row r="107" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A107" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B107" s="14" t="s">
         <v>176</v>
@@ -6260,7 +6290,7 @@
         <v>136</v>
       </c>
       <c r="D107" s="15" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="F107" s="14" t="s">
         <v>424</v>
@@ -6275,7 +6305,7 @@
     </row>
     <row r="108" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A108" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B108" s="14" t="s">
         <v>176</v>
@@ -6290,16 +6320,16 @@
         <v>424</v>
       </c>
       <c r="R108" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AB108" s="14"/>
       <c r="AC108" s="14"/>
       <c r="AD108" s="14"/>
       <c r="AE108" s="14"/>
     </row>
-    <row r="109" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A109" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B109" s="14" t="s">
         <v>176</v>
@@ -6308,33 +6338,14 @@
         <v>136</v>
       </c>
       <c r="D109" s="15" t="s">
-        <v>238</v>
-      </c>
-      <c r="E109" s="14"/>
+        <v>187</v>
+      </c>
       <c r="F109" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="G109" s="14"/>
-      <c r="H109" s="14"/>
-      <c r="I109" s="14"/>
-      <c r="J109" s="14"/>
-      <c r="K109" s="14"/>
-      <c r="L109" s="14"/>
-      <c r="M109" s="14"/>
-      <c r="N109" s="14"/>
-      <c r="O109" s="14"/>
-      <c r="P109" s="14"/>
-      <c r="Q109" s="14"/>
-      <c r="R109" s="15"/>
-      <c r="S109" s="14"/>
-      <c r="T109" s="14"/>
-      <c r="U109" s="14"/>
-      <c r="V109" s="14"/>
-      <c r="W109" s="14"/>
-      <c r="X109" s="14"/>
-      <c r="Y109" s="14"/>
-      <c r="Z109" s="14"/>
-      <c r="AA109" s="14"/>
+      <c r="R109" s="15" t="s">
+        <v>2</v>
+      </c>
       <c r="AB109" s="14"/>
       <c r="AC109" s="14"/>
       <c r="AD109" s="14"/>
@@ -6342,7 +6353,7 @@
     </row>
     <row r="110" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B110" s="14" t="s">
         <v>176</v>
@@ -6351,7 +6362,7 @@
         <v>136</v>
       </c>
       <c r="D110" s="15" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E110" s="14"/>
       <c r="F110" s="14" t="s">
@@ -6383,9 +6394,9 @@
       <c r="AD110" s="14"/>
       <c r="AE110" s="14"/>
     </row>
-    <row r="111" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B111" s="14" t="s">
         <v>176</v>
@@ -6394,12 +6405,33 @@
         <v>136</v>
       </c>
       <c r="D111" s="15" t="s">
-        <v>240</v>
-      </c>
+        <v>239</v>
+      </c>
+      <c r="E111" s="14"/>
       <c r="F111" s="14" t="s">
         <v>424</v>
       </c>
+      <c r="G111" s="14"/>
+      <c r="H111" s="14"/>
+      <c r="I111" s="14"/>
+      <c r="J111" s="14"/>
+      <c r="K111" s="14"/>
+      <c r="L111" s="14"/>
+      <c r="M111" s="14"/>
+      <c r="N111" s="14"/>
+      <c r="O111" s="14"/>
+      <c r="P111" s="14"/>
+      <c r="Q111" s="14"/>
       <c r="R111" s="15"/>
+      <c r="S111" s="14"/>
+      <c r="T111" s="14"/>
+      <c r="U111" s="14"/>
+      <c r="V111" s="14"/>
+      <c r="W111" s="14"/>
+      <c r="X111" s="14"/>
+      <c r="Y111" s="14"/>
+      <c r="Z111" s="14"/>
+      <c r="AA111" s="14"/>
       <c r="AB111" s="14"/>
       <c r="AC111" s="14"/>
       <c r="AD111" s="14"/>
@@ -6407,7 +6439,7 @@
     </row>
     <row r="112" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A112" s="14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B112" s="14" t="s">
         <v>176</v>
@@ -6416,7 +6448,7 @@
         <v>136</v>
       </c>
       <c r="D112" s="15" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F112" s="14" t="s">
         <v>424</v>
@@ -6429,7 +6461,7 @@
     </row>
     <row r="113" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A113" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B113" s="14" t="s">
         <v>176</v>
@@ -6438,7 +6470,7 @@
         <v>136</v>
       </c>
       <c r="D113" s="15" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F113" s="14" t="s">
         <v>424</v>
@@ -6451,7 +6483,7 @@
     </row>
     <row r="114" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A114" s="14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B114" s="14" t="s">
         <v>176</v>
@@ -6459,15 +6491,13 @@
       <c r="C114" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="D114" s="16" t="s">
-        <v>259</v>
+      <c r="D114" s="15" t="s">
+        <v>242</v>
       </c>
       <c r="F114" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="R114" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R114" s="15"/>
       <c r="AB114" s="14"/>
       <c r="AC114" s="14"/>
       <c r="AD114" s="14"/>
@@ -6475,7 +6505,7 @@
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A115" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B115" s="14" t="s">
         <v>176</v>
@@ -6483,8 +6513,8 @@
       <c r="C115" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="D115" s="15" t="s">
-        <v>280</v>
+      <c r="D115" s="16" t="s">
+        <v>259</v>
       </c>
       <c r="F115" s="14" t="s">
         <v>424</v>
@@ -6497,9 +6527,9 @@
       <c r="AD115" s="14"/>
       <c r="AE115" s="14"/>
     </row>
-    <row r="116" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A116" s="14" t="s">
-        <v>281</v>
+        <v>258</v>
       </c>
       <c r="B116" s="14" t="s">
         <v>176</v>
@@ -6508,35 +6538,14 @@
         <v>136</v>
       </c>
       <c r="D116" s="15" t="s">
-        <v>282</v>
-      </c>
-      <c r="E116" s="14"/>
+        <v>280</v>
+      </c>
       <c r="F116" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="G116" s="14"/>
-      <c r="H116" s="14"/>
-      <c r="I116" s="14"/>
-      <c r="J116" s="14"/>
-      <c r="K116" s="14"/>
-      <c r="L116" s="14"/>
-      <c r="M116" s="14"/>
-      <c r="N116" s="14"/>
-      <c r="O116" s="14"/>
-      <c r="P116" s="14"/>
-      <c r="Q116" s="14"/>
       <c r="R116" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="S116" s="14"/>
-      <c r="T116" s="14"/>
-      <c r="U116" s="14"/>
-      <c r="V116" s="14"/>
-      <c r="W116" s="14"/>
-      <c r="X116" s="14"/>
-      <c r="Y116" s="14"/>
-      <c r="Z116" s="14"/>
-      <c r="AA116" s="14"/>
       <c r="AB116" s="14"/>
       <c r="AC116" s="14"/>
       <c r="AD116" s="14"/>
@@ -6544,7 +6553,7 @@
     </row>
     <row r="117" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="14" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="B117" s="14" t="s">
         <v>176</v>
@@ -6553,7 +6562,7 @@
         <v>136</v>
       </c>
       <c r="D117" s="15" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="E117" s="14"/>
       <c r="F117" s="14" t="s">
@@ -6571,7 +6580,7 @@
       <c r="P117" s="14"/>
       <c r="Q117" s="14"/>
       <c r="R117" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S117" s="14"/>
       <c r="T117" s="14"/>
@@ -6589,7 +6598,7 @@
     </row>
     <row r="118" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="14" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B118" s="14" t="s">
         <v>176</v>
@@ -6598,7 +6607,7 @@
         <v>136</v>
       </c>
       <c r="D118" s="15" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E118" s="14"/>
       <c r="F118" s="14" t="s">
@@ -6616,7 +6625,7 @@
       <c r="P118" s="14"/>
       <c r="Q118" s="14"/>
       <c r="R118" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S118" s="14"/>
       <c r="T118" s="14"/>
@@ -6634,7 +6643,7 @@
     </row>
     <row r="119" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B119" s="14" t="s">
         <v>176</v>
@@ -6643,7 +6652,7 @@
         <v>136</v>
       </c>
       <c r="D119" s="15" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="E119" s="14"/>
       <c r="F119" s="14" t="s">
@@ -6679,7 +6688,7 @@
     </row>
     <row r="120" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="14" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="B120" s="14" t="s">
         <v>176</v>
@@ -6688,7 +6697,7 @@
         <v>136</v>
       </c>
       <c r="D120" s="15" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="E120" s="14"/>
       <c r="F120" s="14" t="s">
@@ -6706,7 +6715,7 @@
       <c r="P120" s="14"/>
       <c r="Q120" s="14"/>
       <c r="R120" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S120" s="14"/>
       <c r="T120" s="14"/>
@@ -6724,7 +6733,7 @@
     </row>
     <row r="121" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="14" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B121" s="14" t="s">
         <v>176</v>
@@ -6733,7 +6742,7 @@
         <v>136</v>
       </c>
       <c r="D121" s="15" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="E121" s="14"/>
       <c r="F121" s="14" t="s">
@@ -6751,7 +6760,7 @@
       <c r="P121" s="14"/>
       <c r="Q121" s="14"/>
       <c r="R121" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S121" s="14"/>
       <c r="T121" s="14"/>
@@ -6769,7 +6778,7 @@
     </row>
     <row r="122" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="14" t="s">
-        <v>376</v>
+        <v>297</v>
       </c>
       <c r="B122" s="14" t="s">
         <v>176</v>
@@ -6778,7 +6787,7 @@
         <v>136</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>375</v>
+        <v>298</v>
       </c>
       <c r="E122" s="14"/>
       <c r="F122" s="14" t="s">
@@ -6786,9 +6795,7 @@
       </c>
       <c r="G122" s="14"/>
       <c r="H122" s="14"/>
-      <c r="I122" s="14" t="s">
-        <v>127</v>
-      </c>
+      <c r="I122" s="14"/>
       <c r="J122" s="14"/>
       <c r="K122" s="14"/>
       <c r="L122" s="14"/>
@@ -6797,7 +6804,9 @@
       <c r="O122" s="14"/>
       <c r="P122" s="14"/>
       <c r="Q122" s="14"/>
-      <c r="R122" s="15"/>
+      <c r="R122" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S122" s="14"/>
       <c r="T122" s="14"/>
       <c r="U122" s="14"/>
@@ -6814,7 +6823,7 @@
     </row>
     <row r="123" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="14" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B123" s="14" t="s">
         <v>176</v>
@@ -6823,7 +6832,7 @@
         <v>136</v>
       </c>
       <c r="D123" s="15" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="E123" s="14"/>
       <c r="F123" s="14" t="s">
@@ -6832,7 +6841,7 @@
       <c r="G123" s="14"/>
       <c r="H123" s="14"/>
       <c r="I123" s="14" t="s">
-        <v>382</v>
+        <v>127</v>
       </c>
       <c r="J123" s="14"/>
       <c r="K123" s="14"/>
@@ -6859,7 +6868,7 @@
     </row>
     <row r="124" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="14" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="B124" s="14" t="s">
         <v>176</v>
@@ -6868,7 +6877,7 @@
         <v>136</v>
       </c>
       <c r="D124" s="15" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="E124" s="14"/>
       <c r="F124" s="14" t="s">
@@ -6877,7 +6886,7 @@
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
       <c r="I124" s="14" t="s">
-        <v>126</v>
+        <v>382</v>
       </c>
       <c r="J124" s="14"/>
       <c r="K124" s="14"/>
@@ -6904,7 +6913,7 @@
     </row>
     <row r="125" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="14" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B125" s="14" t="s">
         <v>176</v>
@@ -6913,7 +6922,7 @@
         <v>136</v>
       </c>
       <c r="D125" s="15" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E125" s="14"/>
       <c r="F125" s="14" t="s">
@@ -6922,7 +6931,7 @@
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
       <c r="I125" s="14" t="s">
-        <v>384</v>
+        <v>126</v>
       </c>
       <c r="J125" s="14"/>
       <c r="K125" s="14"/>
@@ -6949,7 +6958,7 @@
     </row>
     <row r="126" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="14" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="B126" s="14" t="s">
         <v>176</v>
@@ -6958,7 +6967,7 @@
         <v>136</v>
       </c>
       <c r="D126" s="15" t="s">
-        <v>181</v>
+        <v>388</v>
       </c>
       <c r="E126" s="14"/>
       <c r="F126" s="14" t="s">
@@ -6966,7 +6975,9 @@
       </c>
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
-      <c r="I126" s="14"/>
+      <c r="I126" s="14" t="s">
+        <v>384</v>
+      </c>
       <c r="J126" s="14"/>
       <c r="K126" s="14"/>
       <c r="L126" s="14"/>
@@ -6991,12 +7002,22 @@
       <c r="AE126" s="14"/>
     </row>
     <row r="127" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="14"/>
-      <c r="B127" s="14"/>
-      <c r="C127" s="14"/>
-      <c r="D127" s="15"/>
+      <c r="A127" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="B127" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C127" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="D127" s="15" t="s">
+        <v>181</v>
+      </c>
       <c r="E127" s="14"/>
-      <c r="F127" s="14"/>
+      <c r="F127" s="14" t="s">
+        <v>424</v>
+      </c>
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
       <c r="I127" s="14"/>
@@ -7089,52 +7110,40 @@
       <c r="AD129" s="14"/>
       <c r="AE129" s="14"/>
     </row>
-    <row r="130" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="14"/>
+      <c r="B130" s="14"/>
+      <c r="C130" s="14"/>
+      <c r="D130" s="15"/>
+      <c r="E130" s="14"/>
+      <c r="F130" s="14"/>
+      <c r="G130" s="14"/>
+      <c r="H130" s="14"/>
+      <c r="I130" s="14"/>
+      <c r="J130" s="14"/>
+      <c r="K130" s="14"/>
+      <c r="L130" s="14"/>
+      <c r="M130" s="14"/>
+      <c r="N130" s="14"/>
+      <c r="O130" s="14"/>
+      <c r="P130" s="14"/>
+      <c r="Q130" s="14"/>
+      <c r="R130" s="15"/>
+      <c r="S130" s="14"/>
+      <c r="T130" s="14"/>
+      <c r="U130" s="14"/>
+      <c r="V130" s="14"/>
+      <c r="W130" s="14"/>
+      <c r="X130" s="14"/>
+      <c r="Y130" s="14"/>
+      <c r="Z130" s="14"/>
+      <c r="AA130" s="14"/>
       <c r="AB130" s="14"/>
       <c r="AC130" s="14"/>
       <c r="AD130" s="14"/>
       <c r="AE130" s="14"/>
     </row>
-    <row r="131" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="14" t="s">
-        <v>270</v>
-      </c>
-      <c r="B131" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="C131" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="D131" s="14"/>
-      <c r="E131" s="14"/>
-      <c r="F131" s="14"/>
-      <c r="G131" s="14"/>
-      <c r="H131" s="14"/>
-      <c r="I131" s="14"/>
-      <c r="J131" s="15" t="s">
-        <v>276</v>
-      </c>
-      <c r="K131" s="15" t="s">
-        <v>277</v>
-      </c>
-      <c r="L131" s="15" t="s">
-        <v>278</v>
-      </c>
-      <c r="M131" s="14"/>
-      <c r="N131" s="14"/>
-      <c r="O131" s="14"/>
-      <c r="P131" s="14"/>
-      <c r="Q131" s="14"/>
-      <c r="R131" s="14"/>
-      <c r="S131" s="14"/>
-      <c r="T131" s="14"/>
-      <c r="U131" s="14"/>
-      <c r="V131" s="14"/>
-      <c r="W131" s="14"/>
-      <c r="X131" s="14"/>
-      <c r="Y131" s="14"/>
-      <c r="Z131" s="14"/>
-      <c r="AA131" s="14"/>
+    <row r="131" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AB131" s="14"/>
       <c r="AC131" s="14"/>
       <c r="AD131" s="14"/>
@@ -7142,7 +7151,7 @@
     </row>
     <row r="132" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="14" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B132" s="14" t="s">
         <v>176</v>
@@ -7157,13 +7166,13 @@
       <c r="H132" s="14"/>
       <c r="I132" s="14"/>
       <c r="J132" s="15" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="K132" s="15" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="L132" s="15" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="M132" s="14"/>
       <c r="N132" s="14"/>
@@ -7185,9 +7194,9 @@
       <c r="AD132" s="14"/>
       <c r="AE132" s="14"/>
     </row>
-    <row r="133" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="14" t="s">
-        <v>362</v>
+        <v>271</v>
       </c>
       <c r="B133" s="14" t="s">
         <v>176</v>
@@ -7195,9 +7204,36 @@
       <c r="C133" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="O133" s="15" t="s">
-        <v>365</v>
-      </c>
+      <c r="D133" s="14"/>
+      <c r="E133" s="14"/>
+      <c r="F133" s="14"/>
+      <c r="G133" s="14"/>
+      <c r="H133" s="14"/>
+      <c r="I133" s="14"/>
+      <c r="J133" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="K133" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="L133" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="M133" s="14"/>
+      <c r="N133" s="14"/>
+      <c r="O133" s="14"/>
+      <c r="P133" s="14"/>
+      <c r="Q133" s="14"/>
+      <c r="R133" s="14"/>
+      <c r="S133" s="14"/>
+      <c r="T133" s="14"/>
+      <c r="U133" s="14"/>
+      <c r="V133" s="14"/>
+      <c r="W133" s="14"/>
+      <c r="X133" s="14"/>
+      <c r="Y133" s="14"/>
+      <c r="Z133" s="14"/>
+      <c r="AA133" s="14"/>
       <c r="AB133" s="14"/>
       <c r="AC133" s="14"/>
       <c r="AD133" s="14"/>
@@ -7205,7 +7241,7 @@
     </row>
     <row r="134" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A134" s="14" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B134" s="14" t="s">
         <v>176</v>
@@ -7214,7 +7250,7 @@
         <v>136</v>
       </c>
       <c r="O134" s="15" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AB134" s="14"/>
       <c r="AC134" s="14"/>
@@ -7223,7 +7259,7 @@
     </row>
     <row r="135" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A135" s="14" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B135" s="14" t="s">
         <v>176</v>
@@ -7232,7 +7268,7 @@
         <v>136</v>
       </c>
       <c r="O135" s="15" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="AB135" s="14"/>
       <c r="AC135" s="14"/>
@@ -7241,7 +7277,7 @@
     </row>
     <row r="136" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A136" s="14" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="B136" s="14" t="s">
         <v>176</v>
@@ -7249,8 +7285,8 @@
       <c r="C136" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="M136" s="14" t="s">
-        <v>374</v>
+      <c r="O136" s="15" t="s">
+        <v>367</v>
       </c>
       <c r="AB136" s="14"/>
       <c r="AC136" s="14"/>
@@ -7258,6 +7294,18 @@
       <c r="AE136" s="14"/>
     </row>
     <row r="137" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A137" s="14" t="s">
+        <v>373</v>
+      </c>
+      <c r="B137" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C137" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="M137" s="14" t="s">
+        <v>374</v>
+      </c>
       <c r="AB137" s="14"/>
       <c r="AC137" s="14"/>
       <c r="AD137" s="14"/>
@@ -8474,6 +8522,12 @@
       <c r="AC339" s="14"/>
       <c r="AD339" s="14"/>
       <c r="AE339" s="14"/>
+    </row>
+    <row r="340" spans="28:31" x14ac:dyDescent="0.25">
+      <c r="AB340" s="14"/>
+      <c r="AC340" s="14"/>
+      <c r="AD340" s="14"/>
+      <c r="AE340" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -8484,7 +8538,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:S105"/>
+  <dimension ref="A1:S106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -8571,16 +8625,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>418</v>
+        <v>437</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>61</v>
+        <v>438</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>113</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>61</v>
+        <v>438</v>
       </c>
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
@@ -10051,35 +10105,42 @@
       <c r="R51" s="14"/>
       <c r="S51" s="14"/>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="16" t="s">
-        <v>160</v>
+        <v>89</v>
       </c>
       <c r="B52" s="20" t="s">
         <v>418</v>
       </c>
-      <c r="C52" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="D52" s="16" t="s">
+      <c r="C52" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D52" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="J52" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O52" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="P52" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q52" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="53" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="E52" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="F52" s="15"/>
+      <c r="G52" s="15"/>
+      <c r="H52" s="14" t="s">
+        <v>424</v>
+      </c>
+      <c r="I52" s="19"/>
+      <c r="J52" s="19"/>
+      <c r="K52" s="19"/>
+      <c r="L52" s="14"/>
+      <c r="M52" s="14"/>
+      <c r="N52" s="14"/>
+      <c r="O52" s="14"/>
+      <c r="P52" s="14"/>
+      <c r="Q52" s="14"/>
+      <c r="R52" s="14"/>
+      <c r="S52" s="14"/>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B53" s="20" t="s">
         <v>418</v>
@@ -10090,18 +10151,9 @@
       <c r="D53" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="E53" s="14"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="14"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="14"/>
       <c r="J53" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="K53" s="14"/>
-      <c r="L53" s="14"/>
-      <c r="M53" s="14"/>
-      <c r="N53" s="14"/>
       <c r="O53" s="14" t="s">
         <v>140</v>
       </c>
@@ -10111,15 +10163,13 @@
       <c r="Q53" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="R53" s="14"/>
-      <c r="S53" s="14"/>
     </row>
     <row r="54" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="16" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>425</v>
+        <v>418</v>
       </c>
       <c r="C54" s="16" t="s">
         <v>0</v>
@@ -10153,13 +10203,13 @@
     </row>
     <row r="55" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="16" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>146</v>
+        <v>425</v>
       </c>
       <c r="C55" s="16" t="s">
-        <v>148</v>
+        <v>0</v>
       </c>
       <c r="D55" s="16" t="s">
         <v>113</v>
@@ -10190,13 +10240,13 @@
     </row>
     <row r="56" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>418</v>
+        <v>146</v>
       </c>
       <c r="C56" s="16" t="s">
-        <v>2</v>
+        <v>148</v>
       </c>
       <c r="D56" s="16" t="s">
         <v>113</v>
@@ -10225,12 +10275,12 @@
       <c r="R56" s="14"/>
       <c r="S56" s="14"/>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
-        <v>165</v>
-      </c>
-      <c r="B57" s="20" t="s">
-        <v>418</v>
+        <v>164</v>
+      </c>
+      <c r="B57" s="18" t="s">
+        <v>437</v>
       </c>
       <c r="C57" s="16" t="s">
         <v>2</v>
@@ -10238,9 +10288,18 @@
       <c r="D57" s="16" t="s">
         <v>113</v>
       </c>
+      <c r="E57" s="14"/>
+      <c r="F57" s="14"/>
+      <c r="G57" s="14"/>
+      <c r="H57" s="14"/>
+      <c r="I57" s="14"/>
       <c r="J57" s="14" t="s">
         <v>135</v>
       </c>
+      <c r="K57" s="14"/>
+      <c r="L57" s="14"/>
+      <c r="M57" s="14"/>
+      <c r="N57" s="14"/>
       <c r="O57" s="14" t="s">
         <v>140</v>
       </c>
@@ -10250,13 +10309,15 @@
       <c r="Q57" s="14" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="58" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="R57" s="14"/>
+      <c r="S57" s="14"/>
+    </row>
+    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58" s="16" t="s">
-        <v>172</v>
-      </c>
-      <c r="B58" s="20" t="s">
-        <v>418</v>
+        <v>165</v>
+      </c>
+      <c r="B58" s="18" t="s">
+        <v>437</v>
       </c>
       <c r="C58" s="16" t="s">
         <v>2</v>
@@ -10264,18 +10325,9 @@
       <c r="D58" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="E58" s="14"/>
-      <c r="F58" s="14"/>
-      <c r="G58" s="14"/>
-      <c r="H58" s="14"/>
-      <c r="I58" s="14"/>
       <c r="J58" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="K58" s="14"/>
-      <c r="L58" s="14"/>
-      <c r="M58" s="14"/>
-      <c r="N58" s="14"/>
       <c r="O58" s="14" t="s">
         <v>140</v>
       </c>
@@ -10285,15 +10337,13 @@
       <c r="Q58" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="R58" s="14"/>
-      <c r="S58" s="14"/>
     </row>
     <row r="59" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B59" s="20" t="s">
-        <v>425</v>
+        <v>418</v>
       </c>
       <c r="C59" s="16" t="s">
         <v>2</v>
@@ -10327,13 +10377,13 @@
     </row>
     <row r="60" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
-        <v>192</v>
+        <v>173</v>
       </c>
       <c r="B60" s="20" t="s">
         <v>425</v>
       </c>
       <c r="C60" s="16" t="s">
-        <v>46</v>
+        <v>2</v>
       </c>
       <c r="D60" s="16" t="s">
         <v>113</v>
@@ -10359,14 +10409,12 @@
       <c r="Q60" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="R60" s="15" t="s">
-        <v>2</v>
-      </c>
+      <c r="R60" s="14"/>
       <c r="S60" s="14"/>
     </row>
     <row r="61" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="16" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B61" s="20" t="s">
         <v>425</v>
@@ -10405,13 +10453,13 @@
     </row>
     <row r="62" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="16" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B62" s="20" t="s">
         <v>425</v>
       </c>
       <c r="C62" s="16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D62" s="16" t="s">
         <v>113</v>
@@ -10437,27 +10485,36 @@
       <c r="Q62" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="R62" s="14"/>
-      <c r="S62" s="15" t="s">
+      <c r="R62" s="15" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S62" s="14"/>
+    </row>
+    <row r="63" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="16" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B63" s="20" t="s">
         <v>425</v>
       </c>
-      <c r="C63" s="15" t="s">
+      <c r="C63" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="D63" s="14" t="s">
+      <c r="D63" s="16" t="s">
         <v>113</v>
       </c>
+      <c r="E63" s="14"/>
+      <c r="F63" s="14"/>
+      <c r="G63" s="14"/>
+      <c r="H63" s="14"/>
+      <c r="I63" s="14"/>
       <c r="J63" s="14" t="s">
         <v>135</v>
       </c>
+      <c r="K63" s="14"/>
+      <c r="L63" s="14"/>
+      <c r="M63" s="14"/>
+      <c r="N63" s="14"/>
       <c r="O63" s="14" t="s">
         <v>140</v>
       </c>
@@ -10467,10 +10524,14 @@
       <c r="Q63" s="14" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="64" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="R63" s="14"/>
+      <c r="S63" s="15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A64" s="16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B64" s="20" t="s">
         <v>425</v>
@@ -10481,18 +10542,9 @@
       <c r="D64" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="E64" s="14"/>
-      <c r="F64" s="14"/>
-      <c r="G64" s="14"/>
-      <c r="H64" s="14"/>
-      <c r="I64" s="14"/>
       <c r="J64" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="K64" s="14"/>
-      <c r="L64" s="14"/>
-      <c r="M64" s="14"/>
-      <c r="N64" s="14"/>
       <c r="O64" s="14" t="s">
         <v>140</v>
       </c>
@@ -10502,14 +10554,10 @@
       <c r="Q64" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="R64" s="14"/>
-      <c r="S64" s="15" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="65" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="16" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B65" s="20" t="s">
         <v>425</v>
@@ -10542,17 +10590,19 @@
         <v>144</v>
       </c>
       <c r="R65" s="14"/>
-      <c r="S65" s="14"/>
+      <c r="S65" s="15" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="66" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="16" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="C66" s="15" t="s">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="D66" s="14" t="s">
         <v>113</v>
@@ -10562,20 +10612,28 @@
       <c r="G66" s="14"/>
       <c r="H66" s="14"/>
       <c r="I66" s="14"/>
-      <c r="J66" s="14"/>
+      <c r="J66" s="14" t="s">
+        <v>135</v>
+      </c>
       <c r="K66" s="14"/>
       <c r="L66" s="14"/>
       <c r="M66" s="14"/>
       <c r="N66" s="14"/>
-      <c r="O66" s="14"/>
-      <c r="P66" s="14"/>
-      <c r="Q66" s="14"/>
+      <c r="O66" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="P66" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q66" s="14" t="s">
+        <v>144</v>
+      </c>
       <c r="R66" s="14"/>
       <c r="S66" s="14"/>
     </row>
     <row r="67" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="16" t="s">
-        <v>266</v>
+        <v>203</v>
       </c>
       <c r="B67" s="20" t="s">
         <v>418</v>
@@ -10583,7 +10641,7 @@
       <c r="C67" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="D67" s="16" t="s">
+      <c r="D67" s="14" t="s">
         <v>113</v>
       </c>
       <c r="E67" s="14"/>
@@ -10591,31 +10649,23 @@
       <c r="G67" s="14"/>
       <c r="H67" s="14"/>
       <c r="I67" s="14"/>
-      <c r="J67" s="14" t="s">
-        <v>135</v>
-      </c>
+      <c r="J67" s="14"/>
       <c r="K67" s="14"/>
       <c r="L67" s="14"/>
       <c r="M67" s="14"/>
       <c r="N67" s="14"/>
-      <c r="O67" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="P67" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q67" s="14" t="s">
-        <v>144</v>
-      </c>
+      <c r="O67" s="14"/>
+      <c r="P67" s="14"/>
+      <c r="Q67" s="14"/>
       <c r="R67" s="14"/>
       <c r="S67" s="14"/>
     </row>
     <row r="68" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="16" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B68" s="20" t="s">
-        <v>425</v>
+        <v>418</v>
       </c>
       <c r="C68" s="15" t="s">
         <v>0</v>
@@ -10649,12 +10699,12 @@
     </row>
     <row r="69" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="16" t="s">
-        <v>349</v>
+        <v>267</v>
       </c>
       <c r="B69" s="20" t="s">
-        <v>418</v>
-      </c>
-      <c r="C69" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="C69" s="15" t="s">
         <v>0</v>
       </c>
       <c r="D69" s="16" t="s">
@@ -10686,7 +10736,7 @@
     </row>
     <row r="70" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="16" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B70" s="20" t="s">
         <v>418</v>
@@ -10723,10 +10773,10 @@
     </row>
     <row r="71" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="16" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B71" s="20" t="s">
-        <v>425</v>
+        <v>418</v>
       </c>
       <c r="C71" s="16" t="s">
         <v>0</v>
@@ -10760,10 +10810,10 @@
     </row>
     <row r="72" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="16" t="s">
-        <v>415</v>
+        <v>351</v>
       </c>
       <c r="B72" s="20" t="s">
-        <v>414</v>
+        <v>425</v>
       </c>
       <c r="C72" s="16" t="s">
         <v>0</v>
@@ -10795,30 +10845,46 @@
       <c r="R72" s="14"/>
       <c r="S72" s="14"/>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A74" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="B74" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="C74" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="D74" s="14" t="s">
+    <row r="73" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="16" t="s">
+        <v>415</v>
+      </c>
+      <c r="B73" s="20" t="s">
+        <v>414</v>
+      </c>
+      <c r="C73" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="D73" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="E74" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="G74" s="21"/>
-      <c r="H74" s="14" t="s">
-        <v>424</v>
-      </c>
+      <c r="E73" s="14"/>
+      <c r="F73" s="14"/>
+      <c r="G73" s="14"/>
+      <c r="H73" s="14"/>
+      <c r="I73" s="14"/>
+      <c r="J73" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K73" s="14"/>
+      <c r="L73" s="14"/>
+      <c r="M73" s="14"/>
+      <c r="N73" s="14"/>
+      <c r="O73" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="P73" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q73" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="R73" s="14"/>
+      <c r="S73" s="14"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A75" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B75" s="15" t="s">
         <v>178</v>
@@ -10839,7 +10905,7 @@
     </row>
     <row r="76" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A76" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B76" s="15" t="s">
         <v>178</v>
@@ -10851,10 +10917,7 @@
         <v>113</v>
       </c>
       <c r="E76" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="F76" s="15" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="G76" s="21"/>
       <c r="H76" s="14" t="s">
@@ -10863,7 +10926,7 @@
     </row>
     <row r="77" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A77" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B77" s="15" t="s">
         <v>178</v>
@@ -10875,7 +10938,10 @@
         <v>113</v>
       </c>
       <c r="E77" s="15" t="s">
-        <v>56</v>
+        <v>52</v>
+      </c>
+      <c r="F77" s="15" t="s">
+        <v>51</v>
       </c>
       <c r="G77" s="21"/>
       <c r="H77" s="14" t="s">
@@ -10884,7 +10950,7 @@
     </row>
     <row r="78" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A78" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B78" s="15" t="s">
         <v>178</v>
@@ -10896,7 +10962,7 @@
         <v>113</v>
       </c>
       <c r="E78" s="15" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="G78" s="21"/>
       <c r="H78" s="14" t="s">
@@ -10905,19 +10971,19 @@
     </row>
     <row r="79" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A79" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B79" s="15" t="s">
         <v>178</v>
       </c>
       <c r="C79" s="15" t="s">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="D79" s="14" t="s">
         <v>113</v>
       </c>
       <c r="E79" s="15" t="s">
-        <v>3</v>
+        <v>81</v>
       </c>
       <c r="G79" s="21"/>
       <c r="H79" s="14" t="s">
@@ -10926,28 +10992,28 @@
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A80" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B80" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C80" s="15" t="s">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="D80" s="14" t="s">
         <v>113</v>
       </c>
       <c r="E80" s="15" t="s">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="G80" s="21"/>
       <c r="H80" s="14" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="81" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A81" s="15" t="s">
-        <v>238</v>
+        <v>186</v>
       </c>
       <c r="B81" s="15" t="s">
         <v>179</v>
@@ -10961,26 +11027,14 @@
       <c r="E81" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="F81" s="14"/>
       <c r="G81" s="21"/>
       <c r="H81" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="I81" s="14"/>
-      <c r="J81" s="14"/>
-      <c r="K81" s="14"/>
-      <c r="L81" s="14"/>
-      <c r="M81" s="14"/>
-      <c r="N81" s="14"/>
-      <c r="O81" s="14"/>
-      <c r="P81" s="14"/>
-      <c r="Q81" s="14"/>
-      <c r="R81" s="14"/>
-      <c r="S81" s="14"/>
-    </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="15" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B82" s="15" t="s">
         <v>179</v>
@@ -10992,19 +11046,28 @@
         <v>113</v>
       </c>
       <c r="E82" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="F82" s="15" t="s">
-        <v>3</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="F82" s="14"/>
       <c r="G82" s="21"/>
       <c r="H82" s="14" t="s">
         <v>424</v>
       </c>
+      <c r="I82" s="14"/>
+      <c r="J82" s="14"/>
+      <c r="K82" s="14"/>
+      <c r="L82" s="14"/>
+      <c r="M82" s="14"/>
+      <c r="N82" s="14"/>
+      <c r="O82" s="14"/>
+      <c r="P82" s="14"/>
+      <c r="Q82" s="14"/>
+      <c r="R82" s="14"/>
+      <c r="S82" s="14"/>
     </row>
     <row r="83" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B83" s="15" t="s">
         <v>179</v>
@@ -11016,7 +11079,10 @@
         <v>113</v>
       </c>
       <c r="E83" s="15" t="s">
-        <v>60</v>
+        <v>3</v>
+      </c>
+      <c r="F83" s="15" t="s">
+        <v>3</v>
       </c>
       <c r="G83" s="21"/>
       <c r="H83" s="14" t="s">
@@ -11025,19 +11091,19 @@
     </row>
     <row r="84" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A84" s="15" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B84" s="15" t="s">
         <v>179</v>
       </c>
       <c r="C84" s="15" t="s">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="D84" s="14" t="s">
         <v>113</v>
       </c>
       <c r="E84" s="15" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G84" s="21"/>
       <c r="H84" s="14" t="s">
@@ -11046,21 +11112,20 @@
     </row>
     <row r="85" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A85" s="15" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B85" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C85" s="15" t="s">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="D85" s="14" t="s">
         <v>113</v>
       </c>
       <c r="E85" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="F85" s="15"/>
+        <v>57</v>
+      </c>
       <c r="G85" s="21"/>
       <c r="H85" s="14" t="s">
         <v>424</v>
@@ -11068,10 +11133,10 @@
     </row>
     <row r="86" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A86" s="15" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B86" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C86" s="15" t="s">
         <v>61</v>
@@ -11088,9 +11153,9 @@
         <v>424</v>
       </c>
     </row>
-    <row r="87" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A87" s="15" t="s">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="B87" s="15" t="s">
         <v>179</v>
@@ -11109,21 +11174,10 @@
       <c r="H87" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="I87" s="14"/>
-      <c r="J87" s="14"/>
-      <c r="K87" s="14"/>
-      <c r="L87" s="14"/>
-      <c r="M87" s="14"/>
-      <c r="N87" s="14"/>
-      <c r="O87" s="14"/>
-      <c r="P87" s="14"/>
-      <c r="Q87" s="14"/>
-      <c r="R87" s="14"/>
-      <c r="S87" s="14"/>
-    </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="15" t="s">
-        <v>280</v>
+        <v>259</v>
       </c>
       <c r="B88" s="15" t="s">
         <v>179</v>
@@ -11135,25 +11189,34 @@
         <v>113</v>
       </c>
       <c r="E88" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="F88" s="15" t="s">
-        <v>3</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="F88" s="15"/>
       <c r="G88" s="21"/>
       <c r="H88" s="14" t="s">
         <v>424</v>
       </c>
+      <c r="I88" s="14"/>
+      <c r="J88" s="14"/>
+      <c r="K88" s="14"/>
+      <c r="L88" s="14"/>
+      <c r="M88" s="14"/>
+      <c r="N88" s="14"/>
+      <c r="O88" s="14"/>
+      <c r="P88" s="14"/>
+      <c r="Q88" s="14"/>
+      <c r="R88" s="14"/>
+      <c r="S88" s="14"/>
     </row>
     <row r="89" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A89" s="15" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="B89" s="15" t="s">
         <v>179</v>
       </c>
       <c r="C89" s="15" t="s">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="D89" s="14" t="s">
         <v>113</v>
@@ -11161,6 +11224,9 @@
       <c r="E89" s="15" t="s">
         <v>3</v>
       </c>
+      <c r="F89" s="15" t="s">
+        <v>3</v>
+      </c>
       <c r="G89" s="21"/>
       <c r="H89" s="14" t="s">
         <v>424</v>
@@ -11168,10 +11234,10 @@
     </row>
     <row r="90" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A90" s="15" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B90" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C90" s="15" t="s">
         <v>3</v>
@@ -11189,10 +11255,10 @@
     </row>
     <row r="91" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A91" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B91" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C91" s="15" t="s">
         <v>3</v>
@@ -11210,10 +11276,10 @@
     </row>
     <row r="92" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A92" s="15" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B92" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C92" s="15" t="s">
         <v>3</v>
@@ -11231,7 +11297,7 @@
     </row>
     <row r="93" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A93" s="15" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B93" s="15" t="s">
         <v>178</v>
@@ -11243,7 +11309,7 @@
         <v>113</v>
       </c>
       <c r="E93" s="15" t="s">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="G93" s="21"/>
       <c r="H93" s="14" t="s">
@@ -11252,7 +11318,7 @@
     </row>
     <row r="94" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A94" s="15" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="B94" s="15" t="s">
         <v>178</v>
@@ -11264,7 +11330,7 @@
         <v>113</v>
       </c>
       <c r="E94" s="15" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="G94" s="21"/>
       <c r="H94" s="14" t="s">
@@ -11273,7 +11339,7 @@
     </row>
     <row r="95" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A95" s="15" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B95" s="15" t="s">
         <v>178</v>
@@ -11284,16 +11350,17 @@
       <c r="D95" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="E95" s="16" t="s">
-        <v>3</v>
-      </c>
+      <c r="E95" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="G95" s="21"/>
       <c r="H95" s="14" t="s">
         <v>424</v>
       </c>
     </row>
     <row r="96" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A96" s="15" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B96" s="15" t="s">
         <v>178</v>
@@ -11313,7 +11380,7 @@
     </row>
     <row r="97" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A97" s="15" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="B97" s="15" t="s">
         <v>178</v>
@@ -11333,7 +11400,7 @@
     </row>
     <row r="98" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A98" s="15" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B98" s="15" t="s">
         <v>178</v>
@@ -11353,27 +11420,27 @@
     </row>
     <row r="99" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A99" s="15" t="s">
-        <v>375</v>
+        <v>300</v>
       </c>
       <c r="B99" s="15" t="s">
         <v>178</v>
       </c>
       <c r="C99" s="15" t="s">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="D99" s="14" t="s">
         <v>113</v>
       </c>
       <c r="E99" s="16" t="s">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="H99" s="14" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="100" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A100" s="15" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="B100" s="15" t="s">
         <v>178</v>
@@ -11387,29 +11454,16 @@
       <c r="E100" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="F100" s="14"/>
-      <c r="G100" s="21"/>
       <c r="H100" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="I100" s="14"/>
-      <c r="J100" s="14"/>
-      <c r="K100" s="14"/>
-      <c r="L100" s="14"/>
-      <c r="M100" s="14"/>
-      <c r="N100" s="14"/>
-      <c r="O100" s="14"/>
-      <c r="P100" s="14"/>
-      <c r="Q100" s="14"/>
-      <c r="R100" s="14"/>
-      <c r="S100" s="14"/>
     </row>
     <row r="101" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="15" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B101" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C101" s="15" t="s">
         <v>46</v>
@@ -11439,32 +11493,28 @@
     </row>
     <row r="102" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="15" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
       <c r="B102" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C102" s="15" t="s">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="D102" s="14" t="s">
         <v>113</v>
       </c>
       <c r="E102" s="16" t="s">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="F102" s="14"/>
-      <c r="G102" s="14"/>
+      <c r="G102" s="21"/>
       <c r="H102" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="I102" s="14" t="s">
-        <v>122</v>
-      </c>
+      <c r="I102" s="14"/>
       <c r="J102" s="14"/>
-      <c r="K102" s="14" t="s">
-        <v>122</v>
-      </c>
+      <c r="K102" s="14"/>
       <c r="L102" s="14"/>
       <c r="M102" s="14"/>
       <c r="N102" s="14"/>
@@ -11476,14 +11526,18 @@
     </row>
     <row r="103" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="15" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B103" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="C103" s="14"/>
-      <c r="D103" s="14"/>
-      <c r="E103" s="15" t="s">
+      <c r="C103" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D103" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="E103" s="16" t="s">
         <v>2</v>
       </c>
       <c r="F103" s="14"/>
@@ -11509,11 +11563,12 @@
     </row>
     <row r="104" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="15" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B104" s="15" t="s">
-        <v>179</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="C104" s="14"/>
       <c r="D104" s="14"/>
       <c r="E104" s="15" t="s">
         <v>2</v>
@@ -11540,17 +11595,28 @@
       <c r="S104" s="14"/>
     </row>
     <row r="105" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="15"/>
-      <c r="B105" s="15"/>
-      <c r="C105" s="15"/>
+      <c r="A105" s="15" t="s">
+        <v>390</v>
+      </c>
+      <c r="B105" s="15" t="s">
+        <v>179</v>
+      </c>
       <c r="D105" s="14"/>
-      <c r="E105" s="16"/>
+      <c r="E105" s="15" t="s">
+        <v>2</v>
+      </c>
       <c r="F105" s="14"/>
       <c r="G105" s="14"/>
-      <c r="H105" s="14"/>
-      <c r="I105" s="14"/>
+      <c r="H105" s="14" t="s">
+        <v>424</v>
+      </c>
+      <c r="I105" s="14" t="s">
+        <v>122</v>
+      </c>
       <c r="J105" s="14"/>
-      <c r="K105" s="14"/>
+      <c r="K105" s="14" t="s">
+        <v>122</v>
+      </c>
       <c r="L105" s="14"/>
       <c r="M105" s="14"/>
       <c r="N105" s="14"/>
@@ -11559,6 +11625,27 @@
       <c r="Q105" s="14"/>
       <c r="R105" s="14"/>
       <c r="S105" s="14"/>
+    </row>
+    <row r="106" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="15"/>
+      <c r="B106" s="15"/>
+      <c r="C106" s="15"/>
+      <c r="D106" s="14"/>
+      <c r="E106" s="16"/>
+      <c r="F106" s="14"/>
+      <c r="G106" s="14"/>
+      <c r="H106" s="14"/>
+      <c r="I106" s="14"/>
+      <c r="J106" s="14"/>
+      <c r="K106" s="14"/>
+      <c r="L106" s="14"/>
+      <c r="M106" s="14"/>
+      <c r="N106" s="14"/>
+      <c r="O106" s="14"/>
+      <c r="P106" s="14"/>
+      <c r="Q106" s="14"/>
+      <c r="R106" s="14"/>
+      <c r="S106" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
updated and added new read me files:
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C5D29EE-7EAE-48F3-83FD-EBC2CDAD636F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F619F628-9506-438F-861D-5F72D71686AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8434,7 +8434,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>419</v>
+        <v>400</v>
       </c>
       <c r="C2" s="15" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
updated DO wave file creation
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42684E92-4E6D-4BF1-84A7-290E53D31816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA7618E-926E-4122-968F-9C70E6576832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9992,8 +9992,8 @@
       <c r="B53" s="20" t="s">
         <v>400</v>
       </c>
-      <c r="C53" s="16" t="s">
-        <v>47</v>
+      <c r="C53" s="15" t="s">
+        <v>2</v>
       </c>
       <c r="D53" s="16" t="s">
         <v>113</v>

</xml_diff>

<commit_message>
updated for congif gile
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA7618E-926E-4122-968F-9C70E6576832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{725FBEC7-9612-4B15-AC9F-52C7CB98E785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3700,7 +3700,7 @@
         <v>136</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E50" s="14"/>
       <c r="F50" s="14"/>
@@ -10263,8 +10263,8 @@
       <c r="A61" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="B61" s="20" t="s">
-        <v>139</v>
+      <c r="B61" s="18" t="s">
+        <v>419</v>
       </c>
       <c r="C61" s="16" t="s">
         <v>46</v>
@@ -10302,8 +10302,8 @@
       <c r="A62" s="16" t="s">
         <v>193</v>
       </c>
-      <c r="B62" s="20" t="s">
-        <v>139</v>
+      <c r="B62" s="18" t="s">
+        <v>419</v>
       </c>
       <c r="C62" s="16" t="s">
         <v>46</v>
@@ -10341,8 +10341,8 @@
       <c r="A63" s="16" t="s">
         <v>196</v>
       </c>
-      <c r="B63" s="20" t="s">
-        <v>139</v>
+      <c r="B63" s="18" t="s">
+        <v>419</v>
       </c>
       <c r="C63" s="16" t="s">
         <v>47</v>
@@ -10380,8 +10380,8 @@
       <c r="A64" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="B64" s="20" t="s">
-        <v>139</v>
+      <c r="B64" s="18" t="s">
+        <v>419</v>
       </c>
       <c r="C64" s="15" t="s">
         <v>47</v>
@@ -10407,7 +10407,7 @@
         <v>198</v>
       </c>
       <c r="B65" s="20" t="s">
-        <v>139</v>
+        <v>400</v>
       </c>
       <c r="C65" s="15" t="s">
         <v>47</v>
@@ -10446,7 +10446,7 @@
         <v>199</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>139</v>
+        <v>400</v>
       </c>
       <c r="C66" s="15" t="s">
         <v>47</v>

</xml_diff>

<commit_message>
updated receiving for no receive loc suggestion
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5352FCC6-8E8B-424F-8F23-4AA9DAE3C767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B9E50F-1F27-40DA-9D84-1D324DED3B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10228,8 +10228,8 @@
       <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="18" t="s">
-        <v>400</v>
+      <c r="B2" s="20" t="s">
+        <v>429</v>
       </c>
       <c r="C2" s="15" t="s">
         <v>70</v>
@@ -10340,8 +10340,8 @@
       <c r="A7" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="20" t="s">
-        <v>429</v>
+      <c r="B7" s="18" t="s">
+        <v>400</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>70</v>

</xml_diff>

<commit_message>
updated tags and scipt for shipments page
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B9E50F-1F27-40DA-9D84-1D324DED3B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8838D410-276B-4E88-9B65-B65639176A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1849" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1850" uniqueCount="481">
   <si>
     <t>1</t>
   </si>
@@ -10229,7 +10229,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>429</v>
+        <v>400</v>
       </c>
       <c r="C2" s="15" t="s">
         <v>70</v>
@@ -10341,7 +10341,7 @@
         <v>48</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>400</v>
+        <v>429</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>70</v>
@@ -11679,7 +11679,9 @@
         <v>406</v>
       </c>
       <c r="J49" s="19"/>
-      <c r="K49" s="19"/>
+      <c r="K49" s="14" t="s">
+        <v>135</v>
+      </c>
       <c r="L49" s="19"/>
       <c r="M49" s="14"/>
       <c r="N49" s="14"/>

</xml_diff>

<commit_message>
updated the olpn the barcode length 20 and ilpn barcode length of 20 for consume ilpn
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8838D410-276B-4E88-9B65-B65639176A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2259F824-671E-4A9A-9BC8-220E59B7A6D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1850" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1853" uniqueCount="483">
   <si>
     <t>1</t>
   </si>
@@ -1471,6 +1471,12 @@
   </si>
   <si>
     <t>FG-000404-00</t>
+  </si>
+  <si>
+    <t>LpnFLag</t>
+  </si>
+  <si>
+    <t>consumeilpn</t>
   </si>
 </sst>
 </file>
@@ -1623,7 +1629,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1661,6 +1667,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2001,7 +2008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH354"/>
+  <dimension ref="A1:AI354"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -2030,9 +2037,10 @@
     <col min="31" max="31" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="32" max="33" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>1</v>
       </c>
@@ -2135,8 +2143,11 @@
       <c r="AH1" s="22" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="2" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI1" s="29" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>205</v>
       </c>
@@ -2181,8 +2192,9 @@
       <c r="AF2" s="14"/>
       <c r="AG2" s="14"/>
       <c r="AH2" s="14"/>
-    </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI2" s="14"/>
+    </row>
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
         <v>206</v>
       </c>
@@ -2206,8 +2218,9 @@
       <c r="AF3" s="14"/>
       <c r="AG3" s="14"/>
       <c r="AH3" s="14"/>
-    </row>
-    <row r="4" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI3" s="14"/>
+    </row>
+    <row r="4" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>207</v>
       </c>
@@ -2256,8 +2269,9 @@
       <c r="AF4" s="14"/>
       <c r="AG4" s="14"/>
       <c r="AH4" s="14"/>
-    </row>
-    <row r="5" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI4" s="14"/>
+    </row>
+    <row r="5" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
         <v>382</v>
       </c>
@@ -2306,8 +2320,9 @@
       <c r="AF5" s="14"/>
       <c r="AG5" s="14"/>
       <c r="AH5" s="14"/>
-    </row>
-    <row r="6" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI5" s="14"/>
+    </row>
+    <row r="6" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>208</v>
       </c>
@@ -2354,8 +2369,9 @@
       <c r="AF6" s="14"/>
       <c r="AG6" s="14"/>
       <c r="AH6" s="14"/>
-    </row>
-    <row r="7" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI6" s="14"/>
+    </row>
+    <row r="7" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>209</v>
       </c>
@@ -2402,8 +2418,9 @@
       <c r="AF7" s="14"/>
       <c r="AG7" s="14"/>
       <c r="AH7" s="14"/>
-    </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI7" s="14"/>
+    </row>
+    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
         <v>210</v>
       </c>
@@ -2430,8 +2447,9 @@
       <c r="AF8" s="14"/>
       <c r="AG8" s="14"/>
       <c r="AH8" s="14"/>
-    </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI8" s="14"/>
+    </row>
+    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
         <v>211</v>
       </c>
@@ -2459,8 +2477,9 @@
       <c r="AF9" s="14"/>
       <c r="AG9" s="14"/>
       <c r="AH9" s="14"/>
-    </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI9" s="14"/>
+    </row>
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
         <v>212</v>
       </c>
@@ -2488,8 +2507,9 @@
       <c r="AF10" s="14"/>
       <c r="AG10" s="14"/>
       <c r="AH10" s="14"/>
-    </row>
-    <row r="11" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI10" s="14"/>
+    </row>
+    <row r="11" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
         <v>213</v>
       </c>
@@ -2536,8 +2556,9 @@
       <c r="AF11" s="14"/>
       <c r="AG11" s="14"/>
       <c r="AH11" s="14"/>
-    </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI11" s="14"/>
+    </row>
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
         <v>214</v>
       </c>
@@ -2564,8 +2585,9 @@
       <c r="AF12" s="14"/>
       <c r="AG12" s="14"/>
       <c r="AH12" s="14"/>
-    </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI12" s="14"/>
+    </row>
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
         <v>215</v>
       </c>
@@ -2592,8 +2614,9 @@
       <c r="AF13" s="14"/>
       <c r="AG13" s="14"/>
       <c r="AH13" s="14"/>
-    </row>
-    <row r="14" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI13" s="14"/>
+    </row>
+    <row r="14" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
         <v>399</v>
       </c>
@@ -2640,8 +2663,9 @@
       <c r="AF14" s="14"/>
       <c r="AG14" s="14"/>
       <c r="AH14" s="14"/>
-    </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI14" s="14"/>
+    </row>
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
         <v>216</v>
       </c>
@@ -2665,8 +2689,9 @@
       <c r="AF15" s="14"/>
       <c r="AG15" s="14"/>
       <c r="AH15" s="14"/>
-    </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI15" s="14"/>
+    </row>
+    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
         <v>217</v>
       </c>
@@ -2690,8 +2715,9 @@
       <c r="AF16" s="14"/>
       <c r="AG16" s="14"/>
       <c r="AH16" s="14"/>
-    </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI16" s="14"/>
+    </row>
+    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
         <v>218</v>
       </c>
@@ -2720,8 +2746,9 @@
       <c r="AF17" s="14"/>
       <c r="AG17" s="14"/>
       <c r="AH17" s="14"/>
-    </row>
-    <row r="18" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI17" s="14"/>
+    </row>
+    <row r="18" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
         <v>219</v>
       </c>
@@ -2750,8 +2777,9 @@
       <c r="AF18" s="14"/>
       <c r="AG18" s="14"/>
       <c r="AH18" s="14"/>
-    </row>
-    <row r="19" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI18" s="14"/>
+    </row>
+    <row r="19" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
         <v>220</v>
       </c>
@@ -2778,8 +2806,9 @@
       <c r="AF19" s="14"/>
       <c r="AG19" s="14"/>
       <c r="AH19" s="14"/>
-    </row>
-    <row r="20" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI19" s="14"/>
+    </row>
+    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
         <v>221</v>
       </c>
@@ -2806,8 +2835,9 @@
       <c r="AF20" s="14"/>
       <c r="AG20" s="14"/>
       <c r="AH20" s="14"/>
-    </row>
-    <row r="21" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI20" s="14"/>
+    </row>
+    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
         <v>222</v>
       </c>
@@ -2835,8 +2865,9 @@
       <c r="AF21" s="14"/>
       <c r="AG21" s="14"/>
       <c r="AH21" s="14"/>
-    </row>
-    <row r="22" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI21" s="14"/>
+    </row>
+    <row r="22" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
         <v>223</v>
       </c>
@@ -2862,8 +2893,9 @@
       <c r="AF22" s="14"/>
       <c r="AG22" s="14"/>
       <c r="AH22" s="14"/>
-    </row>
-    <row r="23" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI22" s="14"/>
+    </row>
+    <row r="23" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
         <v>224</v>
       </c>
@@ -2891,8 +2923,11 @@
       <c r="AF23" s="14"/>
       <c r="AG23" s="14"/>
       <c r="AH23" s="14"/>
-    </row>
-    <row r="24" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI23" s="14" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="24" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
         <v>225</v>
       </c>
@@ -2918,8 +2953,11 @@
       <c r="AF24" s="14"/>
       <c r="AG24" s="14"/>
       <c r="AH24" s="14"/>
-    </row>
-    <row r="25" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI24" s="14" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="25" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
         <v>226</v>
       </c>
@@ -2945,8 +2983,9 @@
       <c r="AF25" s="14"/>
       <c r="AG25" s="14"/>
       <c r="AH25" s="14"/>
-    </row>
-    <row r="26" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI25" s="14"/>
+    </row>
+    <row r="26" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
         <v>227</v>
       </c>
@@ -2972,8 +3011,9 @@
       <c r="AF26" s="14"/>
       <c r="AG26" s="14"/>
       <c r="AH26" s="14"/>
-    </row>
-    <row r="27" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI26" s="14"/>
+    </row>
+    <row r="27" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
         <v>228</v>
       </c>
@@ -2999,8 +3039,9 @@
       <c r="AF27" s="14"/>
       <c r="AG27" s="14"/>
       <c r="AH27" s="14"/>
-    </row>
-    <row r="28" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI27" s="14"/>
+    </row>
+    <row r="28" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
         <v>229</v>
       </c>
@@ -3045,8 +3086,9 @@
       <c r="AF28" s="14"/>
       <c r="AG28" s="14"/>
       <c r="AH28" s="14"/>
-    </row>
-    <row r="29" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI28" s="14"/>
+    </row>
+    <row r="29" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
         <v>230</v>
       </c>
@@ -3091,8 +3133,9 @@
       <c r="AF29" s="14"/>
       <c r="AG29" s="14"/>
       <c r="AH29" s="14"/>
-    </row>
-    <row r="30" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI29" s="14"/>
+    </row>
+    <row r="30" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
         <v>231</v>
       </c>
@@ -3137,8 +3180,9 @@
       <c r="AF30" s="14"/>
       <c r="AG30" s="14"/>
       <c r="AH30" s="14"/>
-    </row>
-    <row r="31" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI30" s="14"/>
+    </row>
+    <row r="31" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
         <v>232</v>
       </c>
@@ -3183,8 +3227,9 @@
       <c r="AF31" s="14"/>
       <c r="AG31" s="14"/>
       <c r="AH31" s="14"/>
-    </row>
-    <row r="32" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI31" s="14"/>
+    </row>
+    <row r="32" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
         <v>233</v>
       </c>
@@ -3229,8 +3274,9 @@
       <c r="AF32" s="14"/>
       <c r="AG32" s="14"/>
       <c r="AH32" s="14"/>
-    </row>
-    <row r="33" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI32" s="14"/>
+    </row>
+    <row r="33" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
         <v>234</v>
       </c>
@@ -3275,8 +3321,9 @@
       <c r="AF33" s="14"/>
       <c r="AG33" s="14"/>
       <c r="AH33" s="14"/>
-    </row>
-    <row r="34" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI33" s="14"/>
+    </row>
+    <row r="34" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
         <v>235</v>
       </c>
@@ -3321,8 +3368,9 @@
       <c r="AF34" s="14"/>
       <c r="AG34" s="14"/>
       <c r="AH34" s="14"/>
-    </row>
-    <row r="35" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI34" s="14"/>
+    </row>
+    <row r="35" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
         <v>236</v>
       </c>
@@ -3367,8 +3415,9 @@
       <c r="AF35" s="14"/>
       <c r="AG35" s="14"/>
       <c r="AH35" s="14"/>
-    </row>
-    <row r="36" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI35" s="14"/>
+    </row>
+    <row r="36" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
         <v>237</v>
       </c>
@@ -3413,8 +3462,9 @@
       <c r="AF36" s="14"/>
       <c r="AG36" s="14"/>
       <c r="AH36" s="14"/>
-    </row>
-    <row r="37" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI36" s="14"/>
+    </row>
+    <row r="37" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
         <v>354</v>
       </c>
@@ -3459,8 +3509,9 @@
       <c r="AF37" s="14"/>
       <c r="AG37" s="14"/>
       <c r="AH37" s="14"/>
-    </row>
-    <row r="38" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI37" s="14"/>
+    </row>
+    <row r="38" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
         <v>355</v>
       </c>
@@ -3505,8 +3556,9 @@
       <c r="AF38" s="14"/>
       <c r="AG38" s="14"/>
       <c r="AH38" s="14"/>
-    </row>
-    <row r="39" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI38" s="14"/>
+    </row>
+    <row r="39" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
         <v>356</v>
       </c>
@@ -3551,8 +3603,9 @@
       <c r="AF39" s="14"/>
       <c r="AG39" s="14"/>
       <c r="AH39" s="14"/>
-    </row>
-    <row r="40" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI39" s="14"/>
+    </row>
+    <row r="40" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
         <v>391</v>
       </c>
@@ -3599,8 +3652,9 @@
       <c r="AF40" s="14"/>
       <c r="AG40" s="14"/>
       <c r="AH40" s="14"/>
-    </row>
-    <row r="41" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI40" s="14"/>
+    </row>
+    <row r="41" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="15" t="s">
         <v>412</v>
       </c>
@@ -3647,8 +3701,9 @@
       <c r="AF41" s="14"/>
       <c r="AG41" s="14"/>
       <c r="AH41" s="14"/>
-    </row>
-    <row r="42" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI41" s="14"/>
+    </row>
+    <row r="42" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
         <v>420</v>
       </c>
@@ -3695,8 +3750,9 @@
       <c r="AF42" s="14"/>
       <c r="AG42" s="14"/>
       <c r="AH42" s="14"/>
-    </row>
-    <row r="43" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI42" s="14"/>
+    </row>
+    <row r="43" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
         <v>353</v>
       </c>
@@ -3741,8 +3797,9 @@
       <c r="AF43" s="14"/>
       <c r="AG43" s="14"/>
       <c r="AH43" s="14"/>
-    </row>
-    <row r="44" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI43" s="14"/>
+    </row>
+    <row r="44" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="15"/>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
@@ -3777,8 +3834,9 @@
       <c r="AF44" s="14"/>
       <c r="AG44" s="14"/>
       <c r="AH44" s="14"/>
-    </row>
-    <row r="45" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI44" s="14"/>
+    </row>
+    <row r="45" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
         <v>138</v>
       </c>
@@ -3827,8 +3885,9 @@
       <c r="AF45" s="14"/>
       <c r="AG45" s="14"/>
       <c r="AH45" s="14"/>
-    </row>
-    <row r="46" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI45" s="14"/>
+    </row>
+    <row r="46" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
         <v>145</v>
       </c>
@@ -3877,8 +3936,9 @@
       <c r="AF46" s="14"/>
       <c r="AG46" s="14"/>
       <c r="AH46" s="14"/>
-    </row>
-    <row r="47" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI46" s="14"/>
+    </row>
+    <row r="47" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
         <v>147</v>
       </c>
@@ -3927,8 +3987,9 @@
       <c r="AF47" s="14"/>
       <c r="AG47" s="14"/>
       <c r="AH47" s="14"/>
-    </row>
-    <row r="48" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI47" s="14"/>
+    </row>
+    <row r="48" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
         <v>154</v>
       </c>
@@ -3979,8 +4040,9 @@
       <c r="AF48" s="14"/>
       <c r="AG48" s="14"/>
       <c r="AH48" s="14"/>
-    </row>
-    <row r="49" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI48" s="14"/>
+    </row>
+    <row r="49" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
         <v>159</v>
       </c>
@@ -4031,8 +4093,9 @@
       <c r="AF49" s="14"/>
       <c r="AG49" s="14"/>
       <c r="AH49" s="14"/>
-    </row>
-    <row r="50" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI49" s="14"/>
+    </row>
+    <row r="50" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
         <v>171</v>
       </c>
@@ -4083,8 +4146,9 @@
       <c r="AF50" s="14"/>
       <c r="AG50" s="14"/>
       <c r="AH50" s="14"/>
-    </row>
-    <row r="51" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI50" s="14"/>
+    </row>
+    <row r="51" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
         <v>175</v>
       </c>
@@ -4135,8 +4199,9 @@
       <c r="AF51" s="14"/>
       <c r="AG51" s="14"/>
       <c r="AH51" s="14"/>
-    </row>
-    <row r="52" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI51" s="14"/>
+    </row>
+    <row r="52" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
         <v>188</v>
       </c>
@@ -4187,8 +4252,9 @@
       <c r="AF52" s="14"/>
       <c r="AG52" s="14"/>
       <c r="AH52" s="14"/>
-    </row>
-    <row r="53" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI52" s="14"/>
+    </row>
+    <row r="53" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
         <v>189</v>
       </c>
@@ -4237,8 +4303,9 @@
       <c r="AF53" s="14"/>
       <c r="AG53" s="14"/>
       <c r="AH53" s="14"/>
-    </row>
-    <row r="54" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI53" s="14"/>
+    </row>
+    <row r="54" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
         <v>190</v>
       </c>
@@ -4287,8 +4354,9 @@
       <c r="AF54" s="14"/>
       <c r="AG54" s="14"/>
       <c r="AH54" s="14"/>
-    </row>
-    <row r="55" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI54" s="14"/>
+    </row>
+    <row r="55" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
         <v>191</v>
       </c>
@@ -4337,8 +4405,9 @@
       <c r="AF55" s="14"/>
       <c r="AG55" s="14"/>
       <c r="AH55" s="14"/>
-    </row>
-    <row r="56" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI55" s="14"/>
+    </row>
+    <row r="56" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
         <v>202</v>
       </c>
@@ -4387,8 +4456,9 @@
       <c r="AF56" s="14"/>
       <c r="AG56" s="14"/>
       <c r="AH56" s="14"/>
-    </row>
-    <row r="57" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI56" s="14"/>
+    </row>
+    <row r="57" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
         <v>260</v>
       </c>
@@ -4441,8 +4511,9 @@
       <c r="AF57" s="14"/>
       <c r="AG57" s="14"/>
       <c r="AH57" s="14"/>
-    </row>
-    <row r="58" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI57" s="14"/>
+    </row>
+    <row r="58" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
         <v>261</v>
       </c>
@@ -4495,8 +4566,9 @@
       <c r="AF58" s="14"/>
       <c r="AG58" s="14"/>
       <c r="AH58" s="14"/>
-    </row>
-    <row r="59" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI58" s="14"/>
+    </row>
+    <row r="59" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
         <v>262</v>
       </c>
@@ -4549,8 +4621,9 @@
       <c r="AF59" s="14"/>
       <c r="AG59" s="14"/>
       <c r="AH59" s="14"/>
-    </row>
-    <row r="60" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI59" s="14"/>
+    </row>
+    <row r="60" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
         <v>263</v>
       </c>
@@ -4605,8 +4678,9 @@
       <c r="AF60" s="14"/>
       <c r="AG60" s="14"/>
       <c r="AH60" s="14"/>
-    </row>
-    <row r="61" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI60" s="14"/>
+    </row>
+    <row r="61" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
         <v>264</v>
       </c>
@@ -4661,8 +4735,9 @@
       <c r="AF61" s="14"/>
       <c r="AG61" s="14"/>
       <c r="AH61" s="14"/>
-    </row>
-    <row r="62" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI61" s="14"/>
+    </row>
+    <row r="62" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
         <v>421</v>
       </c>
@@ -4719,8 +4794,9 @@
       <c r="AH62" s="14" t="s">
         <v>469</v>
       </c>
-    </row>
-    <row r="63" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI62" s="14"/>
+    </row>
+    <row r="63" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
         <v>473</v>
       </c>
@@ -4777,8 +4853,9 @@
       <c r="AH63" s="15" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="64" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI63" s="14"/>
+    </row>
+    <row r="64" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
         <v>477</v>
       </c>
@@ -4835,8 +4912,9 @@
       <c r="AH64" s="15" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="65" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI64" s="14"/>
+    </row>
+    <row r="65" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="14"/>
       <c r="B65" s="14"/>
       <c r="C65" s="14"/>
@@ -4871,8 +4949,9 @@
       <c r="AF65" s="14"/>
       <c r="AG65" s="14"/>
       <c r="AH65" s="14"/>
-    </row>
-    <row r="66" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI65" s="14"/>
+    </row>
+    <row r="66" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
         <v>458</v>
       </c>
@@ -4923,8 +5002,9 @@
       <c r="AH66" s="14" t="s">
         <v>462</v>
       </c>
-    </row>
-    <row r="67" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI66" s="14"/>
+    </row>
+    <row r="67" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
         <v>464</v>
       </c>
@@ -4975,8 +5055,9 @@
       <c r="AH67" s="15" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="68" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI67" s="14"/>
+    </row>
+    <row r="68" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
         <v>434</v>
       </c>
@@ -5025,8 +5106,9 @@
       <c r="AF68" s="14"/>
       <c r="AG68" s="14"/>
       <c r="AH68" s="14"/>
-    </row>
-    <row r="69" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI68" s="14"/>
+    </row>
+    <row r="69" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="14" t="s">
         <v>435</v>
       </c>
@@ -5077,8 +5159,9 @@
       <c r="AH69" s="14" t="s">
         <v>462</v>
       </c>
-    </row>
-    <row r="70" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI69" s="14"/>
+    </row>
+    <row r="70" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="14" t="s">
         <v>436</v>
       </c>
@@ -5127,8 +5210,9 @@
       <c r="AF70" s="14"/>
       <c r="AG70" s="14"/>
       <c r="AH70" s="14"/>
-    </row>
-    <row r="71" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI70" s="14"/>
+    </row>
+    <row r="71" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="14" t="s">
         <v>453</v>
       </c>
@@ -5177,8 +5261,9 @@
       <c r="AF71" s="14"/>
       <c r="AG71" s="14"/>
       <c r="AH71" s="14"/>
-    </row>
-    <row r="72" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI71" s="14"/>
+    </row>
+    <row r="72" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="14" t="s">
         <v>437</v>
       </c>
@@ -5225,8 +5310,9 @@
       <c r="AF72" s="14"/>
       <c r="AG72" s="14"/>
       <c r="AH72" s="14"/>
-    </row>
-    <row r="73" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI72" s="14"/>
+    </row>
+    <row r="73" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="14" t="s">
         <v>440</v>
       </c>
@@ -5275,8 +5361,9 @@
       <c r="AF73" s="14"/>
       <c r="AG73" s="14"/>
       <c r="AH73" s="14"/>
-    </row>
-    <row r="74" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI73" s="14"/>
+    </row>
+    <row r="74" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="14" t="s">
         <v>445</v>
       </c>
@@ -5325,8 +5412,9 @@
       <c r="AF74" s="14"/>
       <c r="AG74" s="14"/>
       <c r="AH74" s="14"/>
-    </row>
-    <row r="75" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI74" s="14"/>
+    </row>
+    <row r="75" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
         <v>446</v>
       </c>
@@ -5373,8 +5461,9 @@
       <c r="AF75" s="14"/>
       <c r="AG75" s="14"/>
       <c r="AH75" s="14"/>
-    </row>
-    <row r="76" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI75" s="14"/>
+    </row>
+    <row r="76" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="14" t="s">
         <v>451</v>
       </c>
@@ -5425,8 +5514,9 @@
         <v>452</v>
       </c>
       <c r="AH76" s="14"/>
-    </row>
-    <row r="77" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI76" s="14"/>
+    </row>
+    <row r="77" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
         <v>466</v>
       </c>
@@ -5479,8 +5569,9 @@
       <c r="AH77" s="14" t="s">
         <v>469</v>
       </c>
-    </row>
-    <row r="78" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI77" s="14"/>
+    </row>
+    <row r="78" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="14"/>
       <c r="B78" s="14"/>
       <c r="C78" s="14"/>
@@ -5515,8 +5606,9 @@
       <c r="AF78" s="14"/>
       <c r="AG78" s="14"/>
       <c r="AH78" s="14"/>
-    </row>
-    <row r="79" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI78" s="14"/>
+    </row>
+    <row r="79" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="14" t="s">
         <v>304</v>
       </c>
@@ -5559,8 +5651,9 @@
       <c r="AF79" s="14"/>
       <c r="AG79" s="14"/>
       <c r="AH79" s="14"/>
-    </row>
-    <row r="80" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI79" s="14"/>
+    </row>
+    <row r="80" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="14" t="s">
         <v>305</v>
       </c>
@@ -5603,8 +5696,9 @@
       <c r="AF80" s="14"/>
       <c r="AG80" s="14"/>
       <c r="AH80" s="14"/>
-    </row>
-    <row r="81" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI80" s="14"/>
+    </row>
+    <row r="81" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="14" t="s">
         <v>306</v>
       </c>
@@ -5651,8 +5745,9 @@
       <c r="AF81" s="14"/>
       <c r="AG81" s="14"/>
       <c r="AH81" s="14"/>
-    </row>
-    <row r="82" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI81" s="14"/>
+    </row>
+    <row r="82" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="14" t="s">
         <v>307</v>
       </c>
@@ -5699,8 +5794,9 @@
       <c r="AF82" s="14"/>
       <c r="AG82" s="14"/>
       <c r="AH82" s="14"/>
-    </row>
-    <row r="83" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI82" s="14"/>
+    </row>
+    <row r="83" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="14" t="s">
         <v>344</v>
       </c>
@@ -5743,8 +5839,9 @@
       <c r="AF83" s="14"/>
       <c r="AG83" s="14"/>
       <c r="AH83" s="14"/>
-    </row>
-    <row r="84" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI83" s="14"/>
+    </row>
+    <row r="84" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="14" t="s">
         <v>345</v>
       </c>
@@ -5787,8 +5884,9 @@
       <c r="AF84" s="14"/>
       <c r="AG84" s="14"/>
       <c r="AH84" s="14"/>
-    </row>
-    <row r="85" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI84" s="14"/>
+    </row>
+    <row r="85" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="14" t="s">
         <v>346</v>
       </c>
@@ -5831,8 +5929,9 @@
       <c r="AF85" s="14"/>
       <c r="AG85" s="14"/>
       <c r="AH85" s="14"/>
-    </row>
-    <row r="86" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI85" s="14"/>
+    </row>
+    <row r="86" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="14" t="s">
         <v>347</v>
       </c>
@@ -5875,8 +5974,9 @@
       <c r="AF86" s="14"/>
       <c r="AG86" s="14"/>
       <c r="AH86" s="14"/>
-    </row>
-    <row r="87" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI86" s="14"/>
+    </row>
+    <row r="87" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="14" t="s">
         <v>352</v>
       </c>
@@ -5917,8 +6017,9 @@
       <c r="AF87" s="14"/>
       <c r="AG87" s="14"/>
       <c r="AH87" s="14"/>
-    </row>
-    <row r="88" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI87" s="14"/>
+    </row>
+    <row r="88" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="14"/>
       <c r="B88" s="14"/>
       <c r="C88" s="14"/>
@@ -5953,8 +6054,9 @@
       <c r="AF88" s="14"/>
       <c r="AG88" s="14"/>
       <c r="AH88" s="14"/>
-    </row>
-    <row r="89" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI88" s="14"/>
+    </row>
+    <row r="89" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="12" t="s">
         <v>367</v>
       </c>
@@ -6001,8 +6103,9 @@
       <c r="AF89" s="14"/>
       <c r="AG89" s="14"/>
       <c r="AH89" s="14"/>
-    </row>
-    <row r="90" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI89" s="14"/>
+    </row>
+    <row r="90" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="12" t="s">
         <v>368</v>
       </c>
@@ -6045,8 +6148,9 @@
       <c r="AF90" s="14"/>
       <c r="AG90" s="14"/>
       <c r="AH90" s="14"/>
-    </row>
-    <row r="91" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI90" s="14"/>
+    </row>
+    <row r="91" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="12" t="s">
         <v>369</v>
       </c>
@@ -6089,8 +6193,9 @@
       <c r="AF91" s="14"/>
       <c r="AG91" s="14"/>
       <c r="AH91" s="14"/>
-    </row>
-    <row r="92" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI91" s="14"/>
+    </row>
+    <row r="92" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="12" t="s">
         <v>370</v>
       </c>
@@ -6133,8 +6238,9 @@
       <c r="AF92" s="14"/>
       <c r="AG92" s="14"/>
       <c r="AH92" s="14"/>
-    </row>
-    <row r="93" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI92" s="14"/>
+    </row>
+    <row r="93" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
         <v>371</v>
       </c>
@@ -6177,8 +6283,9 @@
       <c r="AF93" s="14"/>
       <c r="AG93" s="14"/>
       <c r="AH93" s="14"/>
-    </row>
-    <row r="94" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI93" s="14"/>
+    </row>
+    <row r="94" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="14"/>
       <c r="B94" s="14"/>
       <c r="C94" s="14"/>
@@ -6213,8 +6320,9 @@
       <c r="AF94" s="14"/>
       <c r="AG94" s="14"/>
       <c r="AH94" s="14"/>
-    </row>
-    <row r="95" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI94" s="14"/>
+    </row>
+    <row r="95" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
         <v>308</v>
       </c>
@@ -6269,8 +6377,9 @@
       <c r="AF95" s="12"/>
       <c r="AG95" s="12"/>
       <c r="AH95" s="12"/>
-    </row>
-    <row r="96" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI95" s="12"/>
+    </row>
+    <row r="96" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="12" t="s">
         <v>314</v>
       </c>
@@ -6325,8 +6434,9 @@
       <c r="AF96" s="12"/>
       <c r="AG96" s="12"/>
       <c r="AH96" s="12"/>
-    </row>
-    <row r="97" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI96" s="12"/>
+    </row>
+    <row r="97" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
         <v>315</v>
       </c>
@@ -6379,8 +6489,9 @@
       <c r="AF97" s="12"/>
       <c r="AG97" s="12"/>
       <c r="AH97" s="12"/>
-    </row>
-    <row r="98" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI97" s="12"/>
+    </row>
+    <row r="98" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="12" t="s">
         <v>318</v>
       </c>
@@ -6433,8 +6544,9 @@
       <c r="AF98" s="12"/>
       <c r="AG98" s="12"/>
       <c r="AH98" s="12"/>
-    </row>
-    <row r="99" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI98" s="12"/>
+    </row>
+    <row r="99" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="12" t="s">
         <v>320</v>
       </c>
@@ -6487,8 +6599,9 @@
       <c r="AF99" s="12"/>
       <c r="AG99" s="12"/>
       <c r="AH99" s="12"/>
-    </row>
-    <row r="100" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI99" s="12"/>
+    </row>
+    <row r="100" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="12" t="s">
         <v>322</v>
       </c>
@@ -6541,8 +6654,9 @@
       <c r="AF100" s="12"/>
       <c r="AG100" s="12"/>
       <c r="AH100" s="12"/>
-    </row>
-    <row r="101" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI100" s="12"/>
+    </row>
+    <row r="101" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="12" t="s">
         <v>323</v>
       </c>
@@ -6597,8 +6711,9 @@
       <c r="AF101" s="12"/>
       <c r="AG101" s="12"/>
       <c r="AH101" s="12"/>
-    </row>
-    <row r="102" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI101" s="12"/>
+    </row>
+    <row r="102" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="12" t="s">
         <v>326</v>
       </c>
@@ -6653,8 +6768,9 @@
       <c r="AF102" s="12"/>
       <c r="AG102" s="12"/>
       <c r="AH102" s="12"/>
-    </row>
-    <row r="103" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI102" s="12"/>
+    </row>
+    <row r="103" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="12" t="s">
         <v>328</v>
       </c>
@@ -6709,8 +6825,9 @@
       <c r="AF103" s="12"/>
       <c r="AG103" s="12"/>
       <c r="AH103" s="12"/>
-    </row>
-    <row r="104" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI103" s="12"/>
+    </row>
+    <row r="104" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="12" t="s">
         <v>330</v>
       </c>
@@ -6765,8 +6882,9 @@
       <c r="AF104" s="12"/>
       <c r="AG104" s="12"/>
       <c r="AH104" s="12"/>
-    </row>
-    <row r="105" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI104" s="12"/>
+    </row>
+    <row r="105" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="12" t="s">
         <v>332</v>
       </c>
@@ -6821,8 +6939,9 @@
       <c r="AF105" s="12"/>
       <c r="AG105" s="12"/>
       <c r="AH105" s="12"/>
-    </row>
-    <row r="106" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI105" s="12"/>
+    </row>
+    <row r="106" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="12" t="s">
         <v>334</v>
       </c>
@@ -6877,8 +6996,9 @@
       <c r="AF106" s="12"/>
       <c r="AG106" s="12"/>
       <c r="AH106" s="12"/>
-    </row>
-    <row r="107" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI106" s="12"/>
+    </row>
+    <row r="107" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="12" t="s">
         <v>336</v>
       </c>
@@ -6933,8 +7053,9 @@
       <c r="AF107" s="12"/>
       <c r="AG107" s="12"/>
       <c r="AH107" s="12"/>
-    </row>
-    <row r="108" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI107" s="12"/>
+    </row>
+    <row r="108" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="12"/>
       <c r="B108" s="12"/>
       <c r="C108" s="12"/>
@@ -6969,8 +7090,9 @@
       <c r="AF108" s="12"/>
       <c r="AG108" s="12"/>
       <c r="AH108" s="12"/>
-    </row>
-    <row r="109" spans="1:34" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI108" s="12"/>
+    </row>
+    <row r="109" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="12"/>
       <c r="B109" s="12"/>
       <c r="C109" s="12"/>
@@ -7005,8 +7127,9 @@
       <c r="AF109" s="12"/>
       <c r="AG109" s="12"/>
       <c r="AH109" s="12"/>
-    </row>
-    <row r="110" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI109" s="12"/>
+    </row>
+    <row r="110" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A110" s="14" t="s">
         <v>245</v>
       </c>
@@ -7032,8 +7155,9 @@
       <c r="AF110" s="14"/>
       <c r="AG110" s="14"/>
       <c r="AH110" s="14"/>
-    </row>
-    <row r="111" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI110" s="14"/>
+    </row>
+    <row r="111" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A111" s="14" t="s">
         <v>246</v>
       </c>
@@ -7059,8 +7183,9 @@
       <c r="AF111" s="14"/>
       <c r="AG111" s="14"/>
       <c r="AH111" s="14"/>
-    </row>
-    <row r="112" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI111" s="14"/>
+    </row>
+    <row r="112" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A112" s="14" t="s">
         <v>247</v>
       </c>
@@ -7086,8 +7211,9 @@
       <c r="AF112" s="14"/>
       <c r="AG112" s="14"/>
       <c r="AH112" s="14"/>
-    </row>
-    <row r="113" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI112" s="14"/>
+    </row>
+    <row r="113" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A113" s="14" t="s">
         <v>248</v>
       </c>
@@ -7113,8 +7239,9 @@
       <c r="AF113" s="14"/>
       <c r="AG113" s="14"/>
       <c r="AH113" s="14"/>
-    </row>
-    <row r="114" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI113" s="14"/>
+    </row>
+    <row r="114" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A114" s="14" t="s">
         <v>249</v>
       </c>
@@ -7140,8 +7267,9 @@
       <c r="AF114" s="14"/>
       <c r="AG114" s="14"/>
       <c r="AH114" s="14"/>
-    </row>
-    <row r="115" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI114" s="14"/>
+    </row>
+    <row r="115" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A115" s="14" t="s">
         <v>250</v>
       </c>
@@ -7167,8 +7295,9 @@
       <c r="AF115" s="14"/>
       <c r="AG115" s="14"/>
       <c r="AH115" s="14"/>
-    </row>
-    <row r="116" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI115" s="14"/>
+    </row>
+    <row r="116" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A116" s="14" t="s">
         <v>251</v>
       </c>
@@ -7194,8 +7323,9 @@
       <c r="AF116" s="14"/>
       <c r="AG116" s="14"/>
       <c r="AH116" s="14"/>
-    </row>
-    <row r="117" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI116" s="14"/>
+    </row>
+    <row r="117" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="14" t="s">
         <v>252</v>
       </c>
@@ -7240,8 +7370,9 @@
       <c r="AF117" s="14"/>
       <c r="AG117" s="14"/>
       <c r="AH117" s="14"/>
-    </row>
-    <row r="118" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI117" s="14"/>
+    </row>
+    <row r="118" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="14" t="s">
         <v>253</v>
       </c>
@@ -7286,8 +7417,9 @@
       <c r="AF118" s="14"/>
       <c r="AG118" s="14"/>
       <c r="AH118" s="14"/>
-    </row>
-    <row r="119" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI118" s="14"/>
+    </row>
+    <row r="119" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A119" s="14" t="s">
         <v>254</v>
       </c>
@@ -7311,8 +7443,9 @@
       <c r="AF119" s="14"/>
       <c r="AG119" s="14"/>
       <c r="AH119" s="14"/>
-    </row>
-    <row r="120" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI119" s="14"/>
+    </row>
+    <row r="120" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A120" s="14" t="s">
         <v>255</v>
       </c>
@@ -7336,8 +7469,9 @@
       <c r="AF120" s="14"/>
       <c r="AG120" s="14"/>
       <c r="AH120" s="14"/>
-    </row>
-    <row r="121" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI120" s="14"/>
+    </row>
+    <row r="121" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A121" s="14" t="s">
         <v>256</v>
       </c>
@@ -7361,8 +7495,9 @@
       <c r="AF121" s="14"/>
       <c r="AG121" s="14"/>
       <c r="AH121" s="14"/>
-    </row>
-    <row r="122" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI121" s="14"/>
+    </row>
+    <row r="122" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A122" s="14" t="s">
         <v>257</v>
       </c>
@@ -7388,8 +7523,9 @@
       <c r="AF122" s="14"/>
       <c r="AG122" s="14"/>
       <c r="AH122" s="14"/>
-    </row>
-    <row r="123" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI122" s="14"/>
+    </row>
+    <row r="123" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A123" s="14" t="s">
         <v>258</v>
       </c>
@@ -7415,8 +7551,9 @@
       <c r="AF123" s="14"/>
       <c r="AG123" s="14"/>
       <c r="AH123" s="14"/>
-    </row>
-    <row r="124" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI123" s="14"/>
+    </row>
+    <row r="124" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="14" t="s">
         <v>280</v>
       </c>
@@ -7463,8 +7600,9 @@
       <c r="AF124" s="14"/>
       <c r="AG124" s="14"/>
       <c r="AH124" s="14"/>
-    </row>
-    <row r="125" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI124" s="14"/>
+    </row>
+    <row r="125" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="14" t="s">
         <v>287</v>
       </c>
@@ -7511,8 +7649,9 @@
       <c r="AF125" s="14"/>
       <c r="AG125" s="14"/>
       <c r="AH125" s="14"/>
-    </row>
-    <row r="126" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI125" s="14"/>
+    </row>
+    <row r="126" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="14" t="s">
         <v>289</v>
       </c>
@@ -7559,8 +7698,9 @@
       <c r="AF126" s="14"/>
       <c r="AG126" s="14"/>
       <c r="AH126" s="14"/>
-    </row>
-    <row r="127" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI126" s="14"/>
+    </row>
+    <row r="127" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="14" t="s">
         <v>290</v>
       </c>
@@ -7607,8 +7747,9 @@
       <c r="AF127" s="14"/>
       <c r="AG127" s="14"/>
       <c r="AH127" s="14"/>
-    </row>
-    <row r="128" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI127" s="14"/>
+    </row>
+    <row r="128" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="14" t="s">
         <v>294</v>
       </c>
@@ -7655,8 +7796,9 @@
       <c r="AF128" s="14"/>
       <c r="AG128" s="14"/>
       <c r="AH128" s="14"/>
-    </row>
-    <row r="129" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI128" s="14"/>
+    </row>
+    <row r="129" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="14" t="s">
         <v>296</v>
       </c>
@@ -7703,8 +7845,9 @@
       <c r="AF129" s="14"/>
       <c r="AG129" s="14"/>
       <c r="AH129" s="14"/>
-    </row>
-    <row r="130" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI129" s="14"/>
+    </row>
+    <row r="130" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="14" t="s">
         <v>375</v>
       </c>
@@ -7751,8 +7894,9 @@
       <c r="AF130" s="14"/>
       <c r="AG130" s="14"/>
       <c r="AH130" s="14"/>
-    </row>
-    <row r="131" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI130" s="14"/>
+    </row>
+    <row r="131" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="14" t="s">
         <v>377</v>
       </c>
@@ -7799,8 +7943,9 @@
       <c r="AF131" s="14"/>
       <c r="AG131" s="14"/>
       <c r="AH131" s="14"/>
-    </row>
-    <row r="132" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI131" s="14"/>
+    </row>
+    <row r="132" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="14" t="s">
         <v>384</v>
       </c>
@@ -7847,8 +7992,9 @@
       <c r="AF132" s="14"/>
       <c r="AG132" s="14"/>
       <c r="AH132" s="14"/>
-    </row>
-    <row r="133" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI132" s="14"/>
+    </row>
+    <row r="133" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="14" t="s">
         <v>385</v>
       </c>
@@ -7895,8 +8041,9 @@
       <c r="AF133" s="14"/>
       <c r="AG133" s="14"/>
       <c r="AH133" s="14"/>
-    </row>
-    <row r="134" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI133" s="14"/>
+    </row>
+    <row r="134" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="14" t="s">
         <v>392</v>
       </c>
@@ -7941,8 +8088,9 @@
       <c r="AF134" s="14"/>
       <c r="AG134" s="14"/>
       <c r="AH134" s="14"/>
-    </row>
-    <row r="135" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI134" s="14"/>
+    </row>
+    <row r="135" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="14"/>
       <c r="B135" s="14"/>
       <c r="C135" s="14"/>
@@ -7977,8 +8125,9 @@
       <c r="AF135" s="14"/>
       <c r="AG135" s="14"/>
       <c r="AH135" s="14"/>
-    </row>
-    <row r="136" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI135" s="14"/>
+    </row>
+    <row r="136" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="14"/>
       <c r="B136" s="14"/>
       <c r="C136" s="14"/>
@@ -8013,8 +8162,9 @@
       <c r="AF136" s="14"/>
       <c r="AG136" s="14"/>
       <c r="AH136" s="14"/>
-    </row>
-    <row r="137" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI136" s="14"/>
+    </row>
+    <row r="137" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="14"/>
       <c r="B137" s="14"/>
       <c r="C137" s="14"/>
@@ -8049,8 +8199,9 @@
       <c r="AF137" s="14"/>
       <c r="AG137" s="14"/>
       <c r="AH137" s="14"/>
-    </row>
-    <row r="138" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI137" s="14"/>
+    </row>
+    <row r="138" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB138" s="14"/>
       <c r="AC138" s="14"/>
       <c r="AD138" s="14"/>
@@ -8058,8 +8209,9 @@
       <c r="AF138" s="14"/>
       <c r="AG138" s="14"/>
       <c r="AH138" s="14"/>
-    </row>
-    <row r="139" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI138" s="14"/>
+    </row>
+    <row r="139" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="14" t="s">
         <v>269</v>
       </c>
@@ -8106,8 +8258,9 @@
       <c r="AF139" s="14"/>
       <c r="AG139" s="14"/>
       <c r="AH139" s="14"/>
-    </row>
-    <row r="140" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="AI139" s="14"/>
+    </row>
+    <row r="140" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="14" t="s">
         <v>270</v>
       </c>
@@ -8154,8 +8307,9 @@
       <c r="AF140" s="14"/>
       <c r="AG140" s="14"/>
       <c r="AH140" s="14"/>
-    </row>
-    <row r="141" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI140" s="14"/>
+    </row>
+    <row r="141" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A141" s="14" t="s">
         <v>361</v>
       </c>
@@ -8175,8 +8329,9 @@
       <c r="AF141" s="14"/>
       <c r="AG141" s="14"/>
       <c r="AH141" s="14"/>
-    </row>
-    <row r="142" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI141" s="14"/>
+    </row>
+    <row r="142" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A142" s="14" t="s">
         <v>362</v>
       </c>
@@ -8196,8 +8351,9 @@
       <c r="AF142" s="14"/>
       <c r="AG142" s="14"/>
       <c r="AH142" s="14"/>
-    </row>
-    <row r="143" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI142" s="14"/>
+    </row>
+    <row r="143" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A143" s="14" t="s">
         <v>363</v>
       </c>
@@ -8217,8 +8373,9 @@
       <c r="AF143" s="14"/>
       <c r="AG143" s="14"/>
       <c r="AH143" s="14"/>
-    </row>
-    <row r="144" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI143" s="14"/>
+    </row>
+    <row r="144" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A144" s="14" t="s">
         <v>372</v>
       </c>
@@ -8238,8 +8395,9 @@
       <c r="AF144" s="14"/>
       <c r="AG144" s="14"/>
       <c r="AH144" s="14"/>
-    </row>
-    <row r="145" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI144" s="14"/>
+    </row>
+    <row r="145" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB145" s="14"/>
       <c r="AC145" s="14"/>
       <c r="AD145" s="14"/>
@@ -8247,8 +8405,9 @@
       <c r="AF145" s="14"/>
       <c r="AG145" s="14"/>
       <c r="AH145" s="14"/>
-    </row>
-    <row r="146" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI145" s="14"/>
+    </row>
+    <row r="146" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB146" s="14"/>
       <c r="AC146" s="14"/>
       <c r="AD146" s="14"/>
@@ -8256,8 +8415,9 @@
       <c r="AF146" s="14"/>
       <c r="AG146" s="14"/>
       <c r="AH146" s="14"/>
-    </row>
-    <row r="147" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI146" s="14"/>
+    </row>
+    <row r="147" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB147" s="14"/>
       <c r="AC147" s="14"/>
       <c r="AD147" s="14"/>
@@ -8265,8 +8425,9 @@
       <c r="AF147" s="14"/>
       <c r="AG147" s="14"/>
       <c r="AH147" s="14"/>
-    </row>
-    <row r="148" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI147" s="14"/>
+    </row>
+    <row r="148" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB148" s="14"/>
       <c r="AC148" s="14"/>
       <c r="AD148" s="14"/>
@@ -8274,8 +8435,9 @@
       <c r="AF148" s="14"/>
       <c r="AG148" s="14"/>
       <c r="AH148" s="14"/>
-    </row>
-    <row r="149" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI148" s="14"/>
+    </row>
+    <row r="149" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB149" s="14"/>
       <c r="AC149" s="14"/>
       <c r="AD149" s="14"/>
@@ -8283,8 +8445,9 @@
       <c r="AF149" s="14"/>
       <c r="AG149" s="14"/>
       <c r="AH149" s="14"/>
-    </row>
-    <row r="150" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI149" s="14"/>
+    </row>
+    <row r="150" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB150" s="14"/>
       <c r="AC150" s="14"/>
       <c r="AD150" s="14"/>
@@ -8292,8 +8455,9 @@
       <c r="AF150" s="14"/>
       <c r="AG150" s="14"/>
       <c r="AH150" s="14"/>
-    </row>
-    <row r="151" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI150" s="14"/>
+    </row>
+    <row r="151" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB151" s="14"/>
       <c r="AC151" s="14"/>
       <c r="AD151" s="14"/>
@@ -8301,8 +8465,9 @@
       <c r="AF151" s="14"/>
       <c r="AG151" s="14"/>
       <c r="AH151" s="14"/>
-    </row>
-    <row r="152" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI151" s="14"/>
+    </row>
+    <row r="152" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB152" s="14"/>
       <c r="AC152" s="14"/>
       <c r="AD152" s="14"/>
@@ -8310,8 +8475,9 @@
       <c r="AF152" s="14"/>
       <c r="AG152" s="14"/>
       <c r="AH152" s="14"/>
-    </row>
-    <row r="153" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI152" s="14"/>
+    </row>
+    <row r="153" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB153" s="14"/>
       <c r="AC153" s="14"/>
       <c r="AD153" s="14"/>
@@ -8319,8 +8485,9 @@
       <c r="AF153" s="14"/>
       <c r="AG153" s="14"/>
       <c r="AH153" s="14"/>
-    </row>
-    <row r="154" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI153" s="14"/>
+    </row>
+    <row r="154" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB154" s="14"/>
       <c r="AC154" s="14"/>
       <c r="AD154" s="14"/>
@@ -8328,8 +8495,9 @@
       <c r="AF154" s="14"/>
       <c r="AG154" s="14"/>
       <c r="AH154" s="14"/>
-    </row>
-    <row r="155" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI154" s="14"/>
+    </row>
+    <row r="155" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB155" s="14"/>
       <c r="AC155" s="14"/>
       <c r="AD155" s="14"/>
@@ -8337,8 +8505,9 @@
       <c r="AF155" s="14"/>
       <c r="AG155" s="14"/>
       <c r="AH155" s="14"/>
-    </row>
-    <row r="156" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI155" s="14"/>
+    </row>
+    <row r="156" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB156" s="14"/>
       <c r="AC156" s="14"/>
       <c r="AD156" s="14"/>
@@ -8346,8 +8515,9 @@
       <c r="AF156" s="14"/>
       <c r="AG156" s="14"/>
       <c r="AH156" s="14"/>
-    </row>
-    <row r="157" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI156" s="14"/>
+    </row>
+    <row r="157" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB157" s="14"/>
       <c r="AC157" s="14"/>
       <c r="AD157" s="14"/>
@@ -8355,8 +8525,9 @@
       <c r="AF157" s="14"/>
       <c r="AG157" s="14"/>
       <c r="AH157" s="14"/>
-    </row>
-    <row r="158" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI157" s="14"/>
+    </row>
+    <row r="158" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB158" s="14"/>
       <c r="AC158" s="14"/>
       <c r="AD158" s="14"/>
@@ -8364,8 +8535,9 @@
       <c r="AF158" s="14"/>
       <c r="AG158" s="14"/>
       <c r="AH158" s="14"/>
-    </row>
-    <row r="159" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI158" s="14"/>
+    </row>
+    <row r="159" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB159" s="14"/>
       <c r="AC159" s="14"/>
       <c r="AD159" s="14"/>
@@ -8373,8 +8545,9 @@
       <c r="AF159" s="14"/>
       <c r="AG159" s="14"/>
       <c r="AH159" s="14"/>
-    </row>
-    <row r="160" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI159" s="14"/>
+    </row>
+    <row r="160" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB160" s="14"/>
       <c r="AC160" s="14"/>
       <c r="AD160" s="14"/>
@@ -8382,8 +8555,9 @@
       <c r="AF160" s="14"/>
       <c r="AG160" s="14"/>
       <c r="AH160" s="14"/>
-    </row>
-    <row r="161" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI160" s="14"/>
+    </row>
+    <row r="161" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB161" s="14"/>
       <c r="AC161" s="14"/>
       <c r="AD161" s="14"/>
@@ -8391,8 +8565,9 @@
       <c r="AF161" s="14"/>
       <c r="AG161" s="14"/>
       <c r="AH161" s="14"/>
-    </row>
-    <row r="162" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI161" s="14"/>
+    </row>
+    <row r="162" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB162" s="14"/>
       <c r="AC162" s="14"/>
       <c r="AD162" s="14"/>
@@ -8400,8 +8575,9 @@
       <c r="AF162" s="14"/>
       <c r="AG162" s="14"/>
       <c r="AH162" s="14"/>
-    </row>
-    <row r="163" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI162" s="14"/>
+    </row>
+    <row r="163" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB163" s="14"/>
       <c r="AC163" s="14"/>
       <c r="AD163" s="14"/>
@@ -8409,8 +8585,9 @@
       <c r="AF163" s="14"/>
       <c r="AG163" s="14"/>
       <c r="AH163" s="14"/>
-    </row>
-    <row r="164" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI163" s="14"/>
+    </row>
+    <row r="164" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB164" s="14"/>
       <c r="AC164" s="14"/>
       <c r="AD164" s="14"/>
@@ -8418,8 +8595,9 @@
       <c r="AF164" s="14"/>
       <c r="AG164" s="14"/>
       <c r="AH164" s="14"/>
-    </row>
-    <row r="165" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI164" s="14"/>
+    </row>
+    <row r="165" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB165" s="14"/>
       <c r="AC165" s="14"/>
       <c r="AD165" s="14"/>
@@ -8427,8 +8605,9 @@
       <c r="AF165" s="14"/>
       <c r="AG165" s="14"/>
       <c r="AH165" s="14"/>
-    </row>
-    <row r="166" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI165" s="14"/>
+    </row>
+    <row r="166" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB166" s="14"/>
       <c r="AC166" s="14"/>
       <c r="AD166" s="14"/>
@@ -8436,8 +8615,9 @@
       <c r="AF166" s="14"/>
       <c r="AG166" s="14"/>
       <c r="AH166" s="14"/>
-    </row>
-    <row r="167" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI166" s="14"/>
+    </row>
+    <row r="167" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB167" s="14"/>
       <c r="AC167" s="14"/>
       <c r="AD167" s="14"/>
@@ -8445,8 +8625,9 @@
       <c r="AF167" s="14"/>
       <c r="AG167" s="14"/>
       <c r="AH167" s="14"/>
-    </row>
-    <row r="168" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI167" s="14"/>
+    </row>
+    <row r="168" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB168" s="14"/>
       <c r="AC168" s="14"/>
       <c r="AD168" s="14"/>
@@ -8454,8 +8635,9 @@
       <c r="AF168" s="14"/>
       <c r="AG168" s="14"/>
       <c r="AH168" s="14"/>
-    </row>
-    <row r="169" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI168" s="14"/>
+    </row>
+    <row r="169" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB169" s="14"/>
       <c r="AC169" s="14"/>
       <c r="AD169" s="14"/>
@@ -8463,8 +8645,9 @@
       <c r="AF169" s="14"/>
       <c r="AG169" s="14"/>
       <c r="AH169" s="14"/>
-    </row>
-    <row r="170" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI169" s="14"/>
+    </row>
+    <row r="170" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB170" s="14"/>
       <c r="AC170" s="14"/>
       <c r="AD170" s="14"/>
@@ -8472,8 +8655,9 @@
       <c r="AF170" s="14"/>
       <c r="AG170" s="14"/>
       <c r="AH170" s="14"/>
-    </row>
-    <row r="171" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI170" s="14"/>
+    </row>
+    <row r="171" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB171" s="14"/>
       <c r="AC171" s="14"/>
       <c r="AD171" s="14"/>
@@ -8481,8 +8665,9 @@
       <c r="AF171" s="14"/>
       <c r="AG171" s="14"/>
       <c r="AH171" s="14"/>
-    </row>
-    <row r="172" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI171" s="14"/>
+    </row>
+    <row r="172" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB172" s="14"/>
       <c r="AC172" s="14"/>
       <c r="AD172" s="14"/>
@@ -8490,8 +8675,9 @@
       <c r="AF172" s="14"/>
       <c r="AG172" s="14"/>
       <c r="AH172" s="14"/>
-    </row>
-    <row r="173" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI172" s="14"/>
+    </row>
+    <row r="173" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB173" s="14"/>
       <c r="AC173" s="14"/>
       <c r="AD173" s="14"/>
@@ -8499,8 +8685,9 @@
       <c r="AF173" s="14"/>
       <c r="AG173" s="14"/>
       <c r="AH173" s="14"/>
-    </row>
-    <row r="174" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI173" s="14"/>
+    </row>
+    <row r="174" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB174" s="14"/>
       <c r="AC174" s="14"/>
       <c r="AD174" s="14"/>
@@ -8508,8 +8695,9 @@
       <c r="AF174" s="14"/>
       <c r="AG174" s="14"/>
       <c r="AH174" s="14"/>
-    </row>
-    <row r="175" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI174" s="14"/>
+    </row>
+    <row r="175" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB175" s="14"/>
       <c r="AC175" s="14"/>
       <c r="AD175" s="14"/>
@@ -8517,8 +8705,9 @@
       <c r="AF175" s="14"/>
       <c r="AG175" s="14"/>
       <c r="AH175" s="14"/>
-    </row>
-    <row r="176" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI175" s="14"/>
+    </row>
+    <row r="176" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB176" s="14"/>
       <c r="AC176" s="14"/>
       <c r="AD176" s="14"/>
@@ -8526,8 +8715,9 @@
       <c r="AF176" s="14"/>
       <c r="AG176" s="14"/>
       <c r="AH176" s="14"/>
-    </row>
-    <row r="177" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI176" s="14"/>
+    </row>
+    <row r="177" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB177" s="14"/>
       <c r="AC177" s="14"/>
       <c r="AD177" s="14"/>
@@ -8535,8 +8725,9 @@
       <c r="AF177" s="14"/>
       <c r="AG177" s="14"/>
       <c r="AH177" s="14"/>
-    </row>
-    <row r="178" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI177" s="14"/>
+    </row>
+    <row r="178" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB178" s="14"/>
       <c r="AC178" s="14"/>
       <c r="AD178" s="14"/>
@@ -8544,8 +8735,9 @@
       <c r="AF178" s="14"/>
       <c r="AG178" s="14"/>
       <c r="AH178" s="14"/>
-    </row>
-    <row r="179" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI178" s="14"/>
+    </row>
+    <row r="179" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB179" s="14"/>
       <c r="AC179" s="14"/>
       <c r="AD179" s="14"/>
@@ -8553,8 +8745,9 @@
       <c r="AF179" s="14"/>
       <c r="AG179" s="14"/>
       <c r="AH179" s="14"/>
-    </row>
-    <row r="180" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI179" s="14"/>
+    </row>
+    <row r="180" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB180" s="14"/>
       <c r="AC180" s="14"/>
       <c r="AD180" s="14"/>
@@ -8562,8 +8755,9 @@
       <c r="AF180" s="14"/>
       <c r="AG180" s="14"/>
       <c r="AH180" s="14"/>
-    </row>
-    <row r="181" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI180" s="14"/>
+    </row>
+    <row r="181" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB181" s="14"/>
       <c r="AC181" s="14"/>
       <c r="AD181" s="14"/>
@@ -8571,8 +8765,9 @@
       <c r="AF181" s="14"/>
       <c r="AG181" s="14"/>
       <c r="AH181" s="14"/>
-    </row>
-    <row r="182" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI181" s="14"/>
+    </row>
+    <row r="182" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB182" s="14"/>
       <c r="AC182" s="14"/>
       <c r="AD182" s="14"/>
@@ -8580,8 +8775,9 @@
       <c r="AF182" s="14"/>
       <c r="AG182" s="14"/>
       <c r="AH182" s="14"/>
-    </row>
-    <row r="183" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI182" s="14"/>
+    </row>
+    <row r="183" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB183" s="14"/>
       <c r="AC183" s="14"/>
       <c r="AD183" s="14"/>
@@ -8589,8 +8785,9 @@
       <c r="AF183" s="14"/>
       <c r="AG183" s="14"/>
       <c r="AH183" s="14"/>
-    </row>
-    <row r="184" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI183" s="14"/>
+    </row>
+    <row r="184" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB184" s="14"/>
       <c r="AC184" s="14"/>
       <c r="AD184" s="14"/>
@@ -8598,8 +8795,9 @@
       <c r="AF184" s="14"/>
       <c r="AG184" s="14"/>
       <c r="AH184" s="14"/>
-    </row>
-    <row r="185" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI184" s="14"/>
+    </row>
+    <row r="185" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB185" s="14"/>
       <c r="AC185" s="14"/>
       <c r="AD185" s="14"/>
@@ -8607,8 +8805,9 @@
       <c r="AF185" s="14"/>
       <c r="AG185" s="14"/>
       <c r="AH185" s="14"/>
-    </row>
-    <row r="186" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI185" s="14"/>
+    </row>
+    <row r="186" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB186" s="14"/>
       <c r="AC186" s="14"/>
       <c r="AD186" s="14"/>
@@ -8616,8 +8815,9 @@
       <c r="AF186" s="14"/>
       <c r="AG186" s="14"/>
       <c r="AH186" s="14"/>
-    </row>
-    <row r="187" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI186" s="14"/>
+    </row>
+    <row r="187" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB187" s="14"/>
       <c r="AC187" s="14"/>
       <c r="AD187" s="14"/>
@@ -8625,8 +8825,9 @@
       <c r="AF187" s="14"/>
       <c r="AG187" s="14"/>
       <c r="AH187" s="14"/>
-    </row>
-    <row r="188" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI187" s="14"/>
+    </row>
+    <row r="188" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB188" s="14"/>
       <c r="AC188" s="14"/>
       <c r="AD188" s="14"/>
@@ -8634,8 +8835,9 @@
       <c r="AF188" s="14"/>
       <c r="AG188" s="14"/>
       <c r="AH188" s="14"/>
-    </row>
-    <row r="189" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI188" s="14"/>
+    </row>
+    <row r="189" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB189" s="14"/>
       <c r="AC189" s="14"/>
       <c r="AD189" s="14"/>
@@ -8643,8 +8845,9 @@
       <c r="AF189" s="14"/>
       <c r="AG189" s="14"/>
       <c r="AH189" s="14"/>
-    </row>
-    <row r="190" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI189" s="14"/>
+    </row>
+    <row r="190" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB190" s="14"/>
       <c r="AC190" s="14"/>
       <c r="AD190" s="14"/>
@@ -8652,8 +8855,9 @@
       <c r="AF190" s="14"/>
       <c r="AG190" s="14"/>
       <c r="AH190" s="14"/>
-    </row>
-    <row r="191" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI190" s="14"/>
+    </row>
+    <row r="191" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB191" s="14"/>
       <c r="AC191" s="14"/>
       <c r="AD191" s="14"/>
@@ -8661,8 +8865,9 @@
       <c r="AF191" s="14"/>
       <c r="AG191" s="14"/>
       <c r="AH191" s="14"/>
-    </row>
-    <row r="192" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI191" s="14"/>
+    </row>
+    <row r="192" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB192" s="14"/>
       <c r="AC192" s="14"/>
       <c r="AD192" s="14"/>
@@ -8670,8 +8875,9 @@
       <c r="AF192" s="14"/>
       <c r="AG192" s="14"/>
       <c r="AH192" s="14"/>
-    </row>
-    <row r="193" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI192" s="14"/>
+    </row>
+    <row r="193" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB193" s="14"/>
       <c r="AC193" s="14"/>
       <c r="AD193" s="14"/>
@@ -8679,8 +8885,9 @@
       <c r="AF193" s="14"/>
       <c r="AG193" s="14"/>
       <c r="AH193" s="14"/>
-    </row>
-    <row r="194" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI193" s="14"/>
+    </row>
+    <row r="194" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB194" s="14"/>
       <c r="AC194" s="14"/>
       <c r="AD194" s="14"/>
@@ -8688,8 +8895,9 @@
       <c r="AF194" s="14"/>
       <c r="AG194" s="14"/>
       <c r="AH194" s="14"/>
-    </row>
-    <row r="195" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI194" s="14"/>
+    </row>
+    <row r="195" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB195" s="14"/>
       <c r="AC195" s="14"/>
       <c r="AD195" s="14"/>
@@ -8697,8 +8905,9 @@
       <c r="AF195" s="14"/>
       <c r="AG195" s="14"/>
       <c r="AH195" s="14"/>
-    </row>
-    <row r="196" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI195" s="14"/>
+    </row>
+    <row r="196" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB196" s="14"/>
       <c r="AC196" s="14"/>
       <c r="AD196" s="14"/>
@@ -8706,8 +8915,9 @@
       <c r="AF196" s="14"/>
       <c r="AG196" s="14"/>
       <c r="AH196" s="14"/>
-    </row>
-    <row r="197" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI196" s="14"/>
+    </row>
+    <row r="197" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB197" s="14"/>
       <c r="AC197" s="14"/>
       <c r="AD197" s="14"/>
@@ -8715,8 +8925,9 @@
       <c r="AF197" s="14"/>
       <c r="AG197" s="14"/>
       <c r="AH197" s="14"/>
-    </row>
-    <row r="198" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI197" s="14"/>
+    </row>
+    <row r="198" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB198" s="14"/>
       <c r="AC198" s="14"/>
       <c r="AD198" s="14"/>
@@ -8724,8 +8935,9 @@
       <c r="AF198" s="14"/>
       <c r="AG198" s="14"/>
       <c r="AH198" s="14"/>
-    </row>
-    <row r="199" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI198" s="14"/>
+    </row>
+    <row r="199" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB199" s="14"/>
       <c r="AC199" s="14"/>
       <c r="AD199" s="14"/>
@@ -8733,8 +8945,9 @@
       <c r="AF199" s="14"/>
       <c r="AG199" s="14"/>
       <c r="AH199" s="14"/>
-    </row>
-    <row r="200" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI199" s="14"/>
+    </row>
+    <row r="200" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB200" s="14"/>
       <c r="AC200" s="14"/>
       <c r="AD200" s="14"/>
@@ -8742,8 +8955,9 @@
       <c r="AF200" s="14"/>
       <c r="AG200" s="14"/>
       <c r="AH200" s="14"/>
-    </row>
-    <row r="201" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI200" s="14"/>
+    </row>
+    <row r="201" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB201" s="14"/>
       <c r="AC201" s="14"/>
       <c r="AD201" s="14"/>
@@ -8751,8 +8965,9 @@
       <c r="AF201" s="14"/>
       <c r="AG201" s="14"/>
       <c r="AH201" s="14"/>
-    </row>
-    <row r="202" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI201" s="14"/>
+    </row>
+    <row r="202" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB202" s="14"/>
       <c r="AC202" s="14"/>
       <c r="AD202" s="14"/>
@@ -8760,8 +8975,9 @@
       <c r="AF202" s="14"/>
       <c r="AG202" s="14"/>
       <c r="AH202" s="14"/>
-    </row>
-    <row r="203" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI202" s="14"/>
+    </row>
+    <row r="203" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB203" s="14"/>
       <c r="AC203" s="14"/>
       <c r="AD203" s="14"/>
@@ -8769,8 +8985,9 @@
       <c r="AF203" s="14"/>
       <c r="AG203" s="14"/>
       <c r="AH203" s="14"/>
-    </row>
-    <row r="204" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI203" s="14"/>
+    </row>
+    <row r="204" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB204" s="14"/>
       <c r="AC204" s="14"/>
       <c r="AD204" s="14"/>
@@ -8778,8 +8995,9 @@
       <c r="AF204" s="14"/>
       <c r="AG204" s="14"/>
       <c r="AH204" s="14"/>
-    </row>
-    <row r="205" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI204" s="14"/>
+    </row>
+    <row r="205" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB205" s="14"/>
       <c r="AC205" s="14"/>
       <c r="AD205" s="14"/>
@@ -8787,8 +9005,9 @@
       <c r="AF205" s="14"/>
       <c r="AG205" s="14"/>
       <c r="AH205" s="14"/>
-    </row>
-    <row r="206" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI205" s="14"/>
+    </row>
+    <row r="206" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB206" s="14"/>
       <c r="AC206" s="14"/>
       <c r="AD206" s="14"/>
@@ -8796,8 +9015,9 @@
       <c r="AF206" s="14"/>
       <c r="AG206" s="14"/>
       <c r="AH206" s="14"/>
-    </row>
-    <row r="207" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI206" s="14"/>
+    </row>
+    <row r="207" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB207" s="14"/>
       <c r="AC207" s="14"/>
       <c r="AD207" s="14"/>
@@ -8805,8 +9025,9 @@
       <c r="AF207" s="14"/>
       <c r="AG207" s="14"/>
       <c r="AH207" s="14"/>
-    </row>
-    <row r="208" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI207" s="14"/>
+    </row>
+    <row r="208" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB208" s="14"/>
       <c r="AC208" s="14"/>
       <c r="AD208" s="14"/>
@@ -8814,8 +9035,9 @@
       <c r="AF208" s="14"/>
       <c r="AG208" s="14"/>
       <c r="AH208" s="14"/>
-    </row>
-    <row r="209" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI208" s="14"/>
+    </row>
+    <row r="209" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB209" s="14"/>
       <c r="AC209" s="14"/>
       <c r="AD209" s="14"/>
@@ -8823,8 +9045,9 @@
       <c r="AF209" s="14"/>
       <c r="AG209" s="14"/>
       <c r="AH209" s="14"/>
-    </row>
-    <row r="210" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI209" s="14"/>
+    </row>
+    <row r="210" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB210" s="14"/>
       <c r="AC210" s="14"/>
       <c r="AD210" s="14"/>
@@ -8832,8 +9055,9 @@
       <c r="AF210" s="14"/>
       <c r="AG210" s="14"/>
       <c r="AH210" s="14"/>
-    </row>
-    <row r="211" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI210" s="14"/>
+    </row>
+    <row r="211" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB211" s="14"/>
       <c r="AC211" s="14"/>
       <c r="AD211" s="14"/>
@@ -8841,8 +9065,9 @@
       <c r="AF211" s="14"/>
       <c r="AG211" s="14"/>
       <c r="AH211" s="14"/>
-    </row>
-    <row r="212" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI211" s="14"/>
+    </row>
+    <row r="212" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB212" s="14"/>
       <c r="AC212" s="14"/>
       <c r="AD212" s="14"/>
@@ -8850,8 +9075,9 @@
       <c r="AF212" s="14"/>
       <c r="AG212" s="14"/>
       <c r="AH212" s="14"/>
-    </row>
-    <row r="213" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI212" s="14"/>
+    </row>
+    <row r="213" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB213" s="14"/>
       <c r="AC213" s="14"/>
       <c r="AD213" s="14"/>
@@ -8859,8 +9085,9 @@
       <c r="AF213" s="14"/>
       <c r="AG213" s="14"/>
       <c r="AH213" s="14"/>
-    </row>
-    <row r="214" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI213" s="14"/>
+    </row>
+    <row r="214" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB214" s="14"/>
       <c r="AC214" s="14"/>
       <c r="AD214" s="14"/>
@@ -8868,8 +9095,9 @@
       <c r="AF214" s="14"/>
       <c r="AG214" s="14"/>
       <c r="AH214" s="14"/>
-    </row>
-    <row r="215" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI214" s="14"/>
+    </row>
+    <row r="215" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB215" s="14"/>
       <c r="AC215" s="14"/>
       <c r="AD215" s="14"/>
@@ -8877,8 +9105,9 @@
       <c r="AF215" s="14"/>
       <c r="AG215" s="14"/>
       <c r="AH215" s="14"/>
-    </row>
-    <row r="216" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI215" s="14"/>
+    </row>
+    <row r="216" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB216" s="14"/>
       <c r="AC216" s="14"/>
       <c r="AD216" s="14"/>
@@ -8886,8 +9115,9 @@
       <c r="AF216" s="14"/>
       <c r="AG216" s="14"/>
       <c r="AH216" s="14"/>
-    </row>
-    <row r="217" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI216" s="14"/>
+    </row>
+    <row r="217" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB217" s="14"/>
       <c r="AC217" s="14"/>
       <c r="AD217" s="14"/>
@@ -8895,8 +9125,9 @@
       <c r="AF217" s="14"/>
       <c r="AG217" s="14"/>
       <c r="AH217" s="14"/>
-    </row>
-    <row r="218" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI217" s="14"/>
+    </row>
+    <row r="218" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB218" s="14"/>
       <c r="AC218" s="14"/>
       <c r="AD218" s="14"/>
@@ -8904,8 +9135,9 @@
       <c r="AF218" s="14"/>
       <c r="AG218" s="14"/>
       <c r="AH218" s="14"/>
-    </row>
-    <row r="219" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI218" s="14"/>
+    </row>
+    <row r="219" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB219" s="14"/>
       <c r="AC219" s="14"/>
       <c r="AD219" s="14"/>
@@ -8913,8 +9145,9 @@
       <c r="AF219" s="14"/>
       <c r="AG219" s="14"/>
       <c r="AH219" s="14"/>
-    </row>
-    <row r="220" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI219" s="14"/>
+    </row>
+    <row r="220" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB220" s="14"/>
       <c r="AC220" s="14"/>
       <c r="AD220" s="14"/>
@@ -8922,8 +9155,9 @@
       <c r="AF220" s="14"/>
       <c r="AG220" s="14"/>
       <c r="AH220" s="14"/>
-    </row>
-    <row r="221" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI220" s="14"/>
+    </row>
+    <row r="221" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB221" s="14"/>
       <c r="AC221" s="14"/>
       <c r="AD221" s="14"/>
@@ -8931,8 +9165,9 @@
       <c r="AF221" s="14"/>
       <c r="AG221" s="14"/>
       <c r="AH221" s="14"/>
-    </row>
-    <row r="222" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI221" s="14"/>
+    </row>
+    <row r="222" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB222" s="14"/>
       <c r="AC222" s="14"/>
       <c r="AD222" s="14"/>
@@ -8940,8 +9175,9 @@
       <c r="AF222" s="14"/>
       <c r="AG222" s="14"/>
       <c r="AH222" s="14"/>
-    </row>
-    <row r="223" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI222" s="14"/>
+    </row>
+    <row r="223" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB223" s="14"/>
       <c r="AC223" s="14"/>
       <c r="AD223" s="14"/>
@@ -8949,8 +9185,9 @@
       <c r="AF223" s="14"/>
       <c r="AG223" s="14"/>
       <c r="AH223" s="14"/>
-    </row>
-    <row r="224" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI223" s="14"/>
+    </row>
+    <row r="224" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB224" s="14"/>
       <c r="AC224" s="14"/>
       <c r="AD224" s="14"/>
@@ -8958,8 +9195,9 @@
       <c r="AF224" s="14"/>
       <c r="AG224" s="14"/>
       <c r="AH224" s="14"/>
-    </row>
-    <row r="225" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI224" s="14"/>
+    </row>
+    <row r="225" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB225" s="14"/>
       <c r="AC225" s="14"/>
       <c r="AD225" s="14"/>
@@ -8967,8 +9205,9 @@
       <c r="AF225" s="14"/>
       <c r="AG225" s="14"/>
       <c r="AH225" s="14"/>
-    </row>
-    <row r="226" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI225" s="14"/>
+    </row>
+    <row r="226" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB226" s="14"/>
       <c r="AC226" s="14"/>
       <c r="AD226" s="14"/>
@@ -8976,8 +9215,9 @@
       <c r="AF226" s="14"/>
       <c r="AG226" s="14"/>
       <c r="AH226" s="14"/>
-    </row>
-    <row r="227" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI226" s="14"/>
+    </row>
+    <row r="227" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB227" s="14"/>
       <c r="AC227" s="14"/>
       <c r="AD227" s="14"/>
@@ -8985,8 +9225,9 @@
       <c r="AF227" s="14"/>
       <c r="AG227" s="14"/>
       <c r="AH227" s="14"/>
-    </row>
-    <row r="228" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI227" s="14"/>
+    </row>
+    <row r="228" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB228" s="14"/>
       <c r="AC228" s="14"/>
       <c r="AD228" s="14"/>
@@ -8994,8 +9235,9 @@
       <c r="AF228" s="14"/>
       <c r="AG228" s="14"/>
       <c r="AH228" s="14"/>
-    </row>
-    <row r="229" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI228" s="14"/>
+    </row>
+    <row r="229" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB229" s="14"/>
       <c r="AC229" s="14"/>
       <c r="AD229" s="14"/>
@@ -9003,8 +9245,9 @@
       <c r="AF229" s="14"/>
       <c r="AG229" s="14"/>
       <c r="AH229" s="14"/>
-    </row>
-    <row r="230" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI229" s="14"/>
+    </row>
+    <row r="230" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB230" s="14"/>
       <c r="AC230" s="14"/>
       <c r="AD230" s="14"/>
@@ -9012,8 +9255,9 @@
       <c r="AF230" s="14"/>
       <c r="AG230" s="14"/>
       <c r="AH230" s="14"/>
-    </row>
-    <row r="231" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI230" s="14"/>
+    </row>
+    <row r="231" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB231" s="14"/>
       <c r="AC231" s="14"/>
       <c r="AD231" s="14"/>
@@ -9021,8 +9265,9 @@
       <c r="AF231" s="14"/>
       <c r="AG231" s="14"/>
       <c r="AH231" s="14"/>
-    </row>
-    <row r="232" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI231" s="14"/>
+    </row>
+    <row r="232" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB232" s="14"/>
       <c r="AC232" s="14"/>
       <c r="AD232" s="14"/>
@@ -9030,8 +9275,9 @@
       <c r="AF232" s="14"/>
       <c r="AG232" s="14"/>
       <c r="AH232" s="14"/>
-    </row>
-    <row r="233" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI232" s="14"/>
+    </row>
+    <row r="233" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB233" s="14"/>
       <c r="AC233" s="14"/>
       <c r="AD233" s="14"/>
@@ -9039,8 +9285,9 @@
       <c r="AF233" s="14"/>
       <c r="AG233" s="14"/>
       <c r="AH233" s="14"/>
-    </row>
-    <row r="234" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI233" s="14"/>
+    </row>
+    <row r="234" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB234" s="14"/>
       <c r="AC234" s="14"/>
       <c r="AD234" s="14"/>
@@ -9048,8 +9295,9 @@
       <c r="AF234" s="14"/>
       <c r="AG234" s="14"/>
       <c r="AH234" s="14"/>
-    </row>
-    <row r="235" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI234" s="14"/>
+    </row>
+    <row r="235" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB235" s="14"/>
       <c r="AC235" s="14"/>
       <c r="AD235" s="14"/>
@@ -9057,8 +9305,9 @@
       <c r="AF235" s="14"/>
       <c r="AG235" s="14"/>
       <c r="AH235" s="14"/>
-    </row>
-    <row r="236" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI235" s="14"/>
+    </row>
+    <row r="236" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB236" s="14"/>
       <c r="AC236" s="14"/>
       <c r="AD236" s="14"/>
@@ -9066,8 +9315,9 @@
       <c r="AF236" s="14"/>
       <c r="AG236" s="14"/>
       <c r="AH236" s="14"/>
-    </row>
-    <row r="237" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI236" s="14"/>
+    </row>
+    <row r="237" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB237" s="14"/>
       <c r="AC237" s="14"/>
       <c r="AD237" s="14"/>
@@ -9075,8 +9325,9 @@
       <c r="AF237" s="14"/>
       <c r="AG237" s="14"/>
       <c r="AH237" s="14"/>
-    </row>
-    <row r="238" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI237" s="14"/>
+    </row>
+    <row r="238" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB238" s="14"/>
       <c r="AC238" s="14"/>
       <c r="AD238" s="14"/>
@@ -9084,8 +9335,9 @@
       <c r="AF238" s="14"/>
       <c r="AG238" s="14"/>
       <c r="AH238" s="14"/>
-    </row>
-    <row r="239" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI238" s="14"/>
+    </row>
+    <row r="239" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB239" s="14"/>
       <c r="AC239" s="14"/>
       <c r="AD239" s="14"/>
@@ -9093,8 +9345,9 @@
       <c r="AF239" s="14"/>
       <c r="AG239" s="14"/>
       <c r="AH239" s="14"/>
-    </row>
-    <row r="240" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI239" s="14"/>
+    </row>
+    <row r="240" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB240" s="14"/>
       <c r="AC240" s="14"/>
       <c r="AD240" s="14"/>
@@ -9102,8 +9355,9 @@
       <c r="AF240" s="14"/>
       <c r="AG240" s="14"/>
       <c r="AH240" s="14"/>
-    </row>
-    <row r="241" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI240" s="14"/>
+    </row>
+    <row r="241" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB241" s="14"/>
       <c r="AC241" s="14"/>
       <c r="AD241" s="14"/>
@@ -9111,8 +9365,9 @@
       <c r="AF241" s="14"/>
       <c r="AG241" s="14"/>
       <c r="AH241" s="14"/>
-    </row>
-    <row r="242" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI241" s="14"/>
+    </row>
+    <row r="242" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB242" s="14"/>
       <c r="AC242" s="14"/>
       <c r="AD242" s="14"/>
@@ -9120,8 +9375,9 @@
       <c r="AF242" s="14"/>
       <c r="AG242" s="14"/>
       <c r="AH242" s="14"/>
-    </row>
-    <row r="243" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI242" s="14"/>
+    </row>
+    <row r="243" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB243" s="14"/>
       <c r="AC243" s="14"/>
       <c r="AD243" s="14"/>
@@ -9129,8 +9385,9 @@
       <c r="AF243" s="14"/>
       <c r="AG243" s="14"/>
       <c r="AH243" s="14"/>
-    </row>
-    <row r="244" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI243" s="14"/>
+    </row>
+    <row r="244" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB244" s="14"/>
       <c r="AC244" s="14"/>
       <c r="AD244" s="14"/>
@@ -9138,8 +9395,9 @@
       <c r="AF244" s="14"/>
       <c r="AG244" s="14"/>
       <c r="AH244" s="14"/>
-    </row>
-    <row r="245" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI244" s="14"/>
+    </row>
+    <row r="245" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB245" s="14"/>
       <c r="AC245" s="14"/>
       <c r="AD245" s="14"/>
@@ -9147,8 +9405,9 @@
       <c r="AF245" s="14"/>
       <c r="AG245" s="14"/>
       <c r="AH245" s="14"/>
-    </row>
-    <row r="246" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI245" s="14"/>
+    </row>
+    <row r="246" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB246" s="14"/>
       <c r="AC246" s="14"/>
       <c r="AD246" s="14"/>
@@ -9156,8 +9415,9 @@
       <c r="AF246" s="14"/>
       <c r="AG246" s="14"/>
       <c r="AH246" s="14"/>
-    </row>
-    <row r="247" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI246" s="14"/>
+    </row>
+    <row r="247" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB247" s="14"/>
       <c r="AC247" s="14"/>
       <c r="AD247" s="14"/>
@@ -9165,8 +9425,9 @@
       <c r="AF247" s="14"/>
       <c r="AG247" s="14"/>
       <c r="AH247" s="14"/>
-    </row>
-    <row r="248" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI247" s="14"/>
+    </row>
+    <row r="248" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB248" s="14"/>
       <c r="AC248" s="14"/>
       <c r="AD248" s="14"/>
@@ -9174,8 +9435,9 @@
       <c r="AF248" s="14"/>
       <c r="AG248" s="14"/>
       <c r="AH248" s="14"/>
-    </row>
-    <row r="249" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI248" s="14"/>
+    </row>
+    <row r="249" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB249" s="14"/>
       <c r="AC249" s="14"/>
       <c r="AD249" s="14"/>
@@ -9183,8 +9445,9 @@
       <c r="AF249" s="14"/>
       <c r="AG249" s="14"/>
       <c r="AH249" s="14"/>
-    </row>
-    <row r="250" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI249" s="14"/>
+    </row>
+    <row r="250" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB250" s="14"/>
       <c r="AC250" s="14"/>
       <c r="AD250" s="14"/>
@@ -9192,8 +9455,9 @@
       <c r="AF250" s="14"/>
       <c r="AG250" s="14"/>
       <c r="AH250" s="14"/>
-    </row>
-    <row r="251" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI250" s="14"/>
+    </row>
+    <row r="251" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB251" s="14"/>
       <c r="AC251" s="14"/>
       <c r="AD251" s="14"/>
@@ -9201,8 +9465,9 @@
       <c r="AF251" s="14"/>
       <c r="AG251" s="14"/>
       <c r="AH251" s="14"/>
-    </row>
-    <row r="252" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI251" s="14"/>
+    </row>
+    <row r="252" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB252" s="14"/>
       <c r="AC252" s="14"/>
       <c r="AD252" s="14"/>
@@ -9210,8 +9475,9 @@
       <c r="AF252" s="14"/>
       <c r="AG252" s="14"/>
       <c r="AH252" s="14"/>
-    </row>
-    <row r="253" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI252" s="14"/>
+    </row>
+    <row r="253" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB253" s="14"/>
       <c r="AC253" s="14"/>
       <c r="AD253" s="14"/>
@@ -9219,8 +9485,9 @@
       <c r="AF253" s="14"/>
       <c r="AG253" s="14"/>
       <c r="AH253" s="14"/>
-    </row>
-    <row r="254" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI253" s="14"/>
+    </row>
+    <row r="254" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB254" s="14"/>
       <c r="AC254" s="14"/>
       <c r="AD254" s="14"/>
@@ -9228,8 +9495,9 @@
       <c r="AF254" s="14"/>
       <c r="AG254" s="14"/>
       <c r="AH254" s="14"/>
-    </row>
-    <row r="255" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI254" s="14"/>
+    </row>
+    <row r="255" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB255" s="14"/>
       <c r="AC255" s="14"/>
       <c r="AD255" s="14"/>
@@ -9237,8 +9505,9 @@
       <c r="AF255" s="14"/>
       <c r="AG255" s="14"/>
       <c r="AH255" s="14"/>
-    </row>
-    <row r="256" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI255" s="14"/>
+    </row>
+    <row r="256" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB256" s="14"/>
       <c r="AC256" s="14"/>
       <c r="AD256" s="14"/>
@@ -9246,8 +9515,9 @@
       <c r="AF256" s="14"/>
       <c r="AG256" s="14"/>
       <c r="AH256" s="14"/>
-    </row>
-    <row r="257" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI256" s="14"/>
+    </row>
+    <row r="257" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB257" s="14"/>
       <c r="AC257" s="14"/>
       <c r="AD257" s="14"/>
@@ -9255,8 +9525,9 @@
       <c r="AF257" s="14"/>
       <c r="AG257" s="14"/>
       <c r="AH257" s="14"/>
-    </row>
-    <row r="258" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI257" s="14"/>
+    </row>
+    <row r="258" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB258" s="14"/>
       <c r="AC258" s="14"/>
       <c r="AD258" s="14"/>
@@ -9264,8 +9535,9 @@
       <c r="AF258" s="14"/>
       <c r="AG258" s="14"/>
       <c r="AH258" s="14"/>
-    </row>
-    <row r="259" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI258" s="14"/>
+    </row>
+    <row r="259" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB259" s="14"/>
       <c r="AC259" s="14"/>
       <c r="AD259" s="14"/>
@@ -9273,8 +9545,9 @@
       <c r="AF259" s="14"/>
       <c r="AG259" s="14"/>
       <c r="AH259" s="14"/>
-    </row>
-    <row r="260" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI259" s="14"/>
+    </row>
+    <row r="260" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB260" s="14"/>
       <c r="AC260" s="14"/>
       <c r="AD260" s="14"/>
@@ -9282,8 +9555,9 @@
       <c r="AF260" s="14"/>
       <c r="AG260" s="14"/>
       <c r="AH260" s="14"/>
-    </row>
-    <row r="261" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI260" s="14"/>
+    </row>
+    <row r="261" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB261" s="14"/>
       <c r="AC261" s="14"/>
       <c r="AD261" s="14"/>
@@ -9291,8 +9565,9 @@
       <c r="AF261" s="14"/>
       <c r="AG261" s="14"/>
       <c r="AH261" s="14"/>
-    </row>
-    <row r="262" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI261" s="14"/>
+    </row>
+    <row r="262" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB262" s="14"/>
       <c r="AC262" s="14"/>
       <c r="AD262" s="14"/>
@@ -9300,8 +9575,9 @@
       <c r="AF262" s="14"/>
       <c r="AG262" s="14"/>
       <c r="AH262" s="14"/>
-    </row>
-    <row r="263" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI262" s="14"/>
+    </row>
+    <row r="263" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB263" s="14"/>
       <c r="AC263" s="14"/>
       <c r="AD263" s="14"/>
@@ -9309,8 +9585,9 @@
       <c r="AF263" s="14"/>
       <c r="AG263" s="14"/>
       <c r="AH263" s="14"/>
-    </row>
-    <row r="264" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI263" s="14"/>
+    </row>
+    <row r="264" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB264" s="14"/>
       <c r="AC264" s="14"/>
       <c r="AD264" s="14"/>
@@ -9318,8 +9595,9 @@
       <c r="AF264" s="14"/>
       <c r="AG264" s="14"/>
       <c r="AH264" s="14"/>
-    </row>
-    <row r="265" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI264" s="14"/>
+    </row>
+    <row r="265" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB265" s="14"/>
       <c r="AC265" s="14"/>
       <c r="AD265" s="14"/>
@@ -9327,8 +9605,9 @@
       <c r="AF265" s="14"/>
       <c r="AG265" s="14"/>
       <c r="AH265" s="14"/>
-    </row>
-    <row r="266" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI265" s="14"/>
+    </row>
+    <row r="266" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB266" s="14"/>
       <c r="AC266" s="14"/>
       <c r="AD266" s="14"/>
@@ -9336,8 +9615,9 @@
       <c r="AF266" s="14"/>
       <c r="AG266" s="14"/>
       <c r="AH266" s="14"/>
-    </row>
-    <row r="267" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI266" s="14"/>
+    </row>
+    <row r="267" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB267" s="14"/>
       <c r="AC267" s="14"/>
       <c r="AD267" s="14"/>
@@ -9345,8 +9625,9 @@
       <c r="AF267" s="14"/>
       <c r="AG267" s="14"/>
       <c r="AH267" s="14"/>
-    </row>
-    <row r="268" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI267" s="14"/>
+    </row>
+    <row r="268" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB268" s="14"/>
       <c r="AC268" s="14"/>
       <c r="AD268" s="14"/>
@@ -9354,8 +9635,9 @@
       <c r="AF268" s="14"/>
       <c r="AG268" s="14"/>
       <c r="AH268" s="14"/>
-    </row>
-    <row r="269" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI268" s="14"/>
+    </row>
+    <row r="269" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB269" s="14"/>
       <c r="AC269" s="14"/>
       <c r="AD269" s="14"/>
@@ -9363,8 +9645,9 @@
       <c r="AF269" s="14"/>
       <c r="AG269" s="14"/>
       <c r="AH269" s="14"/>
-    </row>
-    <row r="270" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI269" s="14"/>
+    </row>
+    <row r="270" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB270" s="14"/>
       <c r="AC270" s="14"/>
       <c r="AD270" s="14"/>
@@ -9372,8 +9655,9 @@
       <c r="AF270" s="14"/>
       <c r="AG270" s="14"/>
       <c r="AH270" s="14"/>
-    </row>
-    <row r="271" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI270" s="14"/>
+    </row>
+    <row r="271" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB271" s="14"/>
       <c r="AC271" s="14"/>
       <c r="AD271" s="14"/>
@@ -9381,8 +9665,9 @@
       <c r="AF271" s="14"/>
       <c r="AG271" s="14"/>
       <c r="AH271" s="14"/>
-    </row>
-    <row r="272" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI271" s="14"/>
+    </row>
+    <row r="272" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB272" s="14"/>
       <c r="AC272" s="14"/>
       <c r="AD272" s="14"/>
@@ -9390,8 +9675,9 @@
       <c r="AF272" s="14"/>
       <c r="AG272" s="14"/>
       <c r="AH272" s="14"/>
-    </row>
-    <row r="273" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI272" s="14"/>
+    </row>
+    <row r="273" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB273" s="14"/>
       <c r="AC273" s="14"/>
       <c r="AD273" s="14"/>
@@ -9399,8 +9685,9 @@
       <c r="AF273" s="14"/>
       <c r="AG273" s="14"/>
       <c r="AH273" s="14"/>
-    </row>
-    <row r="274" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI273" s="14"/>
+    </row>
+    <row r="274" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB274" s="14"/>
       <c r="AC274" s="14"/>
       <c r="AD274" s="14"/>
@@ -9408,8 +9695,9 @@
       <c r="AF274" s="14"/>
       <c r="AG274" s="14"/>
       <c r="AH274" s="14"/>
-    </row>
-    <row r="275" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI274" s="14"/>
+    </row>
+    <row r="275" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB275" s="14"/>
       <c r="AC275" s="14"/>
       <c r="AD275" s="14"/>
@@ -9417,8 +9705,9 @@
       <c r="AF275" s="14"/>
       <c r="AG275" s="14"/>
       <c r="AH275" s="14"/>
-    </row>
-    <row r="276" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI275" s="14"/>
+    </row>
+    <row r="276" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB276" s="14"/>
       <c r="AC276" s="14"/>
       <c r="AD276" s="14"/>
@@ -9426,8 +9715,9 @@
       <c r="AF276" s="14"/>
       <c r="AG276" s="14"/>
       <c r="AH276" s="14"/>
-    </row>
-    <row r="277" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI276" s="14"/>
+    </row>
+    <row r="277" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB277" s="14"/>
       <c r="AC277" s="14"/>
       <c r="AD277" s="14"/>
@@ -9435,8 +9725,9 @@
       <c r="AF277" s="14"/>
       <c r="AG277" s="14"/>
       <c r="AH277" s="14"/>
-    </row>
-    <row r="278" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI277" s="14"/>
+    </row>
+    <row r="278" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB278" s="14"/>
       <c r="AC278" s="14"/>
       <c r="AD278" s="14"/>
@@ -9444,8 +9735,9 @@
       <c r="AF278" s="14"/>
       <c r="AG278" s="14"/>
       <c r="AH278" s="14"/>
-    </row>
-    <row r="279" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI278" s="14"/>
+    </row>
+    <row r="279" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB279" s="14"/>
       <c r="AC279" s="14"/>
       <c r="AD279" s="14"/>
@@ -9453,8 +9745,9 @@
       <c r="AF279" s="14"/>
       <c r="AG279" s="14"/>
       <c r="AH279" s="14"/>
-    </row>
-    <row r="280" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI279" s="14"/>
+    </row>
+    <row r="280" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB280" s="14"/>
       <c r="AC280" s="14"/>
       <c r="AD280" s="14"/>
@@ -9462,8 +9755,9 @@
       <c r="AF280" s="14"/>
       <c r="AG280" s="14"/>
       <c r="AH280" s="14"/>
-    </row>
-    <row r="281" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI280" s="14"/>
+    </row>
+    <row r="281" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB281" s="14"/>
       <c r="AC281" s="14"/>
       <c r="AD281" s="14"/>
@@ -9471,8 +9765,9 @@
       <c r="AF281" s="14"/>
       <c r="AG281" s="14"/>
       <c r="AH281" s="14"/>
-    </row>
-    <row r="282" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI281" s="14"/>
+    </row>
+    <row r="282" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB282" s="14"/>
       <c r="AC282" s="14"/>
       <c r="AD282" s="14"/>
@@ -9480,8 +9775,9 @@
       <c r="AF282" s="14"/>
       <c r="AG282" s="14"/>
       <c r="AH282" s="14"/>
-    </row>
-    <row r="283" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI282" s="14"/>
+    </row>
+    <row r="283" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB283" s="14"/>
       <c r="AC283" s="14"/>
       <c r="AD283" s="14"/>
@@ -9489,8 +9785,9 @@
       <c r="AF283" s="14"/>
       <c r="AG283" s="14"/>
       <c r="AH283" s="14"/>
-    </row>
-    <row r="284" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI283" s="14"/>
+    </row>
+    <row r="284" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB284" s="14"/>
       <c r="AC284" s="14"/>
       <c r="AD284" s="14"/>
@@ -9498,8 +9795,9 @@
       <c r="AF284" s="14"/>
       <c r="AG284" s="14"/>
       <c r="AH284" s="14"/>
-    </row>
-    <row r="285" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI284" s="14"/>
+    </row>
+    <row r="285" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB285" s="14"/>
       <c r="AC285" s="14"/>
       <c r="AD285" s="14"/>
@@ -9507,8 +9805,9 @@
       <c r="AF285" s="14"/>
       <c r="AG285" s="14"/>
       <c r="AH285" s="14"/>
-    </row>
-    <row r="286" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI285" s="14"/>
+    </row>
+    <row r="286" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB286" s="14"/>
       <c r="AC286" s="14"/>
       <c r="AD286" s="14"/>
@@ -9516,8 +9815,9 @@
       <c r="AF286" s="14"/>
       <c r="AG286" s="14"/>
       <c r="AH286" s="14"/>
-    </row>
-    <row r="287" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI286" s="14"/>
+    </row>
+    <row r="287" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB287" s="14"/>
       <c r="AC287" s="14"/>
       <c r="AD287" s="14"/>
@@ -9525,8 +9825,9 @@
       <c r="AF287" s="14"/>
       <c r="AG287" s="14"/>
       <c r="AH287" s="14"/>
-    </row>
-    <row r="288" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI287" s="14"/>
+    </row>
+    <row r="288" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB288" s="14"/>
       <c r="AC288" s="14"/>
       <c r="AD288" s="14"/>
@@ -9534,8 +9835,9 @@
       <c r="AF288" s="14"/>
       <c r="AG288" s="14"/>
       <c r="AH288" s="14"/>
-    </row>
-    <row r="289" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI288" s="14"/>
+    </row>
+    <row r="289" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB289" s="14"/>
       <c r="AC289" s="14"/>
       <c r="AD289" s="14"/>
@@ -9543,8 +9845,9 @@
       <c r="AF289" s="14"/>
       <c r="AG289" s="14"/>
       <c r="AH289" s="14"/>
-    </row>
-    <row r="290" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI289" s="14"/>
+    </row>
+    <row r="290" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB290" s="14"/>
       <c r="AC290" s="14"/>
       <c r="AD290" s="14"/>
@@ -9552,8 +9855,9 @@
       <c r="AF290" s="14"/>
       <c r="AG290" s="14"/>
       <c r="AH290" s="14"/>
-    </row>
-    <row r="291" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI290" s="14"/>
+    </row>
+    <row r="291" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB291" s="14"/>
       <c r="AC291" s="14"/>
       <c r="AD291" s="14"/>
@@ -9561,8 +9865,9 @@
       <c r="AF291" s="14"/>
       <c r="AG291" s="14"/>
       <c r="AH291" s="14"/>
-    </row>
-    <row r="292" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI291" s="14"/>
+    </row>
+    <row r="292" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB292" s="14"/>
       <c r="AC292" s="14"/>
       <c r="AD292" s="14"/>
@@ -9570,8 +9875,9 @@
       <c r="AF292" s="14"/>
       <c r="AG292" s="14"/>
       <c r="AH292" s="14"/>
-    </row>
-    <row r="293" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI292" s="14"/>
+    </row>
+    <row r="293" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB293" s="14"/>
       <c r="AC293" s="14"/>
       <c r="AD293" s="14"/>
@@ -9579,8 +9885,9 @@
       <c r="AF293" s="14"/>
       <c r="AG293" s="14"/>
       <c r="AH293" s="14"/>
-    </row>
-    <row r="294" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI293" s="14"/>
+    </row>
+    <row r="294" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB294" s="14"/>
       <c r="AC294" s="14"/>
       <c r="AD294" s="14"/>
@@ -9588,8 +9895,9 @@
       <c r="AF294" s="14"/>
       <c r="AG294" s="14"/>
       <c r="AH294" s="14"/>
-    </row>
-    <row r="295" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI294" s="14"/>
+    </row>
+    <row r="295" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB295" s="14"/>
       <c r="AC295" s="14"/>
       <c r="AD295" s="14"/>
@@ -9597,8 +9905,9 @@
       <c r="AF295" s="14"/>
       <c r="AG295" s="14"/>
       <c r="AH295" s="14"/>
-    </row>
-    <row r="296" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI295" s="14"/>
+    </row>
+    <row r="296" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB296" s="14"/>
       <c r="AC296" s="14"/>
       <c r="AD296" s="14"/>
@@ -9606,8 +9915,9 @@
       <c r="AF296" s="14"/>
       <c r="AG296" s="14"/>
       <c r="AH296" s="14"/>
-    </row>
-    <row r="297" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI296" s="14"/>
+    </row>
+    <row r="297" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB297" s="14"/>
       <c r="AC297" s="14"/>
       <c r="AD297" s="14"/>
@@ -9615,8 +9925,9 @@
       <c r="AF297" s="14"/>
       <c r="AG297" s="14"/>
       <c r="AH297" s="14"/>
-    </row>
-    <row r="298" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI297" s="14"/>
+    </row>
+    <row r="298" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB298" s="14"/>
       <c r="AC298" s="14"/>
       <c r="AD298" s="14"/>
@@ -9624,8 +9935,9 @@
       <c r="AF298" s="14"/>
       <c r="AG298" s="14"/>
       <c r="AH298" s="14"/>
-    </row>
-    <row r="299" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI298" s="14"/>
+    </row>
+    <row r="299" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB299" s="14"/>
       <c r="AC299" s="14"/>
       <c r="AD299" s="14"/>
@@ -9633,8 +9945,9 @@
       <c r="AF299" s="14"/>
       <c r="AG299" s="14"/>
       <c r="AH299" s="14"/>
-    </row>
-    <row r="300" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI299" s="14"/>
+    </row>
+    <row r="300" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB300" s="14"/>
       <c r="AC300" s="14"/>
       <c r="AD300" s="14"/>
@@ -9642,8 +9955,9 @@
       <c r="AF300" s="14"/>
       <c r="AG300" s="14"/>
       <c r="AH300" s="14"/>
-    </row>
-    <row r="301" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI300" s="14"/>
+    </row>
+    <row r="301" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB301" s="14"/>
       <c r="AC301" s="14"/>
       <c r="AD301" s="14"/>
@@ -9651,8 +9965,9 @@
       <c r="AF301" s="14"/>
       <c r="AG301" s="14"/>
       <c r="AH301" s="14"/>
-    </row>
-    <row r="302" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI301" s="14"/>
+    </row>
+    <row r="302" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB302" s="14"/>
       <c r="AC302" s="14"/>
       <c r="AD302" s="14"/>
@@ -9660,8 +9975,9 @@
       <c r="AF302" s="14"/>
       <c r="AG302" s="14"/>
       <c r="AH302" s="14"/>
-    </row>
-    <row r="303" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI302" s="14"/>
+    </row>
+    <row r="303" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB303" s="14"/>
       <c r="AC303" s="14"/>
       <c r="AD303" s="14"/>
@@ -9669,8 +9985,9 @@
       <c r="AF303" s="14"/>
       <c r="AG303" s="14"/>
       <c r="AH303" s="14"/>
-    </row>
-    <row r="304" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI303" s="14"/>
+    </row>
+    <row r="304" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB304" s="14"/>
       <c r="AC304" s="14"/>
       <c r="AD304" s="14"/>
@@ -9678,8 +9995,9 @@
       <c r="AF304" s="14"/>
       <c r="AG304" s="14"/>
       <c r="AH304" s="14"/>
-    </row>
-    <row r="305" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI304" s="14"/>
+    </row>
+    <row r="305" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB305" s="14"/>
       <c r="AC305" s="14"/>
       <c r="AD305" s="14"/>
@@ -9687,8 +10005,9 @@
       <c r="AF305" s="14"/>
       <c r="AG305" s="14"/>
       <c r="AH305" s="14"/>
-    </row>
-    <row r="306" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI305" s="14"/>
+    </row>
+    <row r="306" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB306" s="14"/>
       <c r="AC306" s="14"/>
       <c r="AD306" s="14"/>
@@ -9696,8 +10015,9 @@
       <c r="AF306" s="14"/>
       <c r="AG306" s="14"/>
       <c r="AH306" s="14"/>
-    </row>
-    <row r="307" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI306" s="14"/>
+    </row>
+    <row r="307" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB307" s="14"/>
       <c r="AC307" s="14"/>
       <c r="AD307" s="14"/>
@@ -9705,8 +10025,9 @@
       <c r="AF307" s="14"/>
       <c r="AG307" s="14"/>
       <c r="AH307" s="14"/>
-    </row>
-    <row r="308" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI307" s="14"/>
+    </row>
+    <row r="308" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB308" s="14"/>
       <c r="AC308" s="14"/>
       <c r="AD308" s="14"/>
@@ -9714,8 +10035,9 @@
       <c r="AF308" s="14"/>
       <c r="AG308" s="14"/>
       <c r="AH308" s="14"/>
-    </row>
-    <row r="309" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI308" s="14"/>
+    </row>
+    <row r="309" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB309" s="14"/>
       <c r="AC309" s="14"/>
       <c r="AD309" s="14"/>
@@ -9723,8 +10045,9 @@
       <c r="AF309" s="14"/>
       <c r="AG309" s="14"/>
       <c r="AH309" s="14"/>
-    </row>
-    <row r="310" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI309" s="14"/>
+    </row>
+    <row r="310" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB310" s="14"/>
       <c r="AC310" s="14"/>
       <c r="AD310" s="14"/>
@@ -9732,8 +10055,9 @@
       <c r="AF310" s="14"/>
       <c r="AG310" s="14"/>
       <c r="AH310" s="14"/>
-    </row>
-    <row r="311" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI310" s="14"/>
+    </row>
+    <row r="311" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB311" s="14"/>
       <c r="AC311" s="14"/>
       <c r="AD311" s="14"/>
@@ -9741,8 +10065,9 @@
       <c r="AF311" s="14"/>
       <c r="AG311" s="14"/>
       <c r="AH311" s="14"/>
-    </row>
-    <row r="312" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI311" s="14"/>
+    </row>
+    <row r="312" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB312" s="14"/>
       <c r="AC312" s="14"/>
       <c r="AD312" s="14"/>
@@ -9750,8 +10075,9 @@
       <c r="AF312" s="14"/>
       <c r="AG312" s="14"/>
       <c r="AH312" s="14"/>
-    </row>
-    <row r="313" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI312" s="14"/>
+    </row>
+    <row r="313" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB313" s="14"/>
       <c r="AC313" s="14"/>
       <c r="AD313" s="14"/>
@@ -9759,8 +10085,9 @@
       <c r="AF313" s="14"/>
       <c r="AG313" s="14"/>
       <c r="AH313" s="14"/>
-    </row>
-    <row r="314" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI313" s="14"/>
+    </row>
+    <row r="314" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB314" s="14"/>
       <c r="AC314" s="14"/>
       <c r="AD314" s="14"/>
@@ -9768,8 +10095,9 @@
       <c r="AF314" s="14"/>
       <c r="AG314" s="14"/>
       <c r="AH314" s="14"/>
-    </row>
-    <row r="315" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI314" s="14"/>
+    </row>
+    <row r="315" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB315" s="14"/>
       <c r="AC315" s="14"/>
       <c r="AD315" s="14"/>
@@ -9777,8 +10105,9 @@
       <c r="AF315" s="14"/>
       <c r="AG315" s="14"/>
       <c r="AH315" s="14"/>
-    </row>
-    <row r="316" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI315" s="14"/>
+    </row>
+    <row r="316" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB316" s="14"/>
       <c r="AC316" s="14"/>
       <c r="AD316" s="14"/>
@@ -9786,8 +10115,9 @@
       <c r="AF316" s="14"/>
       <c r="AG316" s="14"/>
       <c r="AH316" s="14"/>
-    </row>
-    <row r="317" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI316" s="14"/>
+    </row>
+    <row r="317" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB317" s="14"/>
       <c r="AC317" s="14"/>
       <c r="AD317" s="14"/>
@@ -9795,8 +10125,9 @@
       <c r="AF317" s="14"/>
       <c r="AG317" s="14"/>
       <c r="AH317" s="14"/>
-    </row>
-    <row r="318" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI317" s="14"/>
+    </row>
+    <row r="318" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB318" s="14"/>
       <c r="AC318" s="14"/>
       <c r="AD318" s="14"/>
@@ -9804,8 +10135,9 @@
       <c r="AF318" s="14"/>
       <c r="AG318" s="14"/>
       <c r="AH318" s="14"/>
-    </row>
-    <row r="319" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI318" s="14"/>
+    </row>
+    <row r="319" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB319" s="14"/>
       <c r="AC319" s="14"/>
       <c r="AD319" s="14"/>
@@ -9813,8 +10145,9 @@
       <c r="AF319" s="14"/>
       <c r="AG319" s="14"/>
       <c r="AH319" s="14"/>
-    </row>
-    <row r="320" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI319" s="14"/>
+    </row>
+    <row r="320" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB320" s="14"/>
       <c r="AC320" s="14"/>
       <c r="AD320" s="14"/>
@@ -9822,8 +10155,9 @@
       <c r="AF320" s="14"/>
       <c r="AG320" s="14"/>
       <c r="AH320" s="14"/>
-    </row>
-    <row r="321" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI320" s="14"/>
+    </row>
+    <row r="321" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB321" s="14"/>
       <c r="AC321" s="14"/>
       <c r="AD321" s="14"/>
@@ -9831,8 +10165,9 @@
       <c r="AF321" s="14"/>
       <c r="AG321" s="14"/>
       <c r="AH321" s="14"/>
-    </row>
-    <row r="322" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI321" s="14"/>
+    </row>
+    <row r="322" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB322" s="14"/>
       <c r="AC322" s="14"/>
       <c r="AD322" s="14"/>
@@ -9840,8 +10175,9 @@
       <c r="AF322" s="14"/>
       <c r="AG322" s="14"/>
       <c r="AH322" s="14"/>
-    </row>
-    <row r="323" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI322" s="14"/>
+    </row>
+    <row r="323" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB323" s="14"/>
       <c r="AC323" s="14"/>
       <c r="AD323" s="14"/>
@@ -9849,8 +10185,9 @@
       <c r="AF323" s="14"/>
       <c r="AG323" s="14"/>
       <c r="AH323" s="14"/>
-    </row>
-    <row r="324" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI323" s="14"/>
+    </row>
+    <row r="324" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB324" s="14"/>
       <c r="AC324" s="14"/>
       <c r="AD324" s="14"/>
@@ -9858,8 +10195,9 @@
       <c r="AF324" s="14"/>
       <c r="AG324" s="14"/>
       <c r="AH324" s="14"/>
-    </row>
-    <row r="325" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI324" s="14"/>
+    </row>
+    <row r="325" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB325" s="14"/>
       <c r="AC325" s="14"/>
       <c r="AD325" s="14"/>
@@ -9867,8 +10205,9 @@
       <c r="AF325" s="14"/>
       <c r="AG325" s="14"/>
       <c r="AH325" s="14"/>
-    </row>
-    <row r="326" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI325" s="14"/>
+    </row>
+    <row r="326" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB326" s="14"/>
       <c r="AC326" s="14"/>
       <c r="AD326" s="14"/>
@@ -9876,8 +10215,9 @@
       <c r="AF326" s="14"/>
       <c r="AG326" s="14"/>
       <c r="AH326" s="14"/>
-    </row>
-    <row r="327" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI326" s="14"/>
+    </row>
+    <row r="327" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB327" s="14"/>
       <c r="AC327" s="14"/>
       <c r="AD327" s="14"/>
@@ -9885,8 +10225,9 @@
       <c r="AF327" s="14"/>
       <c r="AG327" s="14"/>
       <c r="AH327" s="14"/>
-    </row>
-    <row r="328" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI327" s="14"/>
+    </row>
+    <row r="328" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB328" s="14"/>
       <c r="AC328" s="14"/>
       <c r="AD328" s="14"/>
@@ -9894,8 +10235,9 @@
       <c r="AF328" s="14"/>
       <c r="AG328" s="14"/>
       <c r="AH328" s="14"/>
-    </row>
-    <row r="329" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI328" s="14"/>
+    </row>
+    <row r="329" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB329" s="14"/>
       <c r="AC329" s="14"/>
       <c r="AD329" s="14"/>
@@ -9903,8 +10245,9 @@
       <c r="AF329" s="14"/>
       <c r="AG329" s="14"/>
       <c r="AH329" s="14"/>
-    </row>
-    <row r="330" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI329" s="14"/>
+    </row>
+    <row r="330" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB330" s="14"/>
       <c r="AC330" s="14"/>
       <c r="AD330" s="14"/>
@@ -9912,8 +10255,9 @@
       <c r="AF330" s="14"/>
       <c r="AG330" s="14"/>
       <c r="AH330" s="14"/>
-    </row>
-    <row r="331" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI330" s="14"/>
+    </row>
+    <row r="331" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB331" s="14"/>
       <c r="AC331" s="14"/>
       <c r="AD331" s="14"/>
@@ -9921,8 +10265,9 @@
       <c r="AF331" s="14"/>
       <c r="AG331" s="14"/>
       <c r="AH331" s="14"/>
-    </row>
-    <row r="332" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI331" s="14"/>
+    </row>
+    <row r="332" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB332" s="14"/>
       <c r="AC332" s="14"/>
       <c r="AD332" s="14"/>
@@ -9930,8 +10275,9 @@
       <c r="AF332" s="14"/>
       <c r="AG332" s="14"/>
       <c r="AH332" s="14"/>
-    </row>
-    <row r="333" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI332" s="14"/>
+    </row>
+    <row r="333" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB333" s="14"/>
       <c r="AC333" s="14"/>
       <c r="AD333" s="14"/>
@@ -9939,8 +10285,9 @@
       <c r="AF333" s="14"/>
       <c r="AG333" s="14"/>
       <c r="AH333" s="14"/>
-    </row>
-    <row r="334" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI333" s="14"/>
+    </row>
+    <row r="334" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB334" s="14"/>
       <c r="AC334" s="14"/>
       <c r="AD334" s="14"/>
@@ -9948,8 +10295,9 @@
       <c r="AF334" s="14"/>
       <c r="AG334" s="14"/>
       <c r="AH334" s="14"/>
-    </row>
-    <row r="335" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI334" s="14"/>
+    </row>
+    <row r="335" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB335" s="14"/>
       <c r="AC335" s="14"/>
       <c r="AD335" s="14"/>
@@ -9957,8 +10305,9 @@
       <c r="AF335" s="14"/>
       <c r="AG335" s="14"/>
       <c r="AH335" s="14"/>
-    </row>
-    <row r="336" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI335" s="14"/>
+    </row>
+    <row r="336" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB336" s="14"/>
       <c r="AC336" s="14"/>
       <c r="AD336" s="14"/>
@@ -9966,8 +10315,9 @@
       <c r="AF336" s="14"/>
       <c r="AG336" s="14"/>
       <c r="AH336" s="14"/>
-    </row>
-    <row r="337" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI336" s="14"/>
+    </row>
+    <row r="337" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB337" s="14"/>
       <c r="AC337" s="14"/>
       <c r="AD337" s="14"/>
@@ -9975,8 +10325,9 @@
       <c r="AF337" s="14"/>
       <c r="AG337" s="14"/>
       <c r="AH337" s="14"/>
-    </row>
-    <row r="338" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI337" s="14"/>
+    </row>
+    <row r="338" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB338" s="14"/>
       <c r="AC338" s="14"/>
       <c r="AD338" s="14"/>
@@ -9984,8 +10335,9 @@
       <c r="AF338" s="14"/>
       <c r="AG338" s="14"/>
       <c r="AH338" s="14"/>
-    </row>
-    <row r="339" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI338" s="14"/>
+    </row>
+    <row r="339" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB339" s="14"/>
       <c r="AC339" s="14"/>
       <c r="AD339" s="14"/>
@@ -9993,8 +10345,9 @@
       <c r="AF339" s="14"/>
       <c r="AG339" s="14"/>
       <c r="AH339" s="14"/>
-    </row>
-    <row r="340" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI339" s="14"/>
+    </row>
+    <row r="340" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB340" s="14"/>
       <c r="AC340" s="14"/>
       <c r="AD340" s="14"/>
@@ -10002,8 +10355,9 @@
       <c r="AF340" s="14"/>
       <c r="AG340" s="14"/>
       <c r="AH340" s="14"/>
-    </row>
-    <row r="341" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI340" s="14"/>
+    </row>
+    <row r="341" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB341" s="14"/>
       <c r="AC341" s="14"/>
       <c r="AD341" s="14"/>
@@ -10011,8 +10365,9 @@
       <c r="AF341" s="14"/>
       <c r="AG341" s="14"/>
       <c r="AH341" s="14"/>
-    </row>
-    <row r="342" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI341" s="14"/>
+    </row>
+    <row r="342" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB342" s="14"/>
       <c r="AC342" s="14"/>
       <c r="AD342" s="14"/>
@@ -10020,8 +10375,9 @@
       <c r="AF342" s="14"/>
       <c r="AG342" s="14"/>
       <c r="AH342" s="14"/>
-    </row>
-    <row r="343" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI342" s="14"/>
+    </row>
+    <row r="343" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB343" s="14"/>
       <c r="AC343" s="14"/>
       <c r="AD343" s="14"/>
@@ -10029,8 +10385,9 @@
       <c r="AF343" s="14"/>
       <c r="AG343" s="14"/>
       <c r="AH343" s="14"/>
-    </row>
-    <row r="344" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI343" s="14"/>
+    </row>
+    <row r="344" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB344" s="14"/>
       <c r="AC344" s="14"/>
       <c r="AD344" s="14"/>
@@ -10038,8 +10395,9 @@
       <c r="AF344" s="14"/>
       <c r="AG344" s="14"/>
       <c r="AH344" s="14"/>
-    </row>
-    <row r="345" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI344" s="14"/>
+    </row>
+    <row r="345" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB345" s="14"/>
       <c r="AC345" s="14"/>
       <c r="AD345" s="14"/>
@@ -10047,8 +10405,9 @@
       <c r="AF345" s="14"/>
       <c r="AG345" s="14"/>
       <c r="AH345" s="14"/>
-    </row>
-    <row r="346" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI345" s="14"/>
+    </row>
+    <row r="346" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB346" s="14"/>
       <c r="AC346" s="14"/>
       <c r="AD346" s="14"/>
@@ -10056,8 +10415,9 @@
       <c r="AF346" s="14"/>
       <c r="AG346" s="14"/>
       <c r="AH346" s="14"/>
-    </row>
-    <row r="347" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI346" s="14"/>
+    </row>
+    <row r="347" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB347" s="14"/>
       <c r="AC347" s="14"/>
       <c r="AD347" s="14"/>
@@ -10065,8 +10425,9 @@
       <c r="AF347" s="14"/>
       <c r="AG347" s="14"/>
       <c r="AH347" s="14"/>
-    </row>
-    <row r="348" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI347" s="14"/>
+    </row>
+    <row r="348" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB348" s="14"/>
       <c r="AC348" s="14"/>
       <c r="AD348" s="14"/>
@@ -10074,8 +10435,9 @@
       <c r="AF348" s="14"/>
       <c r="AG348" s="14"/>
       <c r="AH348" s="14"/>
-    </row>
-    <row r="349" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI348" s="14"/>
+    </row>
+    <row r="349" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB349" s="14"/>
       <c r="AC349" s="14"/>
       <c r="AD349" s="14"/>
@@ -10083,8 +10445,9 @@
       <c r="AF349" s="14"/>
       <c r="AG349" s="14"/>
       <c r="AH349" s="14"/>
-    </row>
-    <row r="350" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI349" s="14"/>
+    </row>
+    <row r="350" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB350" s="14"/>
       <c r="AC350" s="14"/>
       <c r="AD350" s="14"/>
@@ -10092,8 +10455,9 @@
       <c r="AF350" s="14"/>
       <c r="AG350" s="14"/>
       <c r="AH350" s="14"/>
-    </row>
-    <row r="351" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI350" s="14"/>
+    </row>
+    <row r="351" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB351" s="14"/>
       <c r="AC351" s="14"/>
       <c r="AD351" s="14"/>
@@ -10101,8 +10465,9 @@
       <c r="AF351" s="14"/>
       <c r="AG351" s="14"/>
       <c r="AH351" s="14"/>
-    </row>
-    <row r="352" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI351" s="14"/>
+    </row>
+    <row r="352" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB352" s="14"/>
       <c r="AC352" s="14"/>
       <c r="AD352" s="14"/>
@@ -10110,8 +10475,9 @@
       <c r="AF352" s="14"/>
       <c r="AG352" s="14"/>
       <c r="AH352" s="14"/>
-    </row>
-    <row r="353" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI352" s="14"/>
+    </row>
+    <row r="353" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB353" s="14"/>
       <c r="AC353" s="14"/>
       <c r="AD353" s="14"/>
@@ -10119,8 +10485,9 @@
       <c r="AF353" s="14"/>
       <c r="AG353" s="14"/>
       <c r="AH353" s="14"/>
-    </row>
-    <row r="354" spans="28:34" x14ac:dyDescent="0.25">
+      <c r="AI353" s="14"/>
+    </row>
+    <row r="354" spans="28:35" x14ac:dyDescent="0.25">
       <c r="AB354" s="14"/>
       <c r="AC354" s="14"/>
       <c r="AD354" s="14"/>
@@ -10128,6 +10495,7 @@
       <c r="AF354" s="14"/>
       <c r="AG354" s="14"/>
       <c r="AH354" s="14"/>
+      <c r="AI354" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
updated test data item for adjust olpn
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2259F824-671E-4A9A-9BC8-220E59B7A6D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52495BF8-477C-4AF5-B676-36A230B2F83F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1853" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1853" uniqueCount="482">
   <si>
     <t>1</t>
   </si>
@@ -1240,9 +1240,6 @@
   </si>
   <si>
     <t>OV-Receipt Overage,OV-Receipt Overage</t>
-  </si>
-  <si>
-    <t>FG-000022-01</t>
   </si>
   <si>
     <t>AH</t>
@@ -2132,19 +2129,19 @@
         <v>394</v>
       </c>
       <c r="AE1" s="22" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="AF1" s="22" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="AG1" s="22" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="AH1" s="22" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="AI1" s="29" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="2" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2162,7 +2159,7 @@
       </c>
       <c r="E2" s="15"/>
       <c r="F2" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G2" s="14"/>
       <c r="H2" s="14"/>
@@ -2209,7 +2206,7 @@
       </c>
       <c r="E3" s="15"/>
       <c r="F3" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="AB3" s="14"/>
       <c r="AC3" s="14"/>
@@ -2235,7 +2232,7 @@
       </c>
       <c r="E4" s="15"/>
       <c r="F4" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="14"/>
@@ -2264,7 +2261,7 @@
       <c r="AC4" s="14"/>
       <c r="AD4" s="14"/>
       <c r="AE4" s="27" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AF4" s="14"/>
       <c r="AG4" s="14"/>
@@ -2286,7 +2283,7 @@
       </c>
       <c r="E5" s="15"/>
       <c r="F5" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G5" s="14"/>
       <c r="H5" s="14"/>
@@ -2315,7 +2312,7 @@
       <c r="AC5" s="14"/>
       <c r="AD5" s="14"/>
       <c r="AE5" s="27" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AF5" s="14"/>
       <c r="AG5" s="14"/>
@@ -2337,7 +2334,7 @@
       </c>
       <c r="E6" s="15"/>
       <c r="F6" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G6" s="14"/>
       <c r="H6" s="14"/>
@@ -2364,7 +2361,7 @@
       <c r="AC6" s="14"/>
       <c r="AD6" s="14"/>
       <c r="AE6" s="27" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AF6" s="14"/>
       <c r="AG6" s="14"/>
@@ -2386,7 +2383,7 @@
       </c>
       <c r="E7" s="15"/>
       <c r="F7" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G7" s="14"/>
       <c r="H7" s="14"/>
@@ -2413,7 +2410,7 @@
       <c r="AC7" s="14"/>
       <c r="AD7" s="14"/>
       <c r="AE7" s="27" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AF7" s="14"/>
       <c r="AG7" s="14"/>
@@ -2464,7 +2461,7 @@
       </c>
       <c r="E9" s="15"/>
       <c r="F9" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G9" s="15"/>
       <c r="I9" s="14" t="s">
@@ -2494,7 +2491,7 @@
       </c>
       <c r="E10" s="15"/>
       <c r="F10" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G10" s="15"/>
       <c r="I10" s="14" t="s">
@@ -2524,7 +2521,7 @@
       </c>
       <c r="E11" s="15"/>
       <c r="F11" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G11" s="15"/>
       <c r="H11" s="14"/>
@@ -2573,7 +2570,7 @@
       </c>
       <c r="E12" s="15"/>
       <c r="F12" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I12" s="14" t="s">
         <v>127</v>
@@ -2602,7 +2599,7 @@
       </c>
       <c r="E13" s="15"/>
       <c r="F13" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I13" s="14" t="s">
         <v>128</v>
@@ -2631,7 +2628,7 @@
       </c>
       <c r="E14" s="15"/>
       <c r="F14" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G14" s="14"/>
       <c r="H14" s="14"/>
@@ -2732,7 +2729,7 @@
       </c>
       <c r="E17" s="15"/>
       <c r="F17" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I17" s="14" t="s">
         <v>129</v>
@@ -2741,7 +2738,7 @@
       <c r="AC17" s="14"/>
       <c r="AD17" s="14"/>
       <c r="AE17" s="27" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AF17" s="14"/>
       <c r="AG17" s="14"/>
@@ -2763,7 +2760,7 @@
       </c>
       <c r="E18" s="15"/>
       <c r="F18" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I18" s="14" t="s">
         <v>129</v>
@@ -2772,7 +2769,7 @@
       <c r="AC18" s="14"/>
       <c r="AD18" s="14"/>
       <c r="AE18" s="27" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AF18" s="14"/>
       <c r="AG18" s="14"/>
@@ -2794,7 +2791,7 @@
       </c>
       <c r="E19" s="15"/>
       <c r="F19" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I19" s="14" t="s">
         <v>129</v>
@@ -2823,7 +2820,7 @@
       </c>
       <c r="E20" s="15"/>
       <c r="F20" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I20" s="14" t="s">
         <v>129</v>
@@ -2851,7 +2848,7 @@
         <v>59</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I21" s="14" t="s">
         <v>129</v>
@@ -2860,7 +2857,7 @@
       <c r="AC21" s="14"/>
       <c r="AD21" s="14"/>
       <c r="AE21" s="27" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AF21" s="14"/>
       <c r="AG21" s="14"/>
@@ -2881,7 +2878,7 @@
         <v>60</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I22" s="14" t="s">
         <v>129</v>
@@ -2909,7 +2906,7 @@
         <v>61</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I23" s="14" t="s">
         <v>129</v>
@@ -2918,13 +2915,13 @@
       <c r="AC23" s="14"/>
       <c r="AD23" s="14"/>
       <c r="AE23" s="27" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AF23" s="14"/>
       <c r="AG23" s="14"/>
       <c r="AH23" s="14"/>
       <c r="AI23" s="14" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="24" spans="1:35" x14ac:dyDescent="0.25">
@@ -2941,7 +2938,7 @@
         <v>62</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I24" s="14" t="s">
         <v>127</v>
@@ -2954,7 +2951,7 @@
       <c r="AG24" s="14"/>
       <c r="AH24" s="14"/>
       <c r="AI24" s="14" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="25" spans="1:35" x14ac:dyDescent="0.25">
@@ -2971,7 +2968,7 @@
         <v>63</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I25" s="14" t="s">
         <v>126</v>
@@ -2999,7 +2996,7 @@
         <v>64</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I26" s="14" t="s">
         <v>127</v>
@@ -3027,7 +3024,7 @@
         <v>65</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I27" s="14" t="s">
         <v>128</v>
@@ -3056,7 +3053,7 @@
       </c>
       <c r="E28" s="14"/>
       <c r="F28" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G28" s="14"/>
       <c r="H28" s="14"/>
@@ -3103,7 +3100,7 @@
       </c>
       <c r="E29" s="14"/>
       <c r="F29" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G29" s="14"/>
       <c r="H29" s="14"/>
@@ -3150,7 +3147,7 @@
       </c>
       <c r="E30" s="14"/>
       <c r="F30" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G30" s="14"/>
       <c r="H30" s="14"/>
@@ -3197,7 +3194,7 @@
       </c>
       <c r="E31" s="14"/>
       <c r="F31" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G31" s="14"/>
       <c r="H31" s="14"/>
@@ -3244,7 +3241,7 @@
       </c>
       <c r="E32" s="14"/>
       <c r="F32" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G32" s="14"/>
       <c r="H32" s="14"/>
@@ -3291,7 +3288,7 @@
       </c>
       <c r="E33" s="14"/>
       <c r="F33" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G33" s="14"/>
       <c r="H33" s="14"/>
@@ -3338,7 +3335,7 @@
       </c>
       <c r="E34" s="14"/>
       <c r="F34" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G34" s="14"/>
       <c r="H34" s="14"/>
@@ -3385,7 +3382,7 @@
       </c>
       <c r="E35" s="14"/>
       <c r="F35" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G35" s="14"/>
       <c r="H35" s="14"/>
@@ -3432,7 +3429,7 @@
       </c>
       <c r="E36" s="14"/>
       <c r="F36" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G36" s="14"/>
       <c r="H36" s="14"/>
@@ -3479,7 +3476,7 @@
       </c>
       <c r="E37" s="14"/>
       <c r="F37" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G37" s="14"/>
       <c r="H37" s="14"/>
@@ -3526,7 +3523,7 @@
       </c>
       <c r="E38" s="14"/>
       <c r="F38" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G38" s="14"/>
       <c r="H38" s="14"/>
@@ -3573,7 +3570,7 @@
       </c>
       <c r="E39" s="14"/>
       <c r="F39" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G39" s="14"/>
       <c r="H39" s="14"/>
@@ -3620,7 +3617,7 @@
       </c>
       <c r="E40" s="14"/>
       <c r="F40" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G40" s="14"/>
       <c r="H40" s="14"/>
@@ -3647,7 +3644,7 @@
       <c r="AC40" s="14"/>
       <c r="AD40" s="14"/>
       <c r="AE40" s="27" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="AF40" s="14"/>
       <c r="AG40" s="14"/>
@@ -3656,7 +3653,7 @@
     </row>
     <row r="41" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="15" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>108</v>
@@ -3669,7 +3666,7 @@
       </c>
       <c r="E41" s="14"/>
       <c r="F41" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G41" s="14"/>
       <c r="H41" s="14"/>
@@ -3696,7 +3693,7 @@
       <c r="AC41" s="14"/>
       <c r="AD41" s="14"/>
       <c r="AE41" s="27" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="AF41" s="14"/>
       <c r="AG41" s="14"/>
@@ -3705,7 +3702,7 @@
     </row>
     <row r="42" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>108</v>
@@ -3718,7 +3715,7 @@
       </c>
       <c r="E42" s="14"/>
       <c r="F42" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G42" s="14"/>
       <c r="H42" s="14"/>
@@ -3745,7 +3742,7 @@
       <c r="AC42" s="14"/>
       <c r="AD42" s="14"/>
       <c r="AE42" s="27" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AF42" s="14"/>
       <c r="AG42" s="14"/>
@@ -3767,7 +3764,7 @@
       </c>
       <c r="E43" s="14"/>
       <c r="F43" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G43" s="14"/>
       <c r="H43" s="14"/>
@@ -3876,10 +3873,10 @@
         <v>395</v>
       </c>
       <c r="AC45" s="14" t="s">
+        <v>422</v>
+      </c>
+      <c r="AD45" s="14" t="s">
         <v>423</v>
-      </c>
-      <c r="AD45" s="14" t="s">
-        <v>424</v>
       </c>
       <c r="AE45" s="27"/>
       <c r="AF45" s="14"/>
@@ -4739,7 +4736,7 @@
     </row>
     <row r="62" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B62" s="14" t="s">
         <v>108</v>
@@ -4780,25 +4777,25 @@
       <c r="Z62" s="14"/>
       <c r="AA62" s="14"/>
       <c r="AB62" s="14" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AC62" s="14" t="s">
+        <v>469</v>
+      </c>
+      <c r="AD62" s="14" t="s">
         <v>470</v>
-      </c>
-      <c r="AD62" s="14" t="s">
-        <v>471</v>
       </c>
       <c r="AE62" s="27"/>
       <c r="AF62" s="14"/>
       <c r="AG62" s="14"/>
       <c r="AH62" s="14" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="AI62" s="14"/>
     </row>
     <row r="63" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B63" s="14" t="s">
         <v>108</v>
@@ -4807,7 +4804,7 @@
         <v>136</v>
       </c>
       <c r="D63" s="23" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="E63" s="14"/>
       <c r="F63" s="14"/>
@@ -4839,25 +4836,25 @@
       <c r="Z63" s="14"/>
       <c r="AA63" s="14"/>
       <c r="AB63" s="14" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AC63" s="14" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="AD63" s="14" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="AE63" s="27"/>
       <c r="AF63" s="14"/>
       <c r="AG63" s="14"/>
       <c r="AH63" s="15" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="AI63" s="14"/>
     </row>
     <row r="64" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B64" s="14" t="s">
         <v>108</v>
@@ -4866,7 +4863,7 @@
         <v>136</v>
       </c>
       <c r="D64" s="23" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="E64" s="14"/>
       <c r="F64" s="14"/>
@@ -4898,19 +4895,19 @@
       <c r="Z64" s="14"/>
       <c r="AA64" s="14"/>
       <c r="AB64" s="14" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AC64" s="14" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="AD64" s="14" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="AE64" s="27"/>
       <c r="AF64" s="14"/>
       <c r="AG64" s="14"/>
       <c r="AH64" s="15" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="AI64" s="14"/>
     </row>
@@ -4953,7 +4950,7 @@
     </row>
     <row r="66" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B66" s="14" t="s">
         <v>108</v>
@@ -4962,7 +4959,7 @@
         <v>136</v>
       </c>
       <c r="D66" s="23" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="E66" s="14"/>
       <c r="F66" s="14"/>
@@ -4988,25 +4985,25 @@
       <c r="Z66" s="14"/>
       <c r="AA66" s="14"/>
       <c r="AB66" s="14" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AC66" s="14" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="AD66" s="14" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="AE66" s="27"/>
       <c r="AF66" s="14"/>
       <c r="AG66" s="14"/>
       <c r="AH66" s="14" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="AI66" s="14"/>
     </row>
     <row r="67" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B67" s="14" t="s">
         <v>108</v>
@@ -5015,7 +5012,7 @@
         <v>136</v>
       </c>
       <c r="D67" s="23" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="E67" s="14"/>
       <c r="F67" s="14"/>
@@ -5041,25 +5038,25 @@
       <c r="Z67" s="14"/>
       <c r="AA67" s="14"/>
       <c r="AB67" s="14" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AC67" s="14" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="AD67" s="14" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="AE67" s="27"/>
       <c r="AF67" s="14"/>
       <c r="AG67" s="14"/>
       <c r="AH67" s="15" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="AI67" s="14"/>
     </row>
     <row r="68" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B68" s="14" t="s">
         <v>108</v>
@@ -5068,7 +5065,7 @@
         <v>136</v>
       </c>
       <c r="D68" s="23" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E68" s="14"/>
       <c r="F68" s="14"/>
@@ -5097,10 +5094,10 @@
         <v>395</v>
       </c>
       <c r="AC68" s="14" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="AD68" s="14" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="AE68" s="27"/>
       <c r="AF68" s="14"/>
@@ -5110,7 +5107,7 @@
     </row>
     <row r="69" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="14" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B69" s="14" t="s">
         <v>108</v>
@@ -5119,7 +5116,7 @@
         <v>136</v>
       </c>
       <c r="D69" s="23" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="E69" s="14"/>
       <c r="F69" s="14"/>
@@ -5145,25 +5142,25 @@
       <c r="Z69" s="14"/>
       <c r="AA69" s="14"/>
       <c r="AB69" s="14" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AC69" s="14" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="AD69" s="14" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="AE69" s="27"/>
       <c r="AF69" s="14"/>
       <c r="AG69" s="14"/>
       <c r="AH69" s="14" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="AI69" s="14"/>
     </row>
     <row r="70" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="14" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B70" s="14" t="s">
         <v>108</v>
@@ -5172,7 +5169,7 @@
         <v>136</v>
       </c>
       <c r="D70" s="23" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="E70" s="14"/>
       <c r="F70" s="14"/>
@@ -5201,10 +5198,10 @@
         <v>395</v>
       </c>
       <c r="AC70" s="14" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="AD70" s="14" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="AE70" s="27"/>
       <c r="AF70" s="14"/>
@@ -5214,7 +5211,7 @@
     </row>
     <row r="71" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="14" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B71" s="14" t="s">
         <v>108</v>
@@ -5223,7 +5220,7 @@
         <v>136</v>
       </c>
       <c r="D71" s="23" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E71" s="14"/>
       <c r="F71" s="14"/>
@@ -5252,10 +5249,10 @@
         <v>395</v>
       </c>
       <c r="AC71" s="14" t="s">
+        <v>422</v>
+      </c>
+      <c r="AD71" s="14" t="s">
         <v>423</v>
-      </c>
-      <c r="AD71" s="14" t="s">
-        <v>424</v>
       </c>
       <c r="AE71" s="27"/>
       <c r="AF71" s="14"/>
@@ -5265,7 +5262,7 @@
     </row>
     <row r="72" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="14" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B72" s="14" t="s">
         <v>108</v>
@@ -5274,11 +5271,11 @@
         <v>136</v>
       </c>
       <c r="D72" s="23" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="E72" s="15"/>
       <c r="F72" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G72" s="14"/>
       <c r="H72" s="14"/>
@@ -5314,7 +5311,7 @@
     </row>
     <row r="73" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="14" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B73" s="14" t="s">
         <v>108</v>
@@ -5323,11 +5320,11 @@
         <v>136</v>
       </c>
       <c r="D73" s="23" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E73" s="15"/>
       <c r="F73" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G73" s="14"/>
       <c r="H73" s="14"/>
@@ -5356,7 +5353,7 @@
       <c r="AC73" s="14"/>
       <c r="AD73" s="14"/>
       <c r="AE73" s="27" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AF73" s="14"/>
       <c r="AG73" s="14"/>
@@ -5365,7 +5362,7 @@
     </row>
     <row r="74" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="14" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B74" s="14" t="s">
         <v>108</v>
@@ -5374,7 +5371,7 @@
         <v>136</v>
       </c>
       <c r="D74" s="23" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E74" s="14"/>
       <c r="F74" s="14"/>
@@ -5416,7 +5413,7 @@
     </row>
     <row r="75" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B75" s="14" t="s">
         <v>108</v>
@@ -5425,16 +5422,16 @@
         <v>136</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E75" s="15"/>
       <c r="F75" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G75" s="14"/>
       <c r="H75" s="14"/>
       <c r="I75" s="14" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="J75" s="14"/>
       <c r="K75" s="14"/>
@@ -5465,7 +5462,7 @@
     </row>
     <row r="76" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="14" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B76" s="14" t="s">
         <v>108</v>
@@ -5474,7 +5471,7 @@
         <v>136</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E76" s="14"/>
       <c r="F76" s="14"/>
@@ -5503,22 +5500,22 @@
         <v>395</v>
       </c>
       <c r="AC76" s="14" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="AD76" s="14" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="AE76" s="27"/>
       <c r="AF76" s="14"/>
       <c r="AG76" s="14" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="AH76" s="14"/>
       <c r="AI76" s="14"/>
     </row>
     <row r="77" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B77" s="14" t="s">
         <v>108</v>
@@ -5527,7 +5524,7 @@
         <v>136</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E77" s="14"/>
       <c r="F77" s="14"/>
@@ -5553,21 +5550,21 @@
       <c r="Z77" s="14"/>
       <c r="AA77" s="14"/>
       <c r="AB77" s="14" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AC77" s="14" t="s">
+        <v>469</v>
+      </c>
+      <c r="AD77" s="14" t="s">
         <v>470</v>
-      </c>
-      <c r="AD77" s="14" t="s">
-        <v>471</v>
       </c>
       <c r="AE77" s="27"/>
       <c r="AF77" s="14"/>
       <c r="AG77" s="14" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="AH77" s="14" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="AI77" s="14"/>
     </row>
@@ -5713,7 +5710,7 @@
       </c>
       <c r="E81" s="14"/>
       <c r="F81" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
@@ -5762,7 +5759,7 @@
       </c>
       <c r="E82" s="14"/>
       <c r="F82" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
@@ -6073,13 +6070,13 @@
       <c r="H89" s="14"/>
       <c r="I89" s="14"/>
       <c r="J89" s="13" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="K89" s="15" t="s">
         <v>272</v>
       </c>
       <c r="L89" s="14" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="M89" s="14"/>
       <c r="N89" s="14"/>
@@ -6171,7 +6168,7 @@
       <c r="L91" s="12"/>
       <c r="M91" s="12"/>
       <c r="N91" s="12" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="O91" s="12"/>
       <c r="P91" s="12"/>
@@ -6217,7 +6214,7 @@
       <c r="M92" s="12"/>
       <c r="N92" s="12"/>
       <c r="O92" s="12" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P92" s="12"/>
       <c r="Q92" s="14"/>
@@ -6263,7 +6260,7 @@
       <c r="N93" s="12"/>
       <c r="O93" s="12"/>
       <c r="P93" s="13" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="Q93" s="14"/>
       <c r="R93" s="14"/>
@@ -7143,7 +7140,7 @@
         <v>180</v>
       </c>
       <c r="F110" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R110" s="15" t="s">
         <v>0</v>
@@ -7171,7 +7168,7 @@
         <v>181</v>
       </c>
       <c r="F111" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R111" s="15" t="s">
         <v>0</v>
@@ -7199,7 +7196,7 @@
         <v>182</v>
       </c>
       <c r="F112" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R112" s="15" t="s">
         <v>0</v>
@@ -7227,7 +7224,7 @@
         <v>183</v>
       </c>
       <c r="F113" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R113" s="15" t="s">
         <v>0</v>
@@ -7255,7 +7252,7 @@
         <v>184</v>
       </c>
       <c r="F114" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R114" s="15" t="s">
         <v>0</v>
@@ -7283,7 +7280,7 @@
         <v>187</v>
       </c>
       <c r="F115" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R115" s="15" t="s">
         <v>0</v>
@@ -7311,7 +7308,7 @@
         <v>187</v>
       </c>
       <c r="F116" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R116" s="15" t="s">
         <v>2</v>
@@ -7340,7 +7337,7 @@
       </c>
       <c r="E117" s="14"/>
       <c r="F117" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
@@ -7387,7 +7384,7 @@
       </c>
       <c r="E118" s="14"/>
       <c r="F118" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G118" s="14"/>
       <c r="H118" s="14"/>
@@ -7433,7 +7430,7 @@
         <v>240</v>
       </c>
       <c r="F119" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R119" s="15"/>
       <c r="AB119" s="14"/>
@@ -7459,7 +7456,7 @@
         <v>241</v>
       </c>
       <c r="F120" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R120" s="15"/>
       <c r="AB120" s="14"/>
@@ -7485,7 +7482,7 @@
         <v>242</v>
       </c>
       <c r="F121" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R121" s="15"/>
       <c r="AB121" s="14"/>
@@ -7511,7 +7508,7 @@
         <v>259</v>
       </c>
       <c r="F122" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R122" s="15" t="s">
         <v>0</v>
@@ -7539,7 +7536,7 @@
         <v>279</v>
       </c>
       <c r="F123" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="R123" s="15" t="s">
         <v>0</v>
@@ -7568,7 +7565,7 @@
       </c>
       <c r="E124" s="14"/>
       <c r="F124" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G124" s="14"/>
       <c r="H124" s="14"/>
@@ -7617,7 +7614,7 @@
       </c>
       <c r="E125" s="14"/>
       <c r="F125" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G125" s="14"/>
       <c r="H125" s="14"/>
@@ -7666,7 +7663,7 @@
       </c>
       <c r="E126" s="14"/>
       <c r="F126" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G126" s="14"/>
       <c r="H126" s="14"/>
@@ -7715,7 +7712,7 @@
       </c>
       <c r="E127" s="14"/>
       <c r="F127" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
@@ -7764,7 +7761,7 @@
       </c>
       <c r="E128" s="14"/>
       <c r="F128" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
@@ -7813,7 +7810,7 @@
       </c>
       <c r="E129" s="14"/>
       <c r="F129" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G129" s="14"/>
       <c r="H129" s="14"/>
@@ -7862,7 +7859,7 @@
       </c>
       <c r="E130" s="14"/>
       <c r="F130" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G130" s="14"/>
       <c r="H130" s="14"/>
@@ -7911,7 +7908,7 @@
       </c>
       <c r="E131" s="14"/>
       <c r="F131" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
@@ -7960,7 +7957,7 @@
       </c>
       <c r="E132" s="14"/>
       <c r="F132" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G132" s="14"/>
       <c r="H132" s="14"/>
@@ -8009,7 +8006,7 @@
       </c>
       <c r="E133" s="14"/>
       <c r="F133" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G133" s="14"/>
       <c r="H133" s="14"/>
@@ -8058,7 +8055,7 @@
       </c>
       <c r="E134" s="14"/>
       <c r="F134" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
@@ -10553,7 +10550,7 @@
         <v>112</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="I1" s="17" t="s">
         <v>114</v>
@@ -10612,7 +10609,7 @@
       <c r="G2" s="15"/>
       <c r="H2" s="15"/>
       <c r="I2" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
@@ -10653,7 +10650,7 @@
       <c r="G4" s="15"/>
       <c r="H4" s="15"/>
       <c r="I4" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
@@ -10678,7 +10675,7 @@
       <c r="G5" s="15"/>
       <c r="H5" s="15"/>
       <c r="I5" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
@@ -10686,7 +10683,7 @@
         <v>47</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C6" s="15" t="s">
         <v>70</v>
@@ -10701,7 +10698,7 @@
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
       <c r="I6" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
@@ -10709,7 +10706,7 @@
         <v>48</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>70</v>
@@ -10724,7 +10721,7 @@
       <c r="G7" s="15"/>
       <c r="H7" s="15"/>
       <c r="I7" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
@@ -10742,7 +10739,7 @@
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
       <c r="I8" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J8" s="14" t="s">
         <v>122</v>
@@ -10759,7 +10756,7 @@
         <v>50</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>3</v>
@@ -10774,7 +10771,7 @@
       <c r="G9" s="15"/>
       <c r="H9" s="15"/>
       <c r="I9" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J9" s="14" t="s">
         <v>122</v>
@@ -10803,7 +10800,7 @@
       <c r="G10" s="15"/>
       <c r="H10" s="15"/>
       <c r="I10" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J10" s="14" t="s">
         <v>122</v>
@@ -10832,7 +10829,7 @@
       <c r="G11" s="15"/>
       <c r="H11" s="15"/>
       <c r="I11" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
@@ -10855,7 +10852,7 @@
       <c r="G12" s="15"/>
       <c r="H12" s="15"/>
       <c r="I12" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J12" s="14" t="s">
         <v>124</v>
@@ -10887,7 +10884,7 @@
       <c r="G13" s="15"/>
       <c r="H13" s="15"/>
       <c r="I13" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J13" s="14" t="s">
         <v>401</v>
@@ -10912,7 +10909,7 @@
         <v>92</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="C14" s="15" t="s">
         <v>2</v>
@@ -10927,7 +10924,7 @@
       <c r="G14" s="15"/>
       <c r="H14" s="15"/>
       <c r="I14" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J14" s="14" t="s">
         <v>401</v>
@@ -10952,7 +10949,7 @@
         <v>53</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C15" s="15"/>
       <c r="E15" s="15" t="s">
@@ -10985,7 +10982,7 @@
       <c r="G16" s="15"/>
       <c r="H16" s="15"/>
       <c r="I16" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J16" s="14" t="s">
         <v>122</v>
@@ -11024,13 +11021,13 @@
       <c r="G17" s="15"/>
       <c r="H17" s="15"/>
       <c r="I17" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="M17" s="15" t="s">
         <v>66</v>
       </c>
       <c r="N17" s="14" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
@@ -11052,13 +11049,13 @@
       <c r="G18" s="15"/>
       <c r="H18" s="15"/>
       <c r="I18" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="M18" s="15" t="s">
         <v>56</v>
       </c>
       <c r="N18" s="14" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
@@ -11080,13 +11077,13 @@
       <c r="G19" s="15"/>
       <c r="H19" s="15"/>
       <c r="I19" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="M19" s="15" t="s">
         <v>66</v>
       </c>
       <c r="N19" s="14" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
@@ -11108,13 +11105,13 @@
       <c r="G20" s="15"/>
       <c r="H20" s="15"/>
       <c r="I20" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="M20" s="15" t="s">
         <v>56</v>
       </c>
       <c r="N20" s="14" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
@@ -11136,10 +11133,10 @@
       <c r="G21" s="15"/>
       <c r="H21" s="15"/>
       <c r="I21" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="N21" s="14" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
@@ -11161,10 +11158,10 @@
       <c r="G22" s="15"/>
       <c r="H22" s="15"/>
       <c r="I22" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="N22" s="14" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
@@ -11187,7 +11184,7 @@
       <c r="G23" s="15"/>
       <c r="H23" s="15"/>
       <c r="I23" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="O23" s="14" t="s">
         <v>133</v>
@@ -11198,7 +11195,7 @@
         <v>62</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C24" s="15"/>
       <c r="D24" s="14"/>
@@ -11245,7 +11242,7 @@
       <c r="G25" s="15"/>
       <c r="H25" s="15"/>
       <c r="I25" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J25" s="19" t="s">
         <v>122</v>
@@ -11275,7 +11272,7 @@
       <c r="G26" s="15"/>
       <c r="H26" s="15"/>
       <c r="I26" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.25">
@@ -11298,7 +11295,7 @@
       <c r="G27" s="15"/>
       <c r="H27" s="15"/>
       <c r="I27" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J27" s="19" t="s">
         <v>124</v>
@@ -11328,7 +11325,7 @@
       <c r="G28" s="15"/>
       <c r="H28" s="15"/>
       <c r="I28" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J28" s="19"/>
       <c r="K28" s="19"/>
@@ -11362,7 +11359,7 @@
       <c r="G29" s="15"/>
       <c r="H29" s="15"/>
       <c r="I29" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J29" s="19"/>
       <c r="K29" s="19"/>
@@ -11381,7 +11378,7 @@
         <v>68</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C30" s="15" t="s">
         <v>3</v>
@@ -11396,7 +11393,7 @@
       <c r="G30" s="15"/>
       <c r="H30" s="15"/>
       <c r="I30" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J30" s="19"/>
       <c r="K30" s="19"/>
@@ -11430,7 +11427,7 @@
       <c r="G31" s="15"/>
       <c r="H31" s="15"/>
       <c r="I31" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J31" s="19"/>
       <c r="K31" s="19"/>
@@ -11449,7 +11446,7 @@
         <v>36</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C32" s="15" t="s">
         <v>47</v>
@@ -11464,7 +11461,7 @@
       <c r="G32" s="15"/>
       <c r="H32" s="15"/>
       <c r="I32" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J32" s="19"/>
       <c r="K32" s="19"/>
@@ -11498,7 +11495,7 @@
       <c r="G33" s="15"/>
       <c r="H33" s="15"/>
       <c r="I33" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J33" s="19"/>
       <c r="K33" s="19"/>
@@ -11532,7 +11529,7 @@
       <c r="G34" s="15"/>
       <c r="H34" s="15"/>
       <c r="I34" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J34" s="19"/>
       <c r="K34" s="19"/>
@@ -11566,7 +11563,7 @@
       <c r="G35" s="15"/>
       <c r="H35" s="15"/>
       <c r="I35" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J35" s="19"/>
       <c r="K35" s="19"/>
@@ -11600,7 +11597,7 @@
       <c r="G36" s="15"/>
       <c r="H36" s="15"/>
       <c r="I36" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J36" s="19"/>
       <c r="K36" s="19"/>
@@ -11619,7 +11616,7 @@
         <v>74</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>3</v>
@@ -11634,7 +11631,7 @@
       <c r="G37" s="15"/>
       <c r="H37" s="15"/>
       <c r="I37" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J37" s="19"/>
       <c r="K37" s="19"/>
@@ -11668,7 +11665,7 @@
       <c r="G38" s="15"/>
       <c r="H38" s="15"/>
       <c r="I38" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J38" s="19"/>
       <c r="K38" s="19"/>
@@ -11687,7 +11684,7 @@
         <v>76</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C39" s="15" t="s">
         <v>3</v>
@@ -11702,7 +11699,7 @@
       <c r="G39" s="15"/>
       <c r="H39" s="15"/>
       <c r="I39" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J39" s="19"/>
       <c r="K39" s="19"/>
@@ -11721,7 +11718,7 @@
         <v>77</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C40" s="15" t="s">
         <v>3</v>
@@ -11736,7 +11733,7 @@
       <c r="G40" s="15"/>
       <c r="H40" s="15"/>
       <c r="I40" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J40" s="19"/>
       <c r="K40" s="19"/>
@@ -11755,7 +11752,7 @@
         <v>78</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C41" s="15" t="s">
         <v>3</v>
@@ -11770,7 +11767,7 @@
       <c r="G41" s="15"/>
       <c r="H41" s="15"/>
       <c r="I41" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J41" s="19"/>
       <c r="K41" s="19"/>
@@ -11804,7 +11801,7 @@
       <c r="G42" s="15"/>
       <c r="H42" s="15"/>
       <c r="I42" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J42" s="19"/>
       <c r="K42" s="19"/>
@@ -11823,7 +11820,7 @@
         <v>80</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C43" s="15" t="s">
         <v>47</v>
@@ -11838,7 +11835,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="15"/>
       <c r="I43" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J43" s="19"/>
       <c r="K43" s="19"/>
@@ -11857,7 +11854,7 @@
         <v>81</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C44" s="15" t="s">
         <v>3</v>
@@ -11872,7 +11869,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="15"/>
       <c r="I44" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J44" s="19"/>
       <c r="K44" s="19"/>
@@ -11891,7 +11888,7 @@
         <v>82</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C45" s="15" t="s">
         <v>3</v>
@@ -11906,7 +11903,7 @@
       <c r="G45" s="15"/>
       <c r="H45" s="15"/>
       <c r="I45" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J45" s="19"/>
       <c r="K45" s="19"/>
@@ -11925,7 +11922,7 @@
         <v>83</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C46" s="15" t="s">
         <v>3</v>
@@ -11940,7 +11937,7 @@
       <c r="G46" s="15"/>
       <c r="H46" s="15"/>
       <c r="I46" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J46" s="19"/>
       <c r="K46" s="19"/>
@@ -11959,7 +11956,7 @@
         <v>84</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C47" s="15" t="s">
         <v>47</v>
@@ -11974,7 +11971,7 @@
       <c r="G47" s="15"/>
       <c r="H47" s="15"/>
       <c r="I47" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J47" s="19"/>
       <c r="K47" s="19"/>
@@ -11993,7 +11990,7 @@
         <v>85</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C48" s="15" t="s">
         <v>47</v>
@@ -12010,7 +12007,7 @@
       <c r="G48" s="15"/>
       <c r="H48" s="15"/>
       <c r="I48" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J48" s="19"/>
       <c r="K48" s="19"/>
@@ -12044,7 +12041,7 @@
       <c r="G49" s="15"/>
       <c r="H49" s="15"/>
       <c r="I49" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J49" s="19"/>
       <c r="K49" s="14" t="s">
@@ -12065,7 +12062,7 @@
         <v>87</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C50" s="15" t="s">
         <v>2</v>
@@ -12080,7 +12077,7 @@
       <c r="G50" s="15"/>
       <c r="H50" s="15"/>
       <c r="I50" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J50" s="19"/>
       <c r="K50" s="19"/>
@@ -12114,7 +12111,7 @@
       <c r="G51" s="15"/>
       <c r="H51" s="15"/>
       <c r="I51" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J51" s="19"/>
       <c r="K51" s="19"/>
@@ -12148,7 +12145,7 @@
       <c r="G52" s="15"/>
       <c r="H52" s="15"/>
       <c r="I52" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J52" s="19"/>
       <c r="K52" s="19"/>
@@ -12231,7 +12228,7 @@
         <v>162</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C55" s="16" t="s">
         <v>0</v>
@@ -12306,8 +12303,8 @@
       <c r="A57" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="B57" s="18" t="s">
-        <v>419</v>
+      <c r="B57" s="20" t="s">
+        <v>400</v>
       </c>
       <c r="C57" s="16" t="s">
         <v>2</v>
@@ -12344,8 +12341,8 @@
       <c r="A58" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="B58" s="18" t="s">
-        <v>419</v>
+      <c r="B58" s="20" t="s">
+        <v>400</v>
       </c>
       <c r="C58" s="16" t="s">
         <v>0</v>
@@ -12409,7 +12406,7 @@
         <v>173</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C60" s="16" t="s">
         <v>2</v>
@@ -12487,7 +12484,7 @@
         <v>193</v>
       </c>
       <c r="B62" s="18" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C62" s="16" t="s">
         <v>46</v>
@@ -12739,7 +12736,7 @@
         <v>266</v>
       </c>
       <c r="B69" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C69" s="15" t="s">
         <v>0</v>
@@ -12777,7 +12774,7 @@
         <v>348</v>
       </c>
       <c r="B70" s="20" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C70" s="15" t="s">
         <v>0</v>
@@ -12853,7 +12850,7 @@
         <v>350</v>
       </c>
       <c r="B72" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C72" s="16" t="s">
         <v>0</v>
@@ -12926,10 +12923,10 @@
     </row>
     <row r="74" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="16" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B74" s="20" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C74" s="15" t="s">
         <v>2</v>
@@ -12964,10 +12961,10 @@
     </row>
     <row r="75" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="16" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B75" s="20" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C75" s="15" t="s">
         <v>2</v>
@@ -13002,10 +12999,10 @@
     </row>
     <row r="76" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="16" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B76" s="20" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C76" s="15" t="s">
         <v>2</v>
@@ -13101,7 +13098,7 @@
       <c r="G80" s="21"/>
       <c r="H80" s="21"/>
       <c r="I80" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="81" spans="1:20" x14ac:dyDescent="0.25">
@@ -13123,7 +13120,7 @@
       <c r="G81" s="21"/>
       <c r="H81" s="21"/>
       <c r="I81" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="82" spans="1:20" x14ac:dyDescent="0.25">
@@ -13148,7 +13145,7 @@
       <c r="G82" s="21"/>
       <c r="H82" s="21"/>
       <c r="I82" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="83" spans="1:20" x14ac:dyDescent="0.25">
@@ -13170,7 +13167,7 @@
       <c r="G83" s="21"/>
       <c r="H83" s="21"/>
       <c r="I83" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="84" spans="1:20" x14ac:dyDescent="0.25">
@@ -13192,7 +13189,7 @@
       <c r="G84" s="21"/>
       <c r="H84" s="21"/>
       <c r="I84" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="85" spans="1:20" x14ac:dyDescent="0.25">
@@ -13214,7 +13211,7 @@
       <c r="G85" s="21"/>
       <c r="H85" s="21"/>
       <c r="I85" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="86" spans="1:20" x14ac:dyDescent="0.25">
@@ -13236,7 +13233,7 @@
       <c r="G86" s="21"/>
       <c r="H86" s="21"/>
       <c r="I86" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="87" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -13259,7 +13256,7 @@
       <c r="G87" s="21"/>
       <c r="H87" s="21"/>
       <c r="I87" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J87" s="14"/>
       <c r="K87" s="14"/>
@@ -13295,7 +13292,7 @@
       <c r="G88" s="21"/>
       <c r="H88" s="21"/>
       <c r="I88" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="89" spans="1:20" x14ac:dyDescent="0.25">
@@ -13317,7 +13314,7 @@
       <c r="G89" s="21"/>
       <c r="H89" s="21"/>
       <c r="I89" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="90" spans="1:20" x14ac:dyDescent="0.25">
@@ -13339,7 +13336,7 @@
       <c r="G90" s="21"/>
       <c r="H90" s="21"/>
       <c r="I90" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="91" spans="1:20" x14ac:dyDescent="0.25">
@@ -13362,7 +13359,7 @@
       <c r="G91" s="21"/>
       <c r="H91" s="21"/>
       <c r="I91" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="92" spans="1:20" x14ac:dyDescent="0.25">
@@ -13385,7 +13382,7 @@
       <c r="G92" s="21"/>
       <c r="H92" s="21"/>
       <c r="I92" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="93" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -13408,7 +13405,7 @@
       <c r="G93" s="21"/>
       <c r="H93" s="21"/>
       <c r="I93" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J93" s="14"/>
       <c r="K93" s="14"/>
@@ -13444,7 +13441,7 @@
       <c r="G94" s="21"/>
       <c r="H94" s="21"/>
       <c r="I94" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="95" spans="1:20" x14ac:dyDescent="0.25">
@@ -13466,7 +13463,7 @@
       <c r="G95" s="21"/>
       <c r="H95" s="21"/>
       <c r="I95" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="96" spans="1:20" x14ac:dyDescent="0.25">
@@ -13488,7 +13485,7 @@
       <c r="G96" s="21"/>
       <c r="H96" s="21"/>
       <c r="I96" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="97" spans="1:20" x14ac:dyDescent="0.25">
@@ -13510,7 +13507,7 @@
       <c r="G97" s="21"/>
       <c r="H97" s="21"/>
       <c r="I97" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="98" spans="1:20" x14ac:dyDescent="0.25">
@@ -13532,7 +13529,7 @@
       <c r="G98" s="21"/>
       <c r="H98" s="21"/>
       <c r="I98" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="99" spans="1:20" x14ac:dyDescent="0.25">
@@ -13554,7 +13551,7 @@
       <c r="G99" s="21"/>
       <c r="H99" s="21"/>
       <c r="I99" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="100" spans="1:20" x14ac:dyDescent="0.25">
@@ -13576,7 +13573,7 @@
       <c r="G100" s="21"/>
       <c r="H100" s="21"/>
       <c r="I100" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="101" spans="1:20" x14ac:dyDescent="0.25">
@@ -13596,7 +13593,7 @@
         <v>3</v>
       </c>
       <c r="I101" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="102" spans="1:20" x14ac:dyDescent="0.25">
@@ -13616,7 +13613,7 @@
         <v>3</v>
       </c>
       <c r="I102" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="103" spans="1:20" x14ac:dyDescent="0.25">
@@ -13636,7 +13633,7 @@
         <v>3</v>
       </c>
       <c r="I103" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="104" spans="1:20" x14ac:dyDescent="0.25">
@@ -13656,7 +13653,7 @@
         <v>3</v>
       </c>
       <c r="I104" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="105" spans="1:20" x14ac:dyDescent="0.25">
@@ -13676,7 +13673,7 @@
         <v>46</v>
       </c>
       <c r="I105" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="106" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -13699,7 +13696,7 @@
       <c r="G106" s="21"/>
       <c r="H106" s="21"/>
       <c r="I106" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J106" s="14"/>
       <c r="K106" s="14"/>
@@ -13733,7 +13730,7 @@
       <c r="G107" s="21"/>
       <c r="H107" s="21"/>
       <c r="I107" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J107" s="14"/>
       <c r="K107" s="14"/>
@@ -13767,7 +13764,7 @@
       <c r="G108" s="14"/>
       <c r="H108" s="14"/>
       <c r="I108" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J108" s="14" t="s">
         <v>122</v>
@@ -13801,7 +13798,7 @@
       <c r="G109" s="14"/>
       <c r="H109" s="14"/>
       <c r="I109" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J109" s="14" t="s">
         <v>122</v>
@@ -13834,7 +13831,7 @@
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
       <c r="I110" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J110" s="14" t="s">
         <v>122</v>
@@ -13876,10 +13873,10 @@
     </row>
     <row r="112" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="16" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B112" s="20" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C112" s="15" t="s">
         <v>2</v>
@@ -13914,10 +13911,10 @@
     </row>
     <row r="113" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="16" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B113" s="20" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C113" s="15" t="s">
         <v>2</v>
@@ -13952,7 +13949,7 @@
     </row>
     <row r="114" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="16" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B114" s="20" t="s">
         <v>400</v>
@@ -13990,10 +13987,10 @@
     </row>
     <row r="115" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="16" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B115" s="20" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C115" s="15" t="s">
         <v>46</v>
@@ -14028,10 +14025,10 @@
     </row>
     <row r="116" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="16" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B116" s="18" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C116" s="15" t="s">
         <v>3</v>
@@ -14045,10 +14042,10 @@
       <c r="F116" s="15"/>
       <c r="G116" s="15"/>
       <c r="H116" s="15" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="I116" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J116" s="14"/>
       <c r="K116" s="14"/>
@@ -14064,10 +14061,10 @@
     </row>
     <row r="117" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="16" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B117" s="18" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C117" s="15" t="s">
         <v>3</v>
@@ -14082,7 +14079,7 @@
       <c r="G117" s="15"/>
       <c r="H117" s="15"/>
       <c r="I117" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J117" s="14"/>
       <c r="K117" s="14"/>
@@ -14098,10 +14095,10 @@
     </row>
     <row r="118" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="16" t="s">
+        <v>441</v>
+      </c>
+      <c r="B118" s="18" t="s">
         <v>442</v>
-      </c>
-      <c r="B118" s="18" t="s">
-        <v>443</v>
       </c>
       <c r="C118" s="15" t="s">
         <v>3</v>
@@ -14116,7 +14113,7 @@
       <c r="G118" s="15"/>
       <c r="H118" s="15"/>
       <c r="I118" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J118" s="19"/>
       <c r="K118" s="19"/>
@@ -14132,7 +14129,7 @@
     </row>
     <row r="119" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="16" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B119" s="20" t="s">
         <v>400</v>
@@ -14150,7 +14147,7 @@
       <c r="G119" s="15"/>
       <c r="H119" s="15"/>
       <c r="I119" s="14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J119" s="19" t="s">
         <v>124</v>
@@ -14170,10 +14167,10 @@
     </row>
     <row r="120" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="16" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B120" s="20" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C120" s="15" t="s">
         <v>2</v>
@@ -14208,10 +14205,10 @@
     </row>
     <row r="121" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="16" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B121" s="20" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C121" s="15" t="s">
         <v>2</v>
@@ -14246,7 +14243,7 @@
     </row>
     <row r="122" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="16" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B122" s="20" t="s">
         <v>139</v>

</xml_diff>

<commit_message>
Commit code for scripting completed for validation of 861 and 856 files
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25028"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1971D811-3CAC-463F-9576-8D9C937D6025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A12BEB2-C04C-4C66-A91B-9B79D29015B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1903" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1903" uniqueCount="486">
   <si>
     <t>1</t>
   </si>
@@ -1396,9 +1396,6 @@
   </si>
   <si>
     <t>QSC_DailyRegressionOB01</t>
-  </si>
-  <si>
-    <t>FG-200012-00</t>
   </si>
   <si>
     <t>909</t>
@@ -2156,7 +2153,7 @@
         <v>453</v>
       </c>
       <c r="AI1" s="29" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="2" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2936,7 +2933,7 @@
       <c r="AG23" s="14"/>
       <c r="AH23" s="14"/>
       <c r="AI23" s="14" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="24" spans="1:35" x14ac:dyDescent="0.25">
@@ -2966,7 +2963,7 @@
       <c r="AG24" s="14"/>
       <c r="AH24" s="14"/>
       <c r="AI24" s="14" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="25" spans="1:35" x14ac:dyDescent="0.25">
@@ -4795,22 +4792,22 @@
         <v>419</v>
       </c>
       <c r="AC62" s="14" t="s">
+        <v>466</v>
+      </c>
+      <c r="AD62" s="14" t="s">
         <v>467</v>
-      </c>
-      <c r="AD62" s="14" t="s">
-        <v>468</v>
       </c>
       <c r="AE62" s="27"/>
       <c r="AF62" s="14"/>
       <c r="AG62" s="14"/>
       <c r="AH62" s="14" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="AI62" s="14"/>
     </row>
     <row r="63" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B63" s="14" t="s">
         <v>107</v>
@@ -4819,7 +4816,7 @@
         <v>135</v>
       </c>
       <c r="D63" s="23" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="E63" s="14"/>
       <c r="F63" s="14"/>
@@ -4869,7 +4866,7 @@
     </row>
     <row r="64" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B64" s="14" t="s">
         <v>107</v>
@@ -4878,7 +4875,7 @@
         <v>135</v>
       </c>
       <c r="D64" s="23" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="E64" s="14"/>
       <c r="F64" s="14"/>
@@ -4928,7 +4925,7 @@
     </row>
     <row r="65" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B65" s="14" t="s">
         <v>107</v>
@@ -4937,7 +4934,7 @@
         <v>135</v>
       </c>
       <c r="D65" s="23" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="E65" s="14"/>
       <c r="F65" s="14"/>
@@ -4979,7 +4976,7 @@
     </row>
     <row r="66" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B66" s="14" t="s">
         <v>107</v>
@@ -4988,7 +4985,7 @@
         <v>135</v>
       </c>
       <c r="D66" s="23" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="E66" s="14"/>
       <c r="F66" s="14"/>
@@ -5030,7 +5027,7 @@
     </row>
     <row r="67" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B67" s="14" t="s">
         <v>107</v>
@@ -5039,7 +5036,7 @@
         <v>135</v>
       </c>
       <c r="D67" s="23" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="E67" s="14"/>
       <c r="F67" s="14"/>
@@ -5127,7 +5124,7 @@
         <v>135</v>
       </c>
       <c r="D69" s="23" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="E69" s="14"/>
       <c r="F69" s="14"/>
@@ -5156,7 +5153,7 @@
         <v>419</v>
       </c>
       <c r="AC69" s="14" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="AD69" s="14" t="s">
         <v>451</v>
@@ -5165,13 +5162,13 @@
       <c r="AF69" s="14"/>
       <c r="AG69" s="14"/>
       <c r="AH69" s="14" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="AI69" s="14"/>
     </row>
     <row r="70" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="14" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B70" s="14" t="s">
         <v>107</v>
@@ -5180,7 +5177,7 @@
         <v>135</v>
       </c>
       <c r="D70" s="23" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="E70" s="14"/>
       <c r="F70" s="14"/>
@@ -5284,7 +5281,7 @@
         <v>135</v>
       </c>
       <c r="D72" s="23" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="E72" s="14"/>
       <c r="F72" s="14"/>
@@ -5313,7 +5310,7 @@
         <v>419</v>
       </c>
       <c r="AC72" s="14" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="AD72" s="14" t="s">
         <v>451</v>
@@ -5322,7 +5319,7 @@
       <c r="AF72" s="14"/>
       <c r="AG72" s="14"/>
       <c r="AH72" s="14" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="AI72" s="14"/>
     </row>
@@ -5337,7 +5334,7 @@
         <v>135</v>
       </c>
       <c r="D73" s="23" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="E73" s="14"/>
       <c r="F73" s="14"/>
@@ -5639,7 +5636,7 @@
         <v>135</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="E79" s="14"/>
       <c r="F79" s="14"/>
@@ -5683,7 +5680,7 @@
     </row>
     <row r="80" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="14" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B80" s="14" t="s">
         <v>107</v>
@@ -5692,7 +5689,7 @@
         <v>135</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="E80" s="14"/>
       <c r="F80" s="14"/>
@@ -5721,10 +5718,10 @@
         <v>419</v>
       </c>
       <c r="AC80" s="14" t="s">
+        <v>466</v>
+      </c>
+      <c r="AD80" s="14" t="s">
         <v>467</v>
-      </c>
-      <c r="AD80" s="14" t="s">
-        <v>468</v>
       </c>
       <c r="AE80" s="27"/>
       <c r="AF80" s="14"/>
@@ -5732,7 +5729,7 @@
         <v>449</v>
       </c>
       <c r="AH80" s="14" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="AI80" s="14"/>
     </row>
@@ -12942,7 +12939,7 @@
         <v>346</v>
       </c>
       <c r="B70" s="20" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C70" s="15" t="s">
         <v>0</v>
@@ -13091,7 +13088,7 @@
     </row>
     <row r="74" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="16" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B74" s="20" t="s">
         <v>426</v>
@@ -13129,7 +13126,7 @@
     </row>
     <row r="75" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="16" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B75" s="20" t="s">
         <v>428</v>
@@ -13167,7 +13164,7 @@
     </row>
     <row r="76" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="16" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B76" s="20" t="s">
         <v>428</v>
@@ -13205,7 +13202,7 @@
     </row>
     <row r="77" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="16" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B77" s="20" t="s">
         <v>416</v>
@@ -13245,7 +13242,7 @@
     </row>
     <row r="78" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="16" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B78" s="20" t="s">
         <v>426</v>
@@ -13285,7 +13282,7 @@
     </row>
     <row r="79" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="16" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B79" s="20" t="s">
         <v>416</v>
@@ -14459,10 +14456,10 @@
     </row>
     <row r="123" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="16" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B123" s="20" t="s">
-        <v>456</v>
+        <v>398</v>
       </c>
       <c r="C123" s="15" t="s">
         <v>2</v>
@@ -14497,7 +14494,7 @@
     </row>
     <row r="124" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="16" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B124" s="20" t="s">
         <v>428</v>
@@ -14535,7 +14532,7 @@
     </row>
     <row r="125" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="16" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B125" s="20" t="s">
         <v>398</v>

</xml_diff>

<commit_message>
Commit the TestData xls file and NVI Multiline Xml Template
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A12BEB2-C04C-4C66-A91B-9B79D29015B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CDFBCCF-BEBC-46FE-8963-19462817C2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1903" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1989" uniqueCount="500">
   <si>
     <t>1</t>
   </si>
@@ -1486,6 +1486,48 @@
   </si>
   <si>
     <t>904|903</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario002</t>
+  </si>
+  <si>
+    <t>913|914</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario001</t>
+  </si>
+  <si>
+    <t>915</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario004</t>
+  </si>
+  <si>
+    <t>916|917</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario003</t>
+  </si>
+  <si>
+    <t>912</t>
+  </si>
+  <si>
+    <t>000-081221-003</t>
+  </si>
+  <si>
+    <t>913</t>
+  </si>
+  <si>
+    <t>000-081221-002</t>
+  </si>
+  <si>
+    <t>914</t>
+  </si>
+  <si>
+    <t>916</t>
+  </si>
+  <si>
+    <t>917</t>
   </si>
 </sst>
 </file>
@@ -1638,7 +1680,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1677,6 +1719,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2017,7 +2060,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI357"/>
+  <dimension ref="A1:AI359"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -8290,10 +8333,18 @@
       <c r="AI138" s="14"/>
     </row>
     <row r="139" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="14"/>
-      <c r="B139" s="14"/>
-      <c r="C139" s="14"/>
-      <c r="D139" s="15"/>
+      <c r="A139" s="14" t="s">
+        <v>488</v>
+      </c>
+      <c r="B139" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C139" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D139" s="18" t="s">
+        <v>489</v>
+      </c>
       <c r="E139" s="14"/>
       <c r="F139" s="14"/>
       <c r="G139" s="14"/>
@@ -8306,10 +8357,16 @@
       <c r="N139" s="14"/>
       <c r="O139" s="14"/>
       <c r="P139" s="14"/>
-      <c r="Q139" s="14"/>
-      <c r="R139" s="15"/>
-      <c r="S139" s="14"/>
-      <c r="T139" s="14"/>
+      <c r="Q139" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="R139" s="14"/>
+      <c r="S139" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T139" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U139" s="14"/>
       <c r="V139" s="14"/>
       <c r="W139" s="14"/>
@@ -8317,20 +8374,36 @@
       <c r="Y139" s="14"/>
       <c r="Z139" s="14"/>
       <c r="AA139" s="14"/>
-      <c r="AB139" s="14"/>
-      <c r="AC139" s="14"/>
-      <c r="AD139" s="14"/>
+      <c r="AB139" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC139" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD139" s="14" t="s">
+        <v>393</v>
+      </c>
       <c r="AE139" s="27"/>
       <c r="AF139" s="14"/>
       <c r="AG139" s="14"/>
-      <c r="AH139" s="14"/>
+      <c r="AH139" s="14" t="s">
+        <v>465</v>
+      </c>
       <c r="AI139" s="14"/>
     </row>
     <row r="140" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="14"/>
-      <c r="B140" s="14"/>
-      <c r="C140" s="14"/>
-      <c r="D140" s="15"/>
+      <c r="A140" s="14" t="s">
+        <v>486</v>
+      </c>
+      <c r="B140" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C140" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D140" s="18" t="s">
+        <v>487</v>
+      </c>
       <c r="E140" s="14"/>
       <c r="F140" s="14"/>
       <c r="G140" s="14"/>
@@ -8344,7 +8417,7 @@
       <c r="O140" s="14"/>
       <c r="P140" s="14"/>
       <c r="Q140" s="14"/>
-      <c r="R140" s="15"/>
+      <c r="R140" s="14"/>
       <c r="S140" s="14"/>
       <c r="T140" s="14"/>
       <c r="U140" s="14"/>
@@ -8354,28 +8427,77 @@
       <c r="Y140" s="14"/>
       <c r="Z140" s="14"/>
       <c r="AA140" s="14"/>
-      <c r="AB140" s="14"/>
-      <c r="AC140" s="14"/>
-      <c r="AD140" s="14"/>
+      <c r="AB140" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC140" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD140" s="14" t="s">
+        <v>393</v>
+      </c>
       <c r="AE140" s="27"/>
       <c r="AF140" s="14"/>
       <c r="AG140" s="14"/>
       <c r="AH140" s="14"/>
       <c r="AI140" s="14"/>
     </row>
-    <row r="141" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="AB141" s="14"/>
-      <c r="AC141" s="14"/>
-      <c r="AD141" s="14"/>
+    <row r="141" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="14" t="s">
+        <v>492</v>
+      </c>
+      <c r="B141" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C141" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D141" s="18" t="s">
+        <v>493</v>
+      </c>
+      <c r="E141" s="14"/>
+      <c r="F141" s="14"/>
+      <c r="G141" s="14"/>
+      <c r="H141" s="14"/>
+      <c r="I141" s="14"/>
+      <c r="J141" s="14"/>
+      <c r="K141" s="14"/>
+      <c r="L141" s="14"/>
+      <c r="M141" s="14"/>
+      <c r="N141" s="14"/>
+      <c r="O141" s="14"/>
+      <c r="P141" s="14"/>
+      <c r="Q141" s="14"/>
+      <c r="R141" s="14"/>
+      <c r="S141" s="14"/>
+      <c r="T141" s="14"/>
+      <c r="U141" s="14"/>
+      <c r="V141" s="14"/>
+      <c r="W141" s="14"/>
+      <c r="X141" s="14"/>
+      <c r="Y141" s="14"/>
+      <c r="Z141" s="14"/>
+      <c r="AA141" s="14"/>
+      <c r="AB141" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC141" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD141" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE141" s="27"/>
       <c r="AF141" s="14"/>
       <c r="AG141" s="14"/>
-      <c r="AH141" s="14"/>
+      <c r="AH141" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI141" s="14"/>
     </row>
     <row r="142" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="14" t="s">
-        <v>267</v>
+        <v>490</v>
       </c>
       <c r="B142" s="14" t="s">
         <v>174</v>
@@ -8383,29 +8505,31 @@
       <c r="C142" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D142" s="14"/>
+      <c r="D142" s="18" t="s">
+        <v>491</v>
+      </c>
       <c r="E142" s="14"/>
       <c r="F142" s="14"/>
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
       <c r="I142" s="14"/>
-      <c r="J142" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K142" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L142" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J142" s="14"/>
+      <c r="K142" s="14"/>
+      <c r="L142" s="14"/>
       <c r="M142" s="14"/>
       <c r="N142" s="14"/>
       <c r="O142" s="14"/>
       <c r="P142" s="14"/>
-      <c r="Q142" s="14"/>
+      <c r="Q142" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R142" s="14"/>
-      <c r="S142" s="14"/>
-      <c r="T142" s="14"/>
+      <c r="S142" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T142" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U142" s="14"/>
       <c r="V142" s="14"/>
       <c r="W142" s="14"/>
@@ -8413,46 +8537,42 @@
       <c r="Y142" s="14"/>
       <c r="Z142" s="14"/>
       <c r="AA142" s="14"/>
-      <c r="AB142" s="14"/>
-      <c r="AC142" s="14"/>
-      <c r="AD142" s="14"/>
+      <c r="AB142" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC142" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD142" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE142" s="27"/>
       <c r="AF142" s="14"/>
       <c r="AG142" s="14"/>
-      <c r="AH142" s="14"/>
+      <c r="AH142" s="15" t="s">
+        <v>454</v>
+      </c>
       <c r="AI142" s="14"/>
     </row>
     <row r="143" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="14" t="s">
-        <v>268</v>
-      </c>
-      <c r="B143" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C143" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D143" s="14"/>
+      <c r="A143" s="14"/>
+      <c r="B143" s="14"/>
+      <c r="C143" s="14"/>
+      <c r="D143" s="15"/>
       <c r="E143" s="14"/>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="14"/>
-      <c r="J143" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K143" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L143" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="J143" s="14"/>
+      <c r="K143" s="14"/>
+      <c r="L143" s="14"/>
       <c r="M143" s="14"/>
       <c r="N143" s="14"/>
       <c r="O143" s="14"/>
       <c r="P143" s="14"/>
       <c r="Q143" s="14"/>
-      <c r="R143" s="14"/>
+      <c r="R143" s="15"/>
       <c r="S143" s="14"/>
       <c r="T143" s="14"/>
       <c r="U143" s="14"/>
@@ -8471,9 +8591,9 @@
       <c r="AH143" s="14"/>
       <c r="AI143" s="14"/>
     </row>
-    <row r="144" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="14" t="s">
-        <v>359</v>
+        <v>267</v>
       </c>
       <c r="B144" s="14" t="s">
         <v>174</v>
@@ -8481,9 +8601,36 @@
       <c r="C144" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O144" s="15" t="s">
-        <v>362</v>
-      </c>
+      <c r="D144" s="14"/>
+      <c r="E144" s="14"/>
+      <c r="F144" s="14"/>
+      <c r="G144" s="14"/>
+      <c r="H144" s="14"/>
+      <c r="I144" s="14"/>
+      <c r="J144" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K144" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L144" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M144" s="14"/>
+      <c r="N144" s="14"/>
+      <c r="O144" s="14"/>
+      <c r="P144" s="14"/>
+      <c r="Q144" s="14"/>
+      <c r="R144" s="14"/>
+      <c r="S144" s="14"/>
+      <c r="T144" s="14"/>
+      <c r="U144" s="14"/>
+      <c r="V144" s="14"/>
+      <c r="W144" s="14"/>
+      <c r="X144" s="14"/>
+      <c r="Y144" s="14"/>
+      <c r="Z144" s="14"/>
+      <c r="AA144" s="14"/>
       <c r="AB144" s="14"/>
       <c r="AC144" s="14"/>
       <c r="AD144" s="14"/>
@@ -8493,9 +8640,9 @@
       <c r="AH144" s="14"/>
       <c r="AI144" s="14"/>
     </row>
-    <row r="145" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="14" t="s">
-        <v>360</v>
+        <v>268</v>
       </c>
       <c r="B145" s="14" t="s">
         <v>174</v>
@@ -8503,9 +8650,36 @@
       <c r="C145" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O145" s="15" t="s">
-        <v>363</v>
-      </c>
+      <c r="D145" s="14"/>
+      <c r="E145" s="14"/>
+      <c r="F145" s="14"/>
+      <c r="G145" s="14"/>
+      <c r="H145" s="14"/>
+      <c r="I145" s="14"/>
+      <c r="J145" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K145" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L145" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M145" s="14"/>
+      <c r="N145" s="14"/>
+      <c r="O145" s="14"/>
+      <c r="P145" s="14"/>
+      <c r="Q145" s="14"/>
+      <c r="R145" s="14"/>
+      <c r="S145" s="14"/>
+      <c r="T145" s="14"/>
+      <c r="U145" s="14"/>
+      <c r="V145" s="14"/>
+      <c r="W145" s="14"/>
+      <c r="X145" s="14"/>
+      <c r="Y145" s="14"/>
+      <c r="Z145" s="14"/>
+      <c r="AA145" s="14"/>
       <c r="AB145" s="14"/>
       <c r="AC145" s="14"/>
       <c r="AD145" s="14"/>
@@ -8517,7 +8691,7 @@
     </row>
     <row r="146" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A146" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B146" s="14" t="s">
         <v>174</v>
@@ -8526,7 +8700,7 @@
         <v>135</v>
       </c>
       <c r="O146" s="15" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="AB146" s="14"/>
       <c r="AC146" s="14"/>
@@ -8539,7 +8713,7 @@
     </row>
     <row r="147" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A147" s="14" t="s">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="B147" s="14" t="s">
         <v>174</v>
@@ -8547,8 +8721,8 @@
       <c r="C147" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M147" s="14" t="s">
-        <v>371</v>
+      <c r="O147" s="15" t="s">
+        <v>363</v>
       </c>
       <c r="AB147" s="14"/>
       <c r="AC147" s="14"/>
@@ -8560,6 +8734,18 @@
       <c r="AI147" s="14"/>
     </row>
     <row r="148" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A148" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B148" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C148" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O148" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB148" s="14"/>
       <c r="AC148" s="14"/>
       <c r="AD148" s="14"/>
@@ -8570,6 +8756,18 @@
       <c r="AI148" s="14"/>
     </row>
     <row r="149" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A149" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B149" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C149" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M149" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB149" s="14"/>
       <c r="AC149" s="14"/>
       <c r="AD149" s="14"/>
@@ -10593,7 +10791,7 @@
       <c r="AB351" s="14"/>
       <c r="AC351" s="14"/>
       <c r="AD351" s="14"/>
-      <c r="AE351" s="14"/>
+      <c r="AE351" s="27"/>
       <c r="AF351" s="14"/>
       <c r="AG351" s="14"/>
       <c r="AH351" s="14"/>
@@ -10603,7 +10801,7 @@
       <c r="AB352" s="14"/>
       <c r="AC352" s="14"/>
       <c r="AD352" s="14"/>
-      <c r="AE352" s="14"/>
+      <c r="AE352" s="27"/>
       <c r="AF352" s="14"/>
       <c r="AG352" s="14"/>
       <c r="AH352" s="14"/>
@@ -10659,6 +10857,26 @@
       <c r="AH357" s="14"/>
       <c r="AI357" s="14"/>
     </row>
+    <row r="358" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB358" s="14"/>
+      <c r="AC358" s="14"/>
+      <c r="AD358" s="14"/>
+      <c r="AE358" s="14"/>
+      <c r="AF358" s="14"/>
+      <c r="AG358" s="14"/>
+      <c r="AH358" s="14"/>
+      <c r="AI358" s="14"/>
+    </row>
+    <row r="359" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB359" s="14"/>
+      <c r="AC359" s="14"/>
+      <c r="AD359" s="14"/>
+      <c r="AE359" s="14"/>
+      <c r="AF359" s="14"/>
+      <c r="AG359" s="14"/>
+      <c r="AH359" s="14"/>
+      <c r="AI359" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10668,7 +10886,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T125"/>
+  <dimension ref="A1:T132"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -14568,6 +14786,236 @@
       <c r="S125" s="14"/>
       <c r="T125" s="14"/>
     </row>
+    <row r="127" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="15" t="s">
+        <v>493</v>
+      </c>
+      <c r="B127" s="30" t="s">
+        <v>496</v>
+      </c>
+      <c r="C127" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D127" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E127" s="14"/>
+      <c r="F127" s="14"/>
+      <c r="G127" s="14"/>
+      <c r="H127" s="14"/>
+      <c r="I127" s="14"/>
+      <c r="J127" s="14"/>
+      <c r="K127" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L127" s="14"/>
+      <c r="M127" s="14"/>
+      <c r="N127" s="14"/>
+      <c r="O127" s="14"/>
+      <c r="P127" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q127" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R127" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S127" s="14"/>
+      <c r="T127" s="14"/>
+    </row>
+    <row r="128" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="15" t="s">
+        <v>495</v>
+      </c>
+      <c r="B128" s="30" t="s">
+        <v>496</v>
+      </c>
+      <c r="C128" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D128" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E128" s="14"/>
+      <c r="F128" s="14"/>
+      <c r="G128" s="14"/>
+      <c r="H128" s="14"/>
+      <c r="I128" s="14"/>
+      <c r="J128" s="14"/>
+      <c r="K128" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L128" s="14"/>
+      <c r="M128" s="14"/>
+      <c r="N128" s="14"/>
+      <c r="O128" s="14"/>
+      <c r="P128" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q128" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R128" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S128" s="14"/>
+      <c r="T128" s="15" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="15" t="s">
+        <v>497</v>
+      </c>
+      <c r="B129" s="30" t="s">
+        <v>494</v>
+      </c>
+      <c r="C129" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D129" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E129" s="14"/>
+      <c r="F129" s="14"/>
+      <c r="G129" s="14"/>
+      <c r="H129" s="14"/>
+      <c r="I129" s="14"/>
+      <c r="J129" s="14"/>
+      <c r="K129" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L129" s="14"/>
+      <c r="M129" s="14"/>
+      <c r="N129" s="14"/>
+      <c r="O129" s="14"/>
+      <c r="P129" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q129" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R129" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S129" s="14"/>
+      <c r="T129" s="14"/>
+    </row>
+    <row r="130" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="15" t="s">
+        <v>489</v>
+      </c>
+      <c r="B130" s="14" t="s">
+        <v>494</v>
+      </c>
+      <c r="C130" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D130" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E130" s="14"/>
+      <c r="F130" s="14"/>
+      <c r="G130" s="14"/>
+      <c r="H130" s="14"/>
+      <c r="I130" s="14"/>
+      <c r="J130" s="14"/>
+      <c r="K130" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L130" s="14"/>
+      <c r="M130" s="14"/>
+      <c r="N130" s="14"/>
+      <c r="O130" s="14"/>
+      <c r="P130" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q130" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R130" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S130" s="14"/>
+      <c r="T130" s="14"/>
+    </row>
+    <row r="131" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="15" t="s">
+        <v>498</v>
+      </c>
+      <c r="B131" s="30" t="s">
+        <v>494</v>
+      </c>
+      <c r="C131" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D131" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E131" s="14"/>
+      <c r="F131" s="14"/>
+      <c r="G131" s="14"/>
+      <c r="H131" s="14"/>
+      <c r="I131" s="14"/>
+      <c r="J131" s="14"/>
+      <c r="K131" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L131" s="14"/>
+      <c r="M131" s="14"/>
+      <c r="N131" s="14"/>
+      <c r="O131" s="14"/>
+      <c r="P131" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q131" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R131" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S131" s="14"/>
+      <c r="T131" s="14"/>
+    </row>
+    <row r="132" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="15" t="s">
+        <v>499</v>
+      </c>
+      <c r="B132" s="30" t="s">
+        <v>496</v>
+      </c>
+      <c r="C132" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D132" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E132" s="14"/>
+      <c r="F132" s="14"/>
+      <c r="G132" s="14"/>
+      <c r="H132" s="14"/>
+      <c r="I132" s="14"/>
+      <c r="J132" s="14"/>
+      <c r="K132" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L132" s="14"/>
+      <c r="M132" s="14"/>
+      <c r="N132" s="14"/>
+      <c r="O132" s="14"/>
+      <c r="P132" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q132" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R132" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S132" s="14"/>
+      <c r="T132" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Commit the changes as part of NVI Scenarios added to feature file
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25028"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CDFBCCF-BEBC-46FE-8963-19462817C2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09506360-61A2-4C30-B308-4BE7AE80F4D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1989" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2083" uniqueCount="519">
   <si>
     <t>1</t>
   </si>
@@ -1528,6 +1528,63 @@
   </si>
   <si>
     <t>917</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario026</t>
+  </si>
+  <si>
+    <t>918</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario027</t>
+  </si>
+  <si>
+    <t>919</t>
+  </si>
+  <si>
+    <t>OV-Receipt Overage</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario028</t>
+  </si>
+  <si>
+    <t>920</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario029</t>
+  </si>
+  <si>
+    <t>921|922</t>
+  </si>
+  <si>
+    <t>000-081221-155</t>
+  </si>
+  <si>
+    <t>921</t>
+  </si>
+  <si>
+    <t>922</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario030</t>
+  </si>
+  <si>
+    <t>926|927</t>
+  </si>
+  <si>
+    <t>923</t>
+  </si>
+  <si>
+    <t>924</t>
+  </si>
+  <si>
+    <t>925</t>
+  </si>
+  <si>
+    <t>926</t>
+  </si>
+  <si>
+    <t>927</t>
   </si>
 </sst>
 </file>
@@ -2060,7 +2117,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI359"/>
+  <dimension ref="A1:AI364"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -8296,15 +8353,27 @@
       <c r="AI137" s="14"/>
     </row>
     <row r="138" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A138" s="14"/>
-      <c r="B138" s="14"/>
-      <c r="C138" s="14"/>
-      <c r="D138" s="15"/>
-      <c r="E138" s="14"/>
-      <c r="F138" s="14"/>
+      <c r="A138" s="14" t="s">
+        <v>500</v>
+      </c>
+      <c r="B138" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C138" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D138" s="18" t="s">
+        <v>501</v>
+      </c>
+      <c r="E138" s="15"/>
+      <c r="F138" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
-      <c r="I138" s="14"/>
+      <c r="I138" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J138" s="14"/>
       <c r="K138" s="14"/>
       <c r="L138" s="14"/>
@@ -8313,7 +8382,7 @@
       <c r="O138" s="14"/>
       <c r="P138" s="14"/>
       <c r="Q138" s="14"/>
-      <c r="R138" s="15"/>
+      <c r="R138" s="14"/>
       <c r="S138" s="14"/>
       <c r="T138" s="14"/>
       <c r="U138" s="14"/>
@@ -8326,15 +8395,17 @@
       <c r="AB138" s="14"/>
       <c r="AC138" s="14"/>
       <c r="AD138" s="14"/>
-      <c r="AE138" s="27"/>
+      <c r="AE138" s="27" t="s">
+        <v>415</v>
+      </c>
       <c r="AF138" s="14"/>
       <c r="AG138" s="14"/>
       <c r="AH138" s="14"/>
       <c r="AI138" s="14"/>
     </row>
     <row r="139" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="14" t="s">
-        <v>488</v>
+      <c r="A139" s="15" t="s">
+        <v>502</v>
       </c>
       <c r="B139" s="14" t="s">
         <v>174</v>
@@ -8343,13 +8414,17 @@
         <v>135</v>
       </c>
       <c r="D139" s="18" t="s">
-        <v>489</v>
-      </c>
-      <c r="E139" s="14"/>
-      <c r="F139" s="14"/>
-      <c r="G139" s="14"/>
+        <v>503</v>
+      </c>
+      <c r="E139" s="15"/>
+      <c r="F139" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="G139" s="15"/>
       <c r="H139" s="14"/>
-      <c r="I139" s="14"/>
+      <c r="I139" s="14" t="s">
+        <v>504</v>
+      </c>
       <c r="J139" s="14"/>
       <c r="K139" s="14"/>
       <c r="L139" s="14"/>
@@ -8357,16 +8432,10 @@
       <c r="N139" s="14"/>
       <c r="O139" s="14"/>
       <c r="P139" s="14"/>
-      <c r="Q139" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q139" s="14"/>
       <c r="R139" s="14"/>
-      <c r="S139" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T139" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S139" s="14"/>
+      <c r="T139" s="14"/>
       <c r="U139" s="14"/>
       <c r="V139" s="14"/>
       <c r="W139" s="14"/>
@@ -8374,26 +8443,18 @@
       <c r="Y139" s="14"/>
       <c r="Z139" s="14"/>
       <c r="AA139" s="14"/>
-      <c r="AB139" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC139" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD139" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB139" s="14"/>
+      <c r="AC139" s="14"/>
+      <c r="AD139" s="14"/>
       <c r="AE139" s="27"/>
       <c r="AF139" s="14"/>
       <c r="AG139" s="14"/>
-      <c r="AH139" s="14" t="s">
-        <v>465</v>
-      </c>
+      <c r="AH139" s="14"/>
       <c r="AI139" s="14"/>
     </row>
     <row r="140" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="14" t="s">
-        <v>486</v>
+      <c r="A140" s="15" t="s">
+        <v>505</v>
       </c>
       <c r="B140" s="14" t="s">
         <v>174</v>
@@ -8402,10 +8463,12 @@
         <v>135</v>
       </c>
       <c r="D140" s="18" t="s">
-        <v>487</v>
+        <v>506</v>
       </c>
       <c r="E140" s="14"/>
-      <c r="F140" s="14"/>
+      <c r="F140" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="14"/>
@@ -8427,15 +8490,9 @@
       <c r="Y140" s="14"/>
       <c r="Z140" s="14"/>
       <c r="AA140" s="14"/>
-      <c r="AB140" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC140" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD140" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB140" s="14"/>
+      <c r="AC140" s="14"/>
+      <c r="AD140" s="14"/>
       <c r="AE140" s="27"/>
       <c r="AF140" s="14"/>
       <c r="AG140" s="14"/>
@@ -8443,8 +8500,8 @@
       <c r="AI140" s="14"/>
     </row>
     <row r="141" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="14" t="s">
-        <v>492</v>
+      <c r="A141" s="15" t="s">
+        <v>507</v>
       </c>
       <c r="B141" s="14" t="s">
         <v>174</v>
@@ -8453,10 +8510,12 @@
         <v>135</v>
       </c>
       <c r="D141" s="18" t="s">
-        <v>493</v>
+        <v>508</v>
       </c>
       <c r="E141" s="14"/>
-      <c r="F141" s="14"/>
+      <c r="F141" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
       <c r="I141" s="14"/>
@@ -8478,26 +8537,18 @@
       <c r="Y141" s="14"/>
       <c r="Z141" s="14"/>
       <c r="AA141" s="14"/>
-      <c r="AB141" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC141" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD141" s="14" t="s">
-        <v>451</v>
-      </c>
+      <c r="AB141" s="14"/>
+      <c r="AC141" s="14"/>
+      <c r="AD141" s="14"/>
       <c r="AE141" s="27"/>
       <c r="AF141" s="14"/>
       <c r="AG141" s="14"/>
-      <c r="AH141" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH141" s="14"/>
       <c r="AI141" s="14"/>
     </row>
     <row r="142" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A142" s="14" t="s">
-        <v>490</v>
+      <c r="A142" s="15" t="s">
+        <v>512</v>
       </c>
       <c r="B142" s="14" t="s">
         <v>174</v>
@@ -8506,13 +8557,17 @@
         <v>135</v>
       </c>
       <c r="D142" s="18" t="s">
-        <v>491</v>
-      </c>
-      <c r="E142" s="14"/>
-      <c r="F142" s="14"/>
-      <c r="G142" s="14"/>
+        <v>513</v>
+      </c>
+      <c r="E142" s="15"/>
+      <c r="F142" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="G142" s="15"/>
       <c r="H142" s="14"/>
-      <c r="I142" s="14"/>
+      <c r="I142" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J142" s="14"/>
       <c r="K142" s="14"/>
       <c r="L142" s="14"/>
@@ -8520,16 +8575,10 @@
       <c r="N142" s="14"/>
       <c r="O142" s="14"/>
       <c r="P142" s="14"/>
-      <c r="Q142" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q142" s="14"/>
       <c r="R142" s="14"/>
-      <c r="S142" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T142" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S142" s="14"/>
+      <c r="T142" s="14"/>
       <c r="U142" s="14"/>
       <c r="V142" s="14"/>
       <c r="W142" s="14"/>
@@ -8537,21 +8586,13 @@
       <c r="Y142" s="14"/>
       <c r="Z142" s="14"/>
       <c r="AA142" s="14"/>
-      <c r="AB142" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC142" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD142" s="14" t="s">
-        <v>451</v>
-      </c>
+      <c r="AB142" s="14"/>
+      <c r="AC142" s="14"/>
+      <c r="AD142" s="14"/>
       <c r="AE142" s="27"/>
       <c r="AF142" s="14"/>
       <c r="AG142" s="14"/>
-      <c r="AH142" s="15" t="s">
-        <v>454</v>
-      </c>
+      <c r="AH142" s="14"/>
       <c r="AI142" s="14"/>
     </row>
     <row r="143" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -8593,7 +8634,7 @@
     </row>
     <row r="144" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="14" t="s">
-        <v>267</v>
+        <v>488</v>
       </c>
       <c r="B144" s="14" t="s">
         <v>174</v>
@@ -8601,29 +8642,31 @@
       <c r="C144" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D144" s="14"/>
+      <c r="D144" s="18" t="s">
+        <v>489</v>
+      </c>
       <c r="E144" s="14"/>
       <c r="F144" s="14"/>
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
       <c r="I144" s="14"/>
-      <c r="J144" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K144" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L144" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J144" s="14"/>
+      <c r="K144" s="14"/>
+      <c r="L144" s="14"/>
       <c r="M144" s="14"/>
       <c r="N144" s="14"/>
       <c r="O144" s="14"/>
       <c r="P144" s="14"/>
-      <c r="Q144" s="14"/>
+      <c r="Q144" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R144" s="14"/>
-      <c r="S144" s="14"/>
-      <c r="T144" s="14"/>
+      <c r="S144" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T144" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U144" s="14"/>
       <c r="V144" s="14"/>
       <c r="W144" s="14"/>
@@ -8631,18 +8674,26 @@
       <c r="Y144" s="14"/>
       <c r="Z144" s="14"/>
       <c r="AA144" s="14"/>
-      <c r="AB144" s="14"/>
-      <c r="AC144" s="14"/>
-      <c r="AD144" s="14"/>
+      <c r="AB144" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC144" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD144" s="14" t="s">
+        <v>393</v>
+      </c>
       <c r="AE144" s="27"/>
       <c r="AF144" s="14"/>
       <c r="AG144" s="14"/>
-      <c r="AH144" s="14"/>
+      <c r="AH144" s="14" t="s">
+        <v>465</v>
+      </c>
       <c r="AI144" s="14"/>
     </row>
     <row r="145" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="14" t="s">
-        <v>268</v>
+        <v>486</v>
       </c>
       <c r="B145" s="14" t="s">
         <v>174</v>
@@ -8650,21 +8701,17 @@
       <c r="C145" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D145" s="14"/>
+      <c r="D145" s="18" t="s">
+        <v>487</v>
+      </c>
       <c r="E145" s="14"/>
       <c r="F145" s="14"/>
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="14"/>
-      <c r="J145" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K145" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L145" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="J145" s="14"/>
+      <c r="K145" s="14"/>
+      <c r="L145" s="14"/>
       <c r="M145" s="14"/>
       <c r="N145" s="14"/>
       <c r="O145" s="14"/>
@@ -8680,18 +8727,24 @@
       <c r="Y145" s="14"/>
       <c r="Z145" s="14"/>
       <c r="AA145" s="14"/>
-      <c r="AB145" s="14"/>
-      <c r="AC145" s="14"/>
-      <c r="AD145" s="14"/>
+      <c r="AB145" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC145" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD145" s="14" t="s">
+        <v>393</v>
+      </c>
       <c r="AE145" s="27"/>
       <c r="AF145" s="14"/>
       <c r="AG145" s="14"/>
       <c r="AH145" s="14"/>
       <c r="AI145" s="14"/>
     </row>
-    <row r="146" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="14" t="s">
-        <v>359</v>
+        <v>492</v>
       </c>
       <c r="B146" s="14" t="s">
         <v>174</v>
@@ -8699,21 +8752,52 @@
       <c r="C146" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O146" s="15" t="s">
-        <v>362</v>
-      </c>
-      <c r="AB146" s="14"/>
-      <c r="AC146" s="14"/>
-      <c r="AD146" s="14"/>
+      <c r="D146" s="18" t="s">
+        <v>493</v>
+      </c>
+      <c r="E146" s="14"/>
+      <c r="F146" s="14"/>
+      <c r="G146" s="14"/>
+      <c r="H146" s="14"/>
+      <c r="I146" s="14"/>
+      <c r="J146" s="14"/>
+      <c r="K146" s="14"/>
+      <c r="L146" s="14"/>
+      <c r="M146" s="14"/>
+      <c r="N146" s="14"/>
+      <c r="O146" s="14"/>
+      <c r="P146" s="14"/>
+      <c r="Q146" s="14"/>
+      <c r="R146" s="14"/>
+      <c r="S146" s="14"/>
+      <c r="T146" s="14"/>
+      <c r="U146" s="14"/>
+      <c r="V146" s="14"/>
+      <c r="W146" s="14"/>
+      <c r="X146" s="14"/>
+      <c r="Y146" s="14"/>
+      <c r="Z146" s="14"/>
+      <c r="AA146" s="14"/>
+      <c r="AB146" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC146" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD146" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE146" s="27"/>
       <c r="AF146" s="14"/>
       <c r="AG146" s="14"/>
-      <c r="AH146" s="14"/>
+      <c r="AH146" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI146" s="14"/>
     </row>
-    <row r="147" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="14" t="s">
-        <v>360</v>
+        <v>490</v>
       </c>
       <c r="B147" s="14" t="s">
         <v>174</v>
@@ -8721,31 +8805,83 @@
       <c r="C147" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O147" s="15" t="s">
-        <v>363</v>
-      </c>
-      <c r="AB147" s="14"/>
-      <c r="AC147" s="14"/>
-      <c r="AD147" s="14"/>
+      <c r="D147" s="18" t="s">
+        <v>491</v>
+      </c>
+      <c r="E147" s="14"/>
+      <c r="F147" s="14"/>
+      <c r="G147" s="14"/>
+      <c r="H147" s="14"/>
+      <c r="I147" s="14"/>
+      <c r="J147" s="14"/>
+      <c r="K147" s="14"/>
+      <c r="L147" s="14"/>
+      <c r="M147" s="14"/>
+      <c r="N147" s="14"/>
+      <c r="O147" s="14"/>
+      <c r="P147" s="14"/>
+      <c r="Q147" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="R147" s="14"/>
+      <c r="S147" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T147" s="14" t="s">
+        <v>300</v>
+      </c>
+      <c r="U147" s="14"/>
+      <c r="V147" s="14"/>
+      <c r="W147" s="14"/>
+      <c r="X147" s="14"/>
+      <c r="Y147" s="14"/>
+      <c r="Z147" s="14"/>
+      <c r="AA147" s="14"/>
+      <c r="AB147" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC147" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD147" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE147" s="27"/>
       <c r="AF147" s="14"/>
       <c r="AG147" s="14"/>
-      <c r="AH147" s="14"/>
+      <c r="AH147" s="15" t="s">
+        <v>454</v>
+      </c>
       <c r="AI147" s="14"/>
     </row>
-    <row r="148" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A148" s="14" t="s">
-        <v>361</v>
-      </c>
-      <c r="B148" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C148" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O148" s="15" t="s">
-        <v>364</v>
-      </c>
+    <row r="148" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A148" s="14"/>
+      <c r="B148" s="14"/>
+      <c r="C148" s="14"/>
+      <c r="D148" s="15"/>
+      <c r="E148" s="14"/>
+      <c r="F148" s="14"/>
+      <c r="G148" s="14"/>
+      <c r="H148" s="14"/>
+      <c r="I148" s="14"/>
+      <c r="J148" s="14"/>
+      <c r="K148" s="14"/>
+      <c r="L148" s="14"/>
+      <c r="M148" s="14"/>
+      <c r="N148" s="14"/>
+      <c r="O148" s="14"/>
+      <c r="P148" s="14"/>
+      <c r="Q148" s="14"/>
+      <c r="R148" s="15"/>
+      <c r="S148" s="14"/>
+      <c r="T148" s="14"/>
+      <c r="U148" s="14"/>
+      <c r="V148" s="14"/>
+      <c r="W148" s="14"/>
+      <c r="X148" s="14"/>
+      <c r="Y148" s="14"/>
+      <c r="Z148" s="14"/>
+      <c r="AA148" s="14"/>
       <c r="AB148" s="14"/>
       <c r="AC148" s="14"/>
       <c r="AD148" s="14"/>
@@ -8755,9 +8891,9 @@
       <c r="AH148" s="14"/>
       <c r="AI148" s="14"/>
     </row>
-    <row r="149" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="14" t="s">
-        <v>370</v>
+        <v>267</v>
       </c>
       <c r="B149" s="14" t="s">
         <v>174</v>
@@ -8765,9 +8901,36 @@
       <c r="C149" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M149" s="14" t="s">
-        <v>371</v>
-      </c>
+      <c r="D149" s="14"/>
+      <c r="E149" s="14"/>
+      <c r="F149" s="14"/>
+      <c r="G149" s="14"/>
+      <c r="H149" s="14"/>
+      <c r="I149" s="14"/>
+      <c r="J149" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K149" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L149" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M149" s="14"/>
+      <c r="N149" s="14"/>
+      <c r="O149" s="14"/>
+      <c r="P149" s="14"/>
+      <c r="Q149" s="14"/>
+      <c r="R149" s="14"/>
+      <c r="S149" s="14"/>
+      <c r="T149" s="14"/>
+      <c r="U149" s="14"/>
+      <c r="V149" s="14"/>
+      <c r="W149" s="14"/>
+      <c r="X149" s="14"/>
+      <c r="Y149" s="14"/>
+      <c r="Z149" s="14"/>
+      <c r="AA149" s="14"/>
       <c r="AB149" s="14"/>
       <c r="AC149" s="14"/>
       <c r="AD149" s="14"/>
@@ -8777,7 +8940,46 @@
       <c r="AH149" s="14"/>
       <c r="AI149" s="14"/>
     </row>
-    <row r="150" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="B150" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C150" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D150" s="14"/>
+      <c r="E150" s="14"/>
+      <c r="F150" s="14"/>
+      <c r="G150" s="14"/>
+      <c r="H150" s="14"/>
+      <c r="I150" s="14"/>
+      <c r="J150" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K150" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L150" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M150" s="14"/>
+      <c r="N150" s="14"/>
+      <c r="O150" s="14"/>
+      <c r="P150" s="14"/>
+      <c r="Q150" s="14"/>
+      <c r="R150" s="14"/>
+      <c r="S150" s="14"/>
+      <c r="T150" s="14"/>
+      <c r="U150" s="14"/>
+      <c r="V150" s="14"/>
+      <c r="W150" s="14"/>
+      <c r="X150" s="14"/>
+      <c r="Y150" s="14"/>
+      <c r="Z150" s="14"/>
+      <c r="AA150" s="14"/>
       <c r="AB150" s="14"/>
       <c r="AC150" s="14"/>
       <c r="AD150" s="14"/>
@@ -8788,6 +8990,18 @@
       <c r="AI150" s="14"/>
     </row>
     <row r="151" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A151" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="B151" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C151" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O151" s="15" t="s">
+        <v>362</v>
+      </c>
       <c r="AB151" s="14"/>
       <c r="AC151" s="14"/>
       <c r="AD151" s="14"/>
@@ -8798,6 +9012,18 @@
       <c r="AI151" s="14"/>
     </row>
     <row r="152" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A152" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B152" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C152" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O152" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB152" s="14"/>
       <c r="AC152" s="14"/>
       <c r="AD152" s="14"/>
@@ -8808,6 +9034,18 @@
       <c r="AI152" s="14"/>
     </row>
     <row r="153" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A153" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B153" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C153" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O153" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB153" s="14"/>
       <c r="AC153" s="14"/>
       <c r="AD153" s="14"/>
@@ -8818,6 +9056,18 @@
       <c r="AI153" s="14"/>
     </row>
     <row r="154" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A154" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B154" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C154" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M154" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB154" s="14"/>
       <c r="AC154" s="14"/>
       <c r="AD154" s="14"/>
@@ -10811,7 +11061,7 @@
       <c r="AB353" s="14"/>
       <c r="AC353" s="14"/>
       <c r="AD353" s="14"/>
-      <c r="AE353" s="14"/>
+      <c r="AE353" s="27"/>
       <c r="AF353" s="14"/>
       <c r="AG353" s="14"/>
       <c r="AH353" s="14"/>
@@ -10821,7 +11071,7 @@
       <c r="AB354" s="14"/>
       <c r="AC354" s="14"/>
       <c r="AD354" s="14"/>
-      <c r="AE354" s="14"/>
+      <c r="AE354" s="27"/>
       <c r="AF354" s="14"/>
       <c r="AG354" s="14"/>
       <c r="AH354" s="14"/>
@@ -10831,7 +11081,7 @@
       <c r="AB355" s="14"/>
       <c r="AC355" s="14"/>
       <c r="AD355" s="14"/>
-      <c r="AE355" s="14"/>
+      <c r="AE355" s="27"/>
       <c r="AF355" s="14"/>
       <c r="AG355" s="14"/>
       <c r="AH355" s="14"/>
@@ -10841,7 +11091,7 @@
       <c r="AB356" s="14"/>
       <c r="AC356" s="14"/>
       <c r="AD356" s="14"/>
-      <c r="AE356" s="14"/>
+      <c r="AE356" s="27"/>
       <c r="AF356" s="14"/>
       <c r="AG356" s="14"/>
       <c r="AH356" s="14"/>
@@ -10851,7 +11101,7 @@
       <c r="AB357" s="14"/>
       <c r="AC357" s="14"/>
       <c r="AD357" s="14"/>
-      <c r="AE357" s="14"/>
+      <c r="AE357" s="27"/>
       <c r="AF357" s="14"/>
       <c r="AG357" s="14"/>
       <c r="AH357" s="14"/>
@@ -10877,6 +11127,56 @@
       <c r="AH359" s="14"/>
       <c r="AI359" s="14"/>
     </row>
+    <row r="360" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB360" s="14"/>
+      <c r="AC360" s="14"/>
+      <c r="AD360" s="14"/>
+      <c r="AE360" s="14"/>
+      <c r="AF360" s="14"/>
+      <c r="AG360" s="14"/>
+      <c r="AH360" s="14"/>
+      <c r="AI360" s="14"/>
+    </row>
+    <row r="361" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB361" s="14"/>
+      <c r="AC361" s="14"/>
+      <c r="AD361" s="14"/>
+      <c r="AE361" s="14"/>
+      <c r="AF361" s="14"/>
+      <c r="AG361" s="14"/>
+      <c r="AH361" s="14"/>
+      <c r="AI361" s="14"/>
+    </row>
+    <row r="362" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB362" s="14"/>
+      <c r="AC362" s="14"/>
+      <c r="AD362" s="14"/>
+      <c r="AE362" s="14"/>
+      <c r="AF362" s="14"/>
+      <c r="AG362" s="14"/>
+      <c r="AH362" s="14"/>
+      <c r="AI362" s="14"/>
+    </row>
+    <row r="363" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB363" s="14"/>
+      <c r="AC363" s="14"/>
+      <c r="AD363" s="14"/>
+      <c r="AE363" s="14"/>
+      <c r="AF363" s="14"/>
+      <c r="AG363" s="14"/>
+      <c r="AH363" s="14"/>
+      <c r="AI363" s="14"/>
+    </row>
+    <row r="364" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB364" s="14"/>
+      <c r="AC364" s="14"/>
+      <c r="AD364" s="14"/>
+      <c r="AE364" s="14"/>
+      <c r="AF364" s="14"/>
+      <c r="AG364" s="14"/>
+      <c r="AH364" s="14"/>
+      <c r="AI364" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10886,7 +11186,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T132"/>
+  <dimension ref="A1:T142"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -15016,6 +15316,356 @@
       <c r="S132" s="14"/>
       <c r="T132" s="14"/>
     </row>
+    <row r="133" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="15" t="s">
+        <v>501</v>
+      </c>
+      <c r="B133" s="18" t="s">
+        <v>440</v>
+      </c>
+      <c r="C133" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D133" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E133" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="F133" s="15"/>
+      <c r="G133" s="15"/>
+      <c r="H133" s="15"/>
+      <c r="I133" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J133" s="14"/>
+      <c r="K133" s="14"/>
+      <c r="L133" s="14"/>
+      <c r="M133" s="14"/>
+      <c r="N133" s="14"/>
+      <c r="O133" s="14"/>
+      <c r="P133" s="14"/>
+      <c r="Q133" s="14"/>
+      <c r="R133" s="14"/>
+      <c r="S133" s="14"/>
+      <c r="T133" s="14"/>
+    </row>
+    <row r="134" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="15" t="s">
+        <v>503</v>
+      </c>
+      <c r="B134" s="30" t="s">
+        <v>509</v>
+      </c>
+      <c r="C134" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D134" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E134" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F134" s="15"/>
+      <c r="G134" s="15"/>
+      <c r="H134" s="15"/>
+      <c r="I134" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J134" s="14" t="s">
+        <v>399</v>
+      </c>
+      <c r="K134" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L134" s="14" t="s">
+        <v>399</v>
+      </c>
+      <c r="M134" s="14"/>
+      <c r="N134" s="14"/>
+      <c r="O134" s="14"/>
+      <c r="P134" s="14"/>
+      <c r="Q134" s="14"/>
+      <c r="R134" s="14"/>
+      <c r="S134" s="14"/>
+      <c r="T134" s="14"/>
+    </row>
+    <row r="135" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="15" t="s">
+        <v>506</v>
+      </c>
+      <c r="B135" s="30" t="s">
+        <v>496</v>
+      </c>
+      <c r="C135" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D135" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E135" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F135" s="15"/>
+      <c r="G135" s="15"/>
+      <c r="H135" s="15"/>
+      <c r="I135" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J135" s="14"/>
+      <c r="K135" s="14"/>
+      <c r="L135" s="14"/>
+      <c r="M135" s="14"/>
+      <c r="N135" s="14"/>
+      <c r="O135" s="14"/>
+      <c r="P135" s="14"/>
+      <c r="Q135" s="14"/>
+      <c r="R135" s="14"/>
+      <c r="S135" s="14"/>
+      <c r="T135" s="14"/>
+    </row>
+    <row r="136" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="15" t="s">
+        <v>510</v>
+      </c>
+      <c r="B136" s="30" t="s">
+        <v>496</v>
+      </c>
+      <c r="C136" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D136" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E136" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F136" s="15"/>
+      <c r="G136" s="15"/>
+      <c r="H136" s="15"/>
+      <c r="I136" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J136" s="14"/>
+      <c r="K136" s="14"/>
+      <c r="L136" s="14"/>
+      <c r="M136" s="14"/>
+      <c r="N136" s="14"/>
+      <c r="O136" s="14"/>
+      <c r="P136" s="14"/>
+      <c r="Q136" s="14"/>
+      <c r="R136" s="14"/>
+      <c r="S136" s="14"/>
+      <c r="T136" s="14"/>
+    </row>
+    <row r="137" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="15" t="s">
+        <v>511</v>
+      </c>
+      <c r="B137" s="30" t="s">
+        <v>494</v>
+      </c>
+      <c r="C137" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D137" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E137" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F137" s="15"/>
+      <c r="G137" s="15"/>
+      <c r="H137" s="15"/>
+      <c r="I137" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J137" s="14"/>
+      <c r="K137" s="14"/>
+      <c r="L137" s="14"/>
+      <c r="M137" s="14"/>
+      <c r="N137" s="14"/>
+      <c r="O137" s="14"/>
+      <c r="P137" s="14"/>
+      <c r="Q137" s="14"/>
+      <c r="R137" s="14"/>
+      <c r="S137" s="14"/>
+      <c r="T137" s="14"/>
+    </row>
+    <row r="138" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="15" t="s">
+        <v>514</v>
+      </c>
+      <c r="B138" s="18" t="s">
+        <v>404</v>
+      </c>
+      <c r="C138" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D138" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E138" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="F138" s="15"/>
+      <c r="G138" s="15"/>
+      <c r="H138" s="15"/>
+      <c r="I138" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J138" s="14"/>
+      <c r="K138" s="14"/>
+      <c r="L138" s="14"/>
+      <c r="M138" s="14"/>
+      <c r="N138" s="14"/>
+      <c r="O138" s="14"/>
+      <c r="P138" s="14"/>
+      <c r="Q138" s="14"/>
+      <c r="R138" s="14"/>
+      <c r="S138" s="14"/>
+      <c r="T138" s="14"/>
+    </row>
+    <row r="139" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="15" t="s">
+        <v>515</v>
+      </c>
+      <c r="B139" s="30" t="s">
+        <v>398</v>
+      </c>
+      <c r="C139" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D139" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E139" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="F139" s="15"/>
+      <c r="G139" s="15"/>
+      <c r="H139" s="15"/>
+      <c r="I139" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J139" s="14"/>
+      <c r="K139" s="14"/>
+      <c r="L139" s="14"/>
+      <c r="M139" s="14"/>
+      <c r="N139" s="14"/>
+      <c r="O139" s="14"/>
+      <c r="P139" s="14"/>
+      <c r="Q139" s="14"/>
+      <c r="R139" s="14"/>
+      <c r="S139" s="14"/>
+      <c r="T139" s="14"/>
+    </row>
+    <row r="140" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B140" s="30" t="s">
+        <v>398</v>
+      </c>
+      <c r="C140" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D140" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E140" s="14"/>
+      <c r="F140" s="14"/>
+      <c r="G140" s="14"/>
+      <c r="H140" s="14"/>
+      <c r="I140" s="14"/>
+      <c r="J140" s="14"/>
+      <c r="K140" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L140" s="14"/>
+      <c r="M140" s="14"/>
+      <c r="N140" s="14"/>
+      <c r="O140" s="14"/>
+      <c r="P140" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q140" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R140" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S140" s="14"/>
+      <c r="T140" s="14"/>
+    </row>
+    <row r="141" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="15" t="s">
+        <v>517</v>
+      </c>
+      <c r="B141" s="30" t="s">
+        <v>494</v>
+      </c>
+      <c r="C141" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D141" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E141" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="F141" s="15"/>
+      <c r="G141" s="15"/>
+      <c r="H141" s="15"/>
+      <c r="I141" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J141" s="14"/>
+      <c r="K141" s="14"/>
+      <c r="L141" s="14"/>
+      <c r="M141" s="14"/>
+      <c r="N141" s="14"/>
+      <c r="O141" s="14"/>
+      <c r="P141" s="14"/>
+      <c r="Q141" s="14"/>
+      <c r="R141" s="14"/>
+      <c r="S141" s="14"/>
+      <c r="T141" s="14"/>
+    </row>
+    <row r="142" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="B142" s="30" t="s">
+        <v>496</v>
+      </c>
+      <c r="C142" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D142" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E142" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="F142" s="15"/>
+      <c r="G142" s="15"/>
+      <c r="H142" s="15"/>
+      <c r="I142" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J142" s="14"/>
+      <c r="K142" s="14"/>
+      <c r="L142" s="14"/>
+      <c r="M142" s="14"/>
+      <c r="N142" s="14"/>
+      <c r="O142" s="14"/>
+      <c r="P142" s="14"/>
+      <c r="Q142" s="14"/>
+      <c r="R142" s="14"/>
+      <c r="S142" s="14"/>
+      <c r="T142" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Commit the Testdata and excel file for NVI Inbound scenarios
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25028"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09506360-61A2-4C30-B308-4BE7AE80F4D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{032F975C-1675-4777-8CD1-3424980F6CB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2083" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2157" uniqueCount="531">
   <si>
     <t>1</t>
   </si>
@@ -1585,6 +1585,42 @@
   </si>
   <si>
     <t>927</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario031</t>
+  </si>
+  <si>
+    <t>928</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario032</t>
+  </si>
+  <si>
+    <t>929</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario033</t>
+  </si>
+  <si>
+    <t>930</t>
+  </si>
+  <si>
+    <t>931</t>
+  </si>
+  <si>
+    <t>930|931</t>
+  </si>
+  <si>
+    <t>932</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario034</t>
+  </si>
+  <si>
+    <t>NVI_KelliScenario001</t>
+  </si>
+  <si>
+    <t>933</t>
   </si>
 </sst>
 </file>
@@ -2117,7 +2153,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI364"/>
+  <dimension ref="A1:AI368"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -8596,13 +8632,25 @@
       <c r="AI142" s="14"/>
     </row>
     <row r="143" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="14"/>
-      <c r="B143" s="14"/>
-      <c r="C143" s="14"/>
-      <c r="D143" s="15"/>
-      <c r="E143" s="14"/>
-      <c r="F143" s="14"/>
-      <c r="G143" s="14"/>
+      <c r="A143" s="15" t="s">
+        <v>519</v>
+      </c>
+      <c r="B143" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C143" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D143" s="18" t="s">
+        <v>520</v>
+      </c>
+      <c r="E143" s="15"/>
+      <c r="F143" s="15" t="s">
+        <v>388</v>
+      </c>
+      <c r="G143" s="15" t="s">
+        <v>3</v>
+      </c>
       <c r="H143" s="14"/>
       <c r="I143" s="14"/>
       <c r="J143" s="14"/>
@@ -8613,7 +8661,7 @@
       <c r="O143" s="14"/>
       <c r="P143" s="14"/>
       <c r="Q143" s="14"/>
-      <c r="R143" s="15"/>
+      <c r="R143" s="14"/>
       <c r="S143" s="14"/>
       <c r="T143" s="14"/>
       <c r="U143" s="14"/>
@@ -8633,8 +8681,8 @@
       <c r="AI143" s="14"/>
     </row>
     <row r="144" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A144" s="14" t="s">
-        <v>488</v>
+      <c r="A144" s="15" t="s">
+        <v>521</v>
       </c>
       <c r="B144" s="14" t="s">
         <v>174</v>
@@ -8643,13 +8691,17 @@
         <v>135</v>
       </c>
       <c r="D144" s="18" t="s">
-        <v>489</v>
-      </c>
-      <c r="E144" s="14"/>
-      <c r="F144" s="14"/>
+        <v>522</v>
+      </c>
+      <c r="E144" s="15"/>
+      <c r="F144" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G144" s="14"/>
       <c r="H144" s="14"/>
-      <c r="I144" s="14"/>
+      <c r="I144" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J144" s="14"/>
       <c r="K144" s="14"/>
       <c r="L144" s="14"/>
@@ -8657,16 +8709,10 @@
       <c r="N144" s="14"/>
       <c r="O144" s="14"/>
       <c r="P144" s="14"/>
-      <c r="Q144" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q144" s="14"/>
       <c r="R144" s="14"/>
-      <c r="S144" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T144" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S144" s="14"/>
+      <c r="T144" s="14"/>
       <c r="U144" s="14"/>
       <c r="V144" s="14"/>
       <c r="W144" s="14"/>
@@ -8674,26 +8720,20 @@
       <c r="Y144" s="14"/>
       <c r="Z144" s="14"/>
       <c r="AA144" s="14"/>
-      <c r="AB144" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC144" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD144" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AE144" s="27"/>
+      <c r="AB144" s="14"/>
+      <c r="AC144" s="14"/>
+      <c r="AD144" s="14"/>
+      <c r="AE144" s="27" t="s">
+        <v>415</v>
+      </c>
       <c r="AF144" s="14"/>
       <c r="AG144" s="14"/>
-      <c r="AH144" s="14" t="s">
-        <v>465</v>
-      </c>
+      <c r="AH144" s="14"/>
       <c r="AI144" s="14"/>
     </row>
     <row r="145" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A145" s="14" t="s">
-        <v>486</v>
+      <c r="A145" s="15" t="s">
+        <v>523</v>
       </c>
       <c r="B145" s="14" t="s">
         <v>174</v>
@@ -8702,13 +8742,17 @@
         <v>135</v>
       </c>
       <c r="D145" s="18" t="s">
-        <v>487</v>
-      </c>
-      <c r="E145" s="14"/>
-      <c r="F145" s="14"/>
+        <v>526</v>
+      </c>
+      <c r="E145" s="15"/>
+      <c r="F145" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G145" s="14"/>
       <c r="H145" s="14"/>
-      <c r="I145" s="14"/>
+      <c r="I145" s="14" t="s">
+        <v>401</v>
+      </c>
       <c r="J145" s="14"/>
       <c r="K145" s="14"/>
       <c r="L145" s="14"/>
@@ -8727,15 +8771,9 @@
       <c r="Y145" s="14"/>
       <c r="Z145" s="14"/>
       <c r="AA145" s="14"/>
-      <c r="AB145" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC145" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD145" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB145" s="14"/>
+      <c r="AC145" s="14"/>
+      <c r="AD145" s="14"/>
       <c r="AE145" s="27"/>
       <c r="AF145" s="14"/>
       <c r="AG145" s="14"/>
@@ -8743,8 +8781,8 @@
       <c r="AI145" s="14"/>
     </row>
     <row r="146" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A146" s="14" t="s">
-        <v>492</v>
+      <c r="A146" s="15" t="s">
+        <v>528</v>
       </c>
       <c r="B146" s="14" t="s">
         <v>174</v>
@@ -8753,13 +8791,17 @@
         <v>135</v>
       </c>
       <c r="D146" s="18" t="s">
-        <v>493</v>
-      </c>
-      <c r="E146" s="14"/>
-      <c r="F146" s="14"/>
+        <v>527</v>
+      </c>
+      <c r="E146" s="15"/>
+      <c r="F146" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
-      <c r="I146" s="14"/>
+      <c r="I146" s="14" t="s">
+        <v>126</v>
+      </c>
       <c r="J146" s="14"/>
       <c r="K146" s="14"/>
       <c r="L146" s="14"/>
@@ -8778,36 +8820,20 @@
       <c r="Y146" s="14"/>
       <c r="Z146" s="14"/>
       <c r="AA146" s="14"/>
-      <c r="AB146" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC146" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD146" s="14" t="s">
-        <v>451</v>
-      </c>
+      <c r="AB146" s="14"/>
+      <c r="AC146" s="14"/>
+      <c r="AD146" s="14"/>
       <c r="AE146" s="27"/>
       <c r="AF146" s="14"/>
       <c r="AG146" s="14"/>
-      <c r="AH146" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH146" s="14"/>
       <c r="AI146" s="14"/>
     </row>
     <row r="147" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="14" t="s">
-        <v>490</v>
-      </c>
-      <c r="B147" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C147" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D147" s="18" t="s">
-        <v>491</v>
-      </c>
+      <c r="A147" s="14"/>
+      <c r="B147" s="14"/>
+      <c r="C147" s="14"/>
+      <c r="D147" s="15"/>
       <c r="E147" s="14"/>
       <c r="F147" s="14"/>
       <c r="G147" s="14"/>
@@ -8820,16 +8846,10 @@
       <c r="N147" s="14"/>
       <c r="O147" s="14"/>
       <c r="P147" s="14"/>
-      <c r="Q147" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="R147" s="14"/>
-      <c r="S147" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T147" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="Q147" s="14"/>
+      <c r="R147" s="15"/>
+      <c r="S147" s="14"/>
+      <c r="T147" s="14"/>
       <c r="U147" s="14"/>
       <c r="V147" s="14"/>
       <c r="W147" s="14"/>
@@ -8837,28 +8857,28 @@
       <c r="Y147" s="14"/>
       <c r="Z147" s="14"/>
       <c r="AA147" s="14"/>
-      <c r="AB147" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC147" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD147" s="14" t="s">
-        <v>451</v>
-      </c>
+      <c r="AB147" s="14"/>
+      <c r="AC147" s="14"/>
+      <c r="AD147" s="14"/>
       <c r="AE147" s="27"/>
       <c r="AF147" s="14"/>
       <c r="AG147" s="14"/>
-      <c r="AH147" s="15" t="s">
-        <v>454</v>
-      </c>
+      <c r="AH147" s="14"/>
       <c r="AI147" s="14"/>
     </row>
     <row r="148" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A148" s="14"/>
-      <c r="B148" s="14"/>
-      <c r="C148" s="14"/>
-      <c r="D148" s="15"/>
+      <c r="A148" s="14" t="s">
+        <v>488</v>
+      </c>
+      <c r="B148" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C148" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D148" s="18" t="s">
+        <v>489</v>
+      </c>
       <c r="E148" s="14"/>
       <c r="F148" s="14"/>
       <c r="G148" s="14"/>
@@ -8871,10 +8891,16 @@
       <c r="N148" s="14"/>
       <c r="O148" s="14"/>
       <c r="P148" s="14"/>
-      <c r="Q148" s="14"/>
-      <c r="R148" s="15"/>
-      <c r="S148" s="14"/>
-      <c r="T148" s="14"/>
+      <c r="Q148" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="R148" s="14"/>
+      <c r="S148" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T148" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U148" s="14"/>
       <c r="V148" s="14"/>
       <c r="W148" s="14"/>
@@ -8882,18 +8908,26 @@
       <c r="Y148" s="14"/>
       <c r="Z148" s="14"/>
       <c r="AA148" s="14"/>
-      <c r="AB148" s="14"/>
-      <c r="AC148" s="14"/>
-      <c r="AD148" s="14"/>
+      <c r="AB148" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC148" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD148" s="14" t="s">
+        <v>393</v>
+      </c>
       <c r="AE148" s="27"/>
       <c r="AF148" s="14"/>
       <c r="AG148" s="14"/>
-      <c r="AH148" s="14"/>
+      <c r="AH148" s="14" t="s">
+        <v>465</v>
+      </c>
       <c r="AI148" s="14"/>
     </row>
     <row r="149" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="14" t="s">
-        <v>267</v>
+        <v>486</v>
       </c>
       <c r="B149" s="14" t="s">
         <v>174</v>
@@ -8901,21 +8935,17 @@
       <c r="C149" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D149" s="14"/>
+      <c r="D149" s="18" t="s">
+        <v>487</v>
+      </c>
       <c r="E149" s="14"/>
       <c r="F149" s="14"/>
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="14"/>
-      <c r="J149" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K149" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L149" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J149" s="14"/>
+      <c r="K149" s="14"/>
+      <c r="L149" s="14"/>
       <c r="M149" s="14"/>
       <c r="N149" s="14"/>
       <c r="O149" s="14"/>
@@ -8931,9 +8961,15 @@
       <c r="Y149" s="14"/>
       <c r="Z149" s="14"/>
       <c r="AA149" s="14"/>
-      <c r="AB149" s="14"/>
-      <c r="AC149" s="14"/>
-      <c r="AD149" s="14"/>
+      <c r="AB149" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC149" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD149" s="14" t="s">
+        <v>393</v>
+      </c>
       <c r="AE149" s="27"/>
       <c r="AF149" s="14"/>
       <c r="AG149" s="14"/>
@@ -8942,7 +8978,7 @@
     </row>
     <row r="150" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="14" t="s">
-        <v>268</v>
+        <v>492</v>
       </c>
       <c r="B150" s="14" t="s">
         <v>174</v>
@@ -8950,21 +8986,17 @@
       <c r="C150" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D150" s="14"/>
+      <c r="D150" s="18" t="s">
+        <v>493</v>
+      </c>
       <c r="E150" s="14"/>
       <c r="F150" s="14"/>
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="14"/>
-      <c r="J150" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K150" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L150" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="J150" s="14"/>
+      <c r="K150" s="14"/>
+      <c r="L150" s="14"/>
       <c r="M150" s="14"/>
       <c r="N150" s="14"/>
       <c r="O150" s="14"/>
@@ -8980,18 +9012,26 @@
       <c r="Y150" s="14"/>
       <c r="Z150" s="14"/>
       <c r="AA150" s="14"/>
-      <c r="AB150" s="14"/>
-      <c r="AC150" s="14"/>
-      <c r="AD150" s="14"/>
+      <c r="AB150" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC150" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD150" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE150" s="27"/>
       <c r="AF150" s="14"/>
       <c r="AG150" s="14"/>
-      <c r="AH150" s="14"/>
+      <c r="AH150" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI150" s="14"/>
     </row>
-    <row r="151" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="14" t="s">
-        <v>359</v>
+        <v>490</v>
       </c>
       <c r="B151" s="14" t="s">
         <v>174</v>
@@ -8999,31 +9039,83 @@
       <c r="C151" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O151" s="15" t="s">
-        <v>362</v>
-      </c>
-      <c r="AB151" s="14"/>
-      <c r="AC151" s="14"/>
-      <c r="AD151" s="14"/>
+      <c r="D151" s="18" t="s">
+        <v>491</v>
+      </c>
+      <c r="E151" s="14"/>
+      <c r="F151" s="14"/>
+      <c r="G151" s="14"/>
+      <c r="H151" s="14"/>
+      <c r="I151" s="14"/>
+      <c r="J151" s="14"/>
+      <c r="K151" s="14"/>
+      <c r="L151" s="14"/>
+      <c r="M151" s="14"/>
+      <c r="N151" s="14"/>
+      <c r="O151" s="14"/>
+      <c r="P151" s="14"/>
+      <c r="Q151" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="R151" s="14"/>
+      <c r="S151" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T151" s="14" t="s">
+        <v>300</v>
+      </c>
+      <c r="U151" s="14"/>
+      <c r="V151" s="14"/>
+      <c r="W151" s="14"/>
+      <c r="X151" s="14"/>
+      <c r="Y151" s="14"/>
+      <c r="Z151" s="14"/>
+      <c r="AA151" s="14"/>
+      <c r="AB151" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC151" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD151" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE151" s="27"/>
       <c r="AF151" s="14"/>
       <c r="AG151" s="14"/>
-      <c r="AH151" s="14"/>
+      <c r="AH151" s="15" t="s">
+        <v>454</v>
+      </c>
       <c r="AI151" s="14"/>
     </row>
-    <row r="152" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A152" s="14" t="s">
-        <v>360</v>
-      </c>
-      <c r="B152" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C152" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O152" s="15" t="s">
-        <v>363</v>
-      </c>
+    <row r="152" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="14"/>
+      <c r="B152" s="14"/>
+      <c r="C152" s="14"/>
+      <c r="D152" s="15"/>
+      <c r="E152" s="14"/>
+      <c r="F152" s="14"/>
+      <c r="G152" s="14"/>
+      <c r="H152" s="14"/>
+      <c r="I152" s="14"/>
+      <c r="J152" s="14"/>
+      <c r="K152" s="14"/>
+      <c r="L152" s="14"/>
+      <c r="M152" s="14"/>
+      <c r="N152" s="14"/>
+      <c r="O152" s="14"/>
+      <c r="P152" s="14"/>
+      <c r="Q152" s="14"/>
+      <c r="R152" s="15"/>
+      <c r="S152" s="14"/>
+      <c r="T152" s="14"/>
+      <c r="U152" s="14"/>
+      <c r="V152" s="14"/>
+      <c r="W152" s="14"/>
+      <c r="X152" s="14"/>
+      <c r="Y152" s="14"/>
+      <c r="Z152" s="14"/>
+      <c r="AA152" s="14"/>
       <c r="AB152" s="14"/>
       <c r="AC152" s="14"/>
       <c r="AD152" s="14"/>
@@ -9033,9 +9125,9 @@
       <c r="AH152" s="14"/>
       <c r="AI152" s="14"/>
     </row>
-    <row r="153" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="14" t="s">
-        <v>361</v>
+        <v>267</v>
       </c>
       <c r="B153" s="14" t="s">
         <v>174</v>
@@ -9043,9 +9135,36 @@
       <c r="C153" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O153" s="15" t="s">
-        <v>364</v>
-      </c>
+      <c r="D153" s="14"/>
+      <c r="E153" s="14"/>
+      <c r="F153" s="14"/>
+      <c r="G153" s="14"/>
+      <c r="H153" s="14"/>
+      <c r="I153" s="14"/>
+      <c r="J153" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K153" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L153" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M153" s="14"/>
+      <c r="N153" s="14"/>
+      <c r="O153" s="14"/>
+      <c r="P153" s="14"/>
+      <c r="Q153" s="14"/>
+      <c r="R153" s="14"/>
+      <c r="S153" s="14"/>
+      <c r="T153" s="14"/>
+      <c r="U153" s="14"/>
+      <c r="V153" s="14"/>
+      <c r="W153" s="14"/>
+      <c r="X153" s="14"/>
+      <c r="Y153" s="14"/>
+      <c r="Z153" s="14"/>
+      <c r="AA153" s="14"/>
       <c r="AB153" s="14"/>
       <c r="AC153" s="14"/>
       <c r="AD153" s="14"/>
@@ -9055,9 +9174,9 @@
       <c r="AH153" s="14"/>
       <c r="AI153" s="14"/>
     </row>
-    <row r="154" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="14" t="s">
-        <v>370</v>
+        <v>268</v>
       </c>
       <c r="B154" s="14" t="s">
         <v>174</v>
@@ -9065,9 +9184,36 @@
       <c r="C154" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M154" s="14" t="s">
-        <v>371</v>
-      </c>
+      <c r="D154" s="14"/>
+      <c r="E154" s="14"/>
+      <c r="F154" s="14"/>
+      <c r="G154" s="14"/>
+      <c r="H154" s="14"/>
+      <c r="I154" s="14"/>
+      <c r="J154" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K154" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L154" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M154" s="14"/>
+      <c r="N154" s="14"/>
+      <c r="O154" s="14"/>
+      <c r="P154" s="14"/>
+      <c r="Q154" s="14"/>
+      <c r="R154" s="14"/>
+      <c r="S154" s="14"/>
+      <c r="T154" s="14"/>
+      <c r="U154" s="14"/>
+      <c r="V154" s="14"/>
+      <c r="W154" s="14"/>
+      <c r="X154" s="14"/>
+      <c r="Y154" s="14"/>
+      <c r="Z154" s="14"/>
+      <c r="AA154" s="14"/>
       <c r="AB154" s="14"/>
       <c r="AC154" s="14"/>
       <c r="AD154" s="14"/>
@@ -9078,6 +9224,18 @@
       <c r="AI154" s="14"/>
     </row>
     <row r="155" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A155" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="B155" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C155" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O155" s="15" t="s">
+        <v>362</v>
+      </c>
       <c r="AB155" s="14"/>
       <c r="AC155" s="14"/>
       <c r="AD155" s="14"/>
@@ -9088,6 +9246,18 @@
       <c r="AI155" s="14"/>
     </row>
     <row r="156" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A156" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B156" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C156" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O156" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB156" s="14"/>
       <c r="AC156" s="14"/>
       <c r="AD156" s="14"/>
@@ -9098,6 +9268,18 @@
       <c r="AI156" s="14"/>
     </row>
     <row r="157" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A157" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B157" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C157" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O157" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB157" s="14"/>
       <c r="AC157" s="14"/>
       <c r="AD157" s="14"/>
@@ -9108,6 +9290,18 @@
       <c r="AI157" s="14"/>
     </row>
     <row r="158" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A158" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B158" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C158" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M158" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB158" s="14"/>
       <c r="AC158" s="14"/>
       <c r="AD158" s="14"/>
@@ -9127,7 +9321,42 @@
       <c r="AH159" s="14"/>
       <c r="AI159" s="14"/>
     </row>
-    <row r="160" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="B160" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C160" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D160" s="18" t="s">
+        <v>530</v>
+      </c>
+      <c r="E160" s="15"/>
+      <c r="F160" s="14"/>
+      <c r="G160" s="14"/>
+      <c r="H160" s="14"/>
+      <c r="I160" s="14"/>
+      <c r="J160" s="14"/>
+      <c r="K160" s="14"/>
+      <c r="L160" s="14"/>
+      <c r="M160" s="14"/>
+      <c r="N160" s="14"/>
+      <c r="O160" s="14"/>
+      <c r="P160" s="14"/>
+      <c r="Q160" s="14"/>
+      <c r="R160" s="14"/>
+      <c r="S160" s="14"/>
+      <c r="T160" s="14"/>
+      <c r="U160" s="14"/>
+      <c r="V160" s="14"/>
+      <c r="W160" s="14"/>
+      <c r="X160" s="14"/>
+      <c r="Y160" s="14"/>
+      <c r="Z160" s="14"/>
+      <c r="AA160" s="14"/>
       <c r="AB160" s="14"/>
       <c r="AC160" s="14"/>
       <c r="AD160" s="14"/>
@@ -11111,7 +11340,7 @@
       <c r="AB358" s="14"/>
       <c r="AC358" s="14"/>
       <c r="AD358" s="14"/>
-      <c r="AE358" s="14"/>
+      <c r="AE358" s="27"/>
       <c r="AF358" s="14"/>
       <c r="AG358" s="14"/>
       <c r="AH358" s="14"/>
@@ -11121,7 +11350,7 @@
       <c r="AB359" s="14"/>
       <c r="AC359" s="14"/>
       <c r="AD359" s="14"/>
-      <c r="AE359" s="14"/>
+      <c r="AE359" s="27"/>
       <c r="AF359" s="14"/>
       <c r="AG359" s="14"/>
       <c r="AH359" s="14"/>
@@ -11131,7 +11360,7 @@
       <c r="AB360" s="14"/>
       <c r="AC360" s="14"/>
       <c r="AD360" s="14"/>
-      <c r="AE360" s="14"/>
+      <c r="AE360" s="27"/>
       <c r="AF360" s="14"/>
       <c r="AG360" s="14"/>
       <c r="AH360" s="14"/>
@@ -11141,7 +11370,7 @@
       <c r="AB361" s="14"/>
       <c r="AC361" s="14"/>
       <c r="AD361" s="14"/>
-      <c r="AE361" s="14"/>
+      <c r="AE361" s="27"/>
       <c r="AF361" s="14"/>
       <c r="AG361" s="14"/>
       <c r="AH361" s="14"/>
@@ -11177,6 +11406,46 @@
       <c r="AH364" s="14"/>
       <c r="AI364" s="14"/>
     </row>
+    <row r="365" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB365" s="14"/>
+      <c r="AC365" s="14"/>
+      <c r="AD365" s="14"/>
+      <c r="AE365" s="14"/>
+      <c r="AF365" s="14"/>
+      <c r="AG365" s="14"/>
+      <c r="AH365" s="14"/>
+      <c r="AI365" s="14"/>
+    </row>
+    <row r="366" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB366" s="14"/>
+      <c r="AC366" s="14"/>
+      <c r="AD366" s="14"/>
+      <c r="AE366" s="14"/>
+      <c r="AF366" s="14"/>
+      <c r="AG366" s="14"/>
+      <c r="AH366" s="14"/>
+      <c r="AI366" s="14"/>
+    </row>
+    <row r="367" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB367" s="14"/>
+      <c r="AC367" s="14"/>
+      <c r="AD367" s="14"/>
+      <c r="AE367" s="14"/>
+      <c r="AF367" s="14"/>
+      <c r="AG367" s="14"/>
+      <c r="AH367" s="14"/>
+      <c r="AI367" s="14"/>
+    </row>
+    <row r="368" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB368" s="14"/>
+      <c r="AC368" s="14"/>
+      <c r="AD368" s="14"/>
+      <c r="AE368" s="14"/>
+      <c r="AF368" s="14"/>
+      <c r="AG368" s="14"/>
+      <c r="AH368" s="14"/>
+      <c r="AI368" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11186,7 +11455,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T142"/>
+  <dimension ref="A1:T148"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -15666,6 +15935,228 @@
       <c r="S142" s="14"/>
       <c r="T142" s="14"/>
     </row>
+    <row r="143" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A143" s="15" t="s">
+        <v>520</v>
+      </c>
+      <c r="B143" s="18" t="s">
+        <v>496</v>
+      </c>
+      <c r="C143" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="D143" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E143" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="F143" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="G143" s="15"/>
+      <c r="H143" s="15"/>
+      <c r="I143" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J143" s="14"/>
+      <c r="K143" s="14"/>
+      <c r="L143" s="14"/>
+      <c r="M143" s="14"/>
+      <c r="N143" s="14"/>
+      <c r="O143" s="14"/>
+      <c r="P143" s="14"/>
+      <c r="Q143" s="14"/>
+      <c r="R143" s="14"/>
+      <c r="S143" s="14"/>
+      <c r="T143" s="14"/>
+    </row>
+    <row r="144" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A144" s="16" t="s">
+        <v>522</v>
+      </c>
+      <c r="B144" s="18" t="s">
+        <v>494</v>
+      </c>
+      <c r="C144" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="D144" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E144" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="F144" s="14"/>
+      <c r="G144" s="15"/>
+      <c r="H144" s="15"/>
+      <c r="I144" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J144" s="14"/>
+      <c r="K144" s="14"/>
+      <c r="L144" s="14"/>
+      <c r="M144" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="N144" s="14" t="s">
+        <v>402</v>
+      </c>
+      <c r="O144" s="14"/>
+      <c r="P144" s="14"/>
+      <c r="Q144" s="14"/>
+      <c r="R144" s="14"/>
+      <c r="S144" s="14"/>
+      <c r="T144" s="14"/>
+    </row>
+    <row r="145" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="15" t="s">
+        <v>524</v>
+      </c>
+      <c r="B145" s="18" t="s">
+        <v>496</v>
+      </c>
+      <c r="C145" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D145" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E145" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F145" s="15"/>
+      <c r="G145" s="15"/>
+      <c r="H145" s="15"/>
+      <c r="I145" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J145" s="14" t="s">
+        <v>399</v>
+      </c>
+      <c r="K145" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L145" s="14" t="s">
+        <v>399</v>
+      </c>
+      <c r="M145" s="14"/>
+      <c r="N145" s="14"/>
+      <c r="O145" s="14"/>
+      <c r="P145" s="14"/>
+      <c r="Q145" s="14"/>
+      <c r="R145" s="14"/>
+      <c r="S145" s="14"/>
+      <c r="T145" s="14"/>
+    </row>
+    <row r="146" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A146" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B146" s="18" t="s">
+        <v>496</v>
+      </c>
+      <c r="C146" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D146" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E146" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F146" s="15"/>
+      <c r="G146" s="15"/>
+      <c r="H146" s="15"/>
+      <c r="I146" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J146" s="14" t="s">
+        <v>399</v>
+      </c>
+      <c r="K146" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L146" s="14" t="s">
+        <v>399</v>
+      </c>
+      <c r="M146" s="14"/>
+      <c r="N146" s="14"/>
+      <c r="O146" s="14"/>
+      <c r="P146" s="14"/>
+      <c r="Q146" s="14"/>
+      <c r="R146" s="14"/>
+      <c r="S146" s="14"/>
+      <c r="T146" s="14"/>
+    </row>
+    <row r="147" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A147" s="15" t="s">
+        <v>527</v>
+      </c>
+      <c r="B147" s="18" t="s">
+        <v>494</v>
+      </c>
+      <c r="C147" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D147" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E147" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="F147" s="15"/>
+      <c r="G147" s="15"/>
+      <c r="H147" s="15"/>
+      <c r="I147" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J147" s="14"/>
+      <c r="K147" s="14"/>
+      <c r="L147" s="14"/>
+      <c r="M147" s="14"/>
+      <c r="N147" s="14"/>
+      <c r="O147" s="14"/>
+      <c r="P147" s="14"/>
+      <c r="Q147" s="14"/>
+      <c r="R147" s="14"/>
+      <c r="S147" s="14"/>
+      <c r="T147" s="14"/>
+    </row>
+    <row r="148" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A148" s="15" t="s">
+        <v>530</v>
+      </c>
+      <c r="B148" s="30" t="s">
+        <v>494</v>
+      </c>
+      <c r="C148" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D148" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E148" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="F148" s="15"/>
+      <c r="G148" s="15"/>
+      <c r="H148" s="15"/>
+      <c r="I148" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J148" s="14"/>
+      <c r="K148" s="14"/>
+      <c r="L148" s="14"/>
+      <c r="M148" s="14"/>
+      <c r="N148" s="14"/>
+      <c r="O148" s="14"/>
+      <c r="P148" s="14"/>
+      <c r="Q148" s="14"/>
+      <c r="R148" s="14"/>
+      <c r="S148" s="14"/>
+      <c r="T148" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Commit the code for NVI scenarios added for Parcel Order
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{032F975C-1675-4777-8CD1-3424980F6CB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{968CFE7E-969C-4F0F-965D-6946990424BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2157" uniqueCount="531">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2204" uniqueCount="541">
   <si>
     <t>1</t>
   </si>
@@ -1621,6 +1621,36 @@
   </si>
   <si>
     <t>933</t>
+  </si>
+  <si>
+    <t>934</t>
+  </si>
+  <si>
+    <t>151-10343-001</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario035</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario036</t>
+  </si>
+  <si>
+    <t>935|936</t>
+  </si>
+  <si>
+    <t>935</t>
+  </si>
+  <si>
+    <t>936</t>
+  </si>
+  <si>
+    <t>000-15593-001</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario005</t>
+  </si>
+  <si>
+    <t>937</t>
   </si>
 </sst>
 </file>
@@ -2153,7 +2183,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI368"/>
+  <dimension ref="A1:AI371"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -8830,12 +8860,22 @@
       <c r="AI146" s="14"/>
     </row>
     <row r="147" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="14"/>
-      <c r="B147" s="14"/>
-      <c r="C147" s="14"/>
-      <c r="D147" s="15"/>
+      <c r="A147" s="14" t="s">
+        <v>533</v>
+      </c>
+      <c r="B147" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C147" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D147" s="15" t="s">
+        <v>531</v>
+      </c>
       <c r="E147" s="14"/>
-      <c r="F147" s="14"/>
+      <c r="F147" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="14"/>
@@ -8847,7 +8887,9 @@
       <c r="O147" s="14"/>
       <c r="P147" s="14"/>
       <c r="Q147" s="14"/>
-      <c r="R147" s="15"/>
+      <c r="R147" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S147" s="14"/>
       <c r="T147" s="14"/>
       <c r="U147" s="14"/>
@@ -8867,8 +8909,8 @@
       <c r="AI147" s="14"/>
     </row>
     <row r="148" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A148" s="14" t="s">
-        <v>488</v>
+      <c r="A148" s="15" t="s">
+        <v>534</v>
       </c>
       <c r="B148" s="14" t="s">
         <v>174</v>
@@ -8877,13 +8919,17 @@
         <v>135</v>
       </c>
       <c r="D148" s="18" t="s">
-        <v>489</v>
-      </c>
-      <c r="E148" s="14"/>
-      <c r="F148" s="14"/>
-      <c r="G148" s="14"/>
+        <v>535</v>
+      </c>
+      <c r="E148" s="15"/>
+      <c r="F148" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="G148" s="15"/>
       <c r="H148" s="14"/>
-      <c r="I148" s="14"/>
+      <c r="I148" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J148" s="14"/>
       <c r="K148" s="14"/>
       <c r="L148" s="14"/>
@@ -8891,16 +8937,10 @@
       <c r="N148" s="14"/>
       <c r="O148" s="14"/>
       <c r="P148" s="14"/>
-      <c r="Q148" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q148" s="14"/>
       <c r="R148" s="14"/>
-      <c r="S148" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T148" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S148" s="14"/>
+      <c r="T148" s="14"/>
       <c r="U148" s="14"/>
       <c r="V148" s="14"/>
       <c r="W148" s="14"/>
@@ -8908,36 +8948,20 @@
       <c r="Y148" s="14"/>
       <c r="Z148" s="14"/>
       <c r="AA148" s="14"/>
-      <c r="AB148" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC148" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD148" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB148" s="14"/>
+      <c r="AC148" s="14"/>
+      <c r="AD148" s="14"/>
       <c r="AE148" s="27"/>
       <c r="AF148" s="14"/>
       <c r="AG148" s="14"/>
-      <c r="AH148" s="14" t="s">
-        <v>465</v>
-      </c>
+      <c r="AH148" s="14"/>
       <c r="AI148" s="14"/>
     </row>
     <row r="149" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A149" s="14" t="s">
-        <v>486</v>
-      </c>
-      <c r="B149" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C149" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D149" s="18" t="s">
-        <v>487</v>
-      </c>
+      <c r="A149" s="14"/>
+      <c r="B149" s="14"/>
+      <c r="C149" s="14"/>
+      <c r="D149" s="15"/>
       <c r="E149" s="14"/>
       <c r="F149" s="14"/>
       <c r="G149" s="14"/>
@@ -8951,7 +8975,7 @@
       <c r="O149" s="14"/>
       <c r="P149" s="14"/>
       <c r="Q149" s="14"/>
-      <c r="R149" s="14"/>
+      <c r="R149" s="15"/>
       <c r="S149" s="14"/>
       <c r="T149" s="14"/>
       <c r="U149" s="14"/>
@@ -8961,15 +8985,9 @@
       <c r="Y149" s="14"/>
       <c r="Z149" s="14"/>
       <c r="AA149" s="14"/>
-      <c r="AB149" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC149" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD149" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB149" s="14"/>
+      <c r="AC149" s="14"/>
+      <c r="AD149" s="14"/>
       <c r="AE149" s="27"/>
       <c r="AF149" s="14"/>
       <c r="AG149" s="14"/>
@@ -8978,7 +8996,7 @@
     </row>
     <row r="150" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="14" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="B150" s="14" t="s">
         <v>174</v>
@@ -8987,7 +9005,7 @@
         <v>135</v>
       </c>
       <c r="D150" s="18" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="E150" s="14"/>
       <c r="F150" s="14"/>
@@ -9001,10 +9019,16 @@
       <c r="N150" s="14"/>
       <c r="O150" s="14"/>
       <c r="P150" s="14"/>
-      <c r="Q150" s="14"/>
+      <c r="Q150" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R150" s="14"/>
-      <c r="S150" s="14"/>
-      <c r="T150" s="14"/>
+      <c r="S150" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T150" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U150" s="14"/>
       <c r="V150" s="14"/>
       <c r="W150" s="14"/>
@@ -9013,25 +9037,25 @@
       <c r="Z150" s="14"/>
       <c r="AA150" s="14"/>
       <c r="AB150" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC150" s="14" t="s">
-        <v>457</v>
+        <v>393</v>
       </c>
       <c r="AD150" s="14" t="s">
-        <v>451</v>
+        <v>393</v>
       </c>
       <c r="AE150" s="27"/>
       <c r="AF150" s="14"/>
       <c r="AG150" s="14"/>
       <c r="AH150" s="14" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="AI150" s="14"/>
     </row>
     <row r="151" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="14" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="B151" s="14" t="s">
         <v>174</v>
@@ -9040,7 +9064,7 @@
         <v>135</v>
       </c>
       <c r="D151" s="18" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="E151" s="14"/>
       <c r="F151" s="14"/>
@@ -9054,16 +9078,10 @@
       <c r="N151" s="14"/>
       <c r="O151" s="14"/>
       <c r="P151" s="14"/>
-      <c r="Q151" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q151" s="14"/>
       <c r="R151" s="14"/>
-      <c r="S151" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T151" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S151" s="14"/>
+      <c r="T151" s="14"/>
       <c r="U151" s="14"/>
       <c r="V151" s="14"/>
       <c r="W151" s="14"/>
@@ -9072,27 +9090,33 @@
       <c r="Z151" s="14"/>
       <c r="AA151" s="14"/>
       <c r="AB151" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC151" s="14" t="s">
-        <v>457</v>
+        <v>393</v>
       </c>
       <c r="AD151" s="14" t="s">
-        <v>451</v>
+        <v>393</v>
       </c>
       <c r="AE151" s="27"/>
       <c r="AF151" s="14"/>
       <c r="AG151" s="14"/>
-      <c r="AH151" s="15" t="s">
-        <v>454</v>
-      </c>
+      <c r="AH151" s="14"/>
       <c r="AI151" s="14"/>
     </row>
     <row r="152" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="14"/>
-      <c r="B152" s="14"/>
-      <c r="C152" s="14"/>
-      <c r="D152" s="15"/>
+      <c r="A152" s="14" t="s">
+        <v>492</v>
+      </c>
+      <c r="B152" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C152" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D152" s="18" t="s">
+        <v>493</v>
+      </c>
       <c r="E152" s="14"/>
       <c r="F152" s="14"/>
       <c r="G152" s="14"/>
@@ -9106,7 +9130,7 @@
       <c r="O152" s="14"/>
       <c r="P152" s="14"/>
       <c r="Q152" s="14"/>
-      <c r="R152" s="15"/>
+      <c r="R152" s="14"/>
       <c r="S152" s="14"/>
       <c r="T152" s="14"/>
       <c r="U152" s="14"/>
@@ -9116,18 +9140,26 @@
       <c r="Y152" s="14"/>
       <c r="Z152" s="14"/>
       <c r="AA152" s="14"/>
-      <c r="AB152" s="14"/>
-      <c r="AC152" s="14"/>
-      <c r="AD152" s="14"/>
+      <c r="AB152" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC152" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD152" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE152" s="27"/>
       <c r="AF152" s="14"/>
       <c r="AG152" s="14"/>
-      <c r="AH152" s="14"/>
+      <c r="AH152" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI152" s="14"/>
     </row>
     <row r="153" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="14" t="s">
-        <v>267</v>
+        <v>490</v>
       </c>
       <c r="B153" s="14" t="s">
         <v>174</v>
@@ -9135,29 +9167,31 @@
       <c r="C153" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D153" s="14"/>
+      <c r="D153" s="18" t="s">
+        <v>491</v>
+      </c>
       <c r="E153" s="14"/>
       <c r="F153" s="14"/>
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
       <c r="I153" s="14"/>
-      <c r="J153" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K153" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L153" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J153" s="14"/>
+      <c r="K153" s="14"/>
+      <c r="L153" s="14"/>
       <c r="M153" s="14"/>
       <c r="N153" s="14"/>
       <c r="O153" s="14"/>
       <c r="P153" s="14"/>
-      <c r="Q153" s="14"/>
+      <c r="Q153" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R153" s="14"/>
-      <c r="S153" s="14"/>
-      <c r="T153" s="14"/>
+      <c r="S153" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T153" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U153" s="14"/>
       <c r="V153" s="14"/>
       <c r="W153" s="14"/>
@@ -9165,18 +9199,26 @@
       <c r="Y153" s="14"/>
       <c r="Z153" s="14"/>
       <c r="AA153" s="14"/>
-      <c r="AB153" s="14"/>
-      <c r="AC153" s="14"/>
-      <c r="AD153" s="14"/>
+      <c r="AB153" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC153" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD153" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE153" s="27"/>
       <c r="AF153" s="14"/>
       <c r="AG153" s="14"/>
-      <c r="AH153" s="14"/>
+      <c r="AH153" s="15" t="s">
+        <v>454</v>
+      </c>
       <c r="AI153" s="14"/>
     </row>
     <row r="154" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="14" t="s">
-        <v>268</v>
+        <v>539</v>
       </c>
       <c r="B154" s="14" t="s">
         <v>174</v>
@@ -9184,22 +9226,20 @@
       <c r="C154" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D154" s="14"/>
+      <c r="D154" s="23" t="s">
+        <v>540</v>
+      </c>
       <c r="E154" s="14"/>
       <c r="F154" s="14"/>
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="14"/>
-      <c r="J154" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K154" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L154" s="15" t="s">
-        <v>276</v>
-      </c>
-      <c r="M154" s="14"/>
+      <c r="J154" s="14"/>
+      <c r="K154" s="14"/>
+      <c r="L154" s="14"/>
+      <c r="M154" s="20" t="s">
+        <v>494</v>
+      </c>
       <c r="N154" s="14"/>
       <c r="O154" s="14"/>
       <c r="P154" s="14"/>
@@ -9214,28 +9254,51 @@
       <c r="Y154" s="14"/>
       <c r="Z154" s="14"/>
       <c r="AA154" s="14"/>
-      <c r="AB154" s="14"/>
-      <c r="AC154" s="14"/>
-      <c r="AD154" s="14"/>
+      <c r="AB154" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC154" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD154" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE154" s="27"/>
       <c r="AF154" s="14"/>
       <c r="AG154" s="14"/>
-      <c r="AH154" s="14"/>
+      <c r="AH154" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI154" s="14"/>
     </row>
-    <row r="155" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A155" s="14" t="s">
-        <v>359</v>
-      </c>
-      <c r="B155" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C155" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O155" s="15" t="s">
-        <v>362</v>
-      </c>
+    <row r="155" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="14"/>
+      <c r="B155" s="14"/>
+      <c r="C155" s="14"/>
+      <c r="D155" s="15"/>
+      <c r="E155" s="14"/>
+      <c r="F155" s="14"/>
+      <c r="G155" s="14"/>
+      <c r="H155" s="14"/>
+      <c r="I155" s="14"/>
+      <c r="J155" s="14"/>
+      <c r="K155" s="14"/>
+      <c r="L155" s="14"/>
+      <c r="M155" s="14"/>
+      <c r="N155" s="14"/>
+      <c r="O155" s="14"/>
+      <c r="P155" s="14"/>
+      <c r="Q155" s="14"/>
+      <c r="R155" s="15"/>
+      <c r="S155" s="14"/>
+      <c r="T155" s="14"/>
+      <c r="U155" s="14"/>
+      <c r="V155" s="14"/>
+      <c r="W155" s="14"/>
+      <c r="X155" s="14"/>
+      <c r="Y155" s="14"/>
+      <c r="Z155" s="14"/>
+      <c r="AA155" s="14"/>
       <c r="AB155" s="14"/>
       <c r="AC155" s="14"/>
       <c r="AD155" s="14"/>
@@ -9245,9 +9308,9 @@
       <c r="AH155" s="14"/>
       <c r="AI155" s="14"/>
     </row>
-    <row r="156" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="14" t="s">
-        <v>360</v>
+        <v>267</v>
       </c>
       <c r="B156" s="14" t="s">
         <v>174</v>
@@ -9255,9 +9318,36 @@
       <c r="C156" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O156" s="15" t="s">
-        <v>363</v>
-      </c>
+      <c r="D156" s="14"/>
+      <c r="E156" s="14"/>
+      <c r="F156" s="14"/>
+      <c r="G156" s="14"/>
+      <c r="H156" s="14"/>
+      <c r="I156" s="14"/>
+      <c r="J156" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K156" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L156" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M156" s="14"/>
+      <c r="N156" s="14"/>
+      <c r="O156" s="14"/>
+      <c r="P156" s="14"/>
+      <c r="Q156" s="14"/>
+      <c r="R156" s="14"/>
+      <c r="S156" s="14"/>
+      <c r="T156" s="14"/>
+      <c r="U156" s="14"/>
+      <c r="V156" s="14"/>
+      <c r="W156" s="14"/>
+      <c r="X156" s="14"/>
+      <c r="Y156" s="14"/>
+      <c r="Z156" s="14"/>
+      <c r="AA156" s="14"/>
       <c r="AB156" s="14"/>
       <c r="AC156" s="14"/>
       <c r="AD156" s="14"/>
@@ -9267,9 +9357,9 @@
       <c r="AH156" s="14"/>
       <c r="AI156" s="14"/>
     </row>
-    <row r="157" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="14" t="s">
-        <v>361</v>
+        <v>268</v>
       </c>
       <c r="B157" s="14" t="s">
         <v>174</v>
@@ -9277,9 +9367,36 @@
       <c r="C157" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O157" s="15" t="s">
-        <v>364</v>
-      </c>
+      <c r="D157" s="14"/>
+      <c r="E157" s="14"/>
+      <c r="F157" s="14"/>
+      <c r="G157" s="14"/>
+      <c r="H157" s="14"/>
+      <c r="I157" s="14"/>
+      <c r="J157" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K157" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L157" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M157" s="14"/>
+      <c r="N157" s="14"/>
+      <c r="O157" s="14"/>
+      <c r="P157" s="14"/>
+      <c r="Q157" s="14"/>
+      <c r="R157" s="14"/>
+      <c r="S157" s="14"/>
+      <c r="T157" s="14"/>
+      <c r="U157" s="14"/>
+      <c r="V157" s="14"/>
+      <c r="W157" s="14"/>
+      <c r="X157" s="14"/>
+      <c r="Y157" s="14"/>
+      <c r="Z157" s="14"/>
+      <c r="AA157" s="14"/>
       <c r="AB157" s="14"/>
       <c r="AC157" s="14"/>
       <c r="AD157" s="14"/>
@@ -9291,7 +9408,7 @@
     </row>
     <row r="158" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A158" s="14" t="s">
-        <v>370</v>
+        <v>359</v>
       </c>
       <c r="B158" s="14" t="s">
         <v>174</v>
@@ -9299,8 +9416,8 @@
       <c r="C158" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M158" s="14" t="s">
-        <v>371</v>
+      <c r="O158" s="15" t="s">
+        <v>362</v>
       </c>
       <c r="AB158" s="14"/>
       <c r="AC158" s="14"/>
@@ -9312,6 +9429,18 @@
       <c r="AI158" s="14"/>
     </row>
     <row r="159" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A159" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B159" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C159" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O159" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB159" s="14"/>
       <c r="AC159" s="14"/>
       <c r="AD159" s="14"/>
@@ -9321,9 +9450,9 @@
       <c r="AH159" s="14"/>
       <c r="AI159" s="14"/>
     </row>
-    <row r="160" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A160" s="14" t="s">
-        <v>529</v>
+        <v>361</v>
       </c>
       <c r="B160" s="14" t="s">
         <v>174</v>
@@ -9331,32 +9460,9 @@
       <c r="C160" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D160" s="18" t="s">
-        <v>530</v>
-      </c>
-      <c r="E160" s="15"/>
-      <c r="F160" s="14"/>
-      <c r="G160" s="14"/>
-      <c r="H160" s="14"/>
-      <c r="I160" s="14"/>
-      <c r="J160" s="14"/>
-      <c r="K160" s="14"/>
-      <c r="L160" s="14"/>
-      <c r="M160" s="14"/>
-      <c r="N160" s="14"/>
-      <c r="O160" s="14"/>
-      <c r="P160" s="14"/>
-      <c r="Q160" s="14"/>
-      <c r="R160" s="14"/>
-      <c r="S160" s="14"/>
-      <c r="T160" s="14"/>
-      <c r="U160" s="14"/>
-      <c r="V160" s="14"/>
-      <c r="W160" s="14"/>
-      <c r="X160" s="14"/>
-      <c r="Y160" s="14"/>
-      <c r="Z160" s="14"/>
-      <c r="AA160" s="14"/>
+      <c r="O160" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB160" s="14"/>
       <c r="AC160" s="14"/>
       <c r="AD160" s="14"/>
@@ -9366,7 +9472,19 @@
       <c r="AH160" s="14"/>
       <c r="AI160" s="14"/>
     </row>
-    <row r="161" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A161" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B161" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C161" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M161" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB161" s="14"/>
       <c r="AC161" s="14"/>
       <c r="AD161" s="14"/>
@@ -9376,7 +9494,7 @@
       <c r="AH161" s="14"/>
       <c r="AI161" s="14"/>
     </row>
-    <row r="162" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB162" s="14"/>
       <c r="AC162" s="14"/>
       <c r="AD162" s="14"/>
@@ -9386,7 +9504,42 @@
       <c r="AH162" s="14"/>
       <c r="AI162" s="14"/>
     </row>
-    <row r="163" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="B163" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C163" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D163" s="18" t="s">
+        <v>530</v>
+      </c>
+      <c r="E163" s="15"/>
+      <c r="F163" s="14"/>
+      <c r="G163" s="14"/>
+      <c r="H163" s="14"/>
+      <c r="I163" s="14"/>
+      <c r="J163" s="14"/>
+      <c r="K163" s="14"/>
+      <c r="L163" s="14"/>
+      <c r="M163" s="14"/>
+      <c r="N163" s="14"/>
+      <c r="O163" s="14"/>
+      <c r="P163" s="14"/>
+      <c r="Q163" s="14"/>
+      <c r="R163" s="14"/>
+      <c r="S163" s="14"/>
+      <c r="T163" s="14"/>
+      <c r="U163" s="14"/>
+      <c r="V163" s="14"/>
+      <c r="W163" s="14"/>
+      <c r="X163" s="14"/>
+      <c r="Y163" s="14"/>
+      <c r="Z163" s="14"/>
+      <c r="AA163" s="14"/>
       <c r="AB163" s="14"/>
       <c r="AC163" s="14"/>
       <c r="AD163" s="14"/>
@@ -9396,7 +9549,7 @@
       <c r="AH163" s="14"/>
       <c r="AI163" s="14"/>
     </row>
-    <row r="164" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB164" s="14"/>
       <c r="AC164" s="14"/>
       <c r="AD164" s="14"/>
@@ -9406,7 +9559,7 @@
       <c r="AH164" s="14"/>
       <c r="AI164" s="14"/>
     </row>
-    <row r="165" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB165" s="14"/>
       <c r="AC165" s="14"/>
       <c r="AD165" s="14"/>
@@ -9416,7 +9569,7 @@
       <c r="AH165" s="14"/>
       <c r="AI165" s="14"/>
     </row>
-    <row r="166" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB166" s="14"/>
       <c r="AC166" s="14"/>
       <c r="AD166" s="14"/>
@@ -9426,7 +9579,7 @@
       <c r="AH166" s="14"/>
       <c r="AI166" s="14"/>
     </row>
-    <row r="167" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB167" s="14"/>
       <c r="AC167" s="14"/>
       <c r="AD167" s="14"/>
@@ -9436,7 +9589,7 @@
       <c r="AH167" s="14"/>
       <c r="AI167" s="14"/>
     </row>
-    <row r="168" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB168" s="14"/>
       <c r="AC168" s="14"/>
       <c r="AD168" s="14"/>
@@ -9446,7 +9599,7 @@
       <c r="AH168" s="14"/>
       <c r="AI168" s="14"/>
     </row>
-    <row r="169" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB169" s="14"/>
       <c r="AC169" s="14"/>
       <c r="AD169" s="14"/>
@@ -9456,7 +9609,7 @@
       <c r="AH169" s="14"/>
       <c r="AI169" s="14"/>
     </row>
-    <row r="170" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB170" s="14"/>
       <c r="AC170" s="14"/>
       <c r="AD170" s="14"/>
@@ -9466,7 +9619,7 @@
       <c r="AH170" s="14"/>
       <c r="AI170" s="14"/>
     </row>
-    <row r="171" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB171" s="14"/>
       <c r="AC171" s="14"/>
       <c r="AD171" s="14"/>
@@ -9476,7 +9629,7 @@
       <c r="AH171" s="14"/>
       <c r="AI171" s="14"/>
     </row>
-    <row r="172" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB172" s="14"/>
       <c r="AC172" s="14"/>
       <c r="AD172" s="14"/>
@@ -9486,7 +9639,7 @@
       <c r="AH172" s="14"/>
       <c r="AI172" s="14"/>
     </row>
-    <row r="173" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB173" s="14"/>
       <c r="AC173" s="14"/>
       <c r="AD173" s="14"/>
@@ -9496,7 +9649,7 @@
       <c r="AH173" s="14"/>
       <c r="AI173" s="14"/>
     </row>
-    <row r="174" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB174" s="14"/>
       <c r="AC174" s="14"/>
       <c r="AD174" s="14"/>
@@ -9506,7 +9659,7 @@
       <c r="AH174" s="14"/>
       <c r="AI174" s="14"/>
     </row>
-    <row r="175" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB175" s="14"/>
       <c r="AC175" s="14"/>
       <c r="AD175" s="14"/>
@@ -9516,7 +9669,7 @@
       <c r="AH175" s="14"/>
       <c r="AI175" s="14"/>
     </row>
-    <row r="176" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB176" s="14"/>
       <c r="AC176" s="14"/>
       <c r="AD176" s="14"/>
@@ -11380,7 +11533,7 @@
       <c r="AB362" s="14"/>
       <c r="AC362" s="14"/>
       <c r="AD362" s="14"/>
-      <c r="AE362" s="14"/>
+      <c r="AE362" s="27"/>
       <c r="AF362" s="14"/>
       <c r="AG362" s="14"/>
       <c r="AH362" s="14"/>
@@ -11390,7 +11543,7 @@
       <c r="AB363" s="14"/>
       <c r="AC363" s="14"/>
       <c r="AD363" s="14"/>
-      <c r="AE363" s="14"/>
+      <c r="AE363" s="27"/>
       <c r="AF363" s="14"/>
       <c r="AG363" s="14"/>
       <c r="AH363" s="14"/>
@@ -11400,7 +11553,7 @@
       <c r="AB364" s="14"/>
       <c r="AC364" s="14"/>
       <c r="AD364" s="14"/>
-      <c r="AE364" s="14"/>
+      <c r="AE364" s="27"/>
       <c r="AF364" s="14"/>
       <c r="AG364" s="14"/>
       <c r="AH364" s="14"/>
@@ -11446,6 +11599,36 @@
       <c r="AH368" s="14"/>
       <c r="AI368" s="14"/>
     </row>
+    <row r="369" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB369" s="14"/>
+      <c r="AC369" s="14"/>
+      <c r="AD369" s="14"/>
+      <c r="AE369" s="14"/>
+      <c r="AF369" s="14"/>
+      <c r="AG369" s="14"/>
+      <c r="AH369" s="14"/>
+      <c r="AI369" s="14"/>
+    </row>
+    <row r="370" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB370" s="14"/>
+      <c r="AC370" s="14"/>
+      <c r="AD370" s="14"/>
+      <c r="AE370" s="14"/>
+      <c r="AF370" s="14"/>
+      <c r="AG370" s="14"/>
+      <c r="AH370" s="14"/>
+      <c r="AI370" s="14"/>
+    </row>
+    <row r="371" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB371" s="14"/>
+      <c r="AC371" s="14"/>
+      <c r="AD371" s="14"/>
+      <c r="AE371" s="14"/>
+      <c r="AF371" s="14"/>
+      <c r="AG371" s="14"/>
+      <c r="AH371" s="14"/>
+      <c r="AI371" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11455,7 +11638,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T148"/>
+  <dimension ref="A1:T152"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -16157,6 +16340,146 @@
       <c r="S148" s="14"/>
       <c r="T148" s="14"/>
     </row>
+    <row r="149" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A149" s="15" t="s">
+        <v>531</v>
+      </c>
+      <c r="B149" s="15" t="s">
+        <v>532</v>
+      </c>
+      <c r="C149" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D149" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E149" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F149" s="14"/>
+      <c r="G149" s="21"/>
+      <c r="H149" s="21"/>
+      <c r="I149" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J149" s="14"/>
+      <c r="K149" s="14"/>
+      <c r="L149" s="14"/>
+      <c r="M149" s="14"/>
+      <c r="N149" s="14"/>
+      <c r="O149" s="14"/>
+      <c r="P149" s="14"/>
+      <c r="Q149" s="14"/>
+      <c r="R149" s="14"/>
+      <c r="S149" s="14"/>
+      <c r="T149" s="14"/>
+    </row>
+    <row r="150" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="15" t="s">
+        <v>536</v>
+      </c>
+      <c r="B150" s="15" t="s">
+        <v>532</v>
+      </c>
+      <c r="C150" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D150" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E150" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="F150" s="15"/>
+      <c r="G150" s="15"/>
+      <c r="H150" s="15"/>
+      <c r="I150" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J150" s="14"/>
+      <c r="K150" s="14"/>
+      <c r="L150" s="14"/>
+      <c r="M150" s="14"/>
+      <c r="N150" s="14"/>
+      <c r="O150" s="14"/>
+      <c r="P150" s="14"/>
+      <c r="Q150" s="14"/>
+      <c r="R150" s="14"/>
+      <c r="S150" s="14"/>
+      <c r="T150" s="14"/>
+    </row>
+    <row r="151" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="15" t="s">
+        <v>537</v>
+      </c>
+      <c r="B151" s="30" t="s">
+        <v>538</v>
+      </c>
+      <c r="C151" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D151" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E151" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="F151" s="15"/>
+      <c r="G151" s="15"/>
+      <c r="H151" s="15"/>
+      <c r="I151" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J151" s="14"/>
+      <c r="K151" s="14"/>
+      <c r="L151" s="14"/>
+      <c r="M151" s="14"/>
+      <c r="N151" s="14"/>
+      <c r="O151" s="14"/>
+      <c r="P151" s="14"/>
+      <c r="Q151" s="14"/>
+      <c r="R151" s="14"/>
+      <c r="S151" s="14"/>
+      <c r="T151" s="14"/>
+    </row>
+    <row r="152" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="16" t="s">
+        <v>540</v>
+      </c>
+      <c r="B152" s="20" t="s">
+        <v>494</v>
+      </c>
+      <c r="C152" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D152" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="E152" s="14"/>
+      <c r="F152" s="14"/>
+      <c r="G152" s="14"/>
+      <c r="H152" s="14"/>
+      <c r="I152" s="14"/>
+      <c r="J152" s="14"/>
+      <c r="K152" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L152" s="14"/>
+      <c r="M152" s="14"/>
+      <c r="N152" s="14"/>
+      <c r="O152" s="14"/>
+      <c r="P152" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q152" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R152" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S152" s="14"/>
+      <c r="T152" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Commit the changes done as part of NVI Script execution
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C8DB20-0328-4BC6-8361-2A2CC7977E1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E8D3326-C2BC-4B51-AECE-4A76299124ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1671,193 +1671,193 @@
     <t>939|940</t>
   </si>
   <si>
+    <t>NVI_OBScenario008</t>
+  </si>
+  <si>
+    <t>941</t>
+  </si>
+  <si>
+    <t>000-14268-001</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario009</t>
+  </si>
+  <si>
+    <t>942|943</t>
+  </si>
+  <si>
+    <t>942</t>
+  </si>
+  <si>
+    <t>943</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario011</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario012</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario013</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario014</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario015</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario016</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario017</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario018</t>
+  </si>
+  <si>
+    <t>NVI_OBScenario019</t>
+  </si>
+  <si>
+    <t>944</t>
+  </si>
+  <si>
+    <t>945</t>
+  </si>
+  <si>
+    <t>946</t>
+  </si>
+  <si>
+    <t>947</t>
+  </si>
+  <si>
+    <t>948</t>
+  </si>
+  <si>
+    <t>949</t>
+  </si>
+  <si>
+    <t>945|946</t>
+  </si>
+  <si>
+    <t>948|949</t>
+  </si>
+  <si>
+    <t>950</t>
+  </si>
+  <si>
+    <t>951</t>
+  </si>
+  <si>
+    <t>952</t>
+  </si>
+  <si>
+    <t>953</t>
+  </si>
+  <si>
+    <t>954</t>
+  </si>
+  <si>
+    <t>955</t>
+  </si>
+  <si>
+    <t>956</t>
+  </si>
+  <si>
+    <t>952|953</t>
+  </si>
+  <si>
+    <t>955|956</t>
+  </si>
+  <si>
+    <t>000-15696-001</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario037</t>
+  </si>
+  <si>
+    <t>957</t>
+  </si>
+  <si>
+    <t>958</t>
+  </si>
+  <si>
+    <t>959|960</t>
+  </si>
+  <si>
+    <t>959</t>
+  </si>
+  <si>
+    <t>960</t>
+  </si>
+  <si>
+    <t>961</t>
+  </si>
+  <si>
+    <t>962</t>
+  </si>
+  <si>
+    <t>963</t>
+  </si>
+  <si>
+    <t>964</t>
+  </si>
+  <si>
+    <t>965</t>
+  </si>
+  <si>
+    <t>966</t>
+  </si>
+  <si>
+    <t>967</t>
+  </si>
+  <si>
+    <t>968</t>
+  </si>
+  <si>
+    <t>969</t>
+  </si>
+  <si>
+    <t>970</t>
+  </si>
+  <si>
+    <t>964|965</t>
+  </si>
+  <si>
+    <t>966|967</t>
+  </si>
+  <si>
+    <t>968|969</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario041</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario046</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario038</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario039</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario040</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario042</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario043</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario044</t>
+  </si>
+  <si>
+    <t>NVI_IBScenario045</t>
+  </si>
+  <si>
     <t>000-081221-023</t>
-  </si>
-  <si>
-    <t>NVI_OBScenario008</t>
-  </si>
-  <si>
-    <t>941</t>
-  </si>
-  <si>
-    <t>000-14268-001</t>
-  </si>
-  <si>
-    <t>NVI_OBScenario009</t>
-  </si>
-  <si>
-    <t>942|943</t>
-  </si>
-  <si>
-    <t>942</t>
-  </si>
-  <si>
-    <t>943</t>
-  </si>
-  <si>
-    <t>NVI_OBScenario011</t>
-  </si>
-  <si>
-    <t>NVI_OBScenario012</t>
-  </si>
-  <si>
-    <t>NVI_OBScenario013</t>
-  </si>
-  <si>
-    <t>NVI_OBScenario014</t>
-  </si>
-  <si>
-    <t>NVI_OBScenario015</t>
-  </si>
-  <si>
-    <t>NVI_OBScenario016</t>
-  </si>
-  <si>
-    <t>NVI_OBScenario017</t>
-  </si>
-  <si>
-    <t>NVI_OBScenario018</t>
-  </si>
-  <si>
-    <t>NVI_OBScenario019</t>
-  </si>
-  <si>
-    <t>944</t>
-  </si>
-  <si>
-    <t>945</t>
-  </si>
-  <si>
-    <t>946</t>
-  </si>
-  <si>
-    <t>947</t>
-  </si>
-  <si>
-    <t>948</t>
-  </si>
-  <si>
-    <t>949</t>
-  </si>
-  <si>
-    <t>945|946</t>
-  </si>
-  <si>
-    <t>948|949</t>
-  </si>
-  <si>
-    <t>950</t>
-  </si>
-  <si>
-    <t>951</t>
-  </si>
-  <si>
-    <t>952</t>
-  </si>
-  <si>
-    <t>953</t>
-  </si>
-  <si>
-    <t>954</t>
-  </si>
-  <si>
-    <t>955</t>
-  </si>
-  <si>
-    <t>956</t>
-  </si>
-  <si>
-    <t>952|953</t>
-  </si>
-  <si>
-    <t>955|956</t>
-  </si>
-  <si>
-    <t>000-15696-001</t>
-  </si>
-  <si>
-    <t>NVI_IBScenario037</t>
-  </si>
-  <si>
-    <t>957</t>
-  </si>
-  <si>
-    <t>958</t>
-  </si>
-  <si>
-    <t>959|960</t>
-  </si>
-  <si>
-    <t>959</t>
-  </si>
-  <si>
-    <t>960</t>
-  </si>
-  <si>
-    <t>961</t>
-  </si>
-  <si>
-    <t>962</t>
-  </si>
-  <si>
-    <t>963</t>
-  </si>
-  <si>
-    <t>964</t>
-  </si>
-  <si>
-    <t>965</t>
-  </si>
-  <si>
-    <t>966</t>
-  </si>
-  <si>
-    <t>967</t>
-  </si>
-  <si>
-    <t>968</t>
-  </si>
-  <si>
-    <t>969</t>
-  </si>
-  <si>
-    <t>970</t>
-  </si>
-  <si>
-    <t>964|965</t>
-  </si>
-  <si>
-    <t>966|967</t>
-  </si>
-  <si>
-    <t>968|969</t>
-  </si>
-  <si>
-    <t>NVI_IBScenario041</t>
-  </si>
-  <si>
-    <t>NVI_IBScenario046</t>
-  </si>
-  <si>
-    <t>NVI_IBScenario038</t>
-  </si>
-  <si>
-    <t>NVI_IBScenario039</t>
-  </si>
-  <si>
-    <t>NVI_IBScenario040</t>
-  </si>
-  <si>
-    <t>NVI_IBScenario042</t>
-  </si>
-  <si>
-    <t>NVI_IBScenario043</t>
-  </si>
-  <si>
-    <t>NVI_IBScenario044</t>
-  </si>
-  <si>
-    <t>NVI_IBScenario045</t>
   </si>
 </sst>
 </file>
@@ -9222,7 +9222,7 @@
     </row>
     <row r="150" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="14" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B150" s="14" t="s">
         <v>174</v>
@@ -9231,7 +9231,7 @@
         <v>135</v>
       </c>
       <c r="D150" s="15" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E150" s="14"/>
       <c r="F150" s="14" t="s">
@@ -9271,7 +9271,7 @@
     </row>
     <row r="151" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="14" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B151" s="14" t="s">
         <v>174</v>
@@ -9280,7 +9280,7 @@
         <v>135</v>
       </c>
       <c r="D151" s="15" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E151" s="14"/>
       <c r="F151" s="14" t="s">
@@ -9320,7 +9320,7 @@
     </row>
     <row r="152" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="14" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B152" s="14" t="s">
         <v>174</v>
@@ -9329,7 +9329,7 @@
         <v>135</v>
       </c>
       <c r="D152" s="15" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E152" s="14"/>
       <c r="F152" s="14" t="s">
@@ -9369,7 +9369,7 @@
     </row>
     <row r="153" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="14" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B153" s="14" t="s">
         <v>174</v>
@@ -9378,7 +9378,7 @@
         <v>135</v>
       </c>
       <c r="D153" s="18" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="E153" s="15"/>
       <c r="F153" s="14" t="s">
@@ -9420,7 +9420,7 @@
     </row>
     <row r="154" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="14" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B154" s="14" t="s">
         <v>174</v>
@@ -9429,7 +9429,7 @@
         <v>135</v>
       </c>
       <c r="D154" s="18" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="E154" s="15"/>
       <c r="F154" s="14" t="s">
@@ -9469,7 +9469,7 @@
     </row>
     <row r="155" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="14" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B155" s="14" t="s">
         <v>174</v>
@@ -9478,7 +9478,7 @@
         <v>135</v>
       </c>
       <c r="D155" s="18" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E155" s="14"/>
       <c r="F155" s="14" t="s">
@@ -9516,7 +9516,7 @@
     </row>
     <row r="156" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="14" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B156" s="14" t="s">
         <v>174</v>
@@ -9525,7 +9525,7 @@
         <v>135</v>
       </c>
       <c r="D156" s="18" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="E156" s="14"/>
       <c r="F156" s="14" t="s">
@@ -9563,7 +9563,7 @@
     </row>
     <row r="157" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="14" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B157" s="14" t="s">
         <v>174</v>
@@ -9572,7 +9572,7 @@
         <v>135</v>
       </c>
       <c r="D157" s="18" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="E157" s="15"/>
       <c r="F157" s="14" t="s">
@@ -9612,7 +9612,7 @@
     </row>
     <row r="158" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="14" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B158" s="14" t="s">
         <v>174</v>
@@ -9621,7 +9621,7 @@
         <v>135</v>
       </c>
       <c r="D158" s="18" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E158" s="15"/>
       <c r="F158" s="14" t="s">
@@ -9661,7 +9661,7 @@
     </row>
     <row r="159" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="14" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B159" s="14" t="s">
         <v>174</v>
@@ -9670,7 +9670,7 @@
         <v>135</v>
       </c>
       <c r="D159" s="18" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="E159" s="15"/>
       <c r="F159" s="14" t="s">
@@ -9988,8 +9988,8 @@
       <c r="J165" s="14"/>
       <c r="K165" s="14"/>
       <c r="L165" s="14"/>
-      <c r="M165" s="14" t="s">
-        <v>532</v>
+      <c r="M165" s="20" t="s">
+        <v>609</v>
       </c>
       <c r="N165" s="14"/>
       <c r="O165" s="14"/>
@@ -10132,7 +10132,7 @@
     </row>
     <row r="168" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="14" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B168" s="14" t="s">
         <v>174</v>
@@ -10141,7 +10141,7 @@
         <v>135</v>
       </c>
       <c r="D168" s="18" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E168" s="14"/>
       <c r="F168" s="14"/>
@@ -10187,7 +10187,7 @@
     </row>
     <row r="169" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="14" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B169" s="14" t="s">
         <v>174</v>
@@ -10196,7 +10196,7 @@
         <v>135</v>
       </c>
       <c r="D169" s="18" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="E169" s="14"/>
       <c r="F169" s="14"/>
@@ -10279,7 +10279,7 @@
     </row>
     <row r="171" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="14" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B171" s="14" t="s">
         <v>174</v>
@@ -10288,7 +10288,7 @@
         <v>135</v>
       </c>
       <c r="D171" s="18" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="E171" s="14"/>
       <c r="F171" s="14"/>
@@ -10338,7 +10338,7 @@
     </row>
     <row r="172" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="14" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B172" s="14" t="s">
         <v>174</v>
@@ -10347,7 +10347,7 @@
         <v>135</v>
       </c>
       <c r="D172" s="18" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="E172" s="14"/>
       <c r="F172" s="14"/>
@@ -10389,7 +10389,7 @@
     </row>
     <row r="173" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="14" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B173" s="14" t="s">
         <v>174</v>
@@ -10398,7 +10398,7 @@
         <v>135</v>
       </c>
       <c r="D173" s="18" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="E173" s="14"/>
       <c r="F173" s="14"/>
@@ -10442,7 +10442,7 @@
     </row>
     <row r="174" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="14" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B174" s="14" t="s">
         <v>174</v>
@@ -10451,7 +10451,7 @@
         <v>135</v>
       </c>
       <c r="D174" s="18" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="E174" s="14"/>
       <c r="F174" s="14"/>
@@ -10501,7 +10501,7 @@
     </row>
     <row r="175" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="14" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B175" s="14" t="s">
         <v>174</v>
@@ -10510,7 +10510,7 @@
         <v>135</v>
       </c>
       <c r="D175" s="23" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="E175" s="14"/>
       <c r="F175" s="14"/>
@@ -10521,7 +10521,7 @@
       <c r="K175" s="14"/>
       <c r="L175" s="14"/>
       <c r="M175" s="30" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="N175" s="14"/>
       <c r="O175" s="14"/>
@@ -10556,7 +10556,7 @@
     </row>
     <row r="176" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="14" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B176" s="14" t="s">
         <v>174</v>
@@ -10565,7 +10565,7 @@
         <v>135</v>
       </c>
       <c r="D176" s="23" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="E176" s="14"/>
       <c r="F176" s="14"/>
@@ -10576,7 +10576,7 @@
       <c r="K176" s="14"/>
       <c r="L176" s="14"/>
       <c r="M176" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="N176" s="14"/>
       <c r="O176" s="14"/>
@@ -10609,7 +10609,7 @@
     </row>
     <row r="177" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="14" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B177" s="14" t="s">
         <v>174</v>
@@ -10618,7 +10618,7 @@
         <v>135</v>
       </c>
       <c r="D177" s="23" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="E177" s="14"/>
       <c r="F177" s="14"/>
@@ -10629,7 +10629,7 @@
       <c r="K177" s="14"/>
       <c r="L177" s="14"/>
       <c r="M177" s="14" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="N177" s="14"/>
       <c r="O177" s="14"/>
@@ -10664,7 +10664,7 @@
     </row>
     <row r="178" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="14" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B178" s="14" t="s">
         <v>174</v>
@@ -10673,7 +10673,7 @@
         <v>135</v>
       </c>
       <c r="D178" s="18" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E178" s="14"/>
       <c r="F178" s="14"/>
@@ -10684,7 +10684,7 @@
       <c r="K178" s="14"/>
       <c r="L178" s="14"/>
       <c r="M178" s="14" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="N178" s="14"/>
       <c r="O178" s="14"/>
@@ -10719,7 +10719,7 @@
     </row>
     <row r="179" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="14" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B179" s="14" t="s">
         <v>174</v>
@@ -10728,7 +10728,7 @@
         <v>135</v>
       </c>
       <c r="D179" s="18" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E179" s="14"/>
       <c r="F179" s="14"/>
@@ -10739,7 +10739,7 @@
       <c r="K179" s="14"/>
       <c r="L179" s="31"/>
       <c r="M179" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="N179" s="14"/>
       <c r="O179" s="14"/>
@@ -15768,13 +15768,13 @@
         <v>176</v>
       </c>
       <c r="C83" s="15" t="s">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="D83" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E83" s="15" t="s">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="G83" s="21"/>
       <c r="H83" s="21"/>
@@ -17549,7 +17549,7 @@
         <v>520</v>
       </c>
       <c r="B143" s="18" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="C143" s="15" t="s">
         <v>79</v>
@@ -17873,7 +17873,7 @@
         <v>540</v>
       </c>
       <c r="B152" s="20" t="s">
-        <v>547</v>
+        <v>609</v>
       </c>
       <c r="C152" s="15" t="s">
         <v>2</v>
@@ -18022,7 +18022,7 @@
     </row>
     <row r="156" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="15" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B156" s="20" t="s">
         <v>494</v>
@@ -18060,7 +18060,7 @@
     </row>
     <row r="157" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="15" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B157" s="20" t="s">
         <v>494</v>
@@ -18098,7 +18098,7 @@
     </row>
     <row r="158" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="15" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B158" s="20" t="s">
         <v>494</v>
@@ -18136,10 +18136,10 @@
     </row>
     <row r="159" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="15" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B159" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C159" s="15" t="s">
         <v>2</v>
@@ -18174,10 +18174,10 @@
     </row>
     <row r="160" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="15" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B160" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C160" s="15" t="s">
         <v>0</v>
@@ -18214,10 +18214,10 @@
     </row>
     <row r="161" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="15" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B161" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C161" s="15" t="s">
         <v>0</v>
@@ -18252,10 +18252,10 @@
     </row>
     <row r="162" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="15" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B162" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C162" s="15" t="s">
         <v>0</v>
@@ -18290,10 +18290,10 @@
     </row>
     <row r="163" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="15" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B163" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C163" s="15" t="s">
         <v>2</v>
@@ -18328,10 +18328,10 @@
     </row>
     <row r="164" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="15" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B164" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C164" s="15" t="s">
         <v>2</v>
@@ -18366,10 +18366,10 @@
     </row>
     <row r="165" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="15" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B165" s="30" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C165" s="15" t="s">
         <v>2</v>
@@ -18404,10 +18404,10 @@
     </row>
     <row r="166" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="15" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B166" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C166" s="15" t="s">
         <v>2</v>
@@ -18442,10 +18442,10 @@
     </row>
     <row r="167" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="15" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B167" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C167" s="15" t="s">
         <v>0</v>
@@ -18480,10 +18480,10 @@
     </row>
     <row r="168" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="15" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B168" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C168" s="15" t="s">
         <v>0</v>
@@ -18518,10 +18518,10 @@
     </row>
     <row r="169" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="15" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B169" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C169" s="15" t="s">
         <v>2</v>
@@ -18556,10 +18556,10 @@
     </row>
     <row r="170" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="15" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B170" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C170" s="15" t="s">
         <v>2</v>
@@ -18594,10 +18594,10 @@
     </row>
     <row r="171" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="15" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B171" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C171" s="15" t="s">
         <v>2</v>
@@ -18632,10 +18632,10 @@
     </row>
     <row r="172" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="15" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B172" s="15" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C172" s="15" t="s">
         <v>2</v>
@@ -18666,10 +18666,10 @@
     </row>
     <row r="173" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="15" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B173" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C173" s="15" t="s">
         <v>60</v>
@@ -18700,10 +18700,10 @@
     </row>
     <row r="174" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="15" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B174" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C174" s="15" t="s">
         <v>3</v>
@@ -18734,10 +18734,10 @@
     </row>
     <row r="175" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="15" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B175" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C175" s="15" t="s">
         <v>60</v>
@@ -18768,7 +18768,7 @@
     </row>
     <row r="176" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="15" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B176" s="18" t="s">
         <v>440</v>
@@ -18802,10 +18802,10 @@
     </row>
     <row r="177" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="15" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B177" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C177" s="15" t="s">
         <v>2</v>
@@ -18842,10 +18842,10 @@
     </row>
     <row r="178" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="15" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B178" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C178" s="15" t="s">
         <v>3</v>
@@ -18876,10 +18876,10 @@
     </row>
     <row r="179" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="15" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B179" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C179" s="15" t="s">
         <v>3</v>
@@ -18910,10 +18910,10 @@
     </row>
     <row r="180" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="15" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B180" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C180" s="15" t="s">
         <v>3</v>
@@ -18944,10 +18944,10 @@
     </row>
     <row r="181" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A181" s="15" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B181" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C181" s="15" t="s">
         <v>69</v>
@@ -18978,10 +18978,10 @@
     </row>
     <row r="182" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A182" s="15" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B182" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C182" s="15" t="s">
         <v>69</v>
@@ -19012,10 +19012,10 @@
     </row>
     <row r="183" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A183" s="15" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B183" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C183" s="15" t="s">
         <v>2</v>
@@ -19052,10 +19052,10 @@
     </row>
     <row r="184" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A184" s="15" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B184" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C184" s="15" t="s">
         <v>2</v>
@@ -19092,10 +19092,10 @@
     </row>
     <row r="185" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A185" s="15" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B185" s="30" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C185" s="15" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
Commit after update the Tags for Scenarios to meaningful tag
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E8D3326-C2BC-4B51-AECE-4A76299124ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01465413-FD2F-41C9-B73F-697DA4E27E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2625" uniqueCount="610">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2641" uniqueCount="613">
   <si>
     <t>1</t>
   </si>
@@ -1858,6 +1858,15 @@
   </si>
   <si>
     <t>000-081221-023</t>
+  </si>
+  <si>
+    <t>QSC_DailyRegressionOB11</t>
+  </si>
+  <si>
+    <t>971</t>
+  </si>
+  <si>
+    <t>FG-002182-03</t>
   </si>
 </sst>
 </file>
@@ -2401,7 +2410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI392"/>
+  <dimension ref="A1:AI393"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -6118,10 +6127,18 @@
       <c r="AI80" s="14"/>
     </row>
     <row r="81" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="14"/>
-      <c r="B81" s="14"/>
-      <c r="C81" s="14"/>
-      <c r="D81" s="23"/>
+      <c r="A81" s="14" t="s">
+        <v>610</v>
+      </c>
+      <c r="B81" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="C81" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D81" s="23" t="s">
+        <v>611</v>
+      </c>
       <c r="E81" s="14"/>
       <c r="F81" s="14"/>
       <c r="G81" s="14"/>
@@ -6145,29 +6162,29 @@
       <c r="Y81" s="14"/>
       <c r="Z81" s="14"/>
       <c r="AA81" s="14"/>
-      <c r="AB81" s="14"/>
-      <c r="AC81" s="14"/>
-      <c r="AD81" s="14"/>
+      <c r="AB81" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC81" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD81" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE81" s="27"/>
       <c r="AF81" s="14"/>
       <c r="AG81" s="14"/>
-      <c r="AH81" s="14"/>
+      <c r="AH81" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI81" s="14"/>
     </row>
     <row r="82" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="14" t="s">
-        <v>302</v>
-      </c>
-      <c r="B82" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="C82" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D82" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="E82" s="15"/>
+      <c r="A82" s="14"/>
+      <c r="B82" s="14"/>
+      <c r="C82" s="14"/>
+      <c r="D82" s="23"/>
+      <c r="E82" s="14"/>
       <c r="F82" s="14"/>
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
@@ -6201,7 +6218,7 @@
     </row>
     <row r="83" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B83" s="14" t="s">
         <v>107</v>
@@ -6210,9 +6227,9 @@
         <v>135</v>
       </c>
       <c r="D83" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="E83" s="14"/>
+        <v>0</v>
+      </c>
+      <c r="E83" s="15"/>
       <c r="F83" s="14"/>
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
@@ -6246,7 +6263,7 @@
     </row>
     <row r="84" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="14" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B84" s="14" t="s">
         <v>107</v>
@@ -6255,17 +6272,13 @@
         <v>135</v>
       </c>
       <c r="D84" s="18" t="s">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="E84" s="14"/>
-      <c r="F84" s="14" t="s">
-        <v>403</v>
-      </c>
+      <c r="F84" s="14"/>
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
-      <c r="I84" s="14" t="s">
-        <v>128</v>
-      </c>
+      <c r="I84" s="14"/>
       <c r="J84" s="14"/>
       <c r="K84" s="14"/>
       <c r="L84" s="14"/>
@@ -6295,7 +6308,7 @@
     </row>
     <row r="85" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="14" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B85" s="14" t="s">
         <v>107</v>
@@ -6304,7 +6317,7 @@
         <v>135</v>
       </c>
       <c r="D85" s="18" t="s">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="E85" s="14"/>
       <c r="F85" s="14" t="s">
@@ -6313,7 +6326,7 @@
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
       <c r="I85" s="14" t="s">
-        <v>378</v>
+        <v>128</v>
       </c>
       <c r="J85" s="14"/>
       <c r="K85" s="14"/>
@@ -6344,7 +6357,7 @@
     </row>
     <row r="86" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="14" t="s">
-        <v>342</v>
+        <v>305</v>
       </c>
       <c r="B86" s="14" t="s">
         <v>107</v>
@@ -6352,14 +6365,18 @@
       <c r="C86" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D86" s="25" t="s">
-        <v>346</v>
+      <c r="D86" s="18" t="s">
+        <v>118</v>
       </c>
       <c r="E86" s="14"/>
-      <c r="F86" s="14"/>
+      <c r="F86" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
-      <c r="I86" s="14"/>
+      <c r="I86" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J86" s="14"/>
       <c r="K86" s="14"/>
       <c r="L86" s="14"/>
@@ -6389,7 +6406,7 @@
     </row>
     <row r="87" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="14" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B87" s="14" t="s">
         <v>107</v>
@@ -6397,8 +6414,8 @@
       <c r="C87" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D87" s="18" t="s">
-        <v>349</v>
+      <c r="D87" s="25" t="s">
+        <v>346</v>
       </c>
       <c r="E87" s="14"/>
       <c r="F87" s="14"/>
@@ -6434,7 +6451,7 @@
     </row>
     <row r="88" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="14" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B88" s="14" t="s">
         <v>107</v>
@@ -6442,8 +6459,8 @@
       <c r="C88" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D88" s="25" t="s">
-        <v>346</v>
+      <c r="D88" s="18" t="s">
+        <v>349</v>
       </c>
       <c r="E88" s="14"/>
       <c r="F88" s="14"/>
@@ -6479,7 +6496,7 @@
     </row>
     <row r="89" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="14" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B89" s="14" t="s">
         <v>107</v>
@@ -6487,8 +6504,8 @@
       <c r="C89" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D89" s="18" t="s">
-        <v>349</v>
+      <c r="D89" s="25" t="s">
+        <v>346</v>
       </c>
       <c r="E89" s="14"/>
       <c r="F89" s="14"/>
@@ -6524,7 +6541,7 @@
     </row>
     <row r="90" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="14" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="B90" s="14" t="s">
         <v>107</v>
@@ -6532,7 +6549,9 @@
       <c r="C90" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D90" s="18"/>
+      <c r="D90" s="18" t="s">
+        <v>349</v>
+      </c>
       <c r="E90" s="14"/>
       <c r="F90" s="14"/>
       <c r="G90" s="14"/>
@@ -6567,18 +6586,16 @@
     </row>
     <row r="91" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="14" t="s">
-        <v>529</v>
+        <v>350</v>
       </c>
       <c r="B91" s="14" t="s">
-        <v>174</v>
+        <v>107</v>
       </c>
       <c r="C91" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D91" s="18" t="s">
-        <v>530</v>
-      </c>
-      <c r="E91" s="15"/>
+      <c r="D91" s="18"/>
+      <c r="E91" s="14"/>
       <c r="F91" s="14"/>
       <c r="G91" s="14"/>
       <c r="H91" s="14"/>
@@ -6611,11 +6628,19 @@
       <c r="AI91" s="14"/>
     </row>
     <row r="92" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="14"/>
-      <c r="B92" s="14"/>
-      <c r="C92" s="14"/>
-      <c r="D92" s="18"/>
-      <c r="E92" s="14"/>
+      <c r="A92" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="B92" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C92" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D92" s="18" t="s">
+        <v>530</v>
+      </c>
+      <c r="E92" s="15"/>
       <c r="F92" s="14"/>
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
@@ -6648,30 +6673,18 @@
       <c r="AI92" s="14"/>
     </row>
     <row r="93" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="12" t="s">
-        <v>365</v>
-      </c>
-      <c r="B93" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C93" s="12" t="s">
-        <v>135</v>
-      </c>
+      <c r="A93" s="14"/>
+      <c r="B93" s="14"/>
+      <c r="C93" s="14"/>
       <c r="D93" s="18"/>
       <c r="E93" s="14"/>
       <c r="F93" s="14"/>
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
       <c r="I93" s="14"/>
-      <c r="J93" s="13" t="s">
-        <v>405</v>
-      </c>
-      <c r="K93" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L93" s="14" t="s">
-        <v>406</v>
-      </c>
+      <c r="J93" s="14"/>
+      <c r="K93" s="14"/>
+      <c r="L93" s="14"/>
       <c r="M93" s="14"/>
       <c r="N93" s="14"/>
       <c r="O93" s="14"/>
@@ -6698,7 +6711,7 @@
     </row>
     <row r="94" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="12" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B94" s="12" t="s">
         <v>107</v>
@@ -6712,15 +6725,19 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="14"/>
-      <c r="J94" s="14"/>
-      <c r="K94" s="14"/>
-      <c r="L94" s="12"/>
-      <c r="M94" s="12" t="s">
-        <v>398</v>
-      </c>
-      <c r="N94" s="12"/>
-      <c r="O94" s="12"/>
-      <c r="P94" s="12"/>
+      <c r="J94" s="13" t="s">
+        <v>405</v>
+      </c>
+      <c r="K94" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L94" s="14" t="s">
+        <v>406</v>
+      </c>
+      <c r="M94" s="14"/>
+      <c r="N94" s="14"/>
+      <c r="O94" s="14"/>
+      <c r="P94" s="14"/>
       <c r="Q94" s="14"/>
       <c r="R94" s="14"/>
       <c r="S94" s="14"/>
@@ -6743,7 +6760,7 @@
     </row>
     <row r="95" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B95" s="12" t="s">
         <v>107</v>
@@ -6760,10 +6777,10 @@
       <c r="J95" s="14"/>
       <c r="K95" s="14"/>
       <c r="L95" s="12"/>
-      <c r="M95" s="12"/>
-      <c r="N95" s="12" t="s">
-        <v>410</v>
-      </c>
+      <c r="M95" s="12" t="s">
+        <v>398</v>
+      </c>
+      <c r="N95" s="12"/>
       <c r="O95" s="12"/>
       <c r="P95" s="12"/>
       <c r="Q95" s="14"/>
@@ -6788,7 +6805,7 @@
     </row>
     <row r="96" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="12" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B96" s="12" t="s">
         <v>107</v>
@@ -6806,10 +6823,10 @@
       <c r="K96" s="14"/>
       <c r="L96" s="12"/>
       <c r="M96" s="12"/>
-      <c r="N96" s="12"/>
-      <c r="O96" s="12" t="s">
-        <v>407</v>
-      </c>
+      <c r="N96" s="12" t="s">
+        <v>410</v>
+      </c>
+      <c r="O96" s="12"/>
       <c r="P96" s="12"/>
       <c r="Q96" s="14"/>
       <c r="R96" s="14"/>
@@ -6833,7 +6850,7 @@
     </row>
     <row r="97" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B97" s="12" t="s">
         <v>107</v>
@@ -6852,10 +6869,10 @@
       <c r="L97" s="12"/>
       <c r="M97" s="12"/>
       <c r="N97" s="12"/>
-      <c r="O97" s="12"/>
-      <c r="P97" s="13" t="s">
-        <v>408</v>
-      </c>
+      <c r="O97" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="P97" s="12"/>
       <c r="Q97" s="14"/>
       <c r="R97" s="14"/>
       <c r="S97" s="14"/>
@@ -6877,10 +6894,16 @@
       <c r="AI97" s="14"/>
     </row>
     <row r="98" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="14"/>
-      <c r="B98" s="14"/>
-      <c r="C98" s="14"/>
-      <c r="D98" s="23"/>
+      <c r="A98" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="B98" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C98" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D98" s="18"/>
       <c r="E98" s="14"/>
       <c r="F98" s="14"/>
       <c r="G98" s="14"/>
@@ -6888,11 +6911,13 @@
       <c r="I98" s="14"/>
       <c r="J98" s="14"/>
       <c r="K98" s="14"/>
-      <c r="L98" s="14"/>
-      <c r="M98" s="14"/>
-      <c r="N98" s="14"/>
-      <c r="O98" s="14"/>
-      <c r="P98" s="14"/>
+      <c r="L98" s="12"/>
+      <c r="M98" s="12"/>
+      <c r="N98" s="12"/>
+      <c r="O98" s="12"/>
+      <c r="P98" s="13" t="s">
+        <v>408</v>
+      </c>
       <c r="Q98" s="14"/>
       <c r="R98" s="14"/>
       <c r="S98" s="14"/>
@@ -6913,66 +6938,46 @@
       <c r="AH98" s="14"/>
       <c r="AI98" s="14"/>
     </row>
-    <row r="99" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="12" t="s">
-        <v>306</v>
-      </c>
-      <c r="B99" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C99" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="D99" s="12"/>
-      <c r="E99" s="12"/>
-      <c r="F99" s="12"/>
-      <c r="G99" s="12"/>
-      <c r="H99" s="12"/>
-      <c r="I99" s="12"/>
-      <c r="J99" s="12"/>
-      <c r="K99" s="12"/>
-      <c r="L99" s="12"/>
-      <c r="M99" s="12"/>
-      <c r="N99" s="12"/>
-      <c r="O99" s="12"/>
-      <c r="P99" s="12"/>
-      <c r="Q99" s="12"/>
-      <c r="R99" s="12"/>
-      <c r="S99" s="12"/>
-      <c r="T99" s="12"/>
-      <c r="U99" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="V99" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="W99" s="12" t="s">
-        <v>309</v>
-      </c>
-      <c r="X99" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="Y99" s="12" t="s">
-        <v>311</v>
-      </c>
-      <c r="Z99" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="AA99" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="AB99" s="12"/>
-      <c r="AC99" s="12"/>
-      <c r="AD99" s="12"/>
-      <c r="AE99" s="28"/>
-      <c r="AF99" s="12"/>
-      <c r="AG99" s="12"/>
-      <c r="AH99" s="12"/>
-      <c r="AI99" s="12"/>
+    <row r="99" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="14"/>
+      <c r="B99" s="14"/>
+      <c r="C99" s="14"/>
+      <c r="D99" s="23"/>
+      <c r="E99" s="14"/>
+      <c r="F99" s="14"/>
+      <c r="G99" s="14"/>
+      <c r="H99" s="14"/>
+      <c r="I99" s="14"/>
+      <c r="J99" s="14"/>
+      <c r="K99" s="14"/>
+      <c r="L99" s="14"/>
+      <c r="M99" s="14"/>
+      <c r="N99" s="14"/>
+      <c r="O99" s="14"/>
+      <c r="P99" s="14"/>
+      <c r="Q99" s="14"/>
+      <c r="R99" s="14"/>
+      <c r="S99" s="14"/>
+      <c r="T99" s="14"/>
+      <c r="U99" s="14"/>
+      <c r="V99" s="14"/>
+      <c r="W99" s="14"/>
+      <c r="X99" s="14"/>
+      <c r="Y99" s="14"/>
+      <c r="Z99" s="14"/>
+      <c r="AA99" s="14"/>
+      <c r="AB99" s="14"/>
+      <c r="AC99" s="14"/>
+      <c r="AD99" s="14"/>
+      <c r="AE99" s="27"/>
+      <c r="AF99" s="14"/>
+      <c r="AG99" s="14"/>
+      <c r="AH99" s="14"/>
+      <c r="AI99" s="14"/>
     </row>
     <row r="100" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="12" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="B100" s="12" t="s">
         <v>107</v>
@@ -7029,7 +7034,7 @@
     </row>
     <row r="101" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="12" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B101" s="12" t="s">
         <v>107</v>
@@ -7054,22 +7059,24 @@
       <c r="R101" s="12"/>
       <c r="S101" s="12"/>
       <c r="T101" s="12"/>
-      <c r="U101" s="12" t="s">
+      <c r="U101" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="V101" s="12" t="s">
-        <v>314</v>
+      <c r="V101" s="13" t="s">
+        <v>308</v>
       </c>
       <c r="W101" s="12" t="s">
         <v>309</v>
       </c>
       <c r="X101" s="12" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="Y101" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="Z101" s="12"/>
+      <c r="Z101" s="12" t="s">
+        <v>107</v>
+      </c>
       <c r="AA101" s="12" t="s">
         <v>135</v>
       </c>
@@ -7084,7 +7091,7 @@
     </row>
     <row r="102" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="12" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B102" s="12" t="s">
         <v>107</v>
@@ -7109,25 +7116,25 @@
       <c r="R102" s="12"/>
       <c r="S102" s="12"/>
       <c r="T102" s="12"/>
-      <c r="U102" s="13" t="s">
+      <c r="U102" s="12" t="s">
         <v>307</v>
       </c>
-      <c r="V102" s="13" t="s">
-        <v>317</v>
+      <c r="V102" s="12" t="s">
+        <v>314</v>
       </c>
       <c r="W102" s="12" t="s">
         <v>309</v>
       </c>
       <c r="X102" s="12" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="Y102" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="Z102" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="AA102" s="12"/>
+      <c r="Z102" s="12"/>
+      <c r="AA102" s="12" t="s">
+        <v>135</v>
+      </c>
       <c r="AB102" s="12"/>
       <c r="AC102" s="12"/>
       <c r="AD102" s="12"/>
@@ -7139,7 +7146,7 @@
     </row>
     <row r="103" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="12" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B103" s="12" t="s">
         <v>107</v>
@@ -7164,25 +7171,25 @@
       <c r="R103" s="12"/>
       <c r="S103" s="12"/>
       <c r="T103" s="12"/>
-      <c r="U103" s="12" t="s">
+      <c r="U103" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="V103" s="12" t="s">
-        <v>319</v>
+      <c r="V103" s="13" t="s">
+        <v>317</v>
       </c>
       <c r="W103" s="12" t="s">
         <v>309</v>
       </c>
-      <c r="X103" s="12"/>
+      <c r="X103" s="12" t="s">
+        <v>310</v>
+      </c>
       <c r="Y103" s="12" t="s">
         <v>311</v>
       </c>
       <c r="Z103" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="AA103" s="12" t="s">
-        <v>135</v>
-      </c>
+      <c r="AA103" s="12"/>
       <c r="AB103" s="12"/>
       <c r="AC103" s="12"/>
       <c r="AD103" s="12"/>
@@ -7194,7 +7201,7 @@
     </row>
     <row r="104" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="12" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B104" s="12" t="s">
         <v>107</v>
@@ -7219,16 +7226,16 @@
       <c r="R104" s="12"/>
       <c r="S104" s="12"/>
       <c r="T104" s="12"/>
-      <c r="U104" s="12"/>
+      <c r="U104" s="12" t="s">
+        <v>307</v>
+      </c>
       <c r="V104" s="12" t="s">
         <v>319</v>
       </c>
       <c r="W104" s="12" t="s">
         <v>309</v>
       </c>
-      <c r="X104" s="12" t="s">
-        <v>315</v>
-      </c>
+      <c r="X104" s="12"/>
       <c r="Y104" s="12" t="s">
         <v>311</v>
       </c>
@@ -7249,7 +7256,7 @@
     </row>
     <row r="105" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="12" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B105" s="12" t="s">
         <v>107</v>
@@ -7274,17 +7281,15 @@
       <c r="R105" s="12"/>
       <c r="S105" s="12"/>
       <c r="T105" s="12"/>
-      <c r="U105" s="13" t="s">
-        <v>322</v>
-      </c>
-      <c r="V105" s="13" t="s">
-        <v>323</v>
-      </c>
-      <c r="W105" s="13" t="s">
+      <c r="U105" s="12"/>
+      <c r="V105" s="12" t="s">
+        <v>319</v>
+      </c>
+      <c r="W105" s="12" t="s">
         <v>309</v>
       </c>
       <c r="X105" s="12" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="Y105" s="12" t="s">
         <v>311</v>
@@ -7306,7 +7311,7 @@
     </row>
     <row r="106" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="12" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="B106" s="12" t="s">
         <v>107</v>
@@ -7332,13 +7337,13 @@
       <c r="S106" s="12"/>
       <c r="T106" s="12"/>
       <c r="U106" s="13" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
       <c r="V106" s="13" t="s">
-        <v>308</v>
+        <v>323</v>
       </c>
       <c r="W106" s="13" t="s">
-        <v>325</v>
+        <v>309</v>
       </c>
       <c r="X106" s="12" t="s">
         <v>310</v>
@@ -7363,7 +7368,7 @@
     </row>
     <row r="107" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="12" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B107" s="12" t="s">
         <v>107</v>
@@ -7388,26 +7393,26 @@
       <c r="R107" s="12"/>
       <c r="S107" s="12"/>
       <c r="T107" s="12"/>
-      <c r="U107" s="12" t="s">
+      <c r="U107" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="V107" s="12" t="s">
+      <c r="V107" s="13" t="s">
         <v>308</v>
       </c>
-      <c r="W107" s="12" t="s">
-        <v>309</v>
+      <c r="W107" s="13" t="s">
+        <v>325</v>
       </c>
       <c r="X107" s="12" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="Y107" s="12" t="s">
         <v>311</v>
       </c>
       <c r="Z107" s="12" t="s">
-        <v>174</v>
+        <v>107</v>
       </c>
       <c r="AA107" s="12" t="s">
-        <v>327</v>
+        <v>135</v>
       </c>
       <c r="AB107" s="12"/>
       <c r="AC107" s="12"/>
@@ -7420,7 +7425,7 @@
     </row>
     <row r="108" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="12" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B108" s="12" t="s">
         <v>107</v>
@@ -7448,8 +7453,8 @@
       <c r="U108" s="12" t="s">
         <v>307</v>
       </c>
-      <c r="V108" s="13" t="s">
-        <v>329</v>
+      <c r="V108" s="12" t="s">
+        <v>308</v>
       </c>
       <c r="W108" s="12" t="s">
         <v>309</v>
@@ -7461,10 +7466,10 @@
         <v>311</v>
       </c>
       <c r="Z108" s="12" t="s">
-        <v>107</v>
+        <v>174</v>
       </c>
       <c r="AA108" s="12" t="s">
-        <v>135</v>
+        <v>327</v>
       </c>
       <c r="AB108" s="12"/>
       <c r="AC108" s="12"/>
@@ -7477,7 +7482,7 @@
     </row>
     <row r="109" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="12" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B109" s="12" t="s">
         <v>107</v>
@@ -7505,8 +7510,8 @@
       <c r="U109" s="12" t="s">
         <v>307</v>
       </c>
-      <c r="V109" s="12" t="s">
-        <v>331</v>
+      <c r="V109" s="13" t="s">
+        <v>329</v>
       </c>
       <c r="W109" s="12" t="s">
         <v>309</v>
@@ -7534,7 +7539,7 @@
     </row>
     <row r="110" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="12" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B110" s="12" t="s">
         <v>107</v>
@@ -7563,7 +7568,7 @@
         <v>307</v>
       </c>
       <c r="V110" s="12" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="W110" s="12" t="s">
         <v>309</v>
@@ -7575,7 +7580,7 @@
         <v>311</v>
       </c>
       <c r="Z110" s="12" t="s">
-        <v>327</v>
+        <v>107</v>
       </c>
       <c r="AA110" s="12" t="s">
         <v>135</v>
@@ -7591,7 +7596,7 @@
     </row>
     <row r="111" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="12" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B111" s="12" t="s">
         <v>107</v>
@@ -7626,13 +7631,13 @@
         <v>309</v>
       </c>
       <c r="X111" s="12" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="Y111" s="12" t="s">
         <v>311</v>
       </c>
       <c r="Z111" s="12" t="s">
-        <v>107</v>
+        <v>327</v>
       </c>
       <c r="AA111" s="12" t="s">
         <v>135</v>
@@ -7647,9 +7652,15 @@
       <c r="AI111" s="12"/>
     </row>
     <row r="112" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="12"/>
-      <c r="B112" s="12"/>
-      <c r="C112" s="12"/>
+      <c r="A112" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="B112" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C112" s="12" t="s">
+        <v>135</v>
+      </c>
       <c r="D112" s="12"/>
       <c r="E112" s="12"/>
       <c r="F112" s="12"/>
@@ -7667,13 +7678,27 @@
       <c r="R112" s="12"/>
       <c r="S112" s="12"/>
       <c r="T112" s="12"/>
-      <c r="U112" s="12"/>
-      <c r="V112" s="12"/>
-      <c r="W112" s="12"/>
-      <c r="X112" s="12"/>
-      <c r="Y112" s="12"/>
-      <c r="Z112" s="12"/>
-      <c r="AA112" s="12"/>
+      <c r="U112" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="V112" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="W112" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="X112" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="Y112" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="Z112" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="AA112" s="12" t="s">
+        <v>135</v>
+      </c>
       <c r="AB112" s="12"/>
       <c r="AC112" s="12"/>
       <c r="AD112" s="12"/>
@@ -7720,37 +7745,46 @@
       <c r="AH113" s="12"/>
       <c r="AI113" s="12"/>
     </row>
-    <row r="114" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A114" s="14" t="s">
-        <v>243</v>
-      </c>
-      <c r="B114" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C114" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D114" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="F114" s="14" t="s">
-        <v>403</v>
-      </c>
-      <c r="R114" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB114" s="14"/>
-      <c r="AC114" s="14"/>
-      <c r="AD114" s="14"/>
-      <c r="AE114" s="27"/>
-      <c r="AF114" s="14"/>
-      <c r="AG114" s="14"/>
-      <c r="AH114" s="14"/>
-      <c r="AI114" s="14"/>
+    <row r="114" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="12"/>
+      <c r="B114" s="12"/>
+      <c r="C114" s="12"/>
+      <c r="D114" s="12"/>
+      <c r="E114" s="12"/>
+      <c r="F114" s="12"/>
+      <c r="G114" s="12"/>
+      <c r="H114" s="12"/>
+      <c r="I114" s="12"/>
+      <c r="J114" s="12"/>
+      <c r="K114" s="12"/>
+      <c r="L114" s="12"/>
+      <c r="M114" s="12"/>
+      <c r="N114" s="12"/>
+      <c r="O114" s="12"/>
+      <c r="P114" s="12"/>
+      <c r="Q114" s="12"/>
+      <c r="R114" s="12"/>
+      <c r="S114" s="12"/>
+      <c r="T114" s="12"/>
+      <c r="U114" s="12"/>
+      <c r="V114" s="12"/>
+      <c r="W114" s="12"/>
+      <c r="X114" s="12"/>
+      <c r="Y114" s="12"/>
+      <c r="Z114" s="12"/>
+      <c r="AA114" s="12"/>
+      <c r="AB114" s="12"/>
+      <c r="AC114" s="12"/>
+      <c r="AD114" s="12"/>
+      <c r="AE114" s="28"/>
+      <c r="AF114" s="12"/>
+      <c r="AG114" s="12"/>
+      <c r="AH114" s="12"/>
+      <c r="AI114" s="12"/>
     </row>
     <row r="115" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A115" s="14" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B115" s="14" t="s">
         <v>174</v>
@@ -7759,7 +7793,7 @@
         <v>135</v>
       </c>
       <c r="D115" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F115" s="14" t="s">
         <v>403</v>
@@ -7778,7 +7812,7 @@
     </row>
     <row r="116" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A116" s="14" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B116" s="14" t="s">
         <v>174</v>
@@ -7787,7 +7821,7 @@
         <v>135</v>
       </c>
       <c r="D116" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F116" s="14" t="s">
         <v>403</v>
@@ -7806,7 +7840,7 @@
     </row>
     <row r="117" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A117" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B117" s="14" t="s">
         <v>174</v>
@@ -7815,7 +7849,7 @@
         <v>135</v>
       </c>
       <c r="D117" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F117" s="14" t="s">
         <v>403</v>
@@ -7834,7 +7868,7 @@
     </row>
     <row r="118" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A118" s="14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B118" s="14" t="s">
         <v>174</v>
@@ -7843,7 +7877,7 @@
         <v>135</v>
       </c>
       <c r="D118" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F118" s="14" t="s">
         <v>403</v>
@@ -7862,7 +7896,7 @@
     </row>
     <row r="119" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A119" s="14" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B119" s="14" t="s">
         <v>174</v>
@@ -7871,7 +7905,7 @@
         <v>135</v>
       </c>
       <c r="D119" s="15" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="F119" s="14" t="s">
         <v>403</v>
@@ -7890,7 +7924,7 @@
     </row>
     <row r="120" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A120" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B120" s="14" t="s">
         <v>174</v>
@@ -7905,7 +7939,7 @@
         <v>403</v>
       </c>
       <c r="R120" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AB120" s="14"/>
       <c r="AC120" s="14"/>
@@ -7916,9 +7950,9 @@
       <c r="AH120" s="14"/>
       <c r="AI120" s="14"/>
     </row>
-    <row r="121" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A121" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B121" s="14" t="s">
         <v>174</v>
@@ -7927,33 +7961,14 @@
         <v>135</v>
       </c>
       <c r="D121" s="15" t="s">
-        <v>236</v>
-      </c>
-      <c r="E121" s="14"/>
+        <v>185</v>
+      </c>
       <c r="F121" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G121" s="14"/>
-      <c r="H121" s="14"/>
-      <c r="I121" s="14"/>
-      <c r="J121" s="14"/>
-      <c r="K121" s="14"/>
-      <c r="L121" s="14"/>
-      <c r="M121" s="14"/>
-      <c r="N121" s="14"/>
-      <c r="O121" s="14"/>
-      <c r="P121" s="14"/>
-      <c r="Q121" s="14"/>
-      <c r="R121" s="15"/>
-      <c r="S121" s="14"/>
-      <c r="T121" s="14"/>
-      <c r="U121" s="14"/>
-      <c r="V121" s="14"/>
-      <c r="W121" s="14"/>
-      <c r="X121" s="14"/>
-      <c r="Y121" s="14"/>
-      <c r="Z121" s="14"/>
-      <c r="AA121" s="14"/>
+      <c r="R121" s="15" t="s">
+        <v>2</v>
+      </c>
       <c r="AB121" s="14"/>
       <c r="AC121" s="14"/>
       <c r="AD121" s="14"/>
@@ -7965,7 +7980,7 @@
     </row>
     <row r="122" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B122" s="14" t="s">
         <v>174</v>
@@ -7974,7 +7989,7 @@
         <v>135</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E122" s="14"/>
       <c r="F122" s="14" t="s">
@@ -8010,9 +8025,9 @@
       <c r="AH122" s="14"/>
       <c r="AI122" s="14"/>
     </row>
-    <row r="123" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B123" s="14" t="s">
         <v>174</v>
@@ -8021,12 +8036,33 @@
         <v>135</v>
       </c>
       <c r="D123" s="15" t="s">
-        <v>238</v>
-      </c>
+        <v>237</v>
+      </c>
+      <c r="E123" s="14"/>
       <c r="F123" s="14" t="s">
         <v>403</v>
       </c>
+      <c r="G123" s="14"/>
+      <c r="H123" s="14"/>
+      <c r="I123" s="14"/>
+      <c r="J123" s="14"/>
+      <c r="K123" s="14"/>
+      <c r="L123" s="14"/>
+      <c r="M123" s="14"/>
+      <c r="N123" s="14"/>
+      <c r="O123" s="14"/>
+      <c r="P123" s="14"/>
+      <c r="Q123" s="14"/>
       <c r="R123" s="15"/>
+      <c r="S123" s="14"/>
+      <c r="T123" s="14"/>
+      <c r="U123" s="14"/>
+      <c r="V123" s="14"/>
+      <c r="W123" s="14"/>
+      <c r="X123" s="14"/>
+      <c r="Y123" s="14"/>
+      <c r="Z123" s="14"/>
+      <c r="AA123" s="14"/>
       <c r="AB123" s="14"/>
       <c r="AC123" s="14"/>
       <c r="AD123" s="14"/>
@@ -8038,7 +8074,7 @@
     </row>
     <row r="124" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A124" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B124" s="14" t="s">
         <v>174</v>
@@ -8047,7 +8083,7 @@
         <v>135</v>
       </c>
       <c r="D124" s="15" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F124" s="14" t="s">
         <v>403</v>
@@ -8064,7 +8100,7 @@
     </row>
     <row r="125" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A125" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B125" s="14" t="s">
         <v>174</v>
@@ -8073,7 +8109,7 @@
         <v>135</v>
       </c>
       <c r="D125" s="15" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F125" s="14" t="s">
         <v>403</v>
@@ -8090,7 +8126,7 @@
     </row>
     <row r="126" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A126" s="14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B126" s="14" t="s">
         <v>174</v>
@@ -8098,15 +8134,13 @@
       <c r="C126" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D126" s="16" t="s">
-        <v>257</v>
+      <c r="D126" s="15" t="s">
+        <v>240</v>
       </c>
       <c r="F126" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="R126" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R126" s="15"/>
       <c r="AB126" s="14"/>
       <c r="AC126" s="14"/>
       <c r="AD126" s="14"/>
@@ -8118,7 +8152,7 @@
     </row>
     <row r="127" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A127" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B127" s="14" t="s">
         <v>174</v>
@@ -8126,8 +8160,8 @@
       <c r="C127" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D127" s="15" t="s">
-        <v>277</v>
+      <c r="D127" s="16" t="s">
+        <v>257</v>
       </c>
       <c r="F127" s="14" t="s">
         <v>403</v>
@@ -8144,9 +8178,9 @@
       <c r="AH127" s="14"/>
       <c r="AI127" s="14"/>
     </row>
-    <row r="128" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A128" s="14" t="s">
-        <v>278</v>
+        <v>256</v>
       </c>
       <c r="B128" s="14" t="s">
         <v>174</v>
@@ -8155,35 +8189,14 @@
         <v>135</v>
       </c>
       <c r="D128" s="15" t="s">
-        <v>279</v>
-      </c>
-      <c r="E128" s="14"/>
+        <v>277</v>
+      </c>
       <c r="F128" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G128" s="14"/>
-      <c r="H128" s="14"/>
-      <c r="I128" s="14"/>
-      <c r="J128" s="14"/>
-      <c r="K128" s="14"/>
-      <c r="L128" s="14"/>
-      <c r="M128" s="14"/>
-      <c r="N128" s="14"/>
-      <c r="O128" s="14"/>
-      <c r="P128" s="14"/>
-      <c r="Q128" s="14"/>
       <c r="R128" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="S128" s="14"/>
-      <c r="T128" s="14"/>
-      <c r="U128" s="14"/>
-      <c r="V128" s="14"/>
-      <c r="W128" s="14"/>
-      <c r="X128" s="14"/>
-      <c r="Y128" s="14"/>
-      <c r="Z128" s="14"/>
-      <c r="AA128" s="14"/>
       <c r="AB128" s="14"/>
       <c r="AC128" s="14"/>
       <c r="AD128" s="14"/>
@@ -8195,7 +8208,7 @@
     </row>
     <row r="129" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="14" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="B129" s="14" t="s">
         <v>174</v>
@@ -8204,7 +8217,7 @@
         <v>135</v>
       </c>
       <c r="D129" s="15" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="E129" s="14"/>
       <c r="F129" s="14" t="s">
@@ -8222,7 +8235,7 @@
       <c r="P129" s="14"/>
       <c r="Q129" s="14"/>
       <c r="R129" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S129" s="14"/>
       <c r="T129" s="14"/>
@@ -8244,7 +8257,7 @@
     </row>
     <row r="130" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="14" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B130" s="14" t="s">
         <v>174</v>
@@ -8253,7 +8266,7 @@
         <v>135</v>
       </c>
       <c r="D130" s="15" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E130" s="14"/>
       <c r="F130" s="14" t="s">
@@ -8271,7 +8284,7 @@
       <c r="P130" s="14"/>
       <c r="Q130" s="14"/>
       <c r="R130" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S130" s="14"/>
       <c r="T130" s="14"/>
@@ -8293,7 +8306,7 @@
     </row>
     <row r="131" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="14" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B131" s="14" t="s">
         <v>174</v>
@@ -8302,7 +8315,7 @@
         <v>135</v>
       </c>
       <c r="D131" s="15" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="E131" s="14"/>
       <c r="F131" s="14" t="s">
@@ -8342,7 +8355,7 @@
     </row>
     <row r="132" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="14" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B132" s="14" t="s">
         <v>174</v>
@@ -8351,7 +8364,7 @@
         <v>135</v>
       </c>
       <c r="D132" s="15" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="E132" s="14"/>
       <c r="F132" s="14" t="s">
@@ -8369,7 +8382,7 @@
       <c r="P132" s="14"/>
       <c r="Q132" s="14"/>
       <c r="R132" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S132" s="14"/>
       <c r="T132" s="14"/>
@@ -8391,7 +8404,7 @@
     </row>
     <row r="133" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="14" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B133" s="14" t="s">
         <v>174</v>
@@ -8400,7 +8413,7 @@
         <v>135</v>
       </c>
       <c r="D133" s="15" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E133" s="14"/>
       <c r="F133" s="14" t="s">
@@ -8418,7 +8431,7 @@
       <c r="P133" s="14"/>
       <c r="Q133" s="14"/>
       <c r="R133" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S133" s="14"/>
       <c r="T133" s="14"/>
@@ -8440,7 +8453,7 @@
     </row>
     <row r="134" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="14" t="s">
-        <v>373</v>
+        <v>294</v>
       </c>
       <c r="B134" s="14" t="s">
         <v>174</v>
@@ -8449,7 +8462,7 @@
         <v>135</v>
       </c>
       <c r="D134" s="15" t="s">
-        <v>372</v>
+        <v>295</v>
       </c>
       <c r="E134" s="14"/>
       <c r="F134" s="14" t="s">
@@ -8457,9 +8470,7 @@
       </c>
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
-      <c r="I134" s="14" t="s">
-        <v>126</v>
-      </c>
+      <c r="I134" s="14"/>
       <c r="J134" s="14"/>
       <c r="K134" s="14"/>
       <c r="L134" s="14"/>
@@ -8468,7 +8479,9 @@
       <c r="O134" s="14"/>
       <c r="P134" s="14"/>
       <c r="Q134" s="14"/>
-      <c r="R134" s="15"/>
+      <c r="R134" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S134" s="14"/>
       <c r="T134" s="14"/>
       <c r="U134" s="14"/>
@@ -8489,7 +8502,7 @@
     </row>
     <row r="135" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="14" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B135" s="14" t="s">
         <v>174</v>
@@ -8498,7 +8511,7 @@
         <v>135</v>
       </c>
       <c r="D135" s="15" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="E135" s="14"/>
       <c r="F135" s="14" t="s">
@@ -8507,7 +8520,7 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="14" t="s">
-        <v>379</v>
+        <v>126</v>
       </c>
       <c r="J135" s="14"/>
       <c r="K135" s="14"/>
@@ -8538,7 +8551,7 @@
     </row>
     <row r="136" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="14" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="B136" s="14" t="s">
         <v>174</v>
@@ -8547,7 +8560,7 @@
         <v>135</v>
       </c>
       <c r="D136" s="15" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="E136" s="14"/>
       <c r="F136" s="14" t="s">
@@ -8556,7 +8569,7 @@
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
       <c r="I136" s="14" t="s">
-        <v>125</v>
+        <v>379</v>
       </c>
       <c r="J136" s="14"/>
       <c r="K136" s="14"/>
@@ -8587,7 +8600,7 @@
     </row>
     <row r="137" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="14" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B137" s="14" t="s">
         <v>174</v>
@@ -8596,7 +8609,7 @@
         <v>135</v>
       </c>
       <c r="D137" s="15" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E137" s="14"/>
       <c r="F137" s="14" t="s">
@@ -8605,7 +8618,7 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="14" t="s">
-        <v>381</v>
+        <v>125</v>
       </c>
       <c r="J137" s="14"/>
       <c r="K137" s="14"/>
@@ -8636,7 +8649,7 @@
     </row>
     <row r="138" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="14" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="B138" s="14" t="s">
         <v>174</v>
@@ -8645,7 +8658,7 @@
         <v>135</v>
       </c>
       <c r="D138" s="15" t="s">
-        <v>179</v>
+        <v>385</v>
       </c>
       <c r="E138" s="14"/>
       <c r="F138" s="14" t="s">
@@ -8653,7 +8666,9 @@
       </c>
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
-      <c r="I138" s="14"/>
+      <c r="I138" s="14" t="s">
+        <v>381</v>
+      </c>
       <c r="J138" s="14"/>
       <c r="K138" s="14"/>
       <c r="L138" s="14"/>
@@ -8683,7 +8698,7 @@
     </row>
     <row r="139" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="14" t="s">
-        <v>500</v>
+        <v>390</v>
       </c>
       <c r="B139" s="14" t="s">
         <v>174</v>
@@ -8691,18 +8706,16 @@
       <c r="C139" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D139" s="18" t="s">
-        <v>501</v>
-      </c>
-      <c r="E139" s="15"/>
+      <c r="D139" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="E139" s="14"/>
       <c r="F139" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
-      <c r="I139" s="14" t="s">
-        <v>128</v>
-      </c>
+      <c r="I139" s="14"/>
       <c r="J139" s="14"/>
       <c r="K139" s="14"/>
       <c r="L139" s="14"/>
@@ -8711,7 +8724,7 @@
       <c r="O139" s="14"/>
       <c r="P139" s="14"/>
       <c r="Q139" s="14"/>
-      <c r="R139" s="14"/>
+      <c r="R139" s="15"/>
       <c r="S139" s="14"/>
       <c r="T139" s="14"/>
       <c r="U139" s="14"/>
@@ -8724,17 +8737,15 @@
       <c r="AB139" s="14"/>
       <c r="AC139" s="14"/>
       <c r="AD139" s="14"/>
-      <c r="AE139" s="27" t="s">
-        <v>415</v>
-      </c>
+      <c r="AE139" s="27"/>
       <c r="AF139" s="14"/>
       <c r="AG139" s="14"/>
       <c r="AH139" s="14"/>
       <c r="AI139" s="14"/>
     </row>
     <row r="140" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="15" t="s">
-        <v>502</v>
+      <c r="A140" s="14" t="s">
+        <v>500</v>
       </c>
       <c r="B140" s="14" t="s">
         <v>174</v>
@@ -8743,16 +8754,16 @@
         <v>135</v>
       </c>
       <c r="D140" s="18" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="E140" s="15"/>
       <c r="F140" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G140" s="15"/>
+      <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="14" t="s">
-        <v>504</v>
+        <v>128</v>
       </c>
       <c r="J140" s="14"/>
       <c r="K140" s="14"/>
@@ -8775,7 +8786,9 @@
       <c r="AB140" s="14"/>
       <c r="AC140" s="14"/>
       <c r="AD140" s="14"/>
-      <c r="AE140" s="27"/>
+      <c r="AE140" s="27" t="s">
+        <v>415</v>
+      </c>
       <c r="AF140" s="14"/>
       <c r="AG140" s="14"/>
       <c r="AH140" s="14"/>
@@ -8783,7 +8796,7 @@
     </row>
     <row r="141" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="15" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="B141" s="14" t="s">
         <v>174</v>
@@ -8792,15 +8805,17 @@
         <v>135</v>
       </c>
       <c r="D141" s="18" t="s">
-        <v>506</v>
-      </c>
-      <c r="E141" s="14"/>
+        <v>503</v>
+      </c>
+      <c r="E141" s="15"/>
       <c r="F141" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G141" s="14"/>
+      <c r="G141" s="15"/>
       <c r="H141" s="14"/>
-      <c r="I141" s="14"/>
+      <c r="I141" s="14" t="s">
+        <v>504</v>
+      </c>
       <c r="J141" s="14"/>
       <c r="K141" s="14"/>
       <c r="L141" s="14"/>
@@ -8830,7 +8845,7 @@
     </row>
     <row r="142" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="15" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B142" s="14" t="s">
         <v>174</v>
@@ -8839,7 +8854,7 @@
         <v>135</v>
       </c>
       <c r="D142" s="18" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="E142" s="14"/>
       <c r="F142" s="14" t="s">
@@ -8877,7 +8892,7 @@
     </row>
     <row r="143" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="15" t="s">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="B143" s="14" t="s">
         <v>174</v>
@@ -8886,17 +8901,15 @@
         <v>135</v>
       </c>
       <c r="D143" s="18" t="s">
-        <v>513</v>
-      </c>
-      <c r="E143" s="15"/>
+        <v>508</v>
+      </c>
+      <c r="E143" s="14"/>
       <c r="F143" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G143" s="15"/>
+      <c r="G143" s="14"/>
       <c r="H143" s="14"/>
-      <c r="I143" s="14" t="s">
-        <v>378</v>
-      </c>
+      <c r="I143" s="14"/>
       <c r="J143" s="14"/>
       <c r="K143" s="14"/>
       <c r="L143" s="14"/>
@@ -8926,7 +8939,7 @@
     </row>
     <row r="144" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="15" t="s">
-        <v>519</v>
+        <v>512</v>
       </c>
       <c r="B144" s="14" t="s">
         <v>174</v>
@@ -8935,17 +8948,17 @@
         <v>135</v>
       </c>
       <c r="D144" s="18" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="E144" s="15"/>
-      <c r="F144" s="15" t="s">
-        <v>388</v>
-      </c>
-      <c r="G144" s="15" t="s">
-        <v>3</v>
-      </c>
+      <c r="F144" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="G144" s="15"/>
       <c r="H144" s="14"/>
-      <c r="I144" s="14"/>
+      <c r="I144" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J144" s="14"/>
       <c r="K144" s="14"/>
       <c r="L144" s="14"/>
@@ -8975,7 +8988,7 @@
     </row>
     <row r="145" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="15" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="B145" s="14" t="s">
         <v>174</v>
@@ -8984,17 +8997,17 @@
         <v>135</v>
       </c>
       <c r="D145" s="18" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="E145" s="15"/>
-      <c r="F145" s="14" t="s">
-        <v>403</v>
-      </c>
-      <c r="G145" s="14"/>
+      <c r="F145" s="15" t="s">
+        <v>388</v>
+      </c>
+      <c r="G145" s="15" t="s">
+        <v>3</v>
+      </c>
       <c r="H145" s="14"/>
-      <c r="I145" s="14" t="s">
-        <v>128</v>
-      </c>
+      <c r="I145" s="14"/>
       <c r="J145" s="14"/>
       <c r="K145" s="14"/>
       <c r="L145" s="14"/>
@@ -9016,9 +9029,7 @@
       <c r="AB145" s="14"/>
       <c r="AC145" s="14"/>
       <c r="AD145" s="14"/>
-      <c r="AE145" s="27" t="s">
-        <v>415</v>
-      </c>
+      <c r="AE145" s="27"/>
       <c r="AF145" s="14"/>
       <c r="AG145" s="14"/>
       <c r="AH145" s="14"/>
@@ -9026,7 +9037,7 @@
     </row>
     <row r="146" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="15" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="B146" s="14" t="s">
         <v>174</v>
@@ -9035,7 +9046,7 @@
         <v>135</v>
       </c>
       <c r="D146" s="18" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="E146" s="15"/>
       <c r="F146" s="14" t="s">
@@ -9044,7 +9055,7 @@
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
       <c r="I146" s="14" t="s">
-        <v>401</v>
+        <v>128</v>
       </c>
       <c r="J146" s="14"/>
       <c r="K146" s="14"/>
@@ -9067,7 +9078,9 @@
       <c r="AB146" s="14"/>
       <c r="AC146" s="14"/>
       <c r="AD146" s="14"/>
-      <c r="AE146" s="27"/>
+      <c r="AE146" s="27" t="s">
+        <v>415</v>
+      </c>
       <c r="AF146" s="14"/>
       <c r="AG146" s="14"/>
       <c r="AH146" s="14"/>
@@ -9075,7 +9088,7 @@
     </row>
     <row r="147" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="15" t="s">
-        <v>528</v>
+        <v>523</v>
       </c>
       <c r="B147" s="14" t="s">
         <v>174</v>
@@ -9084,7 +9097,7 @@
         <v>135</v>
       </c>
       <c r="D147" s="18" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E147" s="15"/>
       <c r="F147" s="14" t="s">
@@ -9093,7 +9106,7 @@
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
       <c r="I147" s="14" t="s">
-        <v>126</v>
+        <v>401</v>
       </c>
       <c r="J147" s="14"/>
       <c r="K147" s="14"/>
@@ -9123,8 +9136,8 @@
       <c r="AI147" s="14"/>
     </row>
     <row r="148" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A148" s="14" t="s">
-        <v>533</v>
+      <c r="A148" s="15" t="s">
+        <v>528</v>
       </c>
       <c r="B148" s="14" t="s">
         <v>174</v>
@@ -9132,16 +9145,18 @@
       <c r="C148" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D148" s="15" t="s">
-        <v>531</v>
-      </c>
-      <c r="E148" s="14"/>
+      <c r="D148" s="18" t="s">
+        <v>527</v>
+      </c>
+      <c r="E148" s="15"/>
       <c r="F148" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
-      <c r="I148" s="14"/>
+      <c r="I148" s="14" t="s">
+        <v>126</v>
+      </c>
       <c r="J148" s="14"/>
       <c r="K148" s="14"/>
       <c r="L148" s="14"/>
@@ -9150,9 +9165,7 @@
       <c r="O148" s="14"/>
       <c r="P148" s="14"/>
       <c r="Q148" s="14"/>
-      <c r="R148" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R148" s="14"/>
       <c r="S148" s="14"/>
       <c r="T148" s="14"/>
       <c r="U148" s="14"/>
@@ -9172,8 +9185,8 @@
       <c r="AI148" s="14"/>
     </row>
     <row r="149" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A149" s="15" t="s">
-        <v>534</v>
+      <c r="A149" s="14" t="s">
+        <v>533</v>
       </c>
       <c r="B149" s="14" t="s">
         <v>174</v>
@@ -9181,18 +9194,16 @@
       <c r="C149" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D149" s="18" t="s">
-        <v>535</v>
-      </c>
-      <c r="E149" s="15"/>
+      <c r="D149" s="15" t="s">
+        <v>531</v>
+      </c>
+      <c r="E149" s="14"/>
       <c r="F149" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G149" s="15"/>
+      <c r="G149" s="14"/>
       <c r="H149" s="14"/>
-      <c r="I149" s="14" t="s">
-        <v>378</v>
-      </c>
+      <c r="I149" s="14"/>
       <c r="J149" s="14"/>
       <c r="K149" s="14"/>
       <c r="L149" s="14"/>
@@ -9201,7 +9212,9 @@
       <c r="O149" s="14"/>
       <c r="P149" s="14"/>
       <c r="Q149" s="14"/>
-      <c r="R149" s="14"/>
+      <c r="R149" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S149" s="14"/>
       <c r="T149" s="14"/>
       <c r="U149" s="14"/>
@@ -9221,8 +9234,8 @@
       <c r="AI149" s="14"/>
     </row>
     <row r="150" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="14" t="s">
-        <v>581</v>
+      <c r="A150" s="15" t="s">
+        <v>534</v>
       </c>
       <c r="B150" s="14" t="s">
         <v>174</v>
@@ -9230,16 +9243,18 @@
       <c r="C150" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D150" s="15" t="s">
-        <v>582</v>
-      </c>
-      <c r="E150" s="14"/>
+      <c r="D150" s="18" t="s">
+        <v>535</v>
+      </c>
+      <c r="E150" s="15"/>
       <c r="F150" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G150" s="14"/>
+      <c r="G150" s="15"/>
       <c r="H150" s="14"/>
-      <c r="I150" s="14"/>
+      <c r="I150" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J150" s="14"/>
       <c r="K150" s="14"/>
       <c r="L150" s="14"/>
@@ -9248,9 +9263,7 @@
       <c r="O150" s="14"/>
       <c r="P150" s="14"/>
       <c r="Q150" s="14"/>
-      <c r="R150" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R150" s="14"/>
       <c r="S150" s="14"/>
       <c r="T150" s="14"/>
       <c r="U150" s="14"/>
@@ -9271,7 +9284,7 @@
     </row>
     <row r="151" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="14" t="s">
-        <v>602</v>
+        <v>581</v>
       </c>
       <c r="B151" s="14" t="s">
         <v>174</v>
@@ -9280,7 +9293,7 @@
         <v>135</v>
       </c>
       <c r="D151" s="15" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E151" s="14"/>
       <c r="F151" s="14" t="s">
@@ -9320,7 +9333,7 @@
     </row>
     <row r="152" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="14" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B152" s="14" t="s">
         <v>174</v>
@@ -9329,7 +9342,7 @@
         <v>135</v>
       </c>
       <c r="D152" s="15" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E152" s="14"/>
       <c r="F152" s="14" t="s">
@@ -9369,7 +9382,7 @@
     </row>
     <row r="153" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="14" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B153" s="14" t="s">
         <v>174</v>
@@ -9377,18 +9390,16 @@
       <c r="C153" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D153" s="18" t="s">
-        <v>587</v>
-      </c>
-      <c r="E153" s="15"/>
+      <c r="D153" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="E153" s="14"/>
       <c r="F153" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G153" s="14"/>
       <c r="H153" s="14"/>
-      <c r="I153" s="14" t="s">
-        <v>128</v>
-      </c>
+      <c r="I153" s="14"/>
       <c r="J153" s="14"/>
       <c r="K153" s="14"/>
       <c r="L153" s="14"/>
@@ -9397,7 +9408,9 @@
       <c r="O153" s="14"/>
       <c r="P153" s="14"/>
       <c r="Q153" s="14"/>
-      <c r="R153" s="14"/>
+      <c r="R153" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S153" s="14"/>
       <c r="T153" s="14"/>
       <c r="U153" s="14"/>
@@ -9410,9 +9423,7 @@
       <c r="AB153" s="14"/>
       <c r="AC153" s="14"/>
       <c r="AD153" s="14"/>
-      <c r="AE153" s="27" t="s">
-        <v>415</v>
-      </c>
+      <c r="AE153" s="27"/>
       <c r="AF153" s="14"/>
       <c r="AG153" s="14"/>
       <c r="AH153" s="14"/>
@@ -9420,7 +9431,7 @@
     </row>
     <row r="154" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="14" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="B154" s="14" t="s">
         <v>174</v>
@@ -9429,16 +9440,16 @@
         <v>135</v>
       </c>
       <c r="D154" s="18" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="E154" s="15"/>
       <c r="F154" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G154" s="15"/>
+      <c r="G154" s="14"/>
       <c r="H154" s="14"/>
       <c r="I154" s="14" t="s">
-        <v>504</v>
+        <v>128</v>
       </c>
       <c r="J154" s="14"/>
       <c r="K154" s="14"/>
@@ -9461,7 +9472,9 @@
       <c r="AB154" s="14"/>
       <c r="AC154" s="14"/>
       <c r="AD154" s="14"/>
-      <c r="AE154" s="27"/>
+      <c r="AE154" s="27" t="s">
+        <v>415</v>
+      </c>
       <c r="AF154" s="14"/>
       <c r="AG154" s="14"/>
       <c r="AH154" s="14"/>
@@ -9469,7 +9482,7 @@
     </row>
     <row r="155" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="14" t="s">
-        <v>605</v>
+        <v>600</v>
       </c>
       <c r="B155" s="14" t="s">
         <v>174</v>
@@ -9478,15 +9491,17 @@
         <v>135</v>
       </c>
       <c r="D155" s="18" t="s">
-        <v>589</v>
-      </c>
-      <c r="E155" s="14"/>
+        <v>588</v>
+      </c>
+      <c r="E155" s="15"/>
       <c r="F155" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G155" s="14"/>
+      <c r="G155" s="15"/>
       <c r="H155" s="14"/>
-      <c r="I155" s="14"/>
+      <c r="I155" s="14" t="s">
+        <v>504</v>
+      </c>
       <c r="J155" s="14"/>
       <c r="K155" s="14"/>
       <c r="L155" s="14"/>
@@ -9516,7 +9531,7 @@
     </row>
     <row r="156" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="14" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B156" s="14" t="s">
         <v>174</v>
@@ -9525,7 +9540,7 @@
         <v>135</v>
       </c>
       <c r="D156" s="18" t="s">
-        <v>597</v>
+        <v>589</v>
       </c>
       <c r="E156" s="14"/>
       <c r="F156" s="14" t="s">
@@ -9563,7 +9578,7 @@
     </row>
     <row r="157" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="14" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B157" s="14" t="s">
         <v>174</v>
@@ -9572,17 +9587,15 @@
         <v>135</v>
       </c>
       <c r="D157" s="18" t="s">
-        <v>598</v>
-      </c>
-      <c r="E157" s="15"/>
+        <v>597</v>
+      </c>
+      <c r="E157" s="14"/>
       <c r="F157" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G157" s="15"/>
+      <c r="G157" s="14"/>
       <c r="H157" s="14"/>
-      <c r="I157" s="14" t="s">
-        <v>378</v>
-      </c>
+      <c r="I157" s="14"/>
       <c r="J157" s="14"/>
       <c r="K157" s="14"/>
       <c r="L157" s="14"/>
@@ -9612,7 +9625,7 @@
     </row>
     <row r="158" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="14" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B158" s="14" t="s">
         <v>174</v>
@@ -9621,16 +9634,16 @@
         <v>135</v>
       </c>
       <c r="D158" s="18" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="E158" s="15"/>
       <c r="F158" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G158" s="14"/>
+      <c r="G158" s="15"/>
       <c r="H158" s="14"/>
       <c r="I158" s="14" t="s">
-        <v>401</v>
+        <v>378</v>
       </c>
       <c r="J158" s="14"/>
       <c r="K158" s="14"/>
@@ -9661,7 +9674,7 @@
     </row>
     <row r="159" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="14" t="s">
-        <v>601</v>
+        <v>608</v>
       </c>
       <c r="B159" s="14" t="s">
         <v>174</v>
@@ -9670,7 +9683,7 @@
         <v>135</v>
       </c>
       <c r="D159" s="18" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="E159" s="15"/>
       <c r="F159" s="14" t="s">
@@ -9679,7 +9692,7 @@
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
       <c r="I159" s="14" t="s">
-        <v>126</v>
+        <v>401</v>
       </c>
       <c r="J159" s="14"/>
       <c r="K159" s="14"/>
@@ -9709,15 +9722,27 @@
       <c r="AI159" s="14"/>
     </row>
     <row r="160" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A160" s="14"/>
-      <c r="B160" s="14"/>
-      <c r="C160" s="14"/>
-      <c r="D160" s="15"/>
-      <c r="E160" s="14"/>
-      <c r="F160" s="14"/>
+      <c r="A160" s="14" t="s">
+        <v>601</v>
+      </c>
+      <c r="B160" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C160" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D160" s="18" t="s">
+        <v>596</v>
+      </c>
+      <c r="E160" s="15"/>
+      <c r="F160" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G160" s="14"/>
       <c r="H160" s="14"/>
-      <c r="I160" s="14"/>
+      <c r="I160" s="14" t="s">
+        <v>126</v>
+      </c>
       <c r="J160" s="14"/>
       <c r="K160" s="14"/>
       <c r="L160" s="14"/>
@@ -9726,7 +9751,7 @@
       <c r="O160" s="14"/>
       <c r="P160" s="14"/>
       <c r="Q160" s="14"/>
-      <c r="R160" s="15"/>
+      <c r="R160" s="14"/>
       <c r="S160" s="14"/>
       <c r="T160" s="14"/>
       <c r="U160" s="14"/>
@@ -9746,18 +9771,10 @@
       <c r="AI160" s="14"/>
     </row>
     <row r="161" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A161" s="14" t="s">
-        <v>488</v>
-      </c>
-      <c r="B161" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C161" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D161" s="18" t="s">
-        <v>489</v>
-      </c>
+      <c r="A161" s="14"/>
+      <c r="B161" s="14"/>
+      <c r="C161" s="14"/>
+      <c r="D161" s="15"/>
       <c r="E161" s="14"/>
       <c r="F161" s="14"/>
       <c r="G161" s="14"/>
@@ -9770,16 +9787,10 @@
       <c r="N161" s="14"/>
       <c r="O161" s="14"/>
       <c r="P161" s="14"/>
-      <c r="Q161" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="R161" s="14"/>
-      <c r="S161" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T161" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="Q161" s="14"/>
+      <c r="R161" s="15"/>
+      <c r="S161" s="14"/>
+      <c r="T161" s="14"/>
       <c r="U161" s="14"/>
       <c r="V161" s="14"/>
       <c r="W161" s="14"/>
@@ -9787,26 +9798,18 @@
       <c r="Y161" s="14"/>
       <c r="Z161" s="14"/>
       <c r="AA161" s="14"/>
-      <c r="AB161" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC161" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD161" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB161" s="14"/>
+      <c r="AC161" s="14"/>
+      <c r="AD161" s="14"/>
       <c r="AE161" s="27"/>
       <c r="AF161" s="14"/>
       <c r="AG161" s="14"/>
-      <c r="AH161" s="14" t="s">
-        <v>465</v>
-      </c>
+      <c r="AH161" s="14"/>
       <c r="AI161" s="14"/>
     </row>
     <row r="162" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="14" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B162" s="14" t="s">
         <v>174</v>
@@ -9815,7 +9818,7 @@
         <v>135</v>
       </c>
       <c r="D162" s="18" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="E162" s="14"/>
       <c r="F162" s="14"/>
@@ -9829,10 +9832,16 @@
       <c r="N162" s="14"/>
       <c r="O162" s="14"/>
       <c r="P162" s="14"/>
-      <c r="Q162" s="14"/>
+      <c r="Q162" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R162" s="14"/>
-      <c r="S162" s="14"/>
-      <c r="T162" s="14"/>
+      <c r="S162" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T162" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U162" s="14"/>
       <c r="V162" s="14"/>
       <c r="W162" s="14"/>
@@ -9852,12 +9861,14 @@
       <c r="AE162" s="27"/>
       <c r="AF162" s="14"/>
       <c r="AG162" s="14"/>
-      <c r="AH162" s="14"/>
+      <c r="AH162" s="14" t="s">
+        <v>465</v>
+      </c>
       <c r="AI162" s="14"/>
     </row>
     <row r="163" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="14" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="B163" s="14" t="s">
         <v>174</v>
@@ -9866,7 +9877,7 @@
         <v>135</v>
       </c>
       <c r="D163" s="18" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="E163" s="14"/>
       <c r="F163" s="14"/>
@@ -9892,25 +9903,23 @@
       <c r="Z163" s="14"/>
       <c r="AA163" s="14"/>
       <c r="AB163" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC163" s="14" t="s">
-        <v>457</v>
+        <v>393</v>
       </c>
       <c r="AD163" s="14" t="s">
-        <v>451</v>
+        <v>393</v>
       </c>
       <c r="AE163" s="27"/>
       <c r="AF163" s="14"/>
       <c r="AG163" s="14"/>
-      <c r="AH163" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH163" s="14"/>
       <c r="AI163" s="14"/>
     </row>
     <row r="164" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="14" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B164" s="14" t="s">
         <v>174</v>
@@ -9919,7 +9928,7 @@
         <v>135</v>
       </c>
       <c r="D164" s="18" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="E164" s="14"/>
       <c r="F164" s="14"/>
@@ -9933,16 +9942,10 @@
       <c r="N164" s="14"/>
       <c r="O164" s="14"/>
       <c r="P164" s="14"/>
-      <c r="Q164" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q164" s="14"/>
       <c r="R164" s="14"/>
-      <c r="S164" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T164" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S164" s="14"/>
+      <c r="T164" s="14"/>
       <c r="U164" s="14"/>
       <c r="V164" s="14"/>
       <c r="W164" s="14"/>
@@ -9962,14 +9965,14 @@
       <c r="AE164" s="27"/>
       <c r="AF164" s="14"/>
       <c r="AG164" s="14"/>
-      <c r="AH164" s="15" t="s">
-        <v>454</v>
+      <c r="AH164" s="14" t="s">
+        <v>458</v>
       </c>
       <c r="AI164" s="14"/>
     </row>
     <row r="165" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="14" t="s">
-        <v>539</v>
+        <v>490</v>
       </c>
       <c r="B165" s="14" t="s">
         <v>174</v>
@@ -9977,8 +9980,8 @@
       <c r="C165" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D165" s="23" t="s">
-        <v>540</v>
+      <c r="D165" s="18" t="s">
+        <v>491</v>
       </c>
       <c r="E165" s="14"/>
       <c r="F165" s="14"/>
@@ -9988,16 +9991,20 @@
       <c r="J165" s="14"/>
       <c r="K165" s="14"/>
       <c r="L165" s="14"/>
-      <c r="M165" s="20" t="s">
-        <v>609</v>
-      </c>
+      <c r="M165" s="14"/>
       <c r="N165" s="14"/>
       <c r="O165" s="14"/>
       <c r="P165" s="14"/>
-      <c r="Q165" s="14"/>
+      <c r="Q165" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R165" s="14"/>
-      <c r="S165" s="14"/>
-      <c r="T165" s="14"/>
+      <c r="S165" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T165" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U165" s="14"/>
       <c r="V165" s="14"/>
       <c r="W165" s="14"/>
@@ -10017,14 +10024,14 @@
       <c r="AE165" s="27"/>
       <c r="AF165" s="14"/>
       <c r="AG165" s="14"/>
-      <c r="AH165" s="14" t="s">
-        <v>458</v>
+      <c r="AH165" s="15" t="s">
+        <v>454</v>
       </c>
       <c r="AI165" s="14"/>
     </row>
     <row r="166" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="14" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="B166" s="14" t="s">
         <v>174</v>
@@ -10033,7 +10040,7 @@
         <v>135</v>
       </c>
       <c r="D166" s="23" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="E166" s="14"/>
       <c r="F166" s="14"/>
@@ -10044,7 +10051,7 @@
       <c r="K166" s="14"/>
       <c r="L166" s="14"/>
       <c r="M166" s="20" t="s">
-        <v>494</v>
+        <v>609</v>
       </c>
       <c r="N166" s="14"/>
       <c r="O166" s="14"/>
@@ -10061,23 +10068,25 @@
       <c r="Z166" s="14"/>
       <c r="AA166" s="14"/>
       <c r="AB166" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC166" s="14" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="AD166" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE166" s="27"/>
       <c r="AF166" s="14"/>
       <c r="AG166" s="14"/>
-      <c r="AH166" s="14"/>
+      <c r="AH166" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI166" s="14"/>
     </row>
     <row r="167" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="14" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B167" s="14" t="s">
         <v>174</v>
@@ -10086,7 +10095,7 @@
         <v>135</v>
       </c>
       <c r="D167" s="23" t="s">
-        <v>546</v>
+        <v>541</v>
       </c>
       <c r="E167" s="14"/>
       <c r="F167" s="14"/>
@@ -10114,25 +10123,23 @@
       <c r="Z167" s="14"/>
       <c r="AA167" s="14"/>
       <c r="AB167" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC167" s="14" t="s">
-        <v>457</v>
+        <v>427</v>
       </c>
       <c r="AD167" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE167" s="27"/>
       <c r="AF167" s="14"/>
       <c r="AG167" s="14"/>
-      <c r="AH167" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH167" s="14"/>
       <c r="AI167" s="14"/>
     </row>
     <row r="168" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="14" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="B168" s="14" t="s">
         <v>174</v>
@@ -10140,8 +10147,8 @@
       <c r="C168" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D168" s="18" t="s">
-        <v>548</v>
+      <c r="D168" s="23" t="s">
+        <v>546</v>
       </c>
       <c r="E168" s="14"/>
       <c r="F168" s="14"/>
@@ -10150,7 +10157,7 @@
       <c r="I168" s="14"/>
       <c r="J168" s="14"/>
       <c r="K168" s="14"/>
-      <c r="L168" s="31"/>
+      <c r="L168" s="14"/>
       <c r="M168" s="20" t="s">
         <v>494</v>
       </c>
@@ -10187,7 +10194,7 @@
     </row>
     <row r="169" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="14" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="B169" s="14" t="s">
         <v>174</v>
@@ -10196,7 +10203,7 @@
         <v>135</v>
       </c>
       <c r="D169" s="18" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="E169" s="14"/>
       <c r="F169" s="14"/>
@@ -10205,7 +10212,7 @@
       <c r="I169" s="14"/>
       <c r="J169" s="14"/>
       <c r="K169" s="14"/>
-      <c r="L169" s="14"/>
+      <c r="L169" s="31"/>
       <c r="M169" s="20" t="s">
         <v>494</v>
       </c>
@@ -10224,13 +10231,13 @@
       <c r="Z169" s="14"/>
       <c r="AA169" s="14"/>
       <c r="AB169" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC169" s="14" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="AD169" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE169" s="27"/>
       <c r="AF169" s="14"/>
@@ -10241,10 +10248,18 @@
       <c r="AI169" s="14"/>
     </row>
     <row r="170" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A170" s="14"/>
-      <c r="B170" s="14"/>
-      <c r="C170" s="14"/>
-      <c r="D170" s="18"/>
+      <c r="A170" s="14" t="s">
+        <v>550</v>
+      </c>
+      <c r="B170" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C170" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D170" s="18" t="s">
+        <v>551</v>
+      </c>
       <c r="E170" s="14"/>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -10253,7 +10268,9 @@
       <c r="J170" s="14"/>
       <c r="K170" s="14"/>
       <c r="L170" s="14"/>
-      <c r="M170" s="20"/>
+      <c r="M170" s="20" t="s">
+        <v>494</v>
+      </c>
       <c r="N170" s="14"/>
       <c r="O170" s="14"/>
       <c r="P170" s="14"/>
@@ -10268,28 +10285,28 @@
       <c r="Y170" s="14"/>
       <c r="Z170" s="14"/>
       <c r="AA170" s="14"/>
-      <c r="AB170" s="14"/>
-      <c r="AC170" s="14"/>
-      <c r="AD170" s="14"/>
+      <c r="AB170" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC170" s="14" t="s">
+        <v>427</v>
+      </c>
+      <c r="AD170" s="14" t="s">
+        <v>421</v>
+      </c>
       <c r="AE170" s="27"/>
       <c r="AF170" s="14"/>
       <c r="AG170" s="14"/>
-      <c r="AH170" s="14"/>
+      <c r="AH170" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI170" s="14"/>
     </row>
     <row r="171" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A171" s="14" t="s">
-        <v>554</v>
-      </c>
-      <c r="B171" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C171" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D171" s="18" t="s">
-        <v>566</v>
-      </c>
+      <c r="A171" s="14"/>
+      <c r="B171" s="14"/>
+      <c r="C171" s="14"/>
+      <c r="D171" s="18"/>
       <c r="E171" s="14"/>
       <c r="F171" s="14"/>
       <c r="G171" s="14"/>
@@ -10298,20 +10315,14 @@
       <c r="J171" s="14"/>
       <c r="K171" s="14"/>
       <c r="L171" s="14"/>
-      <c r="M171" s="14"/>
+      <c r="M171" s="20"/>
       <c r="N171" s="14"/>
       <c r="O171" s="14"/>
       <c r="P171" s="14"/>
-      <c r="Q171" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q171" s="14"/>
       <c r="R171" s="14"/>
-      <c r="S171" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T171" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S171" s="14"/>
+      <c r="T171" s="14"/>
       <c r="U171" s="14"/>
       <c r="V171" s="14"/>
       <c r="W171" s="14"/>
@@ -10319,26 +10330,18 @@
       <c r="Y171" s="14"/>
       <c r="Z171" s="14"/>
       <c r="AA171" s="14"/>
-      <c r="AB171" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC171" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD171" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB171" s="14"/>
+      <c r="AC171" s="14"/>
+      <c r="AD171" s="14"/>
       <c r="AE171" s="27"/>
       <c r="AF171" s="14"/>
       <c r="AG171" s="14"/>
-      <c r="AH171" s="14" t="s">
-        <v>465</v>
-      </c>
+      <c r="AH171" s="14"/>
       <c r="AI171" s="14"/>
     </row>
     <row r="172" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="14" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B172" s="14" t="s">
         <v>174</v>
@@ -10347,7 +10350,7 @@
         <v>135</v>
       </c>
       <c r="D172" s="18" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="E172" s="14"/>
       <c r="F172" s="14"/>
@@ -10361,10 +10364,16 @@
       <c r="N172" s="14"/>
       <c r="O172" s="14"/>
       <c r="P172" s="14"/>
-      <c r="Q172" s="14"/>
+      <c r="Q172" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R172" s="14"/>
-      <c r="S172" s="14"/>
-      <c r="T172" s="14"/>
+      <c r="S172" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T172" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U172" s="14"/>
       <c r="V172" s="14"/>
       <c r="W172" s="14"/>
@@ -10384,12 +10393,14 @@
       <c r="AE172" s="27"/>
       <c r="AF172" s="14"/>
       <c r="AG172" s="14"/>
-      <c r="AH172" s="14"/>
+      <c r="AH172" s="14" t="s">
+        <v>465</v>
+      </c>
       <c r="AI172" s="14"/>
     </row>
     <row r="173" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="14" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B173" s="14" t="s">
         <v>174</v>
@@ -10398,7 +10409,7 @@
         <v>135</v>
       </c>
       <c r="D173" s="18" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E173" s="14"/>
       <c r="F173" s="14"/>
@@ -10424,25 +10435,23 @@
       <c r="Z173" s="14"/>
       <c r="AA173" s="14"/>
       <c r="AB173" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC173" s="14" t="s">
-        <v>457</v>
+        <v>393</v>
       </c>
       <c r="AD173" s="14" t="s">
-        <v>451</v>
+        <v>393</v>
       </c>
       <c r="AE173" s="27"/>
       <c r="AF173" s="14"/>
       <c r="AG173" s="14"/>
-      <c r="AH173" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH173" s="14"/>
       <c r="AI173" s="14"/>
     </row>
     <row r="174" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="14" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B174" s="14" t="s">
         <v>174</v>
@@ -10451,7 +10460,7 @@
         <v>135</v>
       </c>
       <c r="D174" s="18" t="s">
-        <v>570</v>
+        <v>563</v>
       </c>
       <c r="E174" s="14"/>
       <c r="F174" s="14"/>
@@ -10465,16 +10474,10 @@
       <c r="N174" s="14"/>
       <c r="O174" s="14"/>
       <c r="P174" s="14"/>
-      <c r="Q174" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q174" s="14"/>
       <c r="R174" s="14"/>
-      <c r="S174" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T174" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S174" s="14"/>
+      <c r="T174" s="14"/>
       <c r="U174" s="14"/>
       <c r="V174" s="14"/>
       <c r="W174" s="14"/>
@@ -10494,14 +10497,14 @@
       <c r="AE174" s="27"/>
       <c r="AF174" s="14"/>
       <c r="AG174" s="14"/>
-      <c r="AH174" s="15" t="s">
-        <v>454</v>
+      <c r="AH174" s="14" t="s">
+        <v>458</v>
       </c>
       <c r="AI174" s="14"/>
     </row>
     <row r="175" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="14" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B175" s="14" t="s">
         <v>174</v>
@@ -10509,8 +10512,8 @@
       <c r="C175" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D175" s="23" t="s">
-        <v>571</v>
+      <c r="D175" s="18" t="s">
+        <v>570</v>
       </c>
       <c r="E175" s="14"/>
       <c r="F175" s="14"/>
@@ -10520,16 +10523,20 @@
       <c r="J175" s="14"/>
       <c r="K175" s="14"/>
       <c r="L175" s="14"/>
-      <c r="M175" s="30" t="s">
-        <v>580</v>
-      </c>
+      <c r="M175" s="14"/>
       <c r="N175" s="14"/>
       <c r="O175" s="14"/>
       <c r="P175" s="14"/>
-      <c r="Q175" s="14"/>
+      <c r="Q175" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R175" s="14"/>
-      <c r="S175" s="14"/>
-      <c r="T175" s="14"/>
+      <c r="S175" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T175" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U175" s="14"/>
       <c r="V175" s="14"/>
       <c r="W175" s="14"/>
@@ -10549,14 +10556,14 @@
       <c r="AE175" s="27"/>
       <c r="AF175" s="14"/>
       <c r="AG175" s="14"/>
-      <c r="AH175" s="14" t="s">
-        <v>458</v>
+      <c r="AH175" s="15" t="s">
+        <v>454</v>
       </c>
       <c r="AI175" s="14"/>
     </row>
     <row r="176" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="14" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B176" s="14" t="s">
         <v>174</v>
@@ -10565,7 +10572,7 @@
         <v>135</v>
       </c>
       <c r="D176" s="23" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="E176" s="14"/>
       <c r="F176" s="14"/>
@@ -10576,7 +10583,7 @@
       <c r="K176" s="14"/>
       <c r="L176" s="14"/>
       <c r="M176" s="30" t="s">
-        <v>549</v>
+        <v>580</v>
       </c>
       <c r="N176" s="14"/>
       <c r="O176" s="14"/>
@@ -10593,23 +10600,25 @@
       <c r="Z176" s="14"/>
       <c r="AA176" s="14"/>
       <c r="AB176" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC176" s="14" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="AD176" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE176" s="27"/>
       <c r="AF176" s="14"/>
       <c r="AG176" s="14"/>
-      <c r="AH176" s="14"/>
+      <c r="AH176" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI176" s="14"/>
     </row>
     <row r="177" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="14" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B177" s="14" t="s">
         <v>174</v>
@@ -10618,7 +10627,7 @@
         <v>135</v>
       </c>
       <c r="D177" s="23" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="E177" s="14"/>
       <c r="F177" s="14"/>
@@ -10628,7 +10637,7 @@
       <c r="J177" s="14"/>
       <c r="K177" s="14"/>
       <c r="L177" s="14"/>
-      <c r="M177" s="14" t="s">
+      <c r="M177" s="30" t="s">
         <v>549</v>
       </c>
       <c r="N177" s="14"/>
@@ -10646,25 +10655,23 @@
       <c r="Z177" s="14"/>
       <c r="AA177" s="14"/>
       <c r="AB177" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC177" s="14" t="s">
-        <v>457</v>
+        <v>427</v>
       </c>
       <c r="AD177" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE177" s="27"/>
       <c r="AF177" s="14"/>
       <c r="AG177" s="14"/>
-      <c r="AH177" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH177" s="14"/>
       <c r="AI177" s="14"/>
     </row>
     <row r="178" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="14" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B178" s="14" t="s">
         <v>174</v>
@@ -10672,8 +10679,8 @@
       <c r="C178" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D178" s="18" t="s">
-        <v>579</v>
+      <c r="D178" s="23" t="s">
+        <v>578</v>
       </c>
       <c r="E178" s="14"/>
       <c r="F178" s="14"/>
@@ -10701,13 +10708,13 @@
       <c r="Z178" s="14"/>
       <c r="AA178" s="14"/>
       <c r="AB178" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC178" s="14" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="AD178" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE178" s="27"/>
       <c r="AF178" s="14"/>
@@ -10719,7 +10726,7 @@
     </row>
     <row r="179" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="14" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B179" s="14" t="s">
         <v>174</v>
@@ -10728,7 +10735,7 @@
         <v>135</v>
       </c>
       <c r="D179" s="18" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E179" s="14"/>
       <c r="F179" s="14"/>
@@ -10737,8 +10744,8 @@
       <c r="I179" s="14"/>
       <c r="J179" s="14"/>
       <c r="K179" s="14"/>
-      <c r="L179" s="31"/>
-      <c r="M179" s="30" t="s">
+      <c r="L179" s="14"/>
+      <c r="M179" s="14" t="s">
         <v>549</v>
       </c>
       <c r="N179" s="14"/>
@@ -10756,13 +10763,13 @@
       <c r="Z179" s="14"/>
       <c r="AA179" s="14"/>
       <c r="AB179" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC179" s="14" t="s">
-        <v>457</v>
+        <v>427</v>
       </c>
       <c r="AD179" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE179" s="27"/>
       <c r="AF179" s="14"/>
@@ -10773,10 +10780,18 @@
       <c r="AI179" s="14"/>
     </row>
     <row r="180" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A180" s="14"/>
-      <c r="B180" s="14"/>
-      <c r="C180" s="14"/>
-      <c r="D180" s="15"/>
+      <c r="A180" s="14" t="s">
+        <v>562</v>
+      </c>
+      <c r="B180" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C180" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D180" s="18" t="s">
+        <v>575</v>
+      </c>
       <c r="E180" s="14"/>
       <c r="F180" s="14"/>
       <c r="G180" s="14"/>
@@ -10784,13 +10799,15 @@
       <c r="I180" s="14"/>
       <c r="J180" s="14"/>
       <c r="K180" s="14"/>
-      <c r="L180" s="14"/>
-      <c r="M180" s="14"/>
+      <c r="L180" s="31"/>
+      <c r="M180" s="30" t="s">
+        <v>549</v>
+      </c>
       <c r="N180" s="14"/>
       <c r="O180" s="14"/>
       <c r="P180" s="14"/>
       <c r="Q180" s="14"/>
-      <c r="R180" s="15"/>
+      <c r="R180" s="14"/>
       <c r="S180" s="14"/>
       <c r="T180" s="14"/>
       <c r="U180" s="14"/>
@@ -10800,46 +10817,42 @@
       <c r="Y180" s="14"/>
       <c r="Z180" s="14"/>
       <c r="AA180" s="14"/>
-      <c r="AB180" s="14"/>
-      <c r="AC180" s="14"/>
-      <c r="AD180" s="14"/>
+      <c r="AB180" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC180" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD180" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE180" s="27"/>
       <c r="AF180" s="14"/>
       <c r="AG180" s="14"/>
-      <c r="AH180" s="14"/>
+      <c r="AH180" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI180" s="14"/>
     </row>
     <row r="181" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A181" s="14" t="s">
-        <v>267</v>
-      </c>
-      <c r="B181" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C181" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D181" s="14"/>
+      <c r="A181" s="14"/>
+      <c r="B181" s="14"/>
+      <c r="C181" s="14"/>
+      <c r="D181" s="15"/>
       <c r="E181" s="14"/>
       <c r="F181" s="14"/>
       <c r="G181" s="14"/>
       <c r="H181" s="14"/>
       <c r="I181" s="14"/>
-      <c r="J181" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K181" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L181" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J181" s="14"/>
+      <c r="K181" s="14"/>
+      <c r="L181" s="14"/>
       <c r="M181" s="14"/>
       <c r="N181" s="14"/>
       <c r="O181" s="14"/>
       <c r="P181" s="14"/>
       <c r="Q181" s="14"/>
-      <c r="R181" s="14"/>
+      <c r="R181" s="15"/>
       <c r="S181" s="14"/>
       <c r="T181" s="14"/>
       <c r="U181" s="14"/>
@@ -10860,7 +10873,7 @@
     </row>
     <row r="182" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A182" s="14" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B182" s="14" t="s">
         <v>174</v>
@@ -10875,13 +10888,13 @@
       <c r="H182" s="14"/>
       <c r="I182" s="14"/>
       <c r="J182" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K182" s="15" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="L182" s="15" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="M182" s="14"/>
       <c r="N182" s="14"/>
@@ -10907,9 +10920,9 @@
       <c r="AH182" s="14"/>
       <c r="AI182" s="14"/>
     </row>
-    <row r="183" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A183" s="14" t="s">
-        <v>359</v>
+        <v>268</v>
       </c>
       <c r="B183" s="14" t="s">
         <v>174</v>
@@ -10917,9 +10930,36 @@
       <c r="C183" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O183" s="15" t="s">
-        <v>362</v>
-      </c>
+      <c r="D183" s="14"/>
+      <c r="E183" s="14"/>
+      <c r="F183" s="14"/>
+      <c r="G183" s="14"/>
+      <c r="H183" s="14"/>
+      <c r="I183" s="14"/>
+      <c r="J183" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K183" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L183" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M183" s="14"/>
+      <c r="N183" s="14"/>
+      <c r="O183" s="14"/>
+      <c r="P183" s="14"/>
+      <c r="Q183" s="14"/>
+      <c r="R183" s="14"/>
+      <c r="S183" s="14"/>
+      <c r="T183" s="14"/>
+      <c r="U183" s="14"/>
+      <c r="V183" s="14"/>
+      <c r="W183" s="14"/>
+      <c r="X183" s="14"/>
+      <c r="Y183" s="14"/>
+      <c r="Z183" s="14"/>
+      <c r="AA183" s="14"/>
       <c r="AB183" s="14"/>
       <c r="AC183" s="14"/>
       <c r="AD183" s="14"/>
@@ -10931,7 +10971,7 @@
     </row>
     <row r="184" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A184" s="14" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B184" s="14" t="s">
         <v>174</v>
@@ -10940,7 +10980,7 @@
         <v>135</v>
       </c>
       <c r="O184" s="15" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AB184" s="14"/>
       <c r="AC184" s="14"/>
@@ -10953,7 +10993,7 @@
     </row>
     <row r="185" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A185" s="14" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B185" s="14" t="s">
         <v>174</v>
@@ -10962,7 +11002,7 @@
         <v>135</v>
       </c>
       <c r="O185" s="15" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AB185" s="14"/>
       <c r="AC185" s="14"/>
@@ -10975,7 +11015,7 @@
     </row>
     <row r="186" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A186" s="14" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="B186" s="14" t="s">
         <v>174</v>
@@ -10983,8 +11023,8 @@
       <c r="C186" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M186" s="14" t="s">
-        <v>371</v>
+      <c r="O186" s="15" t="s">
+        <v>364</v>
       </c>
       <c r="AB186" s="14"/>
       <c r="AC186" s="14"/>
@@ -10996,6 +11036,18 @@
       <c r="AI186" s="14"/>
     </row>
     <row r="187" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A187" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B187" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C187" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M187" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB187" s="14"/>
       <c r="AC187" s="14"/>
       <c r="AD187" s="14"/>
@@ -12989,7 +13041,7 @@
       <c r="AB386" s="14"/>
       <c r="AC386" s="14"/>
       <c r="AD386" s="14"/>
-      <c r="AE386" s="14"/>
+      <c r="AE386" s="27"/>
       <c r="AF386" s="14"/>
       <c r="AG386" s="14"/>
       <c r="AH386" s="14"/>
@@ -13055,6 +13107,16 @@
       <c r="AH392" s="14"/>
       <c r="AI392" s="14"/>
     </row>
+    <row r="393" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB393" s="14"/>
+      <c r="AC393" s="14"/>
+      <c r="AD393" s="14"/>
+      <c r="AE393" s="14"/>
+      <c r="AF393" s="14"/>
+      <c r="AG393" s="14"/>
+      <c r="AH393" s="14"/>
+      <c r="AI393" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13064,7 +13126,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T185"/>
+  <dimension ref="A1:T186"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -17737,7 +17799,7 @@
         <v>530</v>
       </c>
       <c r="B148" s="30" t="s">
-        <v>494</v>
+        <v>549</v>
       </c>
       <c r="C148" s="15" t="s">
         <v>69</v>
@@ -19123,6 +19185,44 @@
       <c r="R185" s="14"/>
       <c r="S185" s="14"/>
       <c r="T185" s="14"/>
+    </row>
+    <row r="186" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="16" t="s">
+        <v>611</v>
+      </c>
+      <c r="B186" s="20" t="s">
+        <v>612</v>
+      </c>
+      <c r="C186" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D186" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="E186" s="14"/>
+      <c r="F186" s="14"/>
+      <c r="G186" s="14"/>
+      <c r="H186" s="14"/>
+      <c r="I186" s="14"/>
+      <c r="J186" s="14"/>
+      <c r="K186" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L186" s="14"/>
+      <c r="M186" s="14"/>
+      <c r="N186" s="14"/>
+      <c r="O186" s="14"/>
+      <c r="P186" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q186" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R186" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S186" s="14"/>
+      <c r="T186" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
Commit latest changes done for APC verify order reached to Manhattan
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01465413-FD2F-41C9-B73F-697DA4E27E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85158EE1-1FBF-4875-B2F4-9DFF9A19216E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2641" uniqueCount="613">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2665" uniqueCount="620">
   <si>
     <t>1</t>
   </si>
@@ -1867,6 +1867,27 @@
   </si>
   <si>
     <t>FG-002182-03</t>
+  </si>
+  <si>
+    <t>APC</t>
+  </si>
+  <si>
+    <t>MM1</t>
+  </si>
+  <si>
+    <t>972</t>
+  </si>
+  <si>
+    <t>APC_IBScenario001</t>
+  </si>
+  <si>
+    <t>APC_KelliScenario001</t>
+  </si>
+  <si>
+    <t>973</t>
+  </si>
+  <si>
+    <t>03P78-25</t>
   </si>
 </sst>
 </file>
@@ -2410,7 +2431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI393"/>
+  <dimension ref="A1:AI396"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -6677,7 +6698,7 @@
       <c r="B93" s="14"/>
       <c r="C93" s="14"/>
       <c r="D93" s="18"/>
-      <c r="E93" s="14"/>
+      <c r="E93" s="15"/>
       <c r="F93" s="14"/>
       <c r="G93" s="14"/>
       <c r="H93" s="14"/>
@@ -6710,30 +6731,26 @@
       <c r="AI93" s="14"/>
     </row>
     <row r="94" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="12" t="s">
-        <v>365</v>
-      </c>
-      <c r="B94" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C94" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="D94" s="18"/>
-      <c r="E94" s="14"/>
+      <c r="A94" s="14" t="s">
+        <v>617</v>
+      </c>
+      <c r="B94" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C94" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D94" s="18" t="s">
+        <v>618</v>
+      </c>
+      <c r="E94" s="15"/>
       <c r="F94" s="14"/>
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="14"/>
-      <c r="J94" s="13" t="s">
-        <v>405</v>
-      </c>
-      <c r="K94" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L94" s="14" t="s">
-        <v>406</v>
-      </c>
+      <c r="J94" s="14"/>
+      <c r="K94" s="14"/>
+      <c r="L94" s="14"/>
       <c r="M94" s="14"/>
       <c r="N94" s="14"/>
       <c r="O94" s="14"/>
@@ -6759,15 +6776,9 @@
       <c r="AI94" s="14"/>
     </row>
     <row r="95" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="12" t="s">
-        <v>366</v>
-      </c>
-      <c r="B95" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C95" s="12" t="s">
-        <v>135</v>
-      </c>
+      <c r="A95" s="14"/>
+      <c r="B95" s="14"/>
+      <c r="C95" s="14"/>
       <c r="D95" s="18"/>
       <c r="E95" s="14"/>
       <c r="F95" s="14"/>
@@ -6776,13 +6787,11 @@
       <c r="I95" s="14"/>
       <c r="J95" s="14"/>
       <c r="K95" s="14"/>
-      <c r="L95" s="12"/>
-      <c r="M95" s="12" t="s">
-        <v>398</v>
-      </c>
-      <c r="N95" s="12"/>
-      <c r="O95" s="12"/>
-      <c r="P95" s="12"/>
+      <c r="L95" s="14"/>
+      <c r="M95" s="14"/>
+      <c r="N95" s="14"/>
+      <c r="O95" s="14"/>
+      <c r="P95" s="14"/>
       <c r="Q95" s="14"/>
       <c r="R95" s="14"/>
       <c r="S95" s="14"/>
@@ -6805,7 +6814,7 @@
     </row>
     <row r="96" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="12" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B96" s="12" t="s">
         <v>107</v>
@@ -6819,15 +6828,19 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="14"/>
-      <c r="J96" s="14"/>
-      <c r="K96" s="14"/>
-      <c r="L96" s="12"/>
-      <c r="M96" s="12"/>
-      <c r="N96" s="12" t="s">
-        <v>410</v>
-      </c>
-      <c r="O96" s="12"/>
-      <c r="P96" s="12"/>
+      <c r="J96" s="13" t="s">
+        <v>405</v>
+      </c>
+      <c r="K96" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L96" s="14" t="s">
+        <v>406</v>
+      </c>
+      <c r="M96" s="14"/>
+      <c r="N96" s="14"/>
+      <c r="O96" s="14"/>
+      <c r="P96" s="14"/>
       <c r="Q96" s="14"/>
       <c r="R96" s="14"/>
       <c r="S96" s="14"/>
@@ -6850,7 +6863,7 @@
     </row>
     <row r="97" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B97" s="12" t="s">
         <v>107</v>
@@ -6867,11 +6880,11 @@
       <c r="J97" s="14"/>
       <c r="K97" s="14"/>
       <c r="L97" s="12"/>
-      <c r="M97" s="12"/>
+      <c r="M97" s="12" t="s">
+        <v>398</v>
+      </c>
       <c r="N97" s="12"/>
-      <c r="O97" s="12" t="s">
-        <v>407</v>
-      </c>
+      <c r="O97" s="12"/>
       <c r="P97" s="12"/>
       <c r="Q97" s="14"/>
       <c r="R97" s="14"/>
@@ -6895,7 +6908,7 @@
     </row>
     <row r="98" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="12" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B98" s="12" t="s">
         <v>107</v>
@@ -6913,11 +6926,11 @@
       <c r="K98" s="14"/>
       <c r="L98" s="12"/>
       <c r="M98" s="12"/>
-      <c r="N98" s="12"/>
+      <c r="N98" s="12" t="s">
+        <v>410</v>
+      </c>
       <c r="O98" s="12"/>
-      <c r="P98" s="13" t="s">
-        <v>408</v>
-      </c>
+      <c r="P98" s="12"/>
       <c r="Q98" s="14"/>
       <c r="R98" s="14"/>
       <c r="S98" s="14"/>
@@ -6939,10 +6952,16 @@
       <c r="AI98" s="14"/>
     </row>
     <row r="99" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="14"/>
-      <c r="B99" s="14"/>
-      <c r="C99" s="14"/>
-      <c r="D99" s="23"/>
+      <c r="A99" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="B99" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C99" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D99" s="18"/>
       <c r="E99" s="14"/>
       <c r="F99" s="14"/>
       <c r="G99" s="14"/>
@@ -6950,11 +6969,13 @@
       <c r="I99" s="14"/>
       <c r="J99" s="14"/>
       <c r="K99" s="14"/>
-      <c r="L99" s="14"/>
-      <c r="M99" s="14"/>
-      <c r="N99" s="14"/>
-      <c r="O99" s="14"/>
-      <c r="P99" s="14"/>
+      <c r="L99" s="12"/>
+      <c r="M99" s="12"/>
+      <c r="N99" s="12"/>
+      <c r="O99" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="P99" s="12"/>
       <c r="Q99" s="14"/>
       <c r="R99" s="14"/>
       <c r="S99" s="14"/>
@@ -6975,9 +6996,9 @@
       <c r="AH99" s="14"/>
       <c r="AI99" s="14"/>
     </row>
-    <row r="100" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="12" t="s">
-        <v>306</v>
+        <v>369</v>
       </c>
       <c r="B100" s="12" t="s">
         <v>107</v>
@@ -6985,113 +7006,81 @@
       <c r="C100" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="D100" s="12"/>
-      <c r="E100" s="12"/>
-      <c r="F100" s="12"/>
-      <c r="G100" s="12"/>
-      <c r="H100" s="12"/>
-      <c r="I100" s="12"/>
-      <c r="J100" s="12"/>
-      <c r="K100" s="12"/>
+      <c r="D100" s="18"/>
+      <c r="E100" s="14"/>
+      <c r="F100" s="14"/>
+      <c r="G100" s="14"/>
+      <c r="H100" s="14"/>
+      <c r="I100" s="14"/>
+      <c r="J100" s="14"/>
+      <c r="K100" s="14"/>
       <c r="L100" s="12"/>
       <c r="M100" s="12"/>
       <c r="N100" s="12"/>
       <c r="O100" s="12"/>
-      <c r="P100" s="12"/>
-      <c r="Q100" s="12"/>
-      <c r="R100" s="12"/>
-      <c r="S100" s="12"/>
-      <c r="T100" s="12"/>
-      <c r="U100" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="V100" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="W100" s="12" t="s">
-        <v>309</v>
-      </c>
-      <c r="X100" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="Y100" s="12" t="s">
-        <v>311</v>
-      </c>
-      <c r="Z100" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="AA100" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="AB100" s="12"/>
-      <c r="AC100" s="12"/>
-      <c r="AD100" s="12"/>
-      <c r="AE100" s="28"/>
-      <c r="AF100" s="12"/>
-      <c r="AG100" s="12"/>
-      <c r="AH100" s="12"/>
-      <c r="AI100" s="12"/>
-    </row>
-    <row r="101" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="12" t="s">
-        <v>312</v>
-      </c>
-      <c r="B101" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C101" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="D101" s="12"/>
-      <c r="E101" s="12"/>
-      <c r="F101" s="12"/>
-      <c r="G101" s="12"/>
-      <c r="H101" s="12"/>
-      <c r="I101" s="12"/>
-      <c r="J101" s="12"/>
-      <c r="K101" s="12"/>
-      <c r="L101" s="12"/>
-      <c r="M101" s="12"/>
-      <c r="N101" s="12"/>
-      <c r="O101" s="12"/>
-      <c r="P101" s="12"/>
-      <c r="Q101" s="12"/>
-      <c r="R101" s="12"/>
-      <c r="S101" s="12"/>
-      <c r="T101" s="12"/>
-      <c r="U101" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="V101" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="W101" s="12" t="s">
-        <v>309</v>
-      </c>
-      <c r="X101" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="Y101" s="12" t="s">
-        <v>311</v>
-      </c>
-      <c r="Z101" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="AA101" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="AB101" s="12"/>
-      <c r="AC101" s="12"/>
-      <c r="AD101" s="12"/>
-      <c r="AE101" s="28"/>
-      <c r="AF101" s="12"/>
-      <c r="AG101" s="12"/>
-      <c r="AH101" s="12"/>
-      <c r="AI101" s="12"/>
+      <c r="P100" s="13" t="s">
+        <v>408</v>
+      </c>
+      <c r="Q100" s="14"/>
+      <c r="R100" s="14"/>
+      <c r="S100" s="14"/>
+      <c r="T100" s="14"/>
+      <c r="U100" s="14"/>
+      <c r="V100" s="14"/>
+      <c r="W100" s="14"/>
+      <c r="X100" s="14"/>
+      <c r="Y100" s="14"/>
+      <c r="Z100" s="14"/>
+      <c r="AA100" s="14"/>
+      <c r="AB100" s="14"/>
+      <c r="AC100" s="14"/>
+      <c r="AD100" s="14"/>
+      <c r="AE100" s="27"/>
+      <c r="AF100" s="14"/>
+      <c r="AG100" s="14"/>
+      <c r="AH100" s="14"/>
+      <c r="AI100" s="14"/>
+    </row>
+    <row r="101" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="14"/>
+      <c r="B101" s="14"/>
+      <c r="C101" s="14"/>
+      <c r="D101" s="23"/>
+      <c r="E101" s="14"/>
+      <c r="F101" s="14"/>
+      <c r="G101" s="14"/>
+      <c r="H101" s="14"/>
+      <c r="I101" s="14"/>
+      <c r="J101" s="14"/>
+      <c r="K101" s="14"/>
+      <c r="L101" s="14"/>
+      <c r="M101" s="14"/>
+      <c r="N101" s="14"/>
+      <c r="O101" s="14"/>
+      <c r="P101" s="14"/>
+      <c r="Q101" s="14"/>
+      <c r="R101" s="14"/>
+      <c r="S101" s="14"/>
+      <c r="T101" s="14"/>
+      <c r="U101" s="14"/>
+      <c r="V101" s="14"/>
+      <c r="W101" s="14"/>
+      <c r="X101" s="14"/>
+      <c r="Y101" s="14"/>
+      <c r="Z101" s="14"/>
+      <c r="AA101" s="14"/>
+      <c r="AB101" s="14"/>
+      <c r="AC101" s="14"/>
+      <c r="AD101" s="14"/>
+      <c r="AE101" s="27"/>
+      <c r="AF101" s="14"/>
+      <c r="AG101" s="14"/>
+      <c r="AH101" s="14"/>
+      <c r="AI101" s="14"/>
     </row>
     <row r="102" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="12" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="B102" s="12" t="s">
         <v>107</v>
@@ -7116,22 +7105,24 @@
       <c r="R102" s="12"/>
       <c r="S102" s="12"/>
       <c r="T102" s="12"/>
-      <c r="U102" s="12" t="s">
+      <c r="U102" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="V102" s="12" t="s">
-        <v>314</v>
+      <c r="V102" s="13" t="s">
+        <v>308</v>
       </c>
       <c r="W102" s="12" t="s">
         <v>309</v>
       </c>
       <c r="X102" s="12" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="Y102" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="Z102" s="12"/>
+      <c r="Z102" s="12" t="s">
+        <v>107</v>
+      </c>
       <c r="AA102" s="12" t="s">
         <v>135</v>
       </c>
@@ -7146,7 +7137,7 @@
     </row>
     <row r="103" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="12" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="B103" s="12" t="s">
         <v>107</v>
@@ -7175,7 +7166,7 @@
         <v>307</v>
       </c>
       <c r="V103" s="13" t="s">
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="W103" s="12" t="s">
         <v>309</v>
@@ -7189,7 +7180,9 @@
       <c r="Z103" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="AA103" s="12"/>
+      <c r="AA103" s="12" t="s">
+        <v>135</v>
+      </c>
       <c r="AB103" s="12"/>
       <c r="AC103" s="12"/>
       <c r="AD103" s="12"/>
@@ -7201,7 +7194,7 @@
     </row>
     <row r="104" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="12" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="B104" s="12" t="s">
         <v>107</v>
@@ -7230,18 +7223,18 @@
         <v>307</v>
       </c>
       <c r="V104" s="12" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="W104" s="12" t="s">
         <v>309</v>
       </c>
-      <c r="X104" s="12"/>
+      <c r="X104" s="12" t="s">
+        <v>315</v>
+      </c>
       <c r="Y104" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="Z104" s="12" t="s">
-        <v>107</v>
-      </c>
+      <c r="Z104" s="12"/>
       <c r="AA104" s="12" t="s">
         <v>135</v>
       </c>
@@ -7256,7 +7249,7 @@
     </row>
     <row r="105" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="12" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B105" s="12" t="s">
         <v>107</v>
@@ -7281,15 +7274,17 @@
       <c r="R105" s="12"/>
       <c r="S105" s="12"/>
       <c r="T105" s="12"/>
-      <c r="U105" s="12"/>
-      <c r="V105" s="12" t="s">
-        <v>319</v>
+      <c r="U105" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="V105" s="13" t="s">
+        <v>317</v>
       </c>
       <c r="W105" s="12" t="s">
         <v>309</v>
       </c>
       <c r="X105" s="12" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="Y105" s="12" t="s">
         <v>311</v>
@@ -7297,9 +7292,7 @@
       <c r="Z105" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="AA105" s="12" t="s">
-        <v>135</v>
-      </c>
+      <c r="AA105" s="12"/>
       <c r="AB105" s="12"/>
       <c r="AC105" s="12"/>
       <c r="AD105" s="12"/>
@@ -7311,7 +7304,7 @@
     </row>
     <row r="106" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="12" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="B106" s="12" t="s">
         <v>107</v>
@@ -7336,18 +7329,16 @@
       <c r="R106" s="12"/>
       <c r="S106" s="12"/>
       <c r="T106" s="12"/>
-      <c r="U106" s="13" t="s">
-        <v>322</v>
-      </c>
-      <c r="V106" s="13" t="s">
-        <v>323</v>
-      </c>
-      <c r="W106" s="13" t="s">
+      <c r="U106" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="V106" s="12" t="s">
+        <v>319</v>
+      </c>
+      <c r="W106" s="12" t="s">
         <v>309</v>
       </c>
-      <c r="X106" s="12" t="s">
-        <v>310</v>
-      </c>
+      <c r="X106" s="12"/>
       <c r="Y106" s="12" t="s">
         <v>311</v>
       </c>
@@ -7368,7 +7359,7 @@
     </row>
     <row r="107" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="12" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B107" s="12" t="s">
         <v>107</v>
@@ -7393,17 +7384,15 @@
       <c r="R107" s="12"/>
       <c r="S107" s="12"/>
       <c r="T107" s="12"/>
-      <c r="U107" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="V107" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="W107" s="13" t="s">
-        <v>325</v>
+      <c r="U107" s="12"/>
+      <c r="V107" s="12" t="s">
+        <v>319</v>
+      </c>
+      <c r="W107" s="12" t="s">
+        <v>309</v>
       </c>
       <c r="X107" s="12" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="Y107" s="12" t="s">
         <v>311</v>
@@ -7425,7 +7414,7 @@
     </row>
     <row r="108" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="12" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="B108" s="12" t="s">
         <v>107</v>
@@ -7450,26 +7439,26 @@
       <c r="R108" s="12"/>
       <c r="S108" s="12"/>
       <c r="T108" s="12"/>
-      <c r="U108" s="12" t="s">
-        <v>307</v>
-      </c>
-      <c r="V108" s="12" t="s">
-        <v>308</v>
-      </c>
-      <c r="W108" s="12" t="s">
+      <c r="U108" s="13" t="s">
+        <v>322</v>
+      </c>
+      <c r="V108" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="W108" s="13" t="s">
         <v>309</v>
       </c>
       <c r="X108" s="12" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="Y108" s="12" t="s">
         <v>311</v>
       </c>
       <c r="Z108" s="12" t="s">
-        <v>174</v>
+        <v>107</v>
       </c>
       <c r="AA108" s="12" t="s">
-        <v>327</v>
+        <v>135</v>
       </c>
       <c r="AB108" s="12"/>
       <c r="AC108" s="12"/>
@@ -7482,7 +7471,7 @@
     </row>
     <row r="109" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="12" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B109" s="12" t="s">
         <v>107</v>
@@ -7507,17 +7496,17 @@
       <c r="R109" s="12"/>
       <c r="S109" s="12"/>
       <c r="T109" s="12"/>
-      <c r="U109" s="12" t="s">
+      <c r="U109" s="13" t="s">
         <v>307</v>
       </c>
       <c r="V109" s="13" t="s">
-        <v>329</v>
-      </c>
-      <c r="W109" s="12" t="s">
-        <v>309</v>
+        <v>308</v>
+      </c>
+      <c r="W109" s="13" t="s">
+        <v>325</v>
       </c>
       <c r="X109" s="12" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="Y109" s="12" t="s">
         <v>311</v>
@@ -7539,7 +7528,7 @@
     </row>
     <row r="110" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="12" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B110" s="12" t="s">
         <v>107</v>
@@ -7568,7 +7557,7 @@
         <v>307</v>
       </c>
       <c r="V110" s="12" t="s">
-        <v>331</v>
+        <v>308</v>
       </c>
       <c r="W110" s="12" t="s">
         <v>309</v>
@@ -7580,10 +7569,10 @@
         <v>311</v>
       </c>
       <c r="Z110" s="12" t="s">
-        <v>107</v>
+        <v>174</v>
       </c>
       <c r="AA110" s="12" t="s">
-        <v>135</v>
+        <v>327</v>
       </c>
       <c r="AB110" s="12"/>
       <c r="AC110" s="12"/>
@@ -7596,7 +7585,7 @@
     </row>
     <row r="111" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="12" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B111" s="12" t="s">
         <v>107</v>
@@ -7624,8 +7613,8 @@
       <c r="U111" s="12" t="s">
         <v>307</v>
       </c>
-      <c r="V111" s="12" t="s">
-        <v>333</v>
+      <c r="V111" s="13" t="s">
+        <v>329</v>
       </c>
       <c r="W111" s="12" t="s">
         <v>309</v>
@@ -7637,7 +7626,7 @@
         <v>311</v>
       </c>
       <c r="Z111" s="12" t="s">
-        <v>327</v>
+        <v>107</v>
       </c>
       <c r="AA111" s="12" t="s">
         <v>135</v>
@@ -7653,7 +7642,7 @@
     </row>
     <row r="112" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="12" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="B112" s="12" t="s">
         <v>107</v>
@@ -7682,13 +7671,13 @@
         <v>307</v>
       </c>
       <c r="V112" s="12" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="W112" s="12" t="s">
         <v>309</v>
       </c>
       <c r="X112" s="12" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="Y112" s="12" t="s">
         <v>311</v>
@@ -7709,9 +7698,15 @@
       <c r="AI112" s="12"/>
     </row>
     <row r="113" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="12"/>
-      <c r="B113" s="12"/>
-      <c r="C113" s="12"/>
+      <c r="A113" s="12" t="s">
+        <v>332</v>
+      </c>
+      <c r="B113" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C113" s="12" t="s">
+        <v>135</v>
+      </c>
       <c r="D113" s="12"/>
       <c r="E113" s="12"/>
       <c r="F113" s="12"/>
@@ -7729,13 +7724,27 @@
       <c r="R113" s="12"/>
       <c r="S113" s="12"/>
       <c r="T113" s="12"/>
-      <c r="U113" s="12"/>
-      <c r="V113" s="12"/>
-      <c r="W113" s="12"/>
-      <c r="X113" s="12"/>
-      <c r="Y113" s="12"/>
-      <c r="Z113" s="12"/>
-      <c r="AA113" s="12"/>
+      <c r="U113" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="V113" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="W113" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="X113" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="Y113" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="Z113" s="12" t="s">
+        <v>327</v>
+      </c>
+      <c r="AA113" s="12" t="s">
+        <v>135</v>
+      </c>
       <c r="AB113" s="12"/>
       <c r="AC113" s="12"/>
       <c r="AD113" s="12"/>
@@ -7746,9 +7755,15 @@
       <c r="AI113" s="12"/>
     </row>
     <row r="114" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="12"/>
-      <c r="B114" s="12"/>
-      <c r="C114" s="12"/>
+      <c r="A114" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="B114" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C114" s="12" t="s">
+        <v>135</v>
+      </c>
       <c r="D114" s="12"/>
       <c r="E114" s="12"/>
       <c r="F114" s="12"/>
@@ -7766,13 +7781,27 @@
       <c r="R114" s="12"/>
       <c r="S114" s="12"/>
       <c r="T114" s="12"/>
-      <c r="U114" s="12"/>
-      <c r="V114" s="12"/>
-      <c r="W114" s="12"/>
-      <c r="X114" s="12"/>
-      <c r="Y114" s="12"/>
-      <c r="Z114" s="12"/>
-      <c r="AA114" s="12"/>
+      <c r="U114" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="V114" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="W114" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="X114" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="Y114" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="Z114" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="AA114" s="12" t="s">
+        <v>135</v>
+      </c>
       <c r="AB114" s="12"/>
       <c r="AC114" s="12"/>
       <c r="AD114" s="12"/>
@@ -7782,65 +7811,83 @@
       <c r="AH114" s="12"/>
       <c r="AI114" s="12"/>
     </row>
-    <row r="115" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A115" s="14" t="s">
-        <v>243</v>
-      </c>
-      <c r="B115" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C115" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D115" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="F115" s="14" t="s">
-        <v>403</v>
-      </c>
-      <c r="R115" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB115" s="14"/>
-      <c r="AC115" s="14"/>
-      <c r="AD115" s="14"/>
-      <c r="AE115" s="27"/>
-      <c r="AF115" s="14"/>
-      <c r="AG115" s="14"/>
-      <c r="AH115" s="14"/>
-      <c r="AI115" s="14"/>
-    </row>
-    <row r="116" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A116" s="14" t="s">
-        <v>244</v>
-      </c>
-      <c r="B116" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C116" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D116" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="F116" s="14" t="s">
-        <v>403</v>
-      </c>
-      <c r="R116" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB116" s="14"/>
-      <c r="AC116" s="14"/>
-      <c r="AD116" s="14"/>
-      <c r="AE116" s="27"/>
-      <c r="AF116" s="14"/>
-      <c r="AG116" s="14"/>
-      <c r="AH116" s="14"/>
-      <c r="AI116" s="14"/>
+    <row r="115" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="12"/>
+      <c r="B115" s="12"/>
+      <c r="C115" s="12"/>
+      <c r="D115" s="12"/>
+      <c r="E115" s="12"/>
+      <c r="F115" s="12"/>
+      <c r="G115" s="12"/>
+      <c r="H115" s="12"/>
+      <c r="I115" s="12"/>
+      <c r="J115" s="12"/>
+      <c r="K115" s="12"/>
+      <c r="L115" s="12"/>
+      <c r="M115" s="12"/>
+      <c r="N115" s="12"/>
+      <c r="O115" s="12"/>
+      <c r="P115" s="12"/>
+      <c r="Q115" s="12"/>
+      <c r="R115" s="12"/>
+      <c r="S115" s="12"/>
+      <c r="T115" s="12"/>
+      <c r="U115" s="12"/>
+      <c r="V115" s="12"/>
+      <c r="W115" s="12"/>
+      <c r="X115" s="12"/>
+      <c r="Y115" s="12"/>
+      <c r="Z115" s="12"/>
+      <c r="AA115" s="12"/>
+      <c r="AB115" s="12"/>
+      <c r="AC115" s="12"/>
+      <c r="AD115" s="12"/>
+      <c r="AE115" s="28"/>
+      <c r="AF115" s="12"/>
+      <c r="AG115" s="12"/>
+      <c r="AH115" s="12"/>
+      <c r="AI115" s="12"/>
+    </row>
+    <row r="116" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="12"/>
+      <c r="B116" s="12"/>
+      <c r="C116" s="12"/>
+      <c r="D116" s="12"/>
+      <c r="E116" s="12"/>
+      <c r="F116" s="12"/>
+      <c r="G116" s="12"/>
+      <c r="H116" s="12"/>
+      <c r="I116" s="12"/>
+      <c r="J116" s="12"/>
+      <c r="K116" s="12"/>
+      <c r="L116" s="12"/>
+      <c r="M116" s="12"/>
+      <c r="N116" s="12"/>
+      <c r="O116" s="12"/>
+      <c r="P116" s="12"/>
+      <c r="Q116" s="12"/>
+      <c r="R116" s="12"/>
+      <c r="S116" s="12"/>
+      <c r="T116" s="12"/>
+      <c r="U116" s="12"/>
+      <c r="V116" s="12"/>
+      <c r="W116" s="12"/>
+      <c r="X116" s="12"/>
+      <c r="Y116" s="12"/>
+      <c r="Z116" s="12"/>
+      <c r="AA116" s="12"/>
+      <c r="AB116" s="12"/>
+      <c r="AC116" s="12"/>
+      <c r="AD116" s="12"/>
+      <c r="AE116" s="28"/>
+      <c r="AF116" s="12"/>
+      <c r="AG116" s="12"/>
+      <c r="AH116" s="12"/>
+      <c r="AI116" s="12"/>
     </row>
     <row r="117" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A117" s="14" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B117" s="14" t="s">
         <v>174</v>
@@ -7849,7 +7896,7 @@
         <v>135</v>
       </c>
       <c r="D117" s="15" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F117" s="14" t="s">
         <v>403</v>
@@ -7868,7 +7915,7 @@
     </row>
     <row r="118" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A118" s="14" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B118" s="14" t="s">
         <v>174</v>
@@ -7877,7 +7924,7 @@
         <v>135</v>
       </c>
       <c r="D118" s="15" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F118" s="14" t="s">
         <v>403</v>
@@ -7896,7 +7943,7 @@
     </row>
     <row r="119" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A119" s="14" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B119" s="14" t="s">
         <v>174</v>
@@ -7905,7 +7952,7 @@
         <v>135</v>
       </c>
       <c r="D119" s="15" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F119" s="14" t="s">
         <v>403</v>
@@ -7924,7 +7971,7 @@
     </row>
     <row r="120" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A120" s="14" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B120" s="14" t="s">
         <v>174</v>
@@ -7933,7 +7980,7 @@
         <v>135</v>
       </c>
       <c r="D120" s="15" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="F120" s="14" t="s">
         <v>403</v>
@@ -7952,7 +7999,7 @@
     </row>
     <row r="121" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A121" s="14" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B121" s="14" t="s">
         <v>174</v>
@@ -7961,13 +8008,13 @@
         <v>135</v>
       </c>
       <c r="D121" s="15" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="F121" s="14" t="s">
         <v>403</v>
       </c>
       <c r="R121" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AB121" s="14"/>
       <c r="AC121" s="14"/>
@@ -7978,9 +8025,9 @@
       <c r="AH121" s="14"/>
       <c r="AI121" s="14"/>
     </row>
-    <row r="122" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A122" s="14" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B122" s="14" t="s">
         <v>174</v>
@@ -7989,33 +8036,14 @@
         <v>135</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>236</v>
-      </c>
-      <c r="E122" s="14"/>
+        <v>185</v>
+      </c>
       <c r="F122" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G122" s="14"/>
-      <c r="H122" s="14"/>
-      <c r="I122" s="14"/>
-      <c r="J122" s="14"/>
-      <c r="K122" s="14"/>
-      <c r="L122" s="14"/>
-      <c r="M122" s="14"/>
-      <c r="N122" s="14"/>
-      <c r="O122" s="14"/>
-      <c r="P122" s="14"/>
-      <c r="Q122" s="14"/>
-      <c r="R122" s="15"/>
-      <c r="S122" s="14"/>
-      <c r="T122" s="14"/>
-      <c r="U122" s="14"/>
-      <c r="V122" s="14"/>
-      <c r="W122" s="14"/>
-      <c r="X122" s="14"/>
-      <c r="Y122" s="14"/>
-      <c r="Z122" s="14"/>
-      <c r="AA122" s="14"/>
+      <c r="R122" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="AB122" s="14"/>
       <c r="AC122" s="14"/>
       <c r="AD122" s="14"/>
@@ -8025,9 +8053,9 @@
       <c r="AH122" s="14"/>
       <c r="AI122" s="14"/>
     </row>
-    <row r="123" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A123" s="14" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B123" s="14" t="s">
         <v>174</v>
@@ -8036,33 +8064,14 @@
         <v>135</v>
       </c>
       <c r="D123" s="15" t="s">
-        <v>237</v>
-      </c>
-      <c r="E123" s="14"/>
+        <v>185</v>
+      </c>
       <c r="F123" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G123" s="14"/>
-      <c r="H123" s="14"/>
-      <c r="I123" s="14"/>
-      <c r="J123" s="14"/>
-      <c r="K123" s="14"/>
-      <c r="L123" s="14"/>
-      <c r="M123" s="14"/>
-      <c r="N123" s="14"/>
-      <c r="O123" s="14"/>
-      <c r="P123" s="14"/>
-      <c r="Q123" s="14"/>
-      <c r="R123" s="15"/>
-      <c r="S123" s="14"/>
-      <c r="T123" s="14"/>
-      <c r="U123" s="14"/>
-      <c r="V123" s="14"/>
-      <c r="W123" s="14"/>
-      <c r="X123" s="14"/>
-      <c r="Y123" s="14"/>
-      <c r="Z123" s="14"/>
-      <c r="AA123" s="14"/>
+      <c r="R123" s="15" t="s">
+        <v>2</v>
+      </c>
       <c r="AB123" s="14"/>
       <c r="AC123" s="14"/>
       <c r="AD123" s="14"/>
@@ -8072,9 +8081,9 @@
       <c r="AH123" s="14"/>
       <c r="AI123" s="14"/>
     </row>
-    <row r="124" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="14" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B124" s="14" t="s">
         <v>174</v>
@@ -8083,12 +8092,33 @@
         <v>135</v>
       </c>
       <c r="D124" s="15" t="s">
-        <v>238</v>
-      </c>
+        <v>236</v>
+      </c>
+      <c r="E124" s="14"/>
       <c r="F124" s="14" t="s">
         <v>403</v>
       </c>
+      <c r="G124" s="14"/>
+      <c r="H124" s="14"/>
+      <c r="I124" s="14"/>
+      <c r="J124" s="14"/>
+      <c r="K124" s="14"/>
+      <c r="L124" s="14"/>
+      <c r="M124" s="14"/>
+      <c r="N124" s="14"/>
+      <c r="O124" s="14"/>
+      <c r="P124" s="14"/>
+      <c r="Q124" s="14"/>
       <c r="R124" s="15"/>
+      <c r="S124" s="14"/>
+      <c r="T124" s="14"/>
+      <c r="U124" s="14"/>
+      <c r="V124" s="14"/>
+      <c r="W124" s="14"/>
+      <c r="X124" s="14"/>
+      <c r="Y124" s="14"/>
+      <c r="Z124" s="14"/>
+      <c r="AA124" s="14"/>
       <c r="AB124" s="14"/>
       <c r="AC124" s="14"/>
       <c r="AD124" s="14"/>
@@ -8098,9 +8128,9 @@
       <c r="AH124" s="14"/>
       <c r="AI124" s="14"/>
     </row>
-    <row r="125" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="14" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B125" s="14" t="s">
         <v>174</v>
@@ -8109,12 +8139,33 @@
         <v>135</v>
       </c>
       <c r="D125" s="15" t="s">
-        <v>239</v>
-      </c>
+        <v>237</v>
+      </c>
+      <c r="E125" s="14"/>
       <c r="F125" s="14" t="s">
         <v>403</v>
       </c>
+      <c r="G125" s="14"/>
+      <c r="H125" s="14"/>
+      <c r="I125" s="14"/>
+      <c r="J125" s="14"/>
+      <c r="K125" s="14"/>
+      <c r="L125" s="14"/>
+      <c r="M125" s="14"/>
+      <c r="N125" s="14"/>
+      <c r="O125" s="14"/>
+      <c r="P125" s="14"/>
+      <c r="Q125" s="14"/>
       <c r="R125" s="15"/>
+      <c r="S125" s="14"/>
+      <c r="T125" s="14"/>
+      <c r="U125" s="14"/>
+      <c r="V125" s="14"/>
+      <c r="W125" s="14"/>
+      <c r="X125" s="14"/>
+      <c r="Y125" s="14"/>
+      <c r="Z125" s="14"/>
+      <c r="AA125" s="14"/>
       <c r="AB125" s="14"/>
       <c r="AC125" s="14"/>
       <c r="AD125" s="14"/>
@@ -8126,7 +8177,7 @@
     </row>
     <row r="126" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A126" s="14" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B126" s="14" t="s">
         <v>174</v>
@@ -8135,7 +8186,7 @@
         <v>135</v>
       </c>
       <c r="D126" s="15" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="F126" s="14" t="s">
         <v>403</v>
@@ -8152,7 +8203,7 @@
     </row>
     <row r="127" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A127" s="14" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B127" s="14" t="s">
         <v>174</v>
@@ -8160,15 +8211,13 @@
       <c r="C127" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D127" s="16" t="s">
-        <v>257</v>
+      <c r="D127" s="15" t="s">
+        <v>239</v>
       </c>
       <c r="F127" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="R127" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R127" s="15"/>
       <c r="AB127" s="14"/>
       <c r="AC127" s="14"/>
       <c r="AD127" s="14"/>
@@ -8180,7 +8229,7 @@
     </row>
     <row r="128" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A128" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B128" s="14" t="s">
         <v>174</v>
@@ -8189,14 +8238,12 @@
         <v>135</v>
       </c>
       <c r="D128" s="15" t="s">
-        <v>277</v>
+        <v>240</v>
       </c>
       <c r="F128" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="R128" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R128" s="15"/>
       <c r="AB128" s="14"/>
       <c r="AC128" s="14"/>
       <c r="AD128" s="14"/>
@@ -8206,9 +8253,9 @@
       <c r="AH128" s="14"/>
       <c r="AI128" s="14"/>
     </row>
-    <row r="129" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A129" s="14" t="s">
-        <v>278</v>
+        <v>255</v>
       </c>
       <c r="B129" s="14" t="s">
         <v>174</v>
@@ -8216,36 +8263,15 @@
       <c r="C129" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D129" s="15" t="s">
-        <v>279</v>
-      </c>
-      <c r="E129" s="14"/>
+      <c r="D129" s="16" t="s">
+        <v>257</v>
+      </c>
       <c r="F129" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G129" s="14"/>
-      <c r="H129" s="14"/>
-      <c r="I129" s="14"/>
-      <c r="J129" s="14"/>
-      <c r="K129" s="14"/>
-      <c r="L129" s="14"/>
-      <c r="M129" s="14"/>
-      <c r="N129" s="14"/>
-      <c r="O129" s="14"/>
-      <c r="P129" s="14"/>
-      <c r="Q129" s="14"/>
       <c r="R129" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="S129" s="14"/>
-      <c r="T129" s="14"/>
-      <c r="U129" s="14"/>
-      <c r="V129" s="14"/>
-      <c r="W129" s="14"/>
-      <c r="X129" s="14"/>
-      <c r="Y129" s="14"/>
-      <c r="Z129" s="14"/>
-      <c r="AA129" s="14"/>
       <c r="AB129" s="14"/>
       <c r="AC129" s="14"/>
       <c r="AD129" s="14"/>
@@ -8255,9 +8281,9 @@
       <c r="AH129" s="14"/>
       <c r="AI129" s="14"/>
     </row>
-    <row r="130" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A130" s="14" t="s">
-        <v>285</v>
+        <v>256</v>
       </c>
       <c r="B130" s="14" t="s">
         <v>174</v>
@@ -8266,35 +8292,14 @@
         <v>135</v>
       </c>
       <c r="D130" s="15" t="s">
-        <v>286</v>
-      </c>
-      <c r="E130" s="14"/>
+        <v>277</v>
+      </c>
       <c r="F130" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G130" s="14"/>
-      <c r="H130" s="14"/>
-      <c r="I130" s="14"/>
-      <c r="J130" s="14"/>
-      <c r="K130" s="14"/>
-      <c r="L130" s="14"/>
-      <c r="M130" s="14"/>
-      <c r="N130" s="14"/>
-      <c r="O130" s="14"/>
-      <c r="P130" s="14"/>
-      <c r="Q130" s="14"/>
       <c r="R130" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="S130" s="14"/>
-      <c r="T130" s="14"/>
-      <c r="U130" s="14"/>
-      <c r="V130" s="14"/>
-      <c r="W130" s="14"/>
-      <c r="X130" s="14"/>
-      <c r="Y130" s="14"/>
-      <c r="Z130" s="14"/>
-      <c r="AA130" s="14"/>
+        <v>0</v>
+      </c>
       <c r="AB130" s="14"/>
       <c r="AC130" s="14"/>
       <c r="AD130" s="14"/>
@@ -8306,7 +8311,7 @@
     </row>
     <row r="131" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="14" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="B131" s="14" t="s">
         <v>174</v>
@@ -8315,7 +8320,7 @@
         <v>135</v>
       </c>
       <c r="D131" s="15" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="E131" s="14"/>
       <c r="F131" s="14" t="s">
@@ -8355,7 +8360,7 @@
     </row>
     <row r="132" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="14" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="B132" s="14" t="s">
         <v>174</v>
@@ -8364,7 +8369,7 @@
         <v>135</v>
       </c>
       <c r="D132" s="15" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E132" s="14"/>
       <c r="F132" s="14" t="s">
@@ -8382,7 +8387,7 @@
       <c r="P132" s="14"/>
       <c r="Q132" s="14"/>
       <c r="R132" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S132" s="14"/>
       <c r="T132" s="14"/>
@@ -8404,7 +8409,7 @@
     </row>
     <row r="133" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="14" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="B133" s="14" t="s">
         <v>174</v>
@@ -8413,7 +8418,7 @@
         <v>135</v>
       </c>
       <c r="D133" s="15" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
       <c r="E133" s="14"/>
       <c r="F133" s="14" t="s">
@@ -8431,7 +8436,7 @@
       <c r="P133" s="14"/>
       <c r="Q133" s="14"/>
       <c r="R133" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S133" s="14"/>
       <c r="T133" s="14"/>
@@ -8453,7 +8458,7 @@
     </row>
     <row r="134" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="14" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="B134" s="14" t="s">
         <v>174</v>
@@ -8462,7 +8467,7 @@
         <v>135</v>
       </c>
       <c r="D134" s="15" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="E134" s="14"/>
       <c r="F134" s="14" t="s">
@@ -8502,7 +8507,7 @@
     </row>
     <row r="135" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="14" t="s">
-        <v>373</v>
+        <v>292</v>
       </c>
       <c r="B135" s="14" t="s">
         <v>174</v>
@@ -8511,7 +8516,7 @@
         <v>135</v>
       </c>
       <c r="D135" s="15" t="s">
-        <v>372</v>
+        <v>293</v>
       </c>
       <c r="E135" s="14"/>
       <c r="F135" s="14" t="s">
@@ -8519,9 +8524,7 @@
       </c>
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
-      <c r="I135" s="14" t="s">
-        <v>126</v>
-      </c>
+      <c r="I135" s="14"/>
       <c r="J135" s="14"/>
       <c r="K135" s="14"/>
       <c r="L135" s="14"/>
@@ -8530,7 +8533,9 @@
       <c r="O135" s="14"/>
       <c r="P135" s="14"/>
       <c r="Q135" s="14"/>
-      <c r="R135" s="15"/>
+      <c r="R135" s="15" t="s">
+        <v>2</v>
+      </c>
       <c r="S135" s="14"/>
       <c r="T135" s="14"/>
       <c r="U135" s="14"/>
@@ -8551,7 +8556,7 @@
     </row>
     <row r="136" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="14" t="s">
-        <v>375</v>
+        <v>294</v>
       </c>
       <c r="B136" s="14" t="s">
         <v>174</v>
@@ -8560,7 +8565,7 @@
         <v>135</v>
       </c>
       <c r="D136" s="15" t="s">
-        <v>374</v>
+        <v>295</v>
       </c>
       <c r="E136" s="14"/>
       <c r="F136" s="14" t="s">
@@ -8568,9 +8573,7 @@
       </c>
       <c r="G136" s="14"/>
       <c r="H136" s="14"/>
-      <c r="I136" s="14" t="s">
-        <v>379</v>
-      </c>
+      <c r="I136" s="14"/>
       <c r="J136" s="14"/>
       <c r="K136" s="14"/>
       <c r="L136" s="14"/>
@@ -8579,7 +8582,9 @@
       <c r="O136" s="14"/>
       <c r="P136" s="14"/>
       <c r="Q136" s="14"/>
-      <c r="R136" s="15"/>
+      <c r="R136" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S136" s="14"/>
       <c r="T136" s="14"/>
       <c r="U136" s="14"/>
@@ -8600,7 +8605,7 @@
     </row>
     <row r="137" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="14" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="B137" s="14" t="s">
         <v>174</v>
@@ -8609,7 +8614,7 @@
         <v>135</v>
       </c>
       <c r="D137" s="15" t="s">
-        <v>384</v>
+        <v>372</v>
       </c>
       <c r="E137" s="14"/>
       <c r="F137" s="14" t="s">
@@ -8618,7 +8623,7 @@
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
       <c r="I137" s="14" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J137" s="14"/>
       <c r="K137" s="14"/>
@@ -8649,7 +8654,7 @@
     </row>
     <row r="138" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="14" t="s">
-        <v>383</v>
+        <v>375</v>
       </c>
       <c r="B138" s="14" t="s">
         <v>174</v>
@@ -8658,7 +8663,7 @@
         <v>135</v>
       </c>
       <c r="D138" s="15" t="s">
-        <v>385</v>
+        <v>374</v>
       </c>
       <c r="E138" s="14"/>
       <c r="F138" s="14" t="s">
@@ -8667,7 +8672,7 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="14" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="J138" s="14"/>
       <c r="K138" s="14"/>
@@ -8698,7 +8703,7 @@
     </row>
     <row r="139" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="14" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="B139" s="14" t="s">
         <v>174</v>
@@ -8707,7 +8712,7 @@
         <v>135</v>
       </c>
       <c r="D139" s="15" t="s">
-        <v>179</v>
+        <v>384</v>
       </c>
       <c r="E139" s="14"/>
       <c r="F139" s="14" t="s">
@@ -8715,7 +8720,9 @@
       </c>
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
-      <c r="I139" s="14"/>
+      <c r="I139" s="14" t="s">
+        <v>125</v>
+      </c>
       <c r="J139" s="14"/>
       <c r="K139" s="14"/>
       <c r="L139" s="14"/>
@@ -8745,7 +8752,7 @@
     </row>
     <row r="140" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="14" t="s">
-        <v>500</v>
+        <v>383</v>
       </c>
       <c r="B140" s="14" t="s">
         <v>174</v>
@@ -8753,17 +8760,17 @@
       <c r="C140" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D140" s="18" t="s">
-        <v>501</v>
-      </c>
-      <c r="E140" s="15"/>
+      <c r="D140" s="15" t="s">
+        <v>385</v>
+      </c>
+      <c r="E140" s="14"/>
       <c r="F140" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="14" t="s">
-        <v>128</v>
+        <v>381</v>
       </c>
       <c r="J140" s="14"/>
       <c r="K140" s="14"/>
@@ -8773,7 +8780,7 @@
       <c r="O140" s="14"/>
       <c r="P140" s="14"/>
       <c r="Q140" s="14"/>
-      <c r="R140" s="14"/>
+      <c r="R140" s="15"/>
       <c r="S140" s="14"/>
       <c r="T140" s="14"/>
       <c r="U140" s="14"/>
@@ -8786,17 +8793,15 @@
       <c r="AB140" s="14"/>
       <c r="AC140" s="14"/>
       <c r="AD140" s="14"/>
-      <c r="AE140" s="27" t="s">
-        <v>415</v>
-      </c>
+      <c r="AE140" s="27"/>
       <c r="AF140" s="14"/>
       <c r="AG140" s="14"/>
       <c r="AH140" s="14"/>
       <c r="AI140" s="14"/>
     </row>
     <row r="141" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="15" t="s">
-        <v>502</v>
+      <c r="A141" s="14" t="s">
+        <v>390</v>
       </c>
       <c r="B141" s="14" t="s">
         <v>174</v>
@@ -8804,18 +8809,16 @@
       <c r="C141" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D141" s="18" t="s">
-        <v>503</v>
-      </c>
-      <c r="E141" s="15"/>
+      <c r="D141" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="E141" s="14"/>
       <c r="F141" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G141" s="15"/>
+      <c r="G141" s="14"/>
       <c r="H141" s="14"/>
-      <c r="I141" s="14" t="s">
-        <v>504</v>
-      </c>
+      <c r="I141" s="14"/>
       <c r="J141" s="14"/>
       <c r="K141" s="14"/>
       <c r="L141" s="14"/>
@@ -8824,7 +8827,7 @@
       <c r="O141" s="14"/>
       <c r="P141" s="14"/>
       <c r="Q141" s="14"/>
-      <c r="R141" s="14"/>
+      <c r="R141" s="15"/>
       <c r="S141" s="14"/>
       <c r="T141" s="14"/>
       <c r="U141" s="14"/>
@@ -8844,8 +8847,8 @@
       <c r="AI141" s="14"/>
     </row>
     <row r="142" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A142" s="15" t="s">
-        <v>505</v>
+      <c r="A142" s="14" t="s">
+        <v>500</v>
       </c>
       <c r="B142" s="14" t="s">
         <v>174</v>
@@ -8854,15 +8857,17 @@
         <v>135</v>
       </c>
       <c r="D142" s="18" t="s">
-        <v>506</v>
-      </c>
-      <c r="E142" s="14"/>
+        <v>501</v>
+      </c>
+      <c r="E142" s="15"/>
       <c r="F142" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
-      <c r="I142" s="14"/>
+      <c r="I142" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J142" s="14"/>
       <c r="K142" s="14"/>
       <c r="L142" s="14"/>
@@ -8884,7 +8889,9 @@
       <c r="AB142" s="14"/>
       <c r="AC142" s="14"/>
       <c r="AD142" s="14"/>
-      <c r="AE142" s="27"/>
+      <c r="AE142" s="27" t="s">
+        <v>415</v>
+      </c>
       <c r="AF142" s="14"/>
       <c r="AG142" s="14"/>
       <c r="AH142" s="14"/>
@@ -8892,7 +8899,7 @@
     </row>
     <row r="143" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="15" t="s">
-        <v>507</v>
+        <v>502</v>
       </c>
       <c r="B143" s="14" t="s">
         <v>174</v>
@@ -8901,15 +8908,17 @@
         <v>135</v>
       </c>
       <c r="D143" s="18" t="s">
-        <v>508</v>
-      </c>
-      <c r="E143" s="14"/>
+        <v>503</v>
+      </c>
+      <c r="E143" s="15"/>
       <c r="F143" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G143" s="14"/>
+      <c r="G143" s="15"/>
       <c r="H143" s="14"/>
-      <c r="I143" s="14"/>
+      <c r="I143" s="14" t="s">
+        <v>504</v>
+      </c>
       <c r="J143" s="14"/>
       <c r="K143" s="14"/>
       <c r="L143" s="14"/>
@@ -8939,7 +8948,7 @@
     </row>
     <row r="144" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="15" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
       <c r="B144" s="14" t="s">
         <v>174</v>
@@ -8948,17 +8957,15 @@
         <v>135</v>
       </c>
       <c r="D144" s="18" t="s">
-        <v>513</v>
-      </c>
-      <c r="E144" s="15"/>
+        <v>506</v>
+      </c>
+      <c r="E144" s="14"/>
       <c r="F144" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G144" s="15"/>
+      <c r="G144" s="14"/>
       <c r="H144" s="14"/>
-      <c r="I144" s="14" t="s">
-        <v>378</v>
-      </c>
+      <c r="I144" s="14"/>
       <c r="J144" s="14"/>
       <c r="K144" s="14"/>
       <c r="L144" s="14"/>
@@ -8988,7 +8995,7 @@
     </row>
     <row r="145" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="15" t="s">
-        <v>519</v>
+        <v>507</v>
       </c>
       <c r="B145" s="14" t="s">
         <v>174</v>
@@ -8997,15 +9004,13 @@
         <v>135</v>
       </c>
       <c r="D145" s="18" t="s">
-        <v>520</v>
-      </c>
-      <c r="E145" s="15"/>
-      <c r="F145" s="15" t="s">
-        <v>388</v>
-      </c>
-      <c r="G145" s="15" t="s">
-        <v>3</v>
-      </c>
+        <v>508</v>
+      </c>
+      <c r="E145" s="14"/>
+      <c r="F145" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="G145" s="14"/>
       <c r="H145" s="14"/>
       <c r="I145" s="14"/>
       <c r="J145" s="14"/>
@@ -9037,7 +9042,7 @@
     </row>
     <row r="146" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="15" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
       <c r="B146" s="14" t="s">
         <v>174</v>
@@ -9046,16 +9051,16 @@
         <v>135</v>
       </c>
       <c r="D146" s="18" t="s">
-        <v>522</v>
+        <v>513</v>
       </c>
       <c r="E146" s="15"/>
       <c r="F146" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G146" s="14"/>
+      <c r="G146" s="15"/>
       <c r="H146" s="14"/>
       <c r="I146" s="14" t="s">
-        <v>128</v>
+        <v>378</v>
       </c>
       <c r="J146" s="14"/>
       <c r="K146" s="14"/>
@@ -9078,9 +9083,7 @@
       <c r="AB146" s="14"/>
       <c r="AC146" s="14"/>
       <c r="AD146" s="14"/>
-      <c r="AE146" s="27" t="s">
-        <v>415</v>
-      </c>
+      <c r="AE146" s="27"/>
       <c r="AF146" s="14"/>
       <c r="AG146" s="14"/>
       <c r="AH146" s="14"/>
@@ -9088,7 +9091,7 @@
     </row>
     <row r="147" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="15" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="B147" s="14" t="s">
         <v>174</v>
@@ -9097,17 +9100,17 @@
         <v>135</v>
       </c>
       <c r="D147" s="18" t="s">
-        <v>526</v>
+        <v>520</v>
       </c>
       <c r="E147" s="15"/>
-      <c r="F147" s="14" t="s">
-        <v>403</v>
-      </c>
-      <c r="G147" s="14"/>
+      <c r="F147" s="15" t="s">
+        <v>388</v>
+      </c>
+      <c r="G147" s="15" t="s">
+        <v>3</v>
+      </c>
       <c r="H147" s="14"/>
-      <c r="I147" s="14" t="s">
-        <v>401</v>
-      </c>
+      <c r="I147" s="14"/>
       <c r="J147" s="14"/>
       <c r="K147" s="14"/>
       <c r="L147" s="14"/>
@@ -9137,7 +9140,7 @@
     </row>
     <row r="148" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="15" t="s">
-        <v>528</v>
+        <v>521</v>
       </c>
       <c r="B148" s="14" t="s">
         <v>174</v>
@@ -9146,7 +9149,7 @@
         <v>135</v>
       </c>
       <c r="D148" s="18" t="s">
-        <v>527</v>
+        <v>522</v>
       </c>
       <c r="E148" s="15"/>
       <c r="F148" s="14" t="s">
@@ -9155,7 +9158,7 @@
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
       <c r="I148" s="14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="J148" s="14"/>
       <c r="K148" s="14"/>
@@ -9178,15 +9181,17 @@
       <c r="AB148" s="14"/>
       <c r="AC148" s="14"/>
       <c r="AD148" s="14"/>
-      <c r="AE148" s="27"/>
+      <c r="AE148" s="27" t="s">
+        <v>415</v>
+      </c>
       <c r="AF148" s="14"/>
       <c r="AG148" s="14"/>
       <c r="AH148" s="14"/>
       <c r="AI148" s="14"/>
     </row>
     <row r="149" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A149" s="14" t="s">
-        <v>533</v>
+      <c r="A149" s="15" t="s">
+        <v>523</v>
       </c>
       <c r="B149" s="14" t="s">
         <v>174</v>
@@ -9194,16 +9199,18 @@
       <c r="C149" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D149" s="15" t="s">
-        <v>531</v>
-      </c>
-      <c r="E149" s="14"/>
+      <c r="D149" s="18" t="s">
+        <v>526</v>
+      </c>
+      <c r="E149" s="15"/>
       <c r="F149" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
-      <c r="I149" s="14"/>
+      <c r="I149" s="14" t="s">
+        <v>401</v>
+      </c>
       <c r="J149" s="14"/>
       <c r="K149" s="14"/>
       <c r="L149" s="14"/>
@@ -9212,9 +9219,7 @@
       <c r="O149" s="14"/>
       <c r="P149" s="14"/>
       <c r="Q149" s="14"/>
-      <c r="R149" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R149" s="14"/>
       <c r="S149" s="14"/>
       <c r="T149" s="14"/>
       <c r="U149" s="14"/>
@@ -9235,7 +9240,7 @@
     </row>
     <row r="150" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="15" t="s">
-        <v>534</v>
+        <v>528</v>
       </c>
       <c r="B150" s="14" t="s">
         <v>174</v>
@@ -9244,16 +9249,16 @@
         <v>135</v>
       </c>
       <c r="D150" s="18" t="s">
-        <v>535</v>
+        <v>527</v>
       </c>
       <c r="E150" s="15"/>
       <c r="F150" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G150" s="15"/>
+      <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="14" t="s">
-        <v>378</v>
+        <v>126</v>
       </c>
       <c r="J150" s="14"/>
       <c r="K150" s="14"/>
@@ -9284,7 +9289,7 @@
     </row>
     <row r="151" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="14" t="s">
-        <v>581</v>
+        <v>533</v>
       </c>
       <c r="B151" s="14" t="s">
         <v>174</v>
@@ -9293,7 +9298,7 @@
         <v>135</v>
       </c>
       <c r="D151" s="15" t="s">
-        <v>582</v>
+        <v>531</v>
       </c>
       <c r="E151" s="14"/>
       <c r="F151" s="14" t="s">
@@ -9332,8 +9337,8 @@
       <c r="AI151" s="14"/>
     </row>
     <row r="152" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="14" t="s">
-        <v>602</v>
+      <c r="A152" s="15" t="s">
+        <v>534</v>
       </c>
       <c r="B152" s="14" t="s">
         <v>174</v>
@@ -9341,16 +9346,18 @@
       <c r="C152" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D152" s="15" t="s">
-        <v>583</v>
-      </c>
-      <c r="E152" s="14"/>
+      <c r="D152" s="18" t="s">
+        <v>535</v>
+      </c>
+      <c r="E152" s="15"/>
       <c r="F152" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G152" s="14"/>
+      <c r="G152" s="15"/>
       <c r="H152" s="14"/>
-      <c r="I152" s="14"/>
+      <c r="I152" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J152" s="14"/>
       <c r="K152" s="14"/>
       <c r="L152" s="14"/>
@@ -9359,9 +9366,7 @@
       <c r="O152" s="14"/>
       <c r="P152" s="14"/>
       <c r="Q152" s="14"/>
-      <c r="R152" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R152" s="14"/>
       <c r="S152" s="14"/>
       <c r="T152" s="14"/>
       <c r="U152" s="14"/>
@@ -9382,7 +9387,7 @@
     </row>
     <row r="153" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="14" t="s">
-        <v>603</v>
+        <v>581</v>
       </c>
       <c r="B153" s="14" t="s">
         <v>174</v>
@@ -9391,7 +9396,7 @@
         <v>135</v>
       </c>
       <c r="D153" s="15" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="E153" s="14"/>
       <c r="F153" s="14" t="s">
@@ -9431,7 +9436,7 @@
     </row>
     <row r="154" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="14" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="B154" s="14" t="s">
         <v>174</v>
@@ -9439,18 +9444,16 @@
       <c r="C154" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D154" s="18" t="s">
-        <v>587</v>
-      </c>
-      <c r="E154" s="15"/>
+      <c r="D154" s="15" t="s">
+        <v>583</v>
+      </c>
+      <c r="E154" s="14"/>
       <c r="F154" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G154" s="14"/>
       <c r="H154" s="14"/>
-      <c r="I154" s="14" t="s">
-        <v>128</v>
-      </c>
+      <c r="I154" s="14"/>
       <c r="J154" s="14"/>
       <c r="K154" s="14"/>
       <c r="L154" s="14"/>
@@ -9459,7 +9462,9 @@
       <c r="O154" s="14"/>
       <c r="P154" s="14"/>
       <c r="Q154" s="14"/>
-      <c r="R154" s="14"/>
+      <c r="R154" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S154" s="14"/>
       <c r="T154" s="14"/>
       <c r="U154" s="14"/>
@@ -9472,9 +9477,7 @@
       <c r="AB154" s="14"/>
       <c r="AC154" s="14"/>
       <c r="AD154" s="14"/>
-      <c r="AE154" s="27" t="s">
-        <v>415</v>
-      </c>
+      <c r="AE154" s="27"/>
       <c r="AF154" s="14"/>
       <c r="AG154" s="14"/>
       <c r="AH154" s="14"/>
@@ -9482,7 +9485,7 @@
     </row>
     <row r="155" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="14" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="B155" s="14" t="s">
         <v>174</v>
@@ -9490,18 +9493,16 @@
       <c r="C155" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D155" s="18" t="s">
-        <v>588</v>
-      </c>
-      <c r="E155" s="15"/>
+      <c r="D155" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="E155" s="14"/>
       <c r="F155" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G155" s="15"/>
+      <c r="G155" s="14"/>
       <c r="H155" s="14"/>
-      <c r="I155" s="14" t="s">
-        <v>504</v>
-      </c>
+      <c r="I155" s="14"/>
       <c r="J155" s="14"/>
       <c r="K155" s="14"/>
       <c r="L155" s="14"/>
@@ -9510,7 +9511,9 @@
       <c r="O155" s="14"/>
       <c r="P155" s="14"/>
       <c r="Q155" s="14"/>
-      <c r="R155" s="14"/>
+      <c r="R155" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S155" s="14"/>
       <c r="T155" s="14"/>
       <c r="U155" s="14"/>
@@ -9531,7 +9534,7 @@
     </row>
     <row r="156" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="14" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B156" s="14" t="s">
         <v>174</v>
@@ -9540,15 +9543,17 @@
         <v>135</v>
       </c>
       <c r="D156" s="18" t="s">
-        <v>589</v>
-      </c>
-      <c r="E156" s="14"/>
+        <v>587</v>
+      </c>
+      <c r="E156" s="15"/>
       <c r="F156" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
-      <c r="I156" s="14"/>
+      <c r="I156" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J156" s="14"/>
       <c r="K156" s="14"/>
       <c r="L156" s="14"/>
@@ -9570,7 +9575,9 @@
       <c r="AB156" s="14"/>
       <c r="AC156" s="14"/>
       <c r="AD156" s="14"/>
-      <c r="AE156" s="27"/>
+      <c r="AE156" s="27" t="s">
+        <v>415</v>
+      </c>
       <c r="AF156" s="14"/>
       <c r="AG156" s="14"/>
       <c r="AH156" s="14"/>
@@ -9578,7 +9585,7 @@
     </row>
     <row r="157" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="14" t="s">
-        <v>606</v>
+        <v>600</v>
       </c>
       <c r="B157" s="14" t="s">
         <v>174</v>
@@ -9587,15 +9594,17 @@
         <v>135</v>
       </c>
       <c r="D157" s="18" t="s">
-        <v>597</v>
-      </c>
-      <c r="E157" s="14"/>
+        <v>588</v>
+      </c>
+      <c r="E157" s="15"/>
       <c r="F157" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G157" s="14"/>
+      <c r="G157" s="15"/>
       <c r="H157" s="14"/>
-      <c r="I157" s="14"/>
+      <c r="I157" s="14" t="s">
+        <v>504</v>
+      </c>
       <c r="J157" s="14"/>
       <c r="K157" s="14"/>
       <c r="L157" s="14"/>
@@ -9625,7 +9634,7 @@
     </row>
     <row r="158" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="14" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B158" s="14" t="s">
         <v>174</v>
@@ -9634,17 +9643,15 @@
         <v>135</v>
       </c>
       <c r="D158" s="18" t="s">
-        <v>598</v>
-      </c>
-      <c r="E158" s="15"/>
+        <v>589</v>
+      </c>
+      <c r="E158" s="14"/>
       <c r="F158" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G158" s="15"/>
+      <c r="G158" s="14"/>
       <c r="H158" s="14"/>
-      <c r="I158" s="14" t="s">
-        <v>378</v>
-      </c>
+      <c r="I158" s="14"/>
       <c r="J158" s="14"/>
       <c r="K158" s="14"/>
       <c r="L158" s="14"/>
@@ -9674,7 +9681,7 @@
     </row>
     <row r="159" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="14" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="B159" s="14" t="s">
         <v>174</v>
@@ -9683,17 +9690,15 @@
         <v>135</v>
       </c>
       <c r="D159" s="18" t="s">
-        <v>599</v>
-      </c>
-      <c r="E159" s="15"/>
+        <v>597</v>
+      </c>
+      <c r="E159" s="14"/>
       <c r="F159" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
-      <c r="I159" s="14" t="s">
-        <v>401</v>
-      </c>
+      <c r="I159" s="14"/>
       <c r="J159" s="14"/>
       <c r="K159" s="14"/>
       <c r="L159" s="14"/>
@@ -9723,7 +9728,7 @@
     </row>
     <row r="160" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="14" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="B160" s="14" t="s">
         <v>174</v>
@@ -9732,16 +9737,16 @@
         <v>135</v>
       </c>
       <c r="D160" s="18" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="E160" s="15"/>
       <c r="F160" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G160" s="14"/>
+      <c r="G160" s="15"/>
       <c r="H160" s="14"/>
       <c r="I160" s="14" t="s">
-        <v>126</v>
+        <v>378</v>
       </c>
       <c r="J160" s="14"/>
       <c r="K160" s="14"/>
@@ -9771,15 +9776,27 @@
       <c r="AI160" s="14"/>
     </row>
     <row r="161" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A161" s="14"/>
-      <c r="B161" s="14"/>
-      <c r="C161" s="14"/>
-      <c r="D161" s="15"/>
-      <c r="E161" s="14"/>
-      <c r="F161" s="14"/>
+      <c r="A161" s="14" t="s">
+        <v>608</v>
+      </c>
+      <c r="B161" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C161" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D161" s="18" t="s">
+        <v>599</v>
+      </c>
+      <c r="E161" s="15"/>
+      <c r="F161" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G161" s="14"/>
       <c r="H161" s="14"/>
-      <c r="I161" s="14"/>
+      <c r="I161" s="14" t="s">
+        <v>401</v>
+      </c>
       <c r="J161" s="14"/>
       <c r="K161" s="14"/>
       <c r="L161" s="14"/>
@@ -9788,7 +9805,7 @@
       <c r="O161" s="14"/>
       <c r="P161" s="14"/>
       <c r="Q161" s="14"/>
-      <c r="R161" s="15"/>
+      <c r="R161" s="14"/>
       <c r="S161" s="14"/>
       <c r="T161" s="14"/>
       <c r="U161" s="14"/>
@@ -9809,7 +9826,7 @@
     </row>
     <row r="162" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="14" t="s">
-        <v>488</v>
+        <v>601</v>
       </c>
       <c r="B162" s="14" t="s">
         <v>174</v>
@@ -9818,13 +9835,17 @@
         <v>135</v>
       </c>
       <c r="D162" s="18" t="s">
-        <v>489</v>
-      </c>
-      <c r="E162" s="14"/>
-      <c r="F162" s="14"/>
+        <v>596</v>
+      </c>
+      <c r="E162" s="15"/>
+      <c r="F162" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
-      <c r="I162" s="14"/>
+      <c r="I162" s="14" t="s">
+        <v>126</v>
+      </c>
       <c r="J162" s="14"/>
       <c r="K162" s="14"/>
       <c r="L162" s="14"/>
@@ -9832,16 +9853,10 @@
       <c r="N162" s="14"/>
       <c r="O162" s="14"/>
       <c r="P162" s="14"/>
-      <c r="Q162" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q162" s="14"/>
       <c r="R162" s="14"/>
-      <c r="S162" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T162" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S162" s="14"/>
+      <c r="T162" s="14"/>
       <c r="U162" s="14"/>
       <c r="V162" s="14"/>
       <c r="W162" s="14"/>
@@ -9849,36 +9864,20 @@
       <c r="Y162" s="14"/>
       <c r="Z162" s="14"/>
       <c r="AA162" s="14"/>
-      <c r="AB162" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC162" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD162" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB162" s="14"/>
+      <c r="AC162" s="14"/>
+      <c r="AD162" s="14"/>
       <c r="AE162" s="27"/>
       <c r="AF162" s="14"/>
       <c r="AG162" s="14"/>
-      <c r="AH162" s="14" t="s">
-        <v>465</v>
-      </c>
+      <c r="AH162" s="14"/>
       <c r="AI162" s="14"/>
     </row>
     <row r="163" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A163" s="14" t="s">
-        <v>486</v>
-      </c>
-      <c r="B163" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C163" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D163" s="18" t="s">
-        <v>487</v>
-      </c>
+      <c r="A163" s="14"/>
+      <c r="B163" s="14"/>
+      <c r="C163" s="14"/>
+      <c r="D163" s="15"/>
       <c r="E163" s="14"/>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -9892,7 +9891,7 @@
       <c r="O163" s="14"/>
       <c r="P163" s="14"/>
       <c r="Q163" s="14"/>
-      <c r="R163" s="14"/>
+      <c r="R163" s="15"/>
       <c r="S163" s="14"/>
       <c r="T163" s="14"/>
       <c r="U163" s="14"/>
@@ -9902,15 +9901,9 @@
       <c r="Y163" s="14"/>
       <c r="Z163" s="14"/>
       <c r="AA163" s="14"/>
-      <c r="AB163" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC163" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD163" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB163" s="14"/>
+      <c r="AC163" s="14"/>
+      <c r="AD163" s="14"/>
       <c r="AE163" s="27"/>
       <c r="AF163" s="14"/>
       <c r="AG163" s="14"/>
@@ -9919,7 +9912,7 @@
     </row>
     <row r="164" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="14" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="B164" s="14" t="s">
         <v>174</v>
@@ -9928,7 +9921,7 @@
         <v>135</v>
       </c>
       <c r="D164" s="18" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="E164" s="14"/>
       <c r="F164" s="14"/>
@@ -9942,10 +9935,16 @@
       <c r="N164" s="14"/>
       <c r="O164" s="14"/>
       <c r="P164" s="14"/>
-      <c r="Q164" s="14"/>
+      <c r="Q164" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R164" s="14"/>
-      <c r="S164" s="14"/>
-      <c r="T164" s="14"/>
+      <c r="S164" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T164" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U164" s="14"/>
       <c r="V164" s="14"/>
       <c r="W164" s="14"/>
@@ -9954,25 +9953,25 @@
       <c r="Z164" s="14"/>
       <c r="AA164" s="14"/>
       <c r="AB164" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC164" s="14" t="s">
-        <v>457</v>
+        <v>393</v>
       </c>
       <c r="AD164" s="14" t="s">
-        <v>451</v>
+        <v>393</v>
       </c>
       <c r="AE164" s="27"/>
       <c r="AF164" s="14"/>
       <c r="AG164" s="14"/>
       <c r="AH164" s="14" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="AI164" s="14"/>
     </row>
     <row r="165" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="14" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="B165" s="14" t="s">
         <v>174</v>
@@ -9981,7 +9980,7 @@
         <v>135</v>
       </c>
       <c r="D165" s="18" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="E165" s="14"/>
       <c r="F165" s="14"/>
@@ -9995,16 +9994,10 @@
       <c r="N165" s="14"/>
       <c r="O165" s="14"/>
       <c r="P165" s="14"/>
-      <c r="Q165" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q165" s="14"/>
       <c r="R165" s="14"/>
-      <c r="S165" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T165" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S165" s="14"/>
+      <c r="T165" s="14"/>
       <c r="U165" s="14"/>
       <c r="V165" s="14"/>
       <c r="W165" s="14"/>
@@ -10013,25 +10006,23 @@
       <c r="Z165" s="14"/>
       <c r="AA165" s="14"/>
       <c r="AB165" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC165" s="14" t="s">
-        <v>457</v>
+        <v>393</v>
       </c>
       <c r="AD165" s="14" t="s">
-        <v>451</v>
+        <v>393</v>
       </c>
       <c r="AE165" s="27"/>
       <c r="AF165" s="14"/>
       <c r="AG165" s="14"/>
-      <c r="AH165" s="15" t="s">
-        <v>454</v>
-      </c>
+      <c r="AH165" s="14"/>
       <c r="AI165" s="14"/>
     </row>
     <row r="166" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="14" t="s">
-        <v>539</v>
+        <v>492</v>
       </c>
       <c r="B166" s="14" t="s">
         <v>174</v>
@@ -10039,8 +10030,8 @@
       <c r="C166" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D166" s="23" t="s">
-        <v>540</v>
+      <c r="D166" s="18" t="s">
+        <v>493</v>
       </c>
       <c r="E166" s="14"/>
       <c r="F166" s="14"/>
@@ -10050,9 +10041,7 @@
       <c r="J166" s="14"/>
       <c r="K166" s="14"/>
       <c r="L166" s="14"/>
-      <c r="M166" s="20" t="s">
-        <v>609</v>
-      </c>
+      <c r="M166" s="14"/>
       <c r="N166" s="14"/>
       <c r="O166" s="14"/>
       <c r="P166" s="14"/>
@@ -10086,7 +10075,7 @@
     </row>
     <row r="167" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="14" t="s">
-        <v>542</v>
+        <v>490</v>
       </c>
       <c r="B167" s="14" t="s">
         <v>174</v>
@@ -10094,8 +10083,8 @@
       <c r="C167" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D167" s="23" t="s">
-        <v>541</v>
+      <c r="D167" s="18" t="s">
+        <v>491</v>
       </c>
       <c r="E167" s="14"/>
       <c r="F167" s="14"/>
@@ -10105,16 +10094,20 @@
       <c r="J167" s="14"/>
       <c r="K167" s="14"/>
       <c r="L167" s="14"/>
-      <c r="M167" s="20" t="s">
-        <v>494</v>
-      </c>
+      <c r="M167" s="14"/>
       <c r="N167" s="14"/>
       <c r="O167" s="14"/>
       <c r="P167" s="14"/>
-      <c r="Q167" s="14"/>
+      <c r="Q167" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R167" s="14"/>
-      <c r="S167" s="14"/>
-      <c r="T167" s="14"/>
+      <c r="S167" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T167" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U167" s="14"/>
       <c r="V167" s="14"/>
       <c r="W167" s="14"/>
@@ -10123,23 +10116,25 @@
       <c r="Z167" s="14"/>
       <c r="AA167" s="14"/>
       <c r="AB167" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC167" s="14" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="AD167" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE167" s="27"/>
       <c r="AF167" s="14"/>
       <c r="AG167" s="14"/>
-      <c r="AH167" s="14"/>
+      <c r="AH167" s="15" t="s">
+        <v>454</v>
+      </c>
       <c r="AI167" s="14"/>
     </row>
     <row r="168" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="14" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="B168" s="14" t="s">
         <v>174</v>
@@ -10148,7 +10143,7 @@
         <v>135</v>
       </c>
       <c r="D168" s="23" t="s">
-        <v>546</v>
+        <v>540</v>
       </c>
       <c r="E168" s="14"/>
       <c r="F168" s="14"/>
@@ -10159,7 +10154,7 @@
       <c r="K168" s="14"/>
       <c r="L168" s="14"/>
       <c r="M168" s="20" t="s">
-        <v>494</v>
+        <v>609</v>
       </c>
       <c r="N168" s="14"/>
       <c r="O168" s="14"/>
@@ -10194,7 +10189,7 @@
     </row>
     <row r="169" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="14" t="s">
-        <v>547</v>
+        <v>542</v>
       </c>
       <c r="B169" s="14" t="s">
         <v>174</v>
@@ -10202,8 +10197,8 @@
       <c r="C169" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D169" s="18" t="s">
-        <v>548</v>
+      <c r="D169" s="23" t="s">
+        <v>541</v>
       </c>
       <c r="E169" s="14"/>
       <c r="F169" s="14"/>
@@ -10212,7 +10207,7 @@
       <c r="I169" s="14"/>
       <c r="J169" s="14"/>
       <c r="K169" s="14"/>
-      <c r="L169" s="31"/>
+      <c r="L169" s="14"/>
       <c r="M169" s="20" t="s">
         <v>494</v>
       </c>
@@ -10231,25 +10226,23 @@
       <c r="Z169" s="14"/>
       <c r="AA169" s="14"/>
       <c r="AB169" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC169" s="14" t="s">
-        <v>457</v>
+        <v>427</v>
       </c>
       <c r="AD169" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE169" s="27"/>
       <c r="AF169" s="14"/>
       <c r="AG169" s="14"/>
-      <c r="AH169" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH169" s="14"/>
       <c r="AI169" s="14"/>
     </row>
     <row r="170" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="14" t="s">
-        <v>550</v>
+        <v>543</v>
       </c>
       <c r="B170" s="14" t="s">
         <v>174</v>
@@ -10257,8 +10250,8 @@
       <c r="C170" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D170" s="18" t="s">
-        <v>551</v>
+      <c r="D170" s="23" t="s">
+        <v>546</v>
       </c>
       <c r="E170" s="14"/>
       <c r="F170" s="14"/>
@@ -10286,13 +10279,13 @@
       <c r="Z170" s="14"/>
       <c r="AA170" s="14"/>
       <c r="AB170" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC170" s="14" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="AD170" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE170" s="27"/>
       <c r="AF170" s="14"/>
@@ -10303,10 +10296,18 @@
       <c r="AI170" s="14"/>
     </row>
     <row r="171" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A171" s="14"/>
-      <c r="B171" s="14"/>
-      <c r="C171" s="14"/>
-      <c r="D171" s="18"/>
+      <c r="A171" s="14" t="s">
+        <v>547</v>
+      </c>
+      <c r="B171" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C171" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D171" s="18" t="s">
+        <v>548</v>
+      </c>
       <c r="E171" s="14"/>
       <c r="F171" s="14"/>
       <c r="G171" s="14"/>
@@ -10314,8 +10315,10 @@
       <c r="I171" s="14"/>
       <c r="J171" s="14"/>
       <c r="K171" s="14"/>
-      <c r="L171" s="14"/>
-      <c r="M171" s="20"/>
+      <c r="L171" s="31"/>
+      <c r="M171" s="20" t="s">
+        <v>494</v>
+      </c>
       <c r="N171" s="14"/>
       <c r="O171" s="14"/>
       <c r="P171" s="14"/>
@@ -10330,18 +10333,26 @@
       <c r="Y171" s="14"/>
       <c r="Z171" s="14"/>
       <c r="AA171" s="14"/>
-      <c r="AB171" s="14"/>
-      <c r="AC171" s="14"/>
-      <c r="AD171" s="14"/>
+      <c r="AB171" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC171" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD171" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE171" s="27"/>
       <c r="AF171" s="14"/>
       <c r="AG171" s="14"/>
-      <c r="AH171" s="14"/>
+      <c r="AH171" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI171" s="14"/>
     </row>
     <row r="172" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="14" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="B172" s="14" t="s">
         <v>174</v>
@@ -10350,7 +10361,7 @@
         <v>135</v>
       </c>
       <c r="D172" s="18" t="s">
-        <v>566</v>
+        <v>551</v>
       </c>
       <c r="E172" s="14"/>
       <c r="F172" s="14"/>
@@ -10360,20 +10371,16 @@
       <c r="J172" s="14"/>
       <c r="K172" s="14"/>
       <c r="L172" s="14"/>
-      <c r="M172" s="14"/>
+      <c r="M172" s="20" t="s">
+        <v>494</v>
+      </c>
       <c r="N172" s="14"/>
       <c r="O172" s="14"/>
       <c r="P172" s="14"/>
-      <c r="Q172" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q172" s="14"/>
       <c r="R172" s="14"/>
-      <c r="S172" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T172" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S172" s="14"/>
+      <c r="T172" s="14"/>
       <c r="U172" s="14"/>
       <c r="V172" s="14"/>
       <c r="W172" s="14"/>
@@ -10385,32 +10392,24 @@
         <v>393</v>
       </c>
       <c r="AC172" s="14" t="s">
-        <v>393</v>
+        <v>427</v>
       </c>
       <c r="AD172" s="14" t="s">
-        <v>393</v>
+        <v>421</v>
       </c>
       <c r="AE172" s="27"/>
       <c r="AF172" s="14"/>
       <c r="AG172" s="14"/>
       <c r="AH172" s="14" t="s">
-        <v>465</v>
+        <v>458</v>
       </c>
       <c r="AI172" s="14"/>
     </row>
     <row r="173" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A173" s="14" t="s">
-        <v>555</v>
-      </c>
-      <c r="B173" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C173" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D173" s="18" t="s">
-        <v>569</v>
-      </c>
+      <c r="A173" s="14"/>
+      <c r="B173" s="14"/>
+      <c r="C173" s="14"/>
+      <c r="D173" s="18"/>
       <c r="E173" s="14"/>
       <c r="F173" s="14"/>
       <c r="G173" s="14"/>
@@ -10419,7 +10418,7 @@
       <c r="J173" s="14"/>
       <c r="K173" s="14"/>
       <c r="L173" s="14"/>
-      <c r="M173" s="14"/>
+      <c r="M173" s="20"/>
       <c r="N173" s="14"/>
       <c r="O173" s="14"/>
       <c r="P173" s="14"/>
@@ -10434,15 +10433,9 @@
       <c r="Y173" s="14"/>
       <c r="Z173" s="14"/>
       <c r="AA173" s="14"/>
-      <c r="AB173" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC173" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD173" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB173" s="14"/>
+      <c r="AC173" s="14"/>
+      <c r="AD173" s="14"/>
       <c r="AE173" s="27"/>
       <c r="AF173" s="14"/>
       <c r="AG173" s="14"/>
@@ -10451,7 +10444,7 @@
     </row>
     <row r="174" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="14" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="B174" s="14" t="s">
         <v>174</v>
@@ -10460,7 +10453,7 @@
         <v>135</v>
       </c>
       <c r="D174" s="18" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="E174" s="14"/>
       <c r="F174" s="14"/>
@@ -10474,10 +10467,16 @@
       <c r="N174" s="14"/>
       <c r="O174" s="14"/>
       <c r="P174" s="14"/>
-      <c r="Q174" s="14"/>
+      <c r="Q174" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R174" s="14"/>
-      <c r="S174" s="14"/>
-      <c r="T174" s="14"/>
+      <c r="S174" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T174" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U174" s="14"/>
       <c r="V174" s="14"/>
       <c r="W174" s="14"/>
@@ -10486,25 +10485,25 @@
       <c r="Z174" s="14"/>
       <c r="AA174" s="14"/>
       <c r="AB174" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC174" s="14" t="s">
-        <v>457</v>
+        <v>393</v>
       </c>
       <c r="AD174" s="14" t="s">
-        <v>451</v>
+        <v>393</v>
       </c>
       <c r="AE174" s="27"/>
       <c r="AF174" s="14"/>
       <c r="AG174" s="14"/>
       <c r="AH174" s="14" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="AI174" s="14"/>
     </row>
     <row r="175" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="14" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="B175" s="14" t="s">
         <v>174</v>
@@ -10513,7 +10512,7 @@
         <v>135</v>
       </c>
       <c r="D175" s="18" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="E175" s="14"/>
       <c r="F175" s="14"/>
@@ -10527,16 +10526,10 @@
       <c r="N175" s="14"/>
       <c r="O175" s="14"/>
       <c r="P175" s="14"/>
-      <c r="Q175" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q175" s="14"/>
       <c r="R175" s="14"/>
-      <c r="S175" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T175" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S175" s="14"/>
+      <c r="T175" s="14"/>
       <c r="U175" s="14"/>
       <c r="V175" s="14"/>
       <c r="W175" s="14"/>
@@ -10545,25 +10538,23 @@
       <c r="Z175" s="14"/>
       <c r="AA175" s="14"/>
       <c r="AB175" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC175" s="14" t="s">
-        <v>457</v>
+        <v>393</v>
       </c>
       <c r="AD175" s="14" t="s">
-        <v>451</v>
+        <v>393</v>
       </c>
       <c r="AE175" s="27"/>
       <c r="AF175" s="14"/>
       <c r="AG175" s="14"/>
-      <c r="AH175" s="15" t="s">
-        <v>454</v>
-      </c>
+      <c r="AH175" s="14"/>
       <c r="AI175" s="14"/>
     </row>
     <row r="176" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="14" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="B176" s="14" t="s">
         <v>174</v>
@@ -10571,8 +10562,8 @@
       <c r="C176" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D176" s="23" t="s">
-        <v>571</v>
+      <c r="D176" s="18" t="s">
+        <v>563</v>
       </c>
       <c r="E176" s="14"/>
       <c r="F176" s="14"/>
@@ -10582,9 +10573,7 @@
       <c r="J176" s="14"/>
       <c r="K176" s="14"/>
       <c r="L176" s="14"/>
-      <c r="M176" s="30" t="s">
-        <v>580</v>
-      </c>
+      <c r="M176" s="14"/>
       <c r="N176" s="14"/>
       <c r="O176" s="14"/>
       <c r="P176" s="14"/>
@@ -10618,7 +10607,7 @@
     </row>
     <row r="177" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="14" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="B177" s="14" t="s">
         <v>174</v>
@@ -10626,8 +10615,8 @@
       <c r="C177" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D177" s="23" t="s">
-        <v>572</v>
+      <c r="D177" s="18" t="s">
+        <v>570</v>
       </c>
       <c r="E177" s="14"/>
       <c r="F177" s="14"/>
@@ -10637,16 +10626,20 @@
       <c r="J177" s="14"/>
       <c r="K177" s="14"/>
       <c r="L177" s="14"/>
-      <c r="M177" s="30" t="s">
-        <v>549</v>
-      </c>
+      <c r="M177" s="14"/>
       <c r="N177" s="14"/>
       <c r="O177" s="14"/>
       <c r="P177" s="14"/>
-      <c r="Q177" s="14"/>
+      <c r="Q177" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R177" s="14"/>
-      <c r="S177" s="14"/>
-      <c r="T177" s="14"/>
+      <c r="S177" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T177" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U177" s="14"/>
       <c r="V177" s="14"/>
       <c r="W177" s="14"/>
@@ -10655,23 +10648,25 @@
       <c r="Z177" s="14"/>
       <c r="AA177" s="14"/>
       <c r="AB177" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC177" s="14" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="AD177" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE177" s="27"/>
       <c r="AF177" s="14"/>
       <c r="AG177" s="14"/>
-      <c r="AH177" s="14"/>
+      <c r="AH177" s="15" t="s">
+        <v>454</v>
+      </c>
       <c r="AI177" s="14"/>
     </row>
     <row r="178" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="14" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B178" s="14" t="s">
         <v>174</v>
@@ -10680,7 +10675,7 @@
         <v>135</v>
       </c>
       <c r="D178" s="23" t="s">
-        <v>578</v>
+        <v>571</v>
       </c>
       <c r="E178" s="14"/>
       <c r="F178" s="14"/>
@@ -10690,8 +10685,8 @@
       <c r="J178" s="14"/>
       <c r="K178" s="14"/>
       <c r="L178" s="14"/>
-      <c r="M178" s="14" t="s">
-        <v>549</v>
+      <c r="M178" s="30" t="s">
+        <v>580</v>
       </c>
       <c r="N178" s="14"/>
       <c r="O178" s="14"/>
@@ -10726,7 +10721,7 @@
     </row>
     <row r="179" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="14" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="B179" s="14" t="s">
         <v>174</v>
@@ -10734,8 +10729,8 @@
       <c r="C179" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D179" s="18" t="s">
-        <v>579</v>
+      <c r="D179" s="23" t="s">
+        <v>572</v>
       </c>
       <c r="E179" s="14"/>
       <c r="F179" s="14"/>
@@ -10745,7 +10740,7 @@
       <c r="J179" s="14"/>
       <c r="K179" s="14"/>
       <c r="L179" s="14"/>
-      <c r="M179" s="14" t="s">
+      <c r="M179" s="30" t="s">
         <v>549</v>
       </c>
       <c r="N179" s="14"/>
@@ -10774,14 +10769,12 @@
       <c r="AE179" s="27"/>
       <c r="AF179" s="14"/>
       <c r="AG179" s="14"/>
-      <c r="AH179" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH179" s="14"/>
       <c r="AI179" s="14"/>
     </row>
     <row r="180" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="14" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="B180" s="14" t="s">
         <v>174</v>
@@ -10789,8 +10782,8 @@
       <c r="C180" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D180" s="18" t="s">
-        <v>575</v>
+      <c r="D180" s="23" t="s">
+        <v>578</v>
       </c>
       <c r="E180" s="14"/>
       <c r="F180" s="14"/>
@@ -10799,8 +10792,8 @@
       <c r="I180" s="14"/>
       <c r="J180" s="14"/>
       <c r="K180" s="14"/>
-      <c r="L180" s="31"/>
-      <c r="M180" s="30" t="s">
+      <c r="L180" s="14"/>
+      <c r="M180" s="14" t="s">
         <v>549</v>
       </c>
       <c r="N180" s="14"/>
@@ -10835,10 +10828,18 @@
       <c r="AI180" s="14"/>
     </row>
     <row r="181" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A181" s="14"/>
-      <c r="B181" s="14"/>
-      <c r="C181" s="14"/>
-      <c r="D181" s="15"/>
+      <c r="A181" s="14" t="s">
+        <v>561</v>
+      </c>
+      <c r="B181" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C181" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D181" s="18" t="s">
+        <v>579</v>
+      </c>
       <c r="E181" s="14"/>
       <c r="F181" s="14"/>
       <c r="G181" s="14"/>
@@ -10847,12 +10848,14 @@
       <c r="J181" s="14"/>
       <c r="K181" s="14"/>
       <c r="L181" s="14"/>
-      <c r="M181" s="14"/>
+      <c r="M181" s="14" t="s">
+        <v>549</v>
+      </c>
       <c r="N181" s="14"/>
       <c r="O181" s="14"/>
       <c r="P181" s="14"/>
       <c r="Q181" s="14"/>
-      <c r="R181" s="15"/>
+      <c r="R181" s="14"/>
       <c r="S181" s="14"/>
       <c r="T181" s="14"/>
       <c r="U181" s="14"/>
@@ -10862,18 +10865,26 @@
       <c r="Y181" s="14"/>
       <c r="Z181" s="14"/>
       <c r="AA181" s="14"/>
-      <c r="AB181" s="14"/>
-      <c r="AC181" s="14"/>
-      <c r="AD181" s="14"/>
+      <c r="AB181" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC181" s="14" t="s">
+        <v>427</v>
+      </c>
+      <c r="AD181" s="14" t="s">
+        <v>421</v>
+      </c>
       <c r="AE181" s="27"/>
       <c r="AF181" s="14"/>
       <c r="AG181" s="14"/>
-      <c r="AH181" s="14"/>
+      <c r="AH181" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI181" s="14"/>
     </row>
     <row r="182" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A182" s="14" t="s">
-        <v>267</v>
+        <v>562</v>
       </c>
       <c r="B182" s="14" t="s">
         <v>174</v>
@@ -10881,22 +10892,20 @@
       <c r="C182" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D182" s="14"/>
+      <c r="D182" s="18" t="s">
+        <v>575</v>
+      </c>
       <c r="E182" s="14"/>
       <c r="F182" s="14"/>
       <c r="G182" s="14"/>
       <c r="H182" s="14"/>
       <c r="I182" s="14"/>
-      <c r="J182" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K182" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L182" s="15" t="s">
-        <v>275</v>
-      </c>
-      <c r="M182" s="14"/>
+      <c r="J182" s="14"/>
+      <c r="K182" s="14"/>
+      <c r="L182" s="31"/>
+      <c r="M182" s="30" t="s">
+        <v>549</v>
+      </c>
       <c r="N182" s="14"/>
       <c r="O182" s="14"/>
       <c r="P182" s="14"/>
@@ -10911,46 +10920,42 @@
       <c r="Y182" s="14"/>
       <c r="Z182" s="14"/>
       <c r="AA182" s="14"/>
-      <c r="AB182" s="14"/>
-      <c r="AC182" s="14"/>
-      <c r="AD182" s="14"/>
+      <c r="AB182" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC182" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD182" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE182" s="27"/>
       <c r="AF182" s="14"/>
       <c r="AG182" s="14"/>
-      <c r="AH182" s="14"/>
+      <c r="AH182" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI182" s="14"/>
     </row>
     <row r="183" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A183" s="14" t="s">
-        <v>268</v>
-      </c>
-      <c r="B183" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C183" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D183" s="14"/>
+      <c r="A183" s="14"/>
+      <c r="B183" s="14"/>
+      <c r="C183" s="14"/>
+      <c r="D183" s="15"/>
       <c r="E183" s="14"/>
       <c r="F183" s="14"/>
       <c r="G183" s="14"/>
       <c r="H183" s="14"/>
       <c r="I183" s="14"/>
-      <c r="J183" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K183" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L183" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="J183" s="14"/>
+      <c r="K183" s="14"/>
+      <c r="L183" s="14"/>
       <c r="M183" s="14"/>
       <c r="N183" s="14"/>
       <c r="O183" s="14"/>
       <c r="P183" s="14"/>
       <c r="Q183" s="14"/>
-      <c r="R183" s="14"/>
+      <c r="R183" s="15"/>
       <c r="S183" s="14"/>
       <c r="T183" s="14"/>
       <c r="U183" s="14"/>
@@ -10969,41 +10974,89 @@
       <c r="AH183" s="14"/>
       <c r="AI183" s="14"/>
     </row>
-    <row r="184" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A184" s="14" t="s">
-        <v>359</v>
+        <v>616</v>
       </c>
       <c r="B184" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C184" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O184" s="15" t="s">
-        <v>362</v>
-      </c>
-      <c r="AB184" s="14"/>
-      <c r="AC184" s="14"/>
-      <c r="AD184" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D184" s="18" t="s">
+        <v>615</v>
+      </c>
+      <c r="E184" s="14"/>
+      <c r="F184" s="14"/>
+      <c r="G184" s="14"/>
+      <c r="H184" s="14"/>
+      <c r="I184" s="14"/>
+      <c r="J184" s="14"/>
+      <c r="K184" s="14"/>
+      <c r="L184" s="31"/>
+      <c r="M184" s="30" t="s">
+        <v>549</v>
+      </c>
+      <c r="N184" s="14"/>
+      <c r="O184" s="14"/>
+      <c r="P184" s="14"/>
+      <c r="Q184" s="14"/>
+      <c r="R184" s="14"/>
+      <c r="S184" s="14"/>
+      <c r="T184" s="14"/>
+      <c r="U184" s="14"/>
+      <c r="V184" s="14"/>
+      <c r="W184" s="14"/>
+      <c r="X184" s="14"/>
+      <c r="Y184" s="14"/>
+      <c r="Z184" s="14"/>
+      <c r="AA184" s="14"/>
+      <c r="AB184" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC184" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD184" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE184" s="27"/>
       <c r="AF184" s="14"/>
       <c r="AG184" s="14"/>
-      <c r="AH184" s="14"/>
+      <c r="AH184" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI184" s="14"/>
     </row>
-    <row r="185" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A185" s="14" t="s">
-        <v>360</v>
-      </c>
-      <c r="B185" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C185" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O185" s="15" t="s">
-        <v>363</v>
-      </c>
+    <row r="185" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="14"/>
+      <c r="B185" s="14"/>
+      <c r="C185" s="14"/>
+      <c r="D185" s="14"/>
+      <c r="E185" s="14"/>
+      <c r="F185" s="14"/>
+      <c r="G185" s="14"/>
+      <c r="H185" s="14"/>
+      <c r="I185" s="14"/>
+      <c r="J185" s="14"/>
+      <c r="K185" s="14"/>
+      <c r="L185" s="14"/>
+      <c r="M185" s="14"/>
+      <c r="N185" s="14"/>
+      <c r="O185" s="14"/>
+      <c r="P185" s="14"/>
+      <c r="Q185" s="14"/>
+      <c r="R185" s="14"/>
+      <c r="S185" s="14"/>
+      <c r="T185" s="14"/>
+      <c r="U185" s="14"/>
+      <c r="V185" s="14"/>
+      <c r="W185" s="14"/>
+      <c r="X185" s="14"/>
+      <c r="Y185" s="14"/>
+      <c r="Z185" s="14"/>
+      <c r="AA185" s="14"/>
       <c r="AB185" s="14"/>
       <c r="AC185" s="14"/>
       <c r="AD185" s="14"/>
@@ -11013,9 +11066,9 @@
       <c r="AH185" s="14"/>
       <c r="AI185" s="14"/>
     </row>
-    <row r="186" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="14" t="s">
-        <v>361</v>
+        <v>267</v>
       </c>
       <c r="B186" s="14" t="s">
         <v>174</v>
@@ -11023,9 +11076,36 @@
       <c r="C186" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O186" s="15" t="s">
-        <v>364</v>
-      </c>
+      <c r="D186" s="14"/>
+      <c r="E186" s="14"/>
+      <c r="F186" s="14"/>
+      <c r="G186" s="14"/>
+      <c r="H186" s="14"/>
+      <c r="I186" s="14"/>
+      <c r="J186" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K186" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L186" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M186" s="14"/>
+      <c r="N186" s="14"/>
+      <c r="O186" s="14"/>
+      <c r="P186" s="14"/>
+      <c r="Q186" s="14"/>
+      <c r="R186" s="14"/>
+      <c r="S186" s="14"/>
+      <c r="T186" s="14"/>
+      <c r="U186" s="14"/>
+      <c r="V186" s="14"/>
+      <c r="W186" s="14"/>
+      <c r="X186" s="14"/>
+      <c r="Y186" s="14"/>
+      <c r="Z186" s="14"/>
+      <c r="AA186" s="14"/>
       <c r="AB186" s="14"/>
       <c r="AC186" s="14"/>
       <c r="AD186" s="14"/>
@@ -11035,9 +11115,9 @@
       <c r="AH186" s="14"/>
       <c r="AI186" s="14"/>
     </row>
-    <row r="187" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="14" t="s">
-        <v>370</v>
+        <v>268</v>
       </c>
       <c r="B187" s="14" t="s">
         <v>174</v>
@@ -11045,9 +11125,36 @@
       <c r="C187" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M187" s="14" t="s">
-        <v>371</v>
-      </c>
+      <c r="D187" s="14"/>
+      <c r="E187" s="14"/>
+      <c r="F187" s="14"/>
+      <c r="G187" s="14"/>
+      <c r="H187" s="14"/>
+      <c r="I187" s="14"/>
+      <c r="J187" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K187" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L187" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M187" s="14"/>
+      <c r="N187" s="14"/>
+      <c r="O187" s="14"/>
+      <c r="P187" s="14"/>
+      <c r="Q187" s="14"/>
+      <c r="R187" s="14"/>
+      <c r="S187" s="14"/>
+      <c r="T187" s="14"/>
+      <c r="U187" s="14"/>
+      <c r="V187" s="14"/>
+      <c r="W187" s="14"/>
+      <c r="X187" s="14"/>
+      <c r="Y187" s="14"/>
+      <c r="Z187" s="14"/>
+      <c r="AA187" s="14"/>
       <c r="AB187" s="14"/>
       <c r="AC187" s="14"/>
       <c r="AD187" s="14"/>
@@ -11058,6 +11165,18 @@
       <c r="AI187" s="14"/>
     </row>
     <row r="188" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A188" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="B188" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C188" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O188" s="15" t="s">
+        <v>362</v>
+      </c>
       <c r="AB188" s="14"/>
       <c r="AC188" s="14"/>
       <c r="AD188" s="14"/>
@@ -11068,6 +11187,18 @@
       <c r="AI188" s="14"/>
     </row>
     <row r="189" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A189" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B189" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C189" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O189" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB189" s="14"/>
       <c r="AC189" s="14"/>
       <c r="AD189" s="14"/>
@@ -11078,6 +11209,18 @@
       <c r="AI189" s="14"/>
     </row>
     <row r="190" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A190" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B190" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C190" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O190" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB190" s="14"/>
       <c r="AC190" s="14"/>
       <c r="AD190" s="14"/>
@@ -11088,6 +11231,18 @@
       <c r="AI190" s="14"/>
     </row>
     <row r="191" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A191" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B191" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C191" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M191" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB191" s="14"/>
       <c r="AC191" s="14"/>
       <c r="AD191" s="14"/>
@@ -13051,7 +13206,7 @@
       <c r="AB387" s="14"/>
       <c r="AC387" s="14"/>
       <c r="AD387" s="14"/>
-      <c r="AE387" s="14"/>
+      <c r="AE387" s="27"/>
       <c r="AF387" s="14"/>
       <c r="AG387" s="14"/>
       <c r="AH387" s="14"/>
@@ -13061,7 +13216,7 @@
       <c r="AB388" s="14"/>
       <c r="AC388" s="14"/>
       <c r="AD388" s="14"/>
-      <c r="AE388" s="14"/>
+      <c r="AE388" s="27"/>
       <c r="AF388" s="14"/>
       <c r="AG388" s="14"/>
       <c r="AH388" s="14"/>
@@ -13071,7 +13226,7 @@
       <c r="AB389" s="14"/>
       <c r="AC389" s="14"/>
       <c r="AD389" s="14"/>
-      <c r="AE389" s="14"/>
+      <c r="AE389" s="27"/>
       <c r="AF389" s="14"/>
       <c r="AG389" s="14"/>
       <c r="AH389" s="14"/>
@@ -13117,6 +13272,36 @@
       <c r="AH393" s="14"/>
       <c r="AI393" s="14"/>
     </row>
+    <row r="394" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB394" s="14"/>
+      <c r="AC394" s="14"/>
+      <c r="AD394" s="14"/>
+      <c r="AE394" s="14"/>
+      <c r="AF394" s="14"/>
+      <c r="AG394" s="14"/>
+      <c r="AH394" s="14"/>
+      <c r="AI394" s="14"/>
+    </row>
+    <row r="395" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB395" s="14"/>
+      <c r="AC395" s="14"/>
+      <c r="AD395" s="14"/>
+      <c r="AE395" s="14"/>
+      <c r="AF395" s="14"/>
+      <c r="AG395" s="14"/>
+      <c r="AH395" s="14"/>
+      <c r="AI395" s="14"/>
+    </row>
+    <row r="396" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB396" s="14"/>
+      <c r="AC396" s="14"/>
+      <c r="AD396" s="14"/>
+      <c r="AE396" s="14"/>
+      <c r="AF396" s="14"/>
+      <c r="AG396" s="14"/>
+      <c r="AH396" s="14"/>
+      <c r="AI396" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13126,7 +13311,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T186"/>
+  <dimension ref="A1:T188"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -19224,6 +19409,72 @@
       <c r="S186" s="14"/>
       <c r="T186" s="14"/>
     </row>
+    <row r="187" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="15" t="s">
+        <v>615</v>
+      </c>
+      <c r="B187" s="20" t="s">
+        <v>398</v>
+      </c>
+      <c r="C187" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D187" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E187" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="F187" s="15"/>
+      <c r="G187" s="15"/>
+      <c r="H187" s="15"/>
+      <c r="I187" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="J187" s="14"/>
+      <c r="K187" s="14"/>
+      <c r="L187" s="14"/>
+      <c r="M187" s="14"/>
+      <c r="N187" s="14"/>
+      <c r="O187" s="14"/>
+      <c r="P187" s="14"/>
+      <c r="Q187" s="14"/>
+      <c r="R187" s="14"/>
+      <c r="S187" s="14"/>
+      <c r="T187" s="14"/>
+    </row>
+    <row r="188" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="15" t="s">
+        <v>618</v>
+      </c>
+      <c r="B188" s="20" t="s">
+        <v>619</v>
+      </c>
+      <c r="C188" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D188" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E188" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F188" s="15"/>
+      <c r="G188" s="15"/>
+      <c r="H188" s="15"/>
+      <c r="I188" s="14"/>
+      <c r="J188" s="14"/>
+      <c r="K188" s="14"/>
+      <c r="L188" s="14"/>
+      <c r="M188" s="14"/>
+      <c r="N188" s="14"/>
+      <c r="O188" s="14"/>
+      <c r="P188" s="14"/>
+      <c r="Q188" s="14"/>
+      <c r="R188" s="14"/>
+      <c r="S188" s="14"/>
+      <c r="T188" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Commit after script developed for APC Automation IB Scenarios
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85158EE1-1FBF-4875-B2F4-9DFF9A19216E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B696DC65-778D-4E11-8A79-39C712858F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2665" uniqueCount="620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2734" uniqueCount="638">
   <si>
     <t>1</t>
   </si>
@@ -1888,6 +1888,60 @@
   </si>
   <si>
     <t>03P78-25</t>
+  </si>
+  <si>
+    <t>03P76-25</t>
+  </si>
+  <si>
+    <t>APC_IBScenario002</t>
+  </si>
+  <si>
+    <t>APC_IBScenario003</t>
+  </si>
+  <si>
+    <t>974</t>
+  </si>
+  <si>
+    <t>975</t>
+  </si>
+  <si>
+    <t>013407-01 01</t>
+  </si>
+  <si>
+    <t>06F16-10</t>
+  </si>
+  <si>
+    <t>PSTG1A0127</t>
+  </si>
+  <si>
+    <t>APC_IBScenario004</t>
+  </si>
+  <si>
+    <t>APC_IBScenario005</t>
+  </si>
+  <si>
+    <t>APC_IBScenario006</t>
+  </si>
+  <si>
+    <t>976</t>
+  </si>
+  <si>
+    <t>977</t>
+  </si>
+  <si>
+    <t>978</t>
+  </si>
+  <si>
+    <t>06F21-26</t>
+  </si>
+  <si>
+    <t>07P02-06</t>
+  </si>
+  <si>
+    <t>07P04-03</t>
+  </si>
+  <si>
+    <t>BX</t>
   </si>
 </sst>
 </file>
@@ -2431,7 +2485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI396"/>
+  <dimension ref="A1:AI401"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -6741,7 +6795,7 @@
         <v>614</v>
       </c>
       <c r="D94" s="18" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="E94" s="15"/>
       <c r="F94" s="14"/>
@@ -10985,7 +11039,7 @@
         <v>614</v>
       </c>
       <c r="D184" s="18" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="E184" s="14"/>
       <c r="F184" s="14"/>
@@ -10995,9 +11049,7 @@
       <c r="J184" s="14"/>
       <c r="K184" s="14"/>
       <c r="L184" s="31"/>
-      <c r="M184" s="30" t="s">
-        <v>549</v>
-      </c>
+      <c r="M184" s="30"/>
       <c r="N184" s="14"/>
       <c r="O184" s="14"/>
       <c r="P184" s="14"/>
@@ -11030,10 +11082,18 @@
       <c r="AI184" s="14"/>
     </row>
     <row r="185" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A185" s="14"/>
-      <c r="B185" s="14"/>
-      <c r="C185" s="14"/>
-      <c r="D185" s="14"/>
+      <c r="A185" s="14" t="s">
+        <v>621</v>
+      </c>
+      <c r="B185" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C185" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D185" s="18" t="s">
+        <v>623</v>
+      </c>
       <c r="E185" s="14"/>
       <c r="F185" s="14"/>
       <c r="G185" s="14"/>
@@ -11041,8 +11101,8 @@
       <c r="I185" s="14"/>
       <c r="J185" s="14"/>
       <c r="K185" s="14"/>
-      <c r="L185" s="14"/>
-      <c r="M185" s="14"/>
+      <c r="L185" s="31"/>
+      <c r="M185" s="30"/>
       <c r="N185" s="14"/>
       <c r="O185" s="14"/>
       <c r="P185" s="14"/>
@@ -11057,41 +11117,45 @@
       <c r="Y185" s="14"/>
       <c r="Z185" s="14"/>
       <c r="AA185" s="14"/>
-      <c r="AB185" s="14"/>
-      <c r="AC185" s="14"/>
-      <c r="AD185" s="14"/>
+      <c r="AB185" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC185" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD185" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE185" s="27"/>
       <c r="AF185" s="14"/>
       <c r="AG185" s="14"/>
-      <c r="AH185" s="14"/>
+      <c r="AH185" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI185" s="14"/>
     </row>
     <row r="186" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="14" t="s">
-        <v>267</v>
+        <v>622</v>
       </c>
       <c r="B186" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C186" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D186" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D186" s="18" t="s">
+        <v>624</v>
+      </c>
       <c r="E186" s="14"/>
       <c r="F186" s="14"/>
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
       <c r="I186" s="14"/>
-      <c r="J186" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K186" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L186" s="15" t="s">
-        <v>275</v>
-      </c>
-      <c r="M186" s="14"/>
+      <c r="J186" s="14"/>
+      <c r="K186" s="14"/>
+      <c r="L186" s="31"/>
+      <c r="M186" s="30"/>
       <c r="N186" s="14"/>
       <c r="O186" s="14"/>
       <c r="P186" s="14"/>
@@ -11106,41 +11170,45 @@
       <c r="Y186" s="14"/>
       <c r="Z186" s="14"/>
       <c r="AA186" s="14"/>
-      <c r="AB186" s="14"/>
-      <c r="AC186" s="14"/>
-      <c r="AD186" s="14"/>
+      <c r="AB186" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC186" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD186" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE186" s="27"/>
       <c r="AF186" s="14"/>
       <c r="AG186" s="14"/>
-      <c r="AH186" s="14"/>
+      <c r="AH186" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI186" s="14"/>
     </row>
     <row r="187" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="14" t="s">
-        <v>268</v>
+        <v>628</v>
       </c>
       <c r="B187" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C187" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D187" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D187" s="18" t="s">
+        <v>631</v>
+      </c>
       <c r="E187" s="14"/>
       <c r="F187" s="14"/>
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
       <c r="I187" s="14"/>
-      <c r="J187" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K187" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L187" s="15" t="s">
-        <v>276</v>
-      </c>
-      <c r="M187" s="14"/>
+      <c r="J187" s="14"/>
+      <c r="K187" s="14"/>
+      <c r="L187" s="31"/>
+      <c r="M187" s="30"/>
       <c r="N187" s="14"/>
       <c r="O187" s="14"/>
       <c r="P187" s="14"/>
@@ -11155,72 +11223,157 @@
       <c r="Y187" s="14"/>
       <c r="Z187" s="14"/>
       <c r="AA187" s="14"/>
-      <c r="AB187" s="14"/>
-      <c r="AC187" s="14"/>
-      <c r="AD187" s="14"/>
+      <c r="AB187" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC187" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD187" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE187" s="27"/>
       <c r="AF187" s="14"/>
       <c r="AG187" s="14"/>
-      <c r="AH187" s="14"/>
+      <c r="AH187" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI187" s="14"/>
     </row>
-    <row r="188" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="14" t="s">
-        <v>359</v>
+        <v>629</v>
       </c>
       <c r="B188" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C188" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O188" s="15" t="s">
-        <v>362</v>
-      </c>
-      <c r="AB188" s="14"/>
-      <c r="AC188" s="14"/>
-      <c r="AD188" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D188" s="18" t="s">
+        <v>632</v>
+      </c>
+      <c r="E188" s="14"/>
+      <c r="F188" s="14"/>
+      <c r="G188" s="14"/>
+      <c r="H188" s="14"/>
+      <c r="I188" s="14"/>
+      <c r="J188" s="14"/>
+      <c r="K188" s="14"/>
+      <c r="L188" s="31"/>
+      <c r="M188" s="30"/>
+      <c r="N188" s="14"/>
+      <c r="O188" s="14"/>
+      <c r="P188" s="14"/>
+      <c r="Q188" s="14"/>
+      <c r="R188" s="14"/>
+      <c r="S188" s="14"/>
+      <c r="T188" s="14"/>
+      <c r="U188" s="14"/>
+      <c r="V188" s="14"/>
+      <c r="W188" s="14"/>
+      <c r="X188" s="14"/>
+      <c r="Y188" s="14"/>
+      <c r="Z188" s="14"/>
+      <c r="AA188" s="14"/>
+      <c r="AB188" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC188" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD188" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE188" s="27"/>
       <c r="AF188" s="14"/>
       <c r="AG188" s="14"/>
-      <c r="AH188" s="14"/>
+      <c r="AH188" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI188" s="14"/>
     </row>
-    <row r="189" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="14" t="s">
-        <v>360</v>
+        <v>630</v>
       </c>
       <c r="B189" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C189" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O189" s="15" t="s">
-        <v>363</v>
-      </c>
-      <c r="AB189" s="14"/>
-      <c r="AC189" s="14"/>
-      <c r="AD189" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D189" s="18" t="s">
+        <v>633</v>
+      </c>
+      <c r="E189" s="14"/>
+      <c r="F189" s="14"/>
+      <c r="G189" s="14"/>
+      <c r="H189" s="14"/>
+      <c r="I189" s="14"/>
+      <c r="J189" s="14"/>
+      <c r="K189" s="14"/>
+      <c r="L189" s="31"/>
+      <c r="M189" s="30"/>
+      <c r="N189" s="14"/>
+      <c r="O189" s="14"/>
+      <c r="P189" s="14"/>
+      <c r="Q189" s="14"/>
+      <c r="R189" s="14"/>
+      <c r="S189" s="14"/>
+      <c r="T189" s="14"/>
+      <c r="U189" s="14"/>
+      <c r="V189" s="14"/>
+      <c r="W189" s="14"/>
+      <c r="X189" s="14"/>
+      <c r="Y189" s="14"/>
+      <c r="Z189" s="14"/>
+      <c r="AA189" s="14"/>
+      <c r="AB189" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC189" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD189" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE189" s="27"/>
       <c r="AF189" s="14"/>
       <c r="AG189" s="14"/>
-      <c r="AH189" s="14"/>
+      <c r="AH189" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI189" s="14"/>
     </row>
-    <row r="190" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A190" s="14" t="s">
-        <v>361</v>
-      </c>
-      <c r="B190" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C190" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O190" s="15" t="s">
-        <v>364</v>
-      </c>
+    <row r="190" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="14"/>
+      <c r="B190" s="14"/>
+      <c r="C190" s="14"/>
+      <c r="D190" s="14"/>
+      <c r="E190" s="14"/>
+      <c r="F190" s="14"/>
+      <c r="G190" s="14"/>
+      <c r="H190" s="14"/>
+      <c r="I190" s="14"/>
+      <c r="J190" s="14"/>
+      <c r="K190" s="14"/>
+      <c r="L190" s="14"/>
+      <c r="M190" s="14"/>
+      <c r="N190" s="14"/>
+      <c r="O190" s="14"/>
+      <c r="P190" s="14"/>
+      <c r="Q190" s="14"/>
+      <c r="R190" s="14"/>
+      <c r="S190" s="14"/>
+      <c r="T190" s="14"/>
+      <c r="U190" s="14"/>
+      <c r="V190" s="14"/>
+      <c r="W190" s="14"/>
+      <c r="X190" s="14"/>
+      <c r="Y190" s="14"/>
+      <c r="Z190" s="14"/>
+      <c r="AA190" s="14"/>
       <c r="AB190" s="14"/>
       <c r="AC190" s="14"/>
       <c r="AD190" s="14"/>
@@ -11230,9 +11383,9 @@
       <c r="AH190" s="14"/>
       <c r="AI190" s="14"/>
     </row>
-    <row r="191" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="14" t="s">
-        <v>370</v>
+        <v>267</v>
       </c>
       <c r="B191" s="14" t="s">
         <v>174</v>
@@ -11240,9 +11393,36 @@
       <c r="C191" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M191" s="14" t="s">
-        <v>371</v>
-      </c>
+      <c r="D191" s="14"/>
+      <c r="E191" s="14"/>
+      <c r="F191" s="14"/>
+      <c r="G191" s="14"/>
+      <c r="H191" s="14"/>
+      <c r="I191" s="14"/>
+      <c r="J191" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K191" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L191" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M191" s="14"/>
+      <c r="N191" s="14"/>
+      <c r="O191" s="14"/>
+      <c r="P191" s="14"/>
+      <c r="Q191" s="14"/>
+      <c r="R191" s="14"/>
+      <c r="S191" s="14"/>
+      <c r="T191" s="14"/>
+      <c r="U191" s="14"/>
+      <c r="V191" s="14"/>
+      <c r="W191" s="14"/>
+      <c r="X191" s="14"/>
+      <c r="Y191" s="14"/>
+      <c r="Z191" s="14"/>
+      <c r="AA191" s="14"/>
       <c r="AB191" s="14"/>
       <c r="AC191" s="14"/>
       <c r="AD191" s="14"/>
@@ -11252,7 +11432,46 @@
       <c r="AH191" s="14"/>
       <c r="AI191" s="14"/>
     </row>
-    <row r="192" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="B192" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C192" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D192" s="14"/>
+      <c r="E192" s="14"/>
+      <c r="F192" s="14"/>
+      <c r="G192" s="14"/>
+      <c r="H192" s="14"/>
+      <c r="I192" s="14"/>
+      <c r="J192" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K192" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L192" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M192" s="14"/>
+      <c r="N192" s="14"/>
+      <c r="O192" s="14"/>
+      <c r="P192" s="14"/>
+      <c r="Q192" s="14"/>
+      <c r="R192" s="14"/>
+      <c r="S192" s="14"/>
+      <c r="T192" s="14"/>
+      <c r="U192" s="14"/>
+      <c r="V192" s="14"/>
+      <c r="W192" s="14"/>
+      <c r="X192" s="14"/>
+      <c r="Y192" s="14"/>
+      <c r="Z192" s="14"/>
+      <c r="AA192" s="14"/>
       <c r="AB192" s="14"/>
       <c r="AC192" s="14"/>
       <c r="AD192" s="14"/>
@@ -11262,7 +11481,19 @@
       <c r="AH192" s="14"/>
       <c r="AI192" s="14"/>
     </row>
-    <row r="193" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A193" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="B193" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C193" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O193" s="15" t="s">
+        <v>362</v>
+      </c>
       <c r="AB193" s="14"/>
       <c r="AC193" s="14"/>
       <c r="AD193" s="14"/>
@@ -11272,7 +11503,19 @@
       <c r="AH193" s="14"/>
       <c r="AI193" s="14"/>
     </row>
-    <row r="194" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A194" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B194" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C194" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O194" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB194" s="14"/>
       <c r="AC194" s="14"/>
       <c r="AD194" s="14"/>
@@ -11282,7 +11525,19 @@
       <c r="AH194" s="14"/>
       <c r="AI194" s="14"/>
     </row>
-    <row r="195" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A195" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B195" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C195" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O195" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB195" s="14"/>
       <c r="AC195" s="14"/>
       <c r="AD195" s="14"/>
@@ -11292,7 +11547,19 @@
       <c r="AH195" s="14"/>
       <c r="AI195" s="14"/>
     </row>
-    <row r="196" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A196" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B196" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C196" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M196" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB196" s="14"/>
       <c r="AC196" s="14"/>
       <c r="AD196" s="14"/>
@@ -11302,7 +11569,7 @@
       <c r="AH196" s="14"/>
       <c r="AI196" s="14"/>
     </row>
-    <row r="197" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB197" s="14"/>
       <c r="AC197" s="14"/>
       <c r="AD197" s="14"/>
@@ -11312,7 +11579,7 @@
       <c r="AH197" s="14"/>
       <c r="AI197" s="14"/>
     </row>
-    <row r="198" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB198" s="14"/>
       <c r="AC198" s="14"/>
       <c r="AD198" s="14"/>
@@ -11322,7 +11589,7 @@
       <c r="AH198" s="14"/>
       <c r="AI198" s="14"/>
     </row>
-    <row r="199" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB199" s="14"/>
       <c r="AC199" s="14"/>
       <c r="AD199" s="14"/>
@@ -11332,7 +11599,7 @@
       <c r="AH199" s="14"/>
       <c r="AI199" s="14"/>
     </row>
-    <row r="200" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB200" s="14"/>
       <c r="AC200" s="14"/>
       <c r="AD200" s="14"/>
@@ -11342,7 +11609,7 @@
       <c r="AH200" s="14"/>
       <c r="AI200" s="14"/>
     </row>
-    <row r="201" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB201" s="14"/>
       <c r="AC201" s="14"/>
       <c r="AD201" s="14"/>
@@ -11352,7 +11619,7 @@
       <c r="AH201" s="14"/>
       <c r="AI201" s="14"/>
     </row>
-    <row r="202" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB202" s="14"/>
       <c r="AC202" s="14"/>
       <c r="AD202" s="14"/>
@@ -11362,7 +11629,7 @@
       <c r="AH202" s="14"/>
       <c r="AI202" s="14"/>
     </row>
-    <row r="203" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB203" s="14"/>
       <c r="AC203" s="14"/>
       <c r="AD203" s="14"/>
@@ -11372,7 +11639,7 @@
       <c r="AH203" s="14"/>
       <c r="AI203" s="14"/>
     </row>
-    <row r="204" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB204" s="14"/>
       <c r="AC204" s="14"/>
       <c r="AD204" s="14"/>
@@ -11382,7 +11649,7 @@
       <c r="AH204" s="14"/>
       <c r="AI204" s="14"/>
     </row>
-    <row r="205" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB205" s="14"/>
       <c r="AC205" s="14"/>
       <c r="AD205" s="14"/>
@@ -11392,7 +11659,7 @@
       <c r="AH205" s="14"/>
       <c r="AI205" s="14"/>
     </row>
-    <row r="206" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB206" s="14"/>
       <c r="AC206" s="14"/>
       <c r="AD206" s="14"/>
@@ -11402,7 +11669,7 @@
       <c r="AH206" s="14"/>
       <c r="AI206" s="14"/>
     </row>
-    <row r="207" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB207" s="14"/>
       <c r="AC207" s="14"/>
       <c r="AD207" s="14"/>
@@ -11412,7 +11679,7 @@
       <c r="AH207" s="14"/>
       <c r="AI207" s="14"/>
     </row>
-    <row r="208" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB208" s="14"/>
       <c r="AC208" s="14"/>
       <c r="AD208" s="14"/>
@@ -13236,7 +13503,7 @@
       <c r="AB390" s="14"/>
       <c r="AC390" s="14"/>
       <c r="AD390" s="14"/>
-      <c r="AE390" s="14"/>
+      <c r="AE390" s="27"/>
       <c r="AF390" s="14"/>
       <c r="AG390" s="14"/>
       <c r="AH390" s="14"/>
@@ -13246,7 +13513,7 @@
       <c r="AB391" s="14"/>
       <c r="AC391" s="14"/>
       <c r="AD391" s="14"/>
-      <c r="AE391" s="14"/>
+      <c r="AE391" s="27"/>
       <c r="AF391" s="14"/>
       <c r="AG391" s="14"/>
       <c r="AH391" s="14"/>
@@ -13256,7 +13523,7 @@
       <c r="AB392" s="14"/>
       <c r="AC392" s="14"/>
       <c r="AD392" s="14"/>
-      <c r="AE392" s="14"/>
+      <c r="AE392" s="27"/>
       <c r="AF392" s="14"/>
       <c r="AG392" s="14"/>
       <c r="AH392" s="14"/>
@@ -13266,7 +13533,7 @@
       <c r="AB393" s="14"/>
       <c r="AC393" s="14"/>
       <c r="AD393" s="14"/>
-      <c r="AE393" s="14"/>
+      <c r="AE393" s="27"/>
       <c r="AF393" s="14"/>
       <c r="AG393" s="14"/>
       <c r="AH393" s="14"/>
@@ -13276,7 +13543,7 @@
       <c r="AB394" s="14"/>
       <c r="AC394" s="14"/>
       <c r="AD394" s="14"/>
-      <c r="AE394" s="14"/>
+      <c r="AE394" s="27"/>
       <c r="AF394" s="14"/>
       <c r="AG394" s="14"/>
       <c r="AH394" s="14"/>
@@ -13302,6 +13569,56 @@
       <c r="AH396" s="14"/>
       <c r="AI396" s="14"/>
     </row>
+    <row r="397" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB397" s="14"/>
+      <c r="AC397" s="14"/>
+      <c r="AD397" s="14"/>
+      <c r="AE397" s="14"/>
+      <c r="AF397" s="14"/>
+      <c r="AG397" s="14"/>
+      <c r="AH397" s="14"/>
+      <c r="AI397" s="14"/>
+    </row>
+    <row r="398" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB398" s="14"/>
+      <c r="AC398" s="14"/>
+      <c r="AD398" s="14"/>
+      <c r="AE398" s="14"/>
+      <c r="AF398" s="14"/>
+      <c r="AG398" s="14"/>
+      <c r="AH398" s="14"/>
+      <c r="AI398" s="14"/>
+    </row>
+    <row r="399" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB399" s="14"/>
+      <c r="AC399" s="14"/>
+      <c r="AD399" s="14"/>
+      <c r="AE399" s="14"/>
+      <c r="AF399" s="14"/>
+      <c r="AG399" s="14"/>
+      <c r="AH399" s="14"/>
+      <c r="AI399" s="14"/>
+    </row>
+    <row r="400" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB400" s="14"/>
+      <c r="AC400" s="14"/>
+      <c r="AD400" s="14"/>
+      <c r="AE400" s="14"/>
+      <c r="AF400" s="14"/>
+      <c r="AG400" s="14"/>
+      <c r="AH400" s="14"/>
+      <c r="AI400" s="14"/>
+    </row>
+    <row r="401" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB401" s="14"/>
+      <c r="AC401" s="14"/>
+      <c r="AD401" s="14"/>
+      <c r="AE401" s="14"/>
+      <c r="AF401" s="14"/>
+      <c r="AG401" s="14"/>
+      <c r="AH401" s="14"/>
+      <c r="AI401" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13311,7 +13628,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T188"/>
+  <dimension ref="A1:T193"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -19414,23 +19731,21 @@
         <v>615</v>
       </c>
       <c r="B187" s="20" t="s">
-        <v>398</v>
+        <v>619</v>
       </c>
       <c r="C187" s="15" t="s">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="D187" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E187" s="15" t="s">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="F187" s="15"/>
       <c r="G187" s="15"/>
       <c r="H187" s="15"/>
-      <c r="I187" s="14" t="s">
-        <v>403</v>
-      </c>
+      <c r="I187" s="14"/>
       <c r="J187" s="14"/>
       <c r="K187" s="14"/>
       <c r="L187" s="14"/>
@@ -19448,21 +19763,23 @@
         <v>618</v>
       </c>
       <c r="B188" s="20" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="C188" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D188" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E188" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F188" s="15"/>
       <c r="G188" s="15"/>
       <c r="H188" s="15"/>
-      <c r="I188" s="14"/>
+      <c r="I188" s="14" t="s">
+        <v>627</v>
+      </c>
       <c r="J188" s="14"/>
       <c r="K188" s="14"/>
       <c r="L188" s="14"/>
@@ -19474,6 +19791,176 @@
       <c r="R188" s="14"/>
       <c r="S188" s="14"/>
       <c r="T188" s="14"/>
+    </row>
+    <row r="189" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="15" t="s">
+        <v>623</v>
+      </c>
+      <c r="B189" s="20" t="s">
+        <v>625</v>
+      </c>
+      <c r="C189" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D189" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E189" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F189" s="15"/>
+      <c r="G189" s="15"/>
+      <c r="H189" s="15"/>
+      <c r="I189" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J189" s="14"/>
+      <c r="K189" s="14"/>
+      <c r="L189" s="14"/>
+      <c r="M189" s="14"/>
+      <c r="N189" s="14"/>
+      <c r="O189" s="14"/>
+      <c r="P189" s="14"/>
+      <c r="Q189" s="14"/>
+      <c r="R189" s="14"/>
+      <c r="S189" s="14"/>
+      <c r="T189" s="14"/>
+    </row>
+    <row r="190" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="15" t="s">
+        <v>624</v>
+      </c>
+      <c r="B190" s="20" t="s">
+        <v>626</v>
+      </c>
+      <c r="C190" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D190" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E190" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F190" s="15"/>
+      <c r="G190" s="15"/>
+      <c r="H190" s="15"/>
+      <c r="I190" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J190" s="14"/>
+      <c r="K190" s="14"/>
+      <c r="L190" s="14"/>
+      <c r="M190" s="14"/>
+      <c r="N190" s="14"/>
+      <c r="O190" s="14"/>
+      <c r="P190" s="14"/>
+      <c r="Q190" s="14"/>
+      <c r="R190" s="14"/>
+      <c r="S190" s="14"/>
+      <c r="T190" s="14"/>
+    </row>
+    <row r="191" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="15" t="s">
+        <v>631</v>
+      </c>
+      <c r="B191" s="20" t="s">
+        <v>634</v>
+      </c>
+      <c r="C191" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D191" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E191" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F191" s="15"/>
+      <c r="G191" s="15"/>
+      <c r="H191" s="15"/>
+      <c r="I191" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J191" s="14"/>
+      <c r="K191" s="14"/>
+      <c r="L191" s="14"/>
+      <c r="M191" s="14"/>
+      <c r="N191" s="14"/>
+      <c r="O191" s="14"/>
+      <c r="P191" s="14"/>
+      <c r="Q191" s="14"/>
+      <c r="R191" s="14"/>
+      <c r="S191" s="14"/>
+      <c r="T191" s="14"/>
+    </row>
+    <row r="192" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="15" t="s">
+        <v>632</v>
+      </c>
+      <c r="B192" s="20" t="s">
+        <v>636</v>
+      </c>
+      <c r="C192" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D192" s="14" t="s">
+        <v>637</v>
+      </c>
+      <c r="E192" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F192" s="15"/>
+      <c r="G192" s="15"/>
+      <c r="H192" s="15"/>
+      <c r="I192" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J192" s="14"/>
+      <c r="K192" s="14"/>
+      <c r="L192" s="14"/>
+      <c r="M192" s="14"/>
+      <c r="N192" s="14"/>
+      <c r="O192" s="14"/>
+      <c r="P192" s="14"/>
+      <c r="Q192" s="14"/>
+      <c r="R192" s="14"/>
+      <c r="S192" s="14"/>
+      <c r="T192" s="14"/>
+    </row>
+    <row r="193" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="15" t="s">
+        <v>633</v>
+      </c>
+      <c r="B193" s="20" t="s">
+        <v>635</v>
+      </c>
+      <c r="C193" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D193" s="14" t="s">
+        <v>637</v>
+      </c>
+      <c r="E193" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F193" s="15"/>
+      <c r="G193" s="15"/>
+      <c r="H193" s="15"/>
+      <c r="I193" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J193" s="14"/>
+      <c r="K193" s="14"/>
+      <c r="L193" s="14"/>
+      <c r="M193" s="14"/>
+      <c r="N193" s="14"/>
+      <c r="O193" s="14"/>
+      <c r="P193" s="14"/>
+      <c r="Q193" s="14"/>
+      <c r="R193" s="14"/>
+      <c r="S193" s="14"/>
+      <c r="T193" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
Commit after added MultiLine scenarios for APC
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B696DC65-778D-4E11-8A79-39C712858F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C360B131-7D99-476B-A0FF-E72ACFD87CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2734" uniqueCount="638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2804" uniqueCount="655">
   <si>
     <t>1</t>
   </si>
@@ -1942,6 +1942,57 @@
   </si>
   <si>
     <t>BX</t>
+  </si>
+  <si>
+    <t>APC_IBScenario007</t>
+  </si>
+  <si>
+    <t>979</t>
+  </si>
+  <si>
+    <t>978|979</t>
+  </si>
+  <si>
+    <t>APC_IBScenario008</t>
+  </si>
+  <si>
+    <t>976|977</t>
+  </si>
+  <si>
+    <t>980</t>
+  </si>
+  <si>
+    <t>01R21-71</t>
+  </si>
+  <si>
+    <t>981</t>
+  </si>
+  <si>
+    <t>01R21-02</t>
+  </si>
+  <si>
+    <t>APC_IBScenario009</t>
+  </si>
+  <si>
+    <t>980|981</t>
+  </si>
+  <si>
+    <t>982</t>
+  </si>
+  <si>
+    <t>983</t>
+  </si>
+  <si>
+    <t>APC_IBScenario010</t>
+  </si>
+  <si>
+    <t>APC_IBScenario011</t>
+  </si>
+  <si>
+    <t>978|982</t>
+  </si>
+  <si>
+    <t>983|982</t>
   </si>
 </sst>
 </file>
@@ -2485,7 +2536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI401"/>
+  <dimension ref="A1:AI406"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -11347,10 +11398,18 @@
       <c r="AI189" s="14"/>
     </row>
     <row r="190" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A190" s="14"/>
-      <c r="B190" s="14"/>
-      <c r="C190" s="14"/>
-      <c r="D190" s="14"/>
+      <c r="A190" s="14" t="s">
+        <v>638</v>
+      </c>
+      <c r="B190" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C190" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D190" s="18" t="s">
+        <v>640</v>
+      </c>
       <c r="E190" s="14"/>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -11358,8 +11417,8 @@
       <c r="I190" s="14"/>
       <c r="J190" s="14"/>
       <c r="K190" s="14"/>
-      <c r="L190" s="14"/>
-      <c r="M190" s="14"/>
+      <c r="L190" s="31"/>
+      <c r="M190" s="30"/>
       <c r="N190" s="14"/>
       <c r="O190" s="14"/>
       <c r="P190" s="14"/>
@@ -11374,41 +11433,45 @@
       <c r="Y190" s="14"/>
       <c r="Z190" s="14"/>
       <c r="AA190" s="14"/>
-      <c r="AB190" s="14"/>
-      <c r="AC190" s="14"/>
-      <c r="AD190" s="14"/>
+      <c r="AB190" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC190" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD190" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE190" s="27"/>
       <c r="AF190" s="14"/>
       <c r="AG190" s="14"/>
-      <c r="AH190" s="14"/>
+      <c r="AH190" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI190" s="14"/>
     </row>
     <row r="191" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="14" t="s">
-        <v>267</v>
+        <v>641</v>
       </c>
       <c r="B191" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C191" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D191" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D191" s="18" t="s">
+        <v>642</v>
+      </c>
       <c r="E191" s="14"/>
       <c r="F191" s="14"/>
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
       <c r="I191" s="14"/>
-      <c r="J191" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K191" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L191" s="15" t="s">
-        <v>275</v>
-      </c>
-      <c r="M191" s="14"/>
+      <c r="J191" s="14"/>
+      <c r="K191" s="14"/>
+      <c r="L191" s="31"/>
+      <c r="M191" s="30"/>
       <c r="N191" s="14"/>
       <c r="O191" s="14"/>
       <c r="P191" s="14"/>
@@ -11423,41 +11486,45 @@
       <c r="Y191" s="14"/>
       <c r="Z191" s="14"/>
       <c r="AA191" s="14"/>
-      <c r="AB191" s="14"/>
-      <c r="AC191" s="14"/>
-      <c r="AD191" s="14"/>
+      <c r="AB191" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC191" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD191" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE191" s="27"/>
       <c r="AF191" s="14"/>
       <c r="AG191" s="14"/>
-      <c r="AH191" s="14"/>
+      <c r="AH191" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI191" s="14"/>
     </row>
     <row r="192" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="14" t="s">
-        <v>268</v>
+        <v>647</v>
       </c>
       <c r="B192" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C192" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D192" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D192" s="18" t="s">
+        <v>648</v>
+      </c>
       <c r="E192" s="14"/>
       <c r="F192" s="14"/>
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
       <c r="I192" s="14"/>
-      <c r="J192" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K192" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L192" s="15" t="s">
-        <v>276</v>
-      </c>
-      <c r="M192" s="14"/>
+      <c r="J192" s="14"/>
+      <c r="K192" s="14"/>
+      <c r="L192" s="31"/>
+      <c r="M192" s="30"/>
       <c r="N192" s="14"/>
       <c r="O192" s="14"/>
       <c r="P192" s="14"/>
@@ -11472,72 +11539,157 @@
       <c r="Y192" s="14"/>
       <c r="Z192" s="14"/>
       <c r="AA192" s="14"/>
-      <c r="AB192" s="14"/>
-      <c r="AC192" s="14"/>
-      <c r="AD192" s="14"/>
+      <c r="AB192" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC192" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD192" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE192" s="27"/>
       <c r="AF192" s="14"/>
       <c r="AG192" s="14"/>
-      <c r="AH192" s="14"/>
+      <c r="AH192" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI192" s="14"/>
     </row>
-    <row r="193" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="14" t="s">
-        <v>359</v>
+        <v>651</v>
       </c>
       <c r="B193" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C193" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O193" s="15" t="s">
-        <v>362</v>
-      </c>
-      <c r="AB193" s="14"/>
-      <c r="AC193" s="14"/>
-      <c r="AD193" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D193" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="E193" s="14"/>
+      <c r="F193" s="14"/>
+      <c r="G193" s="14"/>
+      <c r="H193" s="14"/>
+      <c r="I193" s="14"/>
+      <c r="J193" s="14"/>
+      <c r="K193" s="14"/>
+      <c r="L193" s="31"/>
+      <c r="M193" s="30"/>
+      <c r="N193" s="14"/>
+      <c r="O193" s="14"/>
+      <c r="P193" s="14"/>
+      <c r="Q193" s="14"/>
+      <c r="R193" s="14"/>
+      <c r="S193" s="14"/>
+      <c r="T193" s="14"/>
+      <c r="U193" s="14"/>
+      <c r="V193" s="14"/>
+      <c r="W193" s="14"/>
+      <c r="X193" s="14"/>
+      <c r="Y193" s="14"/>
+      <c r="Z193" s="14"/>
+      <c r="AA193" s="14"/>
+      <c r="AB193" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC193" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD193" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE193" s="27"/>
       <c r="AF193" s="14"/>
       <c r="AG193" s="14"/>
-      <c r="AH193" s="14"/>
+      <c r="AH193" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI193" s="14"/>
     </row>
-    <row r="194" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="14" t="s">
-        <v>360</v>
+        <v>652</v>
       </c>
       <c r="B194" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C194" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O194" s="15" t="s">
-        <v>363</v>
-      </c>
-      <c r="AB194" s="14"/>
-      <c r="AC194" s="14"/>
-      <c r="AD194" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D194" s="18" t="s">
+        <v>654</v>
+      </c>
+      <c r="E194" s="14"/>
+      <c r="F194" s="14"/>
+      <c r="G194" s="14"/>
+      <c r="H194" s="14"/>
+      <c r="I194" s="14"/>
+      <c r="J194" s="14"/>
+      <c r="K194" s="14"/>
+      <c r="L194" s="31"/>
+      <c r="M194" s="30"/>
+      <c r="N194" s="14"/>
+      <c r="O194" s="14"/>
+      <c r="P194" s="14"/>
+      <c r="Q194" s="14"/>
+      <c r="R194" s="14"/>
+      <c r="S194" s="14"/>
+      <c r="T194" s="14"/>
+      <c r="U194" s="14"/>
+      <c r="V194" s="14"/>
+      <c r="W194" s="14"/>
+      <c r="X194" s="14"/>
+      <c r="Y194" s="14"/>
+      <c r="Z194" s="14"/>
+      <c r="AA194" s="14"/>
+      <c r="AB194" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC194" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD194" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE194" s="27"/>
       <c r="AF194" s="14"/>
       <c r="AG194" s="14"/>
-      <c r="AH194" s="14"/>
+      <c r="AH194" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI194" s="14"/>
     </row>
-    <row r="195" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A195" s="14" t="s">
-        <v>361</v>
-      </c>
-      <c r="B195" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C195" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O195" s="15" t="s">
-        <v>364</v>
-      </c>
+    <row r="195" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="14"/>
+      <c r="B195" s="14"/>
+      <c r="C195" s="14"/>
+      <c r="D195" s="14"/>
+      <c r="E195" s="14"/>
+      <c r="F195" s="14"/>
+      <c r="G195" s="14"/>
+      <c r="H195" s="14"/>
+      <c r="I195" s="14"/>
+      <c r="J195" s="14"/>
+      <c r="K195" s="14"/>
+      <c r="L195" s="14"/>
+      <c r="M195" s="14"/>
+      <c r="N195" s="14"/>
+      <c r="O195" s="14"/>
+      <c r="P195" s="14"/>
+      <c r="Q195" s="14"/>
+      <c r="R195" s="14"/>
+      <c r="S195" s="14"/>
+      <c r="T195" s="14"/>
+      <c r="U195" s="14"/>
+      <c r="V195" s="14"/>
+      <c r="W195" s="14"/>
+      <c r="X195" s="14"/>
+      <c r="Y195" s="14"/>
+      <c r="Z195" s="14"/>
+      <c r="AA195" s="14"/>
       <c r="AB195" s="14"/>
       <c r="AC195" s="14"/>
       <c r="AD195" s="14"/>
@@ -11547,9 +11699,9 @@
       <c r="AH195" s="14"/>
       <c r="AI195" s="14"/>
     </row>
-    <row r="196" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="14" t="s">
-        <v>370</v>
+        <v>267</v>
       </c>
       <c r="B196" s="14" t="s">
         <v>174</v>
@@ -11557,9 +11709,36 @@
       <c r="C196" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M196" s="14" t="s">
-        <v>371</v>
-      </c>
+      <c r="D196" s="14"/>
+      <c r="E196" s="14"/>
+      <c r="F196" s="14"/>
+      <c r="G196" s="14"/>
+      <c r="H196" s="14"/>
+      <c r="I196" s="14"/>
+      <c r="J196" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K196" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L196" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M196" s="14"/>
+      <c r="N196" s="14"/>
+      <c r="O196" s="14"/>
+      <c r="P196" s="14"/>
+      <c r="Q196" s="14"/>
+      <c r="R196" s="14"/>
+      <c r="S196" s="14"/>
+      <c r="T196" s="14"/>
+      <c r="U196" s="14"/>
+      <c r="V196" s="14"/>
+      <c r="W196" s="14"/>
+      <c r="X196" s="14"/>
+      <c r="Y196" s="14"/>
+      <c r="Z196" s="14"/>
+      <c r="AA196" s="14"/>
       <c r="AB196" s="14"/>
       <c r="AC196" s="14"/>
       <c r="AD196" s="14"/>
@@ -11569,7 +11748,46 @@
       <c r="AH196" s="14"/>
       <c r="AI196" s="14"/>
     </row>
-    <row r="197" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="B197" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C197" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D197" s="14"/>
+      <c r="E197" s="14"/>
+      <c r="F197" s="14"/>
+      <c r="G197" s="14"/>
+      <c r="H197" s="14"/>
+      <c r="I197" s="14"/>
+      <c r="J197" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K197" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L197" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M197" s="14"/>
+      <c r="N197" s="14"/>
+      <c r="O197" s="14"/>
+      <c r="P197" s="14"/>
+      <c r="Q197" s="14"/>
+      <c r="R197" s="14"/>
+      <c r="S197" s="14"/>
+      <c r="T197" s="14"/>
+      <c r="U197" s="14"/>
+      <c r="V197" s="14"/>
+      <c r="W197" s="14"/>
+      <c r="X197" s="14"/>
+      <c r="Y197" s="14"/>
+      <c r="Z197" s="14"/>
+      <c r="AA197" s="14"/>
       <c r="AB197" s="14"/>
       <c r="AC197" s="14"/>
       <c r="AD197" s="14"/>
@@ -11580,6 +11798,18 @@
       <c r="AI197" s="14"/>
     </row>
     <row r="198" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A198" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="B198" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C198" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O198" s="15" t="s">
+        <v>362</v>
+      </c>
       <c r="AB198" s="14"/>
       <c r="AC198" s="14"/>
       <c r="AD198" s="14"/>
@@ -11590,6 +11820,18 @@
       <c r="AI198" s="14"/>
     </row>
     <row r="199" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A199" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B199" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C199" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O199" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB199" s="14"/>
       <c r="AC199" s="14"/>
       <c r="AD199" s="14"/>
@@ -11600,6 +11842,18 @@
       <c r="AI199" s="14"/>
     </row>
     <row r="200" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A200" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B200" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C200" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O200" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB200" s="14"/>
       <c r="AC200" s="14"/>
       <c r="AD200" s="14"/>
@@ -11610,6 +11864,18 @@
       <c r="AI200" s="14"/>
     </row>
     <row r="201" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A201" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B201" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C201" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M201" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB201" s="14"/>
       <c r="AC201" s="14"/>
       <c r="AD201" s="14"/>
@@ -13553,7 +13819,7 @@
       <c r="AB395" s="14"/>
       <c r="AC395" s="14"/>
       <c r="AD395" s="14"/>
-      <c r="AE395" s="14"/>
+      <c r="AE395" s="27"/>
       <c r="AF395" s="14"/>
       <c r="AG395" s="14"/>
       <c r="AH395" s="14"/>
@@ -13563,7 +13829,7 @@
       <c r="AB396" s="14"/>
       <c r="AC396" s="14"/>
       <c r="AD396" s="14"/>
-      <c r="AE396" s="14"/>
+      <c r="AE396" s="27"/>
       <c r="AF396" s="14"/>
       <c r="AG396" s="14"/>
       <c r="AH396" s="14"/>
@@ -13573,7 +13839,7 @@
       <c r="AB397" s="14"/>
       <c r="AC397" s="14"/>
       <c r="AD397" s="14"/>
-      <c r="AE397" s="14"/>
+      <c r="AE397" s="27"/>
       <c r="AF397" s="14"/>
       <c r="AG397" s="14"/>
       <c r="AH397" s="14"/>
@@ -13583,7 +13849,7 @@
       <c r="AB398" s="14"/>
       <c r="AC398" s="14"/>
       <c r="AD398" s="14"/>
-      <c r="AE398" s="14"/>
+      <c r="AE398" s="27"/>
       <c r="AF398" s="14"/>
       <c r="AG398" s="14"/>
       <c r="AH398" s="14"/>
@@ -13593,7 +13859,7 @@
       <c r="AB399" s="14"/>
       <c r="AC399" s="14"/>
       <c r="AD399" s="14"/>
-      <c r="AE399" s="14"/>
+      <c r="AE399" s="27"/>
       <c r="AF399" s="14"/>
       <c r="AG399" s="14"/>
       <c r="AH399" s="14"/>
@@ -13619,6 +13885,56 @@
       <c r="AH401" s="14"/>
       <c r="AI401" s="14"/>
     </row>
+    <row r="402" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB402" s="14"/>
+      <c r="AC402" s="14"/>
+      <c r="AD402" s="14"/>
+      <c r="AE402" s="14"/>
+      <c r="AF402" s="14"/>
+      <c r="AG402" s="14"/>
+      <c r="AH402" s="14"/>
+      <c r="AI402" s="14"/>
+    </row>
+    <row r="403" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB403" s="14"/>
+      <c r="AC403" s="14"/>
+      <c r="AD403" s="14"/>
+      <c r="AE403" s="14"/>
+      <c r="AF403" s="14"/>
+      <c r="AG403" s="14"/>
+      <c r="AH403" s="14"/>
+      <c r="AI403" s="14"/>
+    </row>
+    <row r="404" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB404" s="14"/>
+      <c r="AC404" s="14"/>
+      <c r="AD404" s="14"/>
+      <c r="AE404" s="14"/>
+      <c r="AF404" s="14"/>
+      <c r="AG404" s="14"/>
+      <c r="AH404" s="14"/>
+      <c r="AI404" s="14"/>
+    </row>
+    <row r="405" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB405" s="14"/>
+      <c r="AC405" s="14"/>
+      <c r="AD405" s="14"/>
+      <c r="AE405" s="14"/>
+      <c r="AF405" s="14"/>
+      <c r="AG405" s="14"/>
+      <c r="AH405" s="14"/>
+      <c r="AI405" s="14"/>
+    </row>
+    <row r="406" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB406" s="14"/>
+      <c r="AC406" s="14"/>
+      <c r="AD406" s="14"/>
+      <c r="AE406" s="14"/>
+      <c r="AF406" s="14"/>
+      <c r="AG406" s="14"/>
+      <c r="AH406" s="14"/>
+      <c r="AI406" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13628,7 +13944,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T193"/>
+  <dimension ref="A1:T198"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -19962,6 +20278,176 @@
       <c r="S193" s="14"/>
       <c r="T193" s="14"/>
     </row>
+    <row r="194" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B194" s="20" t="s">
+        <v>620</v>
+      </c>
+      <c r="C194" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D194" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E194" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F194" s="15"/>
+      <c r="G194" s="15"/>
+      <c r="H194" s="15"/>
+      <c r="I194" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J194" s="14"/>
+      <c r="K194" s="14"/>
+      <c r="L194" s="14"/>
+      <c r="M194" s="14"/>
+      <c r="N194" s="14"/>
+      <c r="O194" s="14"/>
+      <c r="P194" s="14"/>
+      <c r="Q194" s="14"/>
+      <c r="R194" s="14"/>
+      <c r="S194" s="14"/>
+      <c r="T194" s="14"/>
+    </row>
+    <row r="195" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="15" t="s">
+        <v>643</v>
+      </c>
+      <c r="B195" s="20" t="s">
+        <v>644</v>
+      </c>
+      <c r="C195" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D195" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E195" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F195" s="15"/>
+      <c r="G195" s="15"/>
+      <c r="H195" s="15"/>
+      <c r="I195" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J195" s="14"/>
+      <c r="K195" s="14"/>
+      <c r="L195" s="14"/>
+      <c r="M195" s="14"/>
+      <c r="N195" s="14"/>
+      <c r="O195" s="14"/>
+      <c r="P195" s="14"/>
+      <c r="Q195" s="14"/>
+      <c r="R195" s="14"/>
+      <c r="S195" s="14"/>
+      <c r="T195" s="14"/>
+    </row>
+    <row r="196" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="15" t="s">
+        <v>645</v>
+      </c>
+      <c r="B196" s="20" t="s">
+        <v>646</v>
+      </c>
+      <c r="C196" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D196" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E196" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F196" s="15"/>
+      <c r="G196" s="15"/>
+      <c r="H196" s="15"/>
+      <c r="I196" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J196" s="14"/>
+      <c r="K196" s="14"/>
+      <c r="L196" s="14"/>
+      <c r="M196" s="14"/>
+      <c r="N196" s="14"/>
+      <c r="O196" s="14"/>
+      <c r="P196" s="14"/>
+      <c r="Q196" s="14"/>
+      <c r="R196" s="14"/>
+      <c r="S196" s="14"/>
+      <c r="T196" s="14"/>
+    </row>
+    <row r="197" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="15" t="s">
+        <v>649</v>
+      </c>
+      <c r="B197" s="20" t="s">
+        <v>635</v>
+      </c>
+      <c r="C197" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D197" s="14" t="s">
+        <v>637</v>
+      </c>
+      <c r="E197" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F197" s="15"/>
+      <c r="G197" s="15"/>
+      <c r="H197" s="15"/>
+      <c r="I197" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J197" s="14"/>
+      <c r="K197" s="14"/>
+      <c r="L197" s="14"/>
+      <c r="M197" s="14"/>
+      <c r="N197" s="14"/>
+      <c r="O197" s="14"/>
+      <c r="P197" s="14"/>
+      <c r="Q197" s="14"/>
+      <c r="R197" s="14"/>
+      <c r="S197" s="14"/>
+      <c r="T197" s="14"/>
+    </row>
+    <row r="198" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="15" t="s">
+        <v>650</v>
+      </c>
+      <c r="B198" s="20" t="s">
+        <v>635</v>
+      </c>
+      <c r="C198" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D198" s="14" t="s">
+        <v>637</v>
+      </c>
+      <c r="E198" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F198" s="15"/>
+      <c r="G198" s="15"/>
+      <c r="H198" s="15"/>
+      <c r="I198" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J198" s="14"/>
+      <c r="K198" s="14"/>
+      <c r="L198" s="14"/>
+      <c r="M198" s="14"/>
+      <c r="N198" s="14"/>
+      <c r="O198" s="14"/>
+      <c r="P198" s="14"/>
+      <c r="Q198" s="14"/>
+      <c r="R198" s="14"/>
+      <c r="S198" s="14"/>
+      <c r="T198" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Commit code after scripting APC MultiLine IB Scenarios
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C360B131-7D99-476B-A0FF-E72ACFD87CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF884550-870A-4B52-9E23-19B7EFDC3804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2804" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2810" uniqueCount="667">
   <si>
     <t>1</t>
   </si>
@@ -1938,9 +1938,6 @@
     <t>07P02-06</t>
   </si>
   <si>
-    <t>07P04-03</t>
-  </si>
-  <si>
     <t>BX</t>
   </si>
   <si>
@@ -1950,15 +1947,9 @@
     <t>979</t>
   </si>
   <si>
-    <t>978|979</t>
-  </si>
-  <si>
     <t>APC_IBScenario008</t>
   </si>
   <si>
-    <t>976|977</t>
-  </si>
-  <si>
     <t>980</t>
   </si>
   <si>
@@ -1974,9 +1965,6 @@
     <t>APC_IBScenario009</t>
   </si>
   <si>
-    <t>980|981</t>
-  </si>
-  <si>
     <t>982</t>
   </si>
   <si>
@@ -1989,10 +1977,58 @@
     <t>APC_IBScenario011</t>
   </si>
   <si>
-    <t>978|982</t>
-  </si>
-  <si>
-    <t>983|982</t>
+    <t>984</t>
+  </si>
+  <si>
+    <t>06F12-18</t>
+  </si>
+  <si>
+    <t>985</t>
+  </si>
+  <si>
+    <t>986</t>
+  </si>
+  <si>
+    <t>985|986</t>
+  </si>
+  <si>
+    <t>Abaxis</t>
+  </si>
+  <si>
+    <t>Ambient</t>
+  </si>
+  <si>
+    <t>Freezer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dangerous </t>
+  </si>
+  <si>
+    <t>06P17-26</t>
+  </si>
+  <si>
+    <t>Cooler</t>
+  </si>
+  <si>
+    <t>973|979</t>
+  </si>
+  <si>
+    <t>980|975</t>
+  </si>
+  <si>
+    <t>982|983</t>
+  </si>
+  <si>
+    <t>976|976</t>
+  </si>
+  <si>
+    <t>03P84-25</t>
+  </si>
+  <si>
+    <t>016967-00</t>
+  </si>
+  <si>
+    <t>03P51-01</t>
   </si>
 </sst>
 </file>
@@ -11096,7 +11132,9 @@
       <c r="F184" s="14"/>
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
-      <c r="I184" s="14"/>
+      <c r="I184" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J184" s="14"/>
       <c r="K184" s="14"/>
       <c r="L184" s="31"/>
@@ -11115,16 +11153,12 @@
       <c r="Y184" s="14"/>
       <c r="Z184" s="14"/>
       <c r="AA184" s="14"/>
-      <c r="AB184" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC184" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD184" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE184" s="27"/>
+      <c r="AB184" s="14"/>
+      <c r="AC184" s="14"/>
+      <c r="AD184" s="14"/>
+      <c r="AE184" s="27" t="s">
+        <v>659</v>
+      </c>
       <c r="AF184" s="14"/>
       <c r="AG184" s="14"/>
       <c r="AH184" s="14" t="s">
@@ -11149,7 +11183,9 @@
       <c r="F185" s="14"/>
       <c r="G185" s="14"/>
       <c r="H185" s="14"/>
-      <c r="I185" s="14"/>
+      <c r="I185" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J185" s="14"/>
       <c r="K185" s="14"/>
       <c r="L185" s="31"/>
@@ -11168,16 +11204,12 @@
       <c r="Y185" s="14"/>
       <c r="Z185" s="14"/>
       <c r="AA185" s="14"/>
-      <c r="AB185" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC185" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD185" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE185" s="27"/>
+      <c r="AB185" s="14"/>
+      <c r="AC185" s="14"/>
+      <c r="AD185" s="14"/>
+      <c r="AE185" s="27" t="s">
+        <v>655</v>
+      </c>
       <c r="AF185" s="14"/>
       <c r="AG185" s="14"/>
       <c r="AH185" s="14" t="s">
@@ -11202,7 +11234,9 @@
       <c r="F186" s="14"/>
       <c r="G186" s="14"/>
       <c r="H186" s="14"/>
-      <c r="I186" s="14"/>
+      <c r="I186" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J186" s="14"/>
       <c r="K186" s="14"/>
       <c r="L186" s="31"/>
@@ -11221,16 +11255,12 @@
       <c r="Y186" s="14"/>
       <c r="Z186" s="14"/>
       <c r="AA186" s="14"/>
-      <c r="AB186" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC186" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD186" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE186" s="27"/>
+      <c r="AB186" s="14"/>
+      <c r="AC186" s="14"/>
+      <c r="AD186" s="14"/>
+      <c r="AE186" s="27" t="s">
+        <v>655</v>
+      </c>
       <c r="AF186" s="14"/>
       <c r="AG186" s="14"/>
       <c r="AH186" s="14" t="s">
@@ -11255,7 +11285,9 @@
       <c r="F187" s="14"/>
       <c r="G187" s="14"/>
       <c r="H187" s="14"/>
-      <c r="I187" s="14"/>
+      <c r="I187" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J187" s="14"/>
       <c r="K187" s="14"/>
       <c r="L187" s="31"/>
@@ -11274,16 +11306,12 @@
       <c r="Y187" s="14"/>
       <c r="Z187" s="14"/>
       <c r="AA187" s="14"/>
-      <c r="AB187" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC187" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD187" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE187" s="27"/>
+      <c r="AB187" s="14"/>
+      <c r="AC187" s="14"/>
+      <c r="AD187" s="14"/>
+      <c r="AE187" s="27" t="s">
+        <v>657</v>
+      </c>
       <c r="AF187" s="14"/>
       <c r="AG187" s="14"/>
       <c r="AH187" s="14" t="s">
@@ -11308,7 +11336,9 @@
       <c r="F188" s="14"/>
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
-      <c r="I188" s="14"/>
+      <c r="I188" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J188" s="14"/>
       <c r="K188" s="14"/>
       <c r="L188" s="31"/>
@@ -11327,16 +11357,12 @@
       <c r="Y188" s="14"/>
       <c r="Z188" s="14"/>
       <c r="AA188" s="14"/>
-      <c r="AB188" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC188" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD188" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE188" s="27"/>
+      <c r="AB188" s="14"/>
+      <c r="AC188" s="14"/>
+      <c r="AD188" s="14"/>
+      <c r="AE188" s="27" t="s">
+        <v>656</v>
+      </c>
       <c r="AF188" s="14"/>
       <c r="AG188" s="14"/>
       <c r="AH188" s="14" t="s">
@@ -11361,7 +11387,9 @@
       <c r="F189" s="14"/>
       <c r="G189" s="14"/>
       <c r="H189" s="14"/>
-      <c r="I189" s="14"/>
+      <c r="I189" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J189" s="14"/>
       <c r="K189" s="14"/>
       <c r="L189" s="31"/>
@@ -11380,16 +11408,12 @@
       <c r="Y189" s="14"/>
       <c r="Z189" s="14"/>
       <c r="AA189" s="14"/>
-      <c r="AB189" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC189" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD189" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE189" s="27"/>
+      <c r="AB189" s="14"/>
+      <c r="AC189" s="14"/>
+      <c r="AD189" s="14"/>
+      <c r="AE189" s="27" t="s">
+        <v>654</v>
+      </c>
       <c r="AF189" s="14"/>
       <c r="AG189" s="14"/>
       <c r="AH189" s="14" t="s">
@@ -11399,7 +11423,7 @@
     </row>
     <row r="190" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="14" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B190" s="14" t="s">
         <v>613</v>
@@ -11408,13 +11432,15 @@
         <v>614</v>
       </c>
       <c r="D190" s="18" t="s">
-        <v>640</v>
+        <v>660</v>
       </c>
       <c r="E190" s="14"/>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
-      <c r="I190" s="14"/>
+      <c r="I190" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J190" s="14"/>
       <c r="K190" s="14"/>
       <c r="L190" s="31"/>
@@ -11433,16 +11459,12 @@
       <c r="Y190" s="14"/>
       <c r="Z190" s="14"/>
       <c r="AA190" s="14"/>
-      <c r="AB190" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC190" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD190" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE190" s="27"/>
+      <c r="AB190" s="14"/>
+      <c r="AC190" s="14"/>
+      <c r="AD190" s="14"/>
+      <c r="AE190" s="27" t="s">
+        <v>659</v>
+      </c>
       <c r="AF190" s="14"/>
       <c r="AG190" s="14"/>
       <c r="AH190" s="14" t="s">
@@ -11452,7 +11474,7 @@
     </row>
     <row r="191" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="14" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="B191" s="14" t="s">
         <v>613</v>
@@ -11461,13 +11483,15 @@
         <v>614</v>
       </c>
       <c r="D191" s="18" t="s">
-        <v>642</v>
+        <v>653</v>
       </c>
       <c r="E191" s="14"/>
       <c r="F191" s="14"/>
       <c r="G191" s="14"/>
       <c r="H191" s="14"/>
-      <c r="I191" s="14"/>
+      <c r="I191" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J191" s="14"/>
       <c r="K191" s="14"/>
       <c r="L191" s="31"/>
@@ -11486,16 +11510,12 @@
       <c r="Y191" s="14"/>
       <c r="Z191" s="14"/>
       <c r="AA191" s="14"/>
-      <c r="AB191" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC191" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD191" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE191" s="27"/>
+      <c r="AB191" s="14"/>
+      <c r="AC191" s="14"/>
+      <c r="AD191" s="14"/>
+      <c r="AE191" s="27" t="s">
+        <v>655</v>
+      </c>
       <c r="AF191" s="14"/>
       <c r="AG191" s="14"/>
       <c r="AH191" s="14" t="s">
@@ -11505,7 +11525,7 @@
     </row>
     <row r="192" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="14" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="B192" s="14" t="s">
         <v>613</v>
@@ -11514,13 +11534,15 @@
         <v>614</v>
       </c>
       <c r="D192" s="18" t="s">
-        <v>648</v>
+        <v>661</v>
       </c>
       <c r="E192" s="14"/>
       <c r="F192" s="14"/>
       <c r="G192" s="14"/>
       <c r="H192" s="14"/>
-      <c r="I192" s="14"/>
+      <c r="I192" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J192" s="14"/>
       <c r="K192" s="14"/>
       <c r="L192" s="31"/>
@@ -11539,16 +11561,12 @@
       <c r="Y192" s="14"/>
       <c r="Z192" s="14"/>
       <c r="AA192" s="14"/>
-      <c r="AB192" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC192" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD192" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE192" s="27"/>
+      <c r="AB192" s="14"/>
+      <c r="AC192" s="14"/>
+      <c r="AD192" s="14"/>
+      <c r="AE192" s="27" t="s">
+        <v>655</v>
+      </c>
       <c r="AF192" s="14"/>
       <c r="AG192" s="14"/>
       <c r="AH192" s="14" t="s">
@@ -11558,7 +11576,7 @@
     </row>
     <row r="193" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="14" t="s">
-        <v>651</v>
+        <v>647</v>
       </c>
       <c r="B193" s="14" t="s">
         <v>613</v>
@@ -11567,13 +11585,15 @@
         <v>614</v>
       </c>
       <c r="D193" s="18" t="s">
-        <v>653</v>
+        <v>662</v>
       </c>
       <c r="E193" s="14"/>
       <c r="F193" s="14"/>
       <c r="G193" s="14"/>
       <c r="H193" s="14"/>
-      <c r="I193" s="14"/>
+      <c r="I193" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J193" s="14"/>
       <c r="K193" s="14"/>
       <c r="L193" s="31"/>
@@ -11592,26 +11612,20 @@
       <c r="Y193" s="14"/>
       <c r="Z193" s="14"/>
       <c r="AA193" s="14"/>
-      <c r="AB193" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC193" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD193" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE193" s="27"/>
+      <c r="AB193" s="14"/>
+      <c r="AC193" s="14"/>
+      <c r="AD193" s="14"/>
+      <c r="AE193" s="27" t="s">
+        <v>654</v>
+      </c>
       <c r="AF193" s="14"/>
       <c r="AG193" s="14"/>
-      <c r="AH193" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH193" s="14"/>
       <c r="AI193" s="14"/>
     </row>
     <row r="194" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="14" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
       <c r="B194" s="14" t="s">
         <v>613</v>
@@ -11620,13 +11634,15 @@
         <v>614</v>
       </c>
       <c r="D194" s="18" t="s">
-        <v>654</v>
+        <v>663</v>
       </c>
       <c r="E194" s="14"/>
       <c r="F194" s="14"/>
       <c r="G194" s="14"/>
       <c r="H194" s="14"/>
-      <c r="I194" s="14"/>
+      <c r="I194" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J194" s="14"/>
       <c r="K194" s="14"/>
       <c r="L194" s="31"/>
@@ -11645,16 +11661,12 @@
       <c r="Y194" s="14"/>
       <c r="Z194" s="14"/>
       <c r="AA194" s="14"/>
-      <c r="AB194" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC194" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD194" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE194" s="27"/>
+      <c r="AB194" s="14"/>
+      <c r="AC194" s="14"/>
+      <c r="AD194" s="14"/>
+      <c r="AE194" s="27" t="s">
+        <v>656</v>
+      </c>
       <c r="AF194" s="14"/>
       <c r="AG194" s="14"/>
       <c r="AH194" s="14" t="s">
@@ -13944,7 +13956,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T198"/>
+  <dimension ref="A1:T201"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -20215,16 +20227,16 @@
         <v>632</v>
       </c>
       <c r="B192" s="20" t="s">
-        <v>636</v>
+        <v>658</v>
       </c>
       <c r="C192" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D192" s="14" t="s">
-        <v>637</v>
+        <v>112</v>
       </c>
       <c r="E192" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F192" s="15"/>
       <c r="G192" s="15"/>
@@ -20255,7 +20267,7 @@
         <v>2</v>
       </c>
       <c r="D193" s="14" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="E193" s="15" t="s">
         <v>2</v>
@@ -20280,10 +20292,10 @@
     </row>
     <row r="194" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="15" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B194" s="20" t="s">
-        <v>620</v>
+        <v>664</v>
       </c>
       <c r="C194" s="15" t="s">
         <v>0</v>
@@ -20314,10 +20326,10 @@
     </row>
     <row r="195" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="15" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="B195" s="20" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="C195" s="15" t="s">
         <v>0</v>
@@ -20348,10 +20360,10 @@
     </row>
     <row r="196" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="15" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="B196" s="20" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="C196" s="15" t="s">
         <v>0</v>
@@ -20382,7 +20394,7 @@
     </row>
     <row r="197" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="15" t="s">
-        <v>649</v>
+        <v>645</v>
       </c>
       <c r="B197" s="20" t="s">
         <v>635</v>
@@ -20391,7 +20403,7 @@
         <v>2</v>
       </c>
       <c r="D197" s="14" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="E197" s="15" t="s">
         <v>2</v>
@@ -20416,7 +20428,7 @@
     </row>
     <row r="198" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="B198" s="20" t="s">
         <v>635</v>
@@ -20425,7 +20437,7 @@
         <v>2</v>
       </c>
       <c r="D198" s="14" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="E198" s="15" t="s">
         <v>2</v>
@@ -20447,6 +20459,108 @@
       <c r="R198" s="14"/>
       <c r="S198" s="14"/>
       <c r="T198" s="14"/>
+    </row>
+    <row r="199" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="15" t="s">
+        <v>649</v>
+      </c>
+      <c r="B199" s="20" t="s">
+        <v>650</v>
+      </c>
+      <c r="C199" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D199" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E199" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F199" s="15"/>
+      <c r="G199" s="15"/>
+      <c r="H199" s="15"/>
+      <c r="I199" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J199" s="14"/>
+      <c r="K199" s="14"/>
+      <c r="L199" s="14"/>
+      <c r="M199" s="14"/>
+      <c r="N199" s="14"/>
+      <c r="O199" s="14"/>
+      <c r="P199" s="14"/>
+      <c r="Q199" s="14"/>
+      <c r="R199" s="14"/>
+      <c r="S199" s="14"/>
+      <c r="T199" s="14"/>
+    </row>
+    <row r="200" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A200" s="15" t="s">
+        <v>651</v>
+      </c>
+      <c r="B200" s="20" t="s">
+        <v>665</v>
+      </c>
+      <c r="C200" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D200" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E200" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F200" s="15"/>
+      <c r="G200" s="15"/>
+      <c r="H200" s="15"/>
+      <c r="I200" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J200" s="14"/>
+      <c r="K200" s="14"/>
+      <c r="L200" s="14"/>
+      <c r="M200" s="14"/>
+      <c r="N200" s="14"/>
+      <c r="O200" s="14"/>
+      <c r="P200" s="14"/>
+      <c r="Q200" s="14"/>
+      <c r="R200" s="14"/>
+      <c r="S200" s="14"/>
+      <c r="T200" s="14"/>
+    </row>
+    <row r="201" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A201" s="15" t="s">
+        <v>652</v>
+      </c>
+      <c r="B201" s="20" t="s">
+        <v>666</v>
+      </c>
+      <c r="C201" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D201" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E201" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F201" s="15"/>
+      <c r="G201" s="15"/>
+      <c r="H201" s="15"/>
+      <c r="I201" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J201" s="14"/>
+      <c r="K201" s="14"/>
+      <c r="L201" s="14"/>
+      <c r="M201" s="14"/>
+      <c r="N201" s="14"/>
+      <c r="O201" s="14"/>
+      <c r="P201" s="14"/>
+      <c r="Q201" s="14"/>
+      <c r="R201" s="14"/>
+      <c r="S201" s="14"/>
+      <c r="T201" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
Commit after update TestData and minor changes in RFMenuPage and feature file
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF884550-870A-4B52-9E23-19B7EFDC3804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9A3E05D-A194-43F7-BFBC-742E5C96FF54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2004,9 +2004,6 @@
     <t xml:space="preserve">Dangerous </t>
   </si>
   <si>
-    <t>06P17-26</t>
-  </si>
-  <si>
     <t>Cooler</t>
   </si>
   <si>
@@ -2025,10 +2022,13 @@
     <t>03P84-25</t>
   </si>
   <si>
-    <t>016967-00</t>
-  </si>
-  <si>
-    <t>03P51-01</t>
+    <t>06F24-20</t>
+  </si>
+  <si>
+    <t>07P04-07</t>
+  </si>
+  <si>
+    <t>07P04-01</t>
   </si>
 </sst>
 </file>
@@ -11157,7 +11157,7 @@
       <c r="AC184" s="14"/>
       <c r="AD184" s="14"/>
       <c r="AE184" s="27" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="AF184" s="14"/>
       <c r="AG184" s="14"/>
@@ -11432,7 +11432,7 @@
         <v>614</v>
       </c>
       <c r="D190" s="18" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="E190" s="14"/>
       <c r="F190" s="14"/>
@@ -11463,7 +11463,7 @@
       <c r="AC190" s="14"/>
       <c r="AD190" s="14"/>
       <c r="AE190" s="27" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="AF190" s="14"/>
       <c r="AG190" s="14"/>
@@ -11534,7 +11534,7 @@
         <v>614</v>
       </c>
       <c r="D192" s="18" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="E192" s="14"/>
       <c r="F192" s="14"/>
@@ -11585,7 +11585,7 @@
         <v>614</v>
       </c>
       <c r="D193" s="18" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E193" s="14"/>
       <c r="F193" s="14"/>
@@ -11634,7 +11634,7 @@
         <v>614</v>
       </c>
       <c r="D194" s="18" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E194" s="14"/>
       <c r="F194" s="14"/>
@@ -11665,7 +11665,7 @@
       <c r="AC194" s="14"/>
       <c r="AD194" s="14"/>
       <c r="AE194" s="27" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="AF194" s="14"/>
       <c r="AG194" s="14"/>
@@ -20227,13 +20227,13 @@
         <v>632</v>
       </c>
       <c r="B192" s="20" t="s">
-        <v>658</v>
+        <v>666</v>
       </c>
       <c r="C192" s="15" t="s">
         <v>0</v>
       </c>
       <c r="D192" s="14" t="s">
-        <v>112</v>
+        <v>636</v>
       </c>
       <c r="E192" s="15" t="s">
         <v>0</v>
@@ -20295,7 +20295,7 @@
         <v>638</v>
       </c>
       <c r="B194" s="20" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="C194" s="15" t="s">
         <v>0</v>
@@ -20499,13 +20499,13 @@
         <v>651</v>
       </c>
       <c r="B200" s="20" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="C200" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D200" s="14" t="s">
-        <v>112</v>
+        <v>636</v>
       </c>
       <c r="E200" s="15" t="s">
         <v>2</v>
@@ -20533,7 +20533,7 @@
         <v>652</v>
       </c>
       <c r="B201" s="20" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="C201" s="15" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
commit the code after fix Kelli Scenario
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9A3E05D-A194-43F7-BFBC-742E5C96FF54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4AF3B12-0ED9-4807-B440-13CE48F2E0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2810" uniqueCount="667">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2817" uniqueCount="666">
   <si>
     <t>1</t>
   </si>
@@ -1887,9 +1887,6 @@
     <t>973</t>
   </si>
   <si>
-    <t>03P78-25</t>
-  </si>
-  <si>
     <t>03P76-25</t>
   </si>
   <si>
@@ -1905,9 +1902,6 @@
     <t>975</t>
   </si>
   <si>
-    <t>013407-01 01</t>
-  </si>
-  <si>
     <t>06F16-10</t>
   </si>
   <si>
@@ -2016,9 +2010,6 @@
     <t>982|983</t>
   </si>
   <si>
-    <t>976|976</t>
-  </si>
-  <si>
     <t>03P84-25</t>
   </si>
   <si>
@@ -2029,6 +2020,12 @@
   </si>
   <si>
     <t>07P04-01</t>
+  </si>
+  <si>
+    <t>987</t>
+  </si>
+  <si>
+    <t>976|987</t>
   </si>
 </sst>
 </file>
@@ -6910,7 +6907,9 @@
       <c r="AB94" s="14"/>
       <c r="AC94" s="14"/>
       <c r="AD94" s="14"/>
-      <c r="AE94" s="27"/>
+      <c r="AE94" s="27" t="s">
+        <v>656</v>
+      </c>
       <c r="AF94" s="14"/>
       <c r="AG94" s="14"/>
       <c r="AH94" s="14"/>
@@ -11157,7 +11156,7 @@
       <c r="AC184" s="14"/>
       <c r="AD184" s="14"/>
       <c r="AE184" s="27" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="AF184" s="14"/>
       <c r="AG184" s="14"/>
@@ -11168,7 +11167,7 @@
     </row>
     <row r="185" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A185" s="14" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B185" s="14" t="s">
         <v>613</v>
@@ -11177,7 +11176,7 @@
         <v>614</v>
       </c>
       <c r="D185" s="18" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="E185" s="14"/>
       <c r="F185" s="14"/>
@@ -11208,7 +11207,7 @@
       <c r="AC185" s="14"/>
       <c r="AD185" s="14"/>
       <c r="AE185" s="27" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="AF185" s="14"/>
       <c r="AG185" s="14"/>
@@ -11219,7 +11218,7 @@
     </row>
     <row r="186" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="14" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B186" s="14" t="s">
         <v>613</v>
@@ -11228,7 +11227,7 @@
         <v>614</v>
       </c>
       <c r="D186" s="18" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="E186" s="14"/>
       <c r="F186" s="14"/>
@@ -11259,7 +11258,7 @@
       <c r="AC186" s="14"/>
       <c r="AD186" s="14"/>
       <c r="AE186" s="27" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="AF186" s="14"/>
       <c r="AG186" s="14"/>
@@ -11270,7 +11269,7 @@
     </row>
     <row r="187" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="14" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B187" s="14" t="s">
         <v>613</v>
@@ -11279,7 +11278,7 @@
         <v>614</v>
       </c>
       <c r="D187" s="18" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="E187" s="14"/>
       <c r="F187" s="14"/>
@@ -11310,7 +11309,7 @@
       <c r="AC187" s="14"/>
       <c r="AD187" s="14"/>
       <c r="AE187" s="27" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="AF187" s="14"/>
       <c r="AG187" s="14"/>
@@ -11321,7 +11320,7 @@
     </row>
     <row r="188" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="14" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="B188" s="14" t="s">
         <v>613</v>
@@ -11330,7 +11329,7 @@
         <v>614</v>
       </c>
       <c r="D188" s="18" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="E188" s="14"/>
       <c r="F188" s="14"/>
@@ -11361,7 +11360,7 @@
       <c r="AC188" s="14"/>
       <c r="AD188" s="14"/>
       <c r="AE188" s="27" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="AF188" s="14"/>
       <c r="AG188" s="14"/>
@@ -11372,7 +11371,7 @@
     </row>
     <row r="189" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="14" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="B189" s="14" t="s">
         <v>613</v>
@@ -11381,7 +11380,7 @@
         <v>614</v>
       </c>
       <c r="D189" s="18" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="E189" s="14"/>
       <c r="F189" s="14"/>
@@ -11412,7 +11411,7 @@
       <c r="AC189" s="14"/>
       <c r="AD189" s="14"/>
       <c r="AE189" s="27" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="AF189" s="14"/>
       <c r="AG189" s="14"/>
@@ -11423,7 +11422,7 @@
     </row>
     <row r="190" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="14" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B190" s="14" t="s">
         <v>613</v>
@@ -11432,7 +11431,7 @@
         <v>614</v>
       </c>
       <c r="D190" s="18" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="E190" s="14"/>
       <c r="F190" s="14"/>
@@ -11463,7 +11462,7 @@
       <c r="AC190" s="14"/>
       <c r="AD190" s="14"/>
       <c r="AE190" s="27" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="AF190" s="14"/>
       <c r="AG190" s="14"/>
@@ -11474,7 +11473,7 @@
     </row>
     <row r="191" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="14" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="B191" s="14" t="s">
         <v>613</v>
@@ -11483,7 +11482,7 @@
         <v>614</v>
       </c>
       <c r="D191" s="18" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="E191" s="14"/>
       <c r="F191" s="14"/>
@@ -11514,7 +11513,7 @@
       <c r="AC191" s="14"/>
       <c r="AD191" s="14"/>
       <c r="AE191" s="27" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="AF191" s="14"/>
       <c r="AG191" s="14"/>
@@ -11525,7 +11524,7 @@
     </row>
     <row r="192" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="14" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="B192" s="14" t="s">
         <v>613</v>
@@ -11534,7 +11533,7 @@
         <v>614</v>
       </c>
       <c r="D192" s="18" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E192" s="14"/>
       <c r="F192" s="14"/>
@@ -11565,7 +11564,7 @@
       <c r="AC192" s="14"/>
       <c r="AD192" s="14"/>
       <c r="AE192" s="27" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="AF192" s="14"/>
       <c r="AG192" s="14"/>
@@ -11576,7 +11575,7 @@
     </row>
     <row r="193" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="14" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="B193" s="14" t="s">
         <v>613</v>
@@ -11585,7 +11584,7 @@
         <v>614</v>
       </c>
       <c r="D193" s="18" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="E193" s="14"/>
       <c r="F193" s="14"/>
@@ -11616,7 +11615,7 @@
       <c r="AC193" s="14"/>
       <c r="AD193" s="14"/>
       <c r="AE193" s="27" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="AF193" s="14"/>
       <c r="AG193" s="14"/>
@@ -11625,7 +11624,7 @@
     </row>
     <row r="194" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="14" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="B194" s="14" t="s">
         <v>613</v>
@@ -11634,7 +11633,7 @@
         <v>614</v>
       </c>
       <c r="D194" s="18" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="E194" s="14"/>
       <c r="F194" s="14"/>
@@ -11665,7 +11664,7 @@
       <c r="AC194" s="14"/>
       <c r="AD194" s="14"/>
       <c r="AE194" s="27" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="AF194" s="14"/>
       <c r="AG194" s="14"/>
@@ -13956,7 +13955,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T201"/>
+  <dimension ref="A1:T202"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -20059,7 +20058,7 @@
         <v>615</v>
       </c>
       <c r="B187" s="20" t="s">
-        <v>619</v>
+        <v>662</v>
       </c>
       <c r="C187" s="15" t="s">
         <v>0</v>
@@ -20091,7 +20090,7 @@
         <v>618</v>
       </c>
       <c r="B188" s="20" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="C188" s="15" t="s">
         <v>2</v>
@@ -20106,7 +20105,7 @@
       <c r="G188" s="15"/>
       <c r="H188" s="15"/>
       <c r="I188" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J188" s="14"/>
       <c r="K188" s="14"/>
@@ -20122,10 +20121,10 @@
     </row>
     <row r="189" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="15" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B189" s="20" t="s">
-        <v>625</v>
+        <v>662</v>
       </c>
       <c r="C189" s="15" t="s">
         <v>2</v>
@@ -20140,7 +20139,7 @@
       <c r="G189" s="15"/>
       <c r="H189" s="15"/>
       <c r="I189" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J189" s="14"/>
       <c r="K189" s="14"/>
@@ -20156,10 +20155,10 @@
     </row>
     <row r="190" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="15" t="s">
+        <v>623</v>
+      </c>
+      <c r="B190" s="20" t="s">
         <v>624</v>
-      </c>
-      <c r="B190" s="20" t="s">
-        <v>626</v>
       </c>
       <c r="C190" s="15" t="s">
         <v>0</v>
@@ -20174,7 +20173,7 @@
       <c r="G190" s="15"/>
       <c r="H190" s="15"/>
       <c r="I190" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J190" s="14"/>
       <c r="K190" s="14"/>
@@ -20190,10 +20189,10 @@
     </row>
     <row r="191" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="15" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="B191" s="20" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="C191" s="15" t="s">
         <v>2</v>
@@ -20208,7 +20207,7 @@
       <c r="G191" s="15"/>
       <c r="H191" s="15"/>
       <c r="I191" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J191" s="14"/>
       <c r="K191" s="14"/>
@@ -20224,16 +20223,16 @@
     </row>
     <row r="192" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="15" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="B192" s="20" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="C192" s="15" t="s">
         <v>0</v>
       </c>
       <c r="D192" s="14" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="E192" s="15" t="s">
         <v>0</v>
@@ -20242,7 +20241,7 @@
       <c r="G192" s="15"/>
       <c r="H192" s="15"/>
       <c r="I192" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J192" s="14"/>
       <c r="K192" s="14"/>
@@ -20258,16 +20257,16 @@
     </row>
     <row r="193" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="15" t="s">
+        <v>631</v>
+      </c>
+      <c r="B193" s="20" t="s">
         <v>633</v>
-      </c>
-      <c r="B193" s="20" t="s">
-        <v>635</v>
       </c>
       <c r="C193" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D193" s="14" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="E193" s="15" t="s">
         <v>2</v>
@@ -20276,7 +20275,7 @@
       <c r="G193" s="15"/>
       <c r="H193" s="15"/>
       <c r="I193" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J193" s="14"/>
       <c r="K193" s="14"/>
@@ -20292,10 +20291,10 @@
     </row>
     <row r="194" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="15" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="B194" s="20" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="C194" s="15" t="s">
         <v>0</v>
@@ -20310,7 +20309,7 @@
       <c r="G194" s="15"/>
       <c r="H194" s="15"/>
       <c r="I194" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J194" s="14"/>
       <c r="K194" s="14"/>
@@ -20326,10 +20325,10 @@
     </row>
     <row r="195" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="15" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B195" s="20" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C195" s="15" t="s">
         <v>0</v>
@@ -20344,7 +20343,7 @@
       <c r="G195" s="15"/>
       <c r="H195" s="15"/>
       <c r="I195" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J195" s="14"/>
       <c r="K195" s="14"/>
@@ -20360,10 +20359,10 @@
     </row>
     <row r="196" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="15" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="B196" s="20" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="C196" s="15" t="s">
         <v>0</v>
@@ -20378,7 +20377,7 @@
       <c r="G196" s="15"/>
       <c r="H196" s="15"/>
       <c r="I196" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J196" s="14"/>
       <c r="K196" s="14"/>
@@ -20394,16 +20393,16 @@
     </row>
     <row r="197" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="15" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B197" s="20" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="C197" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D197" s="14" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="E197" s="15" t="s">
         <v>2</v>
@@ -20412,7 +20411,7 @@
       <c r="G197" s="15"/>
       <c r="H197" s="15"/>
       <c r="I197" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J197" s="14"/>
       <c r="K197" s="14"/>
@@ -20428,16 +20427,16 @@
     </row>
     <row r="198" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="15" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="B198" s="20" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="C198" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D198" s="14" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="E198" s="15" t="s">
         <v>2</v>
@@ -20446,7 +20445,7 @@
       <c r="G198" s="15"/>
       <c r="H198" s="15"/>
       <c r="I198" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J198" s="14"/>
       <c r="K198" s="14"/>
@@ -20462,10 +20461,10 @@
     </row>
     <row r="199" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="15" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B199" s="20" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C199" s="15" t="s">
         <v>2</v>
@@ -20480,7 +20479,7 @@
       <c r="G199" s="15"/>
       <c r="H199" s="15"/>
       <c r="I199" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J199" s="14"/>
       <c r="K199" s="14"/>
@@ -20496,16 +20495,16 @@
     </row>
     <row r="200" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="15" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B200" s="20" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="C200" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D200" s="14" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="E200" s="15" t="s">
         <v>2</v>
@@ -20514,7 +20513,7 @@
       <c r="G200" s="15"/>
       <c r="H200" s="15"/>
       <c r="I200" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J200" s="14"/>
       <c r="K200" s="14"/>
@@ -20530,10 +20529,10 @@
     </row>
     <row r="201" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="15" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="B201" s="20" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C201" s="15" t="s">
         <v>2</v>
@@ -20548,7 +20547,7 @@
       <c r="G201" s="15"/>
       <c r="H201" s="15"/>
       <c r="I201" s="14" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="J201" s="14"/>
       <c r="K201" s="14"/>
@@ -20561,6 +20560,40 @@
       <c r="R201" s="14"/>
       <c r="S201" s="14"/>
       <c r="T201" s="14"/>
+    </row>
+    <row r="202" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A202" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B202" s="20" t="s">
+        <v>632</v>
+      </c>
+      <c r="C202" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D202" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E202" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F202" s="15"/>
+      <c r="G202" s="15"/>
+      <c r="H202" s="15"/>
+      <c r="I202" s="14" t="s">
+        <v>625</v>
+      </c>
+      <c r="J202" s="14"/>
+      <c r="K202" s="14"/>
+      <c r="L202" s="14"/>
+      <c r="M202" s="14"/>
+      <c r="N202" s="14"/>
+      <c r="O202" s="14"/>
+      <c r="P202" s="14"/>
+      <c r="Q202" s="14"/>
+      <c r="R202" s="14"/>
+      <c r="S202" s="14"/>
+      <c r="T202" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
commit after changes done in config file and AsnsPage
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4AF3B12-0ED9-4807-B440-13CE48F2E0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE446EE3-4E72-4C9F-BA0B-53E4238601B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1887,9 +1887,6 @@
     <t>973</t>
   </si>
   <si>
-    <t>03P76-25</t>
-  </si>
-  <si>
     <t>APC_IBScenario002</t>
   </si>
   <si>
@@ -2026,6 +2023,9 @@
   </si>
   <si>
     <t>976|987</t>
+  </si>
+  <si>
+    <t>03P88-25</t>
   </si>
 </sst>
 </file>
@@ -6908,7 +6908,7 @@
       <c r="AC94" s="14"/>
       <c r="AD94" s="14"/>
       <c r="AE94" s="27" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="AF94" s="14"/>
       <c r="AG94" s="14"/>
@@ -11156,7 +11156,7 @@
       <c r="AC184" s="14"/>
       <c r="AD184" s="14"/>
       <c r="AE184" s="27" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="AF184" s="14"/>
       <c r="AG184" s="14"/>
@@ -11167,7 +11167,7 @@
     </row>
     <row r="185" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A185" s="14" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B185" s="14" t="s">
         <v>613</v>
@@ -11176,7 +11176,7 @@
         <v>614</v>
       </c>
       <c r="D185" s="18" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="E185" s="14"/>
       <c r="F185" s="14"/>
@@ -11207,7 +11207,7 @@
       <c r="AC185" s="14"/>
       <c r="AD185" s="14"/>
       <c r="AE185" s="27" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="AF185" s="14"/>
       <c r="AG185" s="14"/>
@@ -11218,7 +11218,7 @@
     </row>
     <row r="186" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="14" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B186" s="14" t="s">
         <v>613</v>
@@ -11227,7 +11227,7 @@
         <v>614</v>
       </c>
       <c r="D186" s="18" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="E186" s="14"/>
       <c r="F186" s="14"/>
@@ -11258,7 +11258,7 @@
       <c r="AC186" s="14"/>
       <c r="AD186" s="14"/>
       <c r="AE186" s="27" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="AF186" s="14"/>
       <c r="AG186" s="14"/>
@@ -11269,7 +11269,7 @@
     </row>
     <row r="187" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="14" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B187" s="14" t="s">
         <v>613</v>
@@ -11278,7 +11278,7 @@
         <v>614</v>
       </c>
       <c r="D187" s="18" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="E187" s="14"/>
       <c r="F187" s="14"/>
@@ -11309,7 +11309,7 @@
       <c r="AC187" s="14"/>
       <c r="AD187" s="14"/>
       <c r="AE187" s="27" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="AF187" s="14"/>
       <c r="AG187" s="14"/>
@@ -11320,7 +11320,7 @@
     </row>
     <row r="188" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="14" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B188" s="14" t="s">
         <v>613</v>
@@ -11329,7 +11329,7 @@
         <v>614</v>
       </c>
       <c r="D188" s="18" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="E188" s="14"/>
       <c r="F188" s="14"/>
@@ -11360,7 +11360,7 @@
       <c r="AC188" s="14"/>
       <c r="AD188" s="14"/>
       <c r="AE188" s="27" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="AF188" s="14"/>
       <c r="AG188" s="14"/>
@@ -11371,7 +11371,7 @@
     </row>
     <row r="189" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="14" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B189" s="14" t="s">
         <v>613</v>
@@ -11380,7 +11380,7 @@
         <v>614</v>
       </c>
       <c r="D189" s="18" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="E189" s="14"/>
       <c r="F189" s="14"/>
@@ -11411,7 +11411,7 @@
       <c r="AC189" s="14"/>
       <c r="AD189" s="14"/>
       <c r="AE189" s="27" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="AF189" s="14"/>
       <c r="AG189" s="14"/>
@@ -11422,7 +11422,7 @@
     </row>
     <row r="190" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="14" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B190" s="14" t="s">
         <v>613</v>
@@ -11431,7 +11431,7 @@
         <v>614</v>
       </c>
       <c r="D190" s="18" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E190" s="14"/>
       <c r="F190" s="14"/>
@@ -11462,7 +11462,7 @@
       <c r="AC190" s="14"/>
       <c r="AD190" s="14"/>
       <c r="AE190" s="27" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="AF190" s="14"/>
       <c r="AG190" s="14"/>
@@ -11473,7 +11473,7 @@
     </row>
     <row r="191" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="14" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B191" s="14" t="s">
         <v>613</v>
@@ -11482,7 +11482,7 @@
         <v>614</v>
       </c>
       <c r="D191" s="18" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="E191" s="14"/>
       <c r="F191" s="14"/>
@@ -11513,7 +11513,7 @@
       <c r="AC191" s="14"/>
       <c r="AD191" s="14"/>
       <c r="AE191" s="27" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="AF191" s="14"/>
       <c r="AG191" s="14"/>
@@ -11524,7 +11524,7 @@
     </row>
     <row r="192" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="14" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B192" s="14" t="s">
         <v>613</v>
@@ -11533,7 +11533,7 @@
         <v>614</v>
       </c>
       <c r="D192" s="18" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E192" s="14"/>
       <c r="F192" s="14"/>
@@ -11564,7 +11564,7 @@
       <c r="AC192" s="14"/>
       <c r="AD192" s="14"/>
       <c r="AE192" s="27" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="AF192" s="14"/>
       <c r="AG192" s="14"/>
@@ -11575,7 +11575,7 @@
     </row>
     <row r="193" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="14" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B193" s="14" t="s">
         <v>613</v>
@@ -11584,7 +11584,7 @@
         <v>614</v>
       </c>
       <c r="D193" s="18" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E193" s="14"/>
       <c r="F193" s="14"/>
@@ -11615,7 +11615,7 @@
       <c r="AC193" s="14"/>
       <c r="AD193" s="14"/>
       <c r="AE193" s="27" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="AF193" s="14"/>
       <c r="AG193" s="14"/>
@@ -11624,7 +11624,7 @@
     </row>
     <row r="194" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="14" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B194" s="14" t="s">
         <v>613</v>
@@ -11633,7 +11633,7 @@
         <v>614</v>
       </c>
       <c r="D194" s="18" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="E194" s="14"/>
       <c r="F194" s="14"/>
@@ -11664,7 +11664,7 @@
       <c r="AC194" s="14"/>
       <c r="AD194" s="14"/>
       <c r="AE194" s="27" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="AF194" s="14"/>
       <c r="AG194" s="14"/>
@@ -20058,7 +20058,7 @@
         <v>615</v>
       </c>
       <c r="B187" s="20" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C187" s="15" t="s">
         <v>0</v>
@@ -20090,7 +20090,7 @@
         <v>618</v>
       </c>
       <c r="B188" s="20" t="s">
-        <v>619</v>
+        <v>665</v>
       </c>
       <c r="C188" s="15" t="s">
         <v>2</v>
@@ -20105,7 +20105,7 @@
       <c r="G188" s="15"/>
       <c r="H188" s="15"/>
       <c r="I188" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J188" s="14"/>
       <c r="K188" s="14"/>
@@ -20121,10 +20121,10 @@
     </row>
     <row r="189" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="15" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B189" s="20" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C189" s="15" t="s">
         <v>2</v>
@@ -20139,7 +20139,7 @@
       <c r="G189" s="15"/>
       <c r="H189" s="15"/>
       <c r="I189" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J189" s="14"/>
       <c r="K189" s="14"/>
@@ -20155,10 +20155,10 @@
     </row>
     <row r="190" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="15" t="s">
+        <v>622</v>
+      </c>
+      <c r="B190" s="20" t="s">
         <v>623</v>
-      </c>
-      <c r="B190" s="20" t="s">
-        <v>624</v>
       </c>
       <c r="C190" s="15" t="s">
         <v>0</v>
@@ -20173,7 +20173,7 @@
       <c r="G190" s="15"/>
       <c r="H190" s="15"/>
       <c r="I190" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J190" s="14"/>
       <c r="K190" s="14"/>
@@ -20189,10 +20189,10 @@
     </row>
     <row r="191" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="15" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B191" s="20" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C191" s="15" t="s">
         <v>2</v>
@@ -20207,7 +20207,7 @@
       <c r="G191" s="15"/>
       <c r="H191" s="15"/>
       <c r="I191" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J191" s="14"/>
       <c r="K191" s="14"/>
@@ -20223,16 +20223,16 @@
     </row>
     <row r="192" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="15" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B192" s="20" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="C192" s="15" t="s">
         <v>0</v>
       </c>
       <c r="D192" s="14" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="E192" s="15" t="s">
         <v>0</v>
@@ -20241,7 +20241,7 @@
       <c r="G192" s="15"/>
       <c r="H192" s="15"/>
       <c r="I192" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J192" s="14"/>
       <c r="K192" s="14"/>
@@ -20257,16 +20257,16 @@
     </row>
     <row r="193" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="15" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B193" s="20" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="C193" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D193" s="14" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="E193" s="15" t="s">
         <v>2</v>
@@ -20275,7 +20275,7 @@
       <c r="G193" s="15"/>
       <c r="H193" s="15"/>
       <c r="I193" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J193" s="14"/>
       <c r="K193" s="14"/>
@@ -20291,10 +20291,10 @@
     </row>
     <row r="194" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="15" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B194" s="20" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C194" s="15" t="s">
         <v>0</v>
@@ -20309,7 +20309,7 @@
       <c r="G194" s="15"/>
       <c r="H194" s="15"/>
       <c r="I194" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J194" s="14"/>
       <c r="K194" s="14"/>
@@ -20325,10 +20325,10 @@
     </row>
     <row r="195" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="15" t="s">
+        <v>637</v>
+      </c>
+      <c r="B195" s="20" t="s">
         <v>638</v>
-      </c>
-      <c r="B195" s="20" t="s">
-        <v>639</v>
       </c>
       <c r="C195" s="15" t="s">
         <v>0</v>
@@ -20343,7 +20343,7 @@
       <c r="G195" s="15"/>
       <c r="H195" s="15"/>
       <c r="I195" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J195" s="14"/>
       <c r="K195" s="14"/>
@@ -20359,10 +20359,10 @@
     </row>
     <row r="196" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B196" s="20" t="s">
         <v>640</v>
-      </c>
-      <c r="B196" s="20" t="s">
-        <v>641</v>
       </c>
       <c r="C196" s="15" t="s">
         <v>0</v>
@@ -20377,7 +20377,7 @@
       <c r="G196" s="15"/>
       <c r="H196" s="15"/>
       <c r="I196" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J196" s="14"/>
       <c r="K196" s="14"/>
@@ -20393,16 +20393,16 @@
     </row>
     <row r="197" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="15" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B197" s="20" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="C197" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D197" s="14" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="E197" s="15" t="s">
         <v>2</v>
@@ -20411,7 +20411,7 @@
       <c r="G197" s="15"/>
       <c r="H197" s="15"/>
       <c r="I197" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J197" s="14"/>
       <c r="K197" s="14"/>
@@ -20427,16 +20427,16 @@
     </row>
     <row r="198" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="15" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B198" s="20" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="C198" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D198" s="14" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="E198" s="15" t="s">
         <v>2</v>
@@ -20445,7 +20445,7 @@
       <c r="G198" s="15"/>
       <c r="H198" s="15"/>
       <c r="I198" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J198" s="14"/>
       <c r="K198" s="14"/>
@@ -20461,10 +20461,10 @@
     </row>
     <row r="199" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="B199" s="20" t="s">
         <v>647</v>
-      </c>
-      <c r="B199" s="20" t="s">
-        <v>648</v>
       </c>
       <c r="C199" s="15" t="s">
         <v>2</v>
@@ -20479,7 +20479,7 @@
       <c r="G199" s="15"/>
       <c r="H199" s="15"/>
       <c r="I199" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J199" s="14"/>
       <c r="K199" s="14"/>
@@ -20495,16 +20495,16 @@
     </row>
     <row r="200" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="15" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B200" s="20" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="C200" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D200" s="14" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="E200" s="15" t="s">
         <v>2</v>
@@ -20513,7 +20513,7 @@
       <c r="G200" s="15"/>
       <c r="H200" s="15"/>
       <c r="I200" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J200" s="14"/>
       <c r="K200" s="14"/>
@@ -20529,10 +20529,10 @@
     </row>
     <row r="201" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="15" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B201" s="20" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C201" s="15" t="s">
         <v>2</v>
@@ -20547,7 +20547,7 @@
       <c r="G201" s="15"/>
       <c r="H201" s="15"/>
       <c r="I201" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J201" s="14"/>
       <c r="K201" s="14"/>
@@ -20563,10 +20563,10 @@
     </row>
     <row r="202" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="15" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B202" s="20" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C202" s="15" t="s">
         <v>2</v>
@@ -20581,7 +20581,7 @@
       <c r="G202" s="15"/>
       <c r="H202" s="15"/>
       <c r="I202" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J202" s="14"/>
       <c r="K202" s="14"/>

</xml_diff>

<commit_message>
Commit the Excel file after update the Items for Scenario 6 and 10
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE446EE3-4E72-4C9F-BA0B-53E4238601B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F383B566-58BF-4DAB-8E23-10F374A0D7D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2817" uniqueCount="666">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2840" uniqueCount="670">
   <si>
     <t>1</t>
   </si>
@@ -1926,9 +1926,6 @@
     <t>06F21-26</t>
   </si>
   <si>
-    <t>07P02-06</t>
-  </si>
-  <si>
     <t>BX</t>
   </si>
   <si>
@@ -2026,6 +2023,21 @@
   </si>
   <si>
     <t>03P88-25</t>
+  </si>
+  <si>
+    <t>APC_OBScenario01</t>
+  </si>
+  <si>
+    <t>988</t>
+  </si>
+  <si>
+    <t>07P04-15</t>
+  </si>
+  <si>
+    <t>APC_OBScenario02</t>
+  </si>
+  <si>
+    <t>07P02-03</t>
   </si>
 </sst>
 </file>
@@ -2569,7 +2581,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI406"/>
+  <dimension ref="A1:AI409"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -6908,7 +6920,7 @@
       <c r="AC94" s="14"/>
       <c r="AD94" s="14"/>
       <c r="AE94" s="27" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="AF94" s="14"/>
       <c r="AG94" s="14"/>
@@ -11156,7 +11168,7 @@
       <c r="AC184" s="14"/>
       <c r="AD184" s="14"/>
       <c r="AE184" s="27" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="AF184" s="14"/>
       <c r="AG184" s="14"/>
@@ -11207,7 +11219,7 @@
       <c r="AC185" s="14"/>
       <c r="AD185" s="14"/>
       <c r="AE185" s="27" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="AF185" s="14"/>
       <c r="AG185" s="14"/>
@@ -11258,7 +11270,7 @@
       <c r="AC186" s="14"/>
       <c r="AD186" s="14"/>
       <c r="AE186" s="27" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="AF186" s="14"/>
       <c r="AG186" s="14"/>
@@ -11309,7 +11321,7 @@
       <c r="AC187" s="14"/>
       <c r="AD187" s="14"/>
       <c r="AE187" s="27" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="AF187" s="14"/>
       <c r="AG187" s="14"/>
@@ -11360,7 +11372,7 @@
       <c r="AC188" s="14"/>
       <c r="AD188" s="14"/>
       <c r="AE188" s="27" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="AF188" s="14"/>
       <c r="AG188" s="14"/>
@@ -11411,7 +11423,7 @@
       <c r="AC189" s="14"/>
       <c r="AD189" s="14"/>
       <c r="AE189" s="27" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="AF189" s="14"/>
       <c r="AG189" s="14"/>
@@ -11422,7 +11434,7 @@
     </row>
     <row r="190" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="14" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B190" s="14" t="s">
         <v>613</v>
@@ -11431,7 +11443,7 @@
         <v>614</v>
       </c>
       <c r="D190" s="18" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="E190" s="14"/>
       <c r="F190" s="14"/>
@@ -11462,7 +11474,7 @@
       <c r="AC190" s="14"/>
       <c r="AD190" s="14"/>
       <c r="AE190" s="27" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="AF190" s="14"/>
       <c r="AG190" s="14"/>
@@ -11473,7 +11485,7 @@
     </row>
     <row r="191" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="14" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B191" s="14" t="s">
         <v>613</v>
@@ -11482,7 +11494,7 @@
         <v>614</v>
       </c>
       <c r="D191" s="18" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="E191" s="14"/>
       <c r="F191" s="14"/>
@@ -11513,7 +11525,7 @@
       <c r="AC191" s="14"/>
       <c r="AD191" s="14"/>
       <c r="AE191" s="27" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="AF191" s="14"/>
       <c r="AG191" s="14"/>
@@ -11524,7 +11536,7 @@
     </row>
     <row r="192" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="14" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B192" s="14" t="s">
         <v>613</v>
@@ -11533,7 +11545,7 @@
         <v>614</v>
       </c>
       <c r="D192" s="18" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E192" s="14"/>
       <c r="F192" s="14"/>
@@ -11564,7 +11576,7 @@
       <c r="AC192" s="14"/>
       <c r="AD192" s="14"/>
       <c r="AE192" s="27" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="AF192" s="14"/>
       <c r="AG192" s="14"/>
@@ -11575,7 +11587,7 @@
     </row>
     <row r="193" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="14" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B193" s="14" t="s">
         <v>613</v>
@@ -11584,7 +11596,7 @@
         <v>614</v>
       </c>
       <c r="D193" s="18" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E193" s="14"/>
       <c r="F193" s="14"/>
@@ -11615,7 +11627,7 @@
       <c r="AC193" s="14"/>
       <c r="AD193" s="14"/>
       <c r="AE193" s="27" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="AF193" s="14"/>
       <c r="AG193" s="14"/>
@@ -11624,7 +11636,7 @@
     </row>
     <row r="194" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="14" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B194" s="14" t="s">
         <v>613</v>
@@ -11633,7 +11645,7 @@
         <v>614</v>
       </c>
       <c r="D194" s="18" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="E194" s="14"/>
       <c r="F194" s="14"/>
@@ -11664,7 +11676,7 @@
       <c r="AC194" s="14"/>
       <c r="AD194" s="14"/>
       <c r="AE194" s="27" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="AF194" s="14"/>
       <c r="AG194" s="14"/>
@@ -11677,7 +11689,7 @@
       <c r="A195" s="14"/>
       <c r="B195" s="14"/>
       <c r="C195" s="14"/>
-      <c r="D195" s="14"/>
+      <c r="D195" s="18"/>
       <c r="E195" s="14"/>
       <c r="F195" s="14"/>
       <c r="G195" s="14"/>
@@ -11685,8 +11697,8 @@
       <c r="I195" s="14"/>
       <c r="J195" s="14"/>
       <c r="K195" s="14"/>
-      <c r="L195" s="14"/>
-      <c r="M195" s="14"/>
+      <c r="L195" s="31"/>
+      <c r="M195" s="30"/>
       <c r="N195" s="14"/>
       <c r="O195" s="14"/>
       <c r="P195" s="14"/>
@@ -11712,29 +11724,25 @@
     </row>
     <row r="196" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="14" t="s">
-        <v>267</v>
+        <v>665</v>
       </c>
       <c r="B196" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C196" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D196" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D196" s="23" t="s">
+        <v>666</v>
+      </c>
       <c r="E196" s="14"/>
       <c r="F196" s="14"/>
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
       <c r="I196" s="14"/>
-      <c r="J196" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K196" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L196" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J196" s="14"/>
+      <c r="K196" s="14"/>
+      <c r="L196" s="14"/>
       <c r="M196" s="14"/>
       <c r="N196" s="14"/>
       <c r="O196" s="14"/>
@@ -11750,40 +11758,44 @@
       <c r="Y196" s="14"/>
       <c r="Z196" s="14"/>
       <c r="AA196" s="14"/>
-      <c r="AB196" s="14"/>
-      <c r="AC196" s="14"/>
-      <c r="AD196" s="14"/>
+      <c r="AB196" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC196" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD196" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE196" s="27"/>
       <c r="AF196" s="14"/>
       <c r="AG196" s="14"/>
-      <c r="AH196" s="14"/>
+      <c r="AH196" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI196" s="14"/>
     </row>
     <row r="197" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="14" t="s">
-        <v>268</v>
+        <v>668</v>
       </c>
       <c r="B197" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C197" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D197" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D197" s="23" t="s">
+        <v>666</v>
+      </c>
       <c r="E197" s="14"/>
       <c r="F197" s="14"/>
       <c r="G197" s="14"/>
       <c r="H197" s="14"/>
       <c r="I197" s="14"/>
-      <c r="J197" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K197" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L197" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="J197" s="14"/>
+      <c r="K197" s="14"/>
+      <c r="L197" s="14"/>
       <c r="M197" s="14"/>
       <c r="N197" s="14"/>
       <c r="O197" s="14"/>
@@ -11799,28 +11811,49 @@
       <c r="Y197" s="14"/>
       <c r="Z197" s="14"/>
       <c r="AA197" s="14"/>
-      <c r="AB197" s="14"/>
-      <c r="AC197" s="14"/>
-      <c r="AD197" s="14"/>
+      <c r="AB197" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC197" s="14" t="s">
+        <v>420</v>
+      </c>
+      <c r="AD197" s="14" t="s">
+        <v>421</v>
+      </c>
       <c r="AE197" s="27"/>
       <c r="AF197" s="14"/>
       <c r="AG197" s="14"/>
       <c r="AH197" s="14"/>
       <c r="AI197" s="14"/>
     </row>
-    <row r="198" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A198" s="14" t="s">
-        <v>359</v>
-      </c>
-      <c r="B198" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C198" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O198" s="15" t="s">
-        <v>362</v>
-      </c>
+    <row r="198" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="14"/>
+      <c r="B198" s="14"/>
+      <c r="C198" s="14"/>
+      <c r="D198" s="14"/>
+      <c r="E198" s="14"/>
+      <c r="F198" s="14"/>
+      <c r="G198" s="14"/>
+      <c r="H198" s="14"/>
+      <c r="I198" s="14"/>
+      <c r="J198" s="14"/>
+      <c r="K198" s="14"/>
+      <c r="L198" s="14"/>
+      <c r="M198" s="14"/>
+      <c r="N198" s="14"/>
+      <c r="O198" s="14"/>
+      <c r="P198" s="14"/>
+      <c r="Q198" s="14"/>
+      <c r="R198" s="14"/>
+      <c r="S198" s="14"/>
+      <c r="T198" s="14"/>
+      <c r="U198" s="14"/>
+      <c r="V198" s="14"/>
+      <c r="W198" s="14"/>
+      <c r="X198" s="14"/>
+      <c r="Y198" s="14"/>
+      <c r="Z198" s="14"/>
+      <c r="AA198" s="14"/>
       <c r="AB198" s="14"/>
       <c r="AC198" s="14"/>
       <c r="AD198" s="14"/>
@@ -11830,9 +11863,9 @@
       <c r="AH198" s="14"/>
       <c r="AI198" s="14"/>
     </row>
-    <row r="199" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="14" t="s">
-        <v>360</v>
+        <v>267</v>
       </c>
       <c r="B199" s="14" t="s">
         <v>174</v>
@@ -11840,9 +11873,36 @@
       <c r="C199" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O199" s="15" t="s">
-        <v>363</v>
-      </c>
+      <c r="D199" s="14"/>
+      <c r="E199" s="14"/>
+      <c r="F199" s="14"/>
+      <c r="G199" s="14"/>
+      <c r="H199" s="14"/>
+      <c r="I199" s="14"/>
+      <c r="J199" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K199" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L199" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M199" s="14"/>
+      <c r="N199" s="14"/>
+      <c r="O199" s="14"/>
+      <c r="P199" s="14"/>
+      <c r="Q199" s="14"/>
+      <c r="R199" s="14"/>
+      <c r="S199" s="14"/>
+      <c r="T199" s="14"/>
+      <c r="U199" s="14"/>
+      <c r="V199" s="14"/>
+      <c r="W199" s="14"/>
+      <c r="X199" s="14"/>
+      <c r="Y199" s="14"/>
+      <c r="Z199" s="14"/>
+      <c r="AA199" s="14"/>
       <c r="AB199" s="14"/>
       <c r="AC199" s="14"/>
       <c r="AD199" s="14"/>
@@ -11852,9 +11912,9 @@
       <c r="AH199" s="14"/>
       <c r="AI199" s="14"/>
     </row>
-    <row r="200" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="14" t="s">
-        <v>361</v>
+        <v>268</v>
       </c>
       <c r="B200" s="14" t="s">
         <v>174</v>
@@ -11862,9 +11922,36 @@
       <c r="C200" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O200" s="15" t="s">
-        <v>364</v>
-      </c>
+      <c r="D200" s="14"/>
+      <c r="E200" s="14"/>
+      <c r="F200" s="14"/>
+      <c r="G200" s="14"/>
+      <c r="H200" s="14"/>
+      <c r="I200" s="14"/>
+      <c r="J200" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K200" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L200" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M200" s="14"/>
+      <c r="N200" s="14"/>
+      <c r="O200" s="14"/>
+      <c r="P200" s="14"/>
+      <c r="Q200" s="14"/>
+      <c r="R200" s="14"/>
+      <c r="S200" s="14"/>
+      <c r="T200" s="14"/>
+      <c r="U200" s="14"/>
+      <c r="V200" s="14"/>
+      <c r="W200" s="14"/>
+      <c r="X200" s="14"/>
+      <c r="Y200" s="14"/>
+      <c r="Z200" s="14"/>
+      <c r="AA200" s="14"/>
       <c r="AB200" s="14"/>
       <c r="AC200" s="14"/>
       <c r="AD200" s="14"/>
@@ -11876,7 +11963,7 @@
     </row>
     <row r="201" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A201" s="14" t="s">
-        <v>370</v>
+        <v>359</v>
       </c>
       <c r="B201" s="14" t="s">
         <v>174</v>
@@ -11884,8 +11971,8 @@
       <c r="C201" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M201" s="14" t="s">
-        <v>371</v>
+      <c r="O201" s="15" t="s">
+        <v>362</v>
       </c>
       <c r="AB201" s="14"/>
       <c r="AC201" s="14"/>
@@ -11897,6 +11984,18 @@
       <c r="AI201" s="14"/>
     </row>
     <row r="202" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A202" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B202" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C202" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O202" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB202" s="14"/>
       <c r="AC202" s="14"/>
       <c r="AD202" s="14"/>
@@ -11907,6 +12006,18 @@
       <c r="AI202" s="14"/>
     </row>
     <row r="203" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A203" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B203" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C203" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O203" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB203" s="14"/>
       <c r="AC203" s="14"/>
       <c r="AD203" s="14"/>
@@ -11917,6 +12028,18 @@
       <c r="AI203" s="14"/>
     </row>
     <row r="204" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A204" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B204" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C204" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M204" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB204" s="14"/>
       <c r="AC204" s="14"/>
       <c r="AD204" s="14"/>
@@ -13880,7 +14003,7 @@
       <c r="AB400" s="14"/>
       <c r="AC400" s="14"/>
       <c r="AD400" s="14"/>
-      <c r="AE400" s="14"/>
+      <c r="AE400" s="27"/>
       <c r="AF400" s="14"/>
       <c r="AG400" s="14"/>
       <c r="AH400" s="14"/>
@@ -13890,7 +14013,7 @@
       <c r="AB401" s="14"/>
       <c r="AC401" s="14"/>
       <c r="AD401" s="14"/>
-      <c r="AE401" s="14"/>
+      <c r="AE401" s="27"/>
       <c r="AF401" s="14"/>
       <c r="AG401" s="14"/>
       <c r="AH401" s="14"/>
@@ -13900,7 +14023,7 @@
       <c r="AB402" s="14"/>
       <c r="AC402" s="14"/>
       <c r="AD402" s="14"/>
-      <c r="AE402" s="14"/>
+      <c r="AE402" s="27"/>
       <c r="AF402" s="14"/>
       <c r="AG402" s="14"/>
       <c r="AH402" s="14"/>
@@ -13946,6 +14069,36 @@
       <c r="AH406" s="14"/>
       <c r="AI406" s="14"/>
     </row>
+    <row r="407" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB407" s="14"/>
+      <c r="AC407" s="14"/>
+      <c r="AD407" s="14"/>
+      <c r="AE407" s="14"/>
+      <c r="AF407" s="14"/>
+      <c r="AG407" s="14"/>
+      <c r="AH407" s="14"/>
+      <c r="AI407" s="14"/>
+    </row>
+    <row r="408" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB408" s="14"/>
+      <c r="AC408" s="14"/>
+      <c r="AD408" s="14"/>
+      <c r="AE408" s="14"/>
+      <c r="AF408" s="14"/>
+      <c r="AG408" s="14"/>
+      <c r="AH408" s="14"/>
+      <c r="AI408" s="14"/>
+    </row>
+    <row r="409" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB409" s="14"/>
+      <c r="AC409" s="14"/>
+      <c r="AD409" s="14"/>
+      <c r="AE409" s="14"/>
+      <c r="AF409" s="14"/>
+      <c r="AG409" s="14"/>
+      <c r="AH409" s="14"/>
+      <c r="AI409" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13955,7 +14108,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T202"/>
+  <dimension ref="A1:T203"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -20058,7 +20211,7 @@
         <v>615</v>
       </c>
       <c r="B187" s="20" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="C187" s="15" t="s">
         <v>0</v>
@@ -20090,7 +20243,7 @@
         <v>618</v>
       </c>
       <c r="B188" s="20" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="C188" s="15" t="s">
         <v>2</v>
@@ -20124,7 +20277,7 @@
         <v>621</v>
       </c>
       <c r="B189" s="20" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="C189" s="15" t="s">
         <v>2</v>
@@ -20226,13 +20379,13 @@
         <v>629</v>
       </c>
       <c r="B192" s="20" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C192" s="15" t="s">
         <v>0</v>
       </c>
       <c r="D192" s="14" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="E192" s="15" t="s">
         <v>0</v>
@@ -20260,13 +20413,13 @@
         <v>630</v>
       </c>
       <c r="B193" s="20" t="s">
-        <v>632</v>
+        <v>669</v>
       </c>
       <c r="C193" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D193" s="14" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="E193" s="15" t="s">
         <v>2</v>
@@ -20291,10 +20444,10 @@
     </row>
     <row r="194" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="15" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B194" s="20" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="C194" s="15" t="s">
         <v>0</v>
@@ -20325,10 +20478,10 @@
     </row>
     <row r="195" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="15" t="s">
+        <v>636</v>
+      </c>
+      <c r="B195" s="20" t="s">
         <v>637</v>
-      </c>
-      <c r="B195" s="20" t="s">
-        <v>638</v>
       </c>
       <c r="C195" s="15" t="s">
         <v>0</v>
@@ -20359,10 +20512,10 @@
     </row>
     <row r="196" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="15" t="s">
+        <v>638</v>
+      </c>
+      <c r="B196" s="20" t="s">
         <v>639</v>
-      </c>
-      <c r="B196" s="20" t="s">
-        <v>640</v>
       </c>
       <c r="C196" s="15" t="s">
         <v>0</v>
@@ -20393,16 +20546,16 @@
     </row>
     <row r="197" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="15" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B197" s="20" t="s">
-        <v>632</v>
+        <v>669</v>
       </c>
       <c r="C197" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D197" s="14" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="E197" s="15" t="s">
         <v>2</v>
@@ -20427,16 +20580,16 @@
     </row>
     <row r="198" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="15" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B198" s="20" t="s">
-        <v>632</v>
+        <v>669</v>
       </c>
       <c r="C198" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D198" s="14" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="E198" s="15" t="s">
         <v>2</v>
@@ -20461,10 +20614,10 @@
     </row>
     <row r="199" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="15" t="s">
+        <v>645</v>
+      </c>
+      <c r="B199" s="20" t="s">
         <v>646</v>
-      </c>
-      <c r="B199" s="20" t="s">
-        <v>647</v>
       </c>
       <c r="C199" s="15" t="s">
         <v>2</v>
@@ -20495,16 +20648,16 @@
     </row>
     <row r="200" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="15" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B200" s="20" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C200" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D200" s="14" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="E200" s="15" t="s">
         <v>2</v>
@@ -20529,10 +20682,10 @@
     </row>
     <row r="201" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="15" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B201" s="20" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="C201" s="15" t="s">
         <v>2</v>
@@ -20563,7 +20716,7 @@
     </row>
     <row r="202" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="15" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B202" s="20" t="s">
         <v>631</v>
@@ -20594,6 +20747,44 @@
       <c r="R202" s="14"/>
       <c r="S202" s="14"/>
       <c r="T202" s="14"/>
+    </row>
+    <row r="203" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A203" s="16" t="s">
+        <v>666</v>
+      </c>
+      <c r="B203" s="20" t="s">
+        <v>667</v>
+      </c>
+      <c r="C203" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D203" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="E203" s="14"/>
+      <c r="F203" s="14"/>
+      <c r="G203" s="14"/>
+      <c r="H203" s="14"/>
+      <c r="I203" s="14"/>
+      <c r="J203" s="14"/>
+      <c r="K203" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L203" s="14"/>
+      <c r="M203" s="14"/>
+      <c r="N203" s="14"/>
+      <c r="O203" s="14"/>
+      <c r="P203" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q203" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R203" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S203" s="14"/>
+      <c r="T203" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
Commit after changes done for both Inbound and Outbound scenarios scripting
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F383B566-58BF-4DAB-8E23-10F374A0D7D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6136C690-7137-4219-8E51-3CB2C6FEABCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Commit the code for APC Outbound scenarios initial version
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6136C690-7137-4219-8E51-3CB2C6FEABCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BA20D21-9468-41ED-92BD-A416022119F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2840" uniqueCount="670">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2920" uniqueCount="685">
   <si>
     <t>1</t>
   </si>
@@ -2031,13 +2031,58 @@
     <t>988</t>
   </si>
   <si>
+    <t>APC_OBScenario02</t>
+  </si>
+  <si>
+    <t>07P02-03</t>
+  </si>
+  <si>
     <t>07P04-15</t>
   </si>
   <si>
-    <t>APC_OBScenario02</t>
-  </si>
-  <si>
-    <t>07P02-03</t>
+    <t>989</t>
+  </si>
+  <si>
+    <t>APC_OBScenario03</t>
+  </si>
+  <si>
+    <t>07P02-05</t>
+  </si>
+  <si>
+    <t>APC_OBScenario04</t>
+  </si>
+  <si>
+    <t>990</t>
+  </si>
+  <si>
+    <t>APC_OBScenario05</t>
+  </si>
+  <si>
+    <t>991</t>
+  </si>
+  <si>
+    <t>APC_OBScenario06</t>
+  </si>
+  <si>
+    <t>APC_OBScenario07</t>
+  </si>
+  <si>
+    <t>992</t>
+  </si>
+  <si>
+    <t>988|992</t>
+  </si>
+  <si>
+    <t>993</t>
+  </si>
+  <si>
+    <t>994</t>
+  </si>
+  <si>
+    <t>APC_OBScenario08</t>
+  </si>
+  <si>
+    <t>988|994</t>
   </si>
 </sst>
 </file>
@@ -2581,7 +2626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI409"/>
+  <dimension ref="A1:AI415"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -11777,7 +11822,7 @@
     </row>
     <row r="197" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="14" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B197" s="14" t="s">
         <v>613</v>
@@ -11827,10 +11872,18 @@
       <c r="AI197" s="14"/>
     </row>
     <row r="198" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A198" s="14"/>
-      <c r="B198" s="14"/>
-      <c r="C198" s="14"/>
-      <c r="D198" s="14"/>
+      <c r="A198" s="14" t="s">
+        <v>671</v>
+      </c>
+      <c r="B198" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C198" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D198" s="23" t="s">
+        <v>670</v>
+      </c>
       <c r="E198" s="14"/>
       <c r="F198" s="14"/>
       <c r="G198" s="14"/>
@@ -11854,40 +11907,44 @@
       <c r="Y198" s="14"/>
       <c r="Z198" s="14"/>
       <c r="AA198" s="14"/>
-      <c r="AB198" s="14"/>
-      <c r="AC198" s="14"/>
-      <c r="AD198" s="14"/>
+      <c r="AB198" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC198" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD198" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE198" s="27"/>
       <c r="AF198" s="14"/>
       <c r="AG198" s="14"/>
-      <c r="AH198" s="14"/>
+      <c r="AH198" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI198" s="14"/>
     </row>
     <row r="199" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="14" t="s">
-        <v>267</v>
+        <v>673</v>
       </c>
       <c r="B199" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C199" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D199" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D199" s="23" t="s">
+        <v>674</v>
+      </c>
       <c r="E199" s="14"/>
       <c r="F199" s="14"/>
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="14"/>
-      <c r="J199" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K199" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L199" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J199" s="14"/>
+      <c r="K199" s="14"/>
+      <c r="L199" s="14"/>
       <c r="M199" s="14"/>
       <c r="N199" s="14"/>
       <c r="O199" s="14"/>
@@ -11903,40 +11960,44 @@
       <c r="Y199" s="14"/>
       <c r="Z199" s="14"/>
       <c r="AA199" s="14"/>
-      <c r="AB199" s="14"/>
-      <c r="AC199" s="14"/>
-      <c r="AD199" s="14"/>
+      <c r="AB199" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC199" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD199" s="14" t="s">
+        <v>393</v>
+      </c>
       <c r="AE199" s="27"/>
       <c r="AF199" s="14"/>
       <c r="AG199" s="14"/>
-      <c r="AH199" s="14"/>
+      <c r="AH199" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI199" s="14"/>
     </row>
     <row r="200" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="14" t="s">
-        <v>268</v>
+        <v>675</v>
       </c>
       <c r="B200" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C200" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D200" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D200" s="23" t="s">
+        <v>676</v>
+      </c>
       <c r="E200" s="14"/>
       <c r="F200" s="14"/>
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
       <c r="I200" s="14"/>
-      <c r="J200" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K200" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L200" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="J200" s="14"/>
+      <c r="K200" s="14"/>
+      <c r="L200" s="14"/>
       <c r="M200" s="14"/>
       <c r="N200" s="14"/>
       <c r="O200" s="14"/>
@@ -11952,94 +12013,210 @@
       <c r="Y200" s="14"/>
       <c r="Z200" s="14"/>
       <c r="AA200" s="14"/>
-      <c r="AB200" s="14"/>
-      <c r="AC200" s="14"/>
-      <c r="AD200" s="14"/>
+      <c r="AB200" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC200" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD200" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE200" s="27"/>
       <c r="AF200" s="14"/>
       <c r="AG200" s="14"/>
-      <c r="AH200" s="14"/>
+      <c r="AH200" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI200" s="14"/>
     </row>
-    <row r="201" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="14" t="s">
-        <v>359</v>
+        <v>677</v>
       </c>
       <c r="B201" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C201" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O201" s="15" t="s">
-        <v>362</v>
-      </c>
-      <c r="AB201" s="14"/>
-      <c r="AC201" s="14"/>
-      <c r="AD201" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D201" s="23" t="s">
+        <v>676</v>
+      </c>
+      <c r="E201" s="14"/>
+      <c r="F201" s="14"/>
+      <c r="G201" s="14"/>
+      <c r="H201" s="14"/>
+      <c r="I201" s="14"/>
+      <c r="J201" s="14"/>
+      <c r="K201" s="14"/>
+      <c r="L201" s="14"/>
+      <c r="M201" s="14"/>
+      <c r="N201" s="14"/>
+      <c r="O201" s="14"/>
+      <c r="P201" s="14"/>
+      <c r="Q201" s="14"/>
+      <c r="R201" s="14"/>
+      <c r="S201" s="14"/>
+      <c r="T201" s="14"/>
+      <c r="U201" s="14"/>
+      <c r="V201" s="14"/>
+      <c r="W201" s="14"/>
+      <c r="X201" s="14"/>
+      <c r="Y201" s="14"/>
+      <c r="Z201" s="14"/>
+      <c r="AA201" s="14"/>
+      <c r="AB201" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC201" s="14" t="s">
+        <v>420</v>
+      </c>
+      <c r="AD201" s="14" t="s">
+        <v>421</v>
+      </c>
       <c r="AE201" s="27"/>
       <c r="AF201" s="14"/>
       <c r="AG201" s="14"/>
-      <c r="AH201" s="14"/>
+      <c r="AH201" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI201" s="14"/>
     </row>
-    <row r="202" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="14" t="s">
-        <v>360</v>
+        <v>678</v>
       </c>
       <c r="B202" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C202" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O202" s="15" t="s">
-        <v>363</v>
-      </c>
-      <c r="AB202" s="14"/>
-      <c r="AC202" s="14"/>
-      <c r="AD202" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D202" s="18" t="s">
+        <v>680</v>
+      </c>
+      <c r="E202" s="14"/>
+      <c r="F202" s="14"/>
+      <c r="G202" s="14"/>
+      <c r="H202" s="14"/>
+      <c r="I202" s="14"/>
+      <c r="J202" s="14"/>
+      <c r="K202" s="14"/>
+      <c r="L202" s="14"/>
+      <c r="M202" s="14"/>
+      <c r="N202" s="14"/>
+      <c r="O202" s="14"/>
+      <c r="P202" s="14"/>
+      <c r="Q202" s="14"/>
+      <c r="R202" s="14"/>
+      <c r="S202" s="14"/>
+      <c r="T202" s="14"/>
+      <c r="U202" s="14"/>
+      <c r="V202" s="14"/>
+      <c r="W202" s="14"/>
+      <c r="X202" s="14"/>
+      <c r="Y202" s="14"/>
+      <c r="Z202" s="14"/>
+      <c r="AA202" s="14"/>
+      <c r="AB202" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC202" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD202" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE202" s="27"/>
       <c r="AF202" s="14"/>
       <c r="AG202" s="14"/>
-      <c r="AH202" s="14"/>
+      <c r="AH202" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI202" s="14"/>
     </row>
-    <row r="203" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="14" t="s">
-        <v>361</v>
+        <v>683</v>
       </c>
       <c r="B203" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C203" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O203" s="15" t="s">
-        <v>364</v>
-      </c>
-      <c r="AB203" s="14"/>
-      <c r="AC203" s="14"/>
-      <c r="AD203" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D203" s="18" t="s">
+        <v>684</v>
+      </c>
+      <c r="E203" s="14"/>
+      <c r="F203" s="14"/>
+      <c r="G203" s="14"/>
+      <c r="H203" s="14"/>
+      <c r="I203" s="14"/>
+      <c r="J203" s="14"/>
+      <c r="K203" s="14"/>
+      <c r="L203" s="14"/>
+      <c r="M203" s="14"/>
+      <c r="N203" s="14"/>
+      <c r="O203" s="14"/>
+      <c r="P203" s="14"/>
+      <c r="Q203" s="14"/>
+      <c r="R203" s="14"/>
+      <c r="S203" s="14"/>
+      <c r="T203" s="14"/>
+      <c r="U203" s="14"/>
+      <c r="V203" s="14"/>
+      <c r="W203" s="14"/>
+      <c r="X203" s="14"/>
+      <c r="Y203" s="14"/>
+      <c r="Z203" s="14"/>
+      <c r="AA203" s="14"/>
+      <c r="AB203" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC203" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD203" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE203" s="27"/>
       <c r="AF203" s="14"/>
       <c r="AG203" s="14"/>
-      <c r="AH203" s="14"/>
+      <c r="AH203" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI203" s="14"/>
     </row>
-    <row r="204" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A204" s="14" t="s">
-        <v>370</v>
-      </c>
-      <c r="B204" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C204" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="M204" s="14" t="s">
-        <v>371</v>
-      </c>
+    <row r="204" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A204" s="14"/>
+      <c r="B204" s="14"/>
+      <c r="C204" s="14"/>
+      <c r="D204" s="14"/>
+      <c r="E204" s="14"/>
+      <c r="F204" s="14"/>
+      <c r="G204" s="14"/>
+      <c r="H204" s="14"/>
+      <c r="I204" s="14"/>
+      <c r="J204" s="14"/>
+      <c r="K204" s="14"/>
+      <c r="L204" s="14"/>
+      <c r="M204" s="14"/>
+      <c r="N204" s="14"/>
+      <c r="O204" s="14"/>
+      <c r="P204" s="14"/>
+      <c r="Q204" s="14"/>
+      <c r="R204" s="14"/>
+      <c r="S204" s="14"/>
+      <c r="T204" s="14"/>
+      <c r="U204" s="14"/>
+      <c r="V204" s="14"/>
+      <c r="W204" s="14"/>
+      <c r="X204" s="14"/>
+      <c r="Y204" s="14"/>
+      <c r="Z204" s="14"/>
+      <c r="AA204" s="14"/>
       <c r="AB204" s="14"/>
       <c r="AC204" s="14"/>
       <c r="AD204" s="14"/>
@@ -12049,7 +12226,46 @@
       <c r="AH204" s="14"/>
       <c r="AI204" s="14"/>
     </row>
-    <row r="205" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A205" s="14" t="s">
+        <v>267</v>
+      </c>
+      <c r="B205" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C205" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D205" s="14"/>
+      <c r="E205" s="14"/>
+      <c r="F205" s="14"/>
+      <c r="G205" s="14"/>
+      <c r="H205" s="14"/>
+      <c r="I205" s="14"/>
+      <c r="J205" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K205" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L205" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M205" s="14"/>
+      <c r="N205" s="14"/>
+      <c r="O205" s="14"/>
+      <c r="P205" s="14"/>
+      <c r="Q205" s="14"/>
+      <c r="R205" s="14"/>
+      <c r="S205" s="14"/>
+      <c r="T205" s="14"/>
+      <c r="U205" s="14"/>
+      <c r="V205" s="14"/>
+      <c r="W205" s="14"/>
+      <c r="X205" s="14"/>
+      <c r="Y205" s="14"/>
+      <c r="Z205" s="14"/>
+      <c r="AA205" s="14"/>
       <c r="AB205" s="14"/>
       <c r="AC205" s="14"/>
       <c r="AD205" s="14"/>
@@ -12059,7 +12275,46 @@
       <c r="AH205" s="14"/>
       <c r="AI205" s="14"/>
     </row>
-    <row r="206" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A206" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="B206" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C206" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D206" s="14"/>
+      <c r="E206" s="14"/>
+      <c r="F206" s="14"/>
+      <c r="G206" s="14"/>
+      <c r="H206" s="14"/>
+      <c r="I206" s="14"/>
+      <c r="J206" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K206" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L206" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M206" s="14"/>
+      <c r="N206" s="14"/>
+      <c r="O206" s="14"/>
+      <c r="P206" s="14"/>
+      <c r="Q206" s="14"/>
+      <c r="R206" s="14"/>
+      <c r="S206" s="14"/>
+      <c r="T206" s="14"/>
+      <c r="U206" s="14"/>
+      <c r="V206" s="14"/>
+      <c r="W206" s="14"/>
+      <c r="X206" s="14"/>
+      <c r="Y206" s="14"/>
+      <c r="Z206" s="14"/>
+      <c r="AA206" s="14"/>
       <c r="AB206" s="14"/>
       <c r="AC206" s="14"/>
       <c r="AD206" s="14"/>
@@ -12070,6 +12325,18 @@
       <c r="AI206" s="14"/>
     </row>
     <row r="207" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A207" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="B207" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C207" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O207" s="15" t="s">
+        <v>362</v>
+      </c>
       <c r="AB207" s="14"/>
       <c r="AC207" s="14"/>
       <c r="AD207" s="14"/>
@@ -12080,6 +12347,18 @@
       <c r="AI207" s="14"/>
     </row>
     <row r="208" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A208" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B208" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C208" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O208" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB208" s="14"/>
       <c r="AC208" s="14"/>
       <c r="AD208" s="14"/>
@@ -12089,7 +12368,19 @@
       <c r="AH208" s="14"/>
       <c r="AI208" s="14"/>
     </row>
-    <row r="209" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A209" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B209" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C209" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O209" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB209" s="14"/>
       <c r="AC209" s="14"/>
       <c r="AD209" s="14"/>
@@ -12099,7 +12390,19 @@
       <c r="AH209" s="14"/>
       <c r="AI209" s="14"/>
     </row>
-    <row r="210" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A210" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B210" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C210" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M210" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB210" s="14"/>
       <c r="AC210" s="14"/>
       <c r="AD210" s="14"/>
@@ -12109,7 +12412,7 @@
       <c r="AH210" s="14"/>
       <c r="AI210" s="14"/>
     </row>
-    <row r="211" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB211" s="14"/>
       <c r="AC211" s="14"/>
       <c r="AD211" s="14"/>
@@ -12119,7 +12422,7 @@
       <c r="AH211" s="14"/>
       <c r="AI211" s="14"/>
     </row>
-    <row r="212" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB212" s="14"/>
       <c r="AC212" s="14"/>
       <c r="AD212" s="14"/>
@@ -12129,7 +12432,7 @@
       <c r="AH212" s="14"/>
       <c r="AI212" s="14"/>
     </row>
-    <row r="213" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB213" s="14"/>
       <c r="AC213" s="14"/>
       <c r="AD213" s="14"/>
@@ -12139,7 +12442,7 @@
       <c r="AH213" s="14"/>
       <c r="AI213" s="14"/>
     </row>
-    <row r="214" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB214" s="14"/>
       <c r="AC214" s="14"/>
       <c r="AD214" s="14"/>
@@ -12149,7 +12452,7 @@
       <c r="AH214" s="14"/>
       <c r="AI214" s="14"/>
     </row>
-    <row r="215" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB215" s="14"/>
       <c r="AC215" s="14"/>
       <c r="AD215" s="14"/>
@@ -12159,7 +12462,7 @@
       <c r="AH215" s="14"/>
       <c r="AI215" s="14"/>
     </row>
-    <row r="216" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB216" s="14"/>
       <c r="AC216" s="14"/>
       <c r="AD216" s="14"/>
@@ -12169,7 +12472,7 @@
       <c r="AH216" s="14"/>
       <c r="AI216" s="14"/>
     </row>
-    <row r="217" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB217" s="14"/>
       <c r="AC217" s="14"/>
       <c r="AD217" s="14"/>
@@ -12179,7 +12482,7 @@
       <c r="AH217" s="14"/>
       <c r="AI217" s="14"/>
     </row>
-    <row r="218" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB218" s="14"/>
       <c r="AC218" s="14"/>
       <c r="AD218" s="14"/>
@@ -12189,7 +12492,7 @@
       <c r="AH218" s="14"/>
       <c r="AI218" s="14"/>
     </row>
-    <row r="219" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB219" s="14"/>
       <c r="AC219" s="14"/>
       <c r="AD219" s="14"/>
@@ -12199,7 +12502,7 @@
       <c r="AH219" s="14"/>
       <c r="AI219" s="14"/>
     </row>
-    <row r="220" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB220" s="14"/>
       <c r="AC220" s="14"/>
       <c r="AD220" s="14"/>
@@ -12209,7 +12512,7 @@
       <c r="AH220" s="14"/>
       <c r="AI220" s="14"/>
     </row>
-    <row r="221" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB221" s="14"/>
       <c r="AC221" s="14"/>
       <c r="AD221" s="14"/>
@@ -12219,7 +12522,7 @@
       <c r="AH221" s="14"/>
       <c r="AI221" s="14"/>
     </row>
-    <row r="222" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB222" s="14"/>
       <c r="AC222" s="14"/>
       <c r="AD222" s="14"/>
@@ -12229,7 +12532,7 @@
       <c r="AH222" s="14"/>
       <c r="AI222" s="14"/>
     </row>
-    <row r="223" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB223" s="14"/>
       <c r="AC223" s="14"/>
       <c r="AD223" s="14"/>
@@ -12239,7 +12542,7 @@
       <c r="AH223" s="14"/>
       <c r="AI223" s="14"/>
     </row>
-    <row r="224" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB224" s="14"/>
       <c r="AC224" s="14"/>
       <c r="AD224" s="14"/>
@@ -14033,7 +14336,7 @@
       <c r="AB403" s="14"/>
       <c r="AC403" s="14"/>
       <c r="AD403" s="14"/>
-      <c r="AE403" s="14"/>
+      <c r="AE403" s="27"/>
       <c r="AF403" s="14"/>
       <c r="AG403" s="14"/>
       <c r="AH403" s="14"/>
@@ -14043,7 +14346,7 @@
       <c r="AB404" s="14"/>
       <c r="AC404" s="14"/>
       <c r="AD404" s="14"/>
-      <c r="AE404" s="14"/>
+      <c r="AE404" s="27"/>
       <c r="AF404" s="14"/>
       <c r="AG404" s="14"/>
       <c r="AH404" s="14"/>
@@ -14053,7 +14356,7 @@
       <c r="AB405" s="14"/>
       <c r="AC405" s="14"/>
       <c r="AD405" s="14"/>
-      <c r="AE405" s="14"/>
+      <c r="AE405" s="27"/>
       <c r="AF405" s="14"/>
       <c r="AG405" s="14"/>
       <c r="AH405" s="14"/>
@@ -14063,7 +14366,7 @@
       <c r="AB406" s="14"/>
       <c r="AC406" s="14"/>
       <c r="AD406" s="14"/>
-      <c r="AE406" s="14"/>
+      <c r="AE406" s="27"/>
       <c r="AF406" s="14"/>
       <c r="AG406" s="14"/>
       <c r="AH406" s="14"/>
@@ -14073,7 +14376,7 @@
       <c r="AB407" s="14"/>
       <c r="AC407" s="14"/>
       <c r="AD407" s="14"/>
-      <c r="AE407" s="14"/>
+      <c r="AE407" s="27"/>
       <c r="AF407" s="14"/>
       <c r="AG407" s="14"/>
       <c r="AH407" s="14"/>
@@ -14083,7 +14386,7 @@
       <c r="AB408" s="14"/>
       <c r="AC408" s="14"/>
       <c r="AD408" s="14"/>
-      <c r="AE408" s="14"/>
+      <c r="AE408" s="27"/>
       <c r="AF408" s="14"/>
       <c r="AG408" s="14"/>
       <c r="AH408" s="14"/>
@@ -14099,6 +14402,66 @@
       <c r="AH409" s="14"/>
       <c r="AI409" s="14"/>
     </row>
+    <row r="410" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB410" s="14"/>
+      <c r="AC410" s="14"/>
+      <c r="AD410" s="14"/>
+      <c r="AE410" s="14"/>
+      <c r="AF410" s="14"/>
+      <c r="AG410" s="14"/>
+      <c r="AH410" s="14"/>
+      <c r="AI410" s="14"/>
+    </row>
+    <row r="411" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB411" s="14"/>
+      <c r="AC411" s="14"/>
+      <c r="AD411" s="14"/>
+      <c r="AE411" s="14"/>
+      <c r="AF411" s="14"/>
+      <c r="AG411" s="14"/>
+      <c r="AH411" s="14"/>
+      <c r="AI411" s="14"/>
+    </row>
+    <row r="412" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB412" s="14"/>
+      <c r="AC412" s="14"/>
+      <c r="AD412" s="14"/>
+      <c r="AE412" s="14"/>
+      <c r="AF412" s="14"/>
+      <c r="AG412" s="14"/>
+      <c r="AH412" s="14"/>
+      <c r="AI412" s="14"/>
+    </row>
+    <row r="413" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB413" s="14"/>
+      <c r="AC413" s="14"/>
+      <c r="AD413" s="14"/>
+      <c r="AE413" s="14"/>
+      <c r="AF413" s="14"/>
+      <c r="AG413" s="14"/>
+      <c r="AH413" s="14"/>
+      <c r="AI413" s="14"/>
+    </row>
+    <row r="414" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB414" s="14"/>
+      <c r="AC414" s="14"/>
+      <c r="AD414" s="14"/>
+      <c r="AE414" s="14"/>
+      <c r="AF414" s="14"/>
+      <c r="AG414" s="14"/>
+      <c r="AH414" s="14"/>
+      <c r="AI414" s="14"/>
+    </row>
+    <row r="415" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB415" s="14"/>
+      <c r="AC415" s="14"/>
+      <c r="AD415" s="14"/>
+      <c r="AE415" s="14"/>
+      <c r="AF415" s="14"/>
+      <c r="AG415" s="14"/>
+      <c r="AH415" s="14"/>
+      <c r="AI415" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14108,7 +14471,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T203"/>
+  <dimension ref="A1:T209"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -20314,13 +20677,13 @@
         <v>623</v>
       </c>
       <c r="C190" s="15" t="s">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="D190" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E190" s="15" t="s">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="F190" s="15"/>
       <c r="G190" s="15"/>
@@ -20413,7 +20776,7 @@
         <v>630</v>
       </c>
       <c r="B193" s="20" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="C193" s="15" t="s">
         <v>2</v>
@@ -20549,7 +20912,7 @@
         <v>641</v>
       </c>
       <c r="B197" s="20" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="C197" s="15" t="s">
         <v>2</v>
@@ -20583,7 +20946,7 @@
         <v>642</v>
       </c>
       <c r="B198" s="20" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="C198" s="15" t="s">
         <v>2</v>
@@ -20753,7 +21116,7 @@
         <v>666</v>
       </c>
       <c r="B203" s="20" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="C203" s="15" t="s">
         <v>2</v>
@@ -20785,6 +21148,202 @@
       </c>
       <c r="S203" s="14"/>
       <c r="T203" s="14"/>
+    </row>
+    <row r="204" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A204" s="15" t="s">
+        <v>670</v>
+      </c>
+      <c r="B204" s="20" t="s">
+        <v>672</v>
+      </c>
+      <c r="C204" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D204" s="14" t="s">
+        <v>632</v>
+      </c>
+      <c r="E204" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F204" s="15"/>
+      <c r="G204" s="15"/>
+      <c r="H204" s="15"/>
+      <c r="I204" s="14"/>
+      <c r="J204" s="14"/>
+      <c r="K204" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L204" s="14"/>
+      <c r="M204" s="14"/>
+      <c r="N204" s="14"/>
+      <c r="O204" s="14"/>
+      <c r="P204" s="14"/>
+      <c r="Q204" s="14"/>
+      <c r="R204" s="14"/>
+      <c r="S204" s="14"/>
+      <c r="T204" s="14"/>
+    </row>
+    <row r="205" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A205" s="15" t="s">
+        <v>674</v>
+      </c>
+      <c r="B205" s="20" t="s">
+        <v>672</v>
+      </c>
+      <c r="C205" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D205" s="14" t="s">
+        <v>632</v>
+      </c>
+      <c r="E205" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F205" s="15"/>
+      <c r="G205" s="15"/>
+      <c r="H205" s="15"/>
+      <c r="I205" s="14"/>
+      <c r="J205" s="14"/>
+      <c r="K205" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L205" s="14"/>
+      <c r="M205" s="14"/>
+      <c r="N205" s="14"/>
+      <c r="O205" s="14"/>
+      <c r="P205" s="14"/>
+      <c r="Q205" s="14"/>
+      <c r="R205" s="14"/>
+      <c r="S205" s="14"/>
+      <c r="T205" s="14"/>
+    </row>
+    <row r="206" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A206" s="15" t="s">
+        <v>676</v>
+      </c>
+      <c r="B206" s="20" t="s">
+        <v>637</v>
+      </c>
+      <c r="C206" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D206" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E206" s="15"/>
+      <c r="F206" s="15"/>
+      <c r="G206" s="15"/>
+      <c r="H206" s="15"/>
+      <c r="I206" s="14"/>
+      <c r="J206" s="14"/>
+      <c r="K206" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L206" s="14"/>
+      <c r="M206" s="14"/>
+      <c r="N206" s="14"/>
+      <c r="O206" s="14"/>
+      <c r="P206" s="14"/>
+      <c r="Q206" s="14"/>
+      <c r="R206" s="14"/>
+      <c r="S206" s="14"/>
+      <c r="T206" s="14"/>
+    </row>
+    <row r="207" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A207" s="15" t="s">
+        <v>679</v>
+      </c>
+      <c r="B207" s="20" t="s">
+        <v>669</v>
+      </c>
+      <c r="C207" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D207" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E207" s="15"/>
+      <c r="F207" s="15"/>
+      <c r="G207" s="15"/>
+      <c r="H207" s="15"/>
+      <c r="I207" s="14"/>
+      <c r="J207" s="14"/>
+      <c r="K207" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L207" s="14"/>
+      <c r="M207" s="14"/>
+      <c r="N207" s="14"/>
+      <c r="O207" s="14"/>
+      <c r="P207" s="14"/>
+      <c r="Q207" s="14"/>
+      <c r="R207" s="14"/>
+      <c r="S207" s="14"/>
+      <c r="T207" s="14"/>
+    </row>
+    <row r="208" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A208" s="15" t="s">
+        <v>681</v>
+      </c>
+      <c r="B208" s="20" t="s">
+        <v>659</v>
+      </c>
+      <c r="C208" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D208" s="14" t="s">
+        <v>632</v>
+      </c>
+      <c r="E208" s="15"/>
+      <c r="F208" s="15"/>
+      <c r="G208" s="15"/>
+      <c r="H208" s="15"/>
+      <c r="I208" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J208" s="14"/>
+      <c r="K208" s="14"/>
+      <c r="L208" s="14"/>
+      <c r="M208" s="14"/>
+      <c r="N208" s="14"/>
+      <c r="O208" s="14"/>
+      <c r="P208" s="14"/>
+      <c r="Q208" s="14"/>
+      <c r="R208" s="14"/>
+      <c r="S208" s="14"/>
+      <c r="T208" s="14"/>
+    </row>
+    <row r="209" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A209" s="15" t="s">
+        <v>682</v>
+      </c>
+      <c r="B209" s="20" t="s">
+        <v>660</v>
+      </c>
+      <c r="C209" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D209" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E209" s="15"/>
+      <c r="F209" s="15"/>
+      <c r="G209" s="15"/>
+      <c r="H209" s="15"/>
+      <c r="I209" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J209" s="14"/>
+      <c r="K209" s="14"/>
+      <c r="L209" s="14"/>
+      <c r="M209" s="14"/>
+      <c r="N209" s="14"/>
+      <c r="O209" s="14"/>
+      <c r="P209" s="14"/>
+      <c r="Q209" s="14"/>
+      <c r="R209" s="14"/>
+      <c r="S209" s="14"/>
+      <c r="T209" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
commit latest changes for testdata
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BA20D21-9468-41ED-92BD-A416022119F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E08D088-EA38-433F-89C6-9A37330B04DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2920" uniqueCount="685">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2973" uniqueCount="695">
   <si>
     <t>1</t>
   </si>
@@ -2022,9 +2022,6 @@
     <t>976|987</t>
   </si>
   <si>
-    <t>03P88-25</t>
-  </si>
-  <si>
     <t>APC_OBScenario01</t>
   </si>
   <si>
@@ -2046,43 +2043,76 @@
     <t>APC_OBScenario03</t>
   </si>
   <si>
+    <t>APC_OBScenario04</t>
+  </si>
+  <si>
+    <t>990</t>
+  </si>
+  <si>
+    <t>APC_OBScenario05</t>
+  </si>
+  <si>
+    <t>991</t>
+  </si>
+  <si>
+    <t>APC_OBScenario06</t>
+  </si>
+  <si>
+    <t>APC_OBScenario07</t>
+  </si>
+  <si>
+    <t>992</t>
+  </si>
+  <si>
+    <t>988|992</t>
+  </si>
+  <si>
+    <t>993</t>
+  </si>
+  <si>
+    <t>994</t>
+  </si>
+  <si>
+    <t>APC_OBScenario08</t>
+  </si>
+  <si>
+    <t>988|994</t>
+  </si>
+  <si>
+    <t>APC_OBScenario09</t>
+  </si>
+  <si>
+    <t>995</t>
+  </si>
+  <si>
+    <t>996</t>
+  </si>
+  <si>
+    <t>APC_OBScenario10</t>
+  </si>
+  <si>
+    <t>995|996</t>
+  </si>
+  <si>
+    <t>APC_OBScenario11</t>
+  </si>
+  <si>
+    <t>997</t>
+  </si>
+  <si>
+    <t>APC_OBScenario12</t>
+  </si>
+  <si>
+    <t>03P85-25</t>
+  </si>
+  <si>
+    <t>07P05-01</t>
+  </si>
+  <si>
+    <t>APC_OBScenario13</t>
+  </si>
+  <si>
     <t>07P02-05</t>
-  </si>
-  <si>
-    <t>APC_OBScenario04</t>
-  </si>
-  <si>
-    <t>990</t>
-  </si>
-  <si>
-    <t>APC_OBScenario05</t>
-  </si>
-  <si>
-    <t>991</t>
-  </si>
-  <si>
-    <t>APC_OBScenario06</t>
-  </si>
-  <si>
-    <t>APC_OBScenario07</t>
-  </si>
-  <si>
-    <t>992</t>
-  </si>
-  <si>
-    <t>988|992</t>
-  </si>
-  <si>
-    <t>993</t>
-  </si>
-  <si>
-    <t>994</t>
-  </si>
-  <si>
-    <t>APC_OBScenario08</t>
-  </si>
-  <si>
-    <t>988|994</t>
   </si>
 </sst>
 </file>
@@ -2626,7 +2656,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI415"/>
+  <dimension ref="A1:AI420"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -11769,7 +11799,7 @@
     </row>
     <row r="196" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="14" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B196" s="14" t="s">
         <v>613</v>
@@ -11778,7 +11808,7 @@
         <v>614</v>
       </c>
       <c r="D196" s="23" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="E196" s="14"/>
       <c r="F196" s="14"/>
@@ -11822,7 +11852,7 @@
     </row>
     <row r="197" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="14" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B197" s="14" t="s">
         <v>613</v>
@@ -11831,7 +11861,7 @@
         <v>614</v>
       </c>
       <c r="D197" s="23" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="E197" s="14"/>
       <c r="F197" s="14"/>
@@ -11873,7 +11903,7 @@
     </row>
     <row r="198" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="14" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B198" s="14" t="s">
         <v>613</v>
@@ -11882,7 +11912,7 @@
         <v>614</v>
       </c>
       <c r="D198" s="23" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="E198" s="14"/>
       <c r="F198" s="14"/>
@@ -11926,7 +11956,7 @@
     </row>
     <row r="199" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="14" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B199" s="14" t="s">
         <v>613</v>
@@ -11935,7 +11965,7 @@
         <v>614</v>
       </c>
       <c r="D199" s="23" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="E199" s="14"/>
       <c r="F199" s="14"/>
@@ -11964,10 +11994,10 @@
         <v>393</v>
       </c>
       <c r="AC199" s="14" t="s">
-        <v>393</v>
+        <v>420</v>
       </c>
       <c r="AD199" s="14" t="s">
-        <v>393</v>
+        <v>421</v>
       </c>
       <c r="AE199" s="27"/>
       <c r="AF199" s="14"/>
@@ -11979,7 +12009,7 @@
     </row>
     <row r="200" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="14" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="B200" s="14" t="s">
         <v>613</v>
@@ -11988,7 +12018,7 @@
         <v>614</v>
       </c>
       <c r="D200" s="23" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="E200" s="14"/>
       <c r="F200" s="14"/>
@@ -12032,7 +12062,7 @@
     </row>
     <row r="201" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="14" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="B201" s="14" t="s">
         <v>613</v>
@@ -12041,7 +12071,7 @@
         <v>614</v>
       </c>
       <c r="D201" s="23" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="E201" s="14"/>
       <c r="F201" s="14"/>
@@ -12085,7 +12115,7 @@
     </row>
     <row r="202" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="14" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="B202" s="14" t="s">
         <v>613</v>
@@ -12094,7 +12124,7 @@
         <v>614</v>
       </c>
       <c r="D202" s="18" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="E202" s="14"/>
       <c r="F202" s="14"/>
@@ -12138,7 +12168,7 @@
     </row>
     <row r="203" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="14" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="B203" s="14" t="s">
         <v>613</v>
@@ -12147,7 +12177,7 @@
         <v>614</v>
       </c>
       <c r="D203" s="18" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="E203" s="14"/>
       <c r="F203" s="14"/>
@@ -12190,10 +12220,18 @@
       <c r="AI203" s="14"/>
     </row>
     <row r="204" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A204" s="14"/>
-      <c r="B204" s="14"/>
-      <c r="C204" s="14"/>
-      <c r="D204" s="14"/>
+      <c r="A204" s="14" t="s">
+        <v>683</v>
+      </c>
+      <c r="B204" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C204" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D204" s="18" t="s">
+        <v>682</v>
+      </c>
       <c r="E204" s="14"/>
       <c r="F204" s="14"/>
       <c r="G204" s="14"/>
@@ -12217,40 +12255,44 @@
       <c r="Y204" s="14"/>
       <c r="Z204" s="14"/>
       <c r="AA204" s="14"/>
-      <c r="AB204" s="14"/>
-      <c r="AC204" s="14"/>
-      <c r="AD204" s="14"/>
+      <c r="AB204" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC204" s="14" t="s">
+        <v>420</v>
+      </c>
+      <c r="AD204" s="14" t="s">
+        <v>421</v>
+      </c>
       <c r="AE204" s="27"/>
       <c r="AF204" s="14"/>
       <c r="AG204" s="14"/>
-      <c r="AH204" s="14"/>
+      <c r="AH204" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI204" s="14"/>
     </row>
     <row r="205" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="14" t="s">
-        <v>267</v>
+        <v>686</v>
       </c>
       <c r="B205" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C205" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D205" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D205" s="18" t="s">
+        <v>687</v>
+      </c>
       <c r="E205" s="14"/>
       <c r="F205" s="14"/>
       <c r="G205" s="14"/>
       <c r="H205" s="14"/>
       <c r="I205" s="14"/>
-      <c r="J205" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K205" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L205" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J205" s="14"/>
+      <c r="K205" s="14"/>
+      <c r="L205" s="14"/>
       <c r="M205" s="14"/>
       <c r="N205" s="14"/>
       <c r="O205" s="14"/>
@@ -12266,40 +12308,44 @@
       <c r="Y205" s="14"/>
       <c r="Z205" s="14"/>
       <c r="AA205" s="14"/>
-      <c r="AB205" s="14"/>
-      <c r="AC205" s="14"/>
-      <c r="AD205" s="14"/>
+      <c r="AB205" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC205" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD205" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE205" s="27"/>
       <c r="AF205" s="14"/>
       <c r="AG205" s="14"/>
-      <c r="AH205" s="14"/>
+      <c r="AH205" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI205" s="14"/>
     </row>
     <row r="206" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="14" t="s">
-        <v>268</v>
+        <v>688</v>
       </c>
       <c r="B206" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C206" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D206" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D206" s="18" t="s">
+        <v>687</v>
+      </c>
       <c r="E206" s="14"/>
       <c r="F206" s="14"/>
       <c r="G206" s="14"/>
       <c r="H206" s="14"/>
       <c r="I206" s="14"/>
-      <c r="J206" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K206" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L206" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="J206" s="14"/>
+      <c r="K206" s="14"/>
+      <c r="L206" s="14"/>
       <c r="M206" s="14"/>
       <c r="N206" s="14"/>
       <c r="O206" s="14"/>
@@ -12315,72 +12361,157 @@
       <c r="Y206" s="14"/>
       <c r="Z206" s="14"/>
       <c r="AA206" s="14"/>
-      <c r="AB206" s="14"/>
-      <c r="AC206" s="14"/>
-      <c r="AD206" s="14"/>
+      <c r="AB206" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC206" s="14" t="s">
+        <v>420</v>
+      </c>
+      <c r="AD206" s="14" t="s">
+        <v>421</v>
+      </c>
       <c r="AE206" s="27"/>
       <c r="AF206" s="14"/>
       <c r="AG206" s="14"/>
-      <c r="AH206" s="14"/>
+      <c r="AH206" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI206" s="14"/>
     </row>
-    <row r="207" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="14" t="s">
-        <v>359</v>
+        <v>690</v>
       </c>
       <c r="B207" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C207" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O207" s="15" t="s">
-        <v>362</v>
-      </c>
-      <c r="AB207" s="14"/>
-      <c r="AC207" s="14"/>
-      <c r="AD207" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D207" s="23" t="s">
+        <v>689</v>
+      </c>
+      <c r="E207" s="14"/>
+      <c r="F207" s="14"/>
+      <c r="G207" s="14"/>
+      <c r="H207" s="14"/>
+      <c r="I207" s="14"/>
+      <c r="J207" s="14"/>
+      <c r="K207" s="14"/>
+      <c r="L207" s="14"/>
+      <c r="M207" s="14"/>
+      <c r="N207" s="14"/>
+      <c r="O207" s="14"/>
+      <c r="P207" s="14"/>
+      <c r="Q207" s="14"/>
+      <c r="R207" s="14"/>
+      <c r="S207" s="14"/>
+      <c r="T207" s="14"/>
+      <c r="U207" s="14"/>
+      <c r="V207" s="14"/>
+      <c r="W207" s="14"/>
+      <c r="X207" s="14"/>
+      <c r="Y207" s="14"/>
+      <c r="Z207" s="14"/>
+      <c r="AA207" s="14"/>
+      <c r="AB207" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC207" s="14" t="s">
+        <v>420</v>
+      </c>
+      <c r="AD207" s="14" t="s">
+        <v>421</v>
+      </c>
       <c r="AE207" s="27"/>
       <c r="AF207" s="14"/>
       <c r="AG207" s="14"/>
-      <c r="AH207" s="14"/>
+      <c r="AH207" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI207" s="14"/>
     </row>
-    <row r="208" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="14" t="s">
-        <v>360</v>
+        <v>693</v>
       </c>
       <c r="B208" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C208" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O208" s="15" t="s">
-        <v>363</v>
-      </c>
-      <c r="AB208" s="14"/>
-      <c r="AC208" s="14"/>
-      <c r="AD208" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D208" s="23" t="s">
+        <v>689</v>
+      </c>
+      <c r="E208" s="14"/>
+      <c r="F208" s="14"/>
+      <c r="G208" s="14"/>
+      <c r="H208" s="14"/>
+      <c r="I208" s="14"/>
+      <c r="J208" s="14"/>
+      <c r="K208" s="14"/>
+      <c r="L208" s="14"/>
+      <c r="M208" s="14"/>
+      <c r="N208" s="14"/>
+      <c r="O208" s="14"/>
+      <c r="P208" s="14"/>
+      <c r="Q208" s="14"/>
+      <c r="R208" s="14"/>
+      <c r="S208" s="14"/>
+      <c r="T208" s="14"/>
+      <c r="U208" s="14"/>
+      <c r="V208" s="14"/>
+      <c r="W208" s="14"/>
+      <c r="X208" s="14"/>
+      <c r="Y208" s="14"/>
+      <c r="Z208" s="14"/>
+      <c r="AA208" s="14"/>
+      <c r="AB208" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC208" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD208" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE208" s="27"/>
       <c r="AF208" s="14"/>
       <c r="AG208" s="14"/>
-      <c r="AH208" s="14"/>
+      <c r="AH208" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI208" s="14"/>
     </row>
-    <row r="209" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A209" s="14" t="s">
-        <v>361</v>
-      </c>
-      <c r="B209" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C209" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O209" s="15" t="s">
-        <v>364</v>
-      </c>
+    <row r="209" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A209" s="14"/>
+      <c r="B209" s="14"/>
+      <c r="C209" s="14"/>
+      <c r="D209" s="14"/>
+      <c r="E209" s="14"/>
+      <c r="F209" s="14"/>
+      <c r="G209" s="14"/>
+      <c r="H209" s="14"/>
+      <c r="I209" s="14"/>
+      <c r="J209" s="14"/>
+      <c r="K209" s="14"/>
+      <c r="L209" s="14"/>
+      <c r="M209" s="14"/>
+      <c r="N209" s="14"/>
+      <c r="O209" s="14"/>
+      <c r="P209" s="14"/>
+      <c r="Q209" s="14"/>
+      <c r="R209" s="14"/>
+      <c r="S209" s="14"/>
+      <c r="T209" s="14"/>
+      <c r="U209" s="14"/>
+      <c r="V209" s="14"/>
+      <c r="W209" s="14"/>
+      <c r="X209" s="14"/>
+      <c r="Y209" s="14"/>
+      <c r="Z209" s="14"/>
+      <c r="AA209" s="14"/>
       <c r="AB209" s="14"/>
       <c r="AC209" s="14"/>
       <c r="AD209" s="14"/>
@@ -12390,9 +12521,9 @@
       <c r="AH209" s="14"/>
       <c r="AI209" s="14"/>
     </row>
-    <row r="210" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210" s="14" t="s">
-        <v>370</v>
+        <v>267</v>
       </c>
       <c r="B210" s="14" t="s">
         <v>174</v>
@@ -12400,9 +12531,36 @@
       <c r="C210" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M210" s="14" t="s">
-        <v>371</v>
-      </c>
+      <c r="D210" s="14"/>
+      <c r="E210" s="14"/>
+      <c r="F210" s="14"/>
+      <c r="G210" s="14"/>
+      <c r="H210" s="14"/>
+      <c r="I210" s="14"/>
+      <c r="J210" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K210" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L210" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M210" s="14"/>
+      <c r="N210" s="14"/>
+      <c r="O210" s="14"/>
+      <c r="P210" s="14"/>
+      <c r="Q210" s="14"/>
+      <c r="R210" s="14"/>
+      <c r="S210" s="14"/>
+      <c r="T210" s="14"/>
+      <c r="U210" s="14"/>
+      <c r="V210" s="14"/>
+      <c r="W210" s="14"/>
+      <c r="X210" s="14"/>
+      <c r="Y210" s="14"/>
+      <c r="Z210" s="14"/>
+      <c r="AA210" s="14"/>
       <c r="AB210" s="14"/>
       <c r="AC210" s="14"/>
       <c r="AD210" s="14"/>
@@ -12412,7 +12570,46 @@
       <c r="AH210" s="14"/>
       <c r="AI210" s="14"/>
     </row>
-    <row r="211" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A211" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="B211" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C211" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D211" s="14"/>
+      <c r="E211" s="14"/>
+      <c r="F211" s="14"/>
+      <c r="G211" s="14"/>
+      <c r="H211" s="14"/>
+      <c r="I211" s="14"/>
+      <c r="J211" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K211" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L211" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M211" s="14"/>
+      <c r="N211" s="14"/>
+      <c r="O211" s="14"/>
+      <c r="P211" s="14"/>
+      <c r="Q211" s="14"/>
+      <c r="R211" s="14"/>
+      <c r="S211" s="14"/>
+      <c r="T211" s="14"/>
+      <c r="U211" s="14"/>
+      <c r="V211" s="14"/>
+      <c r="W211" s="14"/>
+      <c r="X211" s="14"/>
+      <c r="Y211" s="14"/>
+      <c r="Z211" s="14"/>
+      <c r="AA211" s="14"/>
       <c r="AB211" s="14"/>
       <c r="AC211" s="14"/>
       <c r="AD211" s="14"/>
@@ -12423,6 +12620,18 @@
       <c r="AI211" s="14"/>
     </row>
     <row r="212" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A212" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="B212" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C212" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O212" s="15" t="s">
+        <v>362</v>
+      </c>
       <c r="AB212" s="14"/>
       <c r="AC212" s="14"/>
       <c r="AD212" s="14"/>
@@ -12433,6 +12642,18 @@
       <c r="AI212" s="14"/>
     </row>
     <row r="213" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A213" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B213" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C213" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O213" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB213" s="14"/>
       <c r="AC213" s="14"/>
       <c r="AD213" s="14"/>
@@ -12443,6 +12664,18 @@
       <c r="AI213" s="14"/>
     </row>
     <row r="214" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A214" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B214" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C214" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O214" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB214" s="14"/>
       <c r="AC214" s="14"/>
       <c r="AD214" s="14"/>
@@ -12453,6 +12686,18 @@
       <c r="AI214" s="14"/>
     </row>
     <row r="215" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A215" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B215" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C215" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M215" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB215" s="14"/>
       <c r="AC215" s="14"/>
       <c r="AD215" s="14"/>
@@ -14396,7 +14641,7 @@
       <c r="AB409" s="14"/>
       <c r="AC409" s="14"/>
       <c r="AD409" s="14"/>
-      <c r="AE409" s="14"/>
+      <c r="AE409" s="27"/>
       <c r="AF409" s="14"/>
       <c r="AG409" s="14"/>
       <c r="AH409" s="14"/>
@@ -14406,7 +14651,7 @@
       <c r="AB410" s="14"/>
       <c r="AC410" s="14"/>
       <c r="AD410" s="14"/>
-      <c r="AE410" s="14"/>
+      <c r="AE410" s="27"/>
       <c r="AF410" s="14"/>
       <c r="AG410" s="14"/>
       <c r="AH410" s="14"/>
@@ -14416,7 +14661,7 @@
       <c r="AB411" s="14"/>
       <c r="AC411" s="14"/>
       <c r="AD411" s="14"/>
-      <c r="AE411" s="14"/>
+      <c r="AE411" s="27"/>
       <c r="AF411" s="14"/>
       <c r="AG411" s="14"/>
       <c r="AH411" s="14"/>
@@ -14426,7 +14671,7 @@
       <c r="AB412" s="14"/>
       <c r="AC412" s="14"/>
       <c r="AD412" s="14"/>
-      <c r="AE412" s="14"/>
+      <c r="AE412" s="27"/>
       <c r="AF412" s="14"/>
       <c r="AG412" s="14"/>
       <c r="AH412" s="14"/>
@@ -14436,7 +14681,7 @@
       <c r="AB413" s="14"/>
       <c r="AC413" s="14"/>
       <c r="AD413" s="14"/>
-      <c r="AE413" s="14"/>
+      <c r="AE413" s="27"/>
       <c r="AF413" s="14"/>
       <c r="AG413" s="14"/>
       <c r="AH413" s="14"/>
@@ -14462,6 +14707,56 @@
       <c r="AH415" s="14"/>
       <c r="AI415" s="14"/>
     </row>
+    <row r="416" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB416" s="14"/>
+      <c r="AC416" s="14"/>
+      <c r="AD416" s="14"/>
+      <c r="AE416" s="14"/>
+      <c r="AF416" s="14"/>
+      <c r="AG416" s="14"/>
+      <c r="AH416" s="14"/>
+      <c r="AI416" s="14"/>
+    </row>
+    <row r="417" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB417" s="14"/>
+      <c r="AC417" s="14"/>
+      <c r="AD417" s="14"/>
+      <c r="AE417" s="14"/>
+      <c r="AF417" s="14"/>
+      <c r="AG417" s="14"/>
+      <c r="AH417" s="14"/>
+      <c r="AI417" s="14"/>
+    </row>
+    <row r="418" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB418" s="14"/>
+      <c r="AC418" s="14"/>
+      <c r="AD418" s="14"/>
+      <c r="AE418" s="14"/>
+      <c r="AF418" s="14"/>
+      <c r="AG418" s="14"/>
+      <c r="AH418" s="14"/>
+      <c r="AI418" s="14"/>
+    </row>
+    <row r="419" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB419" s="14"/>
+      <c r="AC419" s="14"/>
+      <c r="AD419" s="14"/>
+      <c r="AE419" s="14"/>
+      <c r="AF419" s="14"/>
+      <c r="AG419" s="14"/>
+      <c r="AH419" s="14"/>
+      <c r="AI419" s="14"/>
+    </row>
+    <row r="420" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB420" s="14"/>
+      <c r="AC420" s="14"/>
+      <c r="AD420" s="14"/>
+      <c r="AE420" s="14"/>
+      <c r="AF420" s="14"/>
+      <c r="AG420" s="14"/>
+      <c r="AH420" s="14"/>
+      <c r="AI420" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14471,7 +14766,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T209"/>
+  <dimension ref="A1:T212"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -20539,7 +20834,7 @@
         <v>612</v>
       </c>
       <c r="C186" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D186" s="16" t="s">
         <v>112</v>
@@ -20606,16 +20901,16 @@
         <v>618</v>
       </c>
       <c r="B188" s="20" t="s">
-        <v>664</v>
+        <v>658</v>
       </c>
       <c r="C188" s="15" t="s">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="D188" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E188" s="15" t="s">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="F188" s="15"/>
       <c r="G188" s="15"/>
@@ -20677,13 +20972,13 @@
         <v>623</v>
       </c>
       <c r="C190" s="15" t="s">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="D190" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E190" s="15" t="s">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="F190" s="15"/>
       <c r="G190" s="15"/>
@@ -20776,7 +21071,7 @@
         <v>630</v>
       </c>
       <c r="B193" s="20" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="C193" s="15" t="s">
         <v>2</v>
@@ -20810,7 +21105,7 @@
         <v>634</v>
       </c>
       <c r="B194" s="20" t="s">
-        <v>658</v>
+        <v>691</v>
       </c>
       <c r="C194" s="15" t="s">
         <v>0</v>
@@ -20912,7 +21207,7 @@
         <v>641</v>
       </c>
       <c r="B197" s="20" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="C197" s="15" t="s">
         <v>2</v>
@@ -20946,7 +21241,7 @@
         <v>642</v>
       </c>
       <c r="B198" s="20" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="C198" s="15" t="s">
         <v>2</v>
@@ -21113,10 +21408,10 @@
     </row>
     <row r="203" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="16" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B203" s="20" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="C203" s="15" t="s">
         <v>2</v>
@@ -21151,20 +21446,18 @@
     </row>
     <row r="204" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A204" s="15" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B204" s="20" t="s">
-        <v>672</v>
+        <v>694</v>
       </c>
       <c r="C204" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="D204" s="14" t="s">
-        <v>632</v>
-      </c>
-      <c r="E204" s="15" t="s">
-        <v>2</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D204" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="E204" s="15"/>
       <c r="F204" s="15"/>
       <c r="G204" s="15"/>
       <c r="H204" s="15"/>
@@ -21185,20 +21478,18 @@
     </row>
     <row r="205" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="15" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="B205" s="20" t="s">
-        <v>672</v>
+        <v>694</v>
       </c>
       <c r="C205" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D205" s="14" t="s">
-        <v>632</v>
-      </c>
-      <c r="E205" s="15" t="s">
-        <v>2</v>
-      </c>
+      <c r="D205" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="E205" s="15"/>
       <c r="F205" s="15"/>
       <c r="G205" s="15"/>
       <c r="H205" s="15"/>
@@ -21219,7 +21510,7 @@
     </row>
     <row r="206" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="15" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="B206" s="20" t="s">
         <v>637</v>
@@ -21251,10 +21542,10 @@
     </row>
     <row r="207" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="15" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="B207" s="20" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="C207" s="15" t="s">
         <v>2</v>
@@ -21283,7 +21574,7 @@
     </row>
     <row r="208" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="15" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="B208" s="20" t="s">
         <v>659</v>
@@ -21315,7 +21606,7 @@
     </row>
     <row r="209" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="15" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="B209" s="20" t="s">
         <v>660</v>
@@ -21344,6 +21635,102 @@
       <c r="R209" s="14"/>
       <c r="S209" s="14"/>
       <c r="T209" s="14"/>
+    </row>
+    <row r="210" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A210" s="15" t="s">
+        <v>684</v>
+      </c>
+      <c r="B210" s="20" t="s">
+        <v>692</v>
+      </c>
+      <c r="C210" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D210" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E210" s="15"/>
+      <c r="F210" s="15"/>
+      <c r="G210" s="15"/>
+      <c r="H210" s="15"/>
+      <c r="I210" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J210" s="14"/>
+      <c r="K210" s="14"/>
+      <c r="L210" s="14"/>
+      <c r="M210" s="14"/>
+      <c r="N210" s="14"/>
+      <c r="O210" s="14"/>
+      <c r="P210" s="14"/>
+      <c r="Q210" s="14"/>
+      <c r="R210" s="14"/>
+      <c r="S210" s="14"/>
+      <c r="T210" s="14"/>
+    </row>
+    <row r="211" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A211" s="15" t="s">
+        <v>685</v>
+      </c>
+      <c r="B211" s="20" t="s">
+        <v>637</v>
+      </c>
+      <c r="C211" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D211" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E211" s="15"/>
+      <c r="F211" s="15"/>
+      <c r="G211" s="15"/>
+      <c r="H211" s="15"/>
+      <c r="I211" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J211" s="14"/>
+      <c r="K211" s="14"/>
+      <c r="L211" s="14"/>
+      <c r="M211" s="14"/>
+      <c r="N211" s="14"/>
+      <c r="O211" s="14"/>
+      <c r="P211" s="14"/>
+      <c r="Q211" s="14"/>
+      <c r="R211" s="14"/>
+      <c r="S211" s="14"/>
+      <c r="T211" s="14"/>
+    </row>
+    <row r="212" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A212" s="15" t="s">
+        <v>689</v>
+      </c>
+      <c r="B212" s="20" t="s">
+        <v>658</v>
+      </c>
+      <c r="C212" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D212" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E212" s="15"/>
+      <c r="F212" s="15"/>
+      <c r="G212" s="15"/>
+      <c r="H212" s="15"/>
+      <c r="I212" s="14"/>
+      <c r="J212" s="14"/>
+      <c r="K212" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L212" s="14"/>
+      <c r="M212" s="14"/>
+      <c r="N212" s="14"/>
+      <c r="O212" s="14"/>
+      <c r="P212" s="14"/>
+      <c r="Q212" s="14"/>
+      <c r="R212" s="14"/>
+      <c r="S212" s="14"/>
+      <c r="T212" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
commit the changes done as part of OB scenario for Lot Item
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E08D088-EA38-433F-89C6-9A37330B04DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1696CD28-42FF-4C93-BFCB-A62808851796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2973" uniqueCount="695">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2988" uniqueCount="697">
   <si>
     <t>1</t>
   </si>
@@ -2113,6 +2113,12 @@
   </si>
   <si>
     <t>07P02-05</t>
+  </si>
+  <si>
+    <t>APC_IBScenario012</t>
+  </si>
+  <si>
+    <t>998</t>
   </si>
 </sst>
 </file>
@@ -2656,7 +2662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI420"/>
+  <dimension ref="A1:AI421"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -11761,15 +11767,25 @@
       <c r="AI194" s="14"/>
     </row>
     <row r="195" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A195" s="14"/>
-      <c r="B195" s="14"/>
-      <c r="C195" s="14"/>
-      <c r="D195" s="18"/>
+      <c r="A195" s="14" t="s">
+        <v>695</v>
+      </c>
+      <c r="B195" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C195" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D195" s="18" t="s">
+        <v>696</v>
+      </c>
       <c r="E195" s="14"/>
       <c r="F195" s="14"/>
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
-      <c r="I195" s="14"/>
+      <c r="I195" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J195" s="14"/>
       <c r="K195" s="14"/>
       <c r="L195" s="31"/>
@@ -11791,25 +11807,21 @@
       <c r="AB195" s="14"/>
       <c r="AC195" s="14"/>
       <c r="AD195" s="14"/>
-      <c r="AE195" s="27"/>
+      <c r="AE195" s="27" t="s">
+        <v>650</v>
+      </c>
       <c r="AF195" s="14"/>
       <c r="AG195" s="14"/>
-      <c r="AH195" s="14"/>
+      <c r="AH195" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI195" s="14"/>
     </row>
     <row r="196" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A196" s="14" t="s">
-        <v>664</v>
-      </c>
-      <c r="B196" s="14" t="s">
-        <v>613</v>
-      </c>
-      <c r="C196" s="14" t="s">
-        <v>614</v>
-      </c>
-      <c r="D196" s="23" t="s">
-        <v>665</v>
-      </c>
+      <c r="A196" s="14"/>
+      <c r="B196" s="14"/>
+      <c r="C196" s="14"/>
+      <c r="D196" s="18"/>
       <c r="E196" s="14"/>
       <c r="F196" s="14"/>
       <c r="G196" s="14"/>
@@ -11817,8 +11829,8 @@
       <c r="I196" s="14"/>
       <c r="J196" s="14"/>
       <c r="K196" s="14"/>
-      <c r="L196" s="14"/>
-      <c r="M196" s="14"/>
+      <c r="L196" s="31"/>
+      <c r="M196" s="30"/>
       <c r="N196" s="14"/>
       <c r="O196" s="14"/>
       <c r="P196" s="14"/>
@@ -11833,26 +11845,18 @@
       <c r="Y196" s="14"/>
       <c r="Z196" s="14"/>
       <c r="AA196" s="14"/>
-      <c r="AB196" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC196" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD196" s="14" t="s">
-        <v>451</v>
-      </c>
+      <c r="AB196" s="14"/>
+      <c r="AC196" s="14"/>
+      <c r="AD196" s="14"/>
       <c r="AE196" s="27"/>
       <c r="AF196" s="14"/>
       <c r="AG196" s="14"/>
-      <c r="AH196" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH196" s="14"/>
       <c r="AI196" s="14"/>
     </row>
     <row r="197" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="14" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B197" s="14" t="s">
         <v>613</v>
@@ -11887,23 +11891,25 @@
       <c r="Z197" s="14"/>
       <c r="AA197" s="14"/>
       <c r="AB197" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC197" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD197" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE197" s="27"/>
       <c r="AF197" s="14"/>
       <c r="AG197" s="14"/>
-      <c r="AH197" s="14"/>
+      <c r="AH197" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI197" s="14"/>
     </row>
     <row r="198" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="14" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="B198" s="14" t="s">
         <v>613</v>
@@ -11912,7 +11918,7 @@
         <v>614</v>
       </c>
       <c r="D198" s="23" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="E198" s="14"/>
       <c r="F198" s="14"/>
@@ -11938,25 +11944,23 @@
       <c r="Z198" s="14"/>
       <c r="AA198" s="14"/>
       <c r="AB198" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC198" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD198" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE198" s="27"/>
       <c r="AF198" s="14"/>
       <c r="AG198" s="14"/>
-      <c r="AH198" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH198" s="14"/>
       <c r="AI198" s="14"/>
     </row>
     <row r="199" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="14" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B199" s="14" t="s">
         <v>613</v>
@@ -11965,7 +11969,7 @@
         <v>614</v>
       </c>
       <c r="D199" s="23" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="E199" s="14"/>
       <c r="F199" s="14"/>
@@ -11991,13 +11995,13 @@
       <c r="Z199" s="14"/>
       <c r="AA199" s="14"/>
       <c r="AB199" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC199" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD199" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE199" s="27"/>
       <c r="AF199" s="14"/>
@@ -12009,7 +12013,7 @@
     </row>
     <row r="200" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="14" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B200" s="14" t="s">
         <v>613</v>
@@ -12018,7 +12022,7 @@
         <v>614</v>
       </c>
       <c r="D200" s="23" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="E200" s="14"/>
       <c r="F200" s="14"/>
@@ -12044,13 +12048,13 @@
       <c r="Z200" s="14"/>
       <c r="AA200" s="14"/>
       <c r="AB200" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC200" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD200" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE200" s="27"/>
       <c r="AF200" s="14"/>
@@ -12062,7 +12066,7 @@
     </row>
     <row r="201" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="14" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="B201" s="14" t="s">
         <v>613</v>
@@ -12097,13 +12101,13 @@
       <c r="Z201" s="14"/>
       <c r="AA201" s="14"/>
       <c r="AB201" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC201" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD201" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE201" s="27"/>
       <c r="AF201" s="14"/>
@@ -12115,7 +12119,7 @@
     </row>
     <row r="202" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="14" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B202" s="14" t="s">
         <v>613</v>
@@ -12123,8 +12127,8 @@
       <c r="C202" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D202" s="18" t="s">
-        <v>678</v>
+      <c r="D202" s="23" t="s">
+        <v>674</v>
       </c>
       <c r="E202" s="14"/>
       <c r="F202" s="14"/>
@@ -12150,13 +12154,13 @@
       <c r="Z202" s="14"/>
       <c r="AA202" s="14"/>
       <c r="AB202" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC202" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD202" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE202" s="27"/>
       <c r="AF202" s="14"/>
@@ -12168,7 +12172,7 @@
     </row>
     <row r="203" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="14" t="s">
-        <v>681</v>
+        <v>676</v>
       </c>
       <c r="B203" s="14" t="s">
         <v>613</v>
@@ -12177,7 +12181,7 @@
         <v>614</v>
       </c>
       <c r="D203" s="18" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="E203" s="14"/>
       <c r="F203" s="14"/>
@@ -12221,7 +12225,7 @@
     </row>
     <row r="204" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A204" s="14" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="B204" s="14" t="s">
         <v>613</v>
@@ -12256,13 +12260,13 @@
       <c r="Z204" s="14"/>
       <c r="AA204" s="14"/>
       <c r="AB204" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC204" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD204" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE204" s="27"/>
       <c r="AF204" s="14"/>
@@ -12274,7 +12278,7 @@
     </row>
     <row r="205" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="14" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="B205" s="14" t="s">
         <v>613</v>
@@ -12283,7 +12287,7 @@
         <v>614</v>
       </c>
       <c r="D205" s="18" t="s">
-        <v>687</v>
+        <v>682</v>
       </c>
       <c r="E205" s="14"/>
       <c r="F205" s="14"/>
@@ -12309,13 +12313,13 @@
       <c r="Z205" s="14"/>
       <c r="AA205" s="14"/>
       <c r="AB205" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC205" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD205" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE205" s="27"/>
       <c r="AF205" s="14"/>
@@ -12327,7 +12331,7 @@
     </row>
     <row r="206" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="14" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B206" s="14" t="s">
         <v>613</v>
@@ -12362,13 +12366,13 @@
       <c r="Z206" s="14"/>
       <c r="AA206" s="14"/>
       <c r="AB206" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC206" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD206" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE206" s="27"/>
       <c r="AF206" s="14"/>
@@ -12380,7 +12384,7 @@
     </row>
     <row r="207" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="14" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="B207" s="14" t="s">
         <v>613</v>
@@ -12388,8 +12392,8 @@
       <c r="C207" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D207" s="23" t="s">
-        <v>689</v>
+      <c r="D207" s="18" t="s">
+        <v>687</v>
       </c>
       <c r="E207" s="14"/>
       <c r="F207" s="14"/>
@@ -12433,7 +12437,7 @@
     </row>
     <row r="208" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="14" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="B208" s="14" t="s">
         <v>613</v>
@@ -12442,7 +12446,7 @@
         <v>614</v>
       </c>
       <c r="D208" s="23" t="s">
-        <v>689</v>
+        <v>669</v>
       </c>
       <c r="E208" s="14"/>
       <c r="F208" s="14"/>
@@ -12468,15 +12472,17 @@
       <c r="Z208" s="14"/>
       <c r="AA208" s="14"/>
       <c r="AB208" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC208" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD208" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE208" s="27"/>
+        <v>421</v>
+      </c>
+      <c r="AE208" s="27" t="s">
+        <v>650</v>
+      </c>
       <c r="AF208" s="14"/>
       <c r="AG208" s="14"/>
       <c r="AH208" s="14" t="s">
@@ -12485,10 +12491,18 @@
       <c r="AI208" s="14"/>
     </row>
     <row r="209" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A209" s="14"/>
-      <c r="B209" s="14"/>
-      <c r="C209" s="14"/>
-      <c r="D209" s="14"/>
+      <c r="A209" s="14" t="s">
+        <v>693</v>
+      </c>
+      <c r="B209" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C209" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D209" s="23" t="s">
+        <v>669</v>
+      </c>
       <c r="E209" s="14"/>
       <c r="F209" s="14"/>
       <c r="G209" s="14"/>
@@ -12512,40 +12526,38 @@
       <c r="Y209" s="14"/>
       <c r="Z209" s="14"/>
       <c r="AA209" s="14"/>
-      <c r="AB209" s="14"/>
-      <c r="AC209" s="14"/>
-      <c r="AD209" s="14"/>
-      <c r="AE209" s="27"/>
+      <c r="AB209" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC209" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD209" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="AE209" s="27" t="s">
+        <v>650</v>
+      </c>
       <c r="AF209" s="14"/>
       <c r="AG209" s="14"/>
-      <c r="AH209" s="14"/>
+      <c r="AH209" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI209" s="14"/>
     </row>
     <row r="210" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A210" s="14" t="s">
-        <v>267</v>
-      </c>
-      <c r="B210" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C210" s="14" t="s">
-        <v>135</v>
-      </c>
+      <c r="A210" s="14"/>
+      <c r="B210" s="14"/>
+      <c r="C210" s="14"/>
       <c r="D210" s="14"/>
       <c r="E210" s="14"/>
       <c r="F210" s="14"/>
       <c r="G210" s="14"/>
       <c r="H210" s="14"/>
       <c r="I210" s="14"/>
-      <c r="J210" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K210" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L210" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J210" s="14"/>
+      <c r="K210" s="14"/>
+      <c r="L210" s="14"/>
       <c r="M210" s="14"/>
       <c r="N210" s="14"/>
       <c r="O210" s="14"/>
@@ -12572,7 +12584,7 @@
     </row>
     <row r="211" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="14" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B211" s="14" t="s">
         <v>174</v>
@@ -12587,13 +12599,13 @@
       <c r="H211" s="14"/>
       <c r="I211" s="14"/>
       <c r="J211" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K211" s="15" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="L211" s="15" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="M211" s="14"/>
       <c r="N211" s="14"/>
@@ -12619,9 +12631,9 @@
       <c r="AH211" s="14"/>
       <c r="AI211" s="14"/>
     </row>
-    <row r="212" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="14" t="s">
-        <v>359</v>
+        <v>268</v>
       </c>
       <c r="B212" s="14" t="s">
         <v>174</v>
@@ -12629,9 +12641,36 @@
       <c r="C212" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O212" s="15" t="s">
-        <v>362</v>
-      </c>
+      <c r="D212" s="14"/>
+      <c r="E212" s="14"/>
+      <c r="F212" s="14"/>
+      <c r="G212" s="14"/>
+      <c r="H212" s="14"/>
+      <c r="I212" s="14"/>
+      <c r="J212" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K212" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L212" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M212" s="14"/>
+      <c r="N212" s="14"/>
+      <c r="O212" s="14"/>
+      <c r="P212" s="14"/>
+      <c r="Q212" s="14"/>
+      <c r="R212" s="14"/>
+      <c r="S212" s="14"/>
+      <c r="T212" s="14"/>
+      <c r="U212" s="14"/>
+      <c r="V212" s="14"/>
+      <c r="W212" s="14"/>
+      <c r="X212" s="14"/>
+      <c r="Y212" s="14"/>
+      <c r="Z212" s="14"/>
+      <c r="AA212" s="14"/>
       <c r="AB212" s="14"/>
       <c r="AC212" s="14"/>
       <c r="AD212" s="14"/>
@@ -12643,7 +12682,7 @@
     </row>
     <row r="213" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A213" s="14" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B213" s="14" t="s">
         <v>174</v>
@@ -12652,7 +12691,7 @@
         <v>135</v>
       </c>
       <c r="O213" s="15" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AB213" s="14"/>
       <c r="AC213" s="14"/>
@@ -12665,7 +12704,7 @@
     </row>
     <row r="214" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A214" s="14" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B214" s="14" t="s">
         <v>174</v>
@@ -12674,7 +12713,7 @@
         <v>135</v>
       </c>
       <c r="O214" s="15" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AB214" s="14"/>
       <c r="AC214" s="14"/>
@@ -12687,7 +12726,7 @@
     </row>
     <row r="215" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A215" s="14" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="B215" s="14" t="s">
         <v>174</v>
@@ -12695,8 +12734,8 @@
       <c r="C215" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M215" s="14" t="s">
-        <v>371</v>
+      <c r="O215" s="15" t="s">
+        <v>364</v>
       </c>
       <c r="AB215" s="14"/>
       <c r="AC215" s="14"/>
@@ -12708,6 +12747,18 @@
       <c r="AI215" s="14"/>
     </row>
     <row r="216" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A216" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B216" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C216" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M216" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB216" s="14"/>
       <c r="AC216" s="14"/>
       <c r="AD216" s="14"/>
@@ -14691,7 +14742,7 @@
       <c r="AB414" s="14"/>
       <c r="AC414" s="14"/>
       <c r="AD414" s="14"/>
-      <c r="AE414" s="14"/>
+      <c r="AE414" s="27"/>
       <c r="AF414" s="14"/>
       <c r="AG414" s="14"/>
       <c r="AH414" s="14"/>
@@ -14757,6 +14808,16 @@
       <c r="AH420" s="14"/>
       <c r="AI420" s="14"/>
     </row>
+    <row r="421" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB421" s="14"/>
+      <c r="AC421" s="14"/>
+      <c r="AD421" s="14"/>
+      <c r="AE421" s="14"/>
+      <c r="AF421" s="14"/>
+      <c r="AG421" s="14"/>
+      <c r="AH421" s="14"/>
+      <c r="AI421" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14766,7 +14827,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T212"/>
+  <dimension ref="A1:T213"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -21455,7 +21516,7 @@
         <v>0</v>
       </c>
       <c r="D204" s="16" t="s">
-        <v>112</v>
+        <v>632</v>
       </c>
       <c r="E204" s="15"/>
       <c r="F204" s="15"/>
@@ -21484,10 +21545,10 @@
         <v>694</v>
       </c>
       <c r="C205" s="15" t="s">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="D205" s="16" t="s">
-        <v>112</v>
+        <v>632</v>
       </c>
       <c r="E205" s="15"/>
       <c r="F205" s="15"/>
@@ -21731,6 +21792,40 @@
       <c r="R212" s="14"/>
       <c r="S212" s="14"/>
       <c r="T212" s="14"/>
+    </row>
+    <row r="213" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A213" s="15" t="s">
+        <v>696</v>
+      </c>
+      <c r="B213" s="20" t="s">
+        <v>694</v>
+      </c>
+      <c r="C213" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D213" s="14" t="s">
+        <v>632</v>
+      </c>
+      <c r="E213" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F213" s="15"/>
+      <c r="G213" s="15"/>
+      <c r="H213" s="15"/>
+      <c r="I213" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J213" s="14"/>
+      <c r="K213" s="14"/>
+      <c r="L213" s="14"/>
+      <c r="M213" s="14"/>
+      <c r="N213" s="14"/>
+      <c r="O213" s="14"/>
+      <c r="P213" s="14"/>
+      <c r="Q213" s="14"/>
+      <c r="R213" s="14"/>
+      <c r="S213" s="14"/>
+      <c r="T213" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
Commit latest code for APC
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1696CD28-42FF-4C93-BFCB-A62808851796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B746E9-77E8-4135-B209-6CF71DC9436F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15390" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2988" uniqueCount="697">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3043" uniqueCount="709">
   <si>
     <t>1</t>
   </si>
@@ -2119,6 +2119,42 @@
   </si>
   <si>
     <t>998</t>
+  </si>
+  <si>
+    <t>Dangerous</t>
+  </si>
+  <si>
+    <t>UNDA</t>
+  </si>
+  <si>
+    <t>UPSN</t>
+  </si>
+  <si>
+    <t>KWEWW</t>
+  </si>
+  <si>
+    <t>KWEO</t>
+  </si>
+  <si>
+    <t>APC_OBScenario14</t>
+  </si>
+  <si>
+    <t>999</t>
+  </si>
+  <si>
+    <t>APC_OBScenario15</t>
+  </si>
+  <si>
+    <t>APC_OBScenario16</t>
+  </si>
+  <si>
+    <t>APC_OBScenario17</t>
+  </si>
+  <si>
+    <t>APC_OBScenario18</t>
+  </si>
+  <si>
+    <t>APC_OBScenario19</t>
   </si>
 </sst>
 </file>
@@ -2662,7 +2698,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI421"/>
+  <dimension ref="A1:AI399"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -12546,10 +12582,18 @@
       <c r="AI209" s="14"/>
     </row>
     <row r="210" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A210" s="14"/>
-      <c r="B210" s="14"/>
-      <c r="C210" s="14"/>
-      <c r="D210" s="14"/>
+      <c r="A210" s="14" t="s">
+        <v>702</v>
+      </c>
+      <c r="B210" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C210" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D210" s="18" t="s">
+        <v>628</v>
+      </c>
       <c r="E210" s="14"/>
       <c r="F210" s="14"/>
       <c r="G210" s="14"/>
@@ -12573,40 +12617,46 @@
       <c r="Y210" s="14"/>
       <c r="Z210" s="14"/>
       <c r="AA210" s="14"/>
-      <c r="AB210" s="14"/>
-      <c r="AC210" s="14"/>
-      <c r="AD210" s="14"/>
-      <c r="AE210" s="27"/>
+      <c r="AB210" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC210" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD210" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="AE210" s="27" t="s">
+        <v>697</v>
+      </c>
       <c r="AF210" s="14"/>
       <c r="AG210" s="14"/>
-      <c r="AH210" s="14"/>
+      <c r="AH210" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI210" s="14"/>
     </row>
     <row r="211" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="14" t="s">
-        <v>267</v>
+        <v>704</v>
       </c>
       <c r="B211" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C211" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D211" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D211" s="18" t="s">
+        <v>665</v>
+      </c>
       <c r="E211" s="14"/>
       <c r="F211" s="14"/>
       <c r="G211" s="14"/>
       <c r="H211" s="14"/>
       <c r="I211" s="14"/>
-      <c r="J211" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K211" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L211" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J211" s="14"/>
+      <c r="K211" s="14"/>
+      <c r="L211" s="14"/>
       <c r="M211" s="14"/>
       <c r="N211" s="14"/>
       <c r="O211" s="14"/>
@@ -12622,40 +12672,46 @@
       <c r="Y211" s="14"/>
       <c r="Z211" s="14"/>
       <c r="AA211" s="14"/>
-      <c r="AB211" s="14"/>
-      <c r="AC211" s="14"/>
-      <c r="AD211" s="14"/>
-      <c r="AE211" s="27"/>
+      <c r="AB211" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC211" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD211" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="AE211" s="27" t="s">
+        <v>651</v>
+      </c>
       <c r="AF211" s="14"/>
       <c r="AG211" s="14"/>
-      <c r="AH211" s="14"/>
+      <c r="AH211" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI211" s="14"/>
     </row>
     <row r="212" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="14" t="s">
-        <v>268</v>
+        <v>705</v>
       </c>
       <c r="B212" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C212" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D212" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D212" s="18" t="s">
+        <v>677</v>
+      </c>
       <c r="E212" s="14"/>
       <c r="F212" s="14"/>
       <c r="G212" s="14"/>
       <c r="H212" s="14"/>
       <c r="I212" s="14"/>
-      <c r="J212" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K212" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L212" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="J212" s="14"/>
+      <c r="K212" s="14"/>
+      <c r="L212" s="14"/>
       <c r="M212" s="14"/>
       <c r="N212" s="14"/>
       <c r="O212" s="14"/>
@@ -12671,94 +12727,210 @@
       <c r="Y212" s="14"/>
       <c r="Z212" s="14"/>
       <c r="AA212" s="14"/>
-      <c r="AB212" s="14"/>
-      <c r="AC212" s="14"/>
-      <c r="AD212" s="14"/>
+      <c r="AB212" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC212" s="14" t="s">
+        <v>698</v>
+      </c>
+      <c r="AD212" s="14" t="s">
+        <v>699</v>
+      </c>
       <c r="AE212" s="27"/>
       <c r="AF212" s="14"/>
       <c r="AG212" s="14"/>
       <c r="AH212" s="14"/>
       <c r="AI212" s="14"/>
     </row>
-    <row r="213" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A213" s="14" t="s">
-        <v>359</v>
+        <v>706</v>
       </c>
       <c r="B213" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C213" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O213" s="15" t="s">
-        <v>362</v>
-      </c>
-      <c r="AB213" s="14"/>
-      <c r="AC213" s="14"/>
-      <c r="AD213" s="14"/>
-      <c r="AE213" s="27"/>
+        <v>614</v>
+      </c>
+      <c r="D213" s="18" t="s">
+        <v>677</v>
+      </c>
+      <c r="E213" s="14"/>
+      <c r="F213" s="14"/>
+      <c r="G213" s="14"/>
+      <c r="H213" s="14"/>
+      <c r="I213" s="14"/>
+      <c r="J213" s="14"/>
+      <c r="K213" s="14"/>
+      <c r="L213" s="14"/>
+      <c r="M213" s="14"/>
+      <c r="N213" s="14"/>
+      <c r="O213" s="14"/>
+      <c r="P213" s="14"/>
+      <c r="Q213" s="14"/>
+      <c r="R213" s="14"/>
+      <c r="S213" s="14"/>
+      <c r="T213" s="14"/>
+      <c r="U213" s="14"/>
+      <c r="V213" s="14"/>
+      <c r="W213" s="14"/>
+      <c r="X213" s="14"/>
+      <c r="Y213" s="14"/>
+      <c r="Z213" s="14"/>
+      <c r="AA213" s="14"/>
+      <c r="AB213" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC213" s="14" t="s">
+        <v>700</v>
+      </c>
+      <c r="AD213" s="14" t="s">
+        <v>701</v>
+      </c>
+      <c r="AE213" s="27" t="s">
+        <v>651</v>
+      </c>
       <c r="AF213" s="14"/>
       <c r="AG213" s="14"/>
       <c r="AH213" s="14"/>
       <c r="AI213" s="14"/>
     </row>
-    <row r="214" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A214" s="14" t="s">
-        <v>360</v>
+        <v>707</v>
       </c>
       <c r="B214" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C214" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O214" s="15" t="s">
-        <v>363</v>
-      </c>
-      <c r="AB214" s="14"/>
-      <c r="AC214" s="14"/>
-      <c r="AD214" s="14"/>
-      <c r="AE214" s="27"/>
+        <v>614</v>
+      </c>
+      <c r="D214" s="18" t="s">
+        <v>628</v>
+      </c>
+      <c r="E214" s="14"/>
+      <c r="F214" s="14"/>
+      <c r="G214" s="14"/>
+      <c r="H214" s="14"/>
+      <c r="I214" s="14"/>
+      <c r="J214" s="14"/>
+      <c r="K214" s="14"/>
+      <c r="L214" s="14"/>
+      <c r="M214" s="14"/>
+      <c r="N214" s="14"/>
+      <c r="O214" s="14"/>
+      <c r="P214" s="14"/>
+      <c r="Q214" s="14"/>
+      <c r="R214" s="14"/>
+      <c r="S214" s="14"/>
+      <c r="T214" s="14"/>
+      <c r="U214" s="14"/>
+      <c r="V214" s="14"/>
+      <c r="W214" s="14"/>
+      <c r="X214" s="14"/>
+      <c r="Y214" s="14"/>
+      <c r="Z214" s="14"/>
+      <c r="AA214" s="14"/>
+      <c r="AB214" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC214" s="14" t="s">
+        <v>698</v>
+      </c>
+      <c r="AD214" s="14" t="s">
+        <v>699</v>
+      </c>
+      <c r="AE214" s="27" t="s">
+        <v>697</v>
+      </c>
       <c r="AF214" s="14"/>
       <c r="AG214" s="14"/>
       <c r="AH214" s="14"/>
       <c r="AI214" s="14"/>
     </row>
-    <row r="215" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A215" s="14" t="s">
-        <v>361</v>
+        <v>708</v>
       </c>
       <c r="B215" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C215" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O215" s="15" t="s">
-        <v>364</v>
-      </c>
-      <c r="AB215" s="14"/>
-      <c r="AC215" s="14"/>
-      <c r="AD215" s="14"/>
-      <c r="AE215" s="27"/>
+        <v>614</v>
+      </c>
+      <c r="D215" s="18" t="s">
+        <v>703</v>
+      </c>
+      <c r="E215" s="14"/>
+      <c r="F215" s="14"/>
+      <c r="G215" s="14"/>
+      <c r="H215" s="14"/>
+      <c r="I215" s="14"/>
+      <c r="J215" s="14"/>
+      <c r="K215" s="14"/>
+      <c r="L215" s="14"/>
+      <c r="M215" s="14"/>
+      <c r="N215" s="14"/>
+      <c r="O215" s="14"/>
+      <c r="P215" s="14"/>
+      <c r="Q215" s="14"/>
+      <c r="R215" s="14"/>
+      <c r="S215" s="14"/>
+      <c r="T215" s="14"/>
+      <c r="U215" s="14"/>
+      <c r="V215" s="14"/>
+      <c r="W215" s="14"/>
+      <c r="X215" s="14"/>
+      <c r="Y215" s="14"/>
+      <c r="Z215" s="14"/>
+      <c r="AA215" s="14"/>
+      <c r="AB215" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC215" s="14" t="s">
+        <v>420</v>
+      </c>
+      <c r="AD215" s="14" t="s">
+        <v>421</v>
+      </c>
+      <c r="AE215" s="27" t="s">
+        <v>654</v>
+      </c>
       <c r="AF215" s="14"/>
       <c r="AG215" s="14"/>
-      <c r="AH215" s="14"/>
+      <c r="AH215" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI215" s="14"/>
     </row>
-    <row r="216" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A216" s="14" t="s">
-        <v>370</v>
-      </c>
-      <c r="B216" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C216" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="M216" s="14" t="s">
-        <v>371</v>
-      </c>
+    <row r="216" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A216" s="14"/>
+      <c r="B216" s="14"/>
+      <c r="C216" s="14"/>
+      <c r="D216" s="14"/>
+      <c r="E216" s="14"/>
+      <c r="F216" s="14"/>
+      <c r="G216" s="14"/>
+      <c r="H216" s="14"/>
+      <c r="I216" s="14"/>
+      <c r="J216" s="14"/>
+      <c r="K216" s="14"/>
+      <c r="L216" s="14"/>
+      <c r="M216" s="14"/>
+      <c r="N216" s="14"/>
+      <c r="O216" s="14"/>
+      <c r="P216" s="14"/>
+      <c r="Q216" s="14"/>
+      <c r="R216" s="14"/>
+      <c r="S216" s="14"/>
+      <c r="T216" s="14"/>
+      <c r="U216" s="14"/>
+      <c r="V216" s="14"/>
+      <c r="W216" s="14"/>
+      <c r="X216" s="14"/>
+      <c r="Y216" s="14"/>
+      <c r="Z216" s="14"/>
+      <c r="AA216" s="14"/>
       <c r="AB216" s="14"/>
       <c r="AC216" s="14"/>
       <c r="AD216" s="14"/>
@@ -12768,7 +12940,46 @@
       <c r="AH216" s="14"/>
       <c r="AI216" s="14"/>
     </row>
-    <row r="217" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A217" s="14" t="s">
+        <v>267</v>
+      </c>
+      <c r="B217" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C217" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D217" s="14"/>
+      <c r="E217" s="14"/>
+      <c r="F217" s="14"/>
+      <c r="G217" s="14"/>
+      <c r="H217" s="14"/>
+      <c r="I217" s="14"/>
+      <c r="J217" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K217" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L217" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M217" s="14"/>
+      <c r="N217" s="14"/>
+      <c r="O217" s="14"/>
+      <c r="P217" s="14"/>
+      <c r="Q217" s="14"/>
+      <c r="R217" s="14"/>
+      <c r="S217" s="14"/>
+      <c r="T217" s="14"/>
+      <c r="U217" s="14"/>
+      <c r="V217" s="14"/>
+      <c r="W217" s="14"/>
+      <c r="X217" s="14"/>
+      <c r="Y217" s="14"/>
+      <c r="Z217" s="14"/>
+      <c r="AA217" s="14"/>
       <c r="AB217" s="14"/>
       <c r="AC217" s="14"/>
       <c r="AD217" s="14"/>
@@ -12778,7 +12989,46 @@
       <c r="AH217" s="14"/>
       <c r="AI217" s="14"/>
     </row>
-    <row r="218" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A218" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="B218" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C218" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D218" s="14"/>
+      <c r="E218" s="14"/>
+      <c r="F218" s="14"/>
+      <c r="G218" s="14"/>
+      <c r="H218" s="14"/>
+      <c r="I218" s="14"/>
+      <c r="J218" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K218" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L218" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M218" s="14"/>
+      <c r="N218" s="14"/>
+      <c r="O218" s="14"/>
+      <c r="P218" s="14"/>
+      <c r="Q218" s="14"/>
+      <c r="R218" s="14"/>
+      <c r="S218" s="14"/>
+      <c r="T218" s="14"/>
+      <c r="U218" s="14"/>
+      <c r="V218" s="14"/>
+      <c r="W218" s="14"/>
+      <c r="X218" s="14"/>
+      <c r="Y218" s="14"/>
+      <c r="Z218" s="14"/>
+      <c r="AA218" s="14"/>
       <c r="AB218" s="14"/>
       <c r="AC218" s="14"/>
       <c r="AD218" s="14"/>
@@ -12789,6 +13039,18 @@
       <c r="AI218" s="14"/>
     </row>
     <row r="219" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A219" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="B219" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C219" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O219" s="15" t="s">
+        <v>362</v>
+      </c>
       <c r="AB219" s="14"/>
       <c r="AC219" s="14"/>
       <c r="AD219" s="14"/>
@@ -12799,6 +13061,18 @@
       <c r="AI219" s="14"/>
     </row>
     <row r="220" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A220" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B220" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C220" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O220" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB220" s="14"/>
       <c r="AC220" s="14"/>
       <c r="AD220" s="14"/>
@@ -12809,6 +13083,18 @@
       <c r="AI220" s="14"/>
     </row>
     <row r="221" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A221" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B221" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C221" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O221" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB221" s="14"/>
       <c r="AC221" s="14"/>
       <c r="AD221" s="14"/>
@@ -12819,6 +13105,18 @@
       <c r="AI221" s="14"/>
     </row>
     <row r="222" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A222" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B222" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C222" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M222" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB222" s="14"/>
       <c r="AC222" s="14"/>
       <c r="AD222" s="14"/>
@@ -14532,7 +14830,7 @@
       <c r="AB393" s="14"/>
       <c r="AC393" s="14"/>
       <c r="AD393" s="14"/>
-      <c r="AE393" s="27"/>
+      <c r="AE393" s="14"/>
       <c r="AF393" s="14"/>
       <c r="AG393" s="14"/>
       <c r="AH393" s="14"/>
@@ -14542,7 +14840,7 @@
       <c r="AB394" s="14"/>
       <c r="AC394" s="14"/>
       <c r="AD394" s="14"/>
-      <c r="AE394" s="27"/>
+      <c r="AE394" s="14"/>
       <c r="AF394" s="14"/>
       <c r="AG394" s="14"/>
       <c r="AH394" s="14"/>
@@ -14552,7 +14850,7 @@
       <c r="AB395" s="14"/>
       <c r="AC395" s="14"/>
       <c r="AD395" s="14"/>
-      <c r="AE395" s="27"/>
+      <c r="AE395" s="14"/>
       <c r="AF395" s="14"/>
       <c r="AG395" s="14"/>
       <c r="AH395" s="14"/>
@@ -14562,7 +14860,7 @@
       <c r="AB396" s="14"/>
       <c r="AC396" s="14"/>
       <c r="AD396" s="14"/>
-      <c r="AE396" s="27"/>
+      <c r="AE396" s="14"/>
       <c r="AF396" s="14"/>
       <c r="AG396" s="14"/>
       <c r="AH396" s="14"/>
@@ -14572,7 +14870,7 @@
       <c r="AB397" s="14"/>
       <c r="AC397" s="14"/>
       <c r="AD397" s="14"/>
-      <c r="AE397" s="27"/>
+      <c r="AE397" s="14"/>
       <c r="AF397" s="14"/>
       <c r="AG397" s="14"/>
       <c r="AH397" s="14"/>
@@ -14582,7 +14880,7 @@
       <c r="AB398" s="14"/>
       <c r="AC398" s="14"/>
       <c r="AD398" s="14"/>
-      <c r="AE398" s="27"/>
+      <c r="AE398" s="14"/>
       <c r="AF398" s="14"/>
       <c r="AG398" s="14"/>
       <c r="AH398" s="14"/>
@@ -14592,231 +14890,11 @@
       <c r="AB399" s="14"/>
       <c r="AC399" s="14"/>
       <c r="AD399" s="14"/>
-      <c r="AE399" s="27"/>
+      <c r="AE399" s="14"/>
       <c r="AF399" s="14"/>
       <c r="AG399" s="14"/>
       <c r="AH399" s="14"/>
       <c r="AI399" s="14"/>
-    </row>
-    <row r="400" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB400" s="14"/>
-      <c r="AC400" s="14"/>
-      <c r="AD400" s="14"/>
-      <c r="AE400" s="27"/>
-      <c r="AF400" s="14"/>
-      <c r="AG400" s="14"/>
-      <c r="AH400" s="14"/>
-      <c r="AI400" s="14"/>
-    </row>
-    <row r="401" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB401" s="14"/>
-      <c r="AC401" s="14"/>
-      <c r="AD401" s="14"/>
-      <c r="AE401" s="27"/>
-      <c r="AF401" s="14"/>
-      <c r="AG401" s="14"/>
-      <c r="AH401" s="14"/>
-      <c r="AI401" s="14"/>
-    </row>
-    <row r="402" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB402" s="14"/>
-      <c r="AC402" s="14"/>
-      <c r="AD402" s="14"/>
-      <c r="AE402" s="27"/>
-      <c r="AF402" s="14"/>
-      <c r="AG402" s="14"/>
-      <c r="AH402" s="14"/>
-      <c r="AI402" s="14"/>
-    </row>
-    <row r="403" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB403" s="14"/>
-      <c r="AC403" s="14"/>
-      <c r="AD403" s="14"/>
-      <c r="AE403" s="27"/>
-      <c r="AF403" s="14"/>
-      <c r="AG403" s="14"/>
-      <c r="AH403" s="14"/>
-      <c r="AI403" s="14"/>
-    </row>
-    <row r="404" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB404" s="14"/>
-      <c r="AC404" s="14"/>
-      <c r="AD404" s="14"/>
-      <c r="AE404" s="27"/>
-      <c r="AF404" s="14"/>
-      <c r="AG404" s="14"/>
-      <c r="AH404" s="14"/>
-      <c r="AI404" s="14"/>
-    </row>
-    <row r="405" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB405" s="14"/>
-      <c r="AC405" s="14"/>
-      <c r="AD405" s="14"/>
-      <c r="AE405" s="27"/>
-      <c r="AF405" s="14"/>
-      <c r="AG405" s="14"/>
-      <c r="AH405" s="14"/>
-      <c r="AI405" s="14"/>
-    </row>
-    <row r="406" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB406" s="14"/>
-      <c r="AC406" s="14"/>
-      <c r="AD406" s="14"/>
-      <c r="AE406" s="27"/>
-      <c r="AF406" s="14"/>
-      <c r="AG406" s="14"/>
-      <c r="AH406" s="14"/>
-      <c r="AI406" s="14"/>
-    </row>
-    <row r="407" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB407" s="14"/>
-      <c r="AC407" s="14"/>
-      <c r="AD407" s="14"/>
-      <c r="AE407" s="27"/>
-      <c r="AF407" s="14"/>
-      <c r="AG407" s="14"/>
-      <c r="AH407" s="14"/>
-      <c r="AI407" s="14"/>
-    </row>
-    <row r="408" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB408" s="14"/>
-      <c r="AC408" s="14"/>
-      <c r="AD408" s="14"/>
-      <c r="AE408" s="27"/>
-      <c r="AF408" s="14"/>
-      <c r="AG408" s="14"/>
-      <c r="AH408" s="14"/>
-      <c r="AI408" s="14"/>
-    </row>
-    <row r="409" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB409" s="14"/>
-      <c r="AC409" s="14"/>
-      <c r="AD409" s="14"/>
-      <c r="AE409" s="27"/>
-      <c r="AF409" s="14"/>
-      <c r="AG409" s="14"/>
-      <c r="AH409" s="14"/>
-      <c r="AI409" s="14"/>
-    </row>
-    <row r="410" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB410" s="14"/>
-      <c r="AC410" s="14"/>
-      <c r="AD410" s="14"/>
-      <c r="AE410" s="27"/>
-      <c r="AF410" s="14"/>
-      <c r="AG410" s="14"/>
-      <c r="AH410" s="14"/>
-      <c r="AI410" s="14"/>
-    </row>
-    <row r="411" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB411" s="14"/>
-      <c r="AC411" s="14"/>
-      <c r="AD411" s="14"/>
-      <c r="AE411" s="27"/>
-      <c r="AF411" s="14"/>
-      <c r="AG411" s="14"/>
-      <c r="AH411" s="14"/>
-      <c r="AI411" s="14"/>
-    </row>
-    <row r="412" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB412" s="14"/>
-      <c r="AC412" s="14"/>
-      <c r="AD412" s="14"/>
-      <c r="AE412" s="27"/>
-      <c r="AF412" s="14"/>
-      <c r="AG412" s="14"/>
-      <c r="AH412" s="14"/>
-      <c r="AI412" s="14"/>
-    </row>
-    <row r="413" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB413" s="14"/>
-      <c r="AC413" s="14"/>
-      <c r="AD413" s="14"/>
-      <c r="AE413" s="27"/>
-      <c r="AF413" s="14"/>
-      <c r="AG413" s="14"/>
-      <c r="AH413" s="14"/>
-      <c r="AI413" s="14"/>
-    </row>
-    <row r="414" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB414" s="14"/>
-      <c r="AC414" s="14"/>
-      <c r="AD414" s="14"/>
-      <c r="AE414" s="27"/>
-      <c r="AF414" s="14"/>
-      <c r="AG414" s="14"/>
-      <c r="AH414" s="14"/>
-      <c r="AI414" s="14"/>
-    </row>
-    <row r="415" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB415" s="14"/>
-      <c r="AC415" s="14"/>
-      <c r="AD415" s="14"/>
-      <c r="AE415" s="14"/>
-      <c r="AF415" s="14"/>
-      <c r="AG415" s="14"/>
-      <c r="AH415" s="14"/>
-      <c r="AI415" s="14"/>
-    </row>
-    <row r="416" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB416" s="14"/>
-      <c r="AC416" s="14"/>
-      <c r="AD416" s="14"/>
-      <c r="AE416" s="14"/>
-      <c r="AF416" s="14"/>
-      <c r="AG416" s="14"/>
-      <c r="AH416" s="14"/>
-      <c r="AI416" s="14"/>
-    </row>
-    <row r="417" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB417" s="14"/>
-      <c r="AC417" s="14"/>
-      <c r="AD417" s="14"/>
-      <c r="AE417" s="14"/>
-      <c r="AF417" s="14"/>
-      <c r="AG417" s="14"/>
-      <c r="AH417" s="14"/>
-      <c r="AI417" s="14"/>
-    </row>
-    <row r="418" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB418" s="14"/>
-      <c r="AC418" s="14"/>
-      <c r="AD418" s="14"/>
-      <c r="AE418" s="14"/>
-      <c r="AF418" s="14"/>
-      <c r="AG418" s="14"/>
-      <c r="AH418" s="14"/>
-      <c r="AI418" s="14"/>
-    </row>
-    <row r="419" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB419" s="14"/>
-      <c r="AC419" s="14"/>
-      <c r="AD419" s="14"/>
-      <c r="AE419" s="14"/>
-      <c r="AF419" s="14"/>
-      <c r="AG419" s="14"/>
-      <c r="AH419" s="14"/>
-      <c r="AI419" s="14"/>
-    </row>
-    <row r="420" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB420" s="14"/>
-      <c r="AC420" s="14"/>
-      <c r="AD420" s="14"/>
-      <c r="AE420" s="14"/>
-      <c r="AF420" s="14"/>
-      <c r="AG420" s="14"/>
-      <c r="AH420" s="14"/>
-      <c r="AI420" s="14"/>
-    </row>
-    <row r="421" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB421" s="14"/>
-      <c r="AC421" s="14"/>
-      <c r="AD421" s="14"/>
-      <c r="AE421" s="14"/>
-      <c r="AF421" s="14"/>
-      <c r="AG421" s="14"/>
-      <c r="AH421" s="14"/>
-      <c r="AI421" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -14827,7 +14905,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T213"/>
+  <dimension ref="A1:T214"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -21827,6 +21905,38 @@
       <c r="S213" s="14"/>
       <c r="T213" s="14"/>
     </row>
+    <row r="214" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A214" s="15" t="s">
+        <v>703</v>
+      </c>
+      <c r="B214" s="30" t="s">
+        <v>658</v>
+      </c>
+      <c r="C214" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D214" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E214" s="15"/>
+      <c r="F214" s="15"/>
+      <c r="G214" s="15"/>
+      <c r="H214" s="15"/>
+      <c r="I214" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J214" s="14"/>
+      <c r="K214" s="14"/>
+      <c r="L214" s="14"/>
+      <c r="M214" s="14"/>
+      <c r="N214" s="14"/>
+      <c r="O214" s="14"/>
+      <c r="P214" s="14"/>
+      <c r="Q214" s="14"/>
+      <c r="R214" s="14"/>
+      <c r="S214" s="14"/>
+      <c r="T214" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
commit the code for 2 new scenarios QSC 4 lines and APC intl high cost
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25629"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B746E9-77E8-4135-B209-6CF71DC9436F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A60254E-AEC9-4624-9413-0E9C86CBB211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15390" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3043" uniqueCount="709">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3059" uniqueCount="713">
   <si>
     <t>1</t>
   </si>
@@ -2155,6 +2155,18 @@
   </si>
   <si>
     <t>APC_OBScenario19</t>
+  </si>
+  <si>
+    <t>APC_OBScenario20</t>
+  </si>
+  <si>
+    <t>FEIP</t>
+  </si>
+  <si>
+    <t>QSC_DailyRegressionOB12</t>
+  </si>
+  <si>
+    <t>112|113|114|115</t>
   </si>
 </sst>
 </file>
@@ -2698,7 +2710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI399"/>
+  <dimension ref="A1:AI401"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -6468,10 +6480,18 @@
       <c r="AI81" s="14"/>
     </row>
     <row r="82" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="14"/>
-      <c r="B82" s="14"/>
-      <c r="C82" s="14"/>
-      <c r="D82" s="23"/>
+      <c r="A82" s="14" t="s">
+        <v>711</v>
+      </c>
+      <c r="B82" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="C82" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D82" s="23" t="s">
+        <v>712</v>
+      </c>
       <c r="E82" s="14"/>
       <c r="F82" s="14"/>
       <c r="G82" s="14"/>
@@ -6495,29 +6515,29 @@
       <c r="Y82" s="14"/>
       <c r="Z82" s="14"/>
       <c r="AA82" s="14"/>
-      <c r="AB82" s="14"/>
-      <c r="AC82" s="14"/>
-      <c r="AD82" s="14"/>
+      <c r="AB82" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC82" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD82" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE82" s="27"/>
       <c r="AF82" s="14"/>
       <c r="AG82" s="14"/>
-      <c r="AH82" s="14"/>
+      <c r="AH82" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI82" s="14"/>
     </row>
     <row r="83" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="14" t="s">
-        <v>302</v>
-      </c>
-      <c r="B83" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="C83" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D83" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="E83" s="15"/>
+      <c r="A83" s="14"/>
+      <c r="B83" s="14"/>
+      <c r="C83" s="14"/>
+      <c r="D83" s="23"/>
+      <c r="E83" s="14"/>
       <c r="F83" s="14"/>
       <c r="G83" s="14"/>
       <c r="H83" s="14"/>
@@ -6551,7 +6571,7 @@
     </row>
     <row r="84" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B84" s="14" t="s">
         <v>107</v>
@@ -6560,9 +6580,9 @@
         <v>135</v>
       </c>
       <c r="D84" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="E84" s="14"/>
+        <v>0</v>
+      </c>
+      <c r="E84" s="15"/>
       <c r="F84" s="14"/>
       <c r="G84" s="14"/>
       <c r="H84" s="14"/>
@@ -6596,7 +6616,7 @@
     </row>
     <row r="85" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="14" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B85" s="14" t="s">
         <v>107</v>
@@ -6605,17 +6625,13 @@
         <v>135</v>
       </c>
       <c r="D85" s="18" t="s">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="E85" s="14"/>
-      <c r="F85" s="14" t="s">
-        <v>403</v>
-      </c>
+      <c r="F85" s="14"/>
       <c r="G85" s="14"/>
       <c r="H85" s="14"/>
-      <c r="I85" s="14" t="s">
-        <v>128</v>
-      </c>
+      <c r="I85" s="14"/>
       <c r="J85" s="14"/>
       <c r="K85" s="14"/>
       <c r="L85" s="14"/>
@@ -6645,7 +6661,7 @@
     </row>
     <row r="86" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="14" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B86" s="14" t="s">
         <v>107</v>
@@ -6654,7 +6670,7 @@
         <v>135</v>
       </c>
       <c r="D86" s="18" t="s">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="E86" s="14"/>
       <c r="F86" s="14" t="s">
@@ -6663,7 +6679,7 @@
       <c r="G86" s="14"/>
       <c r="H86" s="14"/>
       <c r="I86" s="14" t="s">
-        <v>378</v>
+        <v>128</v>
       </c>
       <c r="J86" s="14"/>
       <c r="K86" s="14"/>
@@ -6694,7 +6710,7 @@
     </row>
     <row r="87" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="14" t="s">
-        <v>342</v>
+        <v>305</v>
       </c>
       <c r="B87" s="14" t="s">
         <v>107</v>
@@ -6702,14 +6718,18 @@
       <c r="C87" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D87" s="25" t="s">
-        <v>346</v>
+      <c r="D87" s="18" t="s">
+        <v>118</v>
       </c>
       <c r="E87" s="14"/>
-      <c r="F87" s="14"/>
+      <c r="F87" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G87" s="14"/>
       <c r="H87" s="14"/>
-      <c r="I87" s="14"/>
+      <c r="I87" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J87" s="14"/>
       <c r="K87" s="14"/>
       <c r="L87" s="14"/>
@@ -6739,7 +6759,7 @@
     </row>
     <row r="88" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="14" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B88" s="14" t="s">
         <v>107</v>
@@ -6747,8 +6767,8 @@
       <c r="C88" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D88" s="18" t="s">
-        <v>349</v>
+      <c r="D88" s="25" t="s">
+        <v>346</v>
       </c>
       <c r="E88" s="14"/>
       <c r="F88" s="14"/>
@@ -6784,7 +6804,7 @@
     </row>
     <row r="89" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="14" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B89" s="14" t="s">
         <v>107</v>
@@ -6792,8 +6812,8 @@
       <c r="C89" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D89" s="25" t="s">
-        <v>346</v>
+      <c r="D89" s="18" t="s">
+        <v>349</v>
       </c>
       <c r="E89" s="14"/>
       <c r="F89" s="14"/>
@@ -6829,7 +6849,7 @@
     </row>
     <row r="90" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="14" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B90" s="14" t="s">
         <v>107</v>
@@ -6837,8 +6857,8 @@
       <c r="C90" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D90" s="18" t="s">
-        <v>349</v>
+      <c r="D90" s="25" t="s">
+        <v>346</v>
       </c>
       <c r="E90" s="14"/>
       <c r="F90" s="14"/>
@@ -6874,7 +6894,7 @@
     </row>
     <row r="91" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="14" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="B91" s="14" t="s">
         <v>107</v>
@@ -6882,7 +6902,9 @@
       <c r="C91" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D91" s="18"/>
+      <c r="D91" s="18" t="s">
+        <v>349</v>
+      </c>
       <c r="E91" s="14"/>
       <c r="F91" s="14"/>
       <c r="G91" s="14"/>
@@ -6917,18 +6939,16 @@
     </row>
     <row r="92" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="14" t="s">
-        <v>529</v>
+        <v>350</v>
       </c>
       <c r="B92" s="14" t="s">
-        <v>174</v>
+        <v>107</v>
       </c>
       <c r="C92" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D92" s="18" t="s">
-        <v>530</v>
-      </c>
-      <c r="E92" s="15"/>
+      <c r="D92" s="18"/>
+      <c r="E92" s="14"/>
       <c r="F92" s="14"/>
       <c r="G92" s="14"/>
       <c r="H92" s="14"/>
@@ -6961,10 +6981,18 @@
       <c r="AI92" s="14"/>
     </row>
     <row r="93" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="14"/>
-      <c r="B93" s="14"/>
-      <c r="C93" s="14"/>
-      <c r="D93" s="18"/>
+      <c r="A93" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="B93" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C93" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D93" s="18" t="s">
+        <v>530</v>
+      </c>
       <c r="E93" s="15"/>
       <c r="F93" s="14"/>
       <c r="G93" s="14"/>
@@ -6998,18 +7026,10 @@
       <c r="AI93" s="14"/>
     </row>
     <row r="94" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="14" t="s">
-        <v>617</v>
-      </c>
-      <c r="B94" s="14" t="s">
-        <v>613</v>
-      </c>
-      <c r="C94" s="14" t="s">
-        <v>614</v>
-      </c>
-      <c r="D94" s="18" t="s">
-        <v>615</v>
-      </c>
+      <c r="A94" s="14"/>
+      <c r="B94" s="14"/>
+      <c r="C94" s="14"/>
+      <c r="D94" s="18"/>
       <c r="E94" s="15"/>
       <c r="F94" s="14"/>
       <c r="G94" s="14"/>
@@ -7036,20 +7056,26 @@
       <c r="AB94" s="14"/>
       <c r="AC94" s="14"/>
       <c r="AD94" s="14"/>
-      <c r="AE94" s="27" t="s">
-        <v>654</v>
-      </c>
+      <c r="AE94" s="27"/>
       <c r="AF94" s="14"/>
       <c r="AG94" s="14"/>
       <c r="AH94" s="14"/>
       <c r="AI94" s="14"/>
     </row>
     <row r="95" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="14"/>
-      <c r="B95" s="14"/>
-      <c r="C95" s="14"/>
-      <c r="D95" s="18"/>
-      <c r="E95" s="14"/>
+      <c r="A95" s="14" t="s">
+        <v>617</v>
+      </c>
+      <c r="B95" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C95" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D95" s="18" t="s">
+        <v>615</v>
+      </c>
+      <c r="E95" s="15"/>
       <c r="F95" s="14"/>
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
@@ -7075,37 +7101,27 @@
       <c r="AB95" s="14"/>
       <c r="AC95" s="14"/>
       <c r="AD95" s="14"/>
-      <c r="AE95" s="27"/>
+      <c r="AE95" s="27" t="s">
+        <v>654</v>
+      </c>
       <c r="AF95" s="14"/>
       <c r="AG95" s="14"/>
       <c r="AH95" s="14"/>
       <c r="AI95" s="14"/>
     </row>
     <row r="96" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="12" t="s">
-        <v>365</v>
-      </c>
-      <c r="B96" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C96" s="12" t="s">
-        <v>135</v>
-      </c>
+      <c r="A96" s="14"/>
+      <c r="B96" s="14"/>
+      <c r="C96" s="14"/>
       <c r="D96" s="18"/>
       <c r="E96" s="14"/>
       <c r="F96" s="14"/>
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="14"/>
-      <c r="J96" s="13" t="s">
-        <v>405</v>
-      </c>
-      <c r="K96" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L96" s="14" t="s">
-        <v>406</v>
-      </c>
+      <c r="J96" s="14"/>
+      <c r="K96" s="14"/>
+      <c r="L96" s="14"/>
       <c r="M96" s="14"/>
       <c r="N96" s="14"/>
       <c r="O96" s="14"/>
@@ -7132,7 +7148,7 @@
     </row>
     <row r="97" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B97" s="12" t="s">
         <v>107</v>
@@ -7146,15 +7162,19 @@
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="14"/>
-      <c r="J97" s="14"/>
-      <c r="K97" s="14"/>
-      <c r="L97" s="12"/>
-      <c r="M97" s="12" t="s">
-        <v>398</v>
-      </c>
-      <c r="N97" s="12"/>
-      <c r="O97" s="12"/>
-      <c r="P97" s="12"/>
+      <c r="J97" s="13" t="s">
+        <v>405</v>
+      </c>
+      <c r="K97" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L97" s="14" t="s">
+        <v>406</v>
+      </c>
+      <c r="M97" s="14"/>
+      <c r="N97" s="14"/>
+      <c r="O97" s="14"/>
+      <c r="P97" s="14"/>
       <c r="Q97" s="14"/>
       <c r="R97" s="14"/>
       <c r="S97" s="14"/>
@@ -7177,7 +7197,7 @@
     </row>
     <row r="98" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="12" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B98" s="12" t="s">
         <v>107</v>
@@ -7194,10 +7214,10 @@
       <c r="J98" s="14"/>
       <c r="K98" s="14"/>
       <c r="L98" s="12"/>
-      <c r="M98" s="12"/>
-      <c r="N98" s="12" t="s">
-        <v>410</v>
-      </c>
+      <c r="M98" s="12" t="s">
+        <v>398</v>
+      </c>
+      <c r="N98" s="12"/>
       <c r="O98" s="12"/>
       <c r="P98" s="12"/>
       <c r="Q98" s="14"/>
@@ -7222,7 +7242,7 @@
     </row>
     <row r="99" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="12" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B99" s="12" t="s">
         <v>107</v>
@@ -7240,10 +7260,10 @@
       <c r="K99" s="14"/>
       <c r="L99" s="12"/>
       <c r="M99" s="12"/>
-      <c r="N99" s="12"/>
-      <c r="O99" s="12" t="s">
-        <v>407</v>
-      </c>
+      <c r="N99" s="12" t="s">
+        <v>410</v>
+      </c>
+      <c r="O99" s="12"/>
       <c r="P99" s="12"/>
       <c r="Q99" s="14"/>
       <c r="R99" s="14"/>
@@ -7267,7 +7287,7 @@
     </row>
     <row r="100" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="12" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B100" s="12" t="s">
         <v>107</v>
@@ -7286,10 +7306,10 @@
       <c r="L100" s="12"/>
       <c r="M100" s="12"/>
       <c r="N100" s="12"/>
-      <c r="O100" s="12"/>
-      <c r="P100" s="13" t="s">
-        <v>408</v>
-      </c>
+      <c r="O100" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="P100" s="12"/>
       <c r="Q100" s="14"/>
       <c r="R100" s="14"/>
       <c r="S100" s="14"/>
@@ -7311,10 +7331,16 @@
       <c r="AI100" s="14"/>
     </row>
     <row r="101" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="14"/>
-      <c r="B101" s="14"/>
-      <c r="C101" s="14"/>
-      <c r="D101" s="23"/>
+      <c r="A101" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="B101" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C101" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D101" s="18"/>
       <c r="E101" s="14"/>
       <c r="F101" s="14"/>
       <c r="G101" s="14"/>
@@ -7322,11 +7348,13 @@
       <c r="I101" s="14"/>
       <c r="J101" s="14"/>
       <c r="K101" s="14"/>
-      <c r="L101" s="14"/>
-      <c r="M101" s="14"/>
-      <c r="N101" s="14"/>
-      <c r="O101" s="14"/>
-      <c r="P101" s="14"/>
+      <c r="L101" s="12"/>
+      <c r="M101" s="12"/>
+      <c r="N101" s="12"/>
+      <c r="O101" s="12"/>
+      <c r="P101" s="13" t="s">
+        <v>408</v>
+      </c>
       <c r="Q101" s="14"/>
       <c r="R101" s="14"/>
       <c r="S101" s="14"/>
@@ -7347,66 +7375,46 @@
       <c r="AH101" s="14"/>
       <c r="AI101" s="14"/>
     </row>
-    <row r="102" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="12" t="s">
-        <v>306</v>
-      </c>
-      <c r="B102" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C102" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="D102" s="12"/>
-      <c r="E102" s="12"/>
-      <c r="F102" s="12"/>
-      <c r="G102" s="12"/>
-      <c r="H102" s="12"/>
-      <c r="I102" s="12"/>
-      <c r="J102" s="12"/>
-      <c r="K102" s="12"/>
-      <c r="L102" s="12"/>
-      <c r="M102" s="12"/>
-      <c r="N102" s="12"/>
-      <c r="O102" s="12"/>
-      <c r="P102" s="12"/>
-      <c r="Q102" s="12"/>
-      <c r="R102" s="12"/>
-      <c r="S102" s="12"/>
-      <c r="T102" s="12"/>
-      <c r="U102" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="V102" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="W102" s="12" t="s">
-        <v>309</v>
-      </c>
-      <c r="X102" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="Y102" s="12" t="s">
-        <v>311</v>
-      </c>
-      <c r="Z102" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="AA102" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="AB102" s="12"/>
-      <c r="AC102" s="12"/>
-      <c r="AD102" s="12"/>
-      <c r="AE102" s="28"/>
-      <c r="AF102" s="12"/>
-      <c r="AG102" s="12"/>
-      <c r="AH102" s="12"/>
-      <c r="AI102" s="12"/>
+    <row r="102" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="14"/>
+      <c r="B102" s="14"/>
+      <c r="C102" s="14"/>
+      <c r="D102" s="23"/>
+      <c r="E102" s="14"/>
+      <c r="F102" s="14"/>
+      <c r="G102" s="14"/>
+      <c r="H102" s="14"/>
+      <c r="I102" s="14"/>
+      <c r="J102" s="14"/>
+      <c r="K102" s="14"/>
+      <c r="L102" s="14"/>
+      <c r="M102" s="14"/>
+      <c r="N102" s="14"/>
+      <c r="O102" s="14"/>
+      <c r="P102" s="14"/>
+      <c r="Q102" s="14"/>
+      <c r="R102" s="14"/>
+      <c r="S102" s="14"/>
+      <c r="T102" s="14"/>
+      <c r="U102" s="14"/>
+      <c r="V102" s="14"/>
+      <c r="W102" s="14"/>
+      <c r="X102" s="14"/>
+      <c r="Y102" s="14"/>
+      <c r="Z102" s="14"/>
+      <c r="AA102" s="14"/>
+      <c r="AB102" s="14"/>
+      <c r="AC102" s="14"/>
+      <c r="AD102" s="14"/>
+      <c r="AE102" s="27"/>
+      <c r="AF102" s="14"/>
+      <c r="AG102" s="14"/>
+      <c r="AH102" s="14"/>
+      <c r="AI102" s="14"/>
     </row>
     <row r="103" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="12" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="B103" s="12" t="s">
         <v>107</v>
@@ -7463,7 +7471,7 @@
     </row>
     <row r="104" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="12" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B104" s="12" t="s">
         <v>107</v>
@@ -7488,22 +7496,24 @@
       <c r="R104" s="12"/>
       <c r="S104" s="12"/>
       <c r="T104" s="12"/>
-      <c r="U104" s="12" t="s">
+      <c r="U104" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="V104" s="12" t="s">
-        <v>314</v>
+      <c r="V104" s="13" t="s">
+        <v>308</v>
       </c>
       <c r="W104" s="12" t="s">
         <v>309</v>
       </c>
       <c r="X104" s="12" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="Y104" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="Z104" s="12"/>
+      <c r="Z104" s="12" t="s">
+        <v>107</v>
+      </c>
       <c r="AA104" s="12" t="s">
         <v>135</v>
       </c>
@@ -7518,7 +7528,7 @@
     </row>
     <row r="105" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="12" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B105" s="12" t="s">
         <v>107</v>
@@ -7543,25 +7553,25 @@
       <c r="R105" s="12"/>
       <c r="S105" s="12"/>
       <c r="T105" s="12"/>
-      <c r="U105" s="13" t="s">
+      <c r="U105" s="12" t="s">
         <v>307</v>
       </c>
-      <c r="V105" s="13" t="s">
-        <v>317</v>
+      <c r="V105" s="12" t="s">
+        <v>314</v>
       </c>
       <c r="W105" s="12" t="s">
         <v>309</v>
       </c>
       <c r="X105" s="12" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="Y105" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="Z105" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="AA105" s="12"/>
+      <c r="Z105" s="12"/>
+      <c r="AA105" s="12" t="s">
+        <v>135</v>
+      </c>
       <c r="AB105" s="12"/>
       <c r="AC105" s="12"/>
       <c r="AD105" s="12"/>
@@ -7573,7 +7583,7 @@
     </row>
     <row r="106" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="12" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B106" s="12" t="s">
         <v>107</v>
@@ -7598,25 +7608,25 @@
       <c r="R106" s="12"/>
       <c r="S106" s="12"/>
       <c r="T106" s="12"/>
-      <c r="U106" s="12" t="s">
+      <c r="U106" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="V106" s="12" t="s">
-        <v>319</v>
+      <c r="V106" s="13" t="s">
+        <v>317</v>
       </c>
       <c r="W106" s="12" t="s">
         <v>309</v>
       </c>
-      <c r="X106" s="12"/>
+      <c r="X106" s="12" t="s">
+        <v>310</v>
+      </c>
       <c r="Y106" s="12" t="s">
         <v>311</v>
       </c>
       <c r="Z106" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="AA106" s="12" t="s">
-        <v>135</v>
-      </c>
+      <c r="AA106" s="12"/>
       <c r="AB106" s="12"/>
       <c r="AC106" s="12"/>
       <c r="AD106" s="12"/>
@@ -7628,7 +7638,7 @@
     </row>
     <row r="107" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="12" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B107" s="12" t="s">
         <v>107</v>
@@ -7653,16 +7663,16 @@
       <c r="R107" s="12"/>
       <c r="S107" s="12"/>
       <c r="T107" s="12"/>
-      <c r="U107" s="12"/>
+      <c r="U107" s="12" t="s">
+        <v>307</v>
+      </c>
       <c r="V107" s="12" t="s">
         <v>319</v>
       </c>
       <c r="W107" s="12" t="s">
         <v>309</v>
       </c>
-      <c r="X107" s="12" t="s">
-        <v>315</v>
-      </c>
+      <c r="X107" s="12"/>
       <c r="Y107" s="12" t="s">
         <v>311</v>
       </c>
@@ -7683,7 +7693,7 @@
     </row>
     <row r="108" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="12" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B108" s="12" t="s">
         <v>107</v>
@@ -7708,17 +7718,15 @@
       <c r="R108" s="12"/>
       <c r="S108" s="12"/>
       <c r="T108" s="12"/>
-      <c r="U108" s="13" t="s">
-        <v>322</v>
-      </c>
-      <c r="V108" s="13" t="s">
-        <v>323</v>
-      </c>
-      <c r="W108" s="13" t="s">
+      <c r="U108" s="12"/>
+      <c r="V108" s="12" t="s">
+        <v>319</v>
+      </c>
+      <c r="W108" s="12" t="s">
         <v>309</v>
       </c>
       <c r="X108" s="12" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="Y108" s="12" t="s">
         <v>311</v>
@@ -7740,7 +7748,7 @@
     </row>
     <row r="109" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="12" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="B109" s="12" t="s">
         <v>107</v>
@@ -7766,13 +7774,13 @@
       <c r="S109" s="12"/>
       <c r="T109" s="12"/>
       <c r="U109" s="13" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
       <c r="V109" s="13" t="s">
-        <v>308</v>
+        <v>323</v>
       </c>
       <c r="W109" s="13" t="s">
-        <v>325</v>
+        <v>309</v>
       </c>
       <c r="X109" s="12" t="s">
         <v>310</v>
@@ -7797,7 +7805,7 @@
     </row>
     <row r="110" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="12" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B110" s="12" t="s">
         <v>107</v>
@@ -7822,26 +7830,26 @@
       <c r="R110" s="12"/>
       <c r="S110" s="12"/>
       <c r="T110" s="12"/>
-      <c r="U110" s="12" t="s">
+      <c r="U110" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="V110" s="12" t="s">
+      <c r="V110" s="13" t="s">
         <v>308</v>
       </c>
-      <c r="W110" s="12" t="s">
-        <v>309</v>
+      <c r="W110" s="13" t="s">
+        <v>325</v>
       </c>
       <c r="X110" s="12" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="Y110" s="12" t="s">
         <v>311</v>
       </c>
       <c r="Z110" s="12" t="s">
-        <v>174</v>
+        <v>107</v>
       </c>
       <c r="AA110" s="12" t="s">
-        <v>327</v>
+        <v>135</v>
       </c>
       <c r="AB110" s="12"/>
       <c r="AC110" s="12"/>
@@ -7854,7 +7862,7 @@
     </row>
     <row r="111" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="12" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B111" s="12" t="s">
         <v>107</v>
@@ -7882,8 +7890,8 @@
       <c r="U111" s="12" t="s">
         <v>307</v>
       </c>
-      <c r="V111" s="13" t="s">
-        <v>329</v>
+      <c r="V111" s="12" t="s">
+        <v>308</v>
       </c>
       <c r="W111" s="12" t="s">
         <v>309</v>
@@ -7895,10 +7903,10 @@
         <v>311</v>
       </c>
       <c r="Z111" s="12" t="s">
-        <v>107</v>
+        <v>174</v>
       </c>
       <c r="AA111" s="12" t="s">
-        <v>135</v>
+        <v>327</v>
       </c>
       <c r="AB111" s="12"/>
       <c r="AC111" s="12"/>
@@ -7911,7 +7919,7 @@
     </row>
     <row r="112" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="12" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B112" s="12" t="s">
         <v>107</v>
@@ -7939,8 +7947,8 @@
       <c r="U112" s="12" t="s">
         <v>307</v>
       </c>
-      <c r="V112" s="12" t="s">
-        <v>331</v>
+      <c r="V112" s="13" t="s">
+        <v>329</v>
       </c>
       <c r="W112" s="12" t="s">
         <v>309</v>
@@ -7968,7 +7976,7 @@
     </row>
     <row r="113" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="12" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B113" s="12" t="s">
         <v>107</v>
@@ -7997,7 +8005,7 @@
         <v>307</v>
       </c>
       <c r="V113" s="12" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="W113" s="12" t="s">
         <v>309</v>
@@ -8009,7 +8017,7 @@
         <v>311</v>
       </c>
       <c r="Z113" s="12" t="s">
-        <v>327</v>
+        <v>107</v>
       </c>
       <c r="AA113" s="12" t="s">
         <v>135</v>
@@ -8025,7 +8033,7 @@
     </row>
     <row r="114" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="12" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B114" s="12" t="s">
         <v>107</v>
@@ -8060,13 +8068,13 @@
         <v>309</v>
       </c>
       <c r="X114" s="12" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="Y114" s="12" t="s">
         <v>311</v>
       </c>
       <c r="Z114" s="12" t="s">
-        <v>107</v>
+        <v>327</v>
       </c>
       <c r="AA114" s="12" t="s">
         <v>135</v>
@@ -8081,9 +8089,15 @@
       <c r="AI114" s="12"/>
     </row>
     <row r="115" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="12"/>
-      <c r="B115" s="12"/>
-      <c r="C115" s="12"/>
+      <c r="A115" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="B115" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C115" s="12" t="s">
+        <v>135</v>
+      </c>
       <c r="D115" s="12"/>
       <c r="E115" s="12"/>
       <c r="F115" s="12"/>
@@ -8101,13 +8115,27 @@
       <c r="R115" s="12"/>
       <c r="S115" s="12"/>
       <c r="T115" s="12"/>
-      <c r="U115" s="12"/>
-      <c r="V115" s="12"/>
-      <c r="W115" s="12"/>
-      <c r="X115" s="12"/>
-      <c r="Y115" s="12"/>
-      <c r="Z115" s="12"/>
-      <c r="AA115" s="12"/>
+      <c r="U115" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="V115" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="W115" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="X115" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="Y115" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="Z115" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="AA115" s="12" t="s">
+        <v>135</v>
+      </c>
       <c r="AB115" s="12"/>
       <c r="AC115" s="12"/>
       <c r="AD115" s="12"/>
@@ -8154,37 +8182,46 @@
       <c r="AH116" s="12"/>
       <c r="AI116" s="12"/>
     </row>
-    <row r="117" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A117" s="14" t="s">
-        <v>243</v>
-      </c>
-      <c r="B117" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C117" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D117" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="F117" s="14" t="s">
-        <v>403</v>
-      </c>
-      <c r="R117" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB117" s="14"/>
-      <c r="AC117" s="14"/>
-      <c r="AD117" s="14"/>
-      <c r="AE117" s="27"/>
-      <c r="AF117" s="14"/>
-      <c r="AG117" s="14"/>
-      <c r="AH117" s="14"/>
-      <c r="AI117" s="14"/>
+    <row r="117" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="12"/>
+      <c r="B117" s="12"/>
+      <c r="C117" s="12"/>
+      <c r="D117" s="12"/>
+      <c r="E117" s="12"/>
+      <c r="F117" s="12"/>
+      <c r="G117" s="12"/>
+      <c r="H117" s="12"/>
+      <c r="I117" s="12"/>
+      <c r="J117" s="12"/>
+      <c r="K117" s="12"/>
+      <c r="L117" s="12"/>
+      <c r="M117" s="12"/>
+      <c r="N117" s="12"/>
+      <c r="O117" s="12"/>
+      <c r="P117" s="12"/>
+      <c r="Q117" s="12"/>
+      <c r="R117" s="12"/>
+      <c r="S117" s="12"/>
+      <c r="T117" s="12"/>
+      <c r="U117" s="12"/>
+      <c r="V117" s="12"/>
+      <c r="W117" s="12"/>
+      <c r="X117" s="12"/>
+      <c r="Y117" s="12"/>
+      <c r="Z117" s="12"/>
+      <c r="AA117" s="12"/>
+      <c r="AB117" s="12"/>
+      <c r="AC117" s="12"/>
+      <c r="AD117" s="12"/>
+      <c r="AE117" s="28"/>
+      <c r="AF117" s="12"/>
+      <c r="AG117" s="12"/>
+      <c r="AH117" s="12"/>
+      <c r="AI117" s="12"/>
     </row>
     <row r="118" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A118" s="14" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B118" s="14" t="s">
         <v>174</v>
@@ -8193,7 +8230,7 @@
         <v>135</v>
       </c>
       <c r="D118" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F118" s="14" t="s">
         <v>403</v>
@@ -8212,7 +8249,7 @@
     </row>
     <row r="119" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A119" s="14" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B119" s="14" t="s">
         <v>174</v>
@@ -8221,7 +8258,7 @@
         <v>135</v>
       </c>
       <c r="D119" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F119" s="14" t="s">
         <v>403</v>
@@ -8240,7 +8277,7 @@
     </row>
     <row r="120" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A120" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B120" s="14" t="s">
         <v>174</v>
@@ -8249,7 +8286,7 @@
         <v>135</v>
       </c>
       <c r="D120" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F120" s="14" t="s">
         <v>403</v>
@@ -8268,7 +8305,7 @@
     </row>
     <row r="121" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A121" s="14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B121" s="14" t="s">
         <v>174</v>
@@ -8277,7 +8314,7 @@
         <v>135</v>
       </c>
       <c r="D121" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F121" s="14" t="s">
         <v>403</v>
@@ -8296,7 +8333,7 @@
     </row>
     <row r="122" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A122" s="14" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B122" s="14" t="s">
         <v>174</v>
@@ -8305,7 +8342,7 @@
         <v>135</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="F122" s="14" t="s">
         <v>403</v>
@@ -8324,7 +8361,7 @@
     </row>
     <row r="123" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A123" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B123" s="14" t="s">
         <v>174</v>
@@ -8339,7 +8376,7 @@
         <v>403</v>
       </c>
       <c r="R123" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AB123" s="14"/>
       <c r="AC123" s="14"/>
@@ -8350,9 +8387,9 @@
       <c r="AH123" s="14"/>
       <c r="AI123" s="14"/>
     </row>
-    <row r="124" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A124" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B124" s="14" t="s">
         <v>174</v>
@@ -8361,33 +8398,14 @@
         <v>135</v>
       </c>
       <c r="D124" s="15" t="s">
-        <v>236</v>
-      </c>
-      <c r="E124" s="14"/>
+        <v>185</v>
+      </c>
       <c r="F124" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G124" s="14"/>
-      <c r="H124" s="14"/>
-      <c r="I124" s="14"/>
-      <c r="J124" s="14"/>
-      <c r="K124" s="14"/>
-      <c r="L124" s="14"/>
-      <c r="M124" s="14"/>
-      <c r="N124" s="14"/>
-      <c r="O124" s="14"/>
-      <c r="P124" s="14"/>
-      <c r="Q124" s="14"/>
-      <c r="R124" s="15"/>
-      <c r="S124" s="14"/>
-      <c r="T124" s="14"/>
-      <c r="U124" s="14"/>
-      <c r="V124" s="14"/>
-      <c r="W124" s="14"/>
-      <c r="X124" s="14"/>
-      <c r="Y124" s="14"/>
-      <c r="Z124" s="14"/>
-      <c r="AA124" s="14"/>
+      <c r="R124" s="15" t="s">
+        <v>2</v>
+      </c>
       <c r="AB124" s="14"/>
       <c r="AC124" s="14"/>
       <c r="AD124" s="14"/>
@@ -8399,7 +8417,7 @@
     </row>
     <row r="125" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B125" s="14" t="s">
         <v>174</v>
@@ -8408,7 +8426,7 @@
         <v>135</v>
       </c>
       <c r="D125" s="15" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E125" s="14"/>
       <c r="F125" s="14" t="s">
@@ -8444,9 +8462,9 @@
       <c r="AH125" s="14"/>
       <c r="AI125" s="14"/>
     </row>
-    <row r="126" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B126" s="14" t="s">
         <v>174</v>
@@ -8455,12 +8473,33 @@
         <v>135</v>
       </c>
       <c r="D126" s="15" t="s">
-        <v>238</v>
-      </c>
+        <v>237</v>
+      </c>
+      <c r="E126" s="14"/>
       <c r="F126" s="14" t="s">
         <v>403</v>
       </c>
+      <c r="G126" s="14"/>
+      <c r="H126" s="14"/>
+      <c r="I126" s="14"/>
+      <c r="J126" s="14"/>
+      <c r="K126" s="14"/>
+      <c r="L126" s="14"/>
+      <c r="M126" s="14"/>
+      <c r="N126" s="14"/>
+      <c r="O126" s="14"/>
+      <c r="P126" s="14"/>
+      <c r="Q126" s="14"/>
       <c r="R126" s="15"/>
+      <c r="S126" s="14"/>
+      <c r="T126" s="14"/>
+      <c r="U126" s="14"/>
+      <c r="V126" s="14"/>
+      <c r="W126" s="14"/>
+      <c r="X126" s="14"/>
+      <c r="Y126" s="14"/>
+      <c r="Z126" s="14"/>
+      <c r="AA126" s="14"/>
       <c r="AB126" s="14"/>
       <c r="AC126" s="14"/>
       <c r="AD126" s="14"/>
@@ -8472,7 +8511,7 @@
     </row>
     <row r="127" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A127" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B127" s="14" t="s">
         <v>174</v>
@@ -8481,7 +8520,7 @@
         <v>135</v>
       </c>
       <c r="D127" s="15" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F127" s="14" t="s">
         <v>403</v>
@@ -8498,7 +8537,7 @@
     </row>
     <row r="128" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A128" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B128" s="14" t="s">
         <v>174</v>
@@ -8507,7 +8546,7 @@
         <v>135</v>
       </c>
       <c r="D128" s="15" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F128" s="14" t="s">
         <v>403</v>
@@ -8524,7 +8563,7 @@
     </row>
     <row r="129" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A129" s="14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B129" s="14" t="s">
         <v>174</v>
@@ -8532,15 +8571,13 @@
       <c r="C129" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D129" s="16" t="s">
-        <v>257</v>
+      <c r="D129" s="15" t="s">
+        <v>240</v>
       </c>
       <c r="F129" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="R129" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R129" s="15"/>
       <c r="AB129" s="14"/>
       <c r="AC129" s="14"/>
       <c r="AD129" s="14"/>
@@ -8552,7 +8589,7 @@
     </row>
     <row r="130" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A130" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B130" s="14" t="s">
         <v>174</v>
@@ -8560,8 +8597,8 @@
       <c r="C130" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D130" s="15" t="s">
-        <v>277</v>
+      <c r="D130" s="16" t="s">
+        <v>257</v>
       </c>
       <c r="F130" s="14" t="s">
         <v>403</v>
@@ -8578,9 +8615,9 @@
       <c r="AH130" s="14"/>
       <c r="AI130" s="14"/>
     </row>
-    <row r="131" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A131" s="14" t="s">
-        <v>278</v>
+        <v>256</v>
       </c>
       <c r="B131" s="14" t="s">
         <v>174</v>
@@ -8589,35 +8626,14 @@
         <v>135</v>
       </c>
       <c r="D131" s="15" t="s">
-        <v>279</v>
-      </c>
-      <c r="E131" s="14"/>
+        <v>277</v>
+      </c>
       <c r="F131" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G131" s="14"/>
-      <c r="H131" s="14"/>
-      <c r="I131" s="14"/>
-      <c r="J131" s="14"/>
-      <c r="K131" s="14"/>
-      <c r="L131" s="14"/>
-      <c r="M131" s="14"/>
-      <c r="N131" s="14"/>
-      <c r="O131" s="14"/>
-      <c r="P131" s="14"/>
-      <c r="Q131" s="14"/>
       <c r="R131" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="S131" s="14"/>
-      <c r="T131" s="14"/>
-      <c r="U131" s="14"/>
-      <c r="V131" s="14"/>
-      <c r="W131" s="14"/>
-      <c r="X131" s="14"/>
-      <c r="Y131" s="14"/>
-      <c r="Z131" s="14"/>
-      <c r="AA131" s="14"/>
       <c r="AB131" s="14"/>
       <c r="AC131" s="14"/>
       <c r="AD131" s="14"/>
@@ -8629,7 +8645,7 @@
     </row>
     <row r="132" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="14" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="B132" s="14" t="s">
         <v>174</v>
@@ -8638,7 +8654,7 @@
         <v>135</v>
       </c>
       <c r="D132" s="15" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="E132" s="14"/>
       <c r="F132" s="14" t="s">
@@ -8656,7 +8672,7 @@
       <c r="P132" s="14"/>
       <c r="Q132" s="14"/>
       <c r="R132" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S132" s="14"/>
       <c r="T132" s="14"/>
@@ -8678,7 +8694,7 @@
     </row>
     <row r="133" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="14" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B133" s="14" t="s">
         <v>174</v>
@@ -8687,7 +8703,7 @@
         <v>135</v>
       </c>
       <c r="D133" s="15" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E133" s="14"/>
       <c r="F133" s="14" t="s">
@@ -8705,7 +8721,7 @@
       <c r="P133" s="14"/>
       <c r="Q133" s="14"/>
       <c r="R133" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S133" s="14"/>
       <c r="T133" s="14"/>
@@ -8727,7 +8743,7 @@
     </row>
     <row r="134" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="14" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B134" s="14" t="s">
         <v>174</v>
@@ -8736,7 +8752,7 @@
         <v>135</v>
       </c>
       <c r="D134" s="15" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="E134" s="14"/>
       <c r="F134" s="14" t="s">
@@ -8776,7 +8792,7 @@
     </row>
     <row r="135" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="14" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B135" s="14" t="s">
         <v>174</v>
@@ -8785,7 +8801,7 @@
         <v>135</v>
       </c>
       <c r="D135" s="15" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="E135" s="14"/>
       <c r="F135" s="14" t="s">
@@ -8803,7 +8819,7 @@
       <c r="P135" s="14"/>
       <c r="Q135" s="14"/>
       <c r="R135" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S135" s="14"/>
       <c r="T135" s="14"/>
@@ -8825,7 +8841,7 @@
     </row>
     <row r="136" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="14" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B136" s="14" t="s">
         <v>174</v>
@@ -8834,7 +8850,7 @@
         <v>135</v>
       </c>
       <c r="D136" s="15" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E136" s="14"/>
       <c r="F136" s="14" t="s">
@@ -8852,7 +8868,7 @@
       <c r="P136" s="14"/>
       <c r="Q136" s="14"/>
       <c r="R136" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S136" s="14"/>
       <c r="T136" s="14"/>
@@ -8874,7 +8890,7 @@
     </row>
     <row r="137" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="14" t="s">
-        <v>373</v>
+        <v>294</v>
       </c>
       <c r="B137" s="14" t="s">
         <v>174</v>
@@ -8883,7 +8899,7 @@
         <v>135</v>
       </c>
       <c r="D137" s="15" t="s">
-        <v>372</v>
+        <v>295</v>
       </c>
       <c r="E137" s="14"/>
       <c r="F137" s="14" t="s">
@@ -8891,9 +8907,7 @@
       </c>
       <c r="G137" s="14"/>
       <c r="H137" s="14"/>
-      <c r="I137" s="14" t="s">
-        <v>126</v>
-      </c>
+      <c r="I137" s="14"/>
       <c r="J137" s="14"/>
       <c r="K137" s="14"/>
       <c r="L137" s="14"/>
@@ -8902,7 +8916,9 @@
       <c r="O137" s="14"/>
       <c r="P137" s="14"/>
       <c r="Q137" s="14"/>
-      <c r="R137" s="15"/>
+      <c r="R137" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S137" s="14"/>
       <c r="T137" s="14"/>
       <c r="U137" s="14"/>
@@ -8923,7 +8939,7 @@
     </row>
     <row r="138" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="14" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B138" s="14" t="s">
         <v>174</v>
@@ -8932,7 +8948,7 @@
         <v>135</v>
       </c>
       <c r="D138" s="15" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="E138" s="14"/>
       <c r="F138" s="14" t="s">
@@ -8941,7 +8957,7 @@
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
       <c r="I138" s="14" t="s">
-        <v>379</v>
+        <v>126</v>
       </c>
       <c r="J138" s="14"/>
       <c r="K138" s="14"/>
@@ -8972,7 +8988,7 @@
     </row>
     <row r="139" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="14" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="B139" s="14" t="s">
         <v>174</v>
@@ -8981,7 +8997,7 @@
         <v>135</v>
       </c>
       <c r="D139" s="15" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="E139" s="14"/>
       <c r="F139" s="14" t="s">
@@ -8990,7 +9006,7 @@
       <c r="G139" s="14"/>
       <c r="H139" s="14"/>
       <c r="I139" s="14" t="s">
-        <v>125</v>
+        <v>379</v>
       </c>
       <c r="J139" s="14"/>
       <c r="K139" s="14"/>
@@ -9021,7 +9037,7 @@
     </row>
     <row r="140" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="14" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B140" s="14" t="s">
         <v>174</v>
@@ -9030,7 +9046,7 @@
         <v>135</v>
       </c>
       <c r="D140" s="15" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E140" s="14"/>
       <c r="F140" s="14" t="s">
@@ -9039,7 +9055,7 @@
       <c r="G140" s="14"/>
       <c r="H140" s="14"/>
       <c r="I140" s="14" t="s">
-        <v>381</v>
+        <v>125</v>
       </c>
       <c r="J140" s="14"/>
       <c r="K140" s="14"/>
@@ -9070,7 +9086,7 @@
     </row>
     <row r="141" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="14" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="B141" s="14" t="s">
         <v>174</v>
@@ -9079,7 +9095,7 @@
         <v>135</v>
       </c>
       <c r="D141" s="15" t="s">
-        <v>179</v>
+        <v>385</v>
       </c>
       <c r="E141" s="14"/>
       <c r="F141" s="14" t="s">
@@ -9087,7 +9103,9 @@
       </c>
       <c r="G141" s="14"/>
       <c r="H141" s="14"/>
-      <c r="I141" s="14"/>
+      <c r="I141" s="14" t="s">
+        <v>381</v>
+      </c>
       <c r="J141" s="14"/>
       <c r="K141" s="14"/>
       <c r="L141" s="14"/>
@@ -9117,7 +9135,7 @@
     </row>
     <row r="142" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="14" t="s">
-        <v>500</v>
+        <v>390</v>
       </c>
       <c r="B142" s="14" t="s">
         <v>174</v>
@@ -9125,18 +9143,16 @@
       <c r="C142" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D142" s="18" t="s">
-        <v>501</v>
-      </c>
-      <c r="E142" s="15"/>
+      <c r="D142" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="E142" s="14"/>
       <c r="F142" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
-      <c r="I142" s="14" t="s">
-        <v>128</v>
-      </c>
+      <c r="I142" s="14"/>
       <c r="J142" s="14"/>
       <c r="K142" s="14"/>
       <c r="L142" s="14"/>
@@ -9145,7 +9161,7 @@
       <c r="O142" s="14"/>
       <c r="P142" s="14"/>
       <c r="Q142" s="14"/>
-      <c r="R142" s="14"/>
+      <c r="R142" s="15"/>
       <c r="S142" s="14"/>
       <c r="T142" s="14"/>
       <c r="U142" s="14"/>
@@ -9158,17 +9174,15 @@
       <c r="AB142" s="14"/>
       <c r="AC142" s="14"/>
       <c r="AD142" s="14"/>
-      <c r="AE142" s="27" t="s">
-        <v>415</v>
-      </c>
+      <c r="AE142" s="27"/>
       <c r="AF142" s="14"/>
       <c r="AG142" s="14"/>
       <c r="AH142" s="14"/>
       <c r="AI142" s="14"/>
     </row>
     <row r="143" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="15" t="s">
-        <v>502</v>
+      <c r="A143" s="14" t="s">
+        <v>500</v>
       </c>
       <c r="B143" s="14" t="s">
         <v>174</v>
@@ -9177,16 +9191,16 @@
         <v>135</v>
       </c>
       <c r="D143" s="18" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="E143" s="15"/>
       <c r="F143" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G143" s="15"/>
+      <c r="G143" s="14"/>
       <c r="H143" s="14"/>
       <c r="I143" s="14" t="s">
-        <v>504</v>
+        <v>128</v>
       </c>
       <c r="J143" s="14"/>
       <c r="K143" s="14"/>
@@ -9209,7 +9223,9 @@
       <c r="AB143" s="14"/>
       <c r="AC143" s="14"/>
       <c r="AD143" s="14"/>
-      <c r="AE143" s="27"/>
+      <c r="AE143" s="27" t="s">
+        <v>415</v>
+      </c>
       <c r="AF143" s="14"/>
       <c r="AG143" s="14"/>
       <c r="AH143" s="14"/>
@@ -9217,7 +9233,7 @@
     </row>
     <row r="144" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="15" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="B144" s="14" t="s">
         <v>174</v>
@@ -9226,15 +9242,17 @@
         <v>135</v>
       </c>
       <c r="D144" s="18" t="s">
-        <v>506</v>
-      </c>
-      <c r="E144" s="14"/>
+        <v>503</v>
+      </c>
+      <c r="E144" s="15"/>
       <c r="F144" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G144" s="14"/>
+      <c r="G144" s="15"/>
       <c r="H144" s="14"/>
-      <c r="I144" s="14"/>
+      <c r="I144" s="14" t="s">
+        <v>504</v>
+      </c>
       <c r="J144" s="14"/>
       <c r="K144" s="14"/>
       <c r="L144" s="14"/>
@@ -9264,7 +9282,7 @@
     </row>
     <row r="145" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="15" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B145" s="14" t="s">
         <v>174</v>
@@ -9273,7 +9291,7 @@
         <v>135</v>
       </c>
       <c r="D145" s="18" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="E145" s="14"/>
       <c r="F145" s="14" t="s">
@@ -9311,7 +9329,7 @@
     </row>
     <row r="146" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="15" t="s">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="B146" s="14" t="s">
         <v>174</v>
@@ -9320,17 +9338,15 @@
         <v>135</v>
       </c>
       <c r="D146" s="18" t="s">
-        <v>513</v>
-      </c>
-      <c r="E146" s="15"/>
+        <v>508</v>
+      </c>
+      <c r="E146" s="14"/>
       <c r="F146" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G146" s="15"/>
+      <c r="G146" s="14"/>
       <c r="H146" s="14"/>
-      <c r="I146" s="14" t="s">
-        <v>378</v>
-      </c>
+      <c r="I146" s="14"/>
       <c r="J146" s="14"/>
       <c r="K146" s="14"/>
       <c r="L146" s="14"/>
@@ -9360,7 +9376,7 @@
     </row>
     <row r="147" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="15" t="s">
-        <v>519</v>
+        <v>512</v>
       </c>
       <c r="B147" s="14" t="s">
         <v>174</v>
@@ -9369,17 +9385,17 @@
         <v>135</v>
       </c>
       <c r="D147" s="18" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="E147" s="15"/>
-      <c r="F147" s="15" t="s">
-        <v>388</v>
-      </c>
-      <c r="G147" s="15" t="s">
-        <v>3</v>
-      </c>
+      <c r="F147" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="G147" s="15"/>
       <c r="H147" s="14"/>
-      <c r="I147" s="14"/>
+      <c r="I147" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J147" s="14"/>
       <c r="K147" s="14"/>
       <c r="L147" s="14"/>
@@ -9409,7 +9425,7 @@
     </row>
     <row r="148" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="15" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="B148" s="14" t="s">
         <v>174</v>
@@ -9418,17 +9434,17 @@
         <v>135</v>
       </c>
       <c r="D148" s="18" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="E148" s="15"/>
-      <c r="F148" s="14" t="s">
-        <v>403</v>
-      </c>
-      <c r="G148" s="14"/>
+      <c r="F148" s="15" t="s">
+        <v>388</v>
+      </c>
+      <c r="G148" s="15" t="s">
+        <v>3</v>
+      </c>
       <c r="H148" s="14"/>
-      <c r="I148" s="14" t="s">
-        <v>128</v>
-      </c>
+      <c r="I148" s="14"/>
       <c r="J148" s="14"/>
       <c r="K148" s="14"/>
       <c r="L148" s="14"/>
@@ -9450,9 +9466,7 @@
       <c r="AB148" s="14"/>
       <c r="AC148" s="14"/>
       <c r="AD148" s="14"/>
-      <c r="AE148" s="27" t="s">
-        <v>415</v>
-      </c>
+      <c r="AE148" s="27"/>
       <c r="AF148" s="14"/>
       <c r="AG148" s="14"/>
       <c r="AH148" s="14"/>
@@ -9460,7 +9474,7 @@
     </row>
     <row r="149" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="15" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="B149" s="14" t="s">
         <v>174</v>
@@ -9469,7 +9483,7 @@
         <v>135</v>
       </c>
       <c r="D149" s="18" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="E149" s="15"/>
       <c r="F149" s="14" t="s">
@@ -9478,7 +9492,7 @@
       <c r="G149" s="14"/>
       <c r="H149" s="14"/>
       <c r="I149" s="14" t="s">
-        <v>401</v>
+        <v>128</v>
       </c>
       <c r="J149" s="14"/>
       <c r="K149" s="14"/>
@@ -9501,7 +9515,9 @@
       <c r="AB149" s="14"/>
       <c r="AC149" s="14"/>
       <c r="AD149" s="14"/>
-      <c r="AE149" s="27"/>
+      <c r="AE149" s="27" t="s">
+        <v>415</v>
+      </c>
       <c r="AF149" s="14"/>
       <c r="AG149" s="14"/>
       <c r="AH149" s="14"/>
@@ -9509,7 +9525,7 @@
     </row>
     <row r="150" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="15" t="s">
-        <v>528</v>
+        <v>523</v>
       </c>
       <c r="B150" s="14" t="s">
         <v>174</v>
@@ -9518,7 +9534,7 @@
         <v>135</v>
       </c>
       <c r="D150" s="18" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E150" s="15"/>
       <c r="F150" s="14" t="s">
@@ -9527,7 +9543,7 @@
       <c r="G150" s="14"/>
       <c r="H150" s="14"/>
       <c r="I150" s="14" t="s">
-        <v>126</v>
+        <v>401</v>
       </c>
       <c r="J150" s="14"/>
       <c r="K150" s="14"/>
@@ -9557,8 +9573,8 @@
       <c r="AI150" s="14"/>
     </row>
     <row r="151" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="14" t="s">
-        <v>533</v>
+      <c r="A151" s="15" t="s">
+        <v>528</v>
       </c>
       <c r="B151" s="14" t="s">
         <v>174</v>
@@ -9566,16 +9582,18 @@
       <c r="C151" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D151" s="15" t="s">
-        <v>531</v>
-      </c>
-      <c r="E151" s="14"/>
+      <c r="D151" s="18" t="s">
+        <v>527</v>
+      </c>
+      <c r="E151" s="15"/>
       <c r="F151" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G151" s="14"/>
       <c r="H151" s="14"/>
-      <c r="I151" s="14"/>
+      <c r="I151" s="14" t="s">
+        <v>126</v>
+      </c>
       <c r="J151" s="14"/>
       <c r="K151" s="14"/>
       <c r="L151" s="14"/>
@@ -9584,9 +9602,7 @@
       <c r="O151" s="14"/>
       <c r="P151" s="14"/>
       <c r="Q151" s="14"/>
-      <c r="R151" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R151" s="14"/>
       <c r="S151" s="14"/>
       <c r="T151" s="14"/>
       <c r="U151" s="14"/>
@@ -9606,8 +9622,8 @@
       <c r="AI151" s="14"/>
     </row>
     <row r="152" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="15" t="s">
-        <v>534</v>
+      <c r="A152" s="14" t="s">
+        <v>533</v>
       </c>
       <c r="B152" s="14" t="s">
         <v>174</v>
@@ -9615,18 +9631,16 @@
       <c r="C152" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D152" s="18" t="s">
-        <v>535</v>
-      </c>
-      <c r="E152" s="15"/>
+      <c r="D152" s="15" t="s">
+        <v>531</v>
+      </c>
+      <c r="E152" s="14"/>
       <c r="F152" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G152" s="15"/>
+      <c r="G152" s="14"/>
       <c r="H152" s="14"/>
-      <c r="I152" s="14" t="s">
-        <v>378</v>
-      </c>
+      <c r="I152" s="14"/>
       <c r="J152" s="14"/>
       <c r="K152" s="14"/>
       <c r="L152" s="14"/>
@@ -9635,7 +9649,9 @@
       <c r="O152" s="14"/>
       <c r="P152" s="14"/>
       <c r="Q152" s="14"/>
-      <c r="R152" s="14"/>
+      <c r="R152" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S152" s="14"/>
       <c r="T152" s="14"/>
       <c r="U152" s="14"/>
@@ -9655,8 +9671,8 @@
       <c r="AI152" s="14"/>
     </row>
     <row r="153" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="14" t="s">
-        <v>581</v>
+      <c r="A153" s="15" t="s">
+        <v>534</v>
       </c>
       <c r="B153" s="14" t="s">
         <v>174</v>
@@ -9664,16 +9680,18 @@
       <c r="C153" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D153" s="15" t="s">
-        <v>582</v>
-      </c>
-      <c r="E153" s="14"/>
+      <c r="D153" s="18" t="s">
+        <v>535</v>
+      </c>
+      <c r="E153" s="15"/>
       <c r="F153" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G153" s="14"/>
+      <c r="G153" s="15"/>
       <c r="H153" s="14"/>
-      <c r="I153" s="14"/>
+      <c r="I153" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J153" s="14"/>
       <c r="K153" s="14"/>
       <c r="L153" s="14"/>
@@ -9682,9 +9700,7 @@
       <c r="O153" s="14"/>
       <c r="P153" s="14"/>
       <c r="Q153" s="14"/>
-      <c r="R153" s="15" t="s">
-        <v>0</v>
-      </c>
+      <c r="R153" s="14"/>
       <c r="S153" s="14"/>
       <c r="T153" s="14"/>
       <c r="U153" s="14"/>
@@ -9705,7 +9721,7 @@
     </row>
     <row r="154" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="14" t="s">
-        <v>602</v>
+        <v>581</v>
       </c>
       <c r="B154" s="14" t="s">
         <v>174</v>
@@ -9714,7 +9730,7 @@
         <v>135</v>
       </c>
       <c r="D154" s="15" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E154" s="14"/>
       <c r="F154" s="14" t="s">
@@ -9754,7 +9770,7 @@
     </row>
     <row r="155" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="14" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B155" s="14" t="s">
         <v>174</v>
@@ -9763,7 +9779,7 @@
         <v>135</v>
       </c>
       <c r="D155" s="15" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E155" s="14"/>
       <c r="F155" s="14" t="s">
@@ -9803,7 +9819,7 @@
     </row>
     <row r="156" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="14" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B156" s="14" t="s">
         <v>174</v>
@@ -9811,18 +9827,16 @@
       <c r="C156" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D156" s="18" t="s">
-        <v>587</v>
-      </c>
-      <c r="E156" s="15"/>
+      <c r="D156" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="E156" s="14"/>
       <c r="F156" s="14" t="s">
         <v>403</v>
       </c>
       <c r="G156" s="14"/>
       <c r="H156" s="14"/>
-      <c r="I156" s="14" t="s">
-        <v>128</v>
-      </c>
+      <c r="I156" s="14"/>
       <c r="J156" s="14"/>
       <c r="K156" s="14"/>
       <c r="L156" s="14"/>
@@ -9831,7 +9845,9 @@
       <c r="O156" s="14"/>
       <c r="P156" s="14"/>
       <c r="Q156" s="14"/>
-      <c r="R156" s="14"/>
+      <c r="R156" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="S156" s="14"/>
       <c r="T156" s="14"/>
       <c r="U156" s="14"/>
@@ -9844,9 +9860,7 @@
       <c r="AB156" s="14"/>
       <c r="AC156" s="14"/>
       <c r="AD156" s="14"/>
-      <c r="AE156" s="27" t="s">
-        <v>415</v>
-      </c>
+      <c r="AE156" s="27"/>
       <c r="AF156" s="14"/>
       <c r="AG156" s="14"/>
       <c r="AH156" s="14"/>
@@ -9854,7 +9868,7 @@
     </row>
     <row r="157" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="14" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="B157" s="14" t="s">
         <v>174</v>
@@ -9863,16 +9877,16 @@
         <v>135</v>
       </c>
       <c r="D157" s="18" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="E157" s="15"/>
       <c r="F157" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G157" s="15"/>
+      <c r="G157" s="14"/>
       <c r="H157" s="14"/>
       <c r="I157" s="14" t="s">
-        <v>504</v>
+        <v>128</v>
       </c>
       <c r="J157" s="14"/>
       <c r="K157" s="14"/>
@@ -9895,7 +9909,9 @@
       <c r="AB157" s="14"/>
       <c r="AC157" s="14"/>
       <c r="AD157" s="14"/>
-      <c r="AE157" s="27"/>
+      <c r="AE157" s="27" t="s">
+        <v>415</v>
+      </c>
       <c r="AF157" s="14"/>
       <c r="AG157" s="14"/>
       <c r="AH157" s="14"/>
@@ -9903,7 +9919,7 @@
     </row>
     <row r="158" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="14" t="s">
-        <v>605</v>
+        <v>600</v>
       </c>
       <c r="B158" s="14" t="s">
         <v>174</v>
@@ -9912,15 +9928,17 @@
         <v>135</v>
       </c>
       <c r="D158" s="18" t="s">
-        <v>589</v>
-      </c>
-      <c r="E158" s="14"/>
+        <v>588</v>
+      </c>
+      <c r="E158" s="15"/>
       <c r="F158" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G158" s="14"/>
+      <c r="G158" s="15"/>
       <c r="H158" s="14"/>
-      <c r="I158" s="14"/>
+      <c r="I158" s="14" t="s">
+        <v>504</v>
+      </c>
       <c r="J158" s="14"/>
       <c r="K158" s="14"/>
       <c r="L158" s="14"/>
@@ -9950,7 +9968,7 @@
     </row>
     <row r="159" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="14" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B159" s="14" t="s">
         <v>174</v>
@@ -9959,7 +9977,7 @@
         <v>135</v>
       </c>
       <c r="D159" s="18" t="s">
-        <v>597</v>
+        <v>589</v>
       </c>
       <c r="E159" s="14"/>
       <c r="F159" s="14" t="s">
@@ -9997,7 +10015,7 @@
     </row>
     <row r="160" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="14" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B160" s="14" t="s">
         <v>174</v>
@@ -10006,17 +10024,15 @@
         <v>135</v>
       </c>
       <c r="D160" s="18" t="s">
-        <v>598</v>
-      </c>
-      <c r="E160" s="15"/>
+        <v>597</v>
+      </c>
+      <c r="E160" s="14"/>
       <c r="F160" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G160" s="15"/>
+      <c r="G160" s="14"/>
       <c r="H160" s="14"/>
-      <c r="I160" s="14" t="s">
-        <v>378</v>
-      </c>
+      <c r="I160" s="14"/>
       <c r="J160" s="14"/>
       <c r="K160" s="14"/>
       <c r="L160" s="14"/>
@@ -10046,7 +10062,7 @@
     </row>
     <row r="161" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="14" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B161" s="14" t="s">
         <v>174</v>
@@ -10055,16 +10071,16 @@
         <v>135</v>
       </c>
       <c r="D161" s="18" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="E161" s="15"/>
       <c r="F161" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="G161" s="14"/>
+      <c r="G161" s="15"/>
       <c r="H161" s="14"/>
       <c r="I161" s="14" t="s">
-        <v>401</v>
+        <v>378</v>
       </c>
       <c r="J161" s="14"/>
       <c r="K161" s="14"/>
@@ -10095,7 +10111,7 @@
     </row>
     <row r="162" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="14" t="s">
-        <v>601</v>
+        <v>608</v>
       </c>
       <c r="B162" s="14" t="s">
         <v>174</v>
@@ -10104,7 +10120,7 @@
         <v>135</v>
       </c>
       <c r="D162" s="18" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="E162" s="15"/>
       <c r="F162" s="14" t="s">
@@ -10113,7 +10129,7 @@
       <c r="G162" s="14"/>
       <c r="H162" s="14"/>
       <c r="I162" s="14" t="s">
-        <v>126</v>
+        <v>401</v>
       </c>
       <c r="J162" s="14"/>
       <c r="K162" s="14"/>
@@ -10143,15 +10159,27 @@
       <c r="AI162" s="14"/>
     </row>
     <row r="163" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A163" s="14"/>
-      <c r="B163" s="14"/>
-      <c r="C163" s="14"/>
-      <c r="D163" s="15"/>
-      <c r="E163" s="14"/>
-      <c r="F163" s="14"/>
+      <c r="A163" s="14" t="s">
+        <v>601</v>
+      </c>
+      <c r="B163" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C163" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D163" s="18" t="s">
+        <v>596</v>
+      </c>
+      <c r="E163" s="15"/>
+      <c r="F163" s="14" t="s">
+        <v>403</v>
+      </c>
       <c r="G163" s="14"/>
       <c r="H163" s="14"/>
-      <c r="I163" s="14"/>
+      <c r="I163" s="14" t="s">
+        <v>126</v>
+      </c>
       <c r="J163" s="14"/>
       <c r="K163" s="14"/>
       <c r="L163" s="14"/>
@@ -10160,7 +10188,7 @@
       <c r="O163" s="14"/>
       <c r="P163" s="14"/>
       <c r="Q163" s="14"/>
-      <c r="R163" s="15"/>
+      <c r="R163" s="14"/>
       <c r="S163" s="14"/>
       <c r="T163" s="14"/>
       <c r="U163" s="14"/>
@@ -10180,18 +10208,10 @@
       <c r="AI163" s="14"/>
     </row>
     <row r="164" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A164" s="14" t="s">
-        <v>488</v>
-      </c>
-      <c r="B164" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C164" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D164" s="18" t="s">
-        <v>489</v>
-      </c>
+      <c r="A164" s="14"/>
+      <c r="B164" s="14"/>
+      <c r="C164" s="14"/>
+      <c r="D164" s="15"/>
       <c r="E164" s="14"/>
       <c r="F164" s="14"/>
       <c r="G164" s="14"/>
@@ -10204,16 +10224,10 @@
       <c r="N164" s="14"/>
       <c r="O164" s="14"/>
       <c r="P164" s="14"/>
-      <c r="Q164" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="R164" s="14"/>
-      <c r="S164" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T164" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="Q164" s="14"/>
+      <c r="R164" s="15"/>
+      <c r="S164" s="14"/>
+      <c r="T164" s="14"/>
       <c r="U164" s="14"/>
       <c r="V164" s="14"/>
       <c r="W164" s="14"/>
@@ -10221,26 +10235,18 @@
       <c r="Y164" s="14"/>
       <c r="Z164" s="14"/>
       <c r="AA164" s="14"/>
-      <c r="AB164" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC164" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD164" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB164" s="14"/>
+      <c r="AC164" s="14"/>
+      <c r="AD164" s="14"/>
       <c r="AE164" s="27"/>
       <c r="AF164" s="14"/>
       <c r="AG164" s="14"/>
-      <c r="AH164" s="14" t="s">
-        <v>465</v>
-      </c>
+      <c r="AH164" s="14"/>
       <c r="AI164" s="14"/>
     </row>
     <row r="165" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="14" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B165" s="14" t="s">
         <v>174</v>
@@ -10249,7 +10255,7 @@
         <v>135</v>
       </c>
       <c r="D165" s="18" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="E165" s="14"/>
       <c r="F165" s="14"/>
@@ -10263,10 +10269,16 @@
       <c r="N165" s="14"/>
       <c r="O165" s="14"/>
       <c r="P165" s="14"/>
-      <c r="Q165" s="14"/>
+      <c r="Q165" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R165" s="14"/>
-      <c r="S165" s="14"/>
-      <c r="T165" s="14"/>
+      <c r="S165" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T165" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U165" s="14"/>
       <c r="V165" s="14"/>
       <c r="W165" s="14"/>
@@ -10286,12 +10298,14 @@
       <c r="AE165" s="27"/>
       <c r="AF165" s="14"/>
       <c r="AG165" s="14"/>
-      <c r="AH165" s="14"/>
+      <c r="AH165" s="14" t="s">
+        <v>465</v>
+      </c>
       <c r="AI165" s="14"/>
     </row>
     <row r="166" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="14" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="B166" s="14" t="s">
         <v>174</v>
@@ -10300,7 +10314,7 @@
         <v>135</v>
       </c>
       <c r="D166" s="18" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="E166" s="14"/>
       <c r="F166" s="14"/>
@@ -10326,25 +10340,23 @@
       <c r="Z166" s="14"/>
       <c r="AA166" s="14"/>
       <c r="AB166" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC166" s="14" t="s">
-        <v>457</v>
+        <v>393</v>
       </c>
       <c r="AD166" s="14" t="s">
-        <v>451</v>
+        <v>393</v>
       </c>
       <c r="AE166" s="27"/>
       <c r="AF166" s="14"/>
       <c r="AG166" s="14"/>
-      <c r="AH166" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH166" s="14"/>
       <c r="AI166" s="14"/>
     </row>
     <row r="167" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="14" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B167" s="14" t="s">
         <v>174</v>
@@ -10353,7 +10365,7 @@
         <v>135</v>
       </c>
       <c r="D167" s="18" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="E167" s="14"/>
       <c r="F167" s="14"/>
@@ -10367,16 +10379,10 @@
       <c r="N167" s="14"/>
       <c r="O167" s="14"/>
       <c r="P167" s="14"/>
-      <c r="Q167" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q167" s="14"/>
       <c r="R167" s="14"/>
-      <c r="S167" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T167" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S167" s="14"/>
+      <c r="T167" s="14"/>
       <c r="U167" s="14"/>
       <c r="V167" s="14"/>
       <c r="W167" s="14"/>
@@ -10396,14 +10402,14 @@
       <c r="AE167" s="27"/>
       <c r="AF167" s="14"/>
       <c r="AG167" s="14"/>
-      <c r="AH167" s="15" t="s">
-        <v>454</v>
+      <c r="AH167" s="14" t="s">
+        <v>458</v>
       </c>
       <c r="AI167" s="14"/>
     </row>
     <row r="168" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="14" t="s">
-        <v>539</v>
+        <v>490</v>
       </c>
       <c r="B168" s="14" t="s">
         <v>174</v>
@@ -10411,8 +10417,8 @@
       <c r="C168" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D168" s="23" t="s">
-        <v>540</v>
+      <c r="D168" s="18" t="s">
+        <v>491</v>
       </c>
       <c r="E168" s="14"/>
       <c r="F168" s="14"/>
@@ -10422,16 +10428,20 @@
       <c r="J168" s="14"/>
       <c r="K168" s="14"/>
       <c r="L168" s="14"/>
-      <c r="M168" s="20" t="s">
-        <v>609</v>
-      </c>
+      <c r="M168" s="14"/>
       <c r="N168" s="14"/>
       <c r="O168" s="14"/>
       <c r="P168" s="14"/>
-      <c r="Q168" s="14"/>
+      <c r="Q168" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R168" s="14"/>
-      <c r="S168" s="14"/>
-      <c r="T168" s="14"/>
+      <c r="S168" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T168" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U168" s="14"/>
       <c r="V168" s="14"/>
       <c r="W168" s="14"/>
@@ -10451,14 +10461,14 @@
       <c r="AE168" s="27"/>
       <c r="AF168" s="14"/>
       <c r="AG168" s="14"/>
-      <c r="AH168" s="14" t="s">
-        <v>458</v>
+      <c r="AH168" s="15" t="s">
+        <v>454</v>
       </c>
       <c r="AI168" s="14"/>
     </row>
     <row r="169" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="14" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="B169" s="14" t="s">
         <v>174</v>
@@ -10467,7 +10477,7 @@
         <v>135</v>
       </c>
       <c r="D169" s="23" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="E169" s="14"/>
       <c r="F169" s="14"/>
@@ -10478,7 +10488,7 @@
       <c r="K169" s="14"/>
       <c r="L169" s="14"/>
       <c r="M169" s="20" t="s">
-        <v>494</v>
+        <v>609</v>
       </c>
       <c r="N169" s="14"/>
       <c r="O169" s="14"/>
@@ -10495,23 +10505,25 @@
       <c r="Z169" s="14"/>
       <c r="AA169" s="14"/>
       <c r="AB169" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC169" s="14" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="AD169" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE169" s="27"/>
       <c r="AF169" s="14"/>
       <c r="AG169" s="14"/>
-      <c r="AH169" s="14"/>
+      <c r="AH169" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI169" s="14"/>
     </row>
     <row r="170" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="14" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B170" s="14" t="s">
         <v>174</v>
@@ -10520,7 +10532,7 @@
         <v>135</v>
       </c>
       <c r="D170" s="23" t="s">
-        <v>546</v>
+        <v>541</v>
       </c>
       <c r="E170" s="14"/>
       <c r="F170" s="14"/>
@@ -10548,25 +10560,23 @@
       <c r="Z170" s="14"/>
       <c r="AA170" s="14"/>
       <c r="AB170" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC170" s="14" t="s">
-        <v>457</v>
+        <v>427</v>
       </c>
       <c r="AD170" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE170" s="27"/>
       <c r="AF170" s="14"/>
       <c r="AG170" s="14"/>
-      <c r="AH170" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH170" s="14"/>
       <c r="AI170" s="14"/>
     </row>
     <row r="171" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="14" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="B171" s="14" t="s">
         <v>174</v>
@@ -10574,8 +10584,8 @@
       <c r="C171" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D171" s="18" t="s">
-        <v>548</v>
+      <c r="D171" s="23" t="s">
+        <v>546</v>
       </c>
       <c r="E171" s="14"/>
       <c r="F171" s="14"/>
@@ -10584,7 +10594,7 @@
       <c r="I171" s="14"/>
       <c r="J171" s="14"/>
       <c r="K171" s="14"/>
-      <c r="L171" s="31"/>
+      <c r="L171" s="14"/>
       <c r="M171" s="20" t="s">
         <v>494</v>
       </c>
@@ -10621,7 +10631,7 @@
     </row>
     <row r="172" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="14" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="B172" s="14" t="s">
         <v>174</v>
@@ -10630,7 +10640,7 @@
         <v>135</v>
       </c>
       <c r="D172" s="18" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="E172" s="14"/>
       <c r="F172" s="14"/>
@@ -10639,7 +10649,7 @@
       <c r="I172" s="14"/>
       <c r="J172" s="14"/>
       <c r="K172" s="14"/>
-      <c r="L172" s="14"/>
+      <c r="L172" s="31"/>
       <c r="M172" s="20" t="s">
         <v>494</v>
       </c>
@@ -10658,13 +10668,13 @@
       <c r="Z172" s="14"/>
       <c r="AA172" s="14"/>
       <c r="AB172" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC172" s="14" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="AD172" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE172" s="27"/>
       <c r="AF172" s="14"/>
@@ -10675,10 +10685,18 @@
       <c r="AI172" s="14"/>
     </row>
     <row r="173" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A173" s="14"/>
-      <c r="B173" s="14"/>
-      <c r="C173" s="14"/>
-      <c r="D173" s="18"/>
+      <c r="A173" s="14" t="s">
+        <v>550</v>
+      </c>
+      <c r="B173" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C173" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D173" s="18" t="s">
+        <v>551</v>
+      </c>
       <c r="E173" s="14"/>
       <c r="F173" s="14"/>
       <c r="G173" s="14"/>
@@ -10687,7 +10705,9 @@
       <c r="J173" s="14"/>
       <c r="K173" s="14"/>
       <c r="L173" s="14"/>
-      <c r="M173" s="20"/>
+      <c r="M173" s="20" t="s">
+        <v>494</v>
+      </c>
       <c r="N173" s="14"/>
       <c r="O173" s="14"/>
       <c r="P173" s="14"/>
@@ -10702,28 +10722,28 @@
       <c r="Y173" s="14"/>
       <c r="Z173" s="14"/>
       <c r="AA173" s="14"/>
-      <c r="AB173" s="14"/>
-      <c r="AC173" s="14"/>
-      <c r="AD173" s="14"/>
+      <c r="AB173" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC173" s="14" t="s">
+        <v>427</v>
+      </c>
+      <c r="AD173" s="14" t="s">
+        <v>421</v>
+      </c>
       <c r="AE173" s="27"/>
       <c r="AF173" s="14"/>
       <c r="AG173" s="14"/>
-      <c r="AH173" s="14"/>
+      <c r="AH173" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI173" s="14"/>
     </row>
     <row r="174" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A174" s="14" t="s">
-        <v>554</v>
-      </c>
-      <c r="B174" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C174" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D174" s="18" t="s">
-        <v>566</v>
-      </c>
+      <c r="A174" s="14"/>
+      <c r="B174" s="14"/>
+      <c r="C174" s="14"/>
+      <c r="D174" s="18"/>
       <c r="E174" s="14"/>
       <c r="F174" s="14"/>
       <c r="G174" s="14"/>
@@ -10732,20 +10752,14 @@
       <c r="J174" s="14"/>
       <c r="K174" s="14"/>
       <c r="L174" s="14"/>
-      <c r="M174" s="14"/>
+      <c r="M174" s="20"/>
       <c r="N174" s="14"/>
       <c r="O174" s="14"/>
       <c r="P174" s="14"/>
-      <c r="Q174" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q174" s="14"/>
       <c r="R174" s="14"/>
-      <c r="S174" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T174" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S174" s="14"/>
+      <c r="T174" s="14"/>
       <c r="U174" s="14"/>
       <c r="V174" s="14"/>
       <c r="W174" s="14"/>
@@ -10753,26 +10767,18 @@
       <c r="Y174" s="14"/>
       <c r="Z174" s="14"/>
       <c r="AA174" s="14"/>
-      <c r="AB174" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC174" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AD174" s="14" t="s">
-        <v>393</v>
-      </c>
+      <c r="AB174" s="14"/>
+      <c r="AC174" s="14"/>
+      <c r="AD174" s="14"/>
       <c r="AE174" s="27"/>
       <c r="AF174" s="14"/>
       <c r="AG174" s="14"/>
-      <c r="AH174" s="14" t="s">
-        <v>465</v>
-      </c>
+      <c r="AH174" s="14"/>
       <c r="AI174" s="14"/>
     </row>
     <row r="175" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="14" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B175" s="14" t="s">
         <v>174</v>
@@ -10781,7 +10787,7 @@
         <v>135</v>
       </c>
       <c r="D175" s="18" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="E175" s="14"/>
       <c r="F175" s="14"/>
@@ -10795,10 +10801,16 @@
       <c r="N175" s="14"/>
       <c r="O175" s="14"/>
       <c r="P175" s="14"/>
-      <c r="Q175" s="14"/>
+      <c r="Q175" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R175" s="14"/>
-      <c r="S175" s="14"/>
-      <c r="T175" s="14"/>
+      <c r="S175" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T175" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U175" s="14"/>
       <c r="V175" s="14"/>
       <c r="W175" s="14"/>
@@ -10818,12 +10830,14 @@
       <c r="AE175" s="27"/>
       <c r="AF175" s="14"/>
       <c r="AG175" s="14"/>
-      <c r="AH175" s="14"/>
+      <c r="AH175" s="14" t="s">
+        <v>465</v>
+      </c>
       <c r="AI175" s="14"/>
     </row>
     <row r="176" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="14" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B176" s="14" t="s">
         <v>174</v>
@@ -10832,7 +10846,7 @@
         <v>135</v>
       </c>
       <c r="D176" s="18" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E176" s="14"/>
       <c r="F176" s="14"/>
@@ -10858,25 +10872,23 @@
       <c r="Z176" s="14"/>
       <c r="AA176" s="14"/>
       <c r="AB176" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC176" s="14" t="s">
-        <v>457</v>
+        <v>393</v>
       </c>
       <c r="AD176" s="14" t="s">
-        <v>451</v>
+        <v>393</v>
       </c>
       <c r="AE176" s="27"/>
       <c r="AF176" s="14"/>
       <c r="AG176" s="14"/>
-      <c r="AH176" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH176" s="14"/>
       <c r="AI176" s="14"/>
     </row>
     <row r="177" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="14" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B177" s="14" t="s">
         <v>174</v>
@@ -10885,7 +10897,7 @@
         <v>135</v>
       </c>
       <c r="D177" s="18" t="s">
-        <v>570</v>
+        <v>563</v>
       </c>
       <c r="E177" s="14"/>
       <c r="F177" s="14"/>
@@ -10899,16 +10911,10 @@
       <c r="N177" s="14"/>
       <c r="O177" s="14"/>
       <c r="P177" s="14"/>
-      <c r="Q177" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="Q177" s="14"/>
       <c r="R177" s="14"/>
-      <c r="S177" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="T177" s="14" t="s">
-        <v>300</v>
-      </c>
+      <c r="S177" s="14"/>
+      <c r="T177" s="14"/>
       <c r="U177" s="14"/>
       <c r="V177" s="14"/>
       <c r="W177" s="14"/>
@@ -10928,14 +10934,14 @@
       <c r="AE177" s="27"/>
       <c r="AF177" s="14"/>
       <c r="AG177" s="14"/>
-      <c r="AH177" s="15" t="s">
-        <v>454</v>
+      <c r="AH177" s="14" t="s">
+        <v>458</v>
       </c>
       <c r="AI177" s="14"/>
     </row>
     <row r="178" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="14" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B178" s="14" t="s">
         <v>174</v>
@@ -10943,8 +10949,8 @@
       <c r="C178" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D178" s="23" t="s">
-        <v>571</v>
+      <c r="D178" s="18" t="s">
+        <v>570</v>
       </c>
       <c r="E178" s="14"/>
       <c r="F178" s="14"/>
@@ -10954,16 +10960,20 @@
       <c r="J178" s="14"/>
       <c r="K178" s="14"/>
       <c r="L178" s="14"/>
-      <c r="M178" s="30" t="s">
-        <v>580</v>
-      </c>
+      <c r="M178" s="14"/>
       <c r="N178" s="14"/>
       <c r="O178" s="14"/>
       <c r="P178" s="14"/>
-      <c r="Q178" s="14"/>
+      <c r="Q178" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="R178" s="14"/>
-      <c r="S178" s="14"/>
-      <c r="T178" s="14"/>
+      <c r="S178" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="T178" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="U178" s="14"/>
       <c r="V178" s="14"/>
       <c r="W178" s="14"/>
@@ -10983,14 +10993,14 @@
       <c r="AE178" s="27"/>
       <c r="AF178" s="14"/>
       <c r="AG178" s="14"/>
-      <c r="AH178" s="14" t="s">
-        <v>458</v>
+      <c r="AH178" s="15" t="s">
+        <v>454</v>
       </c>
       <c r="AI178" s="14"/>
     </row>
     <row r="179" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="14" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B179" s="14" t="s">
         <v>174</v>
@@ -10999,7 +11009,7 @@
         <v>135</v>
       </c>
       <c r="D179" s="23" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="E179" s="14"/>
       <c r="F179" s="14"/>
@@ -11010,7 +11020,7 @@
       <c r="K179" s="14"/>
       <c r="L179" s="14"/>
       <c r="M179" s="30" t="s">
-        <v>549</v>
+        <v>580</v>
       </c>
       <c r="N179" s="14"/>
       <c r="O179" s="14"/>
@@ -11027,23 +11037,25 @@
       <c r="Z179" s="14"/>
       <c r="AA179" s="14"/>
       <c r="AB179" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC179" s="14" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="AD179" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE179" s="27"/>
       <c r="AF179" s="14"/>
       <c r="AG179" s="14"/>
-      <c r="AH179" s="14"/>
+      <c r="AH179" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI179" s="14"/>
     </row>
     <row r="180" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="14" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B180" s="14" t="s">
         <v>174</v>
@@ -11052,7 +11064,7 @@
         <v>135</v>
       </c>
       <c r="D180" s="23" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="E180" s="14"/>
       <c r="F180" s="14"/>
@@ -11062,7 +11074,7 @@
       <c r="J180" s="14"/>
       <c r="K180" s="14"/>
       <c r="L180" s="14"/>
-      <c r="M180" s="14" t="s">
+      <c r="M180" s="30" t="s">
         <v>549</v>
       </c>
       <c r="N180" s="14"/>
@@ -11080,25 +11092,23 @@
       <c r="Z180" s="14"/>
       <c r="AA180" s="14"/>
       <c r="AB180" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC180" s="14" t="s">
-        <v>457</v>
+        <v>427</v>
       </c>
       <c r="AD180" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE180" s="27"/>
       <c r="AF180" s="14"/>
       <c r="AG180" s="14"/>
-      <c r="AH180" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH180" s="14"/>
       <c r="AI180" s="14"/>
     </row>
     <row r="181" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A181" s="14" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B181" s="14" t="s">
         <v>174</v>
@@ -11106,8 +11116,8 @@
       <c r="C181" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D181" s="18" t="s">
-        <v>579</v>
+      <c r="D181" s="23" t="s">
+        <v>578</v>
       </c>
       <c r="E181" s="14"/>
       <c r="F181" s="14"/>
@@ -11135,13 +11145,13 @@
       <c r="Z181" s="14"/>
       <c r="AA181" s="14"/>
       <c r="AB181" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC181" s="14" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="AD181" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE181" s="27"/>
       <c r="AF181" s="14"/>
@@ -11153,7 +11163,7 @@
     </row>
     <row r="182" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A182" s="14" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B182" s="14" t="s">
         <v>174</v>
@@ -11162,7 +11172,7 @@
         <v>135</v>
       </c>
       <c r="D182" s="18" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E182" s="14"/>
       <c r="F182" s="14"/>
@@ -11171,8 +11181,8 @@
       <c r="I182" s="14"/>
       <c r="J182" s="14"/>
       <c r="K182" s="14"/>
-      <c r="L182" s="31"/>
-      <c r="M182" s="30" t="s">
+      <c r="L182" s="14"/>
+      <c r="M182" s="14" t="s">
         <v>549</v>
       </c>
       <c r="N182" s="14"/>
@@ -11190,13 +11200,13 @@
       <c r="Z182" s="14"/>
       <c r="AA182" s="14"/>
       <c r="AB182" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC182" s="14" t="s">
-        <v>457</v>
+        <v>427</v>
       </c>
       <c r="AD182" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE182" s="27"/>
       <c r="AF182" s="14"/>
@@ -11207,10 +11217,18 @@
       <c r="AI182" s="14"/>
     </row>
     <row r="183" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A183" s="14"/>
-      <c r="B183" s="14"/>
-      <c r="C183" s="14"/>
-      <c r="D183" s="15"/>
+      <c r="A183" s="14" t="s">
+        <v>562</v>
+      </c>
+      <c r="B183" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C183" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D183" s="18" t="s">
+        <v>575</v>
+      </c>
       <c r="E183" s="14"/>
       <c r="F183" s="14"/>
       <c r="G183" s="14"/>
@@ -11218,13 +11236,15 @@
       <c r="I183" s="14"/>
       <c r="J183" s="14"/>
       <c r="K183" s="14"/>
-      <c r="L183" s="14"/>
-      <c r="M183" s="14"/>
+      <c r="L183" s="31"/>
+      <c r="M183" s="30" t="s">
+        <v>549</v>
+      </c>
       <c r="N183" s="14"/>
       <c r="O183" s="14"/>
       <c r="P183" s="14"/>
       <c r="Q183" s="14"/>
-      <c r="R183" s="15"/>
+      <c r="R183" s="14"/>
       <c r="S183" s="14"/>
       <c r="T183" s="14"/>
       <c r="U183" s="14"/>
@@ -11234,44 +11254,42 @@
       <c r="Y183" s="14"/>
       <c r="Z183" s="14"/>
       <c r="AA183" s="14"/>
-      <c r="AB183" s="14"/>
-      <c r="AC183" s="14"/>
-      <c r="AD183" s="14"/>
+      <c r="AB183" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC183" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD183" s="14" t="s">
+        <v>451</v>
+      </c>
       <c r="AE183" s="27"/>
       <c r="AF183" s="14"/>
       <c r="AG183" s="14"/>
-      <c r="AH183" s="14"/>
+      <c r="AH183" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI183" s="14"/>
     </row>
     <row r="184" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A184" s="14" t="s">
-        <v>616</v>
-      </c>
-      <c r="B184" s="14" t="s">
-        <v>613</v>
-      </c>
-      <c r="C184" s="14" t="s">
-        <v>614</v>
-      </c>
-      <c r="D184" s="18" t="s">
-        <v>618</v>
-      </c>
+      <c r="A184" s="14"/>
+      <c r="B184" s="14"/>
+      <c r="C184" s="14"/>
+      <c r="D184" s="15"/>
       <c r="E184" s="14"/>
       <c r="F184" s="14"/>
       <c r="G184" s="14"/>
       <c r="H184" s="14"/>
-      <c r="I184" s="14" t="s">
-        <v>128</v>
-      </c>
+      <c r="I184" s="14"/>
       <c r="J184" s="14"/>
       <c r="K184" s="14"/>
-      <c r="L184" s="31"/>
-      <c r="M184" s="30"/>
+      <c r="L184" s="14"/>
+      <c r="M184" s="14"/>
       <c r="N184" s="14"/>
       <c r="O184" s="14"/>
       <c r="P184" s="14"/>
       <c r="Q184" s="14"/>
-      <c r="R184" s="14"/>
+      <c r="R184" s="15"/>
       <c r="S184" s="14"/>
       <c r="T184" s="14"/>
       <c r="U184" s="14"/>
@@ -11284,19 +11302,15 @@
       <c r="AB184" s="14"/>
       <c r="AC184" s="14"/>
       <c r="AD184" s="14"/>
-      <c r="AE184" s="27" t="s">
-        <v>654</v>
-      </c>
+      <c r="AE184" s="27"/>
       <c r="AF184" s="14"/>
       <c r="AG184" s="14"/>
-      <c r="AH184" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH184" s="14"/>
       <c r="AI184" s="14"/>
     </row>
     <row r="185" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A185" s="14" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="B185" s="14" t="s">
         <v>613</v>
@@ -11305,7 +11319,7 @@
         <v>614</v>
       </c>
       <c r="D185" s="18" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="E185" s="14"/>
       <c r="F185" s="14"/>
@@ -11336,7 +11350,7 @@
       <c r="AC185" s="14"/>
       <c r="AD185" s="14"/>
       <c r="AE185" s="27" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="AF185" s="14"/>
       <c r="AG185" s="14"/>
@@ -11347,7 +11361,7 @@
     </row>
     <row r="186" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="14" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B186" s="14" t="s">
         <v>613</v>
@@ -11356,7 +11370,7 @@
         <v>614</v>
       </c>
       <c r="D186" s="18" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="E186" s="14"/>
       <c r="F186" s="14"/>
@@ -11398,7 +11412,7 @@
     </row>
     <row r="187" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="14" t="s">
-        <v>625</v>
+        <v>620</v>
       </c>
       <c r="B187" s="14" t="s">
         <v>613</v>
@@ -11407,7 +11421,7 @@
         <v>614</v>
       </c>
       <c r="D187" s="18" t="s">
-        <v>628</v>
+        <v>622</v>
       </c>
       <c r="E187" s="14"/>
       <c r="F187" s="14"/>
@@ -11438,7 +11452,7 @@
       <c r="AC187" s="14"/>
       <c r="AD187" s="14"/>
       <c r="AE187" s="27" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="AF187" s="14"/>
       <c r="AG187" s="14"/>
@@ -11449,7 +11463,7 @@
     </row>
     <row r="188" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="14" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B188" s="14" t="s">
         <v>613</v>
@@ -11458,7 +11472,7 @@
         <v>614</v>
       </c>
       <c r="D188" s="18" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="E188" s="14"/>
       <c r="F188" s="14"/>
@@ -11489,7 +11503,7 @@
       <c r="AC188" s="14"/>
       <c r="AD188" s="14"/>
       <c r="AE188" s="27" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="AF188" s="14"/>
       <c r="AG188" s="14"/>
@@ -11500,7 +11514,7 @@
     </row>
     <row r="189" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="14" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B189" s="14" t="s">
         <v>613</v>
@@ -11509,7 +11523,7 @@
         <v>614</v>
       </c>
       <c r="D189" s="18" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="E189" s="14"/>
       <c r="F189" s="14"/>
@@ -11540,7 +11554,7 @@
       <c r="AC189" s="14"/>
       <c r="AD189" s="14"/>
       <c r="AE189" s="27" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="AF189" s="14"/>
       <c r="AG189" s="14"/>
@@ -11551,7 +11565,7 @@
     </row>
     <row r="190" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="14" t="s">
-        <v>633</v>
+        <v>627</v>
       </c>
       <c r="B190" s="14" t="s">
         <v>613</v>
@@ -11560,14 +11574,14 @@
         <v>614</v>
       </c>
       <c r="D190" s="18" t="s">
-        <v>655</v>
+        <v>630</v>
       </c>
       <c r="E190" s="14"/>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
       <c r="H190" s="14"/>
       <c r="I190" s="14" t="s">
-        <v>378</v>
+        <v>128</v>
       </c>
       <c r="J190" s="14"/>
       <c r="K190" s="14"/>
@@ -11591,7 +11605,7 @@
       <c r="AC190" s="14"/>
       <c r="AD190" s="14"/>
       <c r="AE190" s="27" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="AF190" s="14"/>
       <c r="AG190" s="14"/>
@@ -11602,7 +11616,7 @@
     </row>
     <row r="191" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="14" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="B191" s="14" t="s">
         <v>613</v>
@@ -11611,7 +11625,7 @@
         <v>614</v>
       </c>
       <c r="D191" s="18" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="E191" s="14"/>
       <c r="F191" s="14"/>
@@ -11642,7 +11656,7 @@
       <c r="AC191" s="14"/>
       <c r="AD191" s="14"/>
       <c r="AE191" s="27" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="AF191" s="14"/>
       <c r="AG191" s="14"/>
@@ -11653,7 +11667,7 @@
     </row>
     <row r="192" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="14" t="s">
-        <v>640</v>
+        <v>635</v>
       </c>
       <c r="B192" s="14" t="s">
         <v>613</v>
@@ -11662,7 +11676,7 @@
         <v>614</v>
       </c>
       <c r="D192" s="18" t="s">
-        <v>656</v>
+        <v>649</v>
       </c>
       <c r="E192" s="14"/>
       <c r="F192" s="14"/>
@@ -11704,7 +11718,7 @@
     </row>
     <row r="193" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="14" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="B193" s="14" t="s">
         <v>613</v>
@@ -11713,7 +11727,7 @@
         <v>614</v>
       </c>
       <c r="D193" s="18" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E193" s="14"/>
       <c r="F193" s="14"/>
@@ -11744,16 +11758,18 @@
       <c r="AC193" s="14"/>
       <c r="AD193" s="14"/>
       <c r="AE193" s="27" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="AF193" s="14"/>
       <c r="AG193" s="14"/>
-      <c r="AH193" s="14"/>
+      <c r="AH193" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI193" s="14"/>
     </row>
     <row r="194" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="14" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B194" s="14" t="s">
         <v>613</v>
@@ -11762,7 +11778,7 @@
         <v>614</v>
       </c>
       <c r="D194" s="18" t="s">
-        <v>663</v>
+        <v>657</v>
       </c>
       <c r="E194" s="14"/>
       <c r="F194" s="14"/>
@@ -11793,18 +11809,16 @@
       <c r="AC194" s="14"/>
       <c r="AD194" s="14"/>
       <c r="AE194" s="27" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="AF194" s="14"/>
       <c r="AG194" s="14"/>
-      <c r="AH194" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH194" s="14"/>
       <c r="AI194" s="14"/>
     </row>
     <row r="195" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="14" t="s">
-        <v>695</v>
+        <v>644</v>
       </c>
       <c r="B195" s="14" t="s">
         <v>613</v>
@@ -11813,14 +11827,14 @@
         <v>614</v>
       </c>
       <c r="D195" s="18" t="s">
-        <v>696</v>
+        <v>663</v>
       </c>
       <c r="E195" s="14"/>
       <c r="F195" s="14"/>
       <c r="G195" s="14"/>
       <c r="H195" s="14"/>
       <c r="I195" s="14" t="s">
-        <v>128</v>
+        <v>378</v>
       </c>
       <c r="J195" s="14"/>
       <c r="K195" s="14"/>
@@ -11844,7 +11858,7 @@
       <c r="AC195" s="14"/>
       <c r="AD195" s="14"/>
       <c r="AE195" s="27" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="AF195" s="14"/>
       <c r="AG195" s="14"/>
@@ -11854,15 +11868,25 @@
       <c r="AI195" s="14"/>
     </row>
     <row r="196" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A196" s="14"/>
-      <c r="B196" s="14"/>
-      <c r="C196" s="14"/>
-      <c r="D196" s="18"/>
+      <c r="A196" s="14" t="s">
+        <v>695</v>
+      </c>
+      <c r="B196" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C196" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D196" s="18" t="s">
+        <v>696</v>
+      </c>
       <c r="E196" s="14"/>
       <c r="F196" s="14"/>
       <c r="G196" s="14"/>
       <c r="H196" s="14"/>
-      <c r="I196" s="14"/>
+      <c r="I196" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J196" s="14"/>
       <c r="K196" s="14"/>
       <c r="L196" s="31"/>
@@ -11884,25 +11908,21 @@
       <c r="AB196" s="14"/>
       <c r="AC196" s="14"/>
       <c r="AD196" s="14"/>
-      <c r="AE196" s="27"/>
+      <c r="AE196" s="27" t="s">
+        <v>650</v>
+      </c>
       <c r="AF196" s="14"/>
       <c r="AG196" s="14"/>
-      <c r="AH196" s="14"/>
+      <c r="AH196" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI196" s="14"/>
     </row>
     <row r="197" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A197" s="14" t="s">
-        <v>664</v>
-      </c>
-      <c r="B197" s="14" t="s">
-        <v>613</v>
-      </c>
-      <c r="C197" s="14" t="s">
-        <v>614</v>
-      </c>
-      <c r="D197" s="23" t="s">
-        <v>665</v>
-      </c>
+      <c r="A197" s="14"/>
+      <c r="B197" s="14"/>
+      <c r="C197" s="14"/>
+      <c r="D197" s="18"/>
       <c r="E197" s="14"/>
       <c r="F197" s="14"/>
       <c r="G197" s="14"/>
@@ -11910,8 +11930,8 @@
       <c r="I197" s="14"/>
       <c r="J197" s="14"/>
       <c r="K197" s="14"/>
-      <c r="L197" s="14"/>
-      <c r="M197" s="14"/>
+      <c r="L197" s="31"/>
+      <c r="M197" s="30"/>
       <c r="N197" s="14"/>
       <c r="O197" s="14"/>
       <c r="P197" s="14"/>
@@ -11926,26 +11946,18 @@
       <c r="Y197" s="14"/>
       <c r="Z197" s="14"/>
       <c r="AA197" s="14"/>
-      <c r="AB197" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC197" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD197" s="14" t="s">
-        <v>451</v>
-      </c>
+      <c r="AB197" s="14"/>
+      <c r="AC197" s="14"/>
+      <c r="AD197" s="14"/>
       <c r="AE197" s="27"/>
       <c r="AF197" s="14"/>
       <c r="AG197" s="14"/>
-      <c r="AH197" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH197" s="14"/>
       <c r="AI197" s="14"/>
     </row>
     <row r="198" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="14" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B198" s="14" t="s">
         <v>613</v>
@@ -11980,23 +11992,25 @@
       <c r="Z198" s="14"/>
       <c r="AA198" s="14"/>
       <c r="AB198" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC198" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD198" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE198" s="27"/>
       <c r="AF198" s="14"/>
       <c r="AG198" s="14"/>
-      <c r="AH198" s="14"/>
+      <c r="AH198" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI198" s="14"/>
     </row>
     <row r="199" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="14" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="B199" s="14" t="s">
         <v>613</v>
@@ -12005,7 +12019,7 @@
         <v>614</v>
       </c>
       <c r="D199" s="23" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="E199" s="14"/>
       <c r="F199" s="14"/>
@@ -12031,25 +12045,23 @@
       <c r="Z199" s="14"/>
       <c r="AA199" s="14"/>
       <c r="AB199" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC199" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD199" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE199" s="27"/>
       <c r="AF199" s="14"/>
       <c r="AG199" s="14"/>
-      <c r="AH199" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH199" s="14"/>
       <c r="AI199" s="14"/>
     </row>
     <row r="200" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="14" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B200" s="14" t="s">
         <v>613</v>
@@ -12058,7 +12070,7 @@
         <v>614</v>
       </c>
       <c r="D200" s="23" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="E200" s="14"/>
       <c r="F200" s="14"/>
@@ -12084,13 +12096,13 @@
       <c r="Z200" s="14"/>
       <c r="AA200" s="14"/>
       <c r="AB200" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC200" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD200" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE200" s="27"/>
       <c r="AF200" s="14"/>
@@ -12102,7 +12114,7 @@
     </row>
     <row r="201" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="14" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B201" s="14" t="s">
         <v>613</v>
@@ -12111,7 +12123,7 @@
         <v>614</v>
       </c>
       <c r="D201" s="23" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="E201" s="14"/>
       <c r="F201" s="14"/>
@@ -12137,13 +12149,13 @@
       <c r="Z201" s="14"/>
       <c r="AA201" s="14"/>
       <c r="AB201" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC201" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD201" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE201" s="27"/>
       <c r="AF201" s="14"/>
@@ -12155,7 +12167,7 @@
     </row>
     <row r="202" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="14" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="B202" s="14" t="s">
         <v>613</v>
@@ -12190,13 +12202,13 @@
       <c r="Z202" s="14"/>
       <c r="AA202" s="14"/>
       <c r="AB202" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC202" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD202" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE202" s="27"/>
       <c r="AF202" s="14"/>
@@ -12208,7 +12220,7 @@
     </row>
     <row r="203" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="14" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B203" s="14" t="s">
         <v>613</v>
@@ -12216,8 +12228,8 @@
       <c r="C203" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D203" s="18" t="s">
-        <v>678</v>
+      <c r="D203" s="23" t="s">
+        <v>674</v>
       </c>
       <c r="E203" s="14"/>
       <c r="F203" s="14"/>
@@ -12243,13 +12255,13 @@
       <c r="Z203" s="14"/>
       <c r="AA203" s="14"/>
       <c r="AB203" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC203" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD203" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE203" s="27"/>
       <c r="AF203" s="14"/>
@@ -12261,7 +12273,7 @@
     </row>
     <row r="204" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A204" s="14" t="s">
-        <v>681</v>
+        <v>676</v>
       </c>
       <c r="B204" s="14" t="s">
         <v>613</v>
@@ -12270,7 +12282,7 @@
         <v>614</v>
       </c>
       <c r="D204" s="18" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="E204" s="14"/>
       <c r="F204" s="14"/>
@@ -12314,7 +12326,7 @@
     </row>
     <row r="205" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="14" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="B205" s="14" t="s">
         <v>613</v>
@@ -12349,13 +12361,13 @@
       <c r="Z205" s="14"/>
       <c r="AA205" s="14"/>
       <c r="AB205" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC205" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD205" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE205" s="27"/>
       <c r="AF205" s="14"/>
@@ -12367,7 +12379,7 @@
     </row>
     <row r="206" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="14" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="B206" s="14" t="s">
         <v>613</v>
@@ -12376,7 +12388,7 @@
         <v>614</v>
       </c>
       <c r="D206" s="18" t="s">
-        <v>687</v>
+        <v>682</v>
       </c>
       <c r="E206" s="14"/>
       <c r="F206" s="14"/>
@@ -12402,13 +12414,13 @@
       <c r="Z206" s="14"/>
       <c r="AA206" s="14"/>
       <c r="AB206" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC206" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD206" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE206" s="27"/>
       <c r="AF206" s="14"/>
@@ -12420,7 +12432,7 @@
     </row>
     <row r="207" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="14" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B207" s="14" t="s">
         <v>613</v>
@@ -12455,13 +12467,13 @@
       <c r="Z207" s="14"/>
       <c r="AA207" s="14"/>
       <c r="AB207" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC207" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD207" s="14" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="AE207" s="27"/>
       <c r="AF207" s="14"/>
@@ -12473,7 +12485,7 @@
     </row>
     <row r="208" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="14" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="B208" s="14" t="s">
         <v>613</v>
@@ -12481,8 +12493,8 @@
       <c r="C208" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D208" s="23" t="s">
-        <v>669</v>
+      <c r="D208" s="18" t="s">
+        <v>687</v>
       </c>
       <c r="E208" s="14"/>
       <c r="F208" s="14"/>
@@ -12516,9 +12528,7 @@
       <c r="AD208" s="14" t="s">
         <v>421</v>
       </c>
-      <c r="AE208" s="27" t="s">
-        <v>650</v>
-      </c>
+      <c r="AE208" s="27"/>
       <c r="AF208" s="14"/>
       <c r="AG208" s="14"/>
       <c r="AH208" s="14" t="s">
@@ -12528,7 +12538,7 @@
     </row>
     <row r="209" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="14" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="B209" s="14" t="s">
         <v>613</v>
@@ -12563,13 +12573,13 @@
       <c r="Z209" s="14"/>
       <c r="AA209" s="14"/>
       <c r="AB209" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC209" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD209" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE209" s="27" t="s">
         <v>650</v>
@@ -12583,7 +12593,7 @@
     </row>
     <row r="210" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210" s="14" t="s">
-        <v>702</v>
+        <v>693</v>
       </c>
       <c r="B210" s="14" t="s">
         <v>613</v>
@@ -12591,8 +12601,8 @@
       <c r="C210" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D210" s="18" t="s">
-        <v>628</v>
+      <c r="D210" s="23" t="s">
+        <v>669</v>
       </c>
       <c r="E210" s="14"/>
       <c r="F210" s="14"/>
@@ -12627,7 +12637,7 @@
         <v>451</v>
       </c>
       <c r="AE210" s="27" t="s">
-        <v>697</v>
+        <v>650</v>
       </c>
       <c r="AF210" s="14"/>
       <c r="AG210" s="14"/>
@@ -12638,7 +12648,7 @@
     </row>
     <row r="211" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="14" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="B211" s="14" t="s">
         <v>613</v>
@@ -12647,7 +12657,7 @@
         <v>614</v>
       </c>
       <c r="D211" s="18" t="s">
-        <v>665</v>
+        <v>628</v>
       </c>
       <c r="E211" s="14"/>
       <c r="F211" s="14"/>
@@ -12682,7 +12692,7 @@
         <v>451</v>
       </c>
       <c r="AE211" s="27" t="s">
-        <v>651</v>
+        <v>697</v>
       </c>
       <c r="AF211" s="14"/>
       <c r="AG211" s="14"/>
@@ -12693,7 +12703,7 @@
     </row>
     <row r="212" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="14" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="B212" s="14" t="s">
         <v>613</v>
@@ -12702,7 +12712,7 @@
         <v>614</v>
       </c>
       <c r="D212" s="18" t="s">
-        <v>677</v>
+        <v>665</v>
       </c>
       <c r="E212" s="14"/>
       <c r="F212" s="14"/>
@@ -12731,20 +12741,24 @@
         <v>419</v>
       </c>
       <c r="AC212" s="14" t="s">
-        <v>698</v>
+        <v>457</v>
       </c>
       <c r="AD212" s="14" t="s">
-        <v>699</v>
-      </c>
-      <c r="AE212" s="27"/>
+        <v>451</v>
+      </c>
+      <c r="AE212" s="27" t="s">
+        <v>651</v>
+      </c>
       <c r="AF212" s="14"/>
       <c r="AG212" s="14"/>
-      <c r="AH212" s="14"/>
+      <c r="AH212" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI212" s="14"/>
     </row>
     <row r="213" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A213" s="14" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B213" s="14" t="s">
         <v>613</v>
@@ -12779,17 +12793,15 @@
       <c r="Z213" s="14"/>
       <c r="AA213" s="14"/>
       <c r="AB213" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC213" s="14" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="AD213" s="14" t="s">
-        <v>701</v>
-      </c>
-      <c r="AE213" s="27" t="s">
-        <v>651</v>
-      </c>
+        <v>699</v>
+      </c>
+      <c r="AE213" s="27"/>
       <c r="AF213" s="14"/>
       <c r="AG213" s="14"/>
       <c r="AH213" s="14"/>
@@ -12797,7 +12809,7 @@
     </row>
     <row r="214" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A214" s="14" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="B214" s="14" t="s">
         <v>613</v>
@@ -12806,7 +12818,7 @@
         <v>614</v>
       </c>
       <c r="D214" s="18" t="s">
-        <v>628</v>
+        <v>677</v>
       </c>
       <c r="E214" s="14"/>
       <c r="F214" s="14"/>
@@ -12832,16 +12844,16 @@
       <c r="Z214" s="14"/>
       <c r="AA214" s="14"/>
       <c r="AB214" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC214" s="14" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="AD214" s="14" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="AE214" s="27" t="s">
-        <v>697</v>
+        <v>651</v>
       </c>
       <c r="AF214" s="14"/>
       <c r="AG214" s="14"/>
@@ -12850,7 +12862,7 @@
     </row>
     <row r="215" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A215" s="14" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B215" s="14" t="s">
         <v>613</v>
@@ -12859,7 +12871,7 @@
         <v>614</v>
       </c>
       <c r="D215" s="18" t="s">
-        <v>703</v>
+        <v>628</v>
       </c>
       <c r="E215" s="14"/>
       <c r="F215" s="14"/>
@@ -12885,29 +12897,35 @@
       <c r="Z215" s="14"/>
       <c r="AA215" s="14"/>
       <c r="AB215" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC215" s="14" t="s">
-        <v>420</v>
+        <v>698</v>
       </c>
       <c r="AD215" s="14" t="s">
-        <v>421</v>
+        <v>699</v>
       </c>
       <c r="AE215" s="27" t="s">
-        <v>654</v>
+        <v>697</v>
       </c>
       <c r="AF215" s="14"/>
       <c r="AG215" s="14"/>
-      <c r="AH215" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH215" s="14"/>
       <c r="AI215" s="14"/>
     </row>
     <row r="216" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A216" s="14"/>
-      <c r="B216" s="14"/>
-      <c r="C216" s="14"/>
-      <c r="D216" s="14"/>
+      <c r="A216" s="14" t="s">
+        <v>708</v>
+      </c>
+      <c r="B216" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C216" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D216" s="18" t="s">
+        <v>703</v>
+      </c>
       <c r="E216" s="14"/>
       <c r="F216" s="14"/>
       <c r="G216" s="14"/>
@@ -12931,40 +12949,46 @@
       <c r="Y216" s="14"/>
       <c r="Z216" s="14"/>
       <c r="AA216" s="14"/>
-      <c r="AB216" s="14"/>
-      <c r="AC216" s="14"/>
-      <c r="AD216" s="14"/>
-      <c r="AE216" s="27"/>
+      <c r="AB216" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC216" s="14" t="s">
+        <v>420</v>
+      </c>
+      <c r="AD216" s="14" t="s">
+        <v>421</v>
+      </c>
+      <c r="AE216" s="27" t="s">
+        <v>654</v>
+      </c>
       <c r="AF216" s="14"/>
       <c r="AG216" s="14"/>
-      <c r="AH216" s="14"/>
+      <c r="AH216" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI216" s="14"/>
     </row>
     <row r="217" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A217" s="14" t="s">
-        <v>267</v>
+        <v>709</v>
       </c>
       <c r="B217" s="14" t="s">
-        <v>174</v>
+        <v>613</v>
       </c>
       <c r="C217" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D217" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D217" s="18" t="s">
+        <v>677</v>
+      </c>
       <c r="E217" s="14"/>
       <c r="F217" s="14"/>
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
       <c r="I217" s="14"/>
-      <c r="J217" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K217" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L217" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J217" s="14"/>
+      <c r="K217" s="14"/>
+      <c r="L217" s="14"/>
       <c r="M217" s="14"/>
       <c r="N217" s="14"/>
       <c r="O217" s="14"/>
@@ -12980,40 +13004,36 @@
       <c r="Y217" s="14"/>
       <c r="Z217" s="14"/>
       <c r="AA217" s="14"/>
-      <c r="AB217" s="14"/>
-      <c r="AC217" s="14"/>
-      <c r="AD217" s="14"/>
-      <c r="AE217" s="27"/>
+      <c r="AB217" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC217" s="14" t="s">
+        <v>710</v>
+      </c>
+      <c r="AD217" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="AE217" s="27" t="s">
+        <v>651</v>
+      </c>
       <c r="AF217" s="14"/>
       <c r="AG217" s="14"/>
       <c r="AH217" s="14"/>
       <c r="AI217" s="14"/>
     </row>
     <row r="218" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A218" s="14" t="s">
-        <v>268</v>
-      </c>
-      <c r="B218" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C218" s="14" t="s">
-        <v>135</v>
-      </c>
+      <c r="A218" s="14"/>
+      <c r="B218" s="14"/>
+      <c r="C218" s="14"/>
       <c r="D218" s="14"/>
       <c r="E218" s="14"/>
       <c r="F218" s="14"/>
       <c r="G218" s="14"/>
       <c r="H218" s="14"/>
       <c r="I218" s="14"/>
-      <c r="J218" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K218" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L218" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="J218" s="14"/>
+      <c r="K218" s="14"/>
+      <c r="L218" s="14"/>
       <c r="M218" s="14"/>
       <c r="N218" s="14"/>
       <c r="O218" s="14"/>
@@ -13038,9 +13058,9 @@
       <c r="AH218" s="14"/>
       <c r="AI218" s="14"/>
     </row>
-    <row r="219" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A219" s="14" t="s">
-        <v>359</v>
+        <v>267</v>
       </c>
       <c r="B219" s="14" t="s">
         <v>174</v>
@@ -13048,9 +13068,36 @@
       <c r="C219" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O219" s="15" t="s">
-        <v>362</v>
-      </c>
+      <c r="D219" s="14"/>
+      <c r="E219" s="14"/>
+      <c r="F219" s="14"/>
+      <c r="G219" s="14"/>
+      <c r="H219" s="14"/>
+      <c r="I219" s="14"/>
+      <c r="J219" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K219" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L219" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M219" s="14"/>
+      <c r="N219" s="14"/>
+      <c r="O219" s="14"/>
+      <c r="P219" s="14"/>
+      <c r="Q219" s="14"/>
+      <c r="R219" s="14"/>
+      <c r="S219" s="14"/>
+      <c r="T219" s="14"/>
+      <c r="U219" s="14"/>
+      <c r="V219" s="14"/>
+      <c r="W219" s="14"/>
+      <c r="X219" s="14"/>
+      <c r="Y219" s="14"/>
+      <c r="Z219" s="14"/>
+      <c r="AA219" s="14"/>
       <c r="AB219" s="14"/>
       <c r="AC219" s="14"/>
       <c r="AD219" s="14"/>
@@ -13060,9 +13107,9 @@
       <c r="AH219" s="14"/>
       <c r="AI219" s="14"/>
     </row>
-    <row r="220" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A220" s="14" t="s">
-        <v>360</v>
+        <v>268</v>
       </c>
       <c r="B220" s="14" t="s">
         <v>174</v>
@@ -13070,9 +13117,36 @@
       <c r="C220" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O220" s="15" t="s">
-        <v>363</v>
-      </c>
+      <c r="D220" s="14"/>
+      <c r="E220" s="14"/>
+      <c r="F220" s="14"/>
+      <c r="G220" s="14"/>
+      <c r="H220" s="14"/>
+      <c r="I220" s="14"/>
+      <c r="J220" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K220" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L220" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M220" s="14"/>
+      <c r="N220" s="14"/>
+      <c r="O220" s="14"/>
+      <c r="P220" s="14"/>
+      <c r="Q220" s="14"/>
+      <c r="R220" s="14"/>
+      <c r="S220" s="14"/>
+      <c r="T220" s="14"/>
+      <c r="U220" s="14"/>
+      <c r="V220" s="14"/>
+      <c r="W220" s="14"/>
+      <c r="X220" s="14"/>
+      <c r="Y220" s="14"/>
+      <c r="Z220" s="14"/>
+      <c r="AA220" s="14"/>
       <c r="AB220" s="14"/>
       <c r="AC220" s="14"/>
       <c r="AD220" s="14"/>
@@ -13084,7 +13158,7 @@
     </row>
     <row r="221" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A221" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B221" s="14" t="s">
         <v>174</v>
@@ -13093,7 +13167,7 @@
         <v>135</v>
       </c>
       <c r="O221" s="15" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="AB221" s="14"/>
       <c r="AC221" s="14"/>
@@ -13106,7 +13180,7 @@
     </row>
     <row r="222" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A222" s="14" t="s">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="B222" s="14" t="s">
         <v>174</v>
@@ -13114,8 +13188,8 @@
       <c r="C222" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M222" s="14" t="s">
-        <v>371</v>
+      <c r="O222" s="15" t="s">
+        <v>363</v>
       </c>
       <c r="AB222" s="14"/>
       <c r="AC222" s="14"/>
@@ -13127,6 +13201,18 @@
       <c r="AI222" s="14"/>
     </row>
     <row r="223" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A223" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B223" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C223" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O223" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB223" s="14"/>
       <c r="AC223" s="14"/>
       <c r="AD223" s="14"/>
@@ -13137,6 +13223,18 @@
       <c r="AI223" s="14"/>
     </row>
     <row r="224" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A224" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B224" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C224" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M224" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB224" s="14"/>
       <c r="AC224" s="14"/>
       <c r="AD224" s="14"/>
@@ -14830,7 +14928,7 @@
       <c r="AB393" s="14"/>
       <c r="AC393" s="14"/>
       <c r="AD393" s="14"/>
-      <c r="AE393" s="14"/>
+      <c r="AE393" s="27"/>
       <c r="AF393" s="14"/>
       <c r="AG393" s="14"/>
       <c r="AH393" s="14"/>
@@ -14840,7 +14938,7 @@
       <c r="AB394" s="14"/>
       <c r="AC394" s="14"/>
       <c r="AD394" s="14"/>
-      <c r="AE394" s="14"/>
+      <c r="AE394" s="27"/>
       <c r="AF394" s="14"/>
       <c r="AG394" s="14"/>
       <c r="AH394" s="14"/>
@@ -14895,6 +14993,26 @@
       <c r="AG399" s="14"/>
       <c r="AH399" s="14"/>
       <c r="AI399" s="14"/>
+    </row>
+    <row r="400" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB400" s="14"/>
+      <c r="AC400" s="14"/>
+      <c r="AD400" s="14"/>
+      <c r="AE400" s="14"/>
+      <c r="AF400" s="14"/>
+      <c r="AG400" s="14"/>
+      <c r="AH400" s="14"/>
+      <c r="AI400" s="14"/>
+    </row>
+    <row r="401" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB401" s="14"/>
+      <c r="AC401" s="14"/>
+      <c r="AD401" s="14"/>
+      <c r="AE401" s="14"/>
+      <c r="AF401" s="14"/>
+      <c r="AG401" s="14"/>
+      <c r="AH401" s="14"/>
+      <c r="AI401" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
commit the updated file and script for 2 new scenarios added
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25629"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A60254E-AEC9-4624-9413-0E9C86CBB211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B843A1A5-0E46-4FC6-A0A6-B61D28C1C206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Commit after changes done for Testdata and x12 file and minor modify in 2 java clasess for L5 regression execution
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25629"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B843A1A5-0E46-4FC6-A0A6-B61D28C1C206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{975B38FE-400A-4A11-838C-05D019B1BA13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15390" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3059" uniqueCount="713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3113" uniqueCount="720">
   <si>
     <t>1</t>
   </si>
@@ -1977,9 +1977,6 @@
     <t>986</t>
   </si>
   <si>
-    <t>985|986</t>
-  </si>
-  <si>
     <t>Abaxis</t>
   </si>
   <si>
@@ -1998,9 +1995,6 @@
     <t>973|979</t>
   </si>
   <si>
-    <t>980|975</t>
-  </si>
-  <si>
     <t>982|983</t>
   </si>
   <si>
@@ -2076,97 +2070,124 @@
     <t>APC_OBScenario08</t>
   </si>
   <si>
+    <t>APC_OBScenario09</t>
+  </si>
+  <si>
+    <t>995</t>
+  </si>
+  <si>
+    <t>996</t>
+  </si>
+  <si>
+    <t>APC_OBScenario10</t>
+  </si>
+  <si>
+    <t>995|996</t>
+  </si>
+  <si>
+    <t>APC_OBScenario11</t>
+  </si>
+  <si>
+    <t>997</t>
+  </si>
+  <si>
+    <t>APC_OBScenario12</t>
+  </si>
+  <si>
+    <t>03P85-25</t>
+  </si>
+  <si>
+    <t>07P05-01</t>
+  </si>
+  <si>
+    <t>APC_OBScenario13</t>
+  </si>
+  <si>
+    <t>07P02-05</t>
+  </si>
+  <si>
+    <t>APC_IBScenario012</t>
+  </si>
+  <si>
+    <t>998</t>
+  </si>
+  <si>
+    <t>Dangerous</t>
+  </si>
+  <si>
+    <t>UNDA</t>
+  </si>
+  <si>
+    <t>UPSN</t>
+  </si>
+  <si>
+    <t>KWEWW</t>
+  </si>
+  <si>
+    <t>KWEO</t>
+  </si>
+  <si>
+    <t>APC_OBScenario14</t>
+  </si>
+  <si>
+    <t>999</t>
+  </si>
+  <si>
+    <t>APC_OBScenario15</t>
+  </si>
+  <si>
+    <t>APC_OBScenario16</t>
+  </si>
+  <si>
+    <t>APC_OBScenario17</t>
+  </si>
+  <si>
+    <t>APC_OBScenario18</t>
+  </si>
+  <si>
+    <t>APC_OBScenario19</t>
+  </si>
+  <si>
+    <t>APC_OBScenario20</t>
+  </si>
+  <si>
+    <t>FEIP</t>
+  </si>
+  <si>
+    <t>QSC_DailyRegressionOB12</t>
+  </si>
+  <si>
+    <t>112|113|114|115</t>
+  </si>
+  <si>
+    <t>1000</t>
+  </si>
+  <si>
+    <t>988|986</t>
+  </si>
+  <si>
+    <t>06P28-01</t>
+  </si>
+  <si>
     <t>988|994</t>
   </si>
   <si>
-    <t>APC_OBScenario09</t>
-  </si>
-  <si>
-    <t>995</t>
-  </si>
-  <si>
-    <t>996</t>
-  </si>
-  <si>
-    <t>APC_OBScenario10</t>
-  </si>
-  <si>
-    <t>995|996</t>
-  </si>
-  <si>
-    <t>APC_OBScenario11</t>
-  </si>
-  <si>
-    <t>997</t>
-  </si>
-  <si>
-    <t>APC_OBScenario12</t>
-  </si>
-  <si>
-    <t>03P85-25</t>
-  </si>
-  <si>
-    <t>07P05-01</t>
-  </si>
-  <si>
-    <t>APC_OBScenario13</t>
-  </si>
-  <si>
-    <t>07P02-05</t>
-  </si>
-  <si>
-    <t>APC_IBScenario012</t>
-  </si>
-  <si>
-    <t>998</t>
-  </si>
-  <si>
-    <t>Dangerous</t>
-  </si>
-  <si>
-    <t>UNDA</t>
-  </si>
-  <si>
-    <t>UPSN</t>
-  </si>
-  <si>
-    <t>KWEWW</t>
-  </si>
-  <si>
-    <t>KWEO</t>
-  </si>
-  <si>
-    <t>APC_OBScenario14</t>
-  </si>
-  <si>
-    <t>999</t>
-  </si>
-  <si>
-    <t>APC_OBScenario15</t>
-  </si>
-  <si>
-    <t>APC_OBScenario16</t>
-  </si>
-  <si>
-    <t>APC_OBScenario17</t>
-  </si>
-  <si>
-    <t>APC_OBScenario18</t>
-  </si>
-  <si>
-    <t>APC_OBScenario19</t>
-  </si>
-  <si>
-    <t>APC_OBScenario20</t>
-  </si>
-  <si>
-    <t>FEIP</t>
-  </si>
-  <si>
-    <t>QSC_DailyRegressionOB12</t>
-  </si>
-  <si>
-    <t>112|113|114|115</t>
+    <t>1001</t>
+  </si>
+  <si>
+    <t>013407-01 02</t>
+  </si>
+  <si>
+    <t>1002</t>
+  </si>
+  <si>
+    <t>APC_OBScenario21</t>
+  </si>
+  <si>
+    <t>1003</t>
+  </si>
+  <si>
+    <t>980|1003</t>
   </si>
 </sst>
 </file>
@@ -2710,7 +2731,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI401"/>
+  <dimension ref="A1:AI402"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -6481,7 +6502,7 @@
     </row>
     <row r="82" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="14" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="B82" s="14" t="s">
         <v>107</v>
@@ -6490,7 +6511,7 @@
         <v>135</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="E82" s="14"/>
       <c r="F82" s="14"/>
@@ -7102,7 +7123,7 @@
       <c r="AC95" s="14"/>
       <c r="AD95" s="14"/>
       <c r="AE95" s="27" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="AF95" s="14"/>
       <c r="AG95" s="14"/>
@@ -11350,7 +11371,7 @@
       <c r="AC185" s="14"/>
       <c r="AD185" s="14"/>
       <c r="AE185" s="27" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="AF185" s="14"/>
       <c r="AG185" s="14"/>
@@ -11370,7 +11391,7 @@
         <v>614</v>
       </c>
       <c r="D186" s="18" t="s">
-        <v>621</v>
+        <v>710</v>
       </c>
       <c r="E186" s="14"/>
       <c r="F186" s="14"/>
@@ -11401,7 +11422,7 @@
       <c r="AC186" s="14"/>
       <c r="AD186" s="14"/>
       <c r="AE186" s="27" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="AF186" s="14"/>
       <c r="AG186" s="14"/>
@@ -11452,7 +11473,7 @@
       <c r="AC187" s="14"/>
       <c r="AD187" s="14"/>
       <c r="AE187" s="27" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="AF187" s="14"/>
       <c r="AG187" s="14"/>
@@ -11472,7 +11493,7 @@
         <v>614</v>
       </c>
       <c r="D188" s="18" t="s">
-        <v>628</v>
+        <v>714</v>
       </c>
       <c r="E188" s="14"/>
       <c r="F188" s="14"/>
@@ -11503,7 +11524,7 @@
       <c r="AC188" s="14"/>
       <c r="AD188" s="14"/>
       <c r="AE188" s="27" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="AF188" s="14"/>
       <c r="AG188" s="14"/>
@@ -11554,7 +11575,7 @@
       <c r="AC189" s="14"/>
       <c r="AD189" s="14"/>
       <c r="AE189" s="27" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="AF189" s="14"/>
       <c r="AG189" s="14"/>
@@ -11605,7 +11626,7 @@
       <c r="AC190" s="14"/>
       <c r="AD190" s="14"/>
       <c r="AE190" s="27" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="AF190" s="14"/>
       <c r="AG190" s="14"/>
@@ -11625,7 +11646,7 @@
         <v>614</v>
       </c>
       <c r="D191" s="18" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="E191" s="14"/>
       <c r="F191" s="14"/>
@@ -11656,7 +11677,7 @@
       <c r="AC191" s="14"/>
       <c r="AD191" s="14"/>
       <c r="AE191" s="27" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="AF191" s="14"/>
       <c r="AG191" s="14"/>
@@ -11676,7 +11697,7 @@
         <v>614</v>
       </c>
       <c r="D192" s="18" t="s">
-        <v>649</v>
+        <v>711</v>
       </c>
       <c r="E192" s="14"/>
       <c r="F192" s="14"/>
@@ -11707,7 +11728,7 @@
       <c r="AC192" s="14"/>
       <c r="AD192" s="14"/>
       <c r="AE192" s="27" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="AF192" s="14"/>
       <c r="AG192" s="14"/>
@@ -11727,7 +11748,7 @@
         <v>614</v>
       </c>
       <c r="D193" s="18" t="s">
-        <v>656</v>
+        <v>719</v>
       </c>
       <c r="E193" s="14"/>
       <c r="F193" s="14"/>
@@ -11758,7 +11779,7 @@
       <c r="AC193" s="14"/>
       <c r="AD193" s="14"/>
       <c r="AE193" s="27" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="AF193" s="14"/>
       <c r="AG193" s="14"/>
@@ -11778,7 +11799,7 @@
         <v>614</v>
       </c>
       <c r="D194" s="18" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="E194" s="14"/>
       <c r="F194" s="14"/>
@@ -11809,7 +11830,7 @@
       <c r="AC194" s="14"/>
       <c r="AD194" s="14"/>
       <c r="AE194" s="27" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="AF194" s="14"/>
       <c r="AG194" s="14"/>
@@ -11827,7 +11848,7 @@
         <v>614</v>
       </c>
       <c r="D195" s="18" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="E195" s="14"/>
       <c r="F195" s="14"/>
@@ -11858,7 +11879,7 @@
       <c r="AC195" s="14"/>
       <c r="AD195" s="14"/>
       <c r="AE195" s="27" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="AF195" s="14"/>
       <c r="AG195" s="14"/>
@@ -11869,7 +11890,7 @@
     </row>
     <row r="196" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="14" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
       <c r="B196" s="14" t="s">
         <v>613</v>
@@ -11878,7 +11899,7 @@
         <v>614</v>
       </c>
       <c r="D196" s="18" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="E196" s="14"/>
       <c r="F196" s="14"/>
@@ -11909,7 +11930,7 @@
       <c r="AC196" s="14"/>
       <c r="AD196" s="14"/>
       <c r="AE196" s="27" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="AF196" s="14"/>
       <c r="AG196" s="14"/>
@@ -11957,7 +11978,7 @@
     </row>
     <row r="198" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="14" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="B198" s="14" t="s">
         <v>613</v>
@@ -11966,7 +11987,7 @@
         <v>614</v>
       </c>
       <c r="D198" s="23" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="E198" s="14"/>
       <c r="F198" s="14"/>
@@ -12010,7 +12031,7 @@
     </row>
     <row r="199" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="14" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B199" s="14" t="s">
         <v>613</v>
@@ -12019,7 +12040,7 @@
         <v>614</v>
       </c>
       <c r="D199" s="23" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="E199" s="14"/>
       <c r="F199" s="14"/>
@@ -12061,7 +12082,7 @@
     </row>
     <row r="200" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="14" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B200" s="14" t="s">
         <v>613</v>
@@ -12070,7 +12091,7 @@
         <v>614</v>
       </c>
       <c r="D200" s="23" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="E200" s="14"/>
       <c r="F200" s="14"/>
@@ -12114,7 +12135,7 @@
     </row>
     <row r="201" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="14" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B201" s="14" t="s">
         <v>613</v>
@@ -12123,7 +12144,7 @@
         <v>614</v>
       </c>
       <c r="D201" s="23" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="E201" s="14"/>
       <c r="F201" s="14"/>
@@ -12167,7 +12188,7 @@
     </row>
     <row r="202" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="14" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B202" s="14" t="s">
         <v>613</v>
@@ -12176,7 +12197,7 @@
         <v>614</v>
       </c>
       <c r="D202" s="23" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="E202" s="14"/>
       <c r="F202" s="14"/>
@@ -12220,7 +12241,7 @@
     </row>
     <row r="203" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="14" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="B203" s="14" t="s">
         <v>613</v>
@@ -12229,7 +12250,7 @@
         <v>614</v>
       </c>
       <c r="D203" s="23" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="E203" s="14"/>
       <c r="F203" s="14"/>
@@ -12273,7 +12294,7 @@
     </row>
     <row r="204" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A204" s="14" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="B204" s="14" t="s">
         <v>613</v>
@@ -12282,7 +12303,7 @@
         <v>614</v>
       </c>
       <c r="D204" s="18" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="E204" s="14"/>
       <c r="F204" s="14"/>
@@ -12326,7 +12347,7 @@
     </row>
     <row r="205" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="14" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="B205" s="14" t="s">
         <v>613</v>
@@ -12335,7 +12356,7 @@
         <v>614</v>
       </c>
       <c r="D205" s="18" t="s">
-        <v>682</v>
+        <v>713</v>
       </c>
       <c r="E205" s="14"/>
       <c r="F205" s="14"/>
@@ -12369,7 +12390,9 @@
       <c r="AD205" s="14" t="s">
         <v>451</v>
       </c>
-      <c r="AE205" s="27"/>
+      <c r="AE205" s="27" t="s">
+        <v>650</v>
+      </c>
       <c r="AF205" s="14"/>
       <c r="AG205" s="14"/>
       <c r="AH205" s="14" t="s">
@@ -12379,7 +12402,7 @@
     </row>
     <row r="206" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="14" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="B206" s="14" t="s">
         <v>613</v>
@@ -12388,7 +12411,7 @@
         <v>614</v>
       </c>
       <c r="D206" s="18" t="s">
-        <v>682</v>
+        <v>713</v>
       </c>
       <c r="E206" s="14"/>
       <c r="F206" s="14"/>
@@ -12422,7 +12445,9 @@
       <c r="AD206" s="14" t="s">
         <v>421</v>
       </c>
-      <c r="AE206" s="27"/>
+      <c r="AE206" s="27" t="s">
+        <v>650</v>
+      </c>
       <c r="AF206" s="14"/>
       <c r="AG206" s="14"/>
       <c r="AH206" s="14" t="s">
@@ -12432,7 +12457,7 @@
     </row>
     <row r="207" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="14" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="B207" s="14" t="s">
         <v>613</v>
@@ -12441,7 +12466,7 @@
         <v>614</v>
       </c>
       <c r="D207" s="18" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="E207" s="14"/>
       <c r="F207" s="14"/>
@@ -12485,7 +12510,7 @@
     </row>
     <row r="208" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="14" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="B208" s="14" t="s">
         <v>613</v>
@@ -12494,7 +12519,7 @@
         <v>614</v>
       </c>
       <c r="D208" s="18" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="E208" s="14"/>
       <c r="F208" s="14"/>
@@ -12538,7 +12563,7 @@
     </row>
     <row r="209" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="14" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="B209" s="14" t="s">
         <v>613</v>
@@ -12547,7 +12572,7 @@
         <v>614</v>
       </c>
       <c r="D209" s="23" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="E209" s="14"/>
       <c r="F209" s="14"/>
@@ -12582,7 +12607,7 @@
         <v>421</v>
       </c>
       <c r="AE209" s="27" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="AF209" s="14"/>
       <c r="AG209" s="14"/>
@@ -12593,7 +12618,7 @@
     </row>
     <row r="210" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210" s="14" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="B210" s="14" t="s">
         <v>613</v>
@@ -12602,7 +12627,7 @@
         <v>614</v>
       </c>
       <c r="D210" s="23" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="E210" s="14"/>
       <c r="F210" s="14"/>
@@ -12637,7 +12662,7 @@
         <v>451</v>
       </c>
       <c r="AE210" s="27" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="AF210" s="14"/>
       <c r="AG210" s="14"/>
@@ -12648,7 +12673,7 @@
     </row>
     <row r="211" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="14" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="B211" s="14" t="s">
         <v>613</v>
@@ -12692,7 +12717,7 @@
         <v>451</v>
       </c>
       <c r="AE211" s="27" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="AF211" s="14"/>
       <c r="AG211" s="14"/>
@@ -12703,7 +12728,7 @@
     </row>
     <row r="212" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="14" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="B212" s="14" t="s">
         <v>613</v>
@@ -12712,7 +12737,7 @@
         <v>614</v>
       </c>
       <c r="D212" s="18" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="E212" s="14"/>
       <c r="F212" s="14"/>
@@ -12747,7 +12772,7 @@
         <v>451</v>
       </c>
       <c r="AE212" s="27" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="AF212" s="14"/>
       <c r="AG212" s="14"/>
@@ -12758,7 +12783,7 @@
     </row>
     <row r="213" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A213" s="14" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="B213" s="14" t="s">
         <v>613</v>
@@ -12767,7 +12792,7 @@
         <v>614</v>
       </c>
       <c r="D213" s="18" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="E213" s="14"/>
       <c r="F213" s="14"/>
@@ -12796,10 +12821,10 @@
         <v>419</v>
       </c>
       <c r="AC213" s="14" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="AD213" s="14" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="AE213" s="27"/>
       <c r="AF213" s="14"/>
@@ -12809,7 +12834,7 @@
     </row>
     <row r="214" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A214" s="14" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="B214" s="14" t="s">
         <v>613</v>
@@ -12818,7 +12843,7 @@
         <v>614</v>
       </c>
       <c r="D214" s="18" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="E214" s="14"/>
       <c r="F214" s="14"/>
@@ -12847,13 +12872,13 @@
         <v>393</v>
       </c>
       <c r="AC214" s="14" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="AD214" s="14" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="AE214" s="27" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="AF214" s="14"/>
       <c r="AG214" s="14"/>
@@ -12862,7 +12887,7 @@
     </row>
     <row r="215" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A215" s="14" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="B215" s="14" t="s">
         <v>613</v>
@@ -12900,13 +12925,13 @@
         <v>419</v>
       </c>
       <c r="AC215" s="14" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="AD215" s="14" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="AE215" s="27" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="AF215" s="14"/>
       <c r="AG215" s="14"/>
@@ -12915,7 +12940,7 @@
     </row>
     <row r="216" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A216" s="14" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="B216" s="14" t="s">
         <v>613</v>
@@ -12924,7 +12949,7 @@
         <v>614</v>
       </c>
       <c r="D216" s="18" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="E216" s="14"/>
       <c r="F216" s="14"/>
@@ -12959,7 +12984,7 @@
         <v>421</v>
       </c>
       <c r="AE216" s="27" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="AF216" s="14"/>
       <c r="AG216" s="14"/>
@@ -12970,7 +12995,7 @@
     </row>
     <row r="217" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A217" s="14" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="B217" s="14" t="s">
         <v>613</v>
@@ -12979,7 +13004,7 @@
         <v>614</v>
       </c>
       <c r="D217" s="18" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="E217" s="14"/>
       <c r="F217" s="14"/>
@@ -13008,13 +13033,13 @@
         <v>419</v>
       </c>
       <c r="AC217" s="14" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="AD217" s="14" t="s">
         <v>451</v>
       </c>
       <c r="AE217" s="27" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="AF217" s="14"/>
       <c r="AG217" s="14"/>
@@ -13022,10 +13047,18 @@
       <c r="AI217" s="14"/>
     </row>
     <row r="218" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A218" s="14"/>
-      <c r="B218" s="14"/>
-      <c r="C218" s="14"/>
-      <c r="D218" s="14"/>
+      <c r="A218" s="14" t="s">
+        <v>717</v>
+      </c>
+      <c r="B218" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C218" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D218" s="18" t="s">
+        <v>716</v>
+      </c>
       <c r="E218" s="14"/>
       <c r="F218" s="14"/>
       <c r="G218" s="14"/>
@@ -13049,40 +13082,38 @@
       <c r="Y218" s="14"/>
       <c r="Z218" s="14"/>
       <c r="AA218" s="14"/>
-      <c r="AB218" s="14"/>
-      <c r="AC218" s="14"/>
-      <c r="AD218" s="14"/>
-      <c r="AE218" s="27"/>
+      <c r="AB218" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC218" s="14" t="s">
+        <v>420</v>
+      </c>
+      <c r="AD218" s="14" t="s">
+        <v>421</v>
+      </c>
+      <c r="AE218" s="27" t="s">
+        <v>653</v>
+      </c>
       <c r="AF218" s="14"/>
       <c r="AG218" s="14"/>
-      <c r="AH218" s="14"/>
+      <c r="AH218" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI218" s="14"/>
     </row>
     <row r="219" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A219" s="14" t="s">
-        <v>267</v>
-      </c>
-      <c r="B219" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C219" s="14" t="s">
-        <v>135</v>
-      </c>
+      <c r="A219" s="14"/>
+      <c r="B219" s="14"/>
+      <c r="C219" s="14"/>
       <c r="D219" s="14"/>
       <c r="E219" s="14"/>
       <c r="F219" s="14"/>
       <c r="G219" s="14"/>
       <c r="H219" s="14"/>
       <c r="I219" s="14"/>
-      <c r="J219" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K219" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L219" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J219" s="14"/>
+      <c r="K219" s="14"/>
+      <c r="L219" s="14"/>
       <c r="M219" s="14"/>
       <c r="N219" s="14"/>
       <c r="O219" s="14"/>
@@ -13109,7 +13140,7 @@
     </row>
     <row r="220" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A220" s="14" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B220" s="14" t="s">
         <v>174</v>
@@ -13124,13 +13155,13 @@
       <c r="H220" s="14"/>
       <c r="I220" s="14"/>
       <c r="J220" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K220" s="15" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="L220" s="15" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="M220" s="14"/>
       <c r="N220" s="14"/>
@@ -13156,9 +13187,9 @@
       <c r="AH220" s="14"/>
       <c r="AI220" s="14"/>
     </row>
-    <row r="221" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A221" s="14" t="s">
-        <v>359</v>
+        <v>268</v>
       </c>
       <c r="B221" s="14" t="s">
         <v>174</v>
@@ -13166,9 +13197,36 @@
       <c r="C221" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O221" s="15" t="s">
-        <v>362</v>
-      </c>
+      <c r="D221" s="14"/>
+      <c r="E221" s="14"/>
+      <c r="F221" s="14"/>
+      <c r="G221" s="14"/>
+      <c r="H221" s="14"/>
+      <c r="I221" s="14"/>
+      <c r="J221" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K221" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L221" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M221" s="14"/>
+      <c r="N221" s="14"/>
+      <c r="O221" s="14"/>
+      <c r="P221" s="14"/>
+      <c r="Q221" s="14"/>
+      <c r="R221" s="14"/>
+      <c r="S221" s="14"/>
+      <c r="T221" s="14"/>
+      <c r="U221" s="14"/>
+      <c r="V221" s="14"/>
+      <c r="W221" s="14"/>
+      <c r="X221" s="14"/>
+      <c r="Y221" s="14"/>
+      <c r="Z221" s="14"/>
+      <c r="AA221" s="14"/>
       <c r="AB221" s="14"/>
       <c r="AC221" s="14"/>
       <c r="AD221" s="14"/>
@@ -13180,7 +13238,7 @@
     </row>
     <row r="222" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A222" s="14" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B222" s="14" t="s">
         <v>174</v>
@@ -13189,7 +13247,7 @@
         <v>135</v>
       </c>
       <c r="O222" s="15" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AB222" s="14"/>
       <c r="AC222" s="14"/>
@@ -13202,7 +13260,7 @@
     </row>
     <row r="223" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A223" s="14" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B223" s="14" t="s">
         <v>174</v>
@@ -13211,7 +13269,7 @@
         <v>135</v>
       </c>
       <c r="O223" s="15" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AB223" s="14"/>
       <c r="AC223" s="14"/>
@@ -13224,7 +13282,7 @@
     </row>
     <row r="224" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A224" s="14" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="B224" s="14" t="s">
         <v>174</v>
@@ -13232,8 +13290,8 @@
       <c r="C224" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M224" s="14" t="s">
-        <v>371</v>
+      <c r="O224" s="15" t="s">
+        <v>364</v>
       </c>
       <c r="AB224" s="14"/>
       <c r="AC224" s="14"/>
@@ -13244,7 +13302,19 @@
       <c r="AH224" s="14"/>
       <c r="AI224" s="14"/>
     </row>
-    <row r="225" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A225" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B225" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C225" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M225" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB225" s="14"/>
       <c r="AC225" s="14"/>
       <c r="AD225" s="14"/>
@@ -13254,7 +13324,7 @@
       <c r="AH225" s="14"/>
       <c r="AI225" s="14"/>
     </row>
-    <row r="226" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB226" s="14"/>
       <c r="AC226" s="14"/>
       <c r="AD226" s="14"/>
@@ -13264,7 +13334,7 @@
       <c r="AH226" s="14"/>
       <c r="AI226" s="14"/>
     </row>
-    <row r="227" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB227" s="14"/>
       <c r="AC227" s="14"/>
       <c r="AD227" s="14"/>
@@ -13274,7 +13344,7 @@
       <c r="AH227" s="14"/>
       <c r="AI227" s="14"/>
     </row>
-    <row r="228" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB228" s="14"/>
       <c r="AC228" s="14"/>
       <c r="AD228" s="14"/>
@@ -13284,7 +13354,7 @@
       <c r="AH228" s="14"/>
       <c r="AI228" s="14"/>
     </row>
-    <row r="229" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB229" s="14"/>
       <c r="AC229" s="14"/>
       <c r="AD229" s="14"/>
@@ -13294,7 +13364,7 @@
       <c r="AH229" s="14"/>
       <c r="AI229" s="14"/>
     </row>
-    <row r="230" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB230" s="14"/>
       <c r="AC230" s="14"/>
       <c r="AD230" s="14"/>
@@ -13304,7 +13374,7 @@
       <c r="AH230" s="14"/>
       <c r="AI230" s="14"/>
     </row>
-    <row r="231" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB231" s="14"/>
       <c r="AC231" s="14"/>
       <c r="AD231" s="14"/>
@@ -13314,7 +13384,7 @@
       <c r="AH231" s="14"/>
       <c r="AI231" s="14"/>
     </row>
-    <row r="232" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB232" s="14"/>
       <c r="AC232" s="14"/>
       <c r="AD232" s="14"/>
@@ -13324,7 +13394,7 @@
       <c r="AH232" s="14"/>
       <c r="AI232" s="14"/>
     </row>
-    <row r="233" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB233" s="14"/>
       <c r="AC233" s="14"/>
       <c r="AD233" s="14"/>
@@ -13334,7 +13404,7 @@
       <c r="AH233" s="14"/>
       <c r="AI233" s="14"/>
     </row>
-    <row r="234" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB234" s="14"/>
       <c r="AC234" s="14"/>
       <c r="AD234" s="14"/>
@@ -13344,7 +13414,7 @@
       <c r="AH234" s="14"/>
       <c r="AI234" s="14"/>
     </row>
-    <row r="235" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB235" s="14"/>
       <c r="AC235" s="14"/>
       <c r="AD235" s="14"/>
@@ -13354,7 +13424,7 @@
       <c r="AH235" s="14"/>
       <c r="AI235" s="14"/>
     </row>
-    <row r="236" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB236" s="14"/>
       <c r="AC236" s="14"/>
       <c r="AD236" s="14"/>
@@ -13364,7 +13434,7 @@
       <c r="AH236" s="14"/>
       <c r="AI236" s="14"/>
     </row>
-    <row r="237" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB237" s="14"/>
       <c r="AC237" s="14"/>
       <c r="AD237" s="14"/>
@@ -13374,7 +13444,7 @@
       <c r="AH237" s="14"/>
       <c r="AI237" s="14"/>
     </row>
-    <row r="238" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB238" s="14"/>
       <c r="AC238" s="14"/>
       <c r="AD238" s="14"/>
@@ -13384,7 +13454,7 @@
       <c r="AH238" s="14"/>
       <c r="AI238" s="14"/>
     </row>
-    <row r="239" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB239" s="14"/>
       <c r="AC239" s="14"/>
       <c r="AD239" s="14"/>
@@ -13394,7 +13464,7 @@
       <c r="AH239" s="14"/>
       <c r="AI239" s="14"/>
     </row>
-    <row r="240" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB240" s="14"/>
       <c r="AC240" s="14"/>
       <c r="AD240" s="14"/>
@@ -14948,7 +15018,7 @@
       <c r="AB395" s="14"/>
       <c r="AC395" s="14"/>
       <c r="AD395" s="14"/>
-      <c r="AE395" s="14"/>
+      <c r="AE395" s="27"/>
       <c r="AF395" s="14"/>
       <c r="AG395" s="14"/>
       <c r="AH395" s="14"/>
@@ -15014,6 +15084,16 @@
       <c r="AH401" s="14"/>
       <c r="AI401" s="14"/>
     </row>
+    <row r="402" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB402" s="14"/>
+      <c r="AC402" s="14"/>
+      <c r="AD402" s="14"/>
+      <c r="AE402" s="14"/>
+      <c r="AF402" s="14"/>
+      <c r="AG402" s="14"/>
+      <c r="AH402" s="14"/>
+      <c r="AI402" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15023,7 +15103,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T214"/>
+  <dimension ref="A1:T218"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -21126,16 +21206,16 @@
         <v>615</v>
       </c>
       <c r="B187" s="20" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="C187" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D187" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E187" s="15" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F187" s="15"/>
       <c r="G187" s="15"/>
@@ -21158,16 +21238,16 @@
         <v>618</v>
       </c>
       <c r="B188" s="20" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="C188" s="15" t="s">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="D188" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E188" s="15" t="s">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="F188" s="15"/>
       <c r="G188" s="15"/>
@@ -21192,7 +21272,7 @@
         <v>621</v>
       </c>
       <c r="B189" s="20" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="C189" s="15" t="s">
         <v>2</v>
@@ -21294,7 +21374,7 @@
         <v>629</v>
       </c>
       <c r="B192" s="20" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="C192" s="15" t="s">
         <v>0</v>
@@ -21328,7 +21408,7 @@
         <v>630</v>
       </c>
       <c r="B193" s="20" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="C193" s="15" t="s">
         <v>2</v>
@@ -21362,7 +21442,7 @@
         <v>634</v>
       </c>
       <c r="B194" s="20" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
       <c r="C194" s="15" t="s">
         <v>0</v>
@@ -21399,13 +21479,13 @@
         <v>637</v>
       </c>
       <c r="C195" s="15" t="s">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="D195" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E195" s="15" t="s">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="F195" s="15"/>
       <c r="G195" s="15"/>
@@ -21414,7 +21494,9 @@
         <v>624</v>
       </c>
       <c r="J195" s="14"/>
-      <c r="K195" s="14"/>
+      <c r="K195" s="14" t="s">
+        <v>134</v>
+      </c>
       <c r="L195" s="14"/>
       <c r="M195" s="14"/>
       <c r="N195" s="14"/>
@@ -21464,7 +21546,7 @@
         <v>641</v>
       </c>
       <c r="B197" s="20" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="C197" s="15" t="s">
         <v>2</v>
@@ -21498,7 +21580,7 @@
         <v>642</v>
       </c>
       <c r="B198" s="20" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="C198" s="15" t="s">
         <v>2</v>
@@ -21566,7 +21648,7 @@
         <v>647</v>
       </c>
       <c r="B200" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="C200" s="15" t="s">
         <v>2</v>
@@ -21600,16 +21682,16 @@
         <v>648</v>
       </c>
       <c r="B201" s="20" t="s">
-        <v>660</v>
+        <v>712</v>
       </c>
       <c r="C201" s="15" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="D201" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E201" s="15" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="F201" s="15"/>
       <c r="G201" s="15"/>
@@ -21618,7 +21700,9 @@
         <v>624</v>
       </c>
       <c r="J201" s="14"/>
-      <c r="K201" s="14"/>
+      <c r="K201" s="14" t="s">
+        <v>134</v>
+      </c>
       <c r="L201" s="14"/>
       <c r="M201" s="14"/>
       <c r="N201" s="14"/>
@@ -21631,7 +21715,7 @@
     </row>
     <row r="202" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="15" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="B202" s="20" t="s">
         <v>631</v>
@@ -21665,22 +21749,26 @@
     </row>
     <row r="203" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="16" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="B203" s="20" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="C203" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D203" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="E203" s="14"/>
+      <c r="E203" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="F203" s="14"/>
       <c r="G203" s="14"/>
       <c r="H203" s="14"/>
-      <c r="I203" s="14"/>
+      <c r="I203" s="14" t="s">
+        <v>624</v>
+      </c>
       <c r="J203" s="14"/>
       <c r="K203" s="14" t="s">
         <v>134</v>
@@ -21703,10 +21791,10 @@
     </row>
     <row r="204" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A204" s="15" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="B204" s="20" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="C204" s="15" t="s">
         <v>0</v>
@@ -21735,13 +21823,13 @@
     </row>
     <row r="205" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="15" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="B205" s="20" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="C205" s="15" t="s">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="D205" s="16" t="s">
         <v>632</v>
@@ -21767,7 +21855,7 @@
     </row>
     <row r="206" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="15" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="B206" s="20" t="s">
         <v>637</v>
@@ -21799,13 +21887,13 @@
     </row>
     <row r="207" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="15" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="B207" s="20" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="C207" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D207" s="14" t="s">
         <v>112</v>
@@ -21831,10 +21919,10 @@
     </row>
     <row r="208" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="15" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="B208" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="C208" s="15" t="s">
         <v>2</v>
@@ -21850,7 +21938,9 @@
         <v>624</v>
       </c>
       <c r="J208" s="14"/>
-      <c r="K208" s="14"/>
+      <c r="K208" s="14" t="s">
+        <v>134</v>
+      </c>
       <c r="L208" s="14"/>
       <c r="M208" s="14"/>
       <c r="N208" s="14"/>
@@ -21863,18 +21953,20 @@
     </row>
     <row r="209" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="15" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="B209" s="20" t="s">
-        <v>660</v>
+        <v>712</v>
       </c>
       <c r="C209" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D209" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="E209" s="15"/>
+      <c r="E209" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="F209" s="15"/>
       <c r="G209" s="15"/>
       <c r="H209" s="15"/>
@@ -21882,7 +21974,9 @@
         <v>624</v>
       </c>
       <c r="J209" s="14"/>
-      <c r="K209" s="14"/>
+      <c r="K209" s="14" t="s">
+        <v>134</v>
+      </c>
       <c r="L209" s="14"/>
       <c r="M209" s="14"/>
       <c r="N209" s="14"/>
@@ -21895,10 +21989,10 @@
     </row>
     <row r="210" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210" s="15" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="B210" s="20" t="s">
-        <v>692</v>
+        <v>689</v>
       </c>
       <c r="C210" s="15" t="s">
         <v>0</v>
@@ -21906,7 +22000,9 @@
       <c r="D210" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="E210" s="15"/>
+      <c r="E210" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="F210" s="15"/>
       <c r="G210" s="15"/>
       <c r="H210" s="15"/>
@@ -21914,7 +22010,9 @@
         <v>624</v>
       </c>
       <c r="J210" s="14"/>
-      <c r="K210" s="14"/>
+      <c r="K210" s="14" t="s">
+        <v>134</v>
+      </c>
       <c r="L210" s="14"/>
       <c r="M210" s="14"/>
       <c r="N210" s="14"/>
@@ -21927,7 +22025,7 @@
     </row>
     <row r="211" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="15" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="B211" s="20" t="s">
         <v>637</v>
@@ -21938,7 +22036,9 @@
       <c r="D211" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="E211" s="15"/>
+      <c r="E211" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="F211" s="15"/>
       <c r="G211" s="15"/>
       <c r="H211" s="15"/>
@@ -21946,7 +22046,9 @@
         <v>624</v>
       </c>
       <c r="J211" s="14"/>
-      <c r="K211" s="14"/>
+      <c r="K211" s="14" t="s">
+        <v>134</v>
+      </c>
       <c r="L211" s="14"/>
       <c r="M211" s="14"/>
       <c r="N211" s="14"/>
@@ -21959,10 +22061,10 @@
     </row>
     <row r="212" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="15" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
       <c r="B212" s="20" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="C212" s="15" t="s">
         <v>0</v>
@@ -21991,10 +22093,10 @@
     </row>
     <row r="213" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A213" s="15" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="B213" s="20" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="C213" s="15" t="s">
         <v>0</v>
@@ -22012,7 +22114,9 @@
         <v>624</v>
       </c>
       <c r="J213" s="14"/>
-      <c r="K213" s="14"/>
+      <c r="K213" s="14" t="s">
+        <v>134</v>
+      </c>
       <c r="L213" s="14"/>
       <c r="M213" s="14"/>
       <c r="N213" s="14"/>
@@ -22025,10 +22129,10 @@
     </row>
     <row r="214" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A214" s="15" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="B214" s="30" t="s">
-        <v>658</v>
+        <v>715</v>
       </c>
       <c r="C214" s="15" t="s">
         <v>0</v>
@@ -22036,7 +22140,9 @@
       <c r="D214" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="E214" s="15"/>
+      <c r="E214" s="15" t="s">
+        <v>0</v>
+      </c>
       <c r="F214" s="15"/>
       <c r="G214" s="15"/>
       <c r="H214" s="15"/>
@@ -22044,7 +22150,9 @@
         <v>624</v>
       </c>
       <c r="J214" s="14"/>
-      <c r="K214" s="14"/>
+      <c r="K214" s="14" t="s">
+        <v>134</v>
+      </c>
       <c r="L214" s="14"/>
       <c r="M214" s="14"/>
       <c r="N214" s="14"/>
@@ -22054,6 +22162,152 @@
       <c r="R214" s="14"/>
       <c r="S214" s="14"/>
       <c r="T214" s="14"/>
+    </row>
+    <row r="215" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A215" s="16" t="s">
+        <v>710</v>
+      </c>
+      <c r="B215" s="20" t="s">
+        <v>666</v>
+      </c>
+      <c r="C215" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D215" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="E215" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="F215" s="14"/>
+      <c r="G215" s="14"/>
+      <c r="H215" s="14"/>
+      <c r="I215" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J215" s="14"/>
+      <c r="K215" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L215" s="14"/>
+      <c r="M215" s="14"/>
+      <c r="N215" s="14"/>
+      <c r="O215" s="14"/>
+      <c r="P215" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q215" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R215" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S215" s="14"/>
+      <c r="T215" s="14"/>
+    </row>
+    <row r="216" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A216" s="15" t="s">
+        <v>714</v>
+      </c>
+      <c r="B216" s="20" t="s">
+        <v>631</v>
+      </c>
+      <c r="C216" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D216" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E216" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="F216" s="15"/>
+      <c r="G216" s="15"/>
+      <c r="H216" s="15"/>
+      <c r="I216" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J216" s="14"/>
+      <c r="K216" s="14"/>
+      <c r="L216" s="14"/>
+      <c r="M216" s="14"/>
+      <c r="N216" s="14"/>
+      <c r="O216" s="14"/>
+      <c r="P216" s="14"/>
+      <c r="Q216" s="14"/>
+      <c r="R216" s="14"/>
+      <c r="S216" s="14"/>
+      <c r="T216" s="14"/>
+    </row>
+    <row r="217" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A217" s="15" t="s">
+        <v>716</v>
+      </c>
+      <c r="B217" s="20" t="s">
+        <v>656</v>
+      </c>
+      <c r="C217" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D217" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E217" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F217" s="15"/>
+      <c r="G217" s="15"/>
+      <c r="H217" s="15"/>
+      <c r="I217" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J217" s="14"/>
+      <c r="K217" s="14"/>
+      <c r="L217" s="14"/>
+      <c r="M217" s="14"/>
+      <c r="N217" s="14"/>
+      <c r="O217" s="14"/>
+      <c r="P217" s="14"/>
+      <c r="Q217" s="14"/>
+      <c r="R217" s="14"/>
+      <c r="S217" s="14"/>
+      <c r="T217" s="14"/>
+    </row>
+    <row r="218" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A218" s="15" t="s">
+        <v>718</v>
+      </c>
+      <c r="B218" s="20" t="s">
+        <v>689</v>
+      </c>
+      <c r="C218" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D218" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E218" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F218" s="15"/>
+      <c r="G218" s="15"/>
+      <c r="H218" s="15"/>
+      <c r="I218" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J218" s="14"/>
+      <c r="K218" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L218" s="14"/>
+      <c r="M218" s="14"/>
+      <c r="N218" s="14"/>
+      <c r="O218" s="14"/>
+      <c r="P218" s="14"/>
+      <c r="Q218" s="14"/>
+      <c r="R218" s="14"/>
+      <c r="S218" s="14"/>
+      <c r="T218" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
commit code for O2S create order scenarios script
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{975B38FE-400A-4A11-838C-05D019B1BA13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF43FC44-B3C1-4155-8152-0FF6F6AA73F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15390" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3113" uniqueCount="720">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3144" uniqueCount="731">
   <si>
     <t>1</t>
   </si>
@@ -2188,6 +2188,39 @@
   </si>
   <si>
     <t>980|1003</t>
+  </si>
+  <si>
+    <t>O2S_IntegrationScenario01</t>
+  </si>
+  <si>
+    <t>1004</t>
+  </si>
+  <si>
+    <t>O2S_IntegrationScenario02</t>
+  </si>
+  <si>
+    <t>1006</t>
+  </si>
+  <si>
+    <t>O2S_IntegrationScenario03</t>
+  </si>
+  <si>
+    <t>1004|1004</t>
+  </si>
+  <si>
+    <t>O2S_IntegrationScenario04</t>
+  </si>
+  <si>
+    <t>1004|1005</t>
+  </si>
+  <si>
+    <t>619-00-014</t>
+  </si>
+  <si>
+    <t>1005</t>
+  </si>
+  <si>
+    <t>000-00002-015</t>
   </si>
 </sst>
 </file>
@@ -2731,7 +2764,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI402"/>
+  <dimension ref="A1:AI408"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -13105,7 +13138,7 @@
       <c r="A219" s="14"/>
       <c r="B219" s="14"/>
       <c r="C219" s="14"/>
-      <c r="D219" s="14"/>
+      <c r="D219" s="18"/>
       <c r="E219" s="14"/>
       <c r="F219" s="14"/>
       <c r="G219" s="14"/>
@@ -13139,30 +13172,18 @@
       <c r="AI219" s="14"/>
     </row>
     <row r="220" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A220" s="14" t="s">
-        <v>267</v>
-      </c>
-      <c r="B220" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C220" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D220" s="14"/>
+      <c r="A220" s="14"/>
+      <c r="B220" s="14"/>
+      <c r="C220" s="14"/>
+      <c r="D220" s="18"/>
       <c r="E220" s="14"/>
       <c r="F220" s="14"/>
       <c r="G220" s="14"/>
       <c r="H220" s="14"/>
       <c r="I220" s="14"/>
-      <c r="J220" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K220" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L220" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J220" s="14"/>
+      <c r="K220" s="14"/>
+      <c r="L220" s="14"/>
       <c r="M220" s="14"/>
       <c r="N220" s="14"/>
       <c r="O220" s="14"/>
@@ -13189,7 +13210,7 @@
     </row>
     <row r="221" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A221" s="14" t="s">
-        <v>268</v>
+        <v>720</v>
       </c>
       <c r="B221" s="14" t="s">
         <v>174</v>
@@ -13197,21 +13218,17 @@
       <c r="C221" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D221" s="14"/>
+      <c r="D221" s="18" t="s">
+        <v>721</v>
+      </c>
       <c r="E221" s="14"/>
       <c r="F221" s="14"/>
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
       <c r="I221" s="14"/>
-      <c r="J221" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K221" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L221" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="J221" s="14"/>
+      <c r="K221" s="14"/>
+      <c r="L221" s="14"/>
       <c r="M221" s="14"/>
       <c r="N221" s="14"/>
       <c r="O221" s="14"/>
@@ -13236,9 +13253,9 @@
       <c r="AH221" s="14"/>
       <c r="AI221" s="14"/>
     </row>
-    <row r="222" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A222" s="14" t="s">
-        <v>359</v>
+        <v>722</v>
       </c>
       <c r="B222" s="14" t="s">
         <v>174</v>
@@ -13246,9 +13263,32 @@
       <c r="C222" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O222" s="15" t="s">
-        <v>362</v>
-      </c>
+      <c r="D222" s="18" t="s">
+        <v>723</v>
+      </c>
+      <c r="E222" s="14"/>
+      <c r="F222" s="14"/>
+      <c r="G222" s="14"/>
+      <c r="H222" s="14"/>
+      <c r="I222" s="14"/>
+      <c r="J222" s="14"/>
+      <c r="K222" s="14"/>
+      <c r="L222" s="14"/>
+      <c r="M222" s="14"/>
+      <c r="N222" s="14"/>
+      <c r="O222" s="14"/>
+      <c r="P222" s="14"/>
+      <c r="Q222" s="14"/>
+      <c r="R222" s="14"/>
+      <c r="S222" s="14"/>
+      <c r="T222" s="14"/>
+      <c r="U222" s="14"/>
+      <c r="V222" s="14"/>
+      <c r="W222" s="14"/>
+      <c r="X222" s="14"/>
+      <c r="Y222" s="14"/>
+      <c r="Z222" s="14"/>
+      <c r="AA222" s="14"/>
       <c r="AB222" s="14"/>
       <c r="AC222" s="14"/>
       <c r="AD222" s="14"/>
@@ -13258,9 +13298,9 @@
       <c r="AH222" s="14"/>
       <c r="AI222" s="14"/>
     </row>
-    <row r="223" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A223" s="14" t="s">
-        <v>360</v>
+        <v>724</v>
       </c>
       <c r="B223" s="14" t="s">
         <v>174</v>
@@ -13268,9 +13308,32 @@
       <c r="C223" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O223" s="15" t="s">
-        <v>363</v>
-      </c>
+      <c r="D223" s="18" t="s">
+        <v>725</v>
+      </c>
+      <c r="E223" s="14"/>
+      <c r="F223" s="14"/>
+      <c r="G223" s="14"/>
+      <c r="H223" s="14"/>
+      <c r="I223" s="14"/>
+      <c r="J223" s="14"/>
+      <c r="K223" s="14"/>
+      <c r="L223" s="14"/>
+      <c r="M223" s="14"/>
+      <c r="N223" s="14"/>
+      <c r="O223" s="14"/>
+      <c r="P223" s="14"/>
+      <c r="Q223" s="14"/>
+      <c r="R223" s="14"/>
+      <c r="S223" s="14"/>
+      <c r="T223" s="14"/>
+      <c r="U223" s="14"/>
+      <c r="V223" s="14"/>
+      <c r="W223" s="14"/>
+      <c r="X223" s="14"/>
+      <c r="Y223" s="14"/>
+      <c r="Z223" s="14"/>
+      <c r="AA223" s="14"/>
       <c r="AB223" s="14"/>
       <c r="AC223" s="14"/>
       <c r="AD223" s="14"/>
@@ -13280,9 +13343,9 @@
       <c r="AH223" s="14"/>
       <c r="AI223" s="14"/>
     </row>
-    <row r="224" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A224" s="14" t="s">
-        <v>361</v>
+        <v>726</v>
       </c>
       <c r="B224" s="14" t="s">
         <v>174</v>
@@ -13290,9 +13353,32 @@
       <c r="C224" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O224" s="15" t="s">
-        <v>364</v>
-      </c>
+      <c r="D224" s="18" t="s">
+        <v>727</v>
+      </c>
+      <c r="E224" s="14"/>
+      <c r="F224" s="14"/>
+      <c r="G224" s="14"/>
+      <c r="H224" s="14"/>
+      <c r="I224" s="14"/>
+      <c r="J224" s="14"/>
+      <c r="K224" s="14"/>
+      <c r="L224" s="14"/>
+      <c r="M224" s="14"/>
+      <c r="N224" s="14"/>
+      <c r="O224" s="14"/>
+      <c r="P224" s="14"/>
+      <c r="Q224" s="14"/>
+      <c r="R224" s="14"/>
+      <c r="S224" s="14"/>
+      <c r="T224" s="14"/>
+      <c r="U224" s="14"/>
+      <c r="V224" s="14"/>
+      <c r="W224" s="14"/>
+      <c r="X224" s="14"/>
+      <c r="Y224" s="14"/>
+      <c r="Z224" s="14"/>
+      <c r="AA224" s="14"/>
       <c r="AB224" s="14"/>
       <c r="AC224" s="14"/>
       <c r="AD224" s="14"/>
@@ -13302,19 +13388,34 @@
       <c r="AH224" s="14"/>
       <c r="AI224" s="14"/>
     </row>
-    <row r="225" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A225" s="14" t="s">
-        <v>370</v>
-      </c>
-      <c r="B225" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C225" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="M225" s="14" t="s">
-        <v>371</v>
-      </c>
+    <row r="225" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A225" s="14"/>
+      <c r="B225" s="14"/>
+      <c r="C225" s="14"/>
+      <c r="D225" s="14"/>
+      <c r="E225" s="14"/>
+      <c r="F225" s="14"/>
+      <c r="G225" s="14"/>
+      <c r="H225" s="14"/>
+      <c r="I225" s="14"/>
+      <c r="J225" s="14"/>
+      <c r="K225" s="14"/>
+      <c r="L225" s="14"/>
+      <c r="M225" s="14"/>
+      <c r="N225" s="14"/>
+      <c r="O225" s="14"/>
+      <c r="P225" s="14"/>
+      <c r="Q225" s="14"/>
+      <c r="R225" s="14"/>
+      <c r="S225" s="14"/>
+      <c r="T225" s="14"/>
+      <c r="U225" s="14"/>
+      <c r="V225" s="14"/>
+      <c r="W225" s="14"/>
+      <c r="X225" s="14"/>
+      <c r="Y225" s="14"/>
+      <c r="Z225" s="14"/>
+      <c r="AA225" s="14"/>
       <c r="AB225" s="14"/>
       <c r="AC225" s="14"/>
       <c r="AD225" s="14"/>
@@ -13324,7 +13425,46 @@
       <c r="AH225" s="14"/>
       <c r="AI225" s="14"/>
     </row>
-    <row r="226" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A226" s="14" t="s">
+        <v>267</v>
+      </c>
+      <c r="B226" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C226" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D226" s="14"/>
+      <c r="E226" s="14"/>
+      <c r="F226" s="14"/>
+      <c r="G226" s="14"/>
+      <c r="H226" s="14"/>
+      <c r="I226" s="14"/>
+      <c r="J226" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K226" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L226" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M226" s="14"/>
+      <c r="N226" s="14"/>
+      <c r="O226" s="14"/>
+      <c r="P226" s="14"/>
+      <c r="Q226" s="14"/>
+      <c r="R226" s="14"/>
+      <c r="S226" s="14"/>
+      <c r="T226" s="14"/>
+      <c r="U226" s="14"/>
+      <c r="V226" s="14"/>
+      <c r="W226" s="14"/>
+      <c r="X226" s="14"/>
+      <c r="Y226" s="14"/>
+      <c r="Z226" s="14"/>
+      <c r="AA226" s="14"/>
       <c r="AB226" s="14"/>
       <c r="AC226" s="14"/>
       <c r="AD226" s="14"/>
@@ -13334,7 +13474,46 @@
       <c r="AH226" s="14"/>
       <c r="AI226" s="14"/>
     </row>
-    <row r="227" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A227" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="B227" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C227" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D227" s="14"/>
+      <c r="E227" s="14"/>
+      <c r="F227" s="14"/>
+      <c r="G227" s="14"/>
+      <c r="H227" s="14"/>
+      <c r="I227" s="14"/>
+      <c r="J227" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K227" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L227" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M227" s="14"/>
+      <c r="N227" s="14"/>
+      <c r="O227" s="14"/>
+      <c r="P227" s="14"/>
+      <c r="Q227" s="14"/>
+      <c r="R227" s="14"/>
+      <c r="S227" s="14"/>
+      <c r="T227" s="14"/>
+      <c r="U227" s="14"/>
+      <c r="V227" s="14"/>
+      <c r="W227" s="14"/>
+      <c r="X227" s="14"/>
+      <c r="Y227" s="14"/>
+      <c r="Z227" s="14"/>
+      <c r="AA227" s="14"/>
       <c r="AB227" s="14"/>
       <c r="AC227" s="14"/>
       <c r="AD227" s="14"/>
@@ -13345,6 +13524,18 @@
       <c r="AI227" s="14"/>
     </row>
     <row r="228" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A228" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="B228" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C228" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O228" s="15" t="s">
+        <v>362</v>
+      </c>
       <c r="AB228" s="14"/>
       <c r="AC228" s="14"/>
       <c r="AD228" s="14"/>
@@ -13355,6 +13546,18 @@
       <c r="AI228" s="14"/>
     </row>
     <row r="229" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A229" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B229" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C229" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O229" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB229" s="14"/>
       <c r="AC229" s="14"/>
       <c r="AD229" s="14"/>
@@ -13365,6 +13568,18 @@
       <c r="AI229" s="14"/>
     </row>
     <row r="230" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A230" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B230" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C230" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O230" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB230" s="14"/>
       <c r="AC230" s="14"/>
       <c r="AD230" s="14"/>
@@ -13375,6 +13590,18 @@
       <c r="AI230" s="14"/>
     </row>
     <row r="231" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A231" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B231" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C231" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M231" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB231" s="14"/>
       <c r="AC231" s="14"/>
       <c r="AD231" s="14"/>
@@ -15028,7 +15255,7 @@
       <c r="AB396" s="14"/>
       <c r="AC396" s="14"/>
       <c r="AD396" s="14"/>
-      <c r="AE396" s="14"/>
+      <c r="AE396" s="27"/>
       <c r="AF396" s="14"/>
       <c r="AG396" s="14"/>
       <c r="AH396" s="14"/>
@@ -15038,7 +15265,7 @@
       <c r="AB397" s="14"/>
       <c r="AC397" s="14"/>
       <c r="AD397" s="14"/>
-      <c r="AE397" s="14"/>
+      <c r="AE397" s="27"/>
       <c r="AF397" s="14"/>
       <c r="AG397" s="14"/>
       <c r="AH397" s="14"/>
@@ -15048,7 +15275,7 @@
       <c r="AB398" s="14"/>
       <c r="AC398" s="14"/>
       <c r="AD398" s="14"/>
-      <c r="AE398" s="14"/>
+      <c r="AE398" s="27"/>
       <c r="AF398" s="14"/>
       <c r="AG398" s="14"/>
       <c r="AH398" s="14"/>
@@ -15058,7 +15285,7 @@
       <c r="AB399" s="14"/>
       <c r="AC399" s="14"/>
       <c r="AD399" s="14"/>
-      <c r="AE399" s="14"/>
+      <c r="AE399" s="27"/>
       <c r="AF399" s="14"/>
       <c r="AG399" s="14"/>
       <c r="AH399" s="14"/>
@@ -15068,7 +15295,7 @@
       <c r="AB400" s="14"/>
       <c r="AC400" s="14"/>
       <c r="AD400" s="14"/>
-      <c r="AE400" s="14"/>
+      <c r="AE400" s="27"/>
       <c r="AF400" s="14"/>
       <c r="AG400" s="14"/>
       <c r="AH400" s="14"/>
@@ -15078,7 +15305,7 @@
       <c r="AB401" s="14"/>
       <c r="AC401" s="14"/>
       <c r="AD401" s="14"/>
-      <c r="AE401" s="14"/>
+      <c r="AE401" s="27"/>
       <c r="AF401" s="14"/>
       <c r="AG401" s="14"/>
       <c r="AH401" s="14"/>
@@ -15094,6 +15321,66 @@
       <c r="AH402" s="14"/>
       <c r="AI402" s="14"/>
     </row>
+    <row r="403" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB403" s="14"/>
+      <c r="AC403" s="14"/>
+      <c r="AD403" s="14"/>
+      <c r="AE403" s="14"/>
+      <c r="AF403" s="14"/>
+      <c r="AG403" s="14"/>
+      <c r="AH403" s="14"/>
+      <c r="AI403" s="14"/>
+    </row>
+    <row r="404" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB404" s="14"/>
+      <c r="AC404" s="14"/>
+      <c r="AD404" s="14"/>
+      <c r="AE404" s="14"/>
+      <c r="AF404" s="14"/>
+      <c r="AG404" s="14"/>
+      <c r="AH404" s="14"/>
+      <c r="AI404" s="14"/>
+    </row>
+    <row r="405" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB405" s="14"/>
+      <c r="AC405" s="14"/>
+      <c r="AD405" s="14"/>
+      <c r="AE405" s="14"/>
+      <c r="AF405" s="14"/>
+      <c r="AG405" s="14"/>
+      <c r="AH405" s="14"/>
+      <c r="AI405" s="14"/>
+    </row>
+    <row r="406" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB406" s="14"/>
+      <c r="AC406" s="14"/>
+      <c r="AD406" s="14"/>
+      <c r="AE406" s="14"/>
+      <c r="AF406" s="14"/>
+      <c r="AG406" s="14"/>
+      <c r="AH406" s="14"/>
+      <c r="AI406" s="14"/>
+    </row>
+    <row r="407" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB407" s="14"/>
+      <c r="AC407" s="14"/>
+      <c r="AD407" s="14"/>
+      <c r="AE407" s="14"/>
+      <c r="AF407" s="14"/>
+      <c r="AG407" s="14"/>
+      <c r="AH407" s="14"/>
+      <c r="AI407" s="14"/>
+    </row>
+    <row r="408" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB408" s="14"/>
+      <c r="AC408" s="14"/>
+      <c r="AD408" s="14"/>
+      <c r="AE408" s="14"/>
+      <c r="AF408" s="14"/>
+      <c r="AG408" s="14"/>
+      <c r="AH408" s="14"/>
+      <c r="AI408" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15103,7 +15390,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T218"/>
+  <dimension ref="A1:T221"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -22274,7 +22561,7 @@
       <c r="T217" s="14"/>
     </row>
     <row r="218" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A218" s="15" t="s">
+      <c r="A218" s="16" t="s">
         <v>718</v>
       </c>
       <c r="B218" s="20" t="s">
@@ -22283,15 +22570,15 @@
       <c r="C218" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="D218" s="14" t="s">
+      <c r="D218" s="16" t="s">
         <v>112</v>
       </c>
       <c r="E218" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="F218" s="15"/>
-      <c r="G218" s="15"/>
-      <c r="H218" s="15"/>
+      <c r="F218" s="14"/>
+      <c r="G218" s="14"/>
+      <c r="H218" s="14"/>
       <c r="I218" s="14" t="s">
         <v>624</v>
       </c>
@@ -22308,6 +22595,102 @@
       <c r="R218" s="14"/>
       <c r="S218" s="14"/>
       <c r="T218" s="14"/>
+    </row>
+    <row r="219" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A219" s="16" t="s">
+        <v>721</v>
+      </c>
+      <c r="B219" s="20" t="s">
+        <v>728</v>
+      </c>
+      <c r="C219" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D219" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="E219" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F219" s="14"/>
+      <c r="G219" s="14"/>
+      <c r="H219" s="14"/>
+      <c r="I219" s="14"/>
+      <c r="J219" s="14"/>
+      <c r="K219" s="14"/>
+      <c r="L219" s="14"/>
+      <c r="M219" s="14"/>
+      <c r="N219" s="14"/>
+      <c r="O219" s="14"/>
+      <c r="P219" s="14"/>
+      <c r="Q219" s="14"/>
+      <c r="R219" s="14"/>
+      <c r="S219" s="14"/>
+      <c r="T219" s="14"/>
+    </row>
+    <row r="220" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A220" s="15" t="s">
+        <v>729</v>
+      </c>
+      <c r="B220" s="20" t="s">
+        <v>728</v>
+      </c>
+      <c r="C220" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D220" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E220" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F220" s="15"/>
+      <c r="G220" s="15"/>
+      <c r="H220" s="15"/>
+      <c r="I220" s="14"/>
+      <c r="J220" s="14"/>
+      <c r="K220" s="14"/>
+      <c r="L220" s="14"/>
+      <c r="M220" s="14"/>
+      <c r="N220" s="14"/>
+      <c r="O220" s="14"/>
+      <c r="P220" s="14"/>
+      <c r="Q220" s="14"/>
+      <c r="R220" s="14"/>
+      <c r="S220" s="14"/>
+      <c r="T220" s="14"/>
+    </row>
+    <row r="221" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A221" s="15" t="s">
+        <v>723</v>
+      </c>
+      <c r="B221" s="20" t="s">
+        <v>730</v>
+      </c>
+      <c r="C221" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D221" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E221" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F221" s="15"/>
+      <c r="G221" s="15"/>
+      <c r="H221" s="15"/>
+      <c r="I221" s="14"/>
+      <c r="J221" s="14"/>
+      <c r="K221" s="14"/>
+      <c r="L221" s="14"/>
+      <c r="M221" s="14"/>
+      <c r="N221" s="14"/>
+      <c r="O221" s="14"/>
+      <c r="P221" s="14"/>
+      <c r="Q221" s="14"/>
+      <c r="R221" s="14"/>
+      <c r="S221" s="14"/>
+      <c r="T221" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
Commit script for Create and verify ASN for Vendor Portal module
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE14E1BA-4870-4458-95C5-78EDD514BF3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{507429FE-E851-4644-801C-23EABBFFA112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3180" uniqueCount="738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3218" uniqueCount="744">
   <si>
     <t>1</t>
   </si>
@@ -2242,6 +2242,24 @@
   </si>
   <si>
     <t>APC_KelliScenario004</t>
+  </si>
+  <si>
+    <t>1010</t>
+  </si>
+  <si>
+    <t>APC_IBScenario013</t>
+  </si>
+  <si>
+    <t>APC_IBScenario014</t>
+  </si>
+  <si>
+    <t>1011</t>
+  </si>
+  <si>
+    <t>1012</t>
+  </si>
+  <si>
+    <t>1011|1012</t>
   </si>
 </sst>
 </file>
@@ -2785,7 +2803,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI411"/>
+  <dimension ref="A1:AI413"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -12135,15 +12153,25 @@
       <c r="AI199" s="14"/>
     </row>
     <row r="200" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A200" s="14"/>
-      <c r="B200" s="14"/>
-      <c r="C200" s="14"/>
-      <c r="D200" s="18"/>
+      <c r="A200" s="14" t="s">
+        <v>739</v>
+      </c>
+      <c r="B200" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C200" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D200" s="18" t="s">
+        <v>738</v>
+      </c>
       <c r="E200" s="14"/>
       <c r="F200" s="14"/>
       <c r="G200" s="14"/>
       <c r="H200" s="14"/>
-      <c r="I200" s="14"/>
+      <c r="I200" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J200" s="14"/>
       <c r="K200" s="14"/>
       <c r="L200" s="31"/>
@@ -12165,15 +12193,19 @@
       <c r="AB200" s="14"/>
       <c r="AC200" s="14"/>
       <c r="AD200" s="14"/>
-      <c r="AE200" s="27"/>
+      <c r="AE200" s="27" t="s">
+        <v>650</v>
+      </c>
       <c r="AF200" s="14"/>
       <c r="AG200" s="14"/>
-      <c r="AH200" s="14"/>
+      <c r="AH200" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI200" s="14"/>
     </row>
     <row r="201" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="14" t="s">
-        <v>662</v>
+        <v>740</v>
       </c>
       <c r="B201" s="14" t="s">
         <v>613</v>
@@ -12181,18 +12213,20 @@
       <c r="C201" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D201" s="23" t="s">
-        <v>663</v>
+      <c r="D201" s="18" t="s">
+        <v>743</v>
       </c>
       <c r="E201" s="14"/>
       <c r="F201" s="14"/>
       <c r="G201" s="14"/>
       <c r="H201" s="14"/>
-      <c r="I201" s="14"/>
+      <c r="I201" s="14" t="s">
+        <v>378</v>
+      </c>
       <c r="J201" s="14"/>
       <c r="K201" s="14"/>
-      <c r="L201" s="14"/>
-      <c r="M201" s="14"/>
+      <c r="L201" s="31"/>
+      <c r="M201" s="30"/>
       <c r="N201" s="14"/>
       <c r="O201" s="14"/>
       <c r="P201" s="14"/>
@@ -12207,16 +12241,12 @@
       <c r="Y201" s="14"/>
       <c r="Z201" s="14"/>
       <c r="AA201" s="14"/>
-      <c r="AB201" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="AC201" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD201" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE201" s="27"/>
+      <c r="AB201" s="14"/>
+      <c r="AC201" s="14"/>
+      <c r="AD201" s="14"/>
+      <c r="AE201" s="27" t="s">
+        <v>650</v>
+      </c>
       <c r="AF201" s="14"/>
       <c r="AG201" s="14"/>
       <c r="AH201" s="14" t="s">
@@ -12225,18 +12255,10 @@
       <c r="AI201" s="14"/>
     </row>
     <row r="202" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A202" s="14" t="s">
-        <v>664</v>
-      </c>
-      <c r="B202" s="14" t="s">
-        <v>613</v>
-      </c>
-      <c r="C202" s="14" t="s">
-        <v>614</v>
-      </c>
-      <c r="D202" s="23" t="s">
-        <v>663</v>
-      </c>
+      <c r="A202" s="14"/>
+      <c r="B202" s="14"/>
+      <c r="C202" s="14"/>
+      <c r="D202" s="18"/>
       <c r="E202" s="14"/>
       <c r="F202" s="14"/>
       <c r="G202" s="14"/>
@@ -12244,8 +12266,8 @@
       <c r="I202" s="14"/>
       <c r="J202" s="14"/>
       <c r="K202" s="14"/>
-      <c r="L202" s="14"/>
-      <c r="M202" s="14"/>
+      <c r="L202" s="31"/>
+      <c r="M202" s="30"/>
       <c r="N202" s="14"/>
       <c r="O202" s="14"/>
       <c r="P202" s="14"/>
@@ -12260,15 +12282,9 @@
       <c r="Y202" s="14"/>
       <c r="Z202" s="14"/>
       <c r="AA202" s="14"/>
-      <c r="AB202" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC202" s="14" t="s">
-        <v>420</v>
-      </c>
-      <c r="AD202" s="14" t="s">
-        <v>421</v>
-      </c>
+      <c r="AB202" s="14"/>
+      <c r="AC202" s="14"/>
+      <c r="AD202" s="14"/>
       <c r="AE202" s="27"/>
       <c r="AF202" s="14"/>
       <c r="AG202" s="14"/>
@@ -12277,7 +12293,7 @@
     </row>
     <row r="203" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="14" t="s">
-        <v>668</v>
+        <v>662</v>
       </c>
       <c r="B203" s="14" t="s">
         <v>613</v>
@@ -12286,7 +12302,7 @@
         <v>614</v>
       </c>
       <c r="D203" s="23" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="E203" s="14"/>
       <c r="F203" s="14"/>
@@ -12330,7 +12346,7 @@
     </row>
     <row r="204" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A204" s="14" t="s">
-        <v>669</v>
+        <v>664</v>
       </c>
       <c r="B204" s="14" t="s">
         <v>613</v>
@@ -12339,7 +12355,7 @@
         <v>614</v>
       </c>
       <c r="D204" s="23" t="s">
-        <v>670</v>
+        <v>663</v>
       </c>
       <c r="E204" s="14"/>
       <c r="F204" s="14"/>
@@ -12376,14 +12392,12 @@
       <c r="AE204" s="27"/>
       <c r="AF204" s="14"/>
       <c r="AG204" s="14"/>
-      <c r="AH204" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH204" s="14"/>
       <c r="AI204" s="14"/>
     </row>
     <row r="205" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="14" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="B205" s="14" t="s">
         <v>613</v>
@@ -12392,7 +12406,7 @@
         <v>614</v>
       </c>
       <c r="D205" s="23" t="s">
-        <v>672</v>
+        <v>667</v>
       </c>
       <c r="E205" s="14"/>
       <c r="F205" s="14"/>
@@ -12436,7 +12450,7 @@
     </row>
     <row r="206" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="14" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="B206" s="14" t="s">
         <v>613</v>
@@ -12445,7 +12459,7 @@
         <v>614</v>
       </c>
       <c r="D206" s="23" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="E206" s="14"/>
       <c r="F206" s="14"/>
@@ -12489,7 +12503,7 @@
     </row>
     <row r="207" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="14" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="B207" s="14" t="s">
         <v>613</v>
@@ -12497,8 +12511,8 @@
       <c r="C207" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D207" s="18" t="s">
-        <v>676</v>
+      <c r="D207" s="23" t="s">
+        <v>672</v>
       </c>
       <c r="E207" s="14"/>
       <c r="F207" s="14"/>
@@ -12542,7 +12556,7 @@
     </row>
     <row r="208" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="14" t="s">
-        <v>679</v>
+        <v>673</v>
       </c>
       <c r="B208" s="14" t="s">
         <v>613</v>
@@ -12550,8 +12564,8 @@
       <c r="C208" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D208" s="18" t="s">
-        <v>713</v>
+      <c r="D208" s="23" t="s">
+        <v>672</v>
       </c>
       <c r="E208" s="14"/>
       <c r="F208" s="14"/>
@@ -12577,17 +12591,15 @@
       <c r="Z208" s="14"/>
       <c r="AA208" s="14"/>
       <c r="AB208" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC208" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD208" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE208" s="27" t="s">
-        <v>650</v>
-      </c>
+        <v>421</v>
+      </c>
+      <c r="AE208" s="27"/>
       <c r="AF208" s="14"/>
       <c r="AG208" s="14"/>
       <c r="AH208" s="14" t="s">
@@ -12597,7 +12609,7 @@
     </row>
     <row r="209" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="14" t="s">
-        <v>680</v>
+        <v>674</v>
       </c>
       <c r="B209" s="14" t="s">
         <v>613</v>
@@ -12606,7 +12618,7 @@
         <v>614</v>
       </c>
       <c r="D209" s="18" t="s">
-        <v>713</v>
+        <v>676</v>
       </c>
       <c r="E209" s="14"/>
       <c r="F209" s="14"/>
@@ -12632,17 +12644,15 @@
       <c r="Z209" s="14"/>
       <c r="AA209" s="14"/>
       <c r="AB209" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC209" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD209" s="14" t="s">
-        <v>421</v>
-      </c>
-      <c r="AE209" s="27" t="s">
-        <v>650</v>
-      </c>
+        <v>451</v>
+      </c>
+      <c r="AE209" s="27"/>
       <c r="AF209" s="14"/>
       <c r="AG209" s="14"/>
       <c r="AH209" s="14" t="s">
@@ -12652,7 +12662,7 @@
     </row>
     <row r="210" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210" s="14" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
       <c r="B210" s="14" t="s">
         <v>613</v>
@@ -12661,7 +12671,7 @@
         <v>614</v>
       </c>
       <c r="D210" s="18" t="s">
-        <v>684</v>
+        <v>713</v>
       </c>
       <c r="E210" s="14"/>
       <c r="F210" s="14"/>
@@ -12695,7 +12705,9 @@
       <c r="AD210" s="14" t="s">
         <v>451</v>
       </c>
-      <c r="AE210" s="27"/>
+      <c r="AE210" s="27" t="s">
+        <v>650</v>
+      </c>
       <c r="AF210" s="14"/>
       <c r="AG210" s="14"/>
       <c r="AH210" s="14" t="s">
@@ -12705,7 +12717,7 @@
     </row>
     <row r="211" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="14" t="s">
-        <v>685</v>
+        <v>680</v>
       </c>
       <c r="B211" s="14" t="s">
         <v>613</v>
@@ -12714,7 +12726,7 @@
         <v>614</v>
       </c>
       <c r="D211" s="18" t="s">
-        <v>684</v>
+        <v>713</v>
       </c>
       <c r="E211" s="14"/>
       <c r="F211" s="14"/>
@@ -12748,7 +12760,9 @@
       <c r="AD211" s="14" t="s">
         <v>421</v>
       </c>
-      <c r="AE211" s="27"/>
+      <c r="AE211" s="27" t="s">
+        <v>650</v>
+      </c>
       <c r="AF211" s="14"/>
       <c r="AG211" s="14"/>
       <c r="AH211" s="14" t="s">
@@ -12758,7 +12772,7 @@
     </row>
     <row r="212" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="14" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
       <c r="B212" s="14" t="s">
         <v>613</v>
@@ -12766,8 +12780,8 @@
       <c r="C212" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D212" s="23" t="s">
-        <v>667</v>
+      <c r="D212" s="18" t="s">
+        <v>684</v>
       </c>
       <c r="E212" s="14"/>
       <c r="F212" s="14"/>
@@ -12793,17 +12807,15 @@
       <c r="Z212" s="14"/>
       <c r="AA212" s="14"/>
       <c r="AB212" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC212" s="14" t="s">
-        <v>420</v>
+        <v>457</v>
       </c>
       <c r="AD212" s="14" t="s">
-        <v>421</v>
-      </c>
-      <c r="AE212" s="27" t="s">
-        <v>649</v>
-      </c>
+        <v>451</v>
+      </c>
+      <c r="AE212" s="27"/>
       <c r="AF212" s="14"/>
       <c r="AG212" s="14"/>
       <c r="AH212" s="14" t="s">
@@ -12813,7 +12825,7 @@
     </row>
     <row r="213" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A213" s="14" t="s">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="B213" s="14" t="s">
         <v>613</v>
@@ -12821,8 +12833,8 @@
       <c r="C213" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D213" s="23" t="s">
-        <v>667</v>
+      <c r="D213" s="18" t="s">
+        <v>684</v>
       </c>
       <c r="E213" s="14"/>
       <c r="F213" s="14"/>
@@ -12848,17 +12860,15 @@
       <c r="Z213" s="14"/>
       <c r="AA213" s="14"/>
       <c r="AB213" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC213" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD213" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="AE213" s="27" t="s">
-        <v>649</v>
-      </c>
+        <v>421</v>
+      </c>
+      <c r="AE213" s="27"/>
       <c r="AF213" s="14"/>
       <c r="AG213" s="14"/>
       <c r="AH213" s="14" t="s">
@@ -12868,7 +12878,7 @@
     </row>
     <row r="214" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A214" s="14" t="s">
-        <v>699</v>
+        <v>687</v>
       </c>
       <c r="B214" s="14" t="s">
         <v>613</v>
@@ -12876,8 +12886,8 @@
       <c r="C214" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D214" s="18" t="s">
-        <v>628</v>
+      <c r="D214" s="23" t="s">
+        <v>667</v>
       </c>
       <c r="E214" s="14"/>
       <c r="F214" s="14"/>
@@ -12903,16 +12913,16 @@
       <c r="Z214" s="14"/>
       <c r="AA214" s="14"/>
       <c r="AB214" s="14" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="AC214" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="AD214" s="14" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="AE214" s="27" t="s">
-        <v>694</v>
+        <v>649</v>
       </c>
       <c r="AF214" s="14"/>
       <c r="AG214" s="14"/>
@@ -12923,7 +12933,7 @@
     </row>
     <row r="215" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A215" s="14" t="s">
-        <v>701</v>
+        <v>690</v>
       </c>
       <c r="B215" s="14" t="s">
         <v>613</v>
@@ -12931,8 +12941,8 @@
       <c r="C215" s="14" t="s">
         <v>614</v>
       </c>
-      <c r="D215" s="18" t="s">
-        <v>663</v>
+      <c r="D215" s="23" t="s">
+        <v>667</v>
       </c>
       <c r="E215" s="14"/>
       <c r="F215" s="14"/>
@@ -12967,7 +12977,7 @@
         <v>451</v>
       </c>
       <c r="AE215" s="27" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="AF215" s="14"/>
       <c r="AG215" s="14"/>
@@ -12978,7 +12988,7 @@
     </row>
     <row r="216" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A216" s="14" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="B216" s="14" t="s">
         <v>613</v>
@@ -12987,7 +12997,7 @@
         <v>614</v>
       </c>
       <c r="D216" s="18" t="s">
-        <v>675</v>
+        <v>628</v>
       </c>
       <c r="E216" s="14"/>
       <c r="F216" s="14"/>
@@ -13016,20 +13026,24 @@
         <v>419</v>
       </c>
       <c r="AC216" s="14" t="s">
-        <v>695</v>
+        <v>457</v>
       </c>
       <c r="AD216" s="14" t="s">
-        <v>696</v>
-      </c>
-      <c r="AE216" s="27"/>
+        <v>451</v>
+      </c>
+      <c r="AE216" s="27" t="s">
+        <v>694</v>
+      </c>
       <c r="AF216" s="14"/>
       <c r="AG216" s="14"/>
-      <c r="AH216" s="14"/>
+      <c r="AH216" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI216" s="14"/>
     </row>
     <row r="217" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A217" s="14" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="B217" s="14" t="s">
         <v>613</v>
@@ -13038,7 +13052,7 @@
         <v>614</v>
       </c>
       <c r="D217" s="18" t="s">
-        <v>675</v>
+        <v>663</v>
       </c>
       <c r="E217" s="14"/>
       <c r="F217" s="14"/>
@@ -13064,25 +13078,27 @@
       <c r="Z217" s="14"/>
       <c r="AA217" s="14"/>
       <c r="AB217" s="14" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="AC217" s="14" t="s">
-        <v>697</v>
+        <v>457</v>
       </c>
       <c r="AD217" s="14" t="s">
-        <v>698</v>
+        <v>451</v>
       </c>
       <c r="AE217" s="27" t="s">
         <v>650</v>
       </c>
       <c r="AF217" s="14"/>
       <c r="AG217" s="14"/>
-      <c r="AH217" s="14"/>
+      <c r="AH217" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI217" s="14"/>
     </row>
     <row r="218" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A218" s="14" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="B218" s="14" t="s">
         <v>613</v>
@@ -13091,7 +13107,7 @@
         <v>614</v>
       </c>
       <c r="D218" s="18" t="s">
-        <v>628</v>
+        <v>675</v>
       </c>
       <c r="E218" s="14"/>
       <c r="F218" s="14"/>
@@ -13125,9 +13141,7 @@
       <c r="AD218" s="14" t="s">
         <v>696</v>
       </c>
-      <c r="AE218" s="27" t="s">
-        <v>694</v>
-      </c>
+      <c r="AE218" s="27"/>
       <c r="AF218" s="14"/>
       <c r="AG218" s="14"/>
       <c r="AH218" s="14"/>
@@ -13135,7 +13149,7 @@
     </row>
     <row r="219" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A219" s="14" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="B219" s="14" t="s">
         <v>613</v>
@@ -13144,7 +13158,7 @@
         <v>614</v>
       </c>
       <c r="D219" s="18" t="s">
-        <v>700</v>
+        <v>675</v>
       </c>
       <c r="E219" s="14"/>
       <c r="F219" s="14"/>
@@ -13173,24 +13187,22 @@
         <v>393</v>
       </c>
       <c r="AC219" s="14" t="s">
-        <v>420</v>
+        <v>697</v>
       </c>
       <c r="AD219" s="14" t="s">
-        <v>421</v>
+        <v>698</v>
       </c>
       <c r="AE219" s="27" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="AF219" s="14"/>
       <c r="AG219" s="14"/>
-      <c r="AH219" s="14" t="s">
-        <v>458</v>
-      </c>
+      <c r="AH219" s="14"/>
       <c r="AI219" s="14"/>
     </row>
     <row r="220" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A220" s="14" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B220" s="14" t="s">
         <v>613</v>
@@ -13199,7 +13211,7 @@
         <v>614</v>
       </c>
       <c r="D220" s="18" t="s">
-        <v>675</v>
+        <v>628</v>
       </c>
       <c r="E220" s="14"/>
       <c r="F220" s="14"/>
@@ -13228,13 +13240,13 @@
         <v>419</v>
       </c>
       <c r="AC220" s="14" t="s">
-        <v>707</v>
+        <v>695</v>
       </c>
       <c r="AD220" s="14" t="s">
-        <v>451</v>
+        <v>696</v>
       </c>
       <c r="AE220" s="27" t="s">
-        <v>650</v>
+        <v>694</v>
       </c>
       <c r="AF220" s="14"/>
       <c r="AG220" s="14"/>
@@ -13243,7 +13255,7 @@
     </row>
     <row r="221" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A221" s="14" t="s">
-        <v>717</v>
+        <v>705</v>
       </c>
       <c r="B221" s="14" t="s">
         <v>613</v>
@@ -13252,7 +13264,7 @@
         <v>614</v>
       </c>
       <c r="D221" s="18" t="s">
-        <v>716</v>
+        <v>700</v>
       </c>
       <c r="E221" s="14"/>
       <c r="F221" s="14"/>
@@ -13297,10 +13309,18 @@
       <c r="AI221" s="14"/>
     </row>
     <row r="222" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A222" s="14"/>
-      <c r="B222" s="14"/>
-      <c r="C222" s="14"/>
-      <c r="D222" s="18"/>
+      <c r="A222" s="14" t="s">
+        <v>706</v>
+      </c>
+      <c r="B222" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C222" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D222" s="18" t="s">
+        <v>675</v>
+      </c>
       <c r="E222" s="14"/>
       <c r="F222" s="14"/>
       <c r="G222" s="14"/>
@@ -13324,20 +13344,36 @@
       <c r="Y222" s="14"/>
       <c r="Z222" s="14"/>
       <c r="AA222" s="14"/>
-      <c r="AB222" s="14"/>
-      <c r="AC222" s="14"/>
-      <c r="AD222" s="14"/>
-      <c r="AE222" s="27"/>
+      <c r="AB222" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC222" s="14" t="s">
+        <v>707</v>
+      </c>
+      <c r="AD222" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="AE222" s="27" t="s">
+        <v>650</v>
+      </c>
       <c r="AF222" s="14"/>
       <c r="AG222" s="14"/>
       <c r="AH222" s="14"/>
       <c r="AI222" s="14"/>
     </row>
     <row r="223" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A223" s="14"/>
-      <c r="B223" s="14"/>
-      <c r="C223" s="14"/>
-      <c r="D223" s="18"/>
+      <c r="A223" s="14" t="s">
+        <v>717</v>
+      </c>
+      <c r="B223" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C223" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D223" s="18" t="s">
+        <v>716</v>
+      </c>
       <c r="E223" s="14"/>
       <c r="F223" s="14"/>
       <c r="G223" s="14"/>
@@ -13361,28 +13397,30 @@
       <c r="Y223" s="14"/>
       <c r="Z223" s="14"/>
       <c r="AA223" s="14"/>
-      <c r="AB223" s="14"/>
-      <c r="AC223" s="14"/>
-      <c r="AD223" s="14"/>
-      <c r="AE223" s="27"/>
+      <c r="AB223" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC223" s="14" t="s">
+        <v>420</v>
+      </c>
+      <c r="AD223" s="14" t="s">
+        <v>421</v>
+      </c>
+      <c r="AE223" s="27" t="s">
+        <v>653</v>
+      </c>
       <c r="AF223" s="14"/>
       <c r="AG223" s="14"/>
-      <c r="AH223" s="14"/>
+      <c r="AH223" s="14" t="s">
+        <v>458</v>
+      </c>
       <c r="AI223" s="14"/>
     </row>
     <row r="224" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A224" s="14" t="s">
-        <v>720</v>
-      </c>
-      <c r="B224" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C224" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D224" s="18" t="s">
-        <v>721</v>
-      </c>
+      <c r="A224" s="14"/>
+      <c r="B224" s="14"/>
+      <c r="C224" s="14"/>
+      <c r="D224" s="18"/>
       <c r="E224" s="14"/>
       <c r="F224" s="14"/>
       <c r="G224" s="14"/>
@@ -13391,9 +13429,7 @@
       <c r="J224" s="14"/>
       <c r="K224" s="14"/>
       <c r="L224" s="14"/>
-      <c r="M224" s="14" t="s">
-        <v>728</v>
-      </c>
+      <c r="M224" s="14"/>
       <c r="N224" s="14"/>
       <c r="O224" s="14"/>
       <c r="P224" s="14"/>
@@ -13408,15 +13444,9 @@
       <c r="Y224" s="14"/>
       <c r="Z224" s="14"/>
       <c r="AA224" s="14"/>
-      <c r="AB224" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="AC224" s="14" t="s">
-        <v>427</v>
-      </c>
-      <c r="AD224" s="14" t="s">
-        <v>421</v>
-      </c>
+      <c r="AB224" s="14"/>
+      <c r="AC224" s="14"/>
+      <c r="AD224" s="14"/>
       <c r="AE224" s="27"/>
       <c r="AF224" s="14"/>
       <c r="AG224" s="14"/>
@@ -13424,18 +13454,10 @@
       <c r="AI224" s="14"/>
     </row>
     <row r="225" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A225" s="14" t="s">
-        <v>722</v>
-      </c>
-      <c r="B225" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C225" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D225" s="18" t="s">
-        <v>723</v>
-      </c>
+      <c r="A225" s="14"/>
+      <c r="B225" s="14"/>
+      <c r="C225" s="14"/>
+      <c r="D225" s="18"/>
       <c r="E225" s="14"/>
       <c r="F225" s="14"/>
       <c r="G225" s="14"/>
@@ -13470,7 +13492,7 @@
     </row>
     <row r="226" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A226" s="14" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
       <c r="B226" s="14" t="s">
         <v>174</v>
@@ -13479,7 +13501,7 @@
         <v>135</v>
       </c>
       <c r="D226" s="18" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
       <c r="E226" s="14"/>
       <c r="F226" s="14"/>
@@ -13489,7 +13511,9 @@
       <c r="J226" s="14"/>
       <c r="K226" s="14"/>
       <c r="L226" s="14"/>
-      <c r="M226" s="14"/>
+      <c r="M226" s="14" t="s">
+        <v>728</v>
+      </c>
       <c r="N226" s="14"/>
       <c r="O226" s="14"/>
       <c r="P226" s="14"/>
@@ -13504,9 +13528,15 @@
       <c r="Y226" s="14"/>
       <c r="Z226" s="14"/>
       <c r="AA226" s="14"/>
-      <c r="AB226" s="14"/>
-      <c r="AC226" s="14"/>
-      <c r="AD226" s="14"/>
+      <c r="AB226" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="AC226" s="14" t="s">
+        <v>427</v>
+      </c>
+      <c r="AD226" s="14" t="s">
+        <v>421</v>
+      </c>
       <c r="AE226" s="27"/>
       <c r="AF226" s="14"/>
       <c r="AG226" s="14"/>
@@ -13515,7 +13545,7 @@
     </row>
     <row r="227" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A227" s="14" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
       <c r="B227" s="14" t="s">
         <v>174</v>
@@ -13524,7 +13554,7 @@
         <v>135</v>
       </c>
       <c r="D227" s="18" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
       <c r="E227" s="14"/>
       <c r="F227" s="14"/>
@@ -13559,10 +13589,18 @@
       <c r="AI227" s="14"/>
     </row>
     <row r="228" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A228" s="14"/>
-      <c r="B228" s="14"/>
-      <c r="C228" s="14"/>
-      <c r="D228" s="14"/>
+      <c r="A228" s="14" t="s">
+        <v>724</v>
+      </c>
+      <c r="B228" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C228" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D228" s="18" t="s">
+        <v>725</v>
+      </c>
       <c r="E228" s="14"/>
       <c r="F228" s="14"/>
       <c r="G228" s="14"/>
@@ -13597,7 +13635,7 @@
     </row>
     <row r="229" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A229" s="14" t="s">
-        <v>267</v>
+        <v>726</v>
       </c>
       <c r="B229" s="14" t="s">
         <v>174</v>
@@ -13605,21 +13643,17 @@
       <c r="C229" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D229" s="14"/>
+      <c r="D229" s="18" t="s">
+        <v>727</v>
+      </c>
       <c r="E229" s="14"/>
       <c r="F229" s="14"/>
       <c r="G229" s="14"/>
       <c r="H229" s="14"/>
       <c r="I229" s="14"/>
-      <c r="J229" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K229" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L229" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="J229" s="14"/>
+      <c r="K229" s="14"/>
+      <c r="L229" s="14"/>
       <c r="M229" s="14"/>
       <c r="N229" s="14"/>
       <c r="O229" s="14"/>
@@ -13645,30 +13679,18 @@
       <c r="AI229" s="14"/>
     </row>
     <row r="230" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A230" s="14" t="s">
-        <v>268</v>
-      </c>
-      <c r="B230" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C230" s="14" t="s">
-        <v>135</v>
-      </c>
+      <c r="A230" s="14"/>
+      <c r="B230" s="14"/>
+      <c r="C230" s="14"/>
       <c r="D230" s="14"/>
       <c r="E230" s="14"/>
       <c r="F230" s="14"/>
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
       <c r="I230" s="14"/>
-      <c r="J230" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K230" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L230" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="J230" s="14"/>
+      <c r="K230" s="14"/>
+      <c r="L230" s="14"/>
       <c r="M230" s="14"/>
       <c r="N230" s="14"/>
       <c r="O230" s="14"/>
@@ -13693,9 +13715,9 @@
       <c r="AH230" s="14"/>
       <c r="AI230" s="14"/>
     </row>
-    <row r="231" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A231" s="14" t="s">
-        <v>359</v>
+        <v>267</v>
       </c>
       <c r="B231" s="14" t="s">
         <v>174</v>
@@ -13703,9 +13725,36 @@
       <c r="C231" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O231" s="15" t="s">
-        <v>362</v>
-      </c>
+      <c r="D231" s="14"/>
+      <c r="E231" s="14"/>
+      <c r="F231" s="14"/>
+      <c r="G231" s="14"/>
+      <c r="H231" s="14"/>
+      <c r="I231" s="14"/>
+      <c r="J231" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K231" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L231" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M231" s="14"/>
+      <c r="N231" s="14"/>
+      <c r="O231" s="14"/>
+      <c r="P231" s="14"/>
+      <c r="Q231" s="14"/>
+      <c r="R231" s="14"/>
+      <c r="S231" s="14"/>
+      <c r="T231" s="14"/>
+      <c r="U231" s="14"/>
+      <c r="V231" s="14"/>
+      <c r="W231" s="14"/>
+      <c r="X231" s="14"/>
+      <c r="Y231" s="14"/>
+      <c r="Z231" s="14"/>
+      <c r="AA231" s="14"/>
       <c r="AB231" s="14"/>
       <c r="AC231" s="14"/>
       <c r="AD231" s="14"/>
@@ -13715,9 +13764,9 @@
       <c r="AH231" s="14"/>
       <c r="AI231" s="14"/>
     </row>
-    <row r="232" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A232" s="14" t="s">
-        <v>360</v>
+        <v>268</v>
       </c>
       <c r="B232" s="14" t="s">
         <v>174</v>
@@ -13725,9 +13774,36 @@
       <c r="C232" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="O232" s="15" t="s">
-        <v>363</v>
-      </c>
+      <c r="D232" s="14"/>
+      <c r="E232" s="14"/>
+      <c r="F232" s="14"/>
+      <c r="G232" s="14"/>
+      <c r="H232" s="14"/>
+      <c r="I232" s="14"/>
+      <c r="J232" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K232" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L232" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M232" s="14"/>
+      <c r="N232" s="14"/>
+      <c r="O232" s="14"/>
+      <c r="P232" s="14"/>
+      <c r="Q232" s="14"/>
+      <c r="R232" s="14"/>
+      <c r="S232" s="14"/>
+      <c r="T232" s="14"/>
+      <c r="U232" s="14"/>
+      <c r="V232" s="14"/>
+      <c r="W232" s="14"/>
+      <c r="X232" s="14"/>
+      <c r="Y232" s="14"/>
+      <c r="Z232" s="14"/>
+      <c r="AA232" s="14"/>
       <c r="AB232" s="14"/>
       <c r="AC232" s="14"/>
       <c r="AD232" s="14"/>
@@ -13739,7 +13815,7 @@
     </row>
     <row r="233" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A233" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B233" s="14" t="s">
         <v>174</v>
@@ -13748,7 +13824,7 @@
         <v>135</v>
       </c>
       <c r="O233" s="15" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="AB233" s="14"/>
       <c r="AC233" s="14"/>
@@ -13761,7 +13837,7 @@
     </row>
     <row r="234" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A234" s="14" t="s">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="B234" s="14" t="s">
         <v>174</v>
@@ -13769,8 +13845,8 @@
       <c r="C234" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M234" s="14" t="s">
-        <v>371</v>
+      <c r="O234" s="15" t="s">
+        <v>363</v>
       </c>
       <c r="AB234" s="14"/>
       <c r="AC234" s="14"/>
@@ -13782,6 +13858,18 @@
       <c r="AI234" s="14"/>
     </row>
     <row r="235" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A235" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B235" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C235" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O235" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB235" s="14"/>
       <c r="AC235" s="14"/>
       <c r="AD235" s="14"/>
@@ -13792,6 +13880,18 @@
       <c r="AI235" s="14"/>
     </row>
     <row r="236" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A236" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B236" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C236" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M236" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB236" s="14"/>
       <c r="AC236" s="14"/>
       <c r="AD236" s="14"/>
@@ -15485,7 +15585,7 @@
       <c r="AB405" s="14"/>
       <c r="AC405" s="14"/>
       <c r="AD405" s="14"/>
-      <c r="AE405" s="14"/>
+      <c r="AE405" s="27"/>
       <c r="AF405" s="14"/>
       <c r="AG405" s="14"/>
       <c r="AH405" s="14"/>
@@ -15495,7 +15595,7 @@
       <c r="AB406" s="14"/>
       <c r="AC406" s="14"/>
       <c r="AD406" s="14"/>
-      <c r="AE406" s="14"/>
+      <c r="AE406" s="27"/>
       <c r="AF406" s="14"/>
       <c r="AG406" s="14"/>
       <c r="AH406" s="14"/>
@@ -15551,6 +15651,26 @@
       <c r="AH411" s="14"/>
       <c r="AI411" s="14"/>
     </row>
+    <row r="412" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB412" s="14"/>
+      <c r="AC412" s="14"/>
+      <c r="AD412" s="14"/>
+      <c r="AE412" s="14"/>
+      <c r="AF412" s="14"/>
+      <c r="AG412" s="14"/>
+      <c r="AH412" s="14"/>
+      <c r="AI412" s="14"/>
+    </row>
+    <row r="413" spans="28:35" x14ac:dyDescent="0.25">
+      <c r="AB413" s="14"/>
+      <c r="AC413" s="14"/>
+      <c r="AD413" s="14"/>
+      <c r="AE413" s="14"/>
+      <c r="AF413" s="14"/>
+      <c r="AG413" s="14"/>
+      <c r="AH413" s="14"/>
+      <c r="AI413" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15560,7 +15680,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T224"/>
+  <dimension ref="A1:T227"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -21936,13 +22056,13 @@
         <v>637</v>
       </c>
       <c r="C195" s="15" t="s">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="D195" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E195" s="15" t="s">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="F195" s="15"/>
       <c r="G195" s="15"/>
@@ -22738,13 +22858,13 @@
         <v>689</v>
       </c>
       <c r="C218" s="15" t="s">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="D218" s="16" t="s">
         <v>112</v>
       </c>
       <c r="E218" s="15" t="s">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="F218" s="14"/>
       <c r="G218" s="14"/>
@@ -22961,6 +23081,120 @@
       <c r="R224" s="14"/>
       <c r="S224" s="14"/>
       <c r="T224" s="14"/>
+    </row>
+    <row r="225" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A225" s="16" t="s">
+        <v>738</v>
+      </c>
+      <c r="B225" s="20" t="s">
+        <v>666</v>
+      </c>
+      <c r="C225" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D225" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="E225" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F225" s="14"/>
+      <c r="G225" s="14"/>
+      <c r="H225" s="14"/>
+      <c r="I225" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J225" s="14"/>
+      <c r="K225" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L225" s="14"/>
+      <c r="M225" s="14"/>
+      <c r="N225" s="14"/>
+      <c r="O225" s="14"/>
+      <c r="P225" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q225" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R225" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="S225" s="14"/>
+      <c r="T225" s="14"/>
+    </row>
+    <row r="226" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A226" s="15" t="s">
+        <v>741</v>
+      </c>
+      <c r="B226" s="20" t="s">
+        <v>637</v>
+      </c>
+      <c r="C226" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D226" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E226" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F226" s="15"/>
+      <c r="G226" s="15"/>
+      <c r="H226" s="15"/>
+      <c r="I226" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J226" s="14"/>
+      <c r="K226" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L226" s="14"/>
+      <c r="M226" s="14"/>
+      <c r="N226" s="14"/>
+      <c r="O226" s="14"/>
+      <c r="P226" s="14"/>
+      <c r="Q226" s="14"/>
+      <c r="R226" s="14"/>
+      <c r="S226" s="14"/>
+      <c r="T226" s="14"/>
+    </row>
+    <row r="227" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A227" s="16" t="s">
+        <v>742</v>
+      </c>
+      <c r="B227" s="20" t="s">
+        <v>689</v>
+      </c>
+      <c r="C227" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D227" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="E227" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="F227" s="14"/>
+      <c r="G227" s="14"/>
+      <c r="H227" s="14"/>
+      <c r="I227" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="J227" s="14"/>
+      <c r="K227" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="L227" s="14"/>
+      <c r="M227" s="14"/>
+      <c r="N227" s="14"/>
+      <c r="O227" s="14"/>
+      <c r="P227" s="14"/>
+      <c r="Q227" s="14"/>
+      <c r="R227" s="14"/>
+      <c r="S227" s="14"/>
+      <c r="T227" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
Commit the TestData for sanity suite newly developed
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25629"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{507429FE-E851-4644-801C-23EABBFFA112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA424FBD-A670-4A8E-A53D-AF02449716C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20550" windowHeight="10080" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3218" uniqueCount="744">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3218" uniqueCount="745">
   <si>
     <t>1</t>
   </si>
@@ -2260,6 +2260,9 @@
   </si>
   <si>
     <t>1011|1012</t>
+  </si>
+  <si>
+    <t>000-00002-035</t>
   </si>
 </sst>
 </file>
@@ -22891,7 +22894,7 @@
         <v>721</v>
       </c>
       <c r="B219" s="20" t="s">
-        <v>728</v>
+        <v>744</v>
       </c>
       <c r="C219" s="15" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
Commit the five customer scenarios and vendor portal scenarios update
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA424FBD-A670-4A8E-A53D-AF02449716C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19EDAC81-2B52-4330-8F1C-8343CE4D8835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20550" windowHeight="10080" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3218" uniqueCount="745">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3296" uniqueCount="768">
   <si>
     <t>1</t>
   </si>
@@ -2263,6 +2263,75 @@
   </si>
   <si>
     <t>000-00002-035</t>
+  </si>
+  <si>
+    <t>THH_KelliScenario001</t>
+  </si>
+  <si>
+    <t>THH</t>
+  </si>
+  <si>
+    <t>1013</t>
+  </si>
+  <si>
+    <t>FUJ_KelliScenario001</t>
+  </si>
+  <si>
+    <t>FUJ</t>
+  </si>
+  <si>
+    <t>1014</t>
+  </si>
+  <si>
+    <t>THM_KelliScenario001</t>
+  </si>
+  <si>
+    <t>THM</t>
+  </si>
+  <si>
+    <t>1015</t>
+  </si>
+  <si>
+    <t>TRN_KelliScenario001</t>
+  </si>
+  <si>
+    <t>TRN</t>
+  </si>
+  <si>
+    <t>1016|1017</t>
+  </si>
+  <si>
+    <t>TRON</t>
+  </si>
+  <si>
+    <t>ILW_KelliScenario001</t>
+  </si>
+  <si>
+    <t>ILW</t>
+  </si>
+  <si>
+    <t>1018</t>
+  </si>
+  <si>
+    <t>003-111780-03</t>
+  </si>
+  <si>
+    <t>003X6451-K</t>
+  </si>
+  <si>
+    <t>1295-10-118-1</t>
+  </si>
+  <si>
+    <t>1016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8350202301                     </t>
+  </si>
+  <si>
+    <t>1017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00026315089                        </t>
   </si>
 </sst>
 </file>
@@ -2424,7 +2493,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2465,6 +2534,7 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
@@ -2806,7 +2876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI413"/>
+  <dimension ref="A1:AI400"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="14" customWidth="1"/>
@@ -13682,15 +13752,25 @@
       <c r="AI229" s="14"/>
     </row>
     <row r="230" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A230" s="14"/>
-      <c r="B230" s="14"/>
-      <c r="C230" s="14"/>
-      <c r="D230" s="14"/>
+      <c r="A230" s="14" t="s">
+        <v>745</v>
+      </c>
+      <c r="B230" s="14" t="s">
+        <v>746</v>
+      </c>
+      <c r="C230" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D230" s="18" t="s">
+        <v>747</v>
+      </c>
       <c r="E230" s="14"/>
       <c r="F230" s="14"/>
       <c r="G230" s="14"/>
       <c r="H230" s="14"/>
-      <c r="I230" s="14"/>
+      <c r="I230" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="J230" s="14"/>
       <c r="K230" s="14"/>
       <c r="L230" s="14"/>
@@ -13712,7 +13792,9 @@
       <c r="AB230" s="14"/>
       <c r="AC230" s="14"/>
       <c r="AD230" s="14"/>
-      <c r="AE230" s="27"/>
+      <c r="AE230" s="27" t="s">
+        <v>746</v>
+      </c>
       <c r="AF230" s="14"/>
       <c r="AG230" s="14"/>
       <c r="AH230" s="14"/>
@@ -13720,29 +13802,27 @@
     </row>
     <row r="231" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A231" s="14" t="s">
-        <v>267</v>
+        <v>751</v>
       </c>
       <c r="B231" s="14" t="s">
-        <v>174</v>
+        <v>752</v>
       </c>
       <c r="C231" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D231" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D231" s="18" t="s">
+        <v>753</v>
+      </c>
       <c r="E231" s="14"/>
       <c r="F231" s="14"/>
       <c r="G231" s="14"/>
       <c r="H231" s="14"/>
-      <c r="I231" s="14"/>
-      <c r="J231" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="K231" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="L231" s="15" t="s">
-        <v>275</v>
-      </c>
+      <c r="I231" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="J231" s="14"/>
+      <c r="K231" s="14"/>
+      <c r="L231" s="14"/>
       <c r="M231" s="14"/>
       <c r="N231" s="14"/>
       <c r="O231" s="14"/>
@@ -13761,7 +13841,9 @@
       <c r="AB231" s="14"/>
       <c r="AC231" s="14"/>
       <c r="AD231" s="14"/>
-      <c r="AE231" s="27"/>
+      <c r="AE231" s="27" t="s">
+        <v>752</v>
+      </c>
       <c r="AF231" s="14"/>
       <c r="AG231" s="14"/>
       <c r="AH231" s="14"/>
@@ -13769,29 +13851,27 @@
     </row>
     <row r="232" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A232" s="14" t="s">
-        <v>268</v>
+        <v>754</v>
       </c>
       <c r="B232" s="14" t="s">
-        <v>174</v>
+        <v>755</v>
       </c>
       <c r="C232" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="D232" s="14"/>
+        <v>614</v>
+      </c>
+      <c r="D232" s="18" t="s">
+        <v>756</v>
+      </c>
       <c r="E232" s="14"/>
       <c r="F232" s="14"/>
       <c r="G232" s="14"/>
       <c r="H232" s="14"/>
-      <c r="I232" s="14"/>
-      <c r="J232" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="K232" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="L232" s="15" t="s">
-        <v>276</v>
-      </c>
+      <c r="I232" s="14" t="s">
+        <v>378</v>
+      </c>
+      <c r="J232" s="14"/>
+      <c r="K232" s="14"/>
+      <c r="L232" s="14"/>
       <c r="M232" s="14"/>
       <c r="N232" s="14"/>
       <c r="O232" s="14"/>
@@ -13810,69 +13890,140 @@
       <c r="AB232" s="14"/>
       <c r="AC232" s="14"/>
       <c r="AD232" s="14"/>
-      <c r="AE232" s="27"/>
+      <c r="AE232" s="27" t="s">
+        <v>757</v>
+      </c>
       <c r="AF232" s="14"/>
       <c r="AG232" s="14"/>
       <c r="AH232" s="14"/>
       <c r="AI232" s="14"/>
     </row>
-    <row r="233" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A233" s="14" t="s">
-        <v>359</v>
+        <v>758</v>
       </c>
       <c r="B233" s="14" t="s">
-        <v>174</v>
+        <v>759</v>
       </c>
       <c r="C233" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O233" s="15" t="s">
-        <v>362</v>
-      </c>
+        <v>614</v>
+      </c>
+      <c r="D233" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="E233" s="14"/>
+      <c r="F233" s="14"/>
+      <c r="G233" s="14"/>
+      <c r="H233" s="14"/>
+      <c r="I233" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="J233" s="14"/>
+      <c r="K233" s="14"/>
+      <c r="L233" s="14"/>
+      <c r="M233" s="14"/>
+      <c r="N233" s="14"/>
+      <c r="O233" s="14"/>
+      <c r="P233" s="14"/>
+      <c r="Q233" s="14"/>
+      <c r="R233" s="14"/>
+      <c r="S233" s="14"/>
+      <c r="T233" s="14"/>
+      <c r="U233" s="14"/>
+      <c r="V233" s="14"/>
+      <c r="W233" s="14"/>
+      <c r="X233" s="14"/>
+      <c r="Y233" s="14"/>
+      <c r="Z233" s="14"/>
+      <c r="AA233" s="14"/>
       <c r="AB233" s="14"/>
       <c r="AC233" s="14"/>
       <c r="AD233" s="14"/>
-      <c r="AE233" s="27"/>
+      <c r="AE233" s="27" t="s">
+        <v>759</v>
+      </c>
       <c r="AF233" s="14"/>
       <c r="AG233" s="14"/>
       <c r="AH233" s="14"/>
       <c r="AI233" s="14"/>
     </row>
-    <row r="234" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A234" s="14" t="s">
-        <v>360</v>
+        <v>748</v>
       </c>
       <c r="B234" s="14" t="s">
-        <v>174</v>
+        <v>749</v>
       </c>
       <c r="C234" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O234" s="15" t="s">
-        <v>363</v>
-      </c>
+        <v>614</v>
+      </c>
+      <c r="D234" s="18" t="s">
+        <v>750</v>
+      </c>
+      <c r="E234" s="14"/>
+      <c r="F234" s="14"/>
+      <c r="G234" s="14"/>
+      <c r="H234" s="14"/>
+      <c r="I234" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="J234" s="14"/>
+      <c r="K234" s="14"/>
+      <c r="L234" s="14"/>
+      <c r="M234" s="14"/>
+      <c r="N234" s="14"/>
+      <c r="O234" s="14"/>
+      <c r="P234" s="14"/>
+      <c r="Q234" s="14"/>
+      <c r="R234" s="14"/>
+      <c r="S234" s="14"/>
+      <c r="T234" s="14"/>
+      <c r="U234" s="14"/>
+      <c r="V234" s="14"/>
+      <c r="W234" s="14"/>
+      <c r="X234" s="14"/>
+      <c r="Y234" s="14"/>
+      <c r="Z234" s="14"/>
+      <c r="AA234" s="14"/>
       <c r="AB234" s="14"/>
       <c r="AC234" s="14"/>
       <c r="AD234" s="14"/>
-      <c r="AE234" s="27"/>
+      <c r="AE234" s="27" t="s">
+        <v>749</v>
+      </c>
       <c r="AF234" s="14"/>
       <c r="AG234" s="14"/>
       <c r="AH234" s="14"/>
       <c r="AI234" s="14"/>
     </row>
-    <row r="235" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A235" s="14" t="s">
-        <v>361</v>
-      </c>
-      <c r="B235" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C235" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O235" s="15" t="s">
-        <v>364</v>
-      </c>
+    <row r="235" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A235" s="14"/>
+      <c r="B235" s="14"/>
+      <c r="C235" s="14"/>
+      <c r="D235" s="14"/>
+      <c r="E235" s="14"/>
+      <c r="F235" s="14"/>
+      <c r="G235" s="14"/>
+      <c r="H235" s="14"/>
+      <c r="I235" s="14"/>
+      <c r="J235" s="14"/>
+      <c r="K235" s="14"/>
+      <c r="L235" s="14"/>
+      <c r="M235" s="14"/>
+      <c r="N235" s="14"/>
+      <c r="O235" s="14"/>
+      <c r="P235" s="14"/>
+      <c r="Q235" s="14"/>
+      <c r="R235" s="14"/>
+      <c r="S235" s="14"/>
+      <c r="T235" s="14"/>
+      <c r="U235" s="14"/>
+      <c r="V235" s="14"/>
+      <c r="W235" s="14"/>
+      <c r="X235" s="14"/>
+      <c r="Y235" s="14"/>
+      <c r="Z235" s="14"/>
+      <c r="AA235" s="14"/>
       <c r="AB235" s="14"/>
       <c r="AC235" s="14"/>
       <c r="AD235" s="14"/>
@@ -13882,9 +14033,9 @@
       <c r="AH235" s="14"/>
       <c r="AI235" s="14"/>
     </row>
-    <row r="236" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A236" s="14" t="s">
-        <v>370</v>
+        <v>267</v>
       </c>
       <c r="B236" s="14" t="s">
         <v>174</v>
@@ -13892,9 +14043,36 @@
       <c r="C236" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="M236" s="14" t="s">
-        <v>371</v>
-      </c>
+      <c r="D236" s="14"/>
+      <c r="E236" s="14"/>
+      <c r="F236" s="14"/>
+      <c r="G236" s="14"/>
+      <c r="H236" s="14"/>
+      <c r="I236" s="14"/>
+      <c r="J236" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="K236" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="L236" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="M236" s="14"/>
+      <c r="N236" s="14"/>
+      <c r="O236" s="14"/>
+      <c r="P236" s="14"/>
+      <c r="Q236" s="14"/>
+      <c r="R236" s="14"/>
+      <c r="S236" s="14"/>
+      <c r="T236" s="14"/>
+      <c r="U236" s="14"/>
+      <c r="V236" s="14"/>
+      <c r="W236" s="14"/>
+      <c r="X236" s="14"/>
+      <c r="Y236" s="14"/>
+      <c r="Z236" s="14"/>
+      <c r="AA236" s="14"/>
       <c r="AB236" s="14"/>
       <c r="AC236" s="14"/>
       <c r="AD236" s="14"/>
@@ -13904,7 +14082,46 @@
       <c r="AH236" s="14"/>
       <c r="AI236" s="14"/>
     </row>
-    <row r="237" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A237" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="B237" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C237" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D237" s="14"/>
+      <c r="E237" s="14"/>
+      <c r="F237" s="14"/>
+      <c r="G237" s="14"/>
+      <c r="H237" s="14"/>
+      <c r="I237" s="14"/>
+      <c r="J237" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K237" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L237" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="M237" s="14"/>
+      <c r="N237" s="14"/>
+      <c r="O237" s="14"/>
+      <c r="P237" s="14"/>
+      <c r="Q237" s="14"/>
+      <c r="R237" s="14"/>
+      <c r="S237" s="14"/>
+      <c r="T237" s="14"/>
+      <c r="U237" s="14"/>
+      <c r="V237" s="14"/>
+      <c r="W237" s="14"/>
+      <c r="X237" s="14"/>
+      <c r="Y237" s="14"/>
+      <c r="Z237" s="14"/>
+      <c r="AA237" s="14"/>
       <c r="AB237" s="14"/>
       <c r="AC237" s="14"/>
       <c r="AD237" s="14"/>
@@ -13915,6 +14132,18 @@
       <c r="AI237" s="14"/>
     </row>
     <row r="238" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A238" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="B238" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C238" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O238" s="15" t="s">
+        <v>362</v>
+      </c>
       <c r="AB238" s="14"/>
       <c r="AC238" s="14"/>
       <c r="AD238" s="14"/>
@@ -13925,6 +14154,18 @@
       <c r="AI238" s="14"/>
     </row>
     <row r="239" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A239" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B239" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C239" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O239" s="15" t="s">
+        <v>363</v>
+      </c>
       <c r="AB239" s="14"/>
       <c r="AC239" s="14"/>
       <c r="AD239" s="14"/>
@@ -13935,6 +14176,18 @@
       <c r="AI239" s="14"/>
     </row>
     <row r="240" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A240" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="B240" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C240" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="O240" s="15" t="s">
+        <v>364</v>
+      </c>
       <c r="AB240" s="14"/>
       <c r="AC240" s="14"/>
       <c r="AD240" s="14"/>
@@ -13944,7 +14197,19 @@
       <c r="AH240" s="14"/>
       <c r="AI240" s="14"/>
     </row>
-    <row r="241" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A241" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B241" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C241" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="M241" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="AB241" s="14"/>
       <c r="AC241" s="14"/>
       <c r="AD241" s="14"/>
@@ -13954,7 +14219,7 @@
       <c r="AH241" s="14"/>
       <c r="AI241" s="14"/>
     </row>
-    <row r="242" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB242" s="14"/>
       <c r="AC242" s="14"/>
       <c r="AD242" s="14"/>
@@ -13964,7 +14229,7 @@
       <c r="AH242" s="14"/>
       <c r="AI242" s="14"/>
     </row>
-    <row r="243" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB243" s="14"/>
       <c r="AC243" s="14"/>
       <c r="AD243" s="14"/>
@@ -13974,7 +14239,7 @@
       <c r="AH243" s="14"/>
       <c r="AI243" s="14"/>
     </row>
-    <row r="244" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB244" s="14"/>
       <c r="AC244" s="14"/>
       <c r="AD244" s="14"/>
@@ -13984,7 +14249,7 @@
       <c r="AH244" s="14"/>
       <c r="AI244" s="14"/>
     </row>
-    <row r="245" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB245" s="14"/>
       <c r="AC245" s="14"/>
       <c r="AD245" s="14"/>
@@ -13994,7 +14259,7 @@
       <c r="AH245" s="14"/>
       <c r="AI245" s="14"/>
     </row>
-    <row r="246" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB246" s="14"/>
       <c r="AC246" s="14"/>
       <c r="AD246" s="14"/>
@@ -14004,7 +14269,7 @@
       <c r="AH246" s="14"/>
       <c r="AI246" s="14"/>
     </row>
-    <row r="247" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB247" s="14"/>
       <c r="AC247" s="14"/>
       <c r="AD247" s="14"/>
@@ -14014,7 +14279,7 @@
       <c r="AH247" s="14"/>
       <c r="AI247" s="14"/>
     </row>
-    <row r="248" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB248" s="14"/>
       <c r="AC248" s="14"/>
       <c r="AD248" s="14"/>
@@ -14024,7 +14289,7 @@
       <c r="AH248" s="14"/>
       <c r="AI248" s="14"/>
     </row>
-    <row r="249" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB249" s="14"/>
       <c r="AC249" s="14"/>
       <c r="AD249" s="14"/>
@@ -14034,7 +14299,7 @@
       <c r="AH249" s="14"/>
       <c r="AI249" s="14"/>
     </row>
-    <row r="250" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB250" s="14"/>
       <c r="AC250" s="14"/>
       <c r="AD250" s="14"/>
@@ -14044,7 +14309,7 @@
       <c r="AH250" s="14"/>
       <c r="AI250" s="14"/>
     </row>
-    <row r="251" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB251" s="14"/>
       <c r="AC251" s="14"/>
       <c r="AD251" s="14"/>
@@ -14054,7 +14319,7 @@
       <c r="AH251" s="14"/>
       <c r="AI251" s="14"/>
     </row>
-    <row r="252" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB252" s="14"/>
       <c r="AC252" s="14"/>
       <c r="AD252" s="14"/>
@@ -14064,7 +14329,7 @@
       <c r="AH252" s="14"/>
       <c r="AI252" s="14"/>
     </row>
-    <row r="253" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB253" s="14"/>
       <c r="AC253" s="14"/>
       <c r="AD253" s="14"/>
@@ -14074,7 +14339,7 @@
       <c r="AH253" s="14"/>
       <c r="AI253" s="14"/>
     </row>
-    <row r="254" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB254" s="14"/>
       <c r="AC254" s="14"/>
       <c r="AD254" s="14"/>
@@ -14084,7 +14349,7 @@
       <c r="AH254" s="14"/>
       <c r="AI254" s="14"/>
     </row>
-    <row r="255" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB255" s="14"/>
       <c r="AC255" s="14"/>
       <c r="AD255" s="14"/>
@@ -14094,7 +14359,7 @@
       <c r="AH255" s="14"/>
       <c r="AI255" s="14"/>
     </row>
-    <row r="256" spans="28:35" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AB256" s="14"/>
       <c r="AC256" s="14"/>
       <c r="AD256" s="14"/>
@@ -15478,7 +15743,7 @@
       <c r="AB394" s="14"/>
       <c r="AC394" s="14"/>
       <c r="AD394" s="14"/>
-      <c r="AE394" s="27"/>
+      <c r="AE394" s="14"/>
       <c r="AF394" s="14"/>
       <c r="AG394" s="14"/>
       <c r="AH394" s="14"/>
@@ -15488,7 +15753,7 @@
       <c r="AB395" s="14"/>
       <c r="AC395" s="14"/>
       <c r="AD395" s="14"/>
-      <c r="AE395" s="27"/>
+      <c r="AE395" s="14"/>
       <c r="AF395" s="14"/>
       <c r="AG395" s="14"/>
       <c r="AH395" s="14"/>
@@ -15498,7 +15763,7 @@
       <c r="AB396" s="14"/>
       <c r="AC396" s="14"/>
       <c r="AD396" s="14"/>
-      <c r="AE396" s="27"/>
+      <c r="AE396" s="14"/>
       <c r="AF396" s="14"/>
       <c r="AG396" s="14"/>
       <c r="AH396" s="14"/>
@@ -15508,7 +15773,7 @@
       <c r="AB397" s="14"/>
       <c r="AC397" s="14"/>
       <c r="AD397" s="14"/>
-      <c r="AE397" s="27"/>
+      <c r="AE397" s="14"/>
       <c r="AF397" s="14"/>
       <c r="AG397" s="14"/>
       <c r="AH397" s="14"/>
@@ -15518,7 +15783,7 @@
       <c r="AB398" s="14"/>
       <c r="AC398" s="14"/>
       <c r="AD398" s="14"/>
-      <c r="AE398" s="27"/>
+      <c r="AE398" s="14"/>
       <c r="AF398" s="14"/>
       <c r="AG398" s="14"/>
       <c r="AH398" s="14"/>
@@ -15528,7 +15793,7 @@
       <c r="AB399" s="14"/>
       <c r="AC399" s="14"/>
       <c r="AD399" s="14"/>
-      <c r="AE399" s="27"/>
+      <c r="AE399" s="14"/>
       <c r="AF399" s="14"/>
       <c r="AG399" s="14"/>
       <c r="AH399" s="14"/>
@@ -15538,141 +15803,11 @@
       <c r="AB400" s="14"/>
       <c r="AC400" s="14"/>
       <c r="AD400" s="14"/>
-      <c r="AE400" s="27"/>
+      <c r="AE400" s="14"/>
       <c r="AF400" s="14"/>
       <c r="AG400" s="14"/>
       <c r="AH400" s="14"/>
       <c r="AI400" s="14"/>
-    </row>
-    <row r="401" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB401" s="14"/>
-      <c r="AC401" s="14"/>
-      <c r="AD401" s="14"/>
-      <c r="AE401" s="27"/>
-      <c r="AF401" s="14"/>
-      <c r="AG401" s="14"/>
-      <c r="AH401" s="14"/>
-      <c r="AI401" s="14"/>
-    </row>
-    <row r="402" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB402" s="14"/>
-      <c r="AC402" s="14"/>
-      <c r="AD402" s="14"/>
-      <c r="AE402" s="27"/>
-      <c r="AF402" s="14"/>
-      <c r="AG402" s="14"/>
-      <c r="AH402" s="14"/>
-      <c r="AI402" s="14"/>
-    </row>
-    <row r="403" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB403" s="14"/>
-      <c r="AC403" s="14"/>
-      <c r="AD403" s="14"/>
-      <c r="AE403" s="27"/>
-      <c r="AF403" s="14"/>
-      <c r="AG403" s="14"/>
-      <c r="AH403" s="14"/>
-      <c r="AI403" s="14"/>
-    </row>
-    <row r="404" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB404" s="14"/>
-      <c r="AC404" s="14"/>
-      <c r="AD404" s="14"/>
-      <c r="AE404" s="27"/>
-      <c r="AF404" s="14"/>
-      <c r="AG404" s="14"/>
-      <c r="AH404" s="14"/>
-      <c r="AI404" s="14"/>
-    </row>
-    <row r="405" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB405" s="14"/>
-      <c r="AC405" s="14"/>
-      <c r="AD405" s="14"/>
-      <c r="AE405" s="27"/>
-      <c r="AF405" s="14"/>
-      <c r="AG405" s="14"/>
-      <c r="AH405" s="14"/>
-      <c r="AI405" s="14"/>
-    </row>
-    <row r="406" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB406" s="14"/>
-      <c r="AC406" s="14"/>
-      <c r="AD406" s="14"/>
-      <c r="AE406" s="27"/>
-      <c r="AF406" s="14"/>
-      <c r="AG406" s="14"/>
-      <c r="AH406" s="14"/>
-      <c r="AI406" s="14"/>
-    </row>
-    <row r="407" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB407" s="14"/>
-      <c r="AC407" s="14"/>
-      <c r="AD407" s="14"/>
-      <c r="AE407" s="14"/>
-      <c r="AF407" s="14"/>
-      <c r="AG407" s="14"/>
-      <c r="AH407" s="14"/>
-      <c r="AI407" s="14"/>
-    </row>
-    <row r="408" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB408" s="14"/>
-      <c r="AC408" s="14"/>
-      <c r="AD408" s="14"/>
-      <c r="AE408" s="14"/>
-      <c r="AF408" s="14"/>
-      <c r="AG408" s="14"/>
-      <c r="AH408" s="14"/>
-      <c r="AI408" s="14"/>
-    </row>
-    <row r="409" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB409" s="14"/>
-      <c r="AC409" s="14"/>
-      <c r="AD409" s="14"/>
-      <c r="AE409" s="14"/>
-      <c r="AF409" s="14"/>
-      <c r="AG409" s="14"/>
-      <c r="AH409" s="14"/>
-      <c r="AI409" s="14"/>
-    </row>
-    <row r="410" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB410" s="14"/>
-      <c r="AC410" s="14"/>
-      <c r="AD410" s="14"/>
-      <c r="AE410" s="14"/>
-      <c r="AF410" s="14"/>
-      <c r="AG410" s="14"/>
-      <c r="AH410" s="14"/>
-      <c r="AI410" s="14"/>
-    </row>
-    <row r="411" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB411" s="14"/>
-      <c r="AC411" s="14"/>
-      <c r="AD411" s="14"/>
-      <c r="AE411" s="14"/>
-      <c r="AF411" s="14"/>
-      <c r="AG411" s="14"/>
-      <c r="AH411" s="14"/>
-      <c r="AI411" s="14"/>
-    </row>
-    <row r="412" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB412" s="14"/>
-      <c r="AC412" s="14"/>
-      <c r="AD412" s="14"/>
-      <c r="AE412" s="14"/>
-      <c r="AF412" s="14"/>
-      <c r="AG412" s="14"/>
-      <c r="AH412" s="14"/>
-      <c r="AI412" s="14"/>
-    </row>
-    <row r="413" spans="28:35" x14ac:dyDescent="0.25">
-      <c r="AB413" s="14"/>
-      <c r="AC413" s="14"/>
-      <c r="AD413" s="14"/>
-      <c r="AE413" s="14"/>
-      <c r="AF413" s="14"/>
-      <c r="AG413" s="14"/>
-      <c r="AH413" s="14"/>
-      <c r="AI413" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -15683,7 +15818,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T227"/>
+  <dimension ref="A1:T233"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="14" bestFit="1" customWidth="1"/>
@@ -23199,6 +23334,162 @@
       <c r="S227" s="14"/>
       <c r="T227" s="14"/>
     </row>
+    <row r="228" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A228" s="15" t="s">
+        <v>747</v>
+      </c>
+      <c r="B228" s="30" t="s">
+        <v>761</v>
+      </c>
+      <c r="C228" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D228" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E228" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="I228" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="K228" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="R228" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="229" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A229" s="15" t="s">
+        <v>750</v>
+      </c>
+      <c r="B229" s="30" t="s">
+        <v>762</v>
+      </c>
+      <c r="C229" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D229" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E229" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="I229" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="K229" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="R229" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="230" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A230" s="15" t="s">
+        <v>753</v>
+      </c>
+      <c r="B230" s="32" t="s">
+        <v>763</v>
+      </c>
+      <c r="C230" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D230" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E230" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="I230" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="K230" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="R230" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="231" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A231" s="15" t="s">
+        <v>764</v>
+      </c>
+      <c r="B231" s="15" t="s">
+        <v>765</v>
+      </c>
+      <c r="C231" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D231" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E231" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="I231" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="K231" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="R231" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="232" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A232" s="15" t="s">
+        <v>766</v>
+      </c>
+      <c r="B232" s="15" t="s">
+        <v>765</v>
+      </c>
+      <c r="C232" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D232" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E232" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="I232" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="K232" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="R232" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="233" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A233" s="15" t="s">
+        <v>760</v>
+      </c>
+      <c r="B233" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="C233" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D233" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E233" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="I233" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="K233" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="R233" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Commit after update TestData for THH Customer
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ffd-sys-team\git\eai-3534455-ffd-manhattan-automationtesting\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50BCCF10-0B91-4F1D-83FC-D833C013A62E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA1276B-C557-4EBB-933D-C105DC5F5AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3296" uniqueCount="768">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3310" uniqueCount="771">
   <si>
     <t>ScearioID</t>
   </si>
@@ -2342,6 +2342,15 @@
   </si>
   <si>
     <t>FedEx Will Call</t>
+  </si>
+  <si>
+    <t>THH_KelliScenario002</t>
+  </si>
+  <si>
+    <t>1019</t>
+  </si>
+  <si>
+    <t>1374-200-002</t>
   </si>
 </sst>
 </file>
@@ -2812,7 +2821,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA0C8091-AB5D-461B-B4FE-5D2410DFE16F}">
-  <dimension ref="A1:AI242"/>
+  <dimension ref="A1:AI243"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -14581,15 +14590,25 @@
       <c r="AI235" s="4"/>
     </row>
     <row r="236" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A236" s="4"/>
-      <c r="B236" s="4"/>
-      <c r="C236" s="4"/>
-      <c r="D236" s="4"/>
+      <c r="A236" s="4" t="s">
+        <v>768</v>
+      </c>
+      <c r="B236" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="C236" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D236" s="5" t="s">
+        <v>769</v>
+      </c>
       <c r="E236" s="4"/>
       <c r="F236" s="4"/>
       <c r="G236" s="4"/>
       <c r="H236" s="4"/>
-      <c r="I236" s="4"/>
+      <c r="I236" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="J236" s="4"/>
       <c r="K236" s="4"/>
       <c r="L236" s="4"/>
@@ -14611,37 +14630,27 @@
       <c r="AB236" s="4"/>
       <c r="AC236" s="4"/>
       <c r="AD236" s="4"/>
-      <c r="AE236" s="4"/>
+      <c r="AE236" s="4" t="s">
+        <v>496</v>
+      </c>
       <c r="AF236" s="4"/>
       <c r="AG236" s="4"/>
       <c r="AH236" s="4"/>
       <c r="AI236" s="4"/>
     </row>
     <row r="237" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A237" s="4" t="s">
-        <v>511</v>
-      </c>
-      <c r="B237" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C237" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="A237" s="4"/>
+      <c r="B237" s="4"/>
+      <c r="C237" s="4"/>
       <c r="D237" s="4"/>
       <c r="E237" s="4"/>
       <c r="F237" s="4"/>
       <c r="G237" s="4"/>
       <c r="H237" s="4"/>
       <c r="I237" s="4"/>
-      <c r="J237" s="3" t="s">
-        <v>512</v>
-      </c>
-      <c r="K237" s="3" t="s">
-        <v>513</v>
-      </c>
-      <c r="L237" s="3" t="s">
-        <v>514</v>
-      </c>
+      <c r="J237" s="4"/>
+      <c r="K237" s="4"/>
+      <c r="L237" s="4"/>
       <c r="M237" s="4"/>
       <c r="N237" s="4"/>
       <c r="O237" s="4"/>
@@ -14668,7 +14677,7 @@
     </row>
     <row r="238" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A238" s="4" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="B238" s="4" t="s">
         <v>228</v>
@@ -14683,13 +14692,13 @@
       <c r="H238" s="4"/>
       <c r="I238" s="4"/>
       <c r="J238" s="3" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="K238" s="3" t="s">
-        <v>243</v>
+        <v>513</v>
       </c>
       <c r="L238" s="3" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="M238" s="4"/>
       <c r="N238" s="4"/>
@@ -14717,7 +14726,7 @@
     </row>
     <row r="239" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A239" s="4" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="B239" s="4" t="s">
         <v>228</v>
@@ -14731,14 +14740,18 @@
       <c r="G239" s="4"/>
       <c r="H239" s="4"/>
       <c r="I239" s="4"/>
-      <c r="J239" s="4"/>
-      <c r="K239" s="4"/>
-      <c r="L239" s="4"/>
+      <c r="J239" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="K239" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="L239" s="3" t="s">
+        <v>517</v>
+      </c>
       <c r="M239" s="4"/>
       <c r="N239" s="4"/>
-      <c r="O239" s="3" t="s">
-        <v>519</v>
-      </c>
+      <c r="O239" s="4"/>
       <c r="P239" s="4"/>
       <c r="Q239" s="4"/>
       <c r="R239" s="4"/>
@@ -14762,7 +14775,7 @@
     </row>
     <row r="240" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A240" s="4" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="B240" s="4" t="s">
         <v>228</v>
@@ -14782,7 +14795,7 @@
       <c r="M240" s="4"/>
       <c r="N240" s="4"/>
       <c r="O240" s="3" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="P240" s="4"/>
       <c r="Q240" s="4"/>
@@ -14807,7 +14820,7 @@
     </row>
     <row r="241" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A241" s="4" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="B241" s="4" t="s">
         <v>228</v>
@@ -14827,7 +14840,7 @@
       <c r="M241" s="4"/>
       <c r="N241" s="4"/>
       <c r="O241" s="3" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="P241" s="4"/>
       <c r="Q241" s="4"/>
@@ -14852,7 +14865,7 @@
     </row>
     <row r="242" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A242" s="4" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="B242" s="4" t="s">
         <v>228</v>
@@ -14869,11 +14882,11 @@
       <c r="J242" s="4"/>
       <c r="K242" s="4"/>
       <c r="L242" s="4"/>
-      <c r="M242" s="4" t="s">
-        <v>525</v>
-      </c>
+      <c r="M242" s="4"/>
       <c r="N242" s="4"/>
-      <c r="O242" s="4"/>
+      <c r="O242" s="3" t="s">
+        <v>523</v>
+      </c>
       <c r="P242" s="4"/>
       <c r="Q242" s="4"/>
       <c r="R242" s="4"/>
@@ -14895,6 +14908,51 @@
       <c r="AH242" s="4"/>
       <c r="AI242" s="4"/>
     </row>
+    <row r="243" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A243" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B243" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C243" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D243" s="4"/>
+      <c r="E243" s="4"/>
+      <c r="F243" s="4"/>
+      <c r="G243" s="4"/>
+      <c r="H243" s="4"/>
+      <c r="I243" s="4"/>
+      <c r="J243" s="4"/>
+      <c r="K243" s="4"/>
+      <c r="L243" s="4"/>
+      <c r="M243" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="N243" s="4"/>
+      <c r="O243" s="4"/>
+      <c r="P243" s="4"/>
+      <c r="Q243" s="4"/>
+      <c r="R243" s="4"/>
+      <c r="S243" s="4"/>
+      <c r="T243" s="4"/>
+      <c r="U243" s="4"/>
+      <c r="V243" s="4"/>
+      <c r="W243" s="4"/>
+      <c r="X243" s="4"/>
+      <c r="Y243" s="4"/>
+      <c r="Z243" s="4"/>
+      <c r="AA243" s="4"/>
+      <c r="AB243" s="4"/>
+      <c r="AC243" s="4"/>
+      <c r="AD243" s="4"/>
+      <c r="AE243" s="4"/>
+      <c r="AF243" s="4"/>
+      <c r="AG243" s="4"/>
+      <c r="AH243" s="4"/>
+      <c r="AI243" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14902,7 +14960,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B611D72-2CC2-4CCA-A1E6-2A10215873D6}">
-  <dimension ref="A1:T233"/>
+  <dimension ref="A1:T234"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -23224,6 +23282,44 @@
       <c r="S233" s="4"/>
       <c r="T233" s="4"/>
     </row>
+    <row r="234" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A234" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="B234" s="5" t="s">
+        <v>770</v>
+      </c>
+      <c r="C234" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D234" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E234" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F234" s="4"/>
+      <c r="G234" s="4"/>
+      <c r="H234" s="4"/>
+      <c r="I234" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="J234" s="4"/>
+      <c r="K234" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="L234" s="4"/>
+      <c r="M234" s="4"/>
+      <c r="N234" s="4"/>
+      <c r="O234" s="4"/>
+      <c r="P234" s="4"/>
+      <c r="Q234" s="4"/>
+      <c r="R234" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="S234" s="4"/>
+      <c r="T234" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
commit chromedriver and other classes for four customer OB Scenario
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ffd-sys-team\git\eai-3534455-ffd-manhattan-automationtesting\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ffd-sys-team\git\eai-3534455-ffd-manhattan-automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA1276B-C557-4EBB-933D-C105DC5F5AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8721D447-296C-4CCC-A3F2-E86366ABA4C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3310" uniqueCount="771">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3351" uniqueCount="778">
   <si>
     <t>ScearioID</t>
   </si>
@@ -2351,6 +2351,27 @@
   </si>
   <si>
     <t>1374-200-002</t>
+  </si>
+  <si>
+    <t>1020</t>
+  </si>
+  <si>
+    <t>THH_OBScenario1</t>
+  </si>
+  <si>
+    <t>1021</t>
+  </si>
+  <si>
+    <t>ILW_OBScenario1</t>
+  </si>
+  <si>
+    <t>1022</t>
+  </si>
+  <si>
+    <t>THM_OBScenario1</t>
+  </si>
+  <si>
+    <t>00026315089</t>
   </si>
 </sst>
 </file>
@@ -2821,7 +2842,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA0C8091-AB5D-461B-B4FE-5D2410DFE16F}">
-  <dimension ref="A1:AI243"/>
+  <dimension ref="A1:AI246"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -14140,9 +14161,7 @@
       <c r="J226" s="4"/>
       <c r="K226" s="4"/>
       <c r="L226" s="4"/>
-      <c r="M226" s="4" t="s">
-        <v>488</v>
-      </c>
+      <c r="M226" s="4"/>
       <c r="N226" s="4"/>
       <c r="O226" s="4"/>
       <c r="P226" s="4"/>
@@ -14639,21 +14658,31 @@
       <c r="AI236" s="4"/>
     </row>
     <row r="237" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A237" s="4"/>
-      <c r="B237" s="4"/>
-      <c r="C237" s="4"/>
-      <c r="D237" s="4"/>
+      <c r="A237" s="4" t="s">
+        <v>776</v>
+      </c>
+      <c r="B237" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="C237" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D237" s="5" t="s">
+        <v>771</v>
+      </c>
       <c r="E237" s="4"/>
       <c r="F237" s="4"/>
       <c r="G237" s="4"/>
       <c r="H237" s="4"/>
-      <c r="I237" s="4"/>
+      <c r="I237" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="J237" s="4"/>
       <c r="K237" s="4"/>
       <c r="L237" s="4"/>
-      <c r="M237" s="4"/>
+      <c r="M237" s="3"/>
       <c r="N237" s="4"/>
-      <c r="O237" s="4"/>
+      <c r="O237" s="3"/>
       <c r="P237" s="4"/>
       <c r="Q237" s="4"/>
       <c r="R237" s="4"/>
@@ -14669,7 +14698,9 @@
       <c r="AB237" s="4"/>
       <c r="AC237" s="4"/>
       <c r="AD237" s="4"/>
-      <c r="AE237" s="4"/>
+      <c r="AE237" s="4" t="s">
+        <v>499</v>
+      </c>
       <c r="AF237" s="4"/>
       <c r="AG237" s="4"/>
       <c r="AH237" s="4"/>
@@ -14677,32 +14708,30 @@
     </row>
     <row r="238" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A238" s="4" t="s">
-        <v>511</v>
+        <v>772</v>
       </c>
       <c r="B238" s="4" t="s">
-        <v>228</v>
+        <v>496</v>
       </c>
       <c r="C238" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D238" s="4"/>
+        <v>232</v>
+      </c>
+      <c r="D238" s="5" t="s">
+        <v>773</v>
+      </c>
       <c r="E238" s="4"/>
       <c r="F238" s="4"/>
       <c r="G238" s="4"/>
       <c r="H238" s="4"/>
-      <c r="I238" s="4"/>
-      <c r="J238" s="3" t="s">
-        <v>512</v>
-      </c>
-      <c r="K238" s="3" t="s">
-        <v>513</v>
-      </c>
-      <c r="L238" s="3" t="s">
-        <v>514</v>
-      </c>
-      <c r="M238" s="4"/>
+      <c r="I238" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J238" s="4"/>
+      <c r="K238" s="4"/>
+      <c r="L238" s="4"/>
+      <c r="M238" s="3"/>
       <c r="N238" s="4"/>
-      <c r="O238" s="4"/>
+      <c r="O238" s="3"/>
       <c r="P238" s="4"/>
       <c r="Q238" s="4"/>
       <c r="R238" s="4"/>
@@ -14718,7 +14747,9 @@
       <c r="AB238" s="4"/>
       <c r="AC238" s="4"/>
       <c r="AD238" s="4"/>
-      <c r="AE238" s="4"/>
+      <c r="AE238" s="4" t="s">
+        <v>496</v>
+      </c>
       <c r="AF238" s="4"/>
       <c r="AG238" s="4"/>
       <c r="AH238" s="4"/>
@@ -14726,32 +14757,30 @@
     </row>
     <row r="239" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A239" s="4" t="s">
-        <v>515</v>
+        <v>774</v>
       </c>
       <c r="B239" s="4" t="s">
-        <v>228</v>
+        <v>506</v>
       </c>
       <c r="C239" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D239" s="4"/>
+        <v>232</v>
+      </c>
+      <c r="D239" s="5" t="s">
+        <v>775</v>
+      </c>
       <c r="E239" s="4"/>
       <c r="F239" s="4"/>
       <c r="G239" s="4"/>
       <c r="H239" s="4"/>
-      <c r="I239" s="4"/>
-      <c r="J239" s="3" t="s">
-        <v>516</v>
-      </c>
-      <c r="K239" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="L239" s="3" t="s">
-        <v>517</v>
-      </c>
-      <c r="M239" s="4"/>
+      <c r="I239" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J239" s="4"/>
+      <c r="K239" s="4"/>
+      <c r="L239" s="4"/>
+      <c r="M239" s="3"/>
       <c r="N239" s="4"/>
-      <c r="O239" s="4"/>
+      <c r="O239" s="3"/>
       <c r="P239" s="4"/>
       <c r="Q239" s="4"/>
       <c r="R239" s="4"/>
@@ -14767,22 +14796,18 @@
       <c r="AB239" s="4"/>
       <c r="AC239" s="4"/>
       <c r="AD239" s="4"/>
-      <c r="AE239" s="4"/>
+      <c r="AE239" s="4" t="s">
+        <v>506</v>
+      </c>
       <c r="AF239" s="4"/>
       <c r="AG239" s="4"/>
       <c r="AH239" s="4"/>
       <c r="AI239" s="4"/>
     </row>
     <row r="240" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A240" s="4" t="s">
-        <v>518</v>
-      </c>
-      <c r="B240" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C240" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="A240" s="4"/>
+      <c r="B240" s="4"/>
+      <c r="C240" s="4"/>
       <c r="D240" s="4"/>
       <c r="E240" s="4"/>
       <c r="F240" s="4"/>
@@ -14794,9 +14819,7 @@
       <c r="L240" s="4"/>
       <c r="M240" s="4"/>
       <c r="N240" s="4"/>
-      <c r="O240" s="3" t="s">
-        <v>519</v>
-      </c>
+      <c r="O240" s="4"/>
       <c r="P240" s="4"/>
       <c r="Q240" s="4"/>
       <c r="R240" s="4"/>
@@ -14820,7 +14843,7 @@
     </row>
     <row r="241" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A241" s="4" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
       <c r="B241" s="4" t="s">
         <v>228</v>
@@ -14834,14 +14857,18 @@
       <c r="G241" s="4"/>
       <c r="H241" s="4"/>
       <c r="I241" s="4"/>
-      <c r="J241" s="4"/>
-      <c r="K241" s="4"/>
-      <c r="L241" s="4"/>
+      <c r="J241" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="K241" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="L241" s="3" t="s">
+        <v>514</v>
+      </c>
       <c r="M241" s="4"/>
       <c r="N241" s="4"/>
-      <c r="O241" s="3" t="s">
-        <v>521</v>
-      </c>
+      <c r="O241" s="4"/>
       <c r="P241" s="4"/>
       <c r="Q241" s="4"/>
       <c r="R241" s="4"/>
@@ -14865,7 +14892,7 @@
     </row>
     <row r="242" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A242" s="4" t="s">
-        <v>522</v>
+        <v>515</v>
       </c>
       <c r="B242" s="4" t="s">
         <v>228</v>
@@ -14879,14 +14906,18 @@
       <c r="G242" s="4"/>
       <c r="H242" s="4"/>
       <c r="I242" s="4"/>
-      <c r="J242" s="4"/>
-      <c r="K242" s="4"/>
-      <c r="L242" s="4"/>
+      <c r="J242" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="K242" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="L242" s="3" t="s">
+        <v>517</v>
+      </c>
       <c r="M242" s="4"/>
       <c r="N242" s="4"/>
-      <c r="O242" s="3" t="s">
-        <v>523</v>
-      </c>
+      <c r="O242" s="4"/>
       <c r="P242" s="4"/>
       <c r="Q242" s="4"/>
       <c r="R242" s="4"/>
@@ -14910,7 +14941,7 @@
     </row>
     <row r="243" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A243" s="4" t="s">
-        <v>524</v>
+        <v>518</v>
       </c>
       <c r="B243" s="4" t="s">
         <v>228</v>
@@ -14927,11 +14958,11 @@
       <c r="J243" s="4"/>
       <c r="K243" s="4"/>
       <c r="L243" s="4"/>
-      <c r="M243" s="4" t="s">
-        <v>525</v>
-      </c>
+      <c r="M243" s="4"/>
       <c r="N243" s="4"/>
-      <c r="O243" s="4"/>
+      <c r="O243" s="3" t="s">
+        <v>519</v>
+      </c>
       <c r="P243" s="4"/>
       <c r="Q243" s="4"/>
       <c r="R243" s="4"/>
@@ -14953,6 +14984,141 @@
       <c r="AH243" s="4"/>
       <c r="AI243" s="4"/>
     </row>
+    <row r="244" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A244" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="B244" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C244" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D244" s="4"/>
+      <c r="E244" s="4"/>
+      <c r="F244" s="4"/>
+      <c r="G244" s="4"/>
+      <c r="H244" s="4"/>
+      <c r="I244" s="4"/>
+      <c r="J244" s="4"/>
+      <c r="K244" s="4"/>
+      <c r="L244" s="4"/>
+      <c r="M244" s="4"/>
+      <c r="N244" s="4"/>
+      <c r="O244" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="P244" s="4"/>
+      <c r="Q244" s="4"/>
+      <c r="R244" s="4"/>
+      <c r="S244" s="4"/>
+      <c r="T244" s="4"/>
+      <c r="U244" s="4"/>
+      <c r="V244" s="4"/>
+      <c r="W244" s="4"/>
+      <c r="X244" s="4"/>
+      <c r="Y244" s="4"/>
+      <c r="Z244" s="4"/>
+      <c r="AA244" s="4"/>
+      <c r="AB244" s="4"/>
+      <c r="AC244" s="4"/>
+      <c r="AD244" s="4"/>
+      <c r="AE244" s="4"/>
+      <c r="AF244" s="4"/>
+      <c r="AG244" s="4"/>
+      <c r="AH244" s="4"/>
+      <c r="AI244" s="4"/>
+    </row>
+    <row r="245" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A245" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="B245" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C245" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D245" s="4"/>
+      <c r="E245" s="4"/>
+      <c r="F245" s="4"/>
+      <c r="G245" s="4"/>
+      <c r="H245" s="4"/>
+      <c r="I245" s="4"/>
+      <c r="J245" s="4"/>
+      <c r="K245" s="4"/>
+      <c r="L245" s="4"/>
+      <c r="M245" s="4"/>
+      <c r="N245" s="4"/>
+      <c r="O245" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="P245" s="4"/>
+      <c r="Q245" s="4"/>
+      <c r="R245" s="4"/>
+      <c r="S245" s="4"/>
+      <c r="T245" s="4"/>
+      <c r="U245" s="4"/>
+      <c r="V245" s="4"/>
+      <c r="W245" s="4"/>
+      <c r="X245" s="4"/>
+      <c r="Y245" s="4"/>
+      <c r="Z245" s="4"/>
+      <c r="AA245" s="4"/>
+      <c r="AB245" s="4"/>
+      <c r="AC245" s="4"/>
+      <c r="AD245" s="4"/>
+      <c r="AE245" s="4"/>
+      <c r="AF245" s="4"/>
+      <c r="AG245" s="4"/>
+      <c r="AH245" s="4"/>
+      <c r="AI245" s="4"/>
+    </row>
+    <row r="246" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A246" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B246" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C246" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D246" s="4"/>
+      <c r="E246" s="4"/>
+      <c r="F246" s="4"/>
+      <c r="G246" s="4"/>
+      <c r="H246" s="4"/>
+      <c r="I246" s="4"/>
+      <c r="J246" s="4"/>
+      <c r="K246" s="4"/>
+      <c r="L246" s="4"/>
+      <c r="M246" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="N246" s="4"/>
+      <c r="O246" s="4"/>
+      <c r="P246" s="4"/>
+      <c r="Q246" s="4"/>
+      <c r="R246" s="4"/>
+      <c r="S246" s="4"/>
+      <c r="T246" s="4"/>
+      <c r="U246" s="4"/>
+      <c r="V246" s="4"/>
+      <c r="W246" s="4"/>
+      <c r="X246" s="4"/>
+      <c r="Y246" s="4"/>
+      <c r="Z246" s="4"/>
+      <c r="AA246" s="4"/>
+      <c r="AB246" s="4"/>
+      <c r="AC246" s="4"/>
+      <c r="AD246" s="4"/>
+      <c r="AE246" s="4"/>
+      <c r="AF246" s="4"/>
+      <c r="AG246" s="4"/>
+      <c r="AH246" s="4"/>
+      <c r="AI246" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14960,7 +15126,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B611D72-2CC2-4CCA-A1E6-2A10215873D6}">
-  <dimension ref="A1:T234"/>
+  <dimension ref="A1:T237"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -23320,6 +23486,120 @@
       <c r="S234" s="4"/>
       <c r="T234" s="4"/>
     </row>
+    <row r="235" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A235" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="B235" s="3" t="s">
+        <v>711</v>
+      </c>
+      <c r="C235" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D235" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E235" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F235" s="4"/>
+      <c r="G235" s="4"/>
+      <c r="H235" s="4"/>
+      <c r="I235" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="J235" s="4"/>
+      <c r="K235" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="L235" s="4"/>
+      <c r="M235" s="4"/>
+      <c r="N235" s="4"/>
+      <c r="O235" s="4"/>
+      <c r="P235" s="4"/>
+      <c r="Q235" s="4"/>
+      <c r="R235" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="S235" s="4"/>
+      <c r="T235" s="4"/>
+    </row>
+    <row r="236" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A236" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="B236" s="5" t="s">
+        <v>709</v>
+      </c>
+      <c r="C236" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D236" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E236" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F236" s="4"/>
+      <c r="G236" s="4"/>
+      <c r="H236" s="4"/>
+      <c r="I236" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="J236" s="4"/>
+      <c r="K236" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="L236" s="4"/>
+      <c r="M236" s="4"/>
+      <c r="N236" s="4"/>
+      <c r="O236" s="4"/>
+      <c r="P236" s="4"/>
+      <c r="Q236" s="4"/>
+      <c r="R236" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="S236" s="4"/>
+      <c r="T236" s="4"/>
+    </row>
+    <row r="237" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A237" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="B237" s="3" t="s">
+        <v>777</v>
+      </c>
+      <c r="C237" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D237" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E237" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F237" s="4"/>
+      <c r="G237" s="4"/>
+      <c r="H237" s="4"/>
+      <c r="I237" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="J237" s="4"/>
+      <c r="K237" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="L237" s="4"/>
+      <c r="M237" s="4"/>
+      <c r="N237" s="4"/>
+      <c r="O237" s="4"/>
+      <c r="P237" s="4"/>
+      <c r="Q237" s="4"/>
+      <c r="R237" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="S237" s="4"/>
+      <c r="T237" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Commit for 4 customer Outbound scenario for TRN and ILW customer
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ffd-sys-team\git\eai-3534455-ffd-manhattan-automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8721D447-296C-4CCC-A3F2-E86366ABA4C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99D9E75E-0EF8-4F30-97A6-643BD1C499D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3351" uniqueCount="778">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3373" uniqueCount="784">
   <si>
     <t>ScearioID</t>
   </si>
@@ -2179,9 +2179,6 @@
     <t>1016</t>
   </si>
   <si>
-    <t xml:space="preserve">8350202301                     </t>
-  </si>
-  <si>
     <t>1017</t>
   </si>
   <si>
@@ -2372,6 +2369,27 @@
   </si>
   <si>
     <t>00026315089</t>
+  </si>
+  <si>
+    <t>TRN_OBScenario1</t>
+  </si>
+  <si>
+    <t>1023</t>
+  </si>
+  <si>
+    <t>1024</t>
+  </si>
+  <si>
+    <t>8350202301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8350202301     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">8350202301          </t>
+  </si>
+  <si>
+    <t xml:space="preserve">8350202301  </t>
   </si>
 </sst>
 </file>
@@ -2842,7 +2860,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA0C8091-AB5D-461B-B4FE-5D2410DFE16F}">
-  <dimension ref="A1:AI246"/>
+  <dimension ref="A1:AI247"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -14610,7 +14628,7 @@
     </row>
     <row r="236" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A236" s="4" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="B236" s="4" t="s">
         <v>496</v>
@@ -14619,7 +14637,7 @@
         <v>232</v>
       </c>
       <c r="D236" s="5" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="E236" s="4"/>
       <c r="F236" s="4"/>
@@ -14659,7 +14677,7 @@
     </row>
     <row r="237" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A237" s="4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="B237" s="4" t="s">
         <v>499</v>
@@ -14668,7 +14686,7 @@
         <v>232</v>
       </c>
       <c r="D237" s="5" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E237" s="4"/>
       <c r="F237" s="4"/>
@@ -14708,7 +14726,7 @@
     </row>
     <row r="238" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A238" s="4" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="B238" s="4" t="s">
         <v>496</v>
@@ -14717,7 +14735,7 @@
         <v>232</v>
       </c>
       <c r="D238" s="5" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="E238" s="4"/>
       <c r="F238" s="4"/>
@@ -14757,7 +14775,7 @@
     </row>
     <row r="239" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A239" s="4" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B239" s="4" t="s">
         <v>506</v>
@@ -14766,7 +14784,7 @@
         <v>232</v>
       </c>
       <c r="D239" s="5" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="E239" s="4"/>
       <c r="F239" s="4"/>
@@ -14805,15 +14823,25 @@
       <c r="AI239" s="4"/>
     </row>
     <row r="240" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A240" s="4"/>
-      <c r="B240" s="4"/>
-      <c r="C240" s="4"/>
-      <c r="D240" s="4"/>
+      <c r="A240" s="4" t="s">
+        <v>777</v>
+      </c>
+      <c r="B240" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="C240" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D240" s="5" t="s">
+        <v>778</v>
+      </c>
       <c r="E240" s="4"/>
       <c r="F240" s="4"/>
       <c r="G240" s="4"/>
       <c r="H240" s="4"/>
-      <c r="I240" s="4"/>
+      <c r="I240" s="4" t="s">
+        <v>46</v>
+      </c>
       <c r="J240" s="4"/>
       <c r="K240" s="4"/>
       <c r="L240" s="4"/>
@@ -14835,37 +14863,27 @@
       <c r="AB240" s="4"/>
       <c r="AC240" s="4"/>
       <c r="AD240" s="4"/>
-      <c r="AE240" s="4"/>
+      <c r="AE240" s="4" t="s">
+        <v>504</v>
+      </c>
       <c r="AF240" s="4"/>
       <c r="AG240" s="4"/>
       <c r="AH240" s="4"/>
       <c r="AI240" s="4"/>
     </row>
     <row r="241" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A241" s="4" t="s">
-        <v>511</v>
-      </c>
-      <c r="B241" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C241" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="A241" s="4"/>
+      <c r="B241" s="4"/>
+      <c r="C241" s="4"/>
       <c r="D241" s="4"/>
       <c r="E241" s="4"/>
       <c r="F241" s="4"/>
       <c r="G241" s="4"/>
       <c r="H241" s="4"/>
       <c r="I241" s="4"/>
-      <c r="J241" s="3" t="s">
-        <v>512</v>
-      </c>
-      <c r="K241" s="3" t="s">
-        <v>513</v>
-      </c>
-      <c r="L241" s="3" t="s">
-        <v>514</v>
-      </c>
+      <c r="J241" s="4"/>
+      <c r="K241" s="4"/>
+      <c r="L241" s="4"/>
       <c r="M241" s="4"/>
       <c r="N241" s="4"/>
       <c r="O241" s="4"/>
@@ -14892,7 +14910,7 @@
     </row>
     <row r="242" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A242" s="4" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="B242" s="4" t="s">
         <v>228</v>
@@ -14907,13 +14925,13 @@
       <c r="H242" s="4"/>
       <c r="I242" s="4"/>
       <c r="J242" s="3" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="K242" s="3" t="s">
-        <v>243</v>
+        <v>513</v>
       </c>
       <c r="L242" s="3" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="M242" s="4"/>
       <c r="N242" s="4"/>
@@ -14941,7 +14959,7 @@
     </row>
     <row r="243" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A243" s="4" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="B243" s="4" t="s">
         <v>228</v>
@@ -14955,14 +14973,18 @@
       <c r="G243" s="4"/>
       <c r="H243" s="4"/>
       <c r="I243" s="4"/>
-      <c r="J243" s="4"/>
-      <c r="K243" s="4"/>
-      <c r="L243" s="4"/>
+      <c r="J243" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="K243" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="L243" s="3" t="s">
+        <v>517</v>
+      </c>
       <c r="M243" s="4"/>
       <c r="N243" s="4"/>
-      <c r="O243" s="3" t="s">
-        <v>519</v>
-      </c>
+      <c r="O243" s="4"/>
       <c r="P243" s="4"/>
       <c r="Q243" s="4"/>
       <c r="R243" s="4"/>
@@ -14986,7 +15008,7 @@
     </row>
     <row r="244" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A244" s="4" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="B244" s="4" t="s">
         <v>228</v>
@@ -15006,7 +15028,7 @@
       <c r="M244" s="4"/>
       <c r="N244" s="4"/>
       <c r="O244" s="3" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="P244" s="4"/>
       <c r="Q244" s="4"/>
@@ -15031,7 +15053,7 @@
     </row>
     <row r="245" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A245" s="4" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="B245" s="4" t="s">
         <v>228</v>
@@ -15051,7 +15073,7 @@
       <c r="M245" s="4"/>
       <c r="N245" s="4"/>
       <c r="O245" s="3" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="P245" s="4"/>
       <c r="Q245" s="4"/>
@@ -15076,7 +15098,7 @@
     </row>
     <row r="246" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A246" s="4" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="B246" s="4" t="s">
         <v>228</v>
@@ -15093,11 +15115,11 @@
       <c r="J246" s="4"/>
       <c r="K246" s="4"/>
       <c r="L246" s="4"/>
-      <c r="M246" s="4" t="s">
-        <v>525</v>
-      </c>
+      <c r="M246" s="4"/>
       <c r="N246" s="4"/>
-      <c r="O246" s="4"/>
+      <c r="O246" s="3" t="s">
+        <v>523</v>
+      </c>
       <c r="P246" s="4"/>
       <c r="Q246" s="4"/>
       <c r="R246" s="4"/>
@@ -15119,6 +15141,51 @@
       <c r="AH246" s="4"/>
       <c r="AI246" s="4"/>
     </row>
+    <row r="247" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A247" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B247" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C247" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D247" s="4"/>
+      <c r="E247" s="4"/>
+      <c r="F247" s="4"/>
+      <c r="G247" s="4"/>
+      <c r="H247" s="4"/>
+      <c r="I247" s="4"/>
+      <c r="J247" s="4"/>
+      <c r="K247" s="4"/>
+      <c r="L247" s="4"/>
+      <c r="M247" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="N247" s="4"/>
+      <c r="O247" s="4"/>
+      <c r="P247" s="4"/>
+      <c r="Q247" s="4"/>
+      <c r="R247" s="4"/>
+      <c r="S247" s="4"/>
+      <c r="T247" s="4"/>
+      <c r="U247" s="4"/>
+      <c r="V247" s="4"/>
+      <c r="W247" s="4"/>
+      <c r="X247" s="4"/>
+      <c r="Y247" s="4"/>
+      <c r="Z247" s="4"/>
+      <c r="AA247" s="4"/>
+      <c r="AB247" s="4"/>
+      <c r="AC247" s="4"/>
+      <c r="AD247" s="4"/>
+      <c r="AE247" s="4"/>
+      <c r="AF247" s="4"/>
+      <c r="AG247" s="4"/>
+      <c r="AH247" s="4"/>
+      <c r="AI247" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15126,7 +15193,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B611D72-2CC2-4CCA-A1E6-2A10215873D6}">
-  <dimension ref="A1:T237"/>
+  <dimension ref="A1:T239"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -23339,7 +23406,7 @@
         <v>712</v>
       </c>
       <c r="B231" s="3" t="s">
-        <v>713</v>
+        <v>782</v>
       </c>
       <c r="C231" s="3" t="s">
         <v>38</v>
@@ -23374,10 +23441,10 @@
     </row>
     <row r="232" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A232" s="3" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B232" s="3" t="s">
-        <v>713</v>
+        <v>781</v>
       </c>
       <c r="C232" s="3" t="s">
         <v>38</v>
@@ -23415,7 +23482,7 @@
         <v>507</v>
       </c>
       <c r="B233" s="3" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="C233" s="3" t="s">
         <v>38</v>
@@ -23450,10 +23517,10 @@
     </row>
     <row r="234" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A234" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="B234" s="5" t="s">
         <v>769</v>
-      </c>
-      <c r="B234" s="5" t="s">
-        <v>770</v>
       </c>
       <c r="C234" s="3" t="s">
         <v>38</v>
@@ -23488,7 +23555,7 @@
     </row>
     <row r="235" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A235" s="3" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="B235" s="3" t="s">
         <v>711</v>
@@ -23526,7 +23593,7 @@
     </row>
     <row r="236" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A236" s="3" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="B236" s="5" t="s">
         <v>709</v>
@@ -23564,10 +23631,10 @@
     </row>
     <row r="237" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A237" s="3" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="B237" s="3" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="C237" s="3" t="s">
         <v>38</v>
@@ -23599,6 +23666,82 @@
       </c>
       <c r="S237" s="4"/>
       <c r="T237" s="4"/>
+    </row>
+    <row r="238" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A238" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="B238" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="C238" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D238" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E238" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F238" s="4"/>
+      <c r="G238" s="4"/>
+      <c r="H238" s="4"/>
+      <c r="I238" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="J238" s="4"/>
+      <c r="K238" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="L238" s="4"/>
+      <c r="M238" s="4"/>
+      <c r="N238" s="4"/>
+      <c r="O238" s="4"/>
+      <c r="P238" s="4"/>
+      <c r="Q238" s="4"/>
+      <c r="R238" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="S238" s="4"/>
+      <c r="T238" s="4"/>
+    </row>
+    <row r="239" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A239" s="3" t="s">
+        <v>779</v>
+      </c>
+      <c r="B239" s="3" t="s">
+        <v>783</v>
+      </c>
+      <c r="C239" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D239" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E239" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F239" s="4"/>
+      <c r="G239" s="4"/>
+      <c r="H239" s="4"/>
+      <c r="I239" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="J239" s="4"/>
+      <c r="K239" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="L239" s="4"/>
+      <c r="M239" s="4"/>
+      <c r="N239" s="4"/>
+      <c r="O239" s="4"/>
+      <c r="P239" s="4"/>
+      <c r="Q239" s="4"/>
+      <c r="R239" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="S239" s="4"/>
+      <c r="T239" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23612,10 +23755,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
+        <v>715</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>716</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>717</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -23623,7 +23766,7 @@
         <v>38</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -23631,7 +23774,7 @@
         <v>295</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -23639,7 +23782,7 @@
         <v>49</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -23647,7 +23790,7 @@
         <v>51</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -23655,7 +23798,7 @@
         <v>547</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -23663,7 +23806,7 @@
         <v>549</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -23671,7 +23814,7 @@
         <v>57</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -23679,7 +23822,7 @@
         <v>553</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -23687,7 +23830,7 @@
         <v>60</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -23695,7 +23838,7 @@
         <v>53</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -23703,7 +23846,7 @@
         <v>64</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -23711,7 +23854,7 @@
         <v>70</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -23719,7 +23862,7 @@
         <v>72</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -23727,7 +23870,7 @@
         <v>74</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -23735,7 +23878,7 @@
         <v>76</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -23743,7 +23886,7 @@
         <v>78</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -23751,7 +23894,7 @@
         <v>80</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -23759,7 +23902,7 @@
         <v>82</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -23767,7 +23910,7 @@
         <v>84</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -23775,7 +23918,7 @@
         <v>86</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -23783,7 +23926,7 @@
         <v>89</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -23791,7 +23934,7 @@
         <v>91</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -23799,7 +23942,7 @@
         <v>93</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -23807,7 +23950,7 @@
         <v>95</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -23815,7 +23958,7 @@
         <v>97</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -23823,7 +23966,7 @@
         <v>562</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -23831,7 +23974,7 @@
         <v>563</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -23839,7 +23982,7 @@
         <v>564</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -23847,7 +23990,7 @@
         <v>565</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -23855,7 +23998,7 @@
         <v>103</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -23863,7 +24006,7 @@
         <v>105</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -23871,7 +24014,7 @@
         <v>107</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -23879,7 +24022,7 @@
         <v>566</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -23887,7 +24030,7 @@
         <v>567</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -23895,7 +24038,7 @@
         <v>568</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -23903,7 +24046,7 @@
         <v>569</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -23911,7 +24054,7 @@
         <v>570</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -23919,7 +24062,7 @@
         <v>571</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -23927,7 +24070,7 @@
         <v>572</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -23935,7 +24078,7 @@
         <v>546</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -23943,7 +24086,7 @@
         <v>573</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -23951,7 +24094,7 @@
         <v>574</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -23959,7 +24102,7 @@
         <v>575</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -23967,7 +24110,7 @@
         <v>576</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -23975,7 +24118,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -23983,7 +24126,7 @@
         <v>129</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -23991,7 +24134,7 @@
         <v>121</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -23999,7 +24142,7 @@
         <v>124</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -24007,15 +24150,15 @@
         <v>127</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B51" s="19" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -24023,7 +24166,7 @@
         <v>556</v>
       </c>
       <c r="B52" s="19" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
@@ -24031,127 +24174,127 @@
         <v>558</v>
       </c>
       <c r="B53" s="19" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B54" s="19" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B55" s="19" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B56" s="19" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="B57" s="19" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B58" s="19" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
+        <v>754</v>
+      </c>
+      <c r="B59" s="19" t="s">
         <v>755</v>
-      </c>
-      <c r="B59" s="19" t="s">
-        <v>756</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B60" s="19" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="B61" s="19" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="B62" s="19" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="B63" s="19" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="B64" s="19" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B65" s="19" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
+        <v>763</v>
+      </c>
+      <c r="B67" s="20" t="s">
         <v>764</v>
-      </c>
-      <c r="B67" s="20" t="s">
-        <v>765</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
+        <v>765</v>
+      </c>
+      <c r="B68" s="17" t="s">
         <v>766</v>
-      </c>
-      <c r="B68" s="17" t="s">
-        <v>767</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Commit the latest changes done as part of Vendor Portal customer changes
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ffd-sys-team\git\eai-3534455-ffd-manhattan-automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99D9E75E-0EF8-4F30-97A6-643BD1C499D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB35E375-A530-41EE-A03C-A58C2D3D2965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3373" uniqueCount="784">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3429" uniqueCount="798">
   <si>
     <t>ScearioID</t>
   </si>
@@ -2390,6 +2390,48 @@
   </si>
   <si>
     <t xml:space="preserve">8350202301  </t>
+  </si>
+  <si>
+    <t>ATM_KelliScenario001</t>
+  </si>
+  <si>
+    <t>ATM</t>
+  </si>
+  <si>
+    <t>1025</t>
+  </si>
+  <si>
+    <t>ATMRJ001</t>
+  </si>
+  <si>
+    <t>AMI</t>
+  </si>
+  <si>
+    <t>ATM_KelliScenario002</t>
+  </si>
+  <si>
+    <t>1026</t>
+  </si>
+  <si>
+    <t>ATMLT01</t>
+  </si>
+  <si>
+    <t>ATM_KelliScenario003</t>
+  </si>
+  <si>
+    <t>1027</t>
+  </si>
+  <si>
+    <t>ATMSR01</t>
+  </si>
+  <si>
+    <t>ATM_KelliScenario004</t>
+  </si>
+  <si>
+    <t>1028</t>
+  </si>
+  <si>
+    <t>1025|1028</t>
   </si>
 </sst>
 </file>
@@ -2564,9 +2606,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2604,7 +2646,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2710,7 +2752,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2852,7 +2894,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2860,7 +2902,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA0C8091-AB5D-461B-B4FE-5D2410DFE16F}">
-  <dimension ref="A1:AI247"/>
+  <dimension ref="A1:AI251"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -14872,15 +14914,25 @@
       <c r="AI240" s="4"/>
     </row>
     <row r="241" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A241" s="4"/>
-      <c r="B241" s="4"/>
-      <c r="C241" s="4"/>
-      <c r="D241" s="4"/>
+      <c r="A241" s="4" t="s">
+        <v>784</v>
+      </c>
+      <c r="B241" s="4" t="s">
+        <v>785</v>
+      </c>
+      <c r="C241" s="4" t="s">
+        <v>788</v>
+      </c>
+      <c r="D241" s="5" t="s">
+        <v>786</v>
+      </c>
       <c r="E241" s="4"/>
       <c r="F241" s="4"/>
       <c r="G241" s="4"/>
       <c r="H241" s="4"/>
-      <c r="I241" s="4"/>
+      <c r="I241" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="J241" s="4"/>
       <c r="K241" s="4"/>
       <c r="L241" s="4"/>
@@ -14902,7 +14954,9 @@
       <c r="AB241" s="4"/>
       <c r="AC241" s="4"/>
       <c r="AD241" s="4"/>
-      <c r="AE241" s="4"/>
+      <c r="AE241" s="4" t="s">
+        <v>785</v>
+      </c>
       <c r="AF241" s="4"/>
       <c r="AG241" s="4"/>
       <c r="AH241" s="4"/>
@@ -14910,29 +14964,27 @@
     </row>
     <row r="242" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A242" s="4" t="s">
-        <v>511</v>
+        <v>789</v>
       </c>
       <c r="B242" s="4" t="s">
-        <v>228</v>
+        <v>785</v>
       </c>
       <c r="C242" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D242" s="4"/>
+        <v>788</v>
+      </c>
+      <c r="D242" s="5" t="s">
+        <v>790</v>
+      </c>
       <c r="E242" s="4"/>
       <c r="F242" s="4"/>
       <c r="G242" s="4"/>
       <c r="H242" s="4"/>
-      <c r="I242" s="4"/>
-      <c r="J242" s="3" t="s">
-        <v>512</v>
-      </c>
-      <c r="K242" s="3" t="s">
-        <v>513</v>
-      </c>
-      <c r="L242" s="3" t="s">
-        <v>514</v>
-      </c>
+      <c r="I242" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J242" s="4"/>
+      <c r="K242" s="4"/>
+      <c r="L242" s="4"/>
       <c r="M242" s="4"/>
       <c r="N242" s="4"/>
       <c r="O242" s="4"/>
@@ -14951,7 +15003,9 @@
       <c r="AB242" s="4"/>
       <c r="AC242" s="4"/>
       <c r="AD242" s="4"/>
-      <c r="AE242" s="4"/>
+      <c r="AE242" s="4" t="s">
+        <v>785</v>
+      </c>
       <c r="AF242" s="4"/>
       <c r="AG242" s="4"/>
       <c r="AH242" s="4"/>
@@ -14959,29 +15013,27 @@
     </row>
     <row r="243" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A243" s="4" t="s">
-        <v>515</v>
+        <v>792</v>
       </c>
       <c r="B243" s="4" t="s">
-        <v>228</v>
+        <v>785</v>
       </c>
       <c r="C243" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D243" s="4"/>
+        <v>788</v>
+      </c>
+      <c r="D243" s="5" t="s">
+        <v>793</v>
+      </c>
       <c r="E243" s="4"/>
       <c r="F243" s="4"/>
       <c r="G243" s="4"/>
       <c r="H243" s="4"/>
-      <c r="I243" s="4"/>
-      <c r="J243" s="3" t="s">
-        <v>516</v>
-      </c>
-      <c r="K243" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="L243" s="3" t="s">
-        <v>517</v>
-      </c>
+      <c r="I243" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J243" s="4"/>
+      <c r="K243" s="4"/>
+      <c r="L243" s="4"/>
       <c r="M243" s="4"/>
       <c r="N243" s="4"/>
       <c r="O243" s="4"/>
@@ -15000,7 +15052,9 @@
       <c r="AB243" s="4"/>
       <c r="AC243" s="4"/>
       <c r="AD243" s="4"/>
-      <c r="AE243" s="4"/>
+      <c r="AE243" s="4" t="s">
+        <v>785</v>
+      </c>
       <c r="AF243" s="4"/>
       <c r="AG243" s="4"/>
       <c r="AH243" s="4"/>
@@ -15008,28 +15062,30 @@
     </row>
     <row r="244" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A244" s="4" t="s">
-        <v>518</v>
+        <v>795</v>
       </c>
       <c r="B244" s="4" t="s">
-        <v>228</v>
+        <v>785</v>
       </c>
       <c r="C244" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D244" s="4"/>
+        <v>788</v>
+      </c>
+      <c r="D244" s="5" t="s">
+        <v>797</v>
+      </c>
       <c r="E244" s="4"/>
       <c r="F244" s="4"/>
       <c r="G244" s="4"/>
       <c r="H244" s="4"/>
-      <c r="I244" s="4"/>
+      <c r="I244" s="4" t="s">
+        <v>46</v>
+      </c>
       <c r="J244" s="4"/>
       <c r="K244" s="4"/>
       <c r="L244" s="4"/>
       <c r="M244" s="4"/>
       <c r="N244" s="4"/>
-      <c r="O244" s="3" t="s">
-        <v>519</v>
-      </c>
+      <c r="O244" s="4"/>
       <c r="P244" s="4"/>
       <c r="Q244" s="4"/>
       <c r="R244" s="4"/>
@@ -15045,22 +15101,18 @@
       <c r="AB244" s="4"/>
       <c r="AC244" s="4"/>
       <c r="AD244" s="4"/>
-      <c r="AE244" s="4"/>
+      <c r="AE244" s="4" t="s">
+        <v>785</v>
+      </c>
       <c r="AF244" s="4"/>
       <c r="AG244" s="4"/>
       <c r="AH244" s="4"/>
       <c r="AI244" s="4"/>
     </row>
     <row r="245" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A245" s="4" t="s">
-        <v>520</v>
-      </c>
-      <c r="B245" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C245" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="A245" s="4"/>
+      <c r="B245" s="4"/>
+      <c r="C245" s="4"/>
       <c r="D245" s="4"/>
       <c r="E245" s="4"/>
       <c r="F245" s="4"/>
@@ -15072,9 +15124,7 @@
       <c r="L245" s="4"/>
       <c r="M245" s="4"/>
       <c r="N245" s="4"/>
-      <c r="O245" s="3" t="s">
-        <v>521</v>
-      </c>
+      <c r="O245" s="4"/>
       <c r="P245" s="4"/>
       <c r="Q245" s="4"/>
       <c r="R245" s="4"/>
@@ -15098,7 +15148,7 @@
     </row>
     <row r="246" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A246" s="4" t="s">
-        <v>522</v>
+        <v>511</v>
       </c>
       <c r="B246" s="4" t="s">
         <v>228</v>
@@ -15112,14 +15162,18 @@
       <c r="G246" s="4"/>
       <c r="H246" s="4"/>
       <c r="I246" s="4"/>
-      <c r="J246" s="4"/>
-      <c r="K246" s="4"/>
-      <c r="L246" s="4"/>
+      <c r="J246" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="K246" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="L246" s="3" t="s">
+        <v>514</v>
+      </c>
       <c r="M246" s="4"/>
       <c r="N246" s="4"/>
-      <c r="O246" s="3" t="s">
-        <v>523</v>
-      </c>
+      <c r="O246" s="4"/>
       <c r="P246" s="4"/>
       <c r="Q246" s="4"/>
       <c r="R246" s="4"/>
@@ -15143,7 +15197,7 @@
     </row>
     <row r="247" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A247" s="4" t="s">
-        <v>524</v>
+        <v>515</v>
       </c>
       <c r="B247" s="4" t="s">
         <v>228</v>
@@ -15157,12 +15211,16 @@
       <c r="G247" s="4"/>
       <c r="H247" s="4"/>
       <c r="I247" s="4"/>
-      <c r="J247" s="4"/>
-      <c r="K247" s="4"/>
-      <c r="L247" s="4"/>
-      <c r="M247" s="4" t="s">
-        <v>525</v>
-      </c>
+      <c r="J247" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="K247" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="L247" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="M247" s="4"/>
       <c r="N247" s="4"/>
       <c r="O247" s="4"/>
       <c r="P247" s="4"/>
@@ -15186,6 +15244,186 @@
       <c r="AH247" s="4"/>
       <c r="AI247" s="4"/>
     </row>
+    <row r="248" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A248" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="B248" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C248" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D248" s="4"/>
+      <c r="E248" s="4"/>
+      <c r="F248" s="4"/>
+      <c r="G248" s="4"/>
+      <c r="H248" s="4"/>
+      <c r="I248" s="4"/>
+      <c r="J248" s="4"/>
+      <c r="K248" s="4"/>
+      <c r="L248" s="4"/>
+      <c r="M248" s="4"/>
+      <c r="N248" s="4"/>
+      <c r="O248" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="P248" s="4"/>
+      <c r="Q248" s="4"/>
+      <c r="R248" s="4"/>
+      <c r="S248" s="4"/>
+      <c r="T248" s="4"/>
+      <c r="U248" s="4"/>
+      <c r="V248" s="4"/>
+      <c r="W248" s="4"/>
+      <c r="X248" s="4"/>
+      <c r="Y248" s="4"/>
+      <c r="Z248" s="4"/>
+      <c r="AA248" s="4"/>
+      <c r="AB248" s="4"/>
+      <c r="AC248" s="4"/>
+      <c r="AD248" s="4"/>
+      <c r="AE248" s="4"/>
+      <c r="AF248" s="4"/>
+      <c r="AG248" s="4"/>
+      <c r="AH248" s="4"/>
+      <c r="AI248" s="4"/>
+    </row>
+    <row r="249" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A249" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="B249" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C249" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D249" s="4"/>
+      <c r="E249" s="4"/>
+      <c r="F249" s="4"/>
+      <c r="G249" s="4"/>
+      <c r="H249" s="4"/>
+      <c r="I249" s="4"/>
+      <c r="J249" s="4"/>
+      <c r="K249" s="4"/>
+      <c r="L249" s="4"/>
+      <c r="M249" s="4"/>
+      <c r="N249" s="4"/>
+      <c r="O249" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="P249" s="4"/>
+      <c r="Q249" s="4"/>
+      <c r="R249" s="4"/>
+      <c r="S249" s="4"/>
+      <c r="T249" s="4"/>
+      <c r="U249" s="4"/>
+      <c r="V249" s="4"/>
+      <c r="W249" s="4"/>
+      <c r="X249" s="4"/>
+      <c r="Y249" s="4"/>
+      <c r="Z249" s="4"/>
+      <c r="AA249" s="4"/>
+      <c r="AB249" s="4"/>
+      <c r="AC249" s="4"/>
+      <c r="AD249" s="4"/>
+      <c r="AE249" s="4"/>
+      <c r="AF249" s="4"/>
+      <c r="AG249" s="4"/>
+      <c r="AH249" s="4"/>
+      <c r="AI249" s="4"/>
+    </row>
+    <row r="250" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A250" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="B250" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C250" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D250" s="4"/>
+      <c r="E250" s="4"/>
+      <c r="F250" s="4"/>
+      <c r="G250" s="4"/>
+      <c r="H250" s="4"/>
+      <c r="I250" s="4"/>
+      <c r="J250" s="4"/>
+      <c r="K250" s="4"/>
+      <c r="L250" s="4"/>
+      <c r="M250" s="4"/>
+      <c r="N250" s="4"/>
+      <c r="O250" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="P250" s="4"/>
+      <c r="Q250" s="4"/>
+      <c r="R250" s="4"/>
+      <c r="S250" s="4"/>
+      <c r="T250" s="4"/>
+      <c r="U250" s="4"/>
+      <c r="V250" s="4"/>
+      <c r="W250" s="4"/>
+      <c r="X250" s="4"/>
+      <c r="Y250" s="4"/>
+      <c r="Z250" s="4"/>
+      <c r="AA250" s="4"/>
+      <c r="AB250" s="4"/>
+      <c r="AC250" s="4"/>
+      <c r="AD250" s="4"/>
+      <c r="AE250" s="4"/>
+      <c r="AF250" s="4"/>
+      <c r="AG250" s="4"/>
+      <c r="AH250" s="4"/>
+      <c r="AI250" s="4"/>
+    </row>
+    <row r="251" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A251" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B251" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C251" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D251" s="4"/>
+      <c r="E251" s="4"/>
+      <c r="F251" s="4"/>
+      <c r="G251" s="4"/>
+      <c r="H251" s="4"/>
+      <c r="I251" s="4"/>
+      <c r="J251" s="4"/>
+      <c r="K251" s="4"/>
+      <c r="L251" s="4"/>
+      <c r="M251" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="N251" s="4"/>
+      <c r="O251" s="4"/>
+      <c r="P251" s="4"/>
+      <c r="Q251" s="4"/>
+      <c r="R251" s="4"/>
+      <c r="S251" s="4"/>
+      <c r="T251" s="4"/>
+      <c r="U251" s="4"/>
+      <c r="V251" s="4"/>
+      <c r="W251" s="4"/>
+      <c r="X251" s="4"/>
+      <c r="Y251" s="4"/>
+      <c r="Z251" s="4"/>
+      <c r="AA251" s="4"/>
+      <c r="AB251" s="4"/>
+      <c r="AC251" s="4"/>
+      <c r="AD251" s="4"/>
+      <c r="AE251" s="4"/>
+      <c r="AF251" s="4"/>
+      <c r="AG251" s="4"/>
+      <c r="AH251" s="4"/>
+      <c r="AI251" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15193,7 +15431,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B611D72-2CC2-4CCA-A1E6-2A10215873D6}">
-  <dimension ref="A1:T239"/>
+  <dimension ref="A1:T243"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -23295,13 +23533,13 @@
         <v>709</v>
       </c>
       <c r="C228" s="3" t="s">
-        <v>38</v>
+        <v>549</v>
       </c>
       <c r="D228" s="3" t="s">
         <v>545</v>
       </c>
       <c r="E228" s="3" t="s">
-        <v>38</v>
+        <v>549</v>
       </c>
       <c r="F228" s="4"/>
       <c r="G228" s="4"/>
@@ -23742,6 +23980,158 @@
       </c>
       <c r="S239" s="4"/>
       <c r="T239" s="4"/>
+    </row>
+    <row r="240" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A240" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="B240" s="3" t="s">
+        <v>787</v>
+      </c>
+      <c r="C240" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D240" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E240" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F240" s="4"/>
+      <c r="G240" s="4"/>
+      <c r="H240" s="4"/>
+      <c r="I240" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="J240" s="4"/>
+      <c r="K240" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="L240" s="4"/>
+      <c r="M240" s="4"/>
+      <c r="N240" s="4"/>
+      <c r="O240" s="4"/>
+      <c r="P240" s="4"/>
+      <c r="Q240" s="4"/>
+      <c r="R240" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="S240" s="4"/>
+      <c r="T240" s="4"/>
+    </row>
+    <row r="241" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A241" s="3" t="s">
+        <v>790</v>
+      </c>
+      <c r="B241" s="3" t="s">
+        <v>791</v>
+      </c>
+      <c r="C241" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="D241" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E241" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="F241" s="4"/>
+      <c r="G241" s="4"/>
+      <c r="H241" s="4"/>
+      <c r="I241" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="J241" s="4"/>
+      <c r="K241" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="L241" s="4"/>
+      <c r="M241" s="4"/>
+      <c r="N241" s="4"/>
+      <c r="O241" s="4"/>
+      <c r="P241" s="4"/>
+      <c r="Q241" s="4"/>
+      <c r="R241" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="S241" s="4"/>
+      <c r="T241" s="4"/>
+    </row>
+    <row r="242" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A242" s="3" t="s">
+        <v>793</v>
+      </c>
+      <c r="B242" t="s">
+        <v>794</v>
+      </c>
+      <c r="C242" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D242" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E242" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F242" s="4"/>
+      <c r="G242" s="4"/>
+      <c r="H242" s="4"/>
+      <c r="I242" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="J242" s="4"/>
+      <c r="K242" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="L242" s="4"/>
+      <c r="M242" s="4"/>
+      <c r="N242" s="4"/>
+      <c r="O242" s="4"/>
+      <c r="P242" s="4"/>
+      <c r="Q242" s="4"/>
+      <c r="R242" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="S242" s="4"/>
+      <c r="T242" s="4"/>
+    </row>
+    <row r="243" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A243" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="B243" s="3" t="s">
+        <v>787</v>
+      </c>
+      <c r="C243" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D243" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E243" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F243" s="4"/>
+      <c r="G243" s="4"/>
+      <c r="H243" s="4"/>
+      <c r="I243" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="J243" s="4"/>
+      <c r="K243" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="L243" s="4"/>
+      <c r="M243" s="4"/>
+      <c r="N243" s="4"/>
+      <c r="O243" s="4"/>
+      <c r="P243" s="4"/>
+      <c r="Q243" s="4"/>
+      <c r="R243" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="S243" s="4"/>
+      <c r="T243" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Commit the latest changes for new scenario in 4 customer
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ffd-sys-team\git\eai-3534455-ffd-manhattan-automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F72EBC5F-DE75-4666-BBA4-B0BACAB5BB6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F934BC92-FBE5-4788-B43B-D4E6A17F7231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -23840,13 +23840,13 @@
         <v>768</v>
       </c>
       <c r="C234" s="3" t="s">
-        <v>38</v>
+        <v>295</v>
       </c>
       <c r="D234" s="3" t="s">
         <v>544</v>
       </c>
       <c r="E234" s="3" t="s">
-        <v>38</v>
+        <v>295</v>
       </c>
       <c r="F234" s="4"/>
       <c r="G234" s="4"/>

</xml_diff>

<commit_message>
commit THM scenario for inbound
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ffd-sys-team\git\eai-3534455-ffd-manhattan-automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F934BC92-FBE5-4788-B43B-D4E6A17F7231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C3EB33-959F-4179-B35E-0B0D85D2A875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3459" uniqueCount="808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3481" uniqueCount="814">
   <si>
     <t>ScearioID</t>
   </si>
@@ -2462,6 +2462,24 @@
   </si>
   <si>
     <t>No data found,No data found,No data found</t>
+  </si>
+  <si>
+    <t>THM_KelliScenario002</t>
+  </si>
+  <si>
+    <t>1032</t>
+  </si>
+  <si>
+    <t>1033</t>
+  </si>
+  <si>
+    <t>1032|1033</t>
+  </si>
+  <si>
+    <t>1156519-150</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1301273-108     </t>
   </si>
 </sst>
 </file>
@@ -2932,7 +2950,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA0C8091-AB5D-461B-B4FE-5D2410DFE16F}">
-  <dimension ref="A1:AI252"/>
+  <dimension ref="A1:AI253"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -15189,15 +15207,25 @@
       <c r="AI245" s="4"/>
     </row>
     <row r="246" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A246" s="4"/>
-      <c r="B246" s="4"/>
-      <c r="C246" s="4"/>
-      <c r="D246" s="4"/>
+      <c r="A246" s="4" t="s">
+        <v>808</v>
+      </c>
+      <c r="B246" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="C246" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D246" s="5" t="s">
+        <v>811</v>
+      </c>
       <c r="E246" s="4"/>
       <c r="F246" s="4"/>
       <c r="G246" s="4"/>
       <c r="H246" s="4"/>
-      <c r="I246" s="4"/>
+      <c r="I246" s="4" t="s">
+        <v>46</v>
+      </c>
       <c r="J246" s="4"/>
       <c r="K246" s="4"/>
       <c r="L246" s="4"/>
@@ -15219,37 +15247,27 @@
       <c r="AB246" s="4"/>
       <c r="AC246" s="4"/>
       <c r="AD246" s="4"/>
-      <c r="AE246" s="4"/>
+      <c r="AE246" s="4" t="s">
+        <v>499</v>
+      </c>
       <c r="AF246" s="4"/>
       <c r="AG246" s="4"/>
       <c r="AH246" s="4"/>
       <c r="AI246" s="4"/>
     </row>
     <row r="247" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A247" s="4" t="s">
-        <v>510</v>
-      </c>
-      <c r="B247" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C247" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="A247" s="4"/>
+      <c r="B247" s="4"/>
+      <c r="C247" s="4"/>
       <c r="D247" s="4"/>
       <c r="E247" s="4"/>
       <c r="F247" s="4"/>
       <c r="G247" s="4"/>
       <c r="H247" s="4"/>
       <c r="I247" s="4"/>
-      <c r="J247" s="3" t="s">
-        <v>511</v>
-      </c>
-      <c r="K247" s="3" t="s">
-        <v>512</v>
-      </c>
-      <c r="L247" s="3" t="s">
-        <v>513</v>
-      </c>
+      <c r="J247" s="4"/>
+      <c r="K247" s="4"/>
+      <c r="L247" s="4"/>
       <c r="M247" s="4"/>
       <c r="N247" s="4"/>
       <c r="O247" s="4"/>
@@ -15276,7 +15294,7 @@
     </row>
     <row r="248" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A248" s="4" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="B248" s="4" t="s">
         <v>228</v>
@@ -15291,13 +15309,13 @@
       <c r="H248" s="4"/>
       <c r="I248" s="4"/>
       <c r="J248" s="3" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="K248" s="3" t="s">
-        <v>243</v>
+        <v>512</v>
       </c>
       <c r="L248" s="3" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="M248" s="4"/>
       <c r="N248" s="4"/>
@@ -15325,7 +15343,7 @@
     </row>
     <row r="249" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A249" s="4" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="B249" s="4" t="s">
         <v>228</v>
@@ -15339,14 +15357,18 @@
       <c r="G249" s="4"/>
       <c r="H249" s="4"/>
       <c r="I249" s="4"/>
-      <c r="J249" s="4"/>
-      <c r="K249" s="4"/>
-      <c r="L249" s="4"/>
+      <c r="J249" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="K249" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="L249" s="3" t="s">
+        <v>516</v>
+      </c>
       <c r="M249" s="4"/>
       <c r="N249" s="4"/>
-      <c r="O249" s="3" t="s">
-        <v>518</v>
-      </c>
+      <c r="O249" s="4"/>
       <c r="P249" s="4"/>
       <c r="Q249" s="4"/>
       <c r="R249" s="4"/>
@@ -15370,7 +15392,7 @@
     </row>
     <row r="250" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A250" s="4" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="B250" s="4" t="s">
         <v>228</v>
@@ -15390,7 +15412,7 @@
       <c r="M250" s="4"/>
       <c r="N250" s="4"/>
       <c r="O250" s="3" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="P250" s="4"/>
       <c r="Q250" s="4"/>
@@ -15415,7 +15437,7 @@
     </row>
     <row r="251" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A251" s="4" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="B251" s="4" t="s">
         <v>228</v>
@@ -15435,7 +15457,7 @@
       <c r="M251" s="4"/>
       <c r="N251" s="4"/>
       <c r="O251" s="3" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="P251" s="4"/>
       <c r="Q251" s="4"/>
@@ -15460,7 +15482,7 @@
     </row>
     <row r="252" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A252" s="4" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="B252" s="4" t="s">
         <v>228</v>
@@ -15477,11 +15499,11 @@
       <c r="J252" s="4"/>
       <c r="K252" s="4"/>
       <c r="L252" s="4"/>
-      <c r="M252" s="4" t="s">
-        <v>524</v>
-      </c>
+      <c r="M252" s="4"/>
       <c r="N252" s="4"/>
-      <c r="O252" s="4"/>
+      <c r="O252" s="3" t="s">
+        <v>522</v>
+      </c>
       <c r="P252" s="4"/>
       <c r="Q252" s="4"/>
       <c r="R252" s="4"/>
@@ -15503,6 +15525,51 @@
       <c r="AH252" s="4"/>
       <c r="AI252" s="4"/>
     </row>
+    <row r="253" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A253" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="B253" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C253" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D253" s="4"/>
+      <c r="E253" s="4"/>
+      <c r="F253" s="4"/>
+      <c r="G253" s="4"/>
+      <c r="H253" s="4"/>
+      <c r="I253" s="4"/>
+      <c r="J253" s="4"/>
+      <c r="K253" s="4"/>
+      <c r="L253" s="4"/>
+      <c r="M253" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="N253" s="4"/>
+      <c r="O253" s="4"/>
+      <c r="P253" s="4"/>
+      <c r="Q253" s="4"/>
+      <c r="R253" s="4"/>
+      <c r="S253" s="4"/>
+      <c r="T253" s="4"/>
+      <c r="U253" s="4"/>
+      <c r="V253" s="4"/>
+      <c r="W253" s="4"/>
+      <c r="X253" s="4"/>
+      <c r="Y253" s="4"/>
+      <c r="Z253" s="4"/>
+      <c r="AA253" s="4"/>
+      <c r="AB253" s="4"/>
+      <c r="AC253" s="4"/>
+      <c r="AD253" s="4"/>
+      <c r="AE253" s="4"/>
+      <c r="AF253" s="4"/>
+      <c r="AG253" s="4"/>
+      <c r="AH253" s="4"/>
+      <c r="AI253" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15510,7 +15577,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B611D72-2CC2-4CCA-A1E6-2A10215873D6}">
-  <dimension ref="A1:T246"/>
+  <dimension ref="A1:T248"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -24326,6 +24393,82 @@
       <c r="S246" s="4"/>
       <c r="T246" s="4"/>
     </row>
+    <row r="247" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A247" s="3" t="s">
+        <v>809</v>
+      </c>
+      <c r="B247" s="12" t="s">
+        <v>812</v>
+      </c>
+      <c r="C247" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="D247" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E247" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="F247" s="4"/>
+      <c r="G247" s="4"/>
+      <c r="H247" s="4"/>
+      <c r="I247" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="J247" s="4"/>
+      <c r="K247" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="L247" s="4"/>
+      <c r="M247" s="4"/>
+      <c r="N247" s="4"/>
+      <c r="O247" s="4"/>
+      <c r="P247" s="4"/>
+      <c r="Q247" s="4"/>
+      <c r="R247" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="S247" s="4"/>
+      <c r="T247" s="4"/>
+    </row>
+    <row r="248" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A248" s="3" t="s">
+        <v>810</v>
+      </c>
+      <c r="B248" s="3" t="s">
+        <v>813</v>
+      </c>
+      <c r="C248" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D248" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E248" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F248" s="4"/>
+      <c r="G248" s="4"/>
+      <c r="H248" s="4"/>
+      <c r="I248" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="J248" s="4"/>
+      <c r="K248" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="L248" s="4"/>
+      <c r="M248" s="4"/>
+      <c r="N248" s="4"/>
+      <c r="O248" s="4"/>
+      <c r="P248" s="4"/>
+      <c r="Q248" s="4"/>
+      <c r="R248" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="S248" s="4"/>
+      <c r="T248" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Commit the changes done for 4 customer scenario
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ffd-sys-team\git\eai-3534455-ffd-manhattan-automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C3EB33-959F-4179-B35E-0B0D85D2A875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18320106-5C06-4E3A-ADB7-A61E87D2C211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3481" uniqueCount="814">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3589" uniqueCount="839">
   <si>
     <t>ScearioID</t>
   </si>
@@ -2480,6 +2480,81 @@
   </si>
   <si>
     <t xml:space="preserve">1301273-108     </t>
+  </si>
+  <si>
+    <t>THM_KelliScenario003</t>
+  </si>
+  <si>
+    <t>1034</t>
+  </si>
+  <si>
+    <t>7777777-888</t>
+  </si>
+  <si>
+    <t>1035|1036</t>
+  </si>
+  <si>
+    <t>1035</t>
+  </si>
+  <si>
+    <t>1036</t>
+  </si>
+  <si>
+    <t>187500-101</t>
+  </si>
+  <si>
+    <t>THH_KelliScenario003</t>
+  </si>
+  <si>
+    <t>THH_KelliScenario004</t>
+  </si>
+  <si>
+    <t>1037</t>
+  </si>
+  <si>
+    <t>7777777-999</t>
+  </si>
+  <si>
+    <t>TRN_KelliScenario003</t>
+  </si>
+  <si>
+    <t>1038</t>
+  </si>
+  <si>
+    <t>7777777-777</t>
+  </si>
+  <si>
+    <t>ILW_KelliScenario002</t>
+  </si>
+  <si>
+    <t>1039|1040|1041</t>
+  </si>
+  <si>
+    <t>1039</t>
+  </si>
+  <si>
+    <t>1040</t>
+  </si>
+  <si>
+    <t>1041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00009758080               </t>
+  </si>
+  <si>
+    <t xml:space="preserve">066QL0025                 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">00018110834 </t>
+  </si>
+  <si>
+    <t>ILW_KelliScenario003</t>
+  </si>
+  <si>
+    <t>1042</t>
+  </si>
+  <si>
+    <t>7777777-666</t>
   </si>
 </sst>
 </file>
@@ -2654,9 +2729,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2694,7 +2769,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2800,7 +2875,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2942,7 +3017,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2950,7 +3025,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA0C8091-AB5D-461B-B4FE-5D2410DFE16F}">
-  <dimension ref="A1:AI253"/>
+  <dimension ref="A1:AI259"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -15256,15 +15331,25 @@
       <c r="AI246" s="4"/>
     </row>
     <row r="247" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A247" s="4"/>
-      <c r="B247" s="4"/>
-      <c r="C247" s="4"/>
-      <c r="D247" s="4"/>
+      <c r="A247" s="4" t="s">
+        <v>814</v>
+      </c>
+      <c r="B247" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="C247" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D247" s="5" t="s">
+        <v>815</v>
+      </c>
       <c r="E247" s="4"/>
       <c r="F247" s="4"/>
       <c r="G247" s="4"/>
       <c r="H247" s="4"/>
-      <c r="I247" s="4"/>
+      <c r="I247" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="J247" s="4"/>
       <c r="K247" s="4"/>
       <c r="L247" s="4"/>
@@ -15286,7 +15371,9 @@
       <c r="AB247" s="4"/>
       <c r="AC247" s="4"/>
       <c r="AD247" s="4"/>
-      <c r="AE247" s="4"/>
+      <c r="AE247" s="4" t="s">
+        <v>499</v>
+      </c>
       <c r="AF247" s="4"/>
       <c r="AG247" s="4"/>
       <c r="AH247" s="4"/>
@@ -15294,29 +15381,27 @@
     </row>
     <row r="248" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A248" s="4" t="s">
-        <v>510</v>
+        <v>821</v>
       </c>
       <c r="B248" s="4" t="s">
-        <v>228</v>
+        <v>496</v>
       </c>
       <c r="C248" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D248" s="4"/>
+        <v>232</v>
+      </c>
+      <c r="D248" s="5" t="s">
+        <v>817</v>
+      </c>
       <c r="E248" s="4"/>
       <c r="F248" s="4"/>
       <c r="G248" s="4"/>
       <c r="H248" s="4"/>
-      <c r="I248" s="4"/>
-      <c r="J248" s="3" t="s">
-        <v>511</v>
-      </c>
-      <c r="K248" s="3" t="s">
-        <v>512</v>
-      </c>
-      <c r="L248" s="3" t="s">
-        <v>513</v>
-      </c>
+      <c r="I248" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="J248" s="4"/>
+      <c r="K248" s="4"/>
+      <c r="L248" s="4"/>
       <c r="M248" s="4"/>
       <c r="N248" s="4"/>
       <c r="O248" s="4"/>
@@ -15335,7 +15420,9 @@
       <c r="AB248" s="4"/>
       <c r="AC248" s="4"/>
       <c r="AD248" s="4"/>
-      <c r="AE248" s="4"/>
+      <c r="AE248" s="4" t="s">
+        <v>496</v>
+      </c>
       <c r="AF248" s="4"/>
       <c r="AG248" s="4"/>
       <c r="AH248" s="4"/>
@@ -15343,29 +15430,27 @@
     </row>
     <row r="249" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A249" s="4" t="s">
-        <v>514</v>
+        <v>822</v>
       </c>
       <c r="B249" s="4" t="s">
-        <v>228</v>
+        <v>499</v>
       </c>
       <c r="C249" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D249" s="4"/>
+        <v>232</v>
+      </c>
+      <c r="D249" s="5" t="s">
+        <v>823</v>
+      </c>
       <c r="E249" s="4"/>
       <c r="F249" s="4"/>
       <c r="G249" s="4"/>
       <c r="H249" s="4"/>
-      <c r="I249" s="4"/>
-      <c r="J249" s="3" t="s">
-        <v>515</v>
-      </c>
-      <c r="K249" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="L249" s="3" t="s">
-        <v>516</v>
-      </c>
+      <c r="I249" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J249" s="4"/>
+      <c r="K249" s="4"/>
+      <c r="L249" s="4"/>
       <c r="M249" s="4"/>
       <c r="N249" s="4"/>
       <c r="O249" s="4"/>
@@ -15384,7 +15469,9 @@
       <c r="AB249" s="4"/>
       <c r="AC249" s="4"/>
       <c r="AD249" s="4"/>
-      <c r="AE249" s="4"/>
+      <c r="AE249" s="4" t="s">
+        <v>496</v>
+      </c>
       <c r="AF249" s="4"/>
       <c r="AG249" s="4"/>
       <c r="AH249" s="4"/>
@@ -15392,28 +15479,30 @@
     </row>
     <row r="250" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A250" s="4" t="s">
-        <v>517</v>
+        <v>825</v>
       </c>
       <c r="B250" s="4" t="s">
-        <v>228</v>
+        <v>502</v>
       </c>
       <c r="C250" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D250" s="4"/>
+        <v>232</v>
+      </c>
+      <c r="D250" s="5" t="s">
+        <v>826</v>
+      </c>
       <c r="E250" s="4"/>
       <c r="F250" s="4"/>
       <c r="G250" s="4"/>
       <c r="H250" s="4"/>
-      <c r="I250" s="4"/>
+      <c r="I250" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="J250" s="4"/>
       <c r="K250" s="4"/>
       <c r="L250" s="4"/>
       <c r="M250" s="4"/>
       <c r="N250" s="4"/>
-      <c r="O250" s="3" t="s">
-        <v>518</v>
-      </c>
+      <c r="O250" s="4"/>
       <c r="P250" s="4"/>
       <c r="Q250" s="4"/>
       <c r="R250" s="4"/>
@@ -15429,7 +15518,9 @@
       <c r="AB250" s="4"/>
       <c r="AC250" s="4"/>
       <c r="AD250" s="4"/>
-      <c r="AE250" s="4"/>
+      <c r="AE250" s="4" t="s">
+        <v>503</v>
+      </c>
       <c r="AF250" s="4"/>
       <c r="AG250" s="4"/>
       <c r="AH250" s="4"/>
@@ -15437,28 +15528,30 @@
     </row>
     <row r="251" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A251" s="4" t="s">
-        <v>519</v>
+        <v>828</v>
       </c>
       <c r="B251" s="4" t="s">
-        <v>228</v>
+        <v>505</v>
       </c>
       <c r="C251" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D251" s="4"/>
+        <v>232</v>
+      </c>
+      <c r="D251" s="5" t="s">
+        <v>829</v>
+      </c>
       <c r="E251" s="4"/>
       <c r="F251" s="4"/>
       <c r="G251" s="4"/>
       <c r="H251" s="4"/>
-      <c r="I251" s="4"/>
+      <c r="I251" s="4" t="s">
+        <v>807</v>
+      </c>
       <c r="J251" s="4"/>
       <c r="K251" s="4"/>
       <c r="L251" s="4"/>
       <c r="M251" s="4"/>
       <c r="N251" s="4"/>
-      <c r="O251" s="3" t="s">
-        <v>520</v>
-      </c>
+      <c r="O251" s="4"/>
       <c r="P251" s="4"/>
       <c r="Q251" s="4"/>
       <c r="R251" s="4"/>
@@ -15474,7 +15567,9 @@
       <c r="AB251" s="4"/>
       <c r="AC251" s="4"/>
       <c r="AD251" s="4"/>
-      <c r="AE251" s="4"/>
+      <c r="AE251" s="4" t="s">
+        <v>505</v>
+      </c>
       <c r="AF251" s="4"/>
       <c r="AG251" s="4"/>
       <c r="AH251" s="4"/>
@@ -15482,28 +15577,30 @@
     </row>
     <row r="252" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A252" s="4" t="s">
-        <v>521</v>
+        <v>836</v>
       </c>
       <c r="B252" s="4" t="s">
-        <v>228</v>
+        <v>505</v>
       </c>
       <c r="C252" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D252" s="4"/>
+        <v>232</v>
+      </c>
+      <c r="D252" s="5" t="s">
+        <v>837</v>
+      </c>
       <c r="E252" s="4"/>
       <c r="F252" s="4"/>
       <c r="G252" s="4"/>
       <c r="H252" s="4"/>
-      <c r="I252" s="4"/>
+      <c r="I252" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="J252" s="4"/>
       <c r="K252" s="4"/>
       <c r="L252" s="4"/>
       <c r="M252" s="4"/>
       <c r="N252" s="4"/>
-      <c r="O252" s="3" t="s">
-        <v>522</v>
-      </c>
+      <c r="O252" s="4"/>
       <c r="P252" s="4"/>
       <c r="Q252" s="4"/>
       <c r="R252" s="4"/>
@@ -15519,22 +15616,18 @@
       <c r="AB252" s="4"/>
       <c r="AC252" s="4"/>
       <c r="AD252" s="4"/>
-      <c r="AE252" s="4"/>
+      <c r="AE252" s="4" t="s">
+        <v>505</v>
+      </c>
       <c r="AF252" s="4"/>
       <c r="AG252" s="4"/>
       <c r="AH252" s="4"/>
       <c r="AI252" s="4"/>
     </row>
     <row r="253" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A253" s="4" t="s">
-        <v>523</v>
-      </c>
-      <c r="B253" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C253" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="A253" s="4"/>
+      <c r="B253" s="4"/>
+      <c r="C253" s="4"/>
       <c r="D253" s="4"/>
       <c r="E253" s="4"/>
       <c r="F253" s="4"/>
@@ -15544,9 +15637,7 @@
       <c r="J253" s="4"/>
       <c r="K253" s="4"/>
       <c r="L253" s="4"/>
-      <c r="M253" s="4" t="s">
-        <v>524</v>
-      </c>
+      <c r="M253" s="4"/>
       <c r="N253" s="4"/>
       <c r="O253" s="4"/>
       <c r="P253" s="4"/>
@@ -15570,6 +15661,284 @@
       <c r="AH253" s="4"/>
       <c r="AI253" s="4"/>
     </row>
+    <row r="254" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A254" s="4" t="s">
+        <v>510</v>
+      </c>
+      <c r="B254" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C254" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D254" s="4"/>
+      <c r="E254" s="4"/>
+      <c r="F254" s="4"/>
+      <c r="G254" s="4"/>
+      <c r="H254" s="4"/>
+      <c r="I254" s="4"/>
+      <c r="J254" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="K254" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="L254" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="M254" s="4"/>
+      <c r="N254" s="4"/>
+      <c r="O254" s="4"/>
+      <c r="P254" s="4"/>
+      <c r="Q254" s="4"/>
+      <c r="R254" s="4"/>
+      <c r="S254" s="4"/>
+      <c r="T254" s="4"/>
+      <c r="U254" s="4"/>
+      <c r="V254" s="4"/>
+      <c r="W254" s="4"/>
+      <c r="X254" s="4"/>
+      <c r="Y254" s="4"/>
+      <c r="Z254" s="4"/>
+      <c r="AA254" s="4"/>
+      <c r="AB254" s="4"/>
+      <c r="AC254" s="4"/>
+      <c r="AD254" s="4"/>
+      <c r="AE254" s="4"/>
+      <c r="AF254" s="4"/>
+      <c r="AG254" s="4"/>
+      <c r="AH254" s="4"/>
+      <c r="AI254" s="4"/>
+    </row>
+    <row r="255" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A255" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="B255" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C255" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D255" s="4"/>
+      <c r="E255" s="4"/>
+      <c r="F255" s="4"/>
+      <c r="G255" s="4"/>
+      <c r="H255" s="4"/>
+      <c r="I255" s="4"/>
+      <c r="J255" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="K255" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="L255" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="M255" s="4"/>
+      <c r="N255" s="4"/>
+      <c r="O255" s="4"/>
+      <c r="P255" s="4"/>
+      <c r="Q255" s="4"/>
+      <c r="R255" s="4"/>
+      <c r="S255" s="4"/>
+      <c r="T255" s="4"/>
+      <c r="U255" s="4"/>
+      <c r="V255" s="4"/>
+      <c r="W255" s="4"/>
+      <c r="X255" s="4"/>
+      <c r="Y255" s="4"/>
+      <c r="Z255" s="4"/>
+      <c r="AA255" s="4"/>
+      <c r="AB255" s="4"/>
+      <c r="AC255" s="4"/>
+      <c r="AD255" s="4"/>
+      <c r="AE255" s="4"/>
+      <c r="AF255" s="4"/>
+      <c r="AG255" s="4"/>
+      <c r="AH255" s="4"/>
+      <c r="AI255" s="4"/>
+    </row>
+    <row r="256" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A256" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="B256" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C256" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D256" s="4"/>
+      <c r="E256" s="4"/>
+      <c r="F256" s="4"/>
+      <c r="G256" s="4"/>
+      <c r="H256" s="4"/>
+      <c r="I256" s="4"/>
+      <c r="J256" s="4"/>
+      <c r="K256" s="4"/>
+      <c r="L256" s="4"/>
+      <c r="M256" s="4"/>
+      <c r="N256" s="4"/>
+      <c r="O256" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="P256" s="4"/>
+      <c r="Q256" s="4"/>
+      <c r="R256" s="4"/>
+      <c r="S256" s="4"/>
+      <c r="T256" s="4"/>
+      <c r="U256" s="4"/>
+      <c r="V256" s="4"/>
+      <c r="W256" s="4"/>
+      <c r="X256" s="4"/>
+      <c r="Y256" s="4"/>
+      <c r="Z256" s="4"/>
+      <c r="AA256" s="4"/>
+      <c r="AB256" s="4"/>
+      <c r="AC256" s="4"/>
+      <c r="AD256" s="4"/>
+      <c r="AE256" s="4"/>
+      <c r="AF256" s="4"/>
+      <c r="AG256" s="4"/>
+      <c r="AH256" s="4"/>
+      <c r="AI256" s="4"/>
+    </row>
+    <row r="257" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A257" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="B257" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C257" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D257" s="4"/>
+      <c r="E257" s="4"/>
+      <c r="F257" s="4"/>
+      <c r="G257" s="4"/>
+      <c r="H257" s="4"/>
+      <c r="I257" s="4"/>
+      <c r="J257" s="4"/>
+      <c r="K257" s="4"/>
+      <c r="L257" s="4"/>
+      <c r="M257" s="4"/>
+      <c r="N257" s="4"/>
+      <c r="O257" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="P257" s="4"/>
+      <c r="Q257" s="4"/>
+      <c r="R257" s="4"/>
+      <c r="S257" s="4"/>
+      <c r="T257" s="4"/>
+      <c r="U257" s="4"/>
+      <c r="V257" s="4"/>
+      <c r="W257" s="4"/>
+      <c r="X257" s="4"/>
+      <c r="Y257" s="4"/>
+      <c r="Z257" s="4"/>
+      <c r="AA257" s="4"/>
+      <c r="AB257" s="4"/>
+      <c r="AC257" s="4"/>
+      <c r="AD257" s="4"/>
+      <c r="AE257" s="4"/>
+      <c r="AF257" s="4"/>
+      <c r="AG257" s="4"/>
+      <c r="AH257" s="4"/>
+      <c r="AI257" s="4"/>
+    </row>
+    <row r="258" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A258" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="B258" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C258" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D258" s="4"/>
+      <c r="E258" s="4"/>
+      <c r="F258" s="4"/>
+      <c r="G258" s="4"/>
+      <c r="H258" s="4"/>
+      <c r="I258" s="4"/>
+      <c r="J258" s="4"/>
+      <c r="K258" s="4"/>
+      <c r="L258" s="4"/>
+      <c r="M258" s="4"/>
+      <c r="N258" s="4"/>
+      <c r="O258" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="P258" s="4"/>
+      <c r="Q258" s="4"/>
+      <c r="R258" s="4"/>
+      <c r="S258" s="4"/>
+      <c r="T258" s="4"/>
+      <c r="U258" s="4"/>
+      <c r="V258" s="4"/>
+      <c r="W258" s="4"/>
+      <c r="X258" s="4"/>
+      <c r="Y258" s="4"/>
+      <c r="Z258" s="4"/>
+      <c r="AA258" s="4"/>
+      <c r="AB258" s="4"/>
+      <c r="AC258" s="4"/>
+      <c r="AD258" s="4"/>
+      <c r="AE258" s="4"/>
+      <c r="AF258" s="4"/>
+      <c r="AG258" s="4"/>
+      <c r="AH258" s="4"/>
+      <c r="AI258" s="4"/>
+    </row>
+    <row r="259" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A259" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="B259" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C259" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D259" s="4"/>
+      <c r="E259" s="4"/>
+      <c r="F259" s="4"/>
+      <c r="G259" s="4"/>
+      <c r="H259" s="4"/>
+      <c r="I259" s="4"/>
+      <c r="J259" s="4"/>
+      <c r="K259" s="4"/>
+      <c r="L259" s="4"/>
+      <c r="M259" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="N259" s="4"/>
+      <c r="O259" s="4"/>
+      <c r="P259" s="4"/>
+      <c r="Q259" s="4"/>
+      <c r="R259" s="4"/>
+      <c r="S259" s="4"/>
+      <c r="T259" s="4"/>
+      <c r="U259" s="4"/>
+      <c r="V259" s="4"/>
+      <c r="W259" s="4"/>
+      <c r="X259" s="4"/>
+      <c r="Y259" s="4"/>
+      <c r="Z259" s="4"/>
+      <c r="AA259" s="4"/>
+      <c r="AB259" s="4"/>
+      <c r="AC259" s="4"/>
+      <c r="AD259" s="4"/>
+      <c r="AE259" s="4"/>
+      <c r="AF259" s="4"/>
+      <c r="AG259" s="4"/>
+      <c r="AH259" s="4"/>
+      <c r="AI259" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15577,7 +15946,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B611D72-2CC2-4CCA-A1E6-2A10215873D6}">
-  <dimension ref="A1:T248"/>
+  <dimension ref="A1:T257"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -24469,6 +24838,348 @@
       <c r="S248" s="4"/>
       <c r="T248" s="4"/>
     </row>
+    <row r="249" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A249" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="B249" s="3" t="s">
+        <v>816</v>
+      </c>
+      <c r="C249" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D249" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E249" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F249" s="4"/>
+      <c r="G249" s="4"/>
+      <c r="H249" s="4"/>
+      <c r="I249" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="J249" s="4"/>
+      <c r="K249" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="L249" s="4"/>
+      <c r="M249" s="4"/>
+      <c r="N249" s="4"/>
+      <c r="O249" s="4"/>
+      <c r="P249" s="4"/>
+      <c r="Q249" s="4"/>
+      <c r="R249" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="S249" s="4"/>
+      <c r="T249" s="4"/>
+    </row>
+    <row r="250" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A250" s="3" t="s">
+        <v>818</v>
+      </c>
+      <c r="B250" s="5" t="s">
+        <v>768</v>
+      </c>
+      <c r="C250" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D250" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E250" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F250" s="4"/>
+      <c r="G250" s="4"/>
+      <c r="H250" s="4"/>
+      <c r="I250" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="J250" s="4"/>
+      <c r="K250" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="L250" s="4"/>
+      <c r="M250" s="4"/>
+      <c r="N250" s="4"/>
+      <c r="O250" s="4"/>
+      <c r="P250" s="4"/>
+      <c r="Q250" s="4"/>
+      <c r="R250" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="S250" s="4"/>
+      <c r="T250" s="4"/>
+    </row>
+    <row r="251" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A251" s="3" t="s">
+        <v>819</v>
+      </c>
+      <c r="B251" s="5" t="s">
+        <v>820</v>
+      </c>
+      <c r="C251" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D251" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E251" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F251" s="4"/>
+      <c r="G251" s="4"/>
+      <c r="H251" s="4"/>
+      <c r="I251" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="J251" s="4"/>
+      <c r="K251" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="L251" s="4"/>
+      <c r="M251" s="4"/>
+      <c r="N251" s="4"/>
+      <c r="O251" s="4"/>
+      <c r="P251" s="4"/>
+      <c r="Q251" s="4"/>
+      <c r="R251" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="S251" s="4"/>
+      <c r="T251" s="4"/>
+    </row>
+    <row r="252" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A252" s="3" t="s">
+        <v>823</v>
+      </c>
+      <c r="B252" s="3" t="s">
+        <v>824</v>
+      </c>
+      <c r="C252" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D252" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E252" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F252" s="4"/>
+      <c r="G252" s="4"/>
+      <c r="H252" s="4"/>
+      <c r="I252" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="J252" s="4"/>
+      <c r="K252" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="L252" s="4"/>
+      <c r="M252" s="4"/>
+      <c r="N252" s="4"/>
+      <c r="O252" s="4"/>
+      <c r="P252" s="4"/>
+      <c r="Q252" s="4"/>
+      <c r="R252" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="S252" s="4"/>
+      <c r="T252" s="4"/>
+    </row>
+    <row r="253" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A253" s="3" t="s">
+        <v>826</v>
+      </c>
+      <c r="B253" s="3" t="s">
+        <v>827</v>
+      </c>
+      <c r="C253" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D253" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E253" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F253" s="4"/>
+      <c r="G253" s="4"/>
+      <c r="H253" s="4"/>
+      <c r="I253" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="J253" s="4"/>
+      <c r="K253" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="L253" s="4"/>
+      <c r="M253" s="4"/>
+      <c r="N253" s="4"/>
+      <c r="O253" s="4"/>
+      <c r="P253" s="4"/>
+      <c r="Q253" s="4"/>
+      <c r="R253" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="S253" s="4"/>
+      <c r="T253" s="4"/>
+    </row>
+    <row r="254" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A254" s="3" t="s">
+        <v>830</v>
+      </c>
+      <c r="B254" s="3" t="s">
+        <v>833</v>
+      </c>
+      <c r="C254" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D254" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E254" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F254" s="4"/>
+      <c r="G254" s="4"/>
+      <c r="H254" s="4"/>
+      <c r="I254" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="J254" s="4"/>
+      <c r="K254" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="L254" s="4"/>
+      <c r="M254" s="4"/>
+      <c r="N254" s="4"/>
+      <c r="O254" s="4"/>
+      <c r="P254" s="4"/>
+      <c r="Q254" s="4"/>
+      <c r="R254" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="S254" s="4"/>
+      <c r="T254" s="4"/>
+    </row>
+    <row r="255" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A255" s="3" t="s">
+        <v>831</v>
+      </c>
+      <c r="B255" s="3" t="s">
+        <v>834</v>
+      </c>
+      <c r="C255" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D255" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E255" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F255" s="4"/>
+      <c r="G255" s="4"/>
+      <c r="H255" s="4"/>
+      <c r="I255" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="J255" s="4"/>
+      <c r="K255" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="L255" s="4"/>
+      <c r="M255" s="4"/>
+      <c r="N255" s="4"/>
+      <c r="O255" s="4"/>
+      <c r="P255" s="4"/>
+      <c r="Q255" s="4"/>
+      <c r="R255" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="S255" s="4"/>
+      <c r="T255" s="4"/>
+    </row>
+    <row r="256" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A256" s="3" t="s">
+        <v>832</v>
+      </c>
+      <c r="B256" s="3" t="s">
+        <v>835</v>
+      </c>
+      <c r="C256" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D256" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E256" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F256" s="4"/>
+      <c r="G256" s="4"/>
+      <c r="H256" s="4"/>
+      <c r="I256" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="J256" s="4"/>
+      <c r="K256" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="L256" s="4"/>
+      <c r="M256" s="4"/>
+      <c r="N256" s="4"/>
+      <c r="O256" s="4"/>
+      <c r="P256" s="4"/>
+      <c r="Q256" s="4"/>
+      <c r="R256" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="S256" s="4"/>
+      <c r="T256" s="4"/>
+    </row>
+    <row r="257" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A257" s="3" t="s">
+        <v>837</v>
+      </c>
+      <c r="B257" s="3" t="s">
+        <v>838</v>
+      </c>
+      <c r="C257" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D257" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="E257" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F257" s="4"/>
+      <c r="G257" s="4"/>
+      <c r="H257" s="4"/>
+      <c r="I257" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="J257" s="4"/>
+      <c r="K257" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="L257" s="4"/>
+      <c r="M257" s="4"/>
+      <c r="N257" s="4"/>
+      <c r="O257" s="4"/>
+      <c r="P257" s="4"/>
+      <c r="Q257" s="4"/>
+      <c r="R257" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="S257" s="4"/>
+      <c r="T257" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Commit the Testdata for four custmer
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ffd-sys-team\git\eai-3534455-ffd-manhattan-automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18320106-5C06-4E3A-ADB7-A61E87D2C211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3511C738-D603-4705-9AFC-FFC195A7E01F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
   </bookViews>
@@ -15433,7 +15433,7 @@
         <v>822</v>
       </c>
       <c r="B249" s="4" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C249" s="4" t="s">
         <v>232</v>

</xml_diff>

<commit_message>
commit the changes done for 4 customer IB scenarios
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ffd-sys-team\git\eai-3534455-ffd-manhattan-automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3511C738-D603-4705-9AFC-FFC195A7E01F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D690D2D4-58E5-41EF-9319-B5CA2FD0B4FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{B8F8015F-37F6-4586-B92C-8B20231BA75D}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioData" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3589" uniqueCount="839">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3623" uniqueCount="846">
   <si>
     <t>ScearioID</t>
   </si>
@@ -2555,6 +2555,27 @@
   </si>
   <si>
     <t>7777777-666</t>
+  </si>
+  <si>
+    <t>THH_KelliScenario005</t>
+  </si>
+  <si>
+    <t>ILW_KelliScenario004</t>
+  </si>
+  <si>
+    <t>1043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00000012152     </t>
+  </si>
+  <si>
+    <t>TRN_IBScenario004</t>
+  </si>
+  <si>
+    <t>1044</t>
+  </si>
+  <si>
+    <t>330314</t>
   </si>
 </sst>
 </file>
@@ -3025,7 +3046,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA0C8091-AB5D-461B-B4FE-5D2410DFE16F}">
-  <dimension ref="A1:AI259"/>
+  <dimension ref="A1:AI262"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -15625,15 +15646,25 @@
       <c r="AI252" s="4"/>
     </row>
     <row r="253" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A253" s="4"/>
-      <c r="B253" s="4"/>
-      <c r="C253" s="4"/>
-      <c r="D253" s="4"/>
+      <c r="A253" s="4" t="s">
+        <v>839</v>
+      </c>
+      <c r="B253" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="C253" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D253" s="5" t="s">
+        <v>818</v>
+      </c>
       <c r="E253" s="4"/>
       <c r="F253" s="4"/>
       <c r="G253" s="4"/>
       <c r="H253" s="4"/>
-      <c r="I253" s="4"/>
+      <c r="I253" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="J253" s="4"/>
       <c r="K253" s="4"/>
       <c r="L253" s="4"/>
@@ -15655,7 +15686,9 @@
       <c r="AB253" s="4"/>
       <c r="AC253" s="4"/>
       <c r="AD253" s="4"/>
-      <c r="AE253" s="4"/>
+      <c r="AE253" s="4" t="s">
+        <v>496</v>
+      </c>
       <c r="AF253" s="4"/>
       <c r="AG253" s="4"/>
       <c r="AH253" s="4"/>
@@ -15663,29 +15696,27 @@
     </row>
     <row r="254" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A254" s="4" t="s">
-        <v>510</v>
+        <v>840</v>
       </c>
       <c r="B254" s="4" t="s">
-        <v>228</v>
+        <v>505</v>
       </c>
       <c r="C254" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D254" s="4"/>
+        <v>232</v>
+      </c>
+      <c r="D254" s="5" t="s">
+        <v>841</v>
+      </c>
       <c r="E254" s="4"/>
       <c r="F254" s="4"/>
       <c r="G254" s="4"/>
       <c r="H254" s="4"/>
-      <c r="I254" s="4"/>
-      <c r="J254" s="3" t="s">
-        <v>511</v>
-      </c>
-      <c r="K254" s="3" t="s">
-        <v>512</v>
-      </c>
-      <c r="L254" s="3" t="s">
-        <v>513</v>
-      </c>
+      <c r="I254" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J254" s="4"/>
+      <c r="K254" s="4"/>
+      <c r="L254" s="4"/>
       <c r="M254" s="4"/>
       <c r="N254" s="4"/>
       <c r="O254" s="4"/>
@@ -15704,7 +15735,9 @@
       <c r="AB254" s="4"/>
       <c r="AC254" s="4"/>
       <c r="AD254" s="4"/>
-      <c r="AE254" s="4"/>
+      <c r="AE254" s="4" t="s">
+        <v>505</v>
+      </c>
       <c r="AF254" s="4"/>
       <c r="AG254" s="4"/>
       <c r="AH254" s="4"/>
@@ -15712,29 +15745,27 @@
     </row>
     <row r="255" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A255" s="4" t="s">
-        <v>514</v>
+        <v>843</v>
       </c>
       <c r="B255" s="4" t="s">
-        <v>228</v>
+        <v>502</v>
       </c>
       <c r="C255" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D255" s="4"/>
+        <v>232</v>
+      </c>
+      <c r="D255" s="5" t="s">
+        <v>844</v>
+      </c>
       <c r="E255" s="4"/>
       <c r="F255" s="4"/>
       <c r="G255" s="4"/>
       <c r="H255" s="4"/>
-      <c r="I255" s="4"/>
-      <c r="J255" s="3" t="s">
-        <v>515</v>
-      </c>
-      <c r="K255" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="L255" s="3" t="s">
-        <v>516</v>
-      </c>
+      <c r="I255" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J255" s="4"/>
+      <c r="K255" s="4"/>
+      <c r="L255" s="4"/>
       <c r="M255" s="4"/>
       <c r="N255" s="4"/>
       <c r="O255" s="4"/>
@@ -15753,22 +15784,18 @@
       <c r="AB255" s="4"/>
       <c r="AC255" s="4"/>
       <c r="AD255" s="4"/>
-      <c r="AE255" s="4"/>
+      <c r="AE255" s="4" t="s">
+        <v>503</v>
+      </c>
       <c r="AF255" s="4"/>
       <c r="AG255" s="4"/>
       <c r="AH255" s="4"/>
       <c r="AI255" s="4"/>
     </row>
     <row r="256" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A256" s="4" t="s">
-        <v>517</v>
-      </c>
-      <c r="B256" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C256" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="A256" s="4"/>
+      <c r="B256" s="4"/>
+      <c r="C256" s="4"/>
       <c r="D256" s="4"/>
       <c r="E256" s="4"/>
       <c r="F256" s="4"/>
@@ -15780,9 +15807,7 @@
       <c r="L256" s="4"/>
       <c r="M256" s="4"/>
       <c r="N256" s="4"/>
-      <c r="O256" s="3" t="s">
-        <v>518</v>
-      </c>
+      <c r="O256" s="4"/>
       <c r="P256" s="4"/>
       <c r="Q256" s="4"/>
       <c r="R256" s="4"/>
@@ -15806,7 +15831,7 @@
     </row>
     <row r="257" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A257" s="4" t="s">
-        <v>519</v>
+        <v>510</v>
       </c>
       <c r="B257" s="4" t="s">
         <v>228</v>
@@ -15820,14 +15845,18 @@
       <c r="G257" s="4"/>
       <c r="H257" s="4"/>
       <c r="I257" s="4"/>
-      <c r="J257" s="4"/>
-      <c r="K257" s="4"/>
-      <c r="L257" s="4"/>
+      <c r="J257" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="K257" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="L257" s="3" t="s">
+        <v>513</v>
+      </c>
       <c r="M257" s="4"/>
       <c r="N257" s="4"/>
-      <c r="O257" s="3" t="s">
-        <v>520</v>
-      </c>
+      <c r="O257" s="4"/>
       <c r="P257" s="4"/>
       <c r="Q257" s="4"/>
       <c r="R257" s="4"/>
@@ -15851,7 +15880,7 @@
     </row>
     <row r="258" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A258" s="4" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="B258" s="4" t="s">
         <v>228</v>
@@ -15865,14 +15894,18 @@
       <c r="G258" s="4"/>
       <c r="H258" s="4"/>
       <c r="I258" s="4"/>
-      <c r="J258" s="4"/>
-      <c r="K258" s="4"/>
-      <c r="L258" s="4"/>
+      <c r="J258" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="K258" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="L258" s="3" t="s">
+        <v>516</v>
+      </c>
       <c r="M258" s="4"/>
       <c r="N258" s="4"/>
-      <c r="O258" s="3" t="s">
-        <v>522</v>
-      </c>
+      <c r="O258" s="4"/>
       <c r="P258" s="4"/>
       <c r="Q258" s="4"/>
       <c r="R258" s="4"/>
@@ -15896,7 +15929,7 @@
     </row>
     <row r="259" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A259" s="4" t="s">
-        <v>523</v>
+        <v>517</v>
       </c>
       <c r="B259" s="4" t="s">
         <v>228</v>
@@ -15913,11 +15946,11 @@
       <c r="J259" s="4"/>
       <c r="K259" s="4"/>
       <c r="L259" s="4"/>
-      <c r="M259" s="4" t="s">
-        <v>524</v>
-      </c>
+      <c r="M259" s="4"/>
       <c r="N259" s="4"/>
-      <c r="O259" s="4"/>
+      <c r="O259" s="3" t="s">
+        <v>518</v>
+      </c>
       <c r="P259" s="4"/>
       <c r="Q259" s="4"/>
       <c r="R259" s="4"/>
@@ -15939,6 +15972,141 @@
       <c r="AH259" s="4"/>
       <c r="AI259" s="4"/>
     </row>
+    <row r="260" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A260" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="B260" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C260" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D260" s="4"/>
+      <c r="E260" s="4"/>
+      <c r="F260" s="4"/>
+      <c r="G260" s="4"/>
+      <c r="H260" s="4"/>
+      <c r="I260" s="4"/>
+      <c r="J260" s="4"/>
+      <c r="K260" s="4"/>
+      <c r="L260" s="4"/>
+      <c r="M260" s="4"/>
+      <c r="N260" s="4"/>
+      <c r="O260" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="P260" s="4"/>
+      <c r="Q260" s="4"/>
+      <c r="R260" s="4"/>
+      <c r="S260" s="4"/>
+      <c r="T260" s="4"/>
+      <c r="U260" s="4"/>
+      <c r="V260" s="4"/>
+      <c r="W260" s="4"/>
+      <c r="X260" s="4"/>
+      <c r="Y260" s="4"/>
+      <c r="Z260" s="4"/>
+      <c r="AA260" s="4"/>
+      <c r="AB260" s="4"/>
+      <c r="AC260" s="4"/>
+      <c r="AD260" s="4"/>
+      <c r="AE260" s="4"/>
+      <c r="AF260" s="4"/>
+      <c r="AG260" s="4"/>
+      <c r="AH260" s="4"/>
+      <c r="AI260" s="4"/>
+    </row>
+    <row r="261" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A261" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="B261" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C261" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D261" s="4"/>
+      <c r="E261" s="4"/>
+      <c r="F261" s="4"/>
+      <c r="G261" s="4"/>
+      <c r="H261" s="4"/>
+      <c r="I261" s="4"/>
+      <c r="J261" s="4"/>
+      <c r="K261" s="4"/>
+      <c r="L261" s="4"/>
+      <c r="M261" s="4"/>
+      <c r="N261" s="4"/>
+      <c r="O261" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="P261" s="4"/>
+      <c r="Q261" s="4"/>
+      <c r="R261" s="4"/>
+      <c r="S261" s="4"/>
+      <c r="T261" s="4"/>
+      <c r="U261" s="4"/>
+      <c r="V261" s="4"/>
+      <c r="W261" s="4"/>
+      <c r="X261" s="4"/>
+      <c r="Y261" s="4"/>
+      <c r="Z261" s="4"/>
+      <c r="AA261" s="4"/>
+      <c r="AB261" s="4"/>
+      <c r="AC261" s="4"/>
+      <c r="AD261" s="4"/>
+      <c r="AE261" s="4"/>
+      <c r="AF261" s="4"/>
+      <c r="AG261" s="4"/>
+      <c r="AH261" s="4"/>
+      <c r="AI261" s="4"/>
+    </row>
+    <row r="262" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A262" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="B262" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C262" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D262" s="4"/>
+      <c r="E262" s="4"/>
+      <c r="F262" s="4"/>
+      <c r="G262" s="4"/>
+      <c r="H262" s="4"/>
+      <c r="I262" s="4"/>
+      <c r="J262" s="4"/>
+      <c r="K262" s="4"/>
+      <c r="L262" s="4"/>
+      <c r="M262" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="N262" s="4"/>
+      <c r="O262" s="4"/>
+      <c r="P262" s="4"/>
+      <c r="Q262" s="4"/>
+      <c r="R262" s="4"/>
+      <c r="S262" s="4"/>
+      <c r="T262" s="4"/>
+      <c r="U262" s="4"/>
+      <c r="V262" s="4"/>
+      <c r="W262" s="4"/>
+      <c r="X262" s="4"/>
+      <c r="Y262" s="4"/>
+      <c r="Z262" s="4"/>
+      <c r="AA262" s="4"/>
+      <c r="AB262" s="4"/>
+      <c r="AC262" s="4"/>
+      <c r="AD262" s="4"/>
+      <c r="AE262" s="4"/>
+      <c r="AF262" s="4"/>
+      <c r="AG262" s="4"/>
+      <c r="AH262" s="4"/>
+      <c r="AI262" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15946,7 +16114,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B611D72-2CC2-4CCA-A1E6-2A10215873D6}">
-  <dimension ref="A1:T257"/>
+  <dimension ref="A1:T259"/>
   <sheetFormatPr def